<commit_message>
🤖 Noticias actualizadas 02/06/2026 09:34
</commit_message>
<xml_diff>
--- a/docs/ultimahora.xlsx
+++ b/docs/ultimahora.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Todas las noticias" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Todas las noticias'!$A$1:$E$259</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Todas las noticias'!$A$1:$E$251</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E259"/>
+  <dimension ref="A1:E251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -529,7 +529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 02:30 a. m.</t>
+          <t>02/06/2026 04:06 a. m.</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -544,19 +544,19 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Así opera el pico y placa en Bucaramanga para el martes 2 de junio de 2026</t>
+          <t>Movilidad en Bogotá martes 02 de junio: conozca acá el pico y placa en la ciudad</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/santander/asi-opera-el-pico-y-placa-en-bucaramanga-para-el-martes-2-de-junio-de-3561351</t>
+          <t>https://www.eltiempo.com/bogota/movilidad-en-bogota-martes-02-de-junio-conozca-aca-el-pico-y-placa-en-la-ciudad-3561364</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 02:30 a. m.</t>
+          <t>02/06/2026 04:05 a. m.</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -571,19 +571,19 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>¡Siga la medida de movilidad! Pico y placa en Medellín para el martes 2 de junio de 2026: así funciona la restricción</t>
+          <t>La Organización Meteorológica Mundial elevó al 90 por ciento la probabilidad de llegada del fenómeno de El Niño: 'Su impacto será aún más severo'</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/medellin/siga-la-medida-de-movilidad-pico-y-placa-en-medellin-para-el-martes-2-de-junio-de-2026-asi-funciona-la-restriccion-3561208</t>
+          <t>https://www.eltiempo.com/mundo/mas-regiones/la-organizacion-meteorologica-mundial-elevo-al-90-por-ciento-la-probabilidad-de-llegada-del-fenomeno-de-el-nino-su-impacto-sera-aun-mas-severo-3561365</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 02:30 a. m.</t>
+          <t>02/06/2026 03:00 a. m.</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -598,19 +598,19 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>¡Evite multas! Pico y placa en Cali para el martes 2 de junio de 2026: así opera la medida</t>
+          <t>Grave accidente de carro de alta gama dejó cinco heridos en Dosquebradas: conductor estaría en estado de embriaguez</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/cali/evite-multas-pico-y-placa-en-cali-para-el-martes-2-de-junio-de-2026-asi-opera-la-medida-3561163</t>
+          <t>https://www.eltiempo.com/colombia/otras-ciudades/grave-accidente-de-carro-de-alta-gama-dejo-cinco-heridos-en-dosquebradas-conductor-estaria-en-estado-de-embriaguez-3561362</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 02:25 a. m.</t>
+          <t>02/06/2026 02:40 a. m.</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -625,19 +625,19 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>¡Atención conductores! Pico y placa en Bogotá para el martes 2 de junio de 2026: así funciona la medida</t>
+          <t>¡Atención conductores! Pico y placa en Pereira para el martes 2 de junio de 2026: así regirá la medida</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/bogota/atencion-conductores-pico-y-placa-en-bogota-para-el-martes-2-de-junio-de-2026-asi-funciona-la-medida-3561156</t>
+          <t>https://www.eltiempo.com/colombia/otras-ciudades/atencion-conductores-pico-y-placa-en-pereira-para-el-martes-2-de-junio-de-2026-asi-regira-la-medida-3561352</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 01:21 a. m.</t>
+          <t>02/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -652,19 +652,19 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Temblor hoy en Colombia | Sismo durante la madrugada de este martes 02 de junio: epicentro, magnitud y profundidad</t>
+          <t>Así opera el pico y placa en Bucaramanga para el martes 2 de junio de 2026</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/otras-ciudades/temblor-hoy-en-colombia-sismo-durante-la-madrugada-de-este-martes-02-de-junio-epicentro-magnitud-y-profundidad-3561361</t>
+          <t>https://www.eltiempo.com/colombia/santander/asi-opera-el-pico-y-placa-en-bucaramanga-para-el-martes-2-de-junio-de-3561351</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 12:58 a. m.</t>
+          <t>02/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -679,19 +679,19 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Luto por la muerte del mayor general (r) Javier Alberto Ayala Amaya: reacciones tras fallecimiento del rector de la Universidad Militar Nueva Granada</t>
+          <t>¡Siga la medida de movilidad! Pico y placa en Medellín para el martes 2 de junio de 2026: así funciona la restricción</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/bogota/luto-por-la-muerte-del-mayor-general-r-javier-alberto-ayala-amaya-reacciones-tras-fallecimiento-del-rector-de-la-universidad-militar-nueva-granada-3561360</t>
+          <t>https://www.eltiempo.com/colombia/medellin/siga-la-medida-de-movilidad-pico-y-placa-en-medellin-para-el-martes-2-de-junio-de-2026-asi-funciona-la-restriccion-3561208</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 12:31 a. m.</t>
+          <t>02/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -706,19 +706,19 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>La Personería de Cali solicita acciones preventivas y protección integral ante recientes asesinatos de mujeres</t>
+          <t>¡Evite multas! Pico y placa en Cali para el martes 2 de junio de 2026: así opera la medida</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/cali/la-personeria-de-cali-solicita-acciones-preventivas-y-proteccion-integral-ante-recientes-asesinatos-de-mujeres-3561359</t>
+          <t>https://www.eltiempo.com/colombia/cali/evite-multas-pico-y-placa-en-cali-para-el-martes-2-de-junio-de-2026-asi-opera-la-medida-3561163</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 12:05 a. m.</t>
+          <t>02/06/2026 02:25 a. m.</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -733,19 +733,19 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Disturbios por Champions del PSG en Francia dejan un muerto y 890 detenidos: expertos vinculan la crisis con exclusión de jóvenes en las periferias</t>
+          <t>¡Atención conductores! Pico y placa en Bogotá para el martes 2 de junio de 2026: así funciona la medida</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/europa/disturbios-por-champions-del-psg-en-francia-dejan-un-muerto-y-890-detenidos-expertos-vinculan-la-crisis-con-exclusion-de-jovenes-en-las-periferias-3561226</t>
+          <t>https://www.eltiempo.com/bogota/atencion-conductores-pico-y-placa-en-bogota-para-el-martes-2-de-junio-de-2026-asi-funciona-la-medida-3561156</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 11:15 p. m.</t>
+          <t>02/06/2026 01:21 a. m.</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -760,19 +760,19 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Diferentes sectores hacen un llamado de respaldo a la organización electoral</t>
+          <t>Temblor hoy en Colombia | Sismo durante la madrugada de este martes 02 de junio: epicentro, magnitud y profundidad</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/diferentes-sectores-hacen-un-llamado-de-respaldo-a-la-organizacion-electoral-3561344</t>
+          <t>https://www.eltiempo.com/colombia/otras-ciudades/temblor-hoy-en-colombia-sismo-durante-la-madrugada-de-este-martes-02-de-junio-epicentro-magnitud-y-profundidad-3561361</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 11:14 p. m.</t>
+          <t>02/06/2026 12:58 a. m.</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -787,19 +787,19 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Habló hermana de Alexander Avendaño, joven que murió ahogado en embalse de Guatapé tras presunta pelea: 'Nadie lo ayudaba'</t>
+          <t>Luto por la muerte del mayor general (r) Javier Alberto Ayala Amaya: reacciones tras fallecimiento del rector de la Universidad Militar Nueva Granada</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/medellin/hablo-hermana-de-alexander-avendano-joven-que-murio-ahogado-en-embalse-de-guatape-tras-presunta-pelea-nadie-lo-ayudaba-3561358</t>
+          <t>https://www.eltiempo.com/bogota/luto-por-la-muerte-del-mayor-general-r-javier-alberto-ayala-amaya-reacciones-tras-fallecimiento-del-rector-de-la-universidad-militar-nueva-granada-3561360</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 11:05 p. m.</t>
+          <t>02/06/2026 12:31 a. m.</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -814,19 +814,19 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Junior de Barranquilla vs. Atlético Nacional, primer 'round' de la final de la Liga BetPlay: horario y canal de TV</t>
+          <t>La Personería de Cali solicita acciones preventivas y protección integral ante recientes asesinatos de mujeres</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-colombiano/junior-de-barranquilla-vs-atletico-nacional-primer-round-de-la-final-de-la-liga-betplay-horario-y-canal-de-tv-3561224</t>
+          <t>https://www.eltiempo.com/colombia/cali/la-personeria-de-cali-solicita-acciones-preventivas-y-proteccion-integral-ante-recientes-asesinatos-de-mujeres-3561359</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 11:02 p. m.</t>
+          <t>02/06/2026 12:05 a. m.</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -841,19 +841,19 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Así jugó Colombia contra Costa Rica: Luis Díaz, el más destacado en un encuentro en el que se probaron muchas piezas</t>
+          <t>Disturbios por Champions del PSG en Francia dejan un muerto y 890 detenidos: expertos vinculan la crisis con exclusión de jóvenes en las periferias</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/asi-jugo-colombia-contra-costa-rica-luis-diaz-el-mas-destacado-en-un-encuentro-en-el-que-se-probaron-muchas-piezas-3561357</t>
+          <t>https://www.eltiempo.com/mundo/europa/disturbios-por-champions-del-psg-en-francia-dejan-un-muerto-y-890-detenidos-expertos-vinculan-la-crisis-con-exclusion-de-jovenes-en-las-periferias-3561226</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 10:45 p. m.</t>
+          <t>01/06/2026 11:15 p. m.</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -868,19 +868,19 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>¿Cuándo se conocerán los resultados oficiales de las elecciones presidenciales? El registrador explicó qué sigue en el escrutinio: 'Par de días'</t>
+          <t>Diferentes sectores hacen un llamado de respaldo a la organización electoral</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/cuando-se-conoceran-los-resultados-oficiales-de-las-elecciones-presidenciales-el-registrador-explico-que-sigue-en-el-escrutinio-par-de-dias-3561356</t>
+          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/diferentes-sectores-hacen-un-llamado-de-respaldo-a-la-organizacion-electoral-3561344</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 10:44 p. m.</t>
+          <t>01/06/2026 11:14 p. m.</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -895,19 +895,19 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>¿Quién era el mayor general (r) Javier Alberto Ayala Amaya, rector de la Universidad Militar Nueva Granada, que falleció este 1 de junio?</t>
+          <t>Habló hermana de Alexander Avendaño, joven que murió ahogado en embalse de Guatapé tras presunta pelea: 'Nadie lo ayudaba'</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/bogota/quien-era-el-mayor-general-r-javier-alberto-ayala-amaya-rector-de-la-universidad-militar-nueva-granada-que-fallecio-este-1-de-junio-3561354</t>
+          <t>https://www.eltiempo.com/colombia/medellin/hablo-hermana-de-alexander-avendano-joven-que-murio-ahogado-en-embalse-de-guatape-tras-presunta-pelea-nadie-lo-ayudaba-3561358</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 10:40 p. m.</t>
+          <t>01/06/2026 11:05 p. m.</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -922,19 +922,19 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Kai Trewin, el otro futbolista desconocido que se hace viral antes del Mundial, tal como Tim Payne</t>
+          <t>Junior de Barranquilla vs. Atlético Nacional, primer 'round' de la final de la Liga BetPlay: horario y canal de TV</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/kai-trewin-el-otro-futbolista-desconocido-que-se-hace-viral-antes-del-mundial-tal-como-tim-payne-3561355</t>
+          <t>https://www.eltiempo.com/deportes/futbol-colombiano/junior-de-barranquilla-vs-atletico-nacional-primer-round-de-la-final-de-la-liga-betplay-horario-y-canal-de-tv-3561224</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 10:37 p. m.</t>
+          <t>01/06/2026 11:02 p. m.</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -949,19 +949,19 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>Fiscalía imputó a la alcaldesa de Ibagué, Johana Ximena Aranda, por presuntas irregularidades en un contrato de alimentación animal</t>
+          <t>Así jugó Colombia contra Costa Rica: Luis Díaz, el más destacado en un encuentro en el que se probaron muchas piezas</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/justicia/delitos/fiscalia-imputo-a-johana-ximena-aranda-alcaldesa-de-ibague-y-a-cuatro-personas-mas-por-presuntas-irregularidades-en-contrato-de-alimentacion-animal-3561349</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/asi-jugo-colombia-contra-costa-rica-luis-diaz-el-mas-destacado-en-un-encuentro-en-el-que-se-probaron-muchas-piezas-3561357</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 10:30 p. m.</t>
+          <t>01/06/2026 10:45 p. m.</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -976,19 +976,19 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Venezuela cumple 9 años sin trasplantes de órganos, una deuda que le ha costado la vida de cientos de niños y niñas</t>
+          <t>¿Cuándo se conocerán los resultados oficiales de las elecciones presidenciales? El registrador explicó qué sigue en el escrutinio: 'Par de días'</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/venezuela/venezuela-cumple-9-anos-sin-trasplantes-de-organos-una-deuda-que-le-ha-costado-la-vida-de-cientos-de-ninos-y-ninas-3561242</t>
+          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/cuando-se-conoceran-los-resultados-oficiales-de-las-elecciones-presidenciales-el-registrador-explico-que-sigue-en-el-escrutinio-par-de-dias-3561356</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 10:27 p. m.</t>
+          <t>01/06/2026 10:44 p. m.</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -1003,19 +1003,19 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Néstor Lorenzo y su balance tras ganarle a Costa Rica: ‘Tenemos que mejorar mucho, pero eso se va a dar con el paso de los días’</t>
+          <t>¿Quién era el mayor general (r) Javier Alberto Ayala Amaya, rector de la Universidad Militar Nueva Granada, que falleció este 1 de junio?</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/nestor-lorenzo-y-su-balance-tras-ganarle-a-costa-rica-tenemos-que-mejorar-mucho-pero-eso-se-va-a-dar-con-el-paso-de-los-dias-3561353</t>
+          <t>https://www.eltiempo.com/bogota/quien-era-el-mayor-general-r-javier-alberto-ayala-amaya-rector-de-la-universidad-militar-nueva-granada-que-fallecio-este-1-de-junio-3561354</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 10:25 p. m.</t>
+          <t>01/06/2026 10:40 p. m.</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1030,19 +1030,19 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>América Latina y el Caribe envejece a velocidad récord: Colombia, entre los países más afectados en las próximas décadas</t>
+          <t>Kai Trewin, el otro futbolista desconocido que se hace viral antes del Mundial, tal como Tim Payne</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/latinoamerica/america-latina-y-el-caribe-envejece-a-velocidad-record-colombia-entre-los-paises-mas-afectados-en-las-proximas-decadas-3561188</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/kai-trewin-el-otro-futbolista-desconocido-que-se-hace-viral-antes-del-mundial-tal-como-tim-payne-3561355</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 10:24 p. m.</t>
+          <t>01/06/2026 10:37 p. m.</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
@@ -1057,19 +1057,19 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Una ruta realista para recuperar la seguridad en territorios críticos</t>
+          <t>Fiscalía imputó a la alcaldesa de Ibagué, Johana Ximena Aranda, por presuntas irregularidades en un contrato de alimentación animal</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/una-ruta-realista-para-recuperar-la-seguridad-en-territorios-criticos-3561348</t>
+          <t>https://www.eltiempo.com/justicia/delitos/fiscalia-imputo-a-johana-ximena-aranda-alcaldesa-de-ibague-y-a-cuatro-personas-mas-por-presuntas-irregularidades-en-contrato-de-alimentacion-animal-3561349</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 07:32 a. m.</t>
+          <t>02/06/2026 08:29 a. m.</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1079,24 +1079,24 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Operativo humanitario en Arauca logra liberación de dos retenidos en zona fronteriza</t>
+          <t>Seguidores de Iván Cepeda marcharon en Bogotá y De la Espriella hizo llamado</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/01/operativo-humanitario-en-arauca-logra-liberacion-de-dos-retenidos-en-zona-fronteriza/</t>
+          <t>https://www.lafm.com.co/politica/seguidores-de-ivan-cepeda-marcharon-en-bogota-y-de-la-espriella-hizo-llamadozo-llam-401088</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 07:08 a. m.</t>
+          <t>02/06/2026 03:31 a. m.</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -1106,24 +1106,24 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Alcalde de Bogotá llama a respetar resultados tras jornada electoral en Colombia</t>
+          <t>Siete menores y un adulto mayor heridos por ataque con explosivos en Suárez, Cauca</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/01/alcalde-de-bogota-llama-a-respetar-resultados-tras-jornada-electoral-en-colombia/</t>
+          <t>https://www.lafm.com.co/orden-publico/violento-ataque-de-las-disidencias-de-las-farc-en-suarez-cauca-401086</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 01:00 a. m.</t>
+          <t>02/06/2026 02:41 a. m.</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1133,24 +1133,24 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Pusimos una raya al Tigre</t>
+          <t>“No haré acuerdos”, le dice De la Espriella a quienes anunciaron apoyo a su campaña</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/luis-ernesto-ruiz/2026/06/02/pusimos-una-raya-al-tigre/</t>
+          <t>https://www.lafm.com.co/politica/abelardo-espriella-descarta-acuerdos-politicos-segunda-vuelta-elecciones-2026-401082</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 01:00 a. m.</t>
+          <t>02/06/2026 02:21 a. m.</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
@@ -1160,24 +1160,24 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Luis Ernesto Ruíz</t>
+          <t>Así fue la presentación de Morat en el Estadio Campín antes del partido de Colombia</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/luis-ernesto-ruiz/</t>
+          <t>https://www.lafm.com.co/deportes/seleccion-colombia-mundial-2026-despedida-presentacion-morat-401078</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 01:00 a. m.</t>
+          <t>02/06/2026 02:19 a. m.</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1187,24 +1187,24 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>La cultura como escenario común</t>
+          <t>¿Qué se celebra este 2 de junio en Colombia y por qué es una fecha importante para millones de personas?</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/2026/06/02/la-cultura-como-escenario-comun/</t>
+          <t>https://www.lafm.com.co/sociedad/celebracion-dia-2-de-junio-colombia-2026-401080</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 01:00 a. m.</t>
+          <t>02/06/2026 01:55 a. m.</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -1214,24 +1214,24 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>A Gabriel Latorre Carvajal</t>
+          <t>Imputan a alcaldesa de Ibagué por presuntas irregularidades en contrato de comida para mascotas</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/02/a-gabriel-latorre-carvajal/</t>
+          <t>https://www.lafm.com.co/orden-publico/alcaldesa-ibague-irregularidades-contrato-comida-mascotas-fiscalia-401079</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 01:00 a. m.</t>
+          <t>02/06/2026 01:15 a. m.</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1241,24 +1241,24 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Columnistas</t>
+          <t>Colombia vs. Jordania: Cuándo y dónde ver el partido antes del debut en el mundial 2026</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/</t>
+          <t>https://www.lafm.com.co/deportes/colombia-vs-jordania-cuando-donde-ver-partido-401077</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 01:00 a. m.</t>
+          <t>02/06/2026 12:56 a. m.</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -1268,24 +1268,24 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>Unidos por Colombia</t>
+          <t>Las tres grandes conclusiones que dejó la primera vuelta presidencial en Colombia</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/02/unidos-por-colombia/</t>
+          <t>https://www.lafm.com.co/deportes/primera-vuelta-presidencial-colombia-tres-conclusiones-clave-401076</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 08:11 p. m.</t>
+          <t>02/06/2026 12:21 a. m.</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1295,24 +1295,24 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Cerrejón suspende operaciones en La Guajira: más de 12.000 trabajadores afectados</t>
+          <t>Festivos en Colombia 2026: Cuántos puentes hay junio, cuándo son y qué se celebra</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/01/cerrejon-suspende-operaciones-en-la-guajira-mas-de-12000-trabajadores-afectados/</t>
+          <t>https://www.lafm.com.co/sociedad/puentes-festivos-junio-colombia-2026-dias-fechas-y-celebraciones-401075</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 08:11 p. m.</t>
+          <t>02/06/2026 12:17 a. m.</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -1322,24 +1322,24 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Colombia goleó a Costa Rica por fecha FIFA antes de viajar a Estados Unidos</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/</t>
+          <t>https://www.lafm.com.co/deportes/seleccion-colombia-mundial-2026-resultado-goles-costa-rica-fecha-fifa-401069</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 05:01 p. m.</t>
+          <t>02/06/2026 12:12 a. m.</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1349,24 +1349,24 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Tragedia en Villavicencio: revelan quiénes eran los ocupantes de la avioneta siniestrada</t>
+          <t>Elecciones en Colombia: Registraduría aclara quiénes NO podrán votar en la segunda vuelta</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/01/tragedia-en-villavicencio-revelan-quienes-eran-los-ocupantes-de-la-avioneta-siniestrada/</t>
+          <t>https://www.lafm.com.co/actualidad/elecciones-colombia-2026-segunda-vuelta-quienes-no-pueden-votar-401073</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 05:00 p. m.</t>
+          <t>01/06/2026 11:21 p. m.</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
@@ -1376,24 +1376,24 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>Petro lanza explosiva acusación contra Abelardo De La Espriella: “Detrás de él está el fascismo mafioso”</t>
+          <t>"Le quitaron la ropa, lo golpearon y nadie lo ayudó": familia de Alexander Avendaño pide justicia tras tragedia en Guatapé</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/01/petro-lanza-explosiva-acusacion-contra-abelardo-de-la-espriella-detras-de-el-esta-el-fascismo-mafioso/</t>
+          <t>https://www.lafm.com.co/sociedad/alexander-avendano-guatape-muerte-joven-antioquia-401070</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 02:12 p. m.</t>
+          <t>01/06/2026 10:37 p. m.</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1403,24 +1403,24 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>¿Si votó? Pues estas son las promociones y beneficios que le ofrecen el Estado y sector comercial</t>
+          <t>Se filtran dos nuevos dispositivos de Apple que ya estarían listos para salir al mercado</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/01/si-voto-pues-estas-son-las-promociones-y-beneficios-que-le-ofrecen-el-estado-y-sector-comercial/</t>
+          <t>https://www.lafm.com.co/sociedad/filtracion-nuevos-dispositvos-apple-salir-mercado-2026-401067</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 12:47 p. m.</t>
+          <t>31/05/2026 01:47 p. m.</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
@@ -1430,24 +1430,24 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>Avioneta en Villavicencio se accidentó mientras despegaba: hay cuatro muertos</t>
+          <t>“Tomaré mis propias decisiones; yo mismo me pondré al frente”: Petro tras los resultados de la primera vuelta</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/01/avioneta-en-villavicencio-se-accidento-mientras-despegaba-hay-cuatro-muertos/</t>
+          <t>https://www.lafm.com.co/politica/petro-habla-de-resultados-de-elecciones-y-dice-que-se-pondra-al-frente-renunciara-401046</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 12:34 p. m.</t>
+          <t>18/04/2026 03:41 p. m.</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1457,24 +1457,24 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>¿Quién es la esposa de Iván Cepeda? candidato a la Presidencia de Colombia</t>
+          <t>Tres heridos y 200 familias confinadas por combates en Suárez, Cauca</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/01/quien-es-la-esposa-de-ivan-cepeda-y-cuantos-hijos-tiene-el-candidato-a-la-presidencia-de-colombia/</t>
+          <t>https://www.lafm.com.co/orden-publico/tres-heridos-y-200-familias-confinadas-por-combates-en-suarez-cauca-401087</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 11:41 a. m.</t>
+          <t>27/12/2025 07:07 p. m.</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
@@ -1484,17 +1484,17 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>De la Espriella acepta debatir con Cepeda si antes acepta los resultados de las elecciones</t>
+          <t>DIAN lanza advertencia urgente: estas entidades perderían beneficios tributarios el 30 de junio</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/01/de-la-espriella-acepta-debatir-con-cepeda-si-antes-acepta-los-resultados-de-las-elecciones/</t>
+          <t>https://www.lafm.com.co/economia/dian-beneficios-tributarios-fehca-limite-30-junio-beneficiados-401064</t>
         </is>
       </c>
     </row>
@@ -1507,26 +1507,22 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Capturan a alias ‘Chalia’ en el Chocó</t>
+          <t>Lotería de Cundinamarca: resultado del premio mayor de $10.000 millones hoy 1 de junio de 2026</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/05/31/capturan-a-alias-chalia-en-el-choco/</t>
+          <t>https://www.lafm.com.co/sociedad/loteria-de-cundinamarca-resultado-del-premio-mayor-de-10000-millones-hoy-1-de-junio-de-2026-401081</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="inlineStr">
-        <is>
-          <t>02/06/2026 03:31 a. m.</t>
-        </is>
-      </c>
+      <c r="A39" s="5" t="inlineStr"/>
       <c r="B39" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1539,21 +1535,17 @@
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>Siete menores y un adulto mayor heridos por ataque con explosivos en Suárez, Cauca</t>
+          <t>Colpensiones confirma quiénes pueden trasladarse desde una AFP en 2026: esta es la fecha límite</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/orden-publico/violento-ataque-de-las-disidencias-de-las-farc-en-suarez-cauca-401086</t>
+          <t>https://www.lafm.com.co/economia/traslado-afp-colpensiones-2026-fecha-limite-requisitos-401083</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>02/06/2026 02:35 a. m.</t>
-        </is>
-      </c>
+      <c r="A40" s="2" t="inlineStr"/>
       <c r="B40" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1566,21 +1558,17 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Lotería de Cundinamarca: resultado del premio mayor de $10.000 millones hoy 1 de junio de 2026</t>
+          <t>Fallece Javier Alberto Ayala Amaya, rector de la Universidad Militar Nueva Granada y exgeneral del Ejército</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/sociedad/loteria-de-cundinamarca-resultado-del-premio-mayor-de-10000-millones-hoy-1-de-junio-de-2026-401081</t>
+          <t>https://www.lafm.com.co/actualidad/universidad-militar-nueva-granada-confirma-muerte-rector-javier-alberto-ayala-amaya-401072</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="inlineStr">
-        <is>
-          <t>02/06/2026 02:21 a. m.</t>
-        </is>
-      </c>
+      <c r="A41" s="5" t="inlineStr"/>
       <c r="B41" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1593,19 +1581,19 @@
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>Así fue la presentación de Morat en el Estadio Campín antes del partido de Colombia</t>
+          <t>César Gaviria arremete contra Petro: “gobierne o renuncie, pero no le haga más daño a la democracia”</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/deportes/seleccion-colombia-mundial-2026-despedida-presentacion-morat-401078</t>
+          <t>https://www.lafm.com.co/politica/cesar-gaviria-arremete-contra-petro-gobierne-renuncie-pero-no-le-haga-dano-a-la-democracia-401071</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 02:19 a. m.</t>
+          <t>02/06/2026 07:32 a. m.</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -1615,24 +1603,24 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>¿Qué se celebra este 2 de junio en Colombia y por qué es una fecha importante para millones de personas?</t>
+          <t>Operativo humanitario en Arauca logra liberación de dos retenidos en zona fronteriza</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/sociedad/celebracion-dia-2-de-junio-colombia-2026-401080</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/01/operativo-humanitario-en-arauca-logra-liberacion-de-dos-retenidos-en-zona-fronteriza/</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 01:55 a. m.</t>
+          <t>02/06/2026 07:08 a. m.</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
@@ -1642,24 +1630,24 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>Imputan a alcaldesa de Ibagué por presuntas irregularidades en contrato de comida para mascotas</t>
+          <t>Alcalde de Bogotá llama a respetar resultados tras jornada electoral en Colombia</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/orden-publico/alcaldesa-ibague-irregularidades-contrato-comida-mascotas-fiscalia-401079</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/01/alcalde-de-bogota-llama-a-respetar-resultados-tras-jornada-electoral-en-colombia/</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 01:15 a. m.</t>
+          <t>02/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -1669,24 +1657,24 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Colombia vs. Jordania: Cuándo y dónde ver el partido antes del debut en el mundial 2026</t>
+          <t>Pusimos una raya al Tigre</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/deportes/colombia-vs-jordania-cuando-donde-ver-partido-401077</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/luis-ernesto-ruiz/2026/06/02/pusimos-una-raya-al-tigre/</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 12:56 a. m.</t>
+          <t>02/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
@@ -1696,24 +1684,24 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>Las tres grandes conclusiones que dejó la primera vuelta presidencial en Colombia</t>
+          <t>Luis Ernesto Ruíz</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/deportes/primera-vuelta-presidencial-colombia-tres-conclusiones-clave-401076</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/luis-ernesto-ruiz/</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 12:21 a. m.</t>
+          <t>02/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -1723,24 +1711,24 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Festivos en Colombia 2026: Cuántos puentes hay junio, cuándo son y qué se celebra</t>
+          <t>Unidos por Colombia</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/sociedad/puentes-festivos-junio-colombia-2026-dias-fechas-y-celebraciones-401075</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/02/unidos-por-colombia/</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 12:17 a. m.</t>
+          <t>02/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
@@ -1750,24 +1738,24 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>Colombia goleó a Costa Rica por fecha FIFA antes de viajar a Estados Unidos</t>
+          <t>Columnistas</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/deportes/seleccion-colombia-mundial-2026-resultado-goles-costa-rica-fecha-fifa-401069</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 12:12 a. m.</t>
+          <t>02/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -1777,24 +1765,24 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Elecciones en Colombia: Registraduría aclara quiénes NO podrán votar en la segunda vuelta</t>
+          <t>La cultura como escenario común</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/actualidad/elecciones-colombia-2026-segunda-vuelta-quienes-no-pueden-votar-401073</t>
+          <t>https://www.vanguardia.com/opinion/2026/06/02/la-cultura-como-escenario-comun/</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 11:21 p. m.</t>
+          <t>02/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
@@ -1804,24 +1792,24 @@
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>"Le quitaron la ropa, lo golpearon y nadie lo ayudó": familia de Alexander Avendaño pide justicia tras tragedia en Guatapé</t>
+          <t>A Gabriel Latorre Carvajal</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/sociedad/alexander-avendano-guatape-muerte-joven-antioquia-401070</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/02/a-gabriel-latorre-carvajal/</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 10:37 p. m.</t>
+          <t>01/06/2026 08:11 p. m.</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -1831,24 +1819,24 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>Se filtran dos nuevos dispositivos de Apple que ya estarían listos para salir al mercado</t>
+          <t>Cerrejón suspende operaciones en La Guajira: más de 12.000 trabajadores afectados</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/sociedad/filtracion-nuevos-dispositvos-apple-salir-mercado-2026-401067</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/01/cerrejon-suspende-operaciones-en-la-guajira-mas-de-12000-trabajadores-afectados/</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 05:33 p. m.</t>
+          <t>01/06/2026 08:11 p. m.</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
@@ -1858,24 +1846,24 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>Juez mantiene excluidos los interrogatorios de Nicolás Petro y niega recurso de la Fiscalía</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/orden-publico/nicolas-petro-interrogatorio-excluido-del-proceso-fiscalia-401066</t>
+          <t>https://www.vanguardia.com/colombia/</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>31/05/2026 01:47 p. m.</t>
+          <t>01/06/2026 05:01 p. m.</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -1885,24 +1873,24 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>“Tomaré mis propias decisiones; yo mismo me pondré al frente”: Petro tras los resultados de la primera vuelta</t>
+          <t>Tragedia en Villavicencio: revelan quiénes eran los ocupantes de la avioneta siniestrada</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/petro-habla-de-resultados-de-elecciones-y-dice-que-se-pondra-al-frente-renunciara-401046</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/01/tragedia-en-villavicencio-revelan-quienes-eran-los-ocupantes-de-la-avioneta-siniestrada/</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>18/04/2026 03:41 p. m.</t>
+          <t>01/06/2026 05:00 p. m.</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
@@ -1912,24 +1900,24 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>Tres heridos y 200 familias confinadas por combates en Suárez, Cauca</t>
+          <t>Petro lanza explosiva acusación contra Abelardo De La Espriella: “Detrás de él está el fascismo mafioso”</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/orden-publico/tres-heridos-y-200-familias-confinadas-por-combates-en-suarez-cauca-401087</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/01/petro-lanza-explosiva-acusacion-contra-abelardo-de-la-espriella-detras-de-el-esta-el-fascismo-mafioso/</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>27/12/2025 07:07 p. m.</t>
+          <t>01/06/2026 02:12 p. m.</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -1939,22 +1927,26 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>DIAN lanza advertencia urgente: estas entidades perderían beneficios tributarios el 30 de junio</t>
+          <t>¿Si votó? Pues estas son las promociones y beneficios que le ofrecen el Estado y sector comercial</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/economia/dian-beneficios-tributarios-fehca-limite-30-junio-beneficiados-401064</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/01/si-voto-pues-estas-son-las-promociones-y-beneficios-que-le-ofrecen-el-estado-y-sector-comercial/</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="5" t="inlineStr"/>
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>01/06/2026 12:47 p. m.</t>
+        </is>
+      </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1962,22 +1954,26 @@
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>Colpensiones confirma quiénes pueden trasladarse desde una AFP en 2026: esta es la fecha límite</t>
+          <t>Avioneta en Villavicencio se accidentó mientras despegaba: hay cuatro muertos</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/economia/traslado-afp-colpensiones-2026-fecha-limite-requisitos-401083</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/01/avioneta-en-villavicencio-se-accidento-mientras-despegaba-hay-cuatro-muertos/</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr"/>
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>01/06/2026 12:34 p. m.</t>
+        </is>
+      </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1985,22 +1981,26 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>“No haré acuerdos”, le dice De la Espriella a quienes anunciaron apoyo a su campaña</t>
+          <t>¿Quién es la esposa de Iván Cepeda? candidato a la Presidencia de Colombia</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/abelardo-espriella-descarta-acuerdos-politicos-segunda-vuelta-elecciones-2026-401082</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/01/quien-es-la-esposa-de-ivan-cepeda-y-cuantos-hijos-tiene-el-candidato-a-la-presidencia-de-colombia/</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="5" t="inlineStr"/>
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>01/06/2026 11:41 a. m.</t>
+        </is>
+      </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2008,17 +2008,17 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>Fallece Javier Alberto Ayala Amaya, rector de la Universidad Militar Nueva Granada y exgeneral del Ejército</t>
+          <t>De la Espriella acepta debatir con Cepeda si antes acepta los resultados de las elecciones</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/actualidad/universidad-militar-nueva-granada-confirma-muerte-rector-javier-alberto-ayala-amaya-401072</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/01/de-la-espriella-acepta-debatir-con-cepeda-si-antes-acepta-los-resultados-de-las-elecciones/</t>
         </is>
       </c>
     </row>
@@ -2031,17 +2031,17 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>César Gaviria arremete contra Petro: “gobierne o renuncie, pero no le haga más daño a la democracia”</t>
+          <t>Capturan a alias ‘Chalia’ en el Chocó</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/cesar-gaviria-arremete-contra-petro-gobierne-renuncie-pero-no-le-haga-dano-a-la-democracia-401071</t>
+          <t>https://www.vanguardia.com/colombia/2026/05/31/capturan-a-alias-chalia-en-el-choco/</t>
         </is>
       </c>
     </row>
@@ -2667,11 +2667,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="inlineStr">
-        <is>
-          <t>01/06/2026 09:51 p. m.</t>
-        </is>
-      </c>
+      <c r="A82" s="2" t="inlineStr"/>
       <c r="B82" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3551,12 +3547,12 @@
       </c>
       <c r="D115" s="6" t="inlineStr">
         <is>
-          <t>Directora de la MOE advierte que Petro solo podría liderar la campaña de Iván Cepeda si renuncia a la presidencia</t>
+          <t>Más de 560.000 empleos dependen del sector automotor, pero la informalidad sigue siendo uno de sus mayores desafíos</t>
         </is>
       </c>
       <c r="E115" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/02/directora-de-la-moe-advierte-que-petro-solo-podria-liderar-la-campana-de-ivan-cepeda-si-renuncia-a-la-presidencia/</t>
+          <t>https://www.infobae.com/colombia/2026/06/02/mas-de-560000-empleos-dependen-del-sector-automotor-pero-la-informalidad-sigue-siendo-uno-de-sus-mayores-desafios/</t>
         </is>
       </c>
     </row>
@@ -3578,12 +3574,12 @@
       </c>
       <c r="D116" s="3" t="inlineStr">
         <is>
-          <t>Resultado Baloto y Revancha hoy lunes 1 de junio</t>
+          <t>“La vida de los colombianos no da espera”: Acemi pide que los pacientes críticos sean la prioridad del próximo gobierno</t>
         </is>
       </c>
       <c r="E116" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/02/resultado-baloto-y-revancha-hoy-lunes-1-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/02/la-vida-de-los-colombianos-no-da-espera-acemi-pide-que-los-pacientes-criticos-sean-la-prioridad-del-proximo-gobierno/</t>
         </is>
       </c>
     </row>
@@ -3605,12 +3601,12 @@
       </c>
       <c r="D117" s="6" t="inlineStr">
         <is>
-          <t>TransMilenio cambió el nombre de la estación Calle 26 en Bogotá: así se llamará desde ahora</t>
+          <t>Generales y almirantes en retiro cuestionan a Petro por dudar del preconteo electoral y piden respetar los resultados</t>
         </is>
       </c>
       <c r="E117" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/02/transmilenio-cambio-el-nombre-de-la-estacion-calle-26-en-bogota-asi-se-llamara-desde-ahora/</t>
+          <t>https://www.infobae.com/colombia/2026/06/02/generales-y-almirantes-en-retiro-cuestionan-a-petro-por-dudar-del-preconteo-electoral-y-piden-respetar-los-resultados/</t>
         </is>
       </c>
     </row>
@@ -3632,12 +3628,12 @@
       </c>
       <c r="D118" s="3" t="inlineStr">
         <is>
-          <t>Hallan muerto a un menor de 13 años en un potrero de Valle del Cauca: investigan quiénes están detrás del crimen</t>
+          <t>“Renuncie al cargo y demuestre cómo se ponen 15 millones de votos”: embajador Alfredo Saade le pidió a Petro dejar la Presidencia</t>
         </is>
       </c>
       <c r="E118" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/02/hallan-muerto-a-un-menor-de-13-anos-en-un-potrero-de-valle-del-cauca-investigan-quienes-estan-detras-del-crimen/</t>
+          <t>https://www.infobae.com/colombia/2026/06/02/renuncie-al-cargo-y-demuestre-como-se-ponen-15-millones-de-votos-embajador-alfredo-saade-le-pidio-a-petro-dejar-la-presidencia/</t>
         </is>
       </c>
     </row>
@@ -3659,12 +3655,12 @@
       </c>
       <c r="D119" s="6" t="inlineStr">
         <is>
-          <t>Resultado Lotería de Cundinamarca hoy lunes 1 de junio</t>
+          <t>JEP vuelve a escuchar a Mario Montoya por caso de falsos positivos: exsubalternos lo señalan en 30 testimonios</t>
         </is>
       </c>
       <c r="E119" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/02/resultado-loteria-de-cundinamarca-hoy-lunes-1-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/02/jep-vuelve-a-escuchar-a-mario-montoya-por-caso-de-falsos-positivos-exsubalternos-lo-senalan-en-30-testimonios/</t>
         </is>
       </c>
     </row>
@@ -3686,12 +3682,12 @@
       </c>
       <c r="D120" s="3" t="inlineStr">
         <is>
-          <t>Tras críticas a Abelardo, reviven video de la campaña de Iván Cepeda promoviendo el uso de la camiseta de la Selección</t>
+          <t>“Convocamos a todos los colombianos que quieren un país con esperanza”: José Manuel Restrepo tras el triunfo de Abelardo de la Espriella</t>
         </is>
       </c>
       <c r="E120" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/02/tras-criticas-a-abelardo-reviven-video-de-la-campana-de-ivan-cepeda-promoviendo-el-uso-de-la-camiseta-de-la-seleccion/</t>
+          <t>https://www.infobae.com/colombia/2026/06/02/convocamos-a-todos-los-colombianos-que-quieren-un-pais-con-esperanza-jose-manuel-restrepo-tras-el-triunfo-de-abelardo-de-la-espriella/</t>
         </is>
       </c>
     </row>
@@ -3713,12 +3709,12 @@
       </c>
       <c r="D121" s="6" t="inlineStr">
         <is>
-          <t>Resultado Super Astro Luna HOY: número ganador del lunes 1 de junio</t>
+          <t>Suspensión de Cerrejón genera alerta en La Guajira por riesgo para el empleo y los ingresos regionales</t>
         </is>
       </c>
       <c r="E121" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/02/resultado-super-astro-luna-hoy-numero-ganador-del-lunes-1-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/02/suspension-de-cerrejon-genera-alerta-en-la-guajira-por-riesgo-para-el-empleo-y-los-ingresos-regionales/</t>
         </is>
       </c>
     </row>
@@ -3740,12 +3736,12 @@
       </c>
       <c r="D122" s="3" t="inlineStr">
         <is>
-          <t>Resultado Sinuano Noche hoy 1 de junio</t>
+          <t>Vicky Dávila acusa a Iván Cepeda y Gustavo Petro de querer “incendiar las calles” tras manifestación en Bogotá</t>
         </is>
       </c>
       <c r="E122" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/02/resultado-sinuano-noche-hoy-1-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/02/vicky-davila-acusa-a-ivan-cepeda-y-gustavo-petro-de-querer-incendiar-las-calles-tras-manifestacion-en-bogota/</t>
         </is>
       </c>
     </row>
@@ -3767,12 +3763,12 @@
       </c>
       <c r="D123" s="6" t="inlineStr">
         <is>
-          <t>Pico y Placa: qué autos descansan en Villavicencio este martes 2 de junio</t>
+          <t>Bogotá: la previsión meteorológica para este 2 de junio</t>
         </is>
       </c>
       <c r="E123" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/02/pico-y-placa-que-autos-descansan-en-villavicencio-este-martes-2-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/02/bogota-la-prevision-meteorologica-para-este-2-de-junio/</t>
         </is>
       </c>
     </row>
@@ -3794,12 +3790,12 @@
       </c>
       <c r="D124" s="3" t="inlineStr">
         <is>
-          <t>Tenga en cuenta: así regirá el Pico y Placa en Cartagena este martes 2 de junio</t>
+          <t>Pronóstico del clima en Cali este martes 2 de junio: temperatura, lluvias y viento</t>
         </is>
       </c>
       <c r="E124" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/02/tenga-en-cuenta-asi-regira-el-pico-y-placa-en-cartagena-este-martes-2-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/02/pronostico-del-clima-en-cali-este-martes-2-de-junio-temperatura-lluvias-y-viento/</t>
         </is>
       </c>
     </row>
@@ -3821,12 +3817,12 @@
       </c>
       <c r="D125" s="6" t="inlineStr">
         <is>
-          <t>Pico y Placa en Cali: restricciones vehiculares para evitar multas este martes 2 de junio</t>
+          <t>Clima en Cartagena de Indias: la predicción para este 2 de junio</t>
         </is>
       </c>
       <c r="E125" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/02/pico-y-placa-en-cali-restricciones-vehiculares-para-evitar-multas-este-martes-2-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/02/clima-en-cartagena-de-indias-la-prediccion-para-este-2-de-junio/</t>
         </is>
       </c>
     </row>
@@ -3848,12 +3844,12 @@
       </c>
       <c r="D126" s="3" t="inlineStr">
         <is>
-          <t>En qué barrios de Bogotá habrá cortes de agua este martes</t>
+          <t>¿Cómo estará el clima en Barranquilla?</t>
         </is>
       </c>
       <c r="E126" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/02/en-que-barrios-de-bogota-habra-cortes-de-agua-este-martes/</t>
+          <t>https://www.infobae.com/colombia/2026/06/02/como-estara-el-clima-en-barranquilla/</t>
         </is>
       </c>
     </row>
@@ -3875,12 +3871,12 @@
       </c>
       <c r="D127" s="6" t="inlineStr">
         <is>
-          <t>Cinco menores heridos y 200 familias confinadas por combates entre Ejército y disidencias Farc en Cauca</t>
+          <t>Clima en Colombia: la predicción del tiempo para Medellín este 2 de junio</t>
         </is>
       </c>
       <c r="E127" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/02/cinco-menores-heridos-y-200-familias-confinadas-por-combates-entre-ejercito-y-disidencias-farc-en-cauca/</t>
+          <t>https://www.infobae.com/colombia/2026/06/02/clima-en-colombia-la-prediccion-del-tiempo-para-medellin-este-2-de-junio/</t>
         </is>
       </c>
     </row>
@@ -3902,12 +3898,12 @@
       </c>
       <c r="D128" s="3" t="inlineStr">
         <is>
-          <t>Pico y Placa: qué autos no circulan en Medellín este martes 2 de junio</t>
+          <t>Directora de la MOE advierte que Petro solo podría liderar la campaña de Iván Cepeda si renuncia a la presidencia</t>
         </is>
       </c>
       <c r="E128" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/02/pico-y-placa-que-autos-no-circulan-en-medellin-este-martes-2-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/02/directora-de-la-moe-advierte-que-petro-solo-podria-liderar-la-campana-de-ivan-cepeda-si-renuncia-a-la-presidencia/</t>
         </is>
       </c>
     </row>
@@ -3929,12 +3925,12 @@
       </c>
       <c r="D129" s="6" t="inlineStr">
         <is>
-          <t>Buenas noticias para quienes viajan a Neiva por carretera: Ministerio de Transporte ajustará las tarifas del peaje Villalobos</t>
+          <t>Resultado Baloto y Revancha hoy lunes 1 de junio</t>
         </is>
       </c>
       <c r="E129" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/02/buenas-noticias-para-quienes-viajan-a-neiva-por-carretera-ministerio-de-transporte-ajustara-las-tarifas-del-peaje-villalobos/</t>
+          <t>https://www.infobae.com/colombia/2026/06/02/resultado-baloto-y-revancha-hoy-lunes-1-de-junio/</t>
         </is>
       </c>
     </row>
@@ -3956,12 +3952,12 @@
       </c>
       <c r="D130" s="3" t="inlineStr">
         <is>
-          <t>¿Messi y James juntos? Así se vería el 10 argentino jugando con Colombia según la inteligencia artificial</t>
+          <t>TransMilenio cambió el nombre de la estación Calle 26 en Bogotá: así se llamará desde ahora</t>
         </is>
       </c>
       <c r="E130" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/tecno/2026/06/02/messi-y-james-juntos-asi-se-veria-el-10-argentino-jugando-con-colombia-segun-la-inteligencia-artificial/</t>
+          <t>https://www.infobae.com/colombia/2026/06/02/transmilenio-cambio-el-nombre-de-la-estacion-calle-26-en-bogota-asi-se-llamara-desde-ahora/</t>
         </is>
       </c>
     </row>
@@ -3983,12 +3979,12 @@
       </c>
       <c r="D131" s="6" t="inlineStr">
         <is>
-          <t>“¡Cepeda, jódete!”: desde el estadio El Campín, Vicky Dávila defendió el uso de la camiseta de la selección Colombia en la política</t>
+          <t>Hallan muerto a un menor de 13 años en un potrero de Valle del Cauca: investigan quiénes están detrás del crimen</t>
         </is>
       </c>
       <c r="E131" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/02/cepeda-jodete-desde-el-estadio-el-campin-vicky-davila-defendio-el-uso-de-la-camiseta-de-la-seleccion-colombia-en-la-politica/</t>
+          <t>https://www.infobae.com/colombia/2026/06/02/hallan-muerto-a-un-menor-de-13-anos-en-un-potrero-de-valle-del-cauca-investigan-quienes-estan-detras-del-crimen/</t>
         </is>
       </c>
     </row>
@@ -4010,12 +4006,12 @@
       </c>
       <c r="D132" s="3" t="inlineStr">
         <is>
-          <t>Falcao García se sumó a un nuevo equipo durante el Mundial 2026: “Fichaje de lujo”</t>
+          <t>Resultado Lotería de Cundinamarca hoy lunes 1 de junio</t>
         </is>
       </c>
       <c r="E132" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/02/falcao-garcia-se-sumo-a-un-nuevo-equipo-durante-el-mundial-2026-fichaje-de-lujo/</t>
+          <t>https://www.infobae.com/colombia/2026/06/02/resultado-loteria-de-cundinamarca-hoy-lunes-1-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4037,12 +4033,12 @@
       </c>
       <c r="D133" s="6" t="inlineStr">
         <is>
-          <t>Jugadores de la selección Colombia hablaron después de la victoria ante Costa Rica: “El sueño es ser campeones del Mundo”</t>
+          <t>Tras críticas a Abelardo, reviven video de la campaña de Iván Cepeda promoviendo el uso de la camiseta de la Selección</t>
         </is>
       </c>
       <c r="E133" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/06/02/jugadores-de-la-seleccion-colombia-hablaron-despues-de-la-victoria-ante-costa-rica-el-sueno-es-ser-campeones-del-mundo/</t>
+          <t>https://www.infobae.com/colombia/2026/06/02/tras-criticas-a-abelardo-reviven-video-de-la-campana-de-ivan-cepeda-promoviendo-el-uso-de-la-camiseta-de-la-seleccion/</t>
         </is>
       </c>
     </row>
@@ -4064,19 +4060,19 @@
       </c>
       <c r="D134" s="3" t="inlineStr">
         <is>
-          <t>Iván Duque aplaudió la decisión del Gobierno de Donald Trump de nominar a Nathaniel Morris como embajador de Estados Unidos en Colombia</t>
+          <t>Resultado Super Astro Luna HOY: número ganador del lunes 1 de junio</t>
         </is>
       </c>
       <c r="E134" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/02/ivan-duque-aplaudio-la-decision-del-gobierno-de-donald-trump-de-nominar-a-nathaniel-morris-como-embajador-de-estados-unidos-en-colombia/</t>
+          <t>https://www.infobae.com/colombia/2026/06/02/resultado-super-astro-luna-hoy-numero-ganador-del-lunes-1-de-junio/</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 07:00 p. m.</t>
+          <t>01/06/2026 11:55 p. m.</t>
         </is>
       </c>
       <c r="B135" s="5" t="inlineStr">
@@ -4086,24 +4082,24 @@
       </c>
       <c r="C135" s="5" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D135" s="6" t="inlineStr">
         <is>
-          <t>Duerma informado con las claves de este 1 de junio de 2026</t>
+          <t>Resultados loterías de Cundinamarca, Tolima, Baloto, MiLoto y ColorLoto del 1 de junio de 2026</t>
         </is>
       </c>
       <c r="E135" s="7" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/duerma-informado-con-las-claves-de-este-1-de-junio-de-2026/</t>
+          <t>https://www.bluradio.com/economia/juegos-de-azar/resultados-loterias-de-cundinamarca-tolima-baloto-miloto-y-colorloto-del-1-de-junio-de-2026-so35</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 06:40 p. m.</t>
+          <t>01/06/2026 11:48 p. m.</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
@@ -4113,24 +4109,24 @@
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D136" s="3" t="inlineStr">
         <is>
-          <t>Cepeda no tuvo ventaja en municipios con “riesgo de control criminal”</t>
+          <t>¿Petro entra en la contienda electoral?: Recap - programa completo 1 de junio de 2026</t>
         </is>
       </c>
       <c r="E136" s="4" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/cepeda-no-tuvo-ventaja-en-municipios-con-riesgo-de-control-criminal/</t>
+          <t>https://www.bluradio.com/recap/petro-entra-en-la-contienda-electoral-recap-programa-completo-1-de-junio-de-2026-pr30</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 05:49 p. m.</t>
+          <t>01/06/2026 11:43 p. m.</t>
         </is>
       </c>
       <c r="B137" s="5" t="inlineStr">
@@ -4140,24 +4136,24 @@
       </c>
       <c r="C137" s="5" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D137" s="6" t="inlineStr">
         <is>
-          <t>Campaña de Cepeda ya busca cafés con el centro para segunda vuelta</t>
+          <t>ColorLoto, resultado del lunes 1 de junio de 2026</t>
         </is>
       </c>
       <c r="E137" s="7" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/campana-de-cepeda-ya-busca-cafes-con-el-centro-para-segunda-vuelta/</t>
+          <t>https://www.bluradio.com/economia/juegos-de-azar/colorloto-resultado-del-lunes-1-de-junio-de-2026-so35</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 05:25 p. m.</t>
+          <t>01/06/2026 11:16 p. m.</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
@@ -4167,24 +4163,24 @@
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D138" s="3" t="inlineStr">
         <is>
-          <t>Tras victoria de Abelardo, bajaron tasas de deuda y precio del dólar</t>
+          <t>Taylor Swift pone voz a una nueva canción para la banda sonora de 'Toy Story 5'</t>
         </is>
       </c>
       <c r="E138" s="4" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/tras-victoria-de-abelardo-bajaron-tasas-de-deuda-y-precio-del-dolar/</t>
+          <t>https://www.bluradio.com/entretenimiento/taylor-swift-pone-voz-a-una-nueva-cancion-para-la-banda-sonora-de-toy-story-5-cb20</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 05:21 p. m.</t>
+          <t>01/06/2026 11:13 p. m.</t>
         </is>
       </c>
       <c r="B139" s="5" t="inlineStr">
@@ -4194,24 +4190,24 @@
       </c>
       <c r="C139" s="5" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D139" s="6" t="inlineStr">
         <is>
-          <t>La Silla Vacía invita a los dos candidatos a Micrófono Abierto</t>
+          <t>La importancia de la formación de nuevas figuras de la música latina</t>
         </is>
       </c>
       <c r="E139" s="7" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/la-silla-vacia-invita-a-los-dos-candidatos-a-microfono-abierto/</t>
+          <t>https://www.bluradio.com/sociedad/la-importancia-de-la-formacion-de-nuevas-figuras-de-la-musica-latina-rs15</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 04:42 p. m.</t>
+          <t>01/06/2026 10:56 p. m.</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
@@ -4221,24 +4217,24 @@
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D140" s="3" t="inlineStr">
         <is>
-          <t>Petro convoca a reunión de ministros tras resultados de primera vuelta</t>
+          <t>Kris R, Jay Wheeler y Ela Taubert lideran los estrenos musicales de la semana</t>
         </is>
       </c>
       <c r="E140" s="4" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/petro-convoca-a-reunion-de-ministros-tras-resultados-de-primera-vuelta/</t>
+          <t>https://www.bluradio.com/entretenimiento/kris-r-jay-wheeler-y-ela-taubert-lideran-los-estrenos-musicales-de-la-semana-rs15</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 04:09 p. m.</t>
+          <t>01/06/2026 10:46 p. m.</t>
         </is>
       </c>
       <c r="B141" s="5" t="inlineStr">
@@ -4248,24 +4244,24 @@
       </c>
       <c r="C141" s="5" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D141" s="6" t="inlineStr">
         <is>
-          <t>En la mesa donde votó Iván Cepeda ganó Abelardo</t>
+          <t>¿Qué significa ser pueblerina? El valioso significado que le da Adriana Lucía</t>
         </is>
       </c>
       <c r="E141" s="7" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/en-la-mesa-donde-voto-ivan-cepeda-gano-abelardo/</t>
+          <t>https://www.bluradio.com/entretenimiento/que-significa-ser-pueblerina-el-valioso-significado-que-le-da-adriana-lucia-rs15</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 04:00 p. m.</t>
+          <t>01/06/2026 10:26 p. m.</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
@@ -4275,24 +4271,24 @@
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D142" s="3" t="inlineStr">
         <is>
-          <t>Cepeda y el Pacto se hacen zancadilla con la camiseta de la Selección Colombia</t>
+          <t>"El debate tiene que darse con altura": presidente del CNE previo a segunda vuelta de elecciones</t>
         </is>
       </c>
       <c r="E142" s="4" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/cepeda-y-el-pacto-se-hacen-zancadilla-con-la-camiseta-de-la-seleccion-colombia/</t>
+          <t>https://www.bluradio.com/nacion/elecciones/congreso/el-debate-tiene-que-darse-con-altura-presidente-del-cne-previa-a-segunda-vuelta-de-elecciones-pr30</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 03:15 p. m.</t>
+          <t>01/06/2026 10:18 p. m.</t>
         </is>
       </c>
       <c r="B143" s="5" t="inlineStr">
@@ -4302,24 +4298,24 @@
       </c>
       <c r="C143" s="5" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D143" s="6" t="inlineStr">
         <is>
-          <t>Saade pide a Petro y Benedetti que renuncien para hacer campaña</t>
+          <t>Cerrejón avanza en la reanudación de sus operaciones mineras</t>
         </is>
       </c>
       <c r="E143" s="7" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/saade-pide-a-petro-y-benedetti-que-renuncien-para-hacer-campana/</t>
+          <t>https://www.bluradio.com/regiones/caribe/cerrejon-avanza-en-la-reanudacion-de-sus-operaciones-mineras-so35</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 01:40 p. m.</t>
+          <t>01/06/2026 09:52 p. m.</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
@@ -4329,24 +4325,24 @@
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D144" s="3" t="inlineStr">
         <is>
-          <t>Calculadora de La Silla: qué necesita cada candidato para ganar en segunda</t>
+          <t>Baloto y Revancha, resultado del último sorteo hoy lunes 1 de junio de 2026</t>
         </is>
       </c>
       <c r="E144" s="4" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/calculadora-de-la-silla-que-necesita-cada-candidato-para-ganar-en-segunda/</t>
+          <t>https://www.bluradio.com/economia/juegos-de-azar/baloto-y-revancha-resultado-del-ultimo-sorteo-hoy-lunes-1-de-junio-de-2026-so35</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 01:37 p. m.</t>
+          <t>01/06/2026 09:51 p. m.</t>
         </is>
       </c>
       <c r="B145" s="5" t="inlineStr">
@@ -4356,24 +4352,24 @@
       </c>
       <c r="C145" s="5" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D145" s="6" t="inlineStr">
         <is>
-          <t>Petro se va contra Abelardo y asegura: “vamos a ganar”</t>
+          <t>Lotería del Tolima, resultados del último sorteo hoy lunes 1 de junio de 2026</t>
         </is>
       </c>
       <c r="E145" s="7" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/petro-se-va-contra-abelardo-y-asegura-vamos-a-ganar/</t>
+          <t>https://www.bluradio.com/economia/juegos-de-azar/loteria-del-tolima-resultados-del-ultimo-sorteo-hoy-lunes-1-de-junio-de-2026-so35</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 01:21 p. m.</t>
+          <t>01/06/2026 09:51 p. m.</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
@@ -4383,24 +4379,24 @@
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D146" s="3" t="inlineStr">
         <is>
-          <t>Diario de Campaña: denuncias de fraude y la camiseta de la Selección</t>
+          <t>MiLoto, resultado del último sorteo hoy lunes 1 de junio de 2026</t>
         </is>
       </c>
       <c r="E146" s="4" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/diario-de-campana-denuncias-de-fraude-y-la-camiseta-de-la-seleccion/</t>
+          <t>https://www.bluradio.com/economia/juegos-de-azar/miloto-resultado-del-ultimo-sorteo-hoy-lunes-1-de-junio-de-2026-so35</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 12:55 p. m.</t>
+          <t>01/06/2026 04:30 p. m.</t>
         </is>
       </c>
       <c r="B147" s="5" t="inlineStr">
@@ -4410,24 +4406,24 @@
       </c>
       <c r="C147" s="5" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D147" s="6" t="inlineStr">
         <is>
-          <t>Sheinbaum: “hay que tener respeto por la decisión de Colombia”</t>
+          <t>La FCF responde a Cepeda: no puede impedir uso electoral de la camiseta de la selección, pero piden evitarlo</t>
         </is>
       </c>
       <c r="E147" s="7" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/sheinbaum-hay-que-tener-respeto-por-la-decision-de-colombia/</t>
+          <t>https://cambiocolombia.com/pais/articulo/2026/6/la-fcf-responde-a-cepeda-no-puede-impedir-uso-electoral-de-la-camiseta-de-la-seleccion-pero-piden-evitarlo</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 12:06 p. m.</t>
+          <t>01/06/2026 03:30 p. m.</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
@@ -4437,24 +4433,24 @@
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D148" s="3" t="inlineStr">
         <is>
-          <t>Cepeda ganó en el Caribe y Abelardo se le acerca</t>
+          <t>Ministerioo de Salud elimina Mipres para medicamentos UPC: ¿qué cambió?</t>
         </is>
       </c>
       <c r="E148" s="4" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/cepeda-no-igualo-los-votos-de-petro-en-el-caribe-y-abelardo-le-compite/</t>
+          <t>https://cambiocolombia.com/salud-y-bienestar/articulo/2026/6/ministerioo-de-salud-elimina-mipres-para-medicamentos-upc-que-cambio</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 11:38 a. m.</t>
+          <t>01/06/2026 02:46 p. m.</t>
         </is>
       </c>
       <c r="B149" s="5" t="inlineStr">
@@ -4464,24 +4460,24 @@
       </c>
       <c r="C149" s="5" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D149" s="6" t="inlineStr">
         <is>
-          <t>Partidos inician operación aterrizaje hacia Abelardo</t>
+          <t>Las sanciones que enfrentaría el operador de la lancha donde murió Alexander Avendaño en Guatapé</t>
         </is>
       </c>
       <c r="E149" s="7" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/partidos-inician-operacion-aterrizaje-hacia-abelardo/</t>
+          <t>https://cambiocolombia.com/pais/articulo/2026/6/las-sanciones-que-enfrentaria-el-operador-de-la-lancha-donde-murio-alexander-avendano-en-guatape</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 11:21 a. m.</t>
+          <t>01/06/2026 02:00 p. m.</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
@@ -4491,24 +4487,24 @@
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D150" s="3" t="inlineStr">
         <is>
-          <t>Cepeda dice que no han encontrado evidencias de fraude electoral</t>
+          <t>Cuatro personas murieron en un accidente de avioneta en la ruta Villavicencio – La Macarena</t>
         </is>
       </c>
       <c r="E150" s="4" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/cepeda-dice-que-no-han-encontrado-evidencias-de-fraude-electoral/</t>
+          <t>https://cambiocolombia.com/pais/articulo/2026/6/cuatro-personas-murieron-en-un-accidente-de-avioneta-en-la-ruta-villavicencio-la-macarena</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 10:26 a. m.</t>
+          <t>01/06/2026 01:00 p. m.</t>
         </is>
       </c>
       <c r="B151" s="5" t="inlineStr">
@@ -4518,24 +4514,24 @@
       </c>
       <c r="C151" s="5" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D151" s="6" t="inlineStr">
         <is>
-          <t>Cepeda se queja porque Abelardo usa la camiseta de la Selección Colombia</t>
+          <t>ONU, OEA y Human Rights Watch respaldan a la Registraduría tras críticas de Petro</t>
         </is>
       </c>
       <c r="E151" s="7" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/cepeda-se-queja-porque-abelardo-usa-la-camiseta-de-la-seleccion-colombia/</t>
+          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/onu-oea-y-human-rights-watch-respaldan-a-la-registraduria-tras-criticas-de-petro</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 10:02 a. m.</t>
+          <t>01/06/2026 11:50 a. m.</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
@@ -4545,24 +4541,24 @@
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D152" s="3" t="inlineStr">
         <is>
-          <t>Ordenada, transparente y sin incidentes: el balance de la Unión Europea</t>
+          <t>Iván Cepeda sobre presunto fraude en primera vuelta: “no hemos encontrado irregularidades protuberantes”</t>
         </is>
       </c>
       <c r="E152" s="4" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/ordenada-transparente-y-sin-incidentes-el-balance-de-la-union-europea/</t>
+          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/ivan-cepeda-sobre-presunto-fraude-en-primera-vuelta-no-hemos-encontrado-irregularidades-protuberantes</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 08:33 a. m.</t>
+          <t>01/06/2026 10:30 a. m.</t>
         </is>
       </c>
       <c r="B153" s="5" t="inlineStr">
@@ -4572,24 +4568,24 @@
       </c>
       <c r="C153" s="5" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D153" s="6" t="inlineStr">
         <is>
-          <t>Cepeda retó a debate a Abelardo, quien lo condiciona a que acepte resultados</t>
+          <t>Ecuador elimina aranceles de 100 por ciento a productos colombianos</t>
         </is>
       </c>
       <c r="E153" s="7" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/cepeda-reto-a-debate-a-abelardo-quien-lo-condiciona-a-que-acepte-resultados/</t>
+          <t>https://cambiocolombia.com/economia/articulo/2026/6/ecuador-elimina-aranceles-de-100-por-ciento-a-productos-colombianos</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 07:40 a. m.</t>
+          <t>01/06/2026 10:15 a. m.</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
@@ -4599,24 +4595,24 @@
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D154" s="3" t="inlineStr">
         <is>
-          <t>Desayune informado con las movidas de este 1 de junio de 2026</t>
+          <t>Bogotá registró dos muertos durante la jornada electoral</t>
         </is>
       </c>
       <c r="E154" s="4" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/desayune-informado-con-las-movidas-de-este-1-de-junio-de-2026/</t>
+          <t>https://cambiocolombia.com/pais/articulo/2026/6/bogota-registro-dos-muertos-durante-la-jornada-electoral</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 04:30 p. m.</t>
+          <t>01/06/2026 09:28 a. m.</t>
         </is>
       </c>
       <c r="B155" s="5" t="inlineStr">
@@ -4631,19 +4627,19 @@
       </c>
       <c r="D155" s="6" t="inlineStr">
         <is>
-          <t>La FCF responde a Cepeda: no puede impedir uso electoral de la camiseta de la selección, pero piden evitarlo</t>
+          <t>Los motivos detrás de la impugnación de Petro al preconteo de las elecciones 2026</t>
         </is>
       </c>
       <c r="E155" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/pais/articulo/2026/6/la-fcf-responde-a-cepeda-no-puede-impedir-uso-electoral-de-la-camiseta-de-la-seleccion-pero-piden-evitarlo</t>
+          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/los-motivos-detras-de-la-impugnacion-de-petro-al-preconteo-de-las-elecciones-2026</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 03:30 p. m.</t>
+          <t>31/05/2026 09:45 p. m.</t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
@@ -4658,19 +4654,19 @@
       </c>
       <c r="D156" s="3" t="inlineStr">
         <is>
-          <t>Ministerioo de Salud elimina Mipres para medicamentos UPC: ¿qué cambió?</t>
+          <t>"Ganó la democracia": procurador Eljach celebró la jornada y le recordó a Petro la decisión del Consejo de Estado</t>
         </is>
       </c>
       <c r="E156" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/salud-y-bienestar/articulo/2026/6/ministerioo-de-salud-elimina-mipres-para-medicamentos-upc-que-cambio</t>
+          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/gano-la-democracia-procurador-eljach-celebro-la-jornada-y-le-recordo-a-petro-la-decision-del-consejo-de-estado</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 02:46 p. m.</t>
+          <t>31/05/2026 09:00 p. m.</t>
         </is>
       </c>
       <c r="B157" s="5" t="inlineStr">
@@ -4685,19 +4681,19 @@
       </c>
       <c r="D157" s="6" t="inlineStr">
         <is>
-          <t>Las sanciones que enfrentaría el operador de la lancha donde murió Alexander Avendaño en Guatapé</t>
+          <t>“Petro no es un demócrata”: políticos y figuras públicas reaccionan al rechazo del presidente a los resultados del preconteo</t>
         </is>
       </c>
       <c r="E157" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/pais/articulo/2026/6/las-sanciones-que-enfrentaria-el-operador-de-la-lancha-donde-murio-alexander-avendano-en-guatape</t>
+          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/petro-no-es-un-democrata-politicos-y-figuras-publicas-reaccionan-al-rechazo-del-presidente-a-los-resultados-del-preconteo</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 02:00 p. m.</t>
+          <t>31/05/2026 07:00 p. m.</t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
@@ -4712,19 +4708,19 @@
       </c>
       <c r="D158" s="3" t="inlineStr">
         <is>
-          <t>Cuatro personas murieron en un accidente de avioneta en la ruta Villavicencio – La Macarena</t>
+          <t>¿Cuándo se realizará la segunda vuelta presidencial entre Abelardo de la Espriella e Iván Cepeda?</t>
         </is>
       </c>
       <c r="E158" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/pais/articulo/2026/6/cuatro-personas-murieron-en-un-accidente-de-avioneta-en-la-ruta-villavicencio-la-macarena</t>
+          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/cuando-se-realizara-la-segunda-vuelta-presidencial-entre-abelardo-de-la-espriella-e-ivan-cepeda</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 01:00 p. m.</t>
+          <t>31/05/2026 01:45 p. m.</t>
         </is>
       </c>
       <c r="B159" s="5" t="inlineStr">
@@ -4739,19 +4735,19 @@
       </c>
       <c r="D159" s="6" t="inlineStr">
         <is>
-          <t>ONU, OEA y Human Rights Watch respaldan a la Registraduría tras críticas de Petro</t>
+          <t>¿Mostrar el voto fue participación indebida en política? Expertos analizan actuación de Petro y Benedetti</t>
         </is>
       </c>
       <c r="E159" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/onu-oea-y-human-rights-watch-respaldan-a-la-registraduria-tras-criticas-de-petro</t>
+          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/5/mostrar-el-voto-fue-participacion-indebida-en-politica-expertos-analizan-actuacion-de-petro-y-benedetti</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 11:50 a. m.</t>
+          <t>31/05/2026 12:00 p. m.</t>
         </is>
       </c>
       <c r="B160" s="2" t="inlineStr">
@@ -4766,19 +4762,19 @@
       </c>
       <c r="D160" s="3" t="inlineStr">
         <is>
-          <t>Iván Cepeda sobre presunto fraude en primera vuelta: “no hemos encontrado irregularidades protuberantes”</t>
+          <t>Golpe al Clan del Golfo: Fuerzas Militares bombardean campamento en límites de Chocó y Valle del Cauca</t>
         </is>
       </c>
       <c r="E160" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/ivan-cepeda-sobre-presunto-fraude-en-primera-vuelta-no-hemos-encontrado-irregularidades-protuberantes</t>
+          <t>https://cambiocolombia.com/conflicto-armado-en-colombia/articulo/2026/5/golpe-al-clan-del-golfo-fuerzas-militares-bombardean-campamento-en-limites-de-choco-y-valle-del-cauca</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 10:30 a. m.</t>
+          <t>31/05/2026 09:15 a. m.</t>
         </is>
       </c>
       <c r="B161" s="5" t="inlineStr">
@@ -4793,19 +4789,19 @@
       </c>
       <c r="D161" s="6" t="inlineStr">
         <is>
-          <t>Ecuador elimina aranceles de 100 por ciento a productos colombianos</t>
+          <t>Alcalde Galán insta a la paz y al respeto por los resultados en jornada electoral en Bogotá</t>
         </is>
       </c>
       <c r="E161" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/economia/articulo/2026/6/ecuador-elimina-aranceles-de-100-por-ciento-a-productos-colombianos</t>
+          <t>https://cambiocolombia.com/poder/articulo/2026/5/alcalde-galan-insta-a-la-paz-y-al-respeto-por-los-resultados-en-jornada-electoral-en-bogota</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 10:15 a. m.</t>
+          <t>31/05/2026 06:28 p. m.</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
@@ -4815,24 +4811,24 @@
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D162" s="3" t="inlineStr">
         <is>
-          <t>Bogotá registró dos muertos durante la jornada electoral</t>
+          <t>Paloma Valencia anuncia su unión a Abelardo de la Espriella: “Seguiré en la batalla para derrotar a Iván Cepeda»</t>
         </is>
       </c>
       <c r="E162" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/pais/articulo/2026/6/bogota-registro-dos-muertos-durante-la-jornada-electoral</t>
+          <t>https://canaltrece.com.co/noticias/paloma-valencia-anuncia-su-union-a-abelardo-de-la-espriella-seguire-en-la-batalla-para-derrotar-a-ivan-cepeda/</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 09:28 a. m.</t>
+          <t>31/05/2026 06:22 p. m.</t>
         </is>
       </c>
       <c r="B163" s="5" t="inlineStr">
@@ -4842,24 +4838,24 @@
       </c>
       <c r="C163" s="5" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D163" s="6" t="inlineStr">
         <is>
-          <t>Los motivos detrás de la impugnación de Petro al preconteo de las elecciones 2026</t>
+          <t>El factor Fajardo: Más de un millón de ciudadanos eligen el centro y definen las llaves del balotaje</t>
         </is>
       </c>
       <c r="E163" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/los-motivos-detras-de-la-impugnacion-de-petro-al-preconteo-de-las-elecciones-2026</t>
+          <t>https://canaltrece.com.co/noticias/el-factor-fajardo-mas-de-un-millon-de-ciudadanos-eligen-el-centro-y-definen-las-llaves-del-balotaje/</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>31/05/2026 09:45 p. m.</t>
+          <t>31/05/2026 06:16 p. m.</t>
         </is>
       </c>
       <c r="B164" s="2" t="inlineStr">
@@ -4869,24 +4865,24 @@
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D164" s="3" t="inlineStr">
         <is>
-          <t>"Ganó la democracia": procurador Eljach celebró la jornada y le recordó a Petro la decisión del Consejo de Estado</t>
+          <t>¿Qué regiones votaron por cada candidato?</t>
         </is>
       </c>
       <c r="E164" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/gano-la-democracia-procurador-eljach-celebro-la-jornada-y-le-recordo-a-petro-la-decision-del-consejo-de-estado</t>
+          <t>https://canaltrece.com.co/noticias/que-regiones-votaron-por-cada-candidato/</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="5" t="inlineStr">
         <is>
-          <t>31/05/2026 09:00 p. m.</t>
+          <t>31/05/2026 06:07 p. m.</t>
         </is>
       </c>
       <c r="B165" s="5" t="inlineStr">
@@ -4896,24 +4892,24 @@
       </c>
       <c r="C165" s="5" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D165" s="6" t="inlineStr">
         <is>
-          <t>“Petro no es un demócrata”: políticos y figuras públicas reaccionan al rechazo del presidente a los resultados del preconteo</t>
+          <t>Fiesta en el Malecón del Río: Abelardo de la Espriella celebra el triunfo en primera vuelta y redefine a la derecha</t>
         </is>
       </c>
       <c r="E165" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/petro-no-es-un-democrata-politicos-y-figuras-publicas-reaccionan-al-rechazo-del-presidente-a-los-resultados-del-preconteo</t>
+          <t>https://canaltrece.com.co/noticias/fiesta-en-el-malecon-del-rio-abelardo-de-la-espriella-celebra-el-triunfo-en-primera-vuelta-y-redefine-a-la-derecha/</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>31/05/2026 07:00 p. m.</t>
+          <t>31/05/2026 05:59 p. m.</t>
         </is>
       </c>
       <c r="B166" s="2" t="inlineStr">
@@ -4923,24 +4919,24 @@
       </c>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D166" s="3" t="inlineStr">
         <is>
-          <t>¿Cuándo se realizará la segunda vuelta presidencial entre Abelardo de la Espriella e Iván Cepeda?</t>
+          <t>El ajedrez de la segunda vuelta: Las alianzas clave que definirán el futuro de De la Espriella y Cepeda</t>
         </is>
       </c>
       <c r="E166" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/cuando-se-realizara-la-segunda-vuelta-presidencial-entre-abelardo-de-la-espriella-e-ivan-cepeda</t>
+          <t>https://canaltrece.com.co/noticias/el-ajedrez-de-la-segunda-vuelta-las-alianzas-clave-que-definiran-el-futuro-de-de-la-espriella-y-cepeda/</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="5" t="inlineStr">
         <is>
-          <t>31/05/2026 01:45 p. m.</t>
+          <t>31/05/2026 05:51 p. m.</t>
         </is>
       </c>
       <c r="B167" s="5" t="inlineStr">
@@ -4950,24 +4946,24 @@
       </c>
       <c r="C167" s="5" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D167" s="6" t="inlineStr">
         <is>
-          <t>¿Mostrar el voto fue participación indebida en política? Expertos analizan actuación de Petro y Benedetti</t>
+          <t>Tensión en el Hotel Tequendama: Campaña de Iván Cepeda suspende transmisión en vivo ante resultados adversos</t>
         </is>
       </c>
       <c r="E167" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/5/mostrar-el-voto-fue-participacion-indebida-en-politica-expertos-analizan-actuacion-de-petro-y-benedetti</t>
+          <t>https://canaltrece.com.co/noticias/tension-en-el-hotel-tequendama-campana-de-ivan-cepeda-suspende-transmision-en-vivo-ante-resultados-adversos/</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>31/05/2026 12:00 p. m.</t>
+          <t>31/05/2026 05:19 p. m.</t>
         </is>
       </c>
       <c r="B168" s="2" t="inlineStr">
@@ -4977,24 +4973,24 @@
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D168" s="3" t="inlineStr">
         <is>
-          <t>Golpe al Clan del Golfo: Fuerzas Militares bombardean campamento en límites de Chocó y Valle del Cauca</t>
+          <t>De la Espriella Y Cepeda pasan a segunda vuelta presidencial en Colombia</t>
         </is>
       </c>
       <c r="E168" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/conflicto-armado-en-colombia/articulo/2026/5/golpe-al-clan-del-golfo-fuerzas-militares-bombardean-campamento-en-limites-de-choco-y-valle-del-cauca</t>
+          <t>https://canaltrece.com.co/noticias/de-la-espriella-y-cepeda-pasan-a-segunda-vuelta-presidencial-en-colombia/</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="5" t="inlineStr">
         <is>
-          <t>31/05/2026 09:15 a. m.</t>
+          <t>31/05/2026 04:28 p. m.</t>
         </is>
       </c>
       <c r="B169" s="5" t="inlineStr">
@@ -5004,24 +5000,24 @@
       </c>
       <c r="C169" s="5" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D169" s="6" t="inlineStr">
         <is>
-          <t>Alcalde Galán insta a la paz y al respeto por los resultados en jornada electoral en Bogotá</t>
+          <t>Primeros boletines de la Registraduría: Iván Cepeda y Abelardo de la Espriella lideran los resultados presidenciales</t>
         </is>
       </c>
       <c r="E169" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/poder/articulo/2026/5/alcalde-galan-insta-a-la-paz-y-al-respeto-por-los-resultados-en-jornada-electoral-en-bogota</t>
+          <t>https://canaltrece.com.co/noticias/primeros-boletines-de-la-registraduria-ivan-cepeda-y-abelardo-de-la-espriella-lideran-los-resultados-presidenciales/</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>31/05/2026 06:28 p. m.</t>
+          <t>31/05/2026 04:17 p. m.</t>
         </is>
       </c>
       <c r="B170" s="2" t="inlineStr">
@@ -5036,19 +5032,19 @@
       </c>
       <c r="D170" s="3" t="inlineStr">
         <is>
-          <t>Paloma Valencia anuncia su unión a Abelardo de la Espriella: “Seguiré en la batalla para derrotar a Iván Cepeda»</t>
+          <t>Balance de la Registraduría a las 4:00 p.m.: Así avanza el preconteo y la digitalización de los formularios E-14</t>
         </is>
       </c>
       <c r="E170" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/paloma-valencia-anuncia-su-union-a-abelardo-de-la-espriella-seguire-en-la-batalla-para-derrotar-a-ivan-cepeda/</t>
+          <t>https://canaltrece.com.co/noticias/balance-de-la-registraduria-a-las-400-p-m-asi-avanza-el-preconteo-y-la-digitalizacion-de-los-formularios-e-14/</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="5" t="inlineStr">
         <is>
-          <t>31/05/2026 06:22 p. m.</t>
+          <t>31/05/2026 03:55 p. m.</t>
         </is>
       </c>
       <c r="B171" s="5" t="inlineStr">
@@ -5063,19 +5059,19 @@
       </c>
       <c r="D171" s="6" t="inlineStr">
         <is>
-          <t>El factor Fajardo: Más de un millón de ciudadanos eligen el centro y definen las llaves del balotaje</t>
+          <t>Elecciones 2026 en vivo: resultados y minuto a minuto del preconteo</t>
         </is>
       </c>
       <c r="E171" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/el-factor-fajardo-mas-de-un-millon-de-ciudadanos-eligen-el-centro-y-definen-las-llaves-del-balotaje/</t>
+          <t>https://canaltrece.com.co/noticias/elecciones-2026-en-vivo-resultados-y-minuto-a-minuto-del-preconteo/</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>31/05/2026 06:16 p. m.</t>
+          <t>31/05/2026 02:40 p. m.</t>
         </is>
       </c>
       <c r="B172" s="2" t="inlineStr">
@@ -5090,19 +5086,19 @@
       </c>
       <c r="D172" s="3" t="inlineStr">
         <is>
-          <t>¿Qué regiones votaron por cada candidato?</t>
+          <t>El fenómeno ‘Polymarket’: Se disparan las apuestas que dan a Abelardo de la Espriella como favorito a la Presidencia</t>
         </is>
       </c>
       <c r="E172" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/que-regiones-votaron-por-cada-candidato/</t>
+          <t>https://canaltrece.com.co/noticias/el-fenomeno-polymarket-se-disparan-las-apuestas-que-dan-a-abelardo-de-la-espriella-como-favorito-a-la-presidencia/</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="5" t="inlineStr">
         <is>
-          <t>31/05/2026 06:07 p. m.</t>
+          <t>31/05/2026 01:56 p. m.</t>
         </is>
       </c>
       <c r="B173" s="5" t="inlineStr">
@@ -5117,19 +5113,19 @@
       </c>
       <c r="D173" s="6" t="inlineStr">
         <is>
-          <t>Fiesta en el Malecón del Río: Abelardo de la Espriella celebra el triunfo en primera vuelta y redefine a la derecha</t>
+          <t>Formulario E-14: cómo consultar las actas de las elecciones 2026</t>
         </is>
       </c>
       <c r="E173" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/fiesta-en-el-malecon-del-rio-abelardo-de-la-espriella-celebra-el-triunfo-en-primera-vuelta-y-redefine-a-la-derecha/</t>
+          <t>https://canaltrece.com.co/noticias/formulario-e-14-como-consultar-las-actas-de-las-elecciones-2026/</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>31/05/2026 05:59 p. m.</t>
+          <t>31/05/2026 01:48 p. m.</t>
         </is>
       </c>
       <c r="B174" s="2" t="inlineStr">
@@ -5144,19 +5140,19 @@
       </c>
       <c r="D174" s="3" t="inlineStr">
         <is>
-          <t>El ajedrez de la segunda vuelta: Las alianzas clave que definirán el futuro de De la Espriella y Cepeda</t>
+          <t>¿Cuándo se posesiona el próximo presidente de Colombia en 2026?</t>
         </is>
       </c>
       <c r="E174" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/el-ajedrez-de-la-segunda-vuelta-las-alianzas-clave-que-definiran-el-futuro-de-de-la-espriella-y-cepeda/</t>
+          <t>https://canaltrece.com.co/noticias/cuando-se-posesiona-el-proximo-presidente-de-colombia-en-2026/</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="5" t="inlineStr">
         <is>
-          <t>31/05/2026 05:51 p. m.</t>
+          <t>31/05/2026 01:41 p. m.</t>
         </is>
       </c>
       <c r="B175" s="5" t="inlineStr">
@@ -5171,19 +5167,19 @@
       </c>
       <c r="D175" s="6" t="inlineStr">
         <is>
-          <t>Tensión en el Hotel Tequendama: Campaña de Iván Cepeda suspende transmisión en vivo ante resultados adversos</t>
+          <t>Voto en blanco en Colombia: ¿qué pasa si gana en presidenciales?</t>
         </is>
       </c>
       <c r="E175" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/tension-en-el-hotel-tequendama-campana-de-ivan-cepeda-suspende-transmision-en-vivo-ante-resultados-adversos/</t>
+          <t>https://canaltrece.com.co/noticias/voto-en-blanco-en-colombia-que-pasa-si-gana-en-presidenciales/</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>31/05/2026 05:19 p. m.</t>
+          <t>31/05/2026 01:35 p. m.</t>
         </is>
       </c>
       <c r="B176" s="2" t="inlineStr">
@@ -5198,19 +5194,19 @@
       </c>
       <c r="D176" s="3" t="inlineStr">
         <is>
-          <t>De la Espriella Y Cepeda pasan a segunda vuelta presidencial en Colombia</t>
+          <t>Certificado electoral 2026: beneficios y cómo pedir copia si lo pierde</t>
         </is>
       </c>
       <c r="E176" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/de-la-espriella-y-cepeda-pasan-a-segunda-vuelta-presidencial-en-colombia/</t>
+          <t>https://canaltrece.com.co/noticias/certificado-electoral-2026-beneficios-y-como-pedir-copia-si-lo-pierde/</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="5" t="inlineStr">
         <is>
-          <t>31/05/2026 04:28 p. m.</t>
+          <t>31/05/2026 11:49 a. m.</t>
         </is>
       </c>
       <c r="B177" s="5" t="inlineStr">
@@ -5225,19 +5221,19 @@
       </c>
       <c r="D177" s="6" t="inlineStr">
         <is>
-          <t>Primeros boletines de la Registraduría: Iván Cepeda y Abelardo de la Espriella lideran los resultados presidenciales</t>
+          <t>Delitos electorales 2026: cómo denunciar compra de votos o presiones</t>
         </is>
       </c>
       <c r="E177" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/primeros-boletines-de-la-registraduria-ivan-cepeda-y-abelardo-de-la-espriella-lideran-los-resultados-presidenciales/</t>
+          <t>https://canaltrece.com.co/noticias/delitos-electorales-2026-como-denunciar-compra-de-votos-o-presiones/</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>31/05/2026 04:17 p. m.</t>
+          <t>31/05/2026 11:44 a. m.</t>
         </is>
       </c>
       <c r="B178" s="2" t="inlineStr">
@@ -5252,21 +5248,17 @@
       </c>
       <c r="D178" s="3" t="inlineStr">
         <is>
-          <t>Balance de la Registraduría a las 4:00 p.m.: Así avanza el preconteo y la digitalización de los formularios E-14</t>
+          <t>Elecciones 2026: ¿qué hacer si no aparece en el puesto de votación?</t>
         </is>
       </c>
       <c r="E178" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/balance-de-la-registraduria-a-las-400-p-m-asi-avanza-el-preconteo-y-la-digitalizacion-de-los-formularios-e-14/</t>
+          <t>https://canaltrece.com.co/editorial/elecciones-2026-que-hacer-si-no-aparece-en-el-puesto-de-votacion/</t>
         </is>
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="5" t="inlineStr">
-        <is>
-          <t>31/05/2026 03:55 p. m.</t>
-        </is>
-      </c>
+      <c r="A179" s="5" t="inlineStr"/>
       <c r="B179" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5279,21 +5271,17 @@
       </c>
       <c r="D179" s="6" t="inlineStr">
         <is>
-          <t>Elecciones 2026 en vivo: resultados y minuto a minuto del preconteo</t>
+          <t>Bogotá estrena el Teatro Nancy Kotal de Cortés: Un nuevo templo para el arte, el bilingüismo y la cultura</t>
         </is>
       </c>
       <c r="E179" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/elecciones-2026-en-vivo-resultados-y-minuto-a-minuto-del-preconteo/</t>
+          <t>https://canaltrece.com.co/noticias/bogota-estrena-el-teatro-nancy-kotal-de-cortes-un-nuevo-templo-para-el-arte-el-bilinguismo-y-la-cultura/</t>
         </is>
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="2" t="inlineStr">
-        <is>
-          <t>31/05/2026 02:40 p. m.</t>
-        </is>
-      </c>
+      <c r="A180" s="2" t="inlineStr"/>
       <c r="B180" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5306,21 +5294,17 @@
       </c>
       <c r="D180" s="3" t="inlineStr">
         <is>
-          <t>El fenómeno ‘Polymarket’: Se disparan las apuestas que dan a Abelardo de la Espriella como favorito a la Presidencia</t>
+          <t>Pantallas gigantes y alta tecnología: El Mundial de Fútbol dispara la venta de televisores en Colombia</t>
         </is>
       </c>
       <c r="E180" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/el-fenomeno-polymarket-se-disparan-las-apuestas-que-dan-a-abelardo-de-la-espriella-como-favorito-a-la-presidencia/</t>
+          <t>https://canaltrece.com.co/noticias/pantallas-gigantes-y-alta-tecnologia-el-mundial-de-futbol-dispara-la-venta-de-televisores-en-colombia/</t>
         </is>
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="5" t="inlineStr">
-        <is>
-          <t>31/05/2026 01:56 p. m.</t>
-        </is>
-      </c>
+      <c r="A181" s="5" t="inlineStr"/>
       <c r="B181" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5333,21 +5317,17 @@
       </c>
       <c r="D181" s="6" t="inlineStr">
         <is>
-          <t>Formulario E-14: cómo consultar las actas de las elecciones 2026</t>
+          <t>Nico González: El productor y director musical colombiano que revoluciona el pop latino desde Miami</t>
         </is>
       </c>
       <c r="E181" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/formulario-e-14-como-consultar-las-actas-de-las-elecciones-2026/</t>
+          <t>https://canaltrece.com.co/noticias/nico-gonzalez-el-productor-y-director-musical-colombiano-que-revoluciona-el-pop-latino-desde-miami/</t>
         </is>
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="2" t="inlineStr">
-        <is>
-          <t>31/05/2026 01:48 p. m.</t>
-        </is>
-      </c>
+      <c r="A182" s="2" t="inlineStr"/>
       <c r="B182" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5360,21 +5340,17 @@
       </c>
       <c r="D182" s="3" t="inlineStr">
         <is>
-          <t>¿Cuándo se posesiona el próximo presidente de Colombia en 2026?</t>
+          <t>Claptone regresa a Medellín con su experiencia ‘Claptone &amp; Friends’</t>
         </is>
       </c>
       <c r="E182" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/cuando-se-posesiona-el-proximo-presidente-de-colombia-en-2026/</t>
+          <t>https://canaltrece.com.co/noticias/claptone-regresa-a-medellin-con-su-experiencia-claptone-friends/</t>
         </is>
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="5" t="inlineStr">
-        <is>
-          <t>31/05/2026 01:41 p. m.</t>
-        </is>
-      </c>
+      <c r="A183" s="5" t="inlineStr"/>
       <c r="B183" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5387,21 +5363,17 @@
       </c>
       <c r="D183" s="6" t="inlineStr">
         <is>
-          <t>Voto en blanco en Colombia: ¿qué pasa si gana en presidenciales?</t>
+          <t>El restaurante Inquebrantable de Bogotá recibe el ‘Sello M’: Primer reconocimiento a la cocina mexicana auténtica en Colombia</t>
         </is>
       </c>
       <c r="E183" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/voto-en-blanco-en-colombia-que-pasa-si-gana-en-presidenciales/</t>
+          <t>https://canaltrece.com.co/noticias/el-restaurante-inquebrantable-de-bogota-recibe-el-sello-m-primer-reconocimiento-a-la-cocina-mexicana-autentica-en-colombia/</t>
         </is>
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="2" t="inlineStr">
-        <is>
-          <t>31/05/2026 01:35 p. m.</t>
-        </is>
-      </c>
+      <c r="A184" s="2" t="inlineStr"/>
       <c r="B184" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5414,21 +5386,17 @@
       </c>
       <c r="D184" s="3" t="inlineStr">
         <is>
-          <t>Certificado electoral 2026: beneficios y cómo pedir copia si lo pierde</t>
+          <t>Mau y Ricky estrenan ‘Ricky y Mau’: Su álbum más íntimo, libre y colaborativo hasta la fecha</t>
         </is>
       </c>
       <c r="E184" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/certificado-electoral-2026-beneficios-y-como-pedir-copia-si-lo-pierde/</t>
+          <t>https://canaltrece.com.co/noticias/mau-y-ricky-estrenan-ricky-y-mau-su-album-mas-intimo-libre-y-colaborativo-hasta-la-fecha/</t>
         </is>
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="5" t="inlineStr">
-        <is>
-          <t>31/05/2026 11:49 a. m.</t>
-        </is>
-      </c>
+      <c r="A185" s="5" t="inlineStr"/>
       <c r="B185" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5441,21 +5409,17 @@
       </c>
       <c r="D185" s="6" t="inlineStr">
         <is>
-          <t>Delitos electorales 2026: cómo denunciar compra de votos o presiones</t>
+          <t>Alejandro Saavedra estrena su EP ‘El Malo Soy Yo x Tener Corazón’: La nueva era del merenguetón y el pop urbano</t>
         </is>
       </c>
       <c r="E185" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/delitos-electorales-2026-como-denunciar-compra-de-votos-o-presiones/</t>
+          <t>https://canaltrece.com.co/noticias/alejandro-saavedra-estrena-su-ep-el-malo-soy-yo-x-tener-corazon-la-nueva-era-del-merengueton-y-el-pop-urbano/</t>
         </is>
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="2" t="inlineStr">
-        <is>
-          <t>31/05/2026 11:44 a. m.</t>
-        </is>
-      </c>
+      <c r="A186" s="2" t="inlineStr"/>
       <c r="B186" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5468,12 +5432,12 @@
       </c>
       <c r="D186" s="3" t="inlineStr">
         <is>
-          <t>Elecciones 2026: ¿qué hacer si no aparece en el puesto de votación?</t>
+          <t>Así son Ana Lucía Pineda y Pilar Rueda, las mujeres que aspiran a la Casa de Nariño</t>
         </is>
       </c>
       <c r="E186" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/editorial/elecciones-2026-que-hacer-si-no-aparece-en-el-puesto-de-votacion/</t>
+          <t>https://canaltrece.com.co/noticias/asi-son-ana-lucia-pineda-y-pilar-rueda-las-mujeres-que-aspiran-a-la-casa-de-narino/</t>
         </is>
       </c>
     </row>
@@ -5491,12 +5455,12 @@
       </c>
       <c r="D187" s="6" t="inlineStr">
         <is>
-          <t>Bogotá estrena el Teatro Nancy Kotal de Cortés: Un nuevo templo para el arte, el bilingüismo y la cultura</t>
+          <t>Abelardo de la Espriella responde desde un buque blindado: «No permitiremos que Petro y Cepeda se roben las elecciones»</t>
         </is>
       </c>
       <c r="E187" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/bogota-estrena-el-teatro-nancy-kotal-de-cortes-un-nuevo-templo-para-el-arte-el-bilinguismo-y-la-cultura/</t>
+          <t>https://canaltrece.com.co/noticias/abelardo-de-la-espriella-responde-desde-un-buque-blindado-no-permitiremos-que-petro-y-cepeda-se-roben-las-elecciones/</t>
         </is>
       </c>
     </row>
@@ -5514,12 +5478,12 @@
       </c>
       <c r="D188" s="3" t="inlineStr">
         <is>
-          <t>Pantallas gigantes y alta tecnología: El Mundial de Fútbol dispara la venta de televisores en Colombia</t>
+          <t>Iván Cepeda rompe el silencio: Congela aceptación de resultados, tilda a De la Espriella de «fascismo mafioso» y suma apoyos clave</t>
         </is>
       </c>
       <c r="E188" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/pantallas-gigantes-y-alta-tecnologia-el-mundial-de-futbol-dispara-la-venta-de-televisores-en-colombia/</t>
+          <t>https://canaltrece.com.co/noticias/ivan-cepeda-rompe-el-silencio-congela-aceptacion-de-resultados-tilda-a-de-la-espriella-de-fascismo-mafioso-y-suma-apoyos-clave/</t>
         </is>
       </c>
     </row>
@@ -5537,12 +5501,12 @@
       </c>
       <c r="D189" s="6" t="inlineStr">
         <is>
-          <t>Nico González: El productor y director musical colombiano que revoluciona el pop latino desde Miami</t>
+          <t>Presidente Petro no acepta el preconteo y denuncia graves irregularidades en el software electoral</t>
         </is>
       </c>
       <c r="E189" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/nico-gonzalez-el-productor-y-director-musical-colombiano-que-revoluciona-el-pop-latino-desde-miami/</t>
+          <t>https://canaltrece.com.co/noticias/presidente-petro-no-acepta-el-preconteo-y-denuncia-graves-irregularidades-en-el-software-electoral/</t>
         </is>
       </c>
     </row>
@@ -5560,12 +5524,12 @@
       </c>
       <c r="D190" s="3" t="inlineStr">
         <is>
-          <t>Claptone regresa a Medellín con su experiencia ‘Claptone &amp; Friends’</t>
+          <t>Jornada histórica y pacífica en Colombia: Más de 24 millones de ciudadanos votaron y definieron el balotaje para el 21 de junio</t>
         </is>
       </c>
       <c r="E190" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/claptone-regresa-a-medellin-con-su-experiencia-claptone-friends/</t>
+          <t>https://canaltrece.com.co/noticias/jornada-historica-y-pacifica-en-colombia-mas-de-24-millones-de-ciudadanos-votaron-y-definieron-el-balotaje-para-el-21-de-junio/</t>
         </is>
       </c>
     </row>
@@ -5583,12 +5547,12 @@
       </c>
       <c r="D191" s="6" t="inlineStr">
         <is>
-          <t>El restaurante Inquebrantable de Bogotá recibe el ‘Sello M’: Primer reconocimiento a la cocina mexicana auténtica en Colombia</t>
+          <t>Claudia López rompe el silencio: Pide a Cepeda asumir el liderazgo de su campaña ante el temor de una presidencia de De la Espriella</t>
         </is>
       </c>
       <c r="E191" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/el-restaurante-inquebrantable-de-bogota-recibe-el-sello-m-primer-reconocimiento-a-la-cocina-mexicana-autentica-en-colombia/</t>
+          <t>https://canaltrece.com.co/noticias/claudia-lopez-rompe-el-silencio-pide-a-cepeda-asumir-el-liderazgo-de-su-campana-ante-el-temor-de-una-presidencia-de-de-la-espriella/</t>
         </is>
       </c>
     </row>
@@ -5601,17 +5565,17 @@
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D192" s="3" t="inlineStr">
         <is>
-          <t>Mau y Ricky estrenan ‘Ricky y Mau’: Su álbum más íntimo, libre y colaborativo hasta la fecha</t>
+          <t>“Vamos a dar lo mejor para llevar a Colombia a lo más alto”: Néstor Lorenzo tras el partido de despedida premundialista</t>
         </is>
       </c>
       <c r="E192" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/mau-y-ricky-estrenan-ricky-y-mau-su-album-mas-intimo-libre-y-colaborativo-hasta-la-fecha/</t>
+          <t>https://www.elcolombiano.com/deportes/futbol/nestor-lorenzo-tecnico-seleccion-colombia-vs-costa-rica-despedida-mundial-MD37250837</t>
         </is>
       </c>
     </row>
@@ -5624,17 +5588,17 @@
       </c>
       <c r="C193" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D193" s="6" t="inlineStr">
         <is>
-          <t>Alejandro Saavedra estrena su EP ‘El Malo Soy Yo x Tener Corazón’: La nueva era del merenguetón y el pop urbano</t>
+          <t>Sin guiños al centro, Cepeda y Abelardo se atacaron en sus discursos, ¿cambiarán la estrategia?</t>
         </is>
       </c>
       <c r="E193" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/alejandro-saavedra-estrena-su-ep-el-malo-soy-yo-x-tener-corazon-la-nueva-era-del-merengueton-y-el-pop-urbano/</t>
+          <t>https://www.elcolombiano.com/colombia/politica/elecciones-2026-sin-guinos-centro-cepeda-abelardo-se-atacaron-NC37247684</t>
         </is>
       </c>
     </row>
@@ -5647,17 +5611,17 @@
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D194" s="3" t="inlineStr">
         <is>
-          <t>Así son Ana Lucía Pineda y Pilar Rueda, las mujeres que aspiran a la Casa de Nariño</t>
+          <t>Trump nomina a Nate Morris, “un firme defensor del movimiento MAGA”, como nuevo embajador en Colombia</t>
         </is>
       </c>
       <c r="E194" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/asi-son-ana-lucia-pineda-y-pilar-rueda-las-mujeres-que-aspiran-a-la-casa-de-narino/</t>
+          <t>https://www.elcolombiano.com/internacional/trump-nomina-empresario-nate-morris-embajador-estados-unidos-colombia-EC37246763</t>
         </is>
       </c>
     </row>
@@ -5670,17 +5634,17 @@
       </c>
       <c r="C195" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D195" s="6" t="inlineStr">
         <is>
-          <t>Abelardo de la Espriella responde desde un buque blindado: «No permitiremos que Petro y Cepeda se roben las elecciones»</t>
+          <t>Caso del joven ahogado en embalse de Guatapé: la familia le dio el último adiós y hablaron los primeros testigos</t>
         </is>
       </c>
       <c r="E195" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/abelardo-de-la-espriella-responde-desde-un-buque-blindado-no-permitiremos-que-petro-y-cepeda-se-roben-las-elecciones/</t>
+          <t>https://www.elcolombiano.com/antioquia/hablan-testigos-muerte-joven-embalse-penol-guatape-antioquia-CF37235744</t>
         </is>
       </c>
     </row>
@@ -5693,17 +5657,17 @@
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D196" s="3" t="inlineStr">
         <is>
-          <t>Iván Cepeda rompe el silencio: Congela aceptación de resultados, tilda a De la Espriella de «fascismo mafioso» y suma apoyos clave</t>
+          <t>Fiscalía confirma que 77 personas reportadas como desaparecidas salieron a votar en la primera vuelta presidencial</t>
         </is>
       </c>
       <c r="E196" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/ivan-cepeda-rompe-el-silencio-congela-aceptacion-de-resultados-tilda-a-de-la-espriella-de-fascismo-mafioso-y-suma-apoyos-clave/</t>
+          <t>https://www.elcolombiano.com/colombia/77-personas-desaparecidas-votaron-primera-vuelta-presidencial-NC37242816</t>
         </is>
       </c>
     </row>
@@ -5716,17 +5680,17 @@
       </c>
       <c r="C197" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D197" s="6" t="inlineStr">
         <is>
-          <t>Presidente Petro no acepta el preconteo y denuncia graves irregularidades en el software electoral</t>
+          <t>¿Qué tan cerca estuvieron las encuestas? Vieron la segunda vuelta, pero no el triunfo de Abelardo</t>
         </is>
       </c>
       <c r="E197" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/presidente-petro-no-acepta-el-preconteo-y-denuncia-graves-irregularidades-en-el-software-electoral/</t>
+          <t>https://www.elcolombiano.com/especiales/elecciones-2026/las-encuestas-acertaron-ganadores-primera-vuelta-presidencial-FE37223035</t>
         </is>
       </c>
     </row>
@@ -5739,17 +5703,17 @@
       </c>
       <c r="C198" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D198" s="3" t="inlineStr">
         <is>
-          <t>Jornada histórica y pacífica en Colombia: Más de 24 millones de ciudadanos votaron y definieron el balotaje para el 21 de junio</t>
+          <t>¿Votó o fue jurado? Así puede reclamar hasta un día y medio de descanso remunerado</t>
         </is>
       </c>
       <c r="E198" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/jornada-historica-y-pacifica-en-colombia-mas-de-24-millones-de-ciudadanos-votaron-y-definieron-el-balotaje-para-el-21-de-junio/</t>
+          <t>https://www.elcolombiano.com/negocios/voto-o-fue-jurado-asi-puede-reclamar-hasta-un-dia-y-medio-de-descanso-remunerado-OH37217018</t>
         </is>
       </c>
     </row>
@@ -5762,17 +5726,17 @@
       </c>
       <c r="C199" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D199" s="6" t="inlineStr">
         <is>
-          <t>Claudia López rompe el silencio: Pide a Cepeda asumir el liderazgo de su campaña ante el temor de una presidencia de De la Espriella</t>
+          <t>Corte dice que prepagadas deben justificar afiliaciones sin discriminar; ¿por qué?</t>
         </is>
       </c>
       <c r="E199" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/claudia-lopez-rompe-el-silencio-pide-a-cepeda-asumir-el-liderazgo-de-su-campana-ante-el-temor-de-una-presidencia-de-de-la-espriella/</t>
+          <t>https://www.elcolombiano.com/colombia/salud/corte-constitucional-prepagadas-justificar-afiliaciones-sin-discriminar-HC37246472</t>
         </is>
       </c>
     </row>
@@ -5785,17 +5749,17 @@
       </c>
       <c r="C200" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D200" s="3" t="inlineStr">
         <is>
-          <t>Abelardo de la Espriella tiene el 81 % de probabilidad de ser el presidente de Colombia, según Polymarket</t>
+          <t>Operativo destapa helicóptero con pasado oscuro y motor Rolls-Royce</t>
         </is>
       </c>
       <c r="E200" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/abelardo-de-la-espriella-tiene-el-81-de-probabilidad-de-ser-el-presidente-de-colombia-segun-polymarket/202616/</t>
+          <t>https://www.elcolombiano.com/colombia/ejercito-incauta-helicoptero-de-la-mafia-NG33717192</t>
         </is>
       </c>
     </row>
@@ -5808,17 +5772,17 @@
       </c>
       <c r="C201" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D201" s="6" t="inlineStr">
         <is>
-          <t>“Al mejor estilo de Maduro”: Abelardo de la Espriella reaccionó al apoyo del presidente de Ecuador y arremetió contra Petro y Cepeda</t>
+          <t>Así fue el adiós a Alexánder Avendaño, joven que murió en el embalse El Peñol–Guatapé</t>
         </is>
       </c>
       <c r="E201" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/al-mejor-estilo-de-maduro-abelardo-de-la-espriella-reacciono-al-apoyo-del-presidente-de-ecuador-y-arremetio-contra-petro-y-cepeda/202631/</t>
+          <t>https://www.elcolombiano.com/medellin/entierro-joven-alexander-avendano-san-cristobal-medellin-ahogamiento-embalse-guatape-antioquia-AD37251809</t>
         </is>
       </c>
     </row>
@@ -5831,17 +5795,17 @@
       </c>
       <c r="C202" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D202" s="3" t="inlineStr">
         <is>
-          <t>Miguel Ospino responde a denuncia de Angie Rodríguez: “Afirmaciones irresponsables y carentes de corroboración”</t>
+          <t>¿Podrían responder por omisión quienes acompañaban al joven ahogado en el embalse de Guatapé? Experto explica</t>
         </is>
       </c>
       <c r="E202" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/miguel-ospino-responde-a-denuncia-de-angie-rodriguez-afirmaciones-irresponsables-y-carentes-de-corroboracion/202623/</t>
+          <t>https://www.elcolombiano.com/antioquia/alexander-avendano-consecuencias-penales-por-muerte-embalse-guatape-OC37248633</t>
         </is>
       </c>
     </row>
@@ -5854,17 +5818,17 @@
       </c>
       <c r="C203" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D203" s="6" t="inlineStr">
         <is>
-          <t>Abelardo de la Espriella desmiente supuesto respaldo de Ape Cuello: “Impresentable sujeto”</t>
+          <t>Primera vuelta: cuatro claves para entender cómo cambió el mapa político de Antioquia</t>
         </is>
       </c>
       <c r="E203" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/confidenciales/articulo/abelardo-de-la-espriella-desmiente-supuesto-respaldo-de-ape-cuello-impresentable-sujeto/202628/</t>
+          <t>https://www.elcolombiano.com/antioquia/antioquia-medellin-elecciones-presidenciales-2026-analisis-JC37247583</t>
         </is>
       </c>
     </row>
@@ -5877,17 +5841,17 @@
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D204" s="3" t="inlineStr">
         <is>
-          <t>Dolor en La Victoria: el brutal asesinato de un niño de 13 años que hoy conmociona al Valle del Cauca</t>
+          <t>Ley Yulixa Toloza: iniciativa que busca regular las cirugías estéticas en Colombia</t>
         </is>
       </c>
       <c r="E204" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/dolor-en-la-victoria-el-brutal-asesinato-de-un-nino-de-13-anos-que-hoy-conmociona-al-valle-del-cauca/202606/</t>
+          <t>https://www.elcolombiano.com/colombia/ley-yulixa-toloza-regulacion-cirugias-esteticas-colombia-CC37243643</t>
         </is>
       </c>
     </row>
@@ -5900,17 +5864,17 @@
       </c>
       <c r="C205" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D205" s="6" t="inlineStr">
         <is>
-          <t>Falleció el Mayor General (R) Javier Ayala Amaya, el rector que impulsó una educación para la paz desde la Universidad Militar Nueva Granada</t>
+          <t>Ante riesgos energéticos de El Niño, EPM lanzará campaña prevenvita ¿En qué consistirá?</t>
         </is>
       </c>
       <c r="E205" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/foros-semana/articulo/fallecio-el-mayor-general-r-javier-ayala-amaya-el-rector-que-impulso-una-educacion-para-la-paz-desde-la-universidad-militar-nueva-granada/202630/</t>
+          <t>https://www.elcolombiano.com/antioquia/epm-lanzamiento-campana-prevencion-sequias-embalses-antioquia-EC37247704</t>
         </is>
       </c>
     </row>
@@ -5923,17 +5887,17 @@
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D206" s="3" t="inlineStr">
         <is>
-          <t>Tras los resultados electorales favorables a Abelardo de la Espriella, bajaron el precio del dólar y las tasas de deuda</t>
+          <t>“Crean siempre”: el poderoso mensaje de James Rodríguez y Luis Díaz tras la despedida de la Selección Colombia</t>
         </is>
       </c>
       <c r="E206" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/economia/macroeconomia/articulo/tras-los-resultados-electorales-favorables-a-abelardo-de-la-espriella-bajaron-el-precio-del-dolar-y-las-tasas-de-deuda/202639/</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/james-rodriguez-luis-diaz-despedida-seleccion-colombia-mundial-HC37247761</t>
         </is>
       </c>
     </row>
@@ -5946,17 +5910,17 @@
       </c>
       <c r="C207" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D207" s="6" t="inlineStr">
         <is>
-          <t>Delcy Rodríguez se dirige a Diosdado Cabello y le da una polémica orden que sorprendió en pleno evento público</t>
+          <t>Falcao jugará el Mundial 2026 desde otra cancha: cambia los guayos por el micrófono</t>
         </is>
       </c>
       <c r="E207" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/mundo/articulo/delcy-rodriguez-se-dirige-a-diosdado-cabello-y-le-da-una-polemica-orden-que-sorprendio-en-pleno-evento-publico/202634/</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/falcao-comentara-mundial-2026-con-espn-disney-HC37245354</t>
         </is>
       </c>
     </row>
@@ -5969,17 +5933,17 @@
       </c>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D208" s="3" t="inlineStr">
         <is>
-          <t>¿Quiénes eran las cuatro víctimas del accidente aéreo en Meta? Revelan sus identidades</t>
+          <t>¡Increíble! En Nariño, Antioquia, una vaca tuvo cuatrillizos; ocurre en menos del 1% de los partos</t>
         </is>
       </c>
       <c r="E208" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/quienes-eran-las-cuatro-victimas-del-accidente-aereo-en-meta-revelan-sus-identidades/202642/</t>
+          <t>https://www.elcolombiano.com/antioquia/vaca-narino-antioquia-tuvo-cuatrillizos-suceso-muy-raro-HC37245222</t>
         </is>
       </c>
     </row>
@@ -5992,17 +5956,17 @@
       </c>
       <c r="C209" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D209" s="6" t="inlineStr">
         <is>
-          <t>Colombia bailó a Costa Rica en El Campín y se va sonriendo al Mundial 2026: resultado y goles</t>
+          <t>Más allá de la sequía: Procuraduría advierte impacto del fenómeno de El Niño en la comida, luz y agua del país</t>
         </is>
       </c>
       <c r="E209" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/colombia-bailo-a-costa-rica-en-el-campin-y-se-va-sonriendo-al-mundial-2026-resultado-y-goles/202643/</t>
+          <t>https://www.elcolombiano.com/colombia/procuraduria-advierte-impacto-fenomeno-nino-comida-luz-agua-colombia-FF37238287</t>
         </is>
       </c>
     </row>
@@ -6015,17 +5979,17 @@
       </c>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D210" s="3" t="inlineStr">
         <is>
-          <t>“El enemigo está atacando con misiles balísticos”: se registran nuevos bombardeos en Ucrania</t>
+          <t>Dibu Martínez en alerta: jugará el Mundial 2026 con una fractura en la mano</t>
         </is>
       </c>
       <c r="E210" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/mundo/articulo/el-enemigo-esta-atacando-con-misiles-balisticos-se-registran-nuevos-bombardeos-en-ucrania/202642/</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/dibu-martinez-fractura-mano-mundial-selecion-argentina-KC37243845</t>
         </is>
       </c>
     </row>
@@ -6038,17 +6002,17 @@
       </c>
       <c r="C211" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D211" s="6" t="inlineStr">
         <is>
-          <t>Movilización juvenil se tomó las calles de Bogotá tras la primera vuelta presidencial y respaldó a Iván Cepeda</t>
+          <t>DIM aún no termina el semestre: recibe a Cúcuta en Itagüí buscando los octavos de la Copa BetPlay</t>
         </is>
       </c>
       <c r="E211" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/movilizacion-juvenil-se-tomo-las-calles-de-bogota-tras-la-primera-vuelta-presidencial-y-respaldo-a-ivan-cepeda/202649/</t>
+          <t>https://www.elcolombiano.com/deportes/futbol/dim-vs-cucuta-juego-copa-betplay-fase-de-grupos-clasificacion-octavos-de-final-AF37236464</t>
         </is>
       </c>
     </row>
@@ -6061,17 +6025,17 @@
       </c>
       <c r="C212" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D212" s="3" t="inlineStr">
         <is>
-          <t>James y Juanfer en todo su esplendor: Magistral jugada contra Costa Rica para un golazo de Luis Suárez</t>
+          <t>Las películas y series que llegarán a Netflix, HBO Max, Prime Video y Apple TV en junio 2026</t>
         </is>
       </c>
       <c r="E212" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/james-y-juanfer-en-todo-su-esplendor-magistral-jugada-contra-costa-rica-para-un-golazo-de-luis-suarez/202635/</t>
+          <t>https://www.elcolombiano.com/entretenimiento/television/estrenos-peliculas-series-netflix-hbo-prime-apple-tv-junio-2026-CE37224341</t>
         </is>
       </c>
     </row>
@@ -6084,17 +6048,17 @@
       </c>
       <c r="C213" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D213" s="6" t="inlineStr">
         <is>
-          <t>Alcalde Carlos Fernando Galán agradece a la Selección Colombia por despedirse en Bogotá rumbo al Mundial tras partido con Costa Rica</t>
+          <t>¿Cuál es el más fuerte de los 4 países debutantes en Norteamérica 2026?</t>
         </is>
       </c>
       <c r="E213" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/alcalde-carlos-fernando-galan-agradece-a-la-seleccion-colombia-por-despedirse-en-bogota-rumbo-al-mundial-tras-partido-con-costa-rica/202658/</t>
+          <t>https://www.elcolombiano.com/deportes/futbol/paises-debutantes-mundial-2026-uzbekistan-jordania-cabo-verde-curazao-BC37241527</t>
         </is>
       </c>
     </row>
@@ -6107,17 +6071,17 @@
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D214" s="3" t="inlineStr">
         <is>
-          <t>La reacción de Luis Díaz tras la despedida de la Selección Colombia en El Campín: habló del público en Bogotá</t>
+          <t>Francia se convierte en aliado de Medellín para fortalecer el turismo sostenible, ¿cómo lo hará?</t>
         </is>
       </c>
       <c r="E214" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/la-reaccion-de-luis-diaz-tras-la-despedida-de-la-seleccion-colombia-en-el-campin-hablo-del-publico-en-bogota/202651/</t>
+          <t>https://www.elcolombiano.com/medellin/alianza-con-francia-para-turismo-sostenible-medellin-antioquia-DC37241013</t>
         </is>
       </c>
     </row>
@@ -6130,17 +6094,17 @@
       </c>
       <c r="C215" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D215" s="6" t="inlineStr">
         <is>
-          <t>¿Los vehículos eléctricos livianos son seguros para circular por ciclorrutas? Lo que se debate en el Concejo de Bogotá</t>
+          <t>Venezuela rompe su récord exportador de petróleo desde las sanciones de 2019</t>
         </is>
       </c>
       <c r="E215" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/vehiculos/articulo/los-vehiculos-electricos-livianos-son-seguros-para-circular-por-ciclorrutas-lo-que-se-debate-en-el-concejo-de-bogota/202642/</t>
+          <t>https://www.elcolombiano.com/negocios/exportaciones-petroleo-venezuela-mayo-2026-pdvsa-colombia-HC37241240</t>
         </is>
       </c>
     </row>
@@ -6153,17 +6117,17 @@
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D216" s="3" t="inlineStr">
         <is>
-          <t>¿Cuándo vuelve a jugar la Selección Colombia? Fecha, hora y rival del próximo partido</t>
+          <t>Procurador Eljach controvierte a Petro por querer desconocer preconteo: “no hay evidencia o reclamaciones que resolver”</t>
         </is>
       </c>
       <c r="E216" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/cuando-vuelve-a-jugar-la-seleccion-colombia-fecha-hora-y-rival-del-proximo-partido/202613/</t>
+          <t>https://www.elcolombiano.com/colombia/procuraduria-gregorio-eljach-dice-que-no-hay-evidencia-de-fraude-DC37241075</t>
         </is>
       </c>
     </row>
@@ -6176,17 +6140,17 @@
       </c>
       <c r="C217" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D217" s="6" t="inlineStr">
         <is>
-          <t>Meta, TikTok y YouTube acuerdan millonaria compensación por dañar la salud mental de estudiantes y para evitar un juicio histórico</t>
+          <t>En Antioquia se vendieron casi 25.000 carros nuevos en los primeros cinco meses de 2026</t>
         </is>
       </c>
       <c r="E217" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/tecnologia/articulo/meta-tiktok-y-youtube-acuerdan-millonaria-compensacion-por-danar-la-salud-mental-de-estudiantes-y-para-evitar-un-juicio-historico/202611/</t>
+          <t>https://www.elcolombiano.com/negocios/venta-carros-nuevos-medellin-antioquia-2026-IF37239023</t>
         </is>
       </c>
     </row>
@@ -6199,17 +6163,17 @@
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D218" s="3" t="inlineStr">
         <is>
-          <t>“Es una vergüenza”: Juliana Galvis rompió el silencio, defendió a Abelardo y frenó las versiones de fraude electoral</t>
+          <t>Descarga mortal en Doradal: un rayo acabó con 25 cabezas de ganado</t>
         </is>
       </c>
       <c r="E218" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/gente/articulo/es-una-verguenza-juliana-galvis-rompio-el-silencio-defendio-a-abelardo-y-freno-las-versiones-de-fraude-electoral/202621/</t>
+          <t>https://www.elcolombiano.com/antioquia/descarga-mortal-doradal-rayo-acabo-25-cabezas-ganado-LF37238614</t>
         </is>
       </c>
     </row>
@@ -6222,17 +6186,17 @@
       </c>
       <c r="C219" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D219" s="6" t="inlineStr">
         <is>
-          <t>Falcao García consiguió nuevo trabajo y así fue su presentación oficial: “Bienvenido ídolo”</t>
+          <t>De la Espriella ganó hasta en Venezuela: así votaron los colombianos en el exterior en la primera vuelta presidencial</t>
         </is>
       </c>
       <c r="E219" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/falcao-garcia-consiguio-nuevo-trabajo-y-asi-fue-su-presentacion-oficial-bienvenido-idolo/202657/</t>
+          <t>https://www.elcolombiano.com/internacional/resultados-elecciones-colombianos-exterior-primera-vuelta-2026-DF37236577</t>
         </is>
       </c>
     </row>
@@ -6245,17 +6209,17 @@
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D220" s="3" t="inlineStr">
         <is>
-          <t>Novia de James Rodríguez publicó inesperada fotografía antes del partido de la Selección Colombia</t>
+          <t>¿Quiénes ya anunciaron su apoyo para la segunda vuelta? Miguel Uribe Londoño y el Partido Conservador ya dijeron que se van con De la Espriella</t>
         </is>
       </c>
       <c r="E220" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/gente/articulo/la-tierna-foto-que-compartio-la-novia-de-james-rodriguez-antes-del-partido-de-la-seleccion-colombia/202634/</t>
+          <t>https://www.elcolombiano.com/especiales/elecciones-2026/apoyo-miguel-uribe-londono-partido-conservador-de-la-espriella-EF37237113</t>
         </is>
       </c>
     </row>
@@ -6268,17 +6232,17 @@
       </c>
       <c r="C221" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D221" s="6" t="inlineStr">
         <is>
-          <t>‘The Economist’ reconoce que Abelardo de la Espriella sería el próximo presidente</t>
+          <t>Las propuestas económicas de Cepeda y De la Espriella que definirán la segunda vuelta presidencial en Colombia</t>
         </is>
       </c>
       <c r="E221" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/the-economist-reconoce-que-abelardo-de-la-espriella-seria-el-proximo-presidente/202611/</t>
+          <t>https://www.elcolombiano.com/negocios/propuestas-economicas-cepeda-abelardo-segunda-vuelta-presidencia-DH37213734</t>
         </is>
       </c>
     </row>
@@ -6296,12 +6260,12 @@
       </c>
       <c r="D222" s="3" t="inlineStr">
         <is>
-          <t>Le recuerdan a Petro cuando usaba la camiseta de la Selección Colombia en la campaña de 2022, lo que ahora critica Cepeda</t>
+          <t>Abelardo de la Espriella tiene el 81 % de probabilidad de ser el presidente de Colombia, según Polymarket</t>
         </is>
       </c>
       <c r="E222" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/le-recuerdan-a-petro-cuando-usaba-la-camiseta-de-la-seleccion-colombia-en-la-campana-de-2022-lo-que-ahora-critica-cepeda/202628/</t>
+          <t>https://www.semana.com/politica/articulo/abelardo-de-la-espriella-tiene-el-81-de-probabilidad-de-ser-el-presidente-de-colombia-segun-polymarket/202616/</t>
         </is>
       </c>
     </row>
@@ -6319,12 +6283,12 @@
       </c>
       <c r="D223" s="6" t="inlineStr">
         <is>
-          <t>Primer funcionario del Gobierno le pidió públicamente a Gustavo Petro que renuncie a la Presidencia: “Victoria o muerte”</t>
+          <t>“Al mejor estilo de Maduro”: Abelardo de la Espriella reaccionó al apoyo del presidente de Ecuador y arremetió contra Petro y Cepeda</t>
         </is>
       </c>
       <c r="E223" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/primer-funcionario-del-gobierno-le-pidio-publicamente-a-gustavo-petro-que-renuncie-a-la-presidencia-victoria-o-muerte/202625/</t>
+          <t>https://www.semana.com/politica/articulo/al-mejor-estilo-de-maduro-abelardo-de-la-espriella-reacciono-al-apoyo-del-presidente-de-ecuador-y-arremetio-contra-petro-y-cepeda/202631/</t>
         </is>
       </c>
     </row>
@@ -6342,12 +6306,12 @@
       </c>
       <c r="D224" s="3" t="inlineStr">
         <is>
-          <t>Miguel Uribe Londoño dice que “entramado criminal que tiene tomado el Gobierno de Gustavo Petro” está detrás del crimen de su hijo</t>
+          <t>Miguel Ospino responde a denuncia de Angie Rodríguez: “Afirmaciones irresponsables y carentes de corroboración”</t>
         </is>
       </c>
       <c r="E224" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/semana-tv/semana-el-debate/articulo/miguel-uribe-londono-dice-que-entramado-criminal-que-tiene-tomado-el-gobierno-de-gustavo-petro-esta-detras-del-crimen-de-su-hijo/202645/</t>
+          <t>https://www.semana.com/nacion/articulo/miguel-ospino-responde-a-denuncia-de-angie-rodriguez-afirmaciones-irresponsables-y-carentes-de-corroboracion/202623/</t>
         </is>
       </c>
     </row>
@@ -6365,12 +6329,12 @@
       </c>
       <c r="D225" s="6" t="inlineStr">
         <is>
-          <t>Imputan cargos a alcaldesa de Ibagué por presuntas irregularidades en contrato para compra de comida para animales de un centro de protección</t>
+          <t>Abelardo de la Espriella desmiente supuesto respaldo de Ape Cuello: “Impresentable sujeto”</t>
         </is>
       </c>
       <c r="E225" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/armenia/articulo/imputan-cargos-a-alcaldesa-de-ibague-por-presuntas-irregularidades-en-contrato-para-compra-de-comida-para-animales-de-un-centro-de-proteccion/202642/</t>
+          <t>https://www.semana.com/confidenciales/articulo/abelardo-de-la-espriella-desmiente-supuesto-respaldo-de-ape-cuello-impresentable-sujeto/202628/</t>
         </is>
       </c>
     </row>
@@ -6388,12 +6352,12 @@
       </c>
       <c r="D226" s="3" t="inlineStr">
         <is>
-          <t>Hombre murió en plena vía pública en medio de las elecciones por esta prenda de vestir</t>
+          <t>Dolor en La Victoria: el brutal asesinato de un niño de 13 años que hoy conmociona al Valle del Cauca</t>
         </is>
       </c>
       <c r="E226" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/hombre-murio-en-plena-via-publica-en-medio-de-las-elecciones-por-esta-prenda-de-vestir/202615/</t>
+          <t>https://www.semana.com/nacion/articulo/dolor-en-la-victoria-el-brutal-asesinato-de-un-nino-de-13-anos-que-hoy-conmociona-al-valle-del-cauca/202606/</t>
         </is>
       </c>
     </row>
@@ -6411,12 +6375,12 @@
       </c>
       <c r="D227" s="6" t="inlineStr">
         <is>
-          <t>Barbosa redujo en un 82 % su deuda con acreedores y ejecuta obras de infraestructura por miles de millones de pesos</t>
+          <t>Falleció el Mayor General (R) Javier Ayala Amaya, el rector que impulsó una educación para la paz desde la Universidad Militar Nueva Granada</t>
         </is>
       </c>
       <c r="E227" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/medellin/articulo/barbosa-redujo-en-un-82-su-deuda-con-acreedores-y-ejecuta-obras-de-infraestructura-por-miles-de-millones-de-pesos/202605/</t>
+          <t>https://www.semana.com/foros-semana/articulo/fallecio-el-mayor-general-r-javier-ayala-amaya-el-rector-que-impulso-una-educacion-para-la-paz-desde-la-universidad-militar-nueva-granada/202630/</t>
         </is>
       </c>
     </row>
@@ -6434,12 +6398,12 @@
       </c>
       <c r="D228" s="3" t="inlineStr">
         <is>
-          <t>Cali busca posicionarse como referente global de transformación urbana en Cumbre de Ciudades en Singapur</t>
+          <t>Tras los resultados electorales favorables a Abelardo de la Espriella, bajaron el precio del dólar y las tasas de deuda</t>
         </is>
       </c>
       <c r="E228" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/cali/articulo/cali-busca-posicionarse-como-referente-global-de-transformacion-urbana-en-cumbre-de-ciudades-en-singapur/202633/</t>
+          <t>https://www.semana.com/economia/macroeconomia/articulo/tras-los-resultados-electorales-favorables-a-abelardo-de-la-espriella-bajaron-el-precio-del-dolar-y-las-tasas-de-deuda/202639/</t>
         </is>
       </c>
     </row>
@@ -6457,12 +6421,12 @@
       </c>
       <c r="D229" s="6" t="inlineStr">
         <is>
-          <t>Wendy Sepúlveda no resistió: murió la joven atacada con gasolina por su expareja en Neiva</t>
+          <t>Delcy Rodríguez se dirige a Diosdado Cabello y le da una polémica orden que sorprendió en pleno evento público</t>
         </is>
       </c>
       <c r="E229" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/wendy-sepulveda-no-resistio-murio-la-joven-atacada-con-gasolina-por-su-expareja-en-neiva/202645/</t>
+          <t>https://www.semana.com/mundo/articulo/delcy-rodriguez-se-dirige-a-diosdado-cabello-y-le-da-una-polemica-orden-que-sorprendio-en-pleno-evento-publico/202634/</t>
         </is>
       </c>
     </row>
@@ -6475,17 +6439,17 @@
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D230" s="3" t="inlineStr">
         <is>
-          <t>“Vamos a dar lo mejor para llevar a Colombia a lo más alto”: Néstor Lorenzo tras el partido de despedida premundialista</t>
+          <t>¿Quiénes eran las cuatro víctimas del accidente aéreo en Meta? Revelan sus identidades</t>
         </is>
       </c>
       <c r="E230" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/deportes/futbol/nestor-lorenzo-tecnico-seleccion-colombia-vs-costa-rica-despedida-mundial-MD37250837</t>
+          <t>https://www.semana.com/nacion/articulo/quienes-eran-las-cuatro-victimas-del-accidente-aereo-en-meta-revelan-sus-identidades/202642/</t>
         </is>
       </c>
     </row>
@@ -6498,17 +6462,17 @@
       </c>
       <c r="C231" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D231" s="6" t="inlineStr">
         <is>
-          <t>Sin guiños al centro, Cepeda y Abelardo se atacaron en sus discursos, ¿cambiarán la estrategia?</t>
+          <t>Colombia bailó a Costa Rica en El Campín y se va sonriendo al Mundial 2026: resultado y goles</t>
         </is>
       </c>
       <c r="E231" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/politica/elecciones-2026-sin-guinos-centro-cepeda-abelardo-se-atacaron-NC37247684</t>
+          <t>https://www.semana.com/deportes/articulo/colombia-bailo-a-costa-rica-en-el-campin-y-se-va-sonriendo-al-mundial-2026-resultado-y-goles/202643/</t>
         </is>
       </c>
     </row>
@@ -6521,17 +6485,17 @@
       </c>
       <c r="C232" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D232" s="3" t="inlineStr">
         <is>
-          <t>Trump nomina a Nate Morris, “un firme defensor del movimiento MAGA”, como nuevo embajador en Colombia</t>
+          <t>“El enemigo está atacando con misiles balísticos”: se registran nuevos bombardeos en Ucrania</t>
         </is>
       </c>
       <c r="E232" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/internacional/trump-nomina-empresario-nate-morris-embajador-estados-unidos-colombia-EC37246763</t>
+          <t>https://www.semana.com/mundo/articulo/el-enemigo-esta-atacando-con-misiles-balisticos-se-registran-nuevos-bombardeos-en-ucrania/202642/</t>
         </is>
       </c>
     </row>
@@ -6544,17 +6508,17 @@
       </c>
       <c r="C233" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D233" s="6" t="inlineStr">
         <is>
-          <t>Caso del joven ahogado en embalse de Guatapé: la familia le dio el último adiós y hablaron los primeros testigos</t>
+          <t>Movilización juvenil se tomó las calles de Bogotá tras la primera vuelta presidencial y respaldó a Iván Cepeda</t>
         </is>
       </c>
       <c r="E233" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/antioquia/hablan-testigos-muerte-joven-embalse-penol-guatape-antioquia-CF37235744</t>
+          <t>https://www.semana.com/politica/articulo/movilizacion-juvenil-se-tomo-las-calles-de-bogota-tras-la-primera-vuelta-presidencial-y-respaldo-a-ivan-cepeda/202649/</t>
         </is>
       </c>
     </row>
@@ -6567,17 +6531,17 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D234" s="3" t="inlineStr">
         <is>
-          <t>Fiscalía confirma que 77 personas reportadas como desaparecidas salieron a votar en la primera vuelta presidencial</t>
+          <t>James y Juanfer en todo su esplendor: Magistral jugada contra Costa Rica para un golazo de Luis Suárez</t>
         </is>
       </c>
       <c r="E234" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/77-personas-desaparecidas-votaron-primera-vuelta-presidencial-NC37242816</t>
+          <t>https://www.semana.com/deportes/articulo/james-y-juanfer-en-todo-su-esplendor-magistral-jugada-contra-costa-rica-para-un-golazo-de-luis-suarez/202635/</t>
         </is>
       </c>
     </row>
@@ -6590,17 +6554,17 @@
       </c>
       <c r="C235" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D235" s="6" t="inlineStr">
         <is>
-          <t>¿Qué tan cerca estuvieron las encuestas? Vieron la segunda vuelta, pero no el triunfo de Abelardo</t>
+          <t>Alcalde Carlos Fernando Galán agradece a la Selección Colombia por despedirse en Bogotá rumbo al Mundial tras partido con Costa Rica</t>
         </is>
       </c>
       <c r="E235" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/elecciones-2026/las-encuestas-acertaron-ganadores-primera-vuelta-presidencial-FE37223035</t>
+          <t>https://www.semana.com/deportes/articulo/alcalde-carlos-fernando-galan-agradece-a-la-seleccion-colombia-por-despedirse-en-bogota-rumbo-al-mundial-tras-partido-con-costa-rica/202658/</t>
         </is>
       </c>
     </row>
@@ -6613,17 +6577,17 @@
       </c>
       <c r="C236" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D236" s="3" t="inlineStr">
         <is>
-          <t>¿Votó o fue jurado? Así puede reclamar hasta un día y medio de descanso remunerado</t>
+          <t>La reacción de Luis Díaz tras la despedida de la Selección Colombia en El Campín: habló del público en Bogotá</t>
         </is>
       </c>
       <c r="E236" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/negocios/voto-o-fue-jurado-asi-puede-reclamar-hasta-un-dia-y-medio-de-descanso-remunerado-OH37217018</t>
+          <t>https://www.semana.com/deportes/articulo/la-reaccion-de-luis-diaz-tras-la-despedida-de-la-seleccion-colombia-en-el-campin-hablo-del-publico-en-bogota/202651/</t>
         </is>
       </c>
     </row>
@@ -6636,17 +6600,17 @@
       </c>
       <c r="C237" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D237" s="6" t="inlineStr">
         <is>
-          <t>Corte dice que prepagadas deben justificar afiliaciones sin discriminar; ¿por qué?</t>
+          <t>¿Los vehículos eléctricos livianos son seguros para circular por ciclorrutas? Lo que se debate en el Concejo de Bogotá</t>
         </is>
       </c>
       <c r="E237" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/salud/corte-constitucional-prepagadas-justificar-afiliaciones-sin-discriminar-HC37246472</t>
+          <t>https://www.semana.com/vehiculos/articulo/los-vehiculos-electricos-livianos-son-seguros-para-circular-por-ciclorrutas-lo-que-se-debate-en-el-concejo-de-bogota/202642/</t>
         </is>
       </c>
     </row>
@@ -6659,17 +6623,17 @@
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D238" s="3" t="inlineStr">
         <is>
-          <t>Operativo destapa helicóptero con pasado oscuro y motor Rolls-Royce</t>
+          <t>¿Cuándo vuelve a jugar la Selección Colombia? Fecha, hora y rival del próximo partido</t>
         </is>
       </c>
       <c r="E238" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/ejercito-incauta-helicoptero-de-la-mafia-NG33717192</t>
+          <t>https://www.semana.com/deportes/articulo/cuando-vuelve-a-jugar-la-seleccion-colombia-fecha-hora-y-rival-del-proximo-partido/202613/</t>
         </is>
       </c>
     </row>
@@ -6682,17 +6646,17 @@
       </c>
       <c r="C239" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D239" s="6" t="inlineStr">
         <is>
-          <t>Así fue el adiós a Alexánder Avendaño, joven que murió en el embalse El Peñol–Guatapé</t>
+          <t>Meta, TikTok y YouTube acuerdan millonaria compensación por dañar la salud mental de estudiantes y para evitar un juicio histórico</t>
         </is>
       </c>
       <c r="E239" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/medellin/entierro-joven-alexander-avendano-san-cristobal-medellin-ahogamiento-embalse-guatape-antioquia-AD37251809</t>
+          <t>https://www.semana.com/tecnologia/articulo/meta-tiktok-y-youtube-acuerdan-millonaria-compensacion-por-danar-la-salud-mental-de-estudiantes-y-para-evitar-un-juicio-historico/202611/</t>
         </is>
       </c>
     </row>
@@ -6705,17 +6669,17 @@
       </c>
       <c r="C240" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D240" s="3" t="inlineStr">
         <is>
-          <t>¿Podrían responder por omisión quienes acompañaban al joven ahogado en el embalse de Guatapé? Experto explica</t>
+          <t>“Es una vergüenza”: Juliana Galvis rompió el silencio, defendió a Abelardo y frenó las versiones de fraude electoral</t>
         </is>
       </c>
       <c r="E240" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/antioquia/alexander-avendano-consecuencias-penales-por-muerte-embalse-guatape-OC37248633</t>
+          <t>https://www.semana.com/gente/articulo/es-una-verguenza-juliana-galvis-rompio-el-silencio-defendio-a-abelardo-y-freno-las-versiones-de-fraude-electoral/202621/</t>
         </is>
       </c>
     </row>
@@ -6728,17 +6692,17 @@
       </c>
       <c r="C241" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D241" s="6" t="inlineStr">
         <is>
-          <t>Primera vuelta: cuatro claves para entender cómo cambió el mapa político de Antioquia</t>
+          <t>Falcao García consiguió nuevo trabajo y así fue su presentación oficial: “Bienvenido ídolo”</t>
         </is>
       </c>
       <c r="E241" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/antioquia/antioquia-medellin-elecciones-presidenciales-2026-analisis-JC37247583</t>
+          <t>https://www.semana.com/deportes/articulo/falcao-garcia-consiguio-nuevo-trabajo-y-asi-fue-su-presentacion-oficial-bienvenido-idolo/202657/</t>
         </is>
       </c>
     </row>
@@ -6751,17 +6715,17 @@
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D242" s="3" t="inlineStr">
         <is>
-          <t>Ley Yulixa Toloza: iniciativa que busca regular las cirugías estéticas en Colombia</t>
+          <t>Novia de James Rodríguez publicó inesperada fotografía antes del partido de la Selección Colombia</t>
         </is>
       </c>
       <c r="E242" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/ley-yulixa-toloza-regulacion-cirugias-esteticas-colombia-CC37243643</t>
+          <t>https://www.semana.com/gente/articulo/la-tierna-foto-que-compartio-la-novia-de-james-rodriguez-antes-del-partido-de-la-seleccion-colombia/202634/</t>
         </is>
       </c>
     </row>
@@ -6774,17 +6738,17 @@
       </c>
       <c r="C243" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D243" s="6" t="inlineStr">
         <is>
-          <t>Ante riesgos energéticos de El Niño, EPM lanzará campaña prevenvita ¿En qué consistirá?</t>
+          <t>‘The Economist’ reconoce que Abelardo de la Espriella sería el próximo presidente</t>
         </is>
       </c>
       <c r="E243" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/antioquia/epm-lanzamiento-campana-prevencion-sequias-embalses-antioquia-EC37247704</t>
+          <t>https://www.semana.com/politica/articulo/the-economist-reconoce-que-abelardo-de-la-espriella-seria-el-proximo-presidente/202611/</t>
         </is>
       </c>
     </row>
@@ -6797,17 +6761,17 @@
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D244" s="3" t="inlineStr">
         <is>
-          <t>“Crean siempre”: el poderoso mensaje de James Rodríguez y Luis Díaz tras la despedida de la Selección Colombia</t>
+          <t>Le recuerdan a Petro cuando usaba la camiseta de la Selección Colombia en la campaña de 2022, lo que ahora critica Cepeda</t>
         </is>
       </c>
       <c r="E244" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/mundial-2026/james-rodriguez-luis-diaz-despedida-seleccion-colombia-mundial-HC37247761</t>
+          <t>https://www.semana.com/politica/articulo/le-recuerdan-a-petro-cuando-usaba-la-camiseta-de-la-seleccion-colombia-en-la-campana-de-2022-lo-que-ahora-critica-cepeda/202628/</t>
         </is>
       </c>
     </row>
@@ -6820,17 +6784,17 @@
       </c>
       <c r="C245" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D245" s="6" t="inlineStr">
         <is>
-          <t>Falcao jugará el Mundial 2026 desde otra cancha: cambia los guayos por el micrófono</t>
+          <t>Primer funcionario del Gobierno le pidió públicamente a Gustavo Petro que renuncie a la Presidencia: “Victoria o muerte”</t>
         </is>
       </c>
       <c r="E245" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/mundial-2026/falcao-comentara-mundial-2026-con-espn-disney-HC37245354</t>
+          <t>https://www.semana.com/politica/articulo/primer-funcionario-del-gobierno-le-pidio-publicamente-a-gustavo-petro-que-renuncie-a-la-presidencia-victoria-o-muerte/202625/</t>
         </is>
       </c>
     </row>
@@ -6843,17 +6807,17 @@
       </c>
       <c r="C246" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D246" s="3" t="inlineStr">
         <is>
-          <t>¡Increíble! En Nariño, Antioquia, una vaca tuvo cuatrillizos; ocurre en menos del 1% de los partos</t>
+          <t>Miguel Uribe Londoño dice que “entramado criminal que tiene tomado el Gobierno de Gustavo Petro” está detrás del crimen de su hijo</t>
         </is>
       </c>
       <c r="E246" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/antioquia/vaca-narino-antioquia-tuvo-cuatrillizos-suceso-muy-raro-HC37245222</t>
+          <t>https://www.semana.com/semana-tv/semana-el-debate/articulo/miguel-uribe-londono-dice-que-entramado-criminal-que-tiene-tomado-el-gobierno-de-gustavo-petro-esta-detras-del-crimen-de-su-hijo/202645/</t>
         </is>
       </c>
     </row>
@@ -6866,17 +6830,17 @@
       </c>
       <c r="C247" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D247" s="6" t="inlineStr">
         <is>
-          <t>Más allá de la sequía: Procuraduría advierte impacto del fenómeno de El Niño en la comida, luz y agua del país</t>
+          <t>Imputan cargos a alcaldesa de Ibagué por presuntas irregularidades en contrato para compra de comida para animales de un centro de protección</t>
         </is>
       </c>
       <c r="E247" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/procuraduria-advierte-impacto-fenomeno-nino-comida-luz-agua-colombia-FF37238287</t>
+          <t>https://www.semana.com/nacion/armenia/articulo/imputan-cargos-a-alcaldesa-de-ibague-por-presuntas-irregularidades-en-contrato-para-compra-de-comida-para-animales-de-un-centro-de-proteccion/202642/</t>
         </is>
       </c>
     </row>
@@ -6889,17 +6853,17 @@
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D248" s="3" t="inlineStr">
         <is>
-          <t>Dibu Martínez en alerta: jugará el Mundial 2026 con una fractura en la mano</t>
+          <t>Hombre murió en plena vía pública en medio de las elecciones por esta prenda de vestir</t>
         </is>
       </c>
       <c r="E248" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/mundial-2026/dibu-martinez-fractura-mano-mundial-selecion-argentina-KC37243845</t>
+          <t>https://www.semana.com/nacion/articulo/hombre-murio-en-plena-via-publica-en-medio-de-las-elecciones-por-esta-prenda-de-vestir/202615/</t>
         </is>
       </c>
     </row>
@@ -6912,17 +6876,17 @@
       </c>
       <c r="C249" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D249" s="6" t="inlineStr">
         <is>
-          <t>DIM aún no termina el semestre: recibe a Cúcuta en Itagüí buscando los octavos de la Copa BetPlay</t>
+          <t>Barbosa redujo en un 82 % su deuda con acreedores y ejecuta obras de infraestructura por miles de millones de pesos</t>
         </is>
       </c>
       <c r="E249" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/deportes/futbol/dim-vs-cucuta-juego-copa-betplay-fase-de-grupos-clasificacion-octavos-de-final-AF37236464</t>
+          <t>https://www.semana.com/nacion/medellin/articulo/barbosa-redujo-en-un-82-su-deuda-con-acreedores-y-ejecuta-obras-de-infraestructura-por-miles-de-millones-de-pesos/202605/</t>
         </is>
       </c>
     </row>
@@ -6935,17 +6899,17 @@
       </c>
       <c r="C250" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D250" s="3" t="inlineStr">
         <is>
-          <t>Las películas y series que llegarán a Netflix, HBO Max, Prime Video y Apple TV en junio 2026</t>
+          <t>Cali busca posicionarse como referente global de transformación urbana en Cumbre de Ciudades en Singapur</t>
         </is>
       </c>
       <c r="E250" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/entretenimiento/television/estrenos-peliculas-series-netflix-hbo-prime-apple-tv-junio-2026-CE37224341</t>
+          <t>https://www.semana.com/nacion/cali/articulo/cali-busca-posicionarse-como-referente-global-de-transformacion-urbana-en-cumbre-de-ciudades-en-singapur/202633/</t>
         </is>
       </c>
     </row>
@@ -6958,206 +6922,22 @@
       </c>
       <c r="C251" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D251" s="6" t="inlineStr">
         <is>
-          <t>¿Cuál es el más fuerte de los 4 países debutantes en Norteamérica 2026?</t>
+          <t>Wendy Sepúlveda no resistió: murió la joven atacada con gasolina por su expareja en Neiva</t>
         </is>
       </c>
       <c r="E251" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/deportes/futbol/paises-debutantes-mundial-2026-uzbekistan-jordania-cabo-verde-curazao-BC37241527</t>
-        </is>
-      </c>
-    </row>
-    <row r="252">
-      <c r="A252" s="2" t="inlineStr"/>
-      <c r="B252" s="2" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C252" s="2" t="inlineStr">
-        <is>
-          <t>El Colombiano</t>
-        </is>
-      </c>
-      <c r="D252" s="3" t="inlineStr">
-        <is>
-          <t>Francia se convierte en aliado de Medellín para fortalecer el turismo sostenible, ¿cómo lo hará?</t>
-        </is>
-      </c>
-      <c r="E252" s="4" t="inlineStr">
-        <is>
-          <t>https://www.elcolombiano.com/medellin/alianza-con-francia-para-turismo-sostenible-medellin-antioquia-DC37241013</t>
-        </is>
-      </c>
-    </row>
-    <row r="253">
-      <c r="A253" s="5" t="inlineStr"/>
-      <c r="B253" s="5" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C253" s="5" t="inlineStr">
-        <is>
-          <t>El Colombiano</t>
-        </is>
-      </c>
-      <c r="D253" s="6" t="inlineStr">
-        <is>
-          <t>Venezuela rompe su récord exportador de petróleo desde las sanciones de 2019</t>
-        </is>
-      </c>
-      <c r="E253" s="7" t="inlineStr">
-        <is>
-          <t>https://www.elcolombiano.com/negocios/exportaciones-petroleo-venezuela-mayo-2026-pdvsa-colombia-HC37241240</t>
-        </is>
-      </c>
-    </row>
-    <row r="254">
-      <c r="A254" s="2" t="inlineStr"/>
-      <c r="B254" s="2" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C254" s="2" t="inlineStr">
-        <is>
-          <t>El Colombiano</t>
-        </is>
-      </c>
-      <c r="D254" s="3" t="inlineStr">
-        <is>
-          <t>Procurador Eljach controvierte a Petro por querer desconocer preconteo: “no hay evidencia o reclamaciones que resolver”</t>
-        </is>
-      </c>
-      <c r="E254" s="4" t="inlineStr">
-        <is>
-          <t>https://www.elcolombiano.com/colombia/procuraduria-gregorio-eljach-dice-que-no-hay-evidencia-de-fraude-DC37241075</t>
-        </is>
-      </c>
-    </row>
-    <row r="255">
-      <c r="A255" s="5" t="inlineStr"/>
-      <c r="B255" s="5" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C255" s="5" t="inlineStr">
-        <is>
-          <t>El Colombiano</t>
-        </is>
-      </c>
-      <c r="D255" s="6" t="inlineStr">
-        <is>
-          <t>En Antioquia se vendieron casi 25.000 carros nuevos en los primeros cinco meses de 2026</t>
-        </is>
-      </c>
-      <c r="E255" s="7" t="inlineStr">
-        <is>
-          <t>https://www.elcolombiano.com/negocios/venta-carros-nuevos-medellin-antioquia-2026-IF37239023</t>
-        </is>
-      </c>
-    </row>
-    <row r="256">
-      <c r="A256" s="2" t="inlineStr"/>
-      <c r="B256" s="2" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C256" s="2" t="inlineStr">
-        <is>
-          <t>El Colombiano</t>
-        </is>
-      </c>
-      <c r="D256" s="3" t="inlineStr">
-        <is>
-          <t>Descarga mortal en Doradal: un rayo acabó con 25 cabezas de ganado</t>
-        </is>
-      </c>
-      <c r="E256" s="4" t="inlineStr">
-        <is>
-          <t>https://www.elcolombiano.com/antioquia/descarga-mortal-doradal-rayo-acabo-25-cabezas-ganado-LF37238614</t>
-        </is>
-      </c>
-    </row>
-    <row r="257">
-      <c r="A257" s="5" t="inlineStr"/>
-      <c r="B257" s="5" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C257" s="5" t="inlineStr">
-        <is>
-          <t>El Colombiano</t>
-        </is>
-      </c>
-      <c r="D257" s="6" t="inlineStr">
-        <is>
-          <t>De la Espriella ganó hasta en Venezuela: así votaron los colombianos en el exterior en la primera vuelta presidencial</t>
-        </is>
-      </c>
-      <c r="E257" s="7" t="inlineStr">
-        <is>
-          <t>https://www.elcolombiano.com/internacional/resultados-elecciones-colombianos-exterior-primera-vuelta-2026-DF37236577</t>
-        </is>
-      </c>
-    </row>
-    <row r="258">
-      <c r="A258" s="2" t="inlineStr"/>
-      <c r="B258" s="2" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C258" s="2" t="inlineStr">
-        <is>
-          <t>El Colombiano</t>
-        </is>
-      </c>
-      <c r="D258" s="3" t="inlineStr">
-        <is>
-          <t>¿Quiénes ya anunciaron su apoyo para la segunda vuelta? Miguel Uribe Londoño y el Partido Conservador ya dijeron que se van con De la Espriella</t>
-        </is>
-      </c>
-      <c r="E258" s="4" t="inlineStr">
-        <is>
-          <t>https://www.elcolombiano.com/especiales/elecciones-2026/apoyo-miguel-uribe-londono-partido-conservador-de-la-espriella-EF37237113</t>
-        </is>
-      </c>
-    </row>
-    <row r="259">
-      <c r="A259" s="5" t="inlineStr"/>
-      <c r="B259" s="5" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C259" s="5" t="inlineStr">
-        <is>
-          <t>El Colombiano</t>
-        </is>
-      </c>
-      <c r="D259" s="6" t="inlineStr">
-        <is>
-          <t>Las propuestas económicas de Cepeda y De la Espriella que definirán la segunda vuelta presidencial en Colombia</t>
-        </is>
-      </c>
-      <c r="E259" s="7" t="inlineStr">
-        <is>
-          <t>https://www.elcolombiano.com/negocios/propuestas-economicas-cepeda-abelardo-segunda-vuelta-presidencia-DH37213734</t>
+          <t>https://www.semana.com/nacion/articulo/wendy-sepulveda-no-resistio-murio-la-joven-atacada-con-gasolina-por-su-expareja-en-neiva/202645/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E259"/>
+  <autoFilter ref="A1:E251"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
@@ -7409,14 +7189,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E249" r:id="rId248"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E250" r:id="rId249"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E251" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E252" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E253" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E254" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E255" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E256" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E257" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E258" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E259" r:id="rId258"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Noticias actualizadas 03/06/2026 09:09
</commit_message>
<xml_diff>
--- a/docs/ultimahora.xlsx
+++ b/docs/ultimahora.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Todas las noticias" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Todas las noticias'!$A$1:$E$279</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Todas las noticias'!$A$1:$E$276</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E279"/>
+  <dimension ref="A1:E276"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -515,7 +515,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 01:09 a. m.</t>
+          <t>03/06/2026 04:04 a. m.</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -530,19 +530,19 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Senadora Andrea Padilla denunció que MinAmbiente conocía desde hace un año la crisis de los 350 cocodrilos sin alimento; el Ministerio respondió</t>
+          <t>Movilidad en Bogotá miércoles 03 de junio: conozca acá el pico y placa en la ciudad</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/vida/medio-ambiente/senadora-andrea-padilla-denuncio-que-minambiente-conocia-desde-hace-un-ano-la-crisis-de-los-350-cocodrilos-sin-alimento-el-ministerio-respondio-3561665</t>
+          <t>https://www.eltiempo.com/bogota/movilidad-en-bogota-miercoles-03-de-junio-conozca-aca-el-pico-y-placa-en-la-ciudad-3561668</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 12:01 a. m.</t>
+          <t>03/06/2026 03:33 a. m.</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -557,19 +557,19 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>Murió Edgar Morin, referente mundial del pensamiento complejo</t>
+          <t>Vendaval, granizo y árboles caídos: la estela de destrucción que dejó fuerte tormenta en Cartago</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/contenido-comercial/murio-edgar-morin-referente-mundial-del-pensamiento-complejo-3561445</t>
+          <t>https://www.eltiempo.com/colombia/cali/vendaval-granizo-y-arboles-caidos-la-estela-de-destruccion-que-dejo-fuerte-tormenta-en-cartago-3561664</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 11:25 p. m.</t>
+          <t>03/06/2026 02:44 a. m.</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -584,19 +584,19 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Millonario monto que habría pedido familia de Valeria Afanador en conciliación previa a imputación por homicidio culposo: abogado de colegio dio cifra</t>
+          <t>República Democrática del Congo elevó a 344 los casos confirmados de ébola por brote del virus Bundibugyo: 60 personas han muerto</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/bogota/millonario-monto-que-habria-pedido-familia-de-valeria-afanador-en-conciliacion-previa-a-imputacion-por-homicidio-culposo-abogado-de-colegio-dio-cifra-3561662</t>
+          <t>https://www.eltiempo.com/mundo/africa/republica-democratica-del-congo-elevo-a-344-los-casos-confirmados-de-ebola-por-brote-del-virus-bundibugyo-60-personas-han-muerto-3561667</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 11:05 p. m.</t>
+          <t>03/06/2026 02:35 a. m.</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -611,19 +611,19 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Pasajero intentó abrir las puertas de un avión que cubría la ruta Puerto Rico-Chicago en pleno vuelo, lo que provocó aterrizaje de emergencia en Miami</t>
+          <t>¡Atención conductores! Pico y placa en Pereira para el miércoles 3 de junio de 2026: así regirá la medida</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/pasajero-intento-abrir-las-puertas-de-un-avion-que-cubria-la-ruta-puerto-rico-chicago-en-pleno-vuelo-y-provoco-aterrizaje-de-emergencia-en-miami-3561654</t>
+          <t>https://www.eltiempo.com/colombia/otras-ciudades/atencion-conductores-pico-y-placa-en-pereira-para-el-miercoles-3-de-junio-de-2026-asi-regira-la-medida-3561538</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 11:02 p. m.</t>
+          <t>03/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -638,19 +638,19 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Diego Arias piensa en la remontada de Nacional en la final contra Junior: ‘Lo importante es estar juntos en los momentos duros’</t>
+          <t>¡Ojo, conductor! Pico y placa en Bucaramanga para el miércoles 3 de junio de 2026</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-colombiano/diego-arias-piensa-en-la-remontada-de-nacional-en-la-final-contra-junior-lo-importante-es-estar-juntos-en-los-momentos-duros-3561663</t>
+          <t>https://www.eltiempo.com/colombia/santander/ojo-conductor-pico-y-placa-en-bucaramanga-para-el-miercoles-3-de-junio-de-3561540</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 10:55 p. m.</t>
+          <t>03/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -665,19 +665,19 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Atlético Nacional mereció la goleada que se llevó en la ida de la final contra Junior: calificaciones individuales</t>
+          <t>¡Siga la medida de movilidad! Pico y placa en Medellín para el miércoles 3 de junio de 2026: así funciona la restricción</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-colombiano/atletico-nacional-merecio-la-goleada-que-se-llevo-en-la-ida-de-la-final-contra-junior-calificaciones-individuales-3561661</t>
+          <t>https://www.eltiempo.com/colombia/medellin/siga-la-medida-de-movilidad-pico-y-placa-en-medellin-para-el-miercoles-3-de-junio-de-2026-asi-funciona-la-restriccion-3561535</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 10:52 p. m.</t>
+          <t>03/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -692,19 +692,19 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Abelardo de la Espriella agradeció la felicitación del presidente Donald Trump por triunfo en la primera vuelta electoral: 'Estoy muy honrado'</t>
+          <t>¡Evite multas! Pico y placa en Cali para el miércoles 3 de junio de 2026: así opera la medida</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/abelardo-de-la-espriella-agradecio-la-felicitacion-y-apoyo-del-presidente-donald-trump-a-su-campana-estoy-muy-honrado-3561660</t>
+          <t>https://www.eltiempo.com/colombia/cali/evite-multas-pico-y-placa-en-cali-para-el-miercoles-3-de-junio-de-2026-asi-opera-la-medida-3561529</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 10:41 p. m.</t>
+          <t>03/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -719,19 +719,19 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Chavismo inaugura 'club para abuelos', con peluquería y centro médico, en casa expropiada al opositor Leopoldo López en Venezuela</t>
+          <t>¡Pilas en las vías! Pico y placa en Bogotá para el miércoles 3 de junio de 2026</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/venezuela/chavismo-inaugura-club-para-abuelos-con-peluqueria-y-centro-medico-en-casa-expropiada-al-opositor-leopoldo-lopez-en-venezuela-3561525</t>
+          <t>https://www.eltiempo.com/bogota/pilas-en-las-vias-pico-y-placa-en-bogota-para-el-miercoles-3-de-junio-de-3561528</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 10:39 p. m.</t>
+          <t>03/06/2026 02:08 a. m.</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -746,19 +746,19 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Luis Fernando Muriel, el mejor de Junior en el primer asalto de la final: calificaciones individuales</t>
+          <t>Ministerio de Defensa aseguró que nunca solicitó a Estados Unidos sanciones financieras al oro colombiano ni su inclusión en una 'lista negra'</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-colombiano/luis-fernando-muriel-el-mejor-de-junior-en-el-primer-asalto-de-la-final-calificaciones-individuales-3561659</t>
+          <t>https://www.eltiempo.com/politica/gobierno/ministerio-de-defensa-aseguro-que-nunca-solicito-a-estados-unidos-sanciones-financieras-al-oro-colombiano-ni-su-inclusion-en-una-lista-negra-3561666</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 10:37 p. m.</t>
+          <t>03/06/2026 01:09 a. m.</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -773,19 +773,19 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Más de 600 familias campesinas de Montelíbano (Córdoba) reciben 1.254 hectáreas tras más de tres décadas de espera</t>
+          <t>Senadora Andrea Padilla denunció que MinAmbiente conocía desde hace un año la crisis de los 350 cocodrilos sin alimento; el Ministerio respondió</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/otras-ciudades/mas-de-600-familias-campesinas-de-montelibano-cordoba-reciben-1-254-hectareas-tras-mas-de-tres-decadas-de-espera-3561658</t>
+          <t>https://www.eltiempo.com/vida/medio-ambiente/senadora-andrea-padilla-denuncio-que-minambiente-conocia-desde-hace-un-ano-la-crisis-de-los-350-cocodrilos-sin-alimento-el-ministerio-respondio-3561665</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 10:34 p. m.</t>
+          <t>03/06/2026 12:01 a. m.</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -800,19 +800,19 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Las marcas colombianas se 'pusieron la 10' y lanzaron prendas para apoyar a la Selección con estilo: véalas y anímese a crear su outfit futbolero</t>
+          <t>Murió Edgar Morin, referente mundial del pensamiento complejo</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/vida/tendencias/las-marcas-colombianas-se-pusieron-la-10-y-lanzaron-prendas-para-apoyar-a-la-seleccion-con-estilo-vealas-y-animese-a-crear-su-outfit-futbolero-3561578</t>
+          <t>https://www.eltiempo.com/contenido-comercial/murio-edgar-morin-referente-mundial-del-pensamiento-complejo-3561445</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 10:30 p. m.</t>
+          <t>02/06/2026 11:25 p. m.</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -827,19 +827,19 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>¿Podrá por fin Keiko Fujimori ganar la presidencia en Perú y consolidar el giro a la derecha en América Latina? / Análisis de Mauricio Vargas</t>
+          <t>Millonario monto que habría pedido familia de Valeria Afanador en conciliación previa a imputación por homicidio culposo: abogado de colegio dio cifra</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/latinoamerica/podra-por-fin-keiko-fujimori-ganar-la-presidencia-en-peru-y-consolidar-el-giro-a-la-derecha-en-america-latina-analisis-de-mauricio-vargas-3561595</t>
+          <t>https://www.eltiempo.com/bogota/millonario-monto-que-habria-pedido-familia-de-valeria-afanador-en-conciliacion-previa-a-imputacion-por-homicidio-culposo-abogado-de-colegio-dio-cifra-3561662</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 10:24 p. m.</t>
+          <t>02/06/2026 11:05 p. m.</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -854,19 +854,19 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Junior de Barranquilla, con un panorama favorable para el bicampeonato: nunca se ha remontado una ventaja de tres goles en una final</t>
+          <t>Pasajero intentó abrir las puertas de un avión que cubría la ruta Puerto Rico-Chicago en pleno vuelo, lo que provocó aterrizaje de emergencia en Miami</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-colombiano/junior-de-barranquilla-con-un-panorama-favorable-para-el-bicampeonato-nunca-se-ha-remontado-una-ventaja-de-tres-goles-en-una-final-3561657</t>
+          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/pasajero-intento-abrir-las-puertas-de-un-avion-que-cubria-la-ruta-puerto-rico-chicago-en-pleno-vuelo-y-provoco-aterrizaje-de-emergencia-en-miami-3561654</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 10:20 p. m.</t>
+          <t>02/06/2026 11:02 p. m.</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -881,19 +881,19 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Luis Fernando Muriel, la figura en la ida de la final, se ilusiona con la estrella para Junior: 'Todo nos salió a pedir de boca'</t>
+          <t>Diego Arias piensa en la remontada de Nacional en la final contra Junior: ‘Lo importante es estar juntos en los momentos duros’</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-colombiano/luis-fernando-muriel-la-figura-en-la-ida-de-la-final-se-ilusiona-con-la-estrella-para-junior-todo-nos-salio-a-pedir-de-boca-3561656</t>
+          <t>https://www.eltiempo.com/deportes/futbol-colombiano/diego-arias-piensa-en-la-remontada-de-nacional-en-la-final-contra-junior-lo-importante-es-estar-juntos-en-los-momentos-duros-3561663</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 10:13 p. m.</t>
+          <t>02/06/2026 10:55 p. m.</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -908,19 +908,19 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Las 10 razones por las que el sistema electoral colombiano demostró un sólido funcionamiento en la primera vuelta del 31 de mayo</t>
+          <t>Atlético Nacional mereció la goleada que se llevó en la ida de la final contra Junior: calificaciones individuales</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/las-10-razones-por-las-que-el-sistema-electoral-colombiano-demostro-un-solido-funcionamiento-en-la-primera-vuelta-del-31-de-mayo-3561653</t>
+          <t>https://www.eltiempo.com/deportes/futbol-colombiano/atletico-nacional-merecio-la-goleada-que-se-llevo-en-la-ida-de-la-final-contra-junior-calificaciones-individuales-3561661</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 10:01 p. m.</t>
+          <t>02/06/2026 10:52 p. m.</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -935,19 +935,19 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>Desprotección rampante</t>
+          <t>Abelardo de la Espriella agradeció la felicitación del presidente Donald Trump por triunfo en la primera vuelta electoral: 'Estoy muy honrado'</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/caricaturas/desproteccion-rampante-3561632</t>
+          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/abelardo-de-la-espriella-agradecio-la-felicitacion-y-apoyo-del-presidente-donald-trump-a-su-campana-estoy-muy-honrado-3561660</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 10:01 p. m.</t>
+          <t>02/06/2026 10:41 p. m.</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -962,19 +962,19 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Experiencia</t>
+          <t>Chavismo inaugura 'club para abuelos', con peluquería y centro médico, en casa expropiada al opositor Leopoldo López en Venezuela</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/caricaturas/experiencia-3561631</t>
+          <t>https://www.eltiempo.com/mundo/venezuela/chavismo-inaugura-club-para-abuelos-con-peluqueria-y-centro-medico-en-casa-expropiada-al-opositor-leopoldo-lopez-en-venezuela-3561525</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 10:01 p. m.</t>
+          <t>02/06/2026 10:39 p. m.</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -989,19 +989,19 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Solitario mensaje</t>
+          <t>Luis Fernando Muriel, el mejor de Junior en el primer asalto de la final: calificaciones individuales</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/caricaturas/solitario-mensaje-3561630</t>
+          <t>https://www.eltiempo.com/deportes/futbol-colombiano/luis-fernando-muriel-el-mejor-de-junior-en-el-primer-asalto-de-la-final-calificaciones-individuales-3561659</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 10:01 p. m.</t>
+          <t>02/06/2026 10:37 p. m.</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1016,19 +1016,19 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Legítimas y transparentes</t>
+          <t>Más de 600 familias campesinas de Montelíbano (Córdoba) reciben 1.254 hectáreas tras más de tres décadas de espera</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/editorial/legitimas-y-transparentes-3561627</t>
+          <t>https://www.eltiempo.com/colombia/otras-ciudades/mas-de-600-familias-campesinas-de-montelibano-cordoba-reciben-1-254-hectareas-tras-mas-de-tres-decadas-de-espera-3561658</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 10:01 p. m.</t>
+          <t>02/06/2026 10:34 p. m.</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
@@ -1043,19 +1043,19 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>El Ejército está de luto</t>
+          <t>Las marcas colombianas se 'pusieron la 10' y lanzaron prendas para apoyar a la Selección con estilo: véalas y anímese a crear su outfit futbolero</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/cartas/el-ejercito-esta-de-luto-3561616</t>
+          <t>https://www.eltiempo.com/vida/tendencias/las-marcas-colombianas-se-pusieron-la-10-y-lanzaron-prendas-para-apoyar-a-la-seleccion-con-estilo-vealas-y-animese-a-crear-su-outfit-futbolero-3561578</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 03:04 a. m.</t>
+          <t>03/06/2026 09:05 a. m.</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1070,19 +1070,19 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Un militar muerto y otro herido tras ataque con dron en el Catatumbo</t>
+          <t>Registraduría responde a Petro y aclara información sobre el proceso electoral</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/orden-publico/un-militar-muerto-y-otro-herido-tras-ataque-con-dron-en-el-catatumbo-401206</t>
+          <t>https://www.lafm.com.co/actualidad/registraduria-responde-a-petro-y-aclara-informacion-sobre-el-proceso-electoral-401208</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 02:20 a. m.</t>
+          <t>03/06/2026 02:37 a. m.</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -1097,19 +1097,19 @@
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Último sorteo de la Lotería de la Cruz Roja: resultado premio mayor hoy 2 de junio</t>
+          <t>Experto advierte que denuncias de Petro sobre supuesto fraude podrían favorecer a Abelardo de la Espriella</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/sociedad/ultimo-sorteo-de-la-loteria-de-la-cruz-roja-resultado-premio-mayor-hoy-2-de-junio-401201</t>
+          <t>https://www.lafm.com.co/politica/petro-denuncia-fraude-electoral-favorece-aberlado-de-la-espriella-segunda-vuelta-401203</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 01:54 a. m.</t>
+          <t>03/06/2026 02:20 a. m.</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1124,19 +1124,19 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Abelardo de la Espriella prometió relacionarse con EEUU "como nunca antes" tras apoyo de Trump</t>
+          <t>Último sorteo de la Lotería de la Cruz Roja: resultado premio mayor hoy 2 de junio</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/abelardo-de-la-espriella-promete-relacion-historica-colombia-eeuu-tras-respaldo-trump-401199</t>
+          <t>https://www.lafm.com.co/sociedad/ultimo-sorteo-de-la-loteria-de-la-cruz-roja-resultado-premio-mayor-hoy-2-de-junio-401201</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 12:42 a. m.</t>
+          <t>03/06/2026 01:54 a. m.</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
@@ -1151,19 +1151,19 @@
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>¿Qué está pasando con el volcán Puracé y por qué preocupa a las autoridades?</t>
+          <t>Abelardo de la Espriella prometió relacionarse con EEUU "como nunca antes" tras apoyo de Trump</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/actualidad/volcan-purace-ceniza-creciente-alerta-amarilla-sintomas-respiratorios-401197</t>
+          <t>https://www.lafm.com.co/politica/abelardo-de-la-espriella-promete-relacion-historica-colombia-eeuu-tras-respaldo-trump-401199</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 12:26 a. m.</t>
+          <t>03/06/2026 12:42 a. m.</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1178,19 +1178,19 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>¿Quién es el empresario de Before club que dijo que había que “fumigar” a Abelardo de la Espriella?</t>
+          <t>¿Qué está pasando con el volcán Puracé y por qué preocupa a las autoridades?</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/actualidad/before-club-dueno-frase-contra-abelardo-de-la-espriella-relacion-protestas-bogota-401193</t>
+          <t>https://www.lafm.com.co/actualidad/volcan-purace-ceniza-creciente-alerta-amarilla-sintomas-respiratorios-401197</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 12:04 a. m.</t>
+          <t>03/06/2026 12:26 a. m.</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -1205,19 +1205,19 @@
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>Junior Goleó a Nacional entre el humo y la fiesta; se define todo en Medellín</t>
+          <t>¿Quién es el empresario de Before club que dijo que había que “fumigar” a Abelardo de la Espriella?</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/deportes/liga-betplay-final-ida-junior-nacional-goles-resultados-401191</t>
+          <t>https://www.lafm.com.co/actualidad/before-club-dueno-frase-contra-abelardo-de-la-espriella-relacion-protestas-bogota-401193</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 11:24 p. m.</t>
+          <t>03/06/2026 12:04 a. m.</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1232,19 +1232,19 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Junior goleó a Atlético Nacional por la ida de la final de la Liga Betplay 2026-I</t>
+          <t>Junior Goleó a Nacional entre el humo y la fiesta; se define todo en Medellín</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/deportes/final-liga-betplay-2026-junior-vs-nacional-fpc-401187</t>
+          <t>https://www.lafm.com.co/deportes/liga-betplay-final-ida-junior-nacional-goles-resultados-401191</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 11:05 p. m.</t>
+          <t>02/06/2026 11:24 p. m.</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -1259,12 +1259,12 @@
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>¿El voto en blanco favorece al candidato ganador? Expertos aclaran el mito que vuelve en cada elección</t>
+          <t>Junior goleó a Atlético Nacional por la ida de la final de la Liga Betplay 2026-I</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/voto-en-blanco-ayuda-al-ganador-mito-expertos-aclaran-verdad-elecciones-colombia-2026-401183</t>
+          <t>https://www.lafm.com.co/deportes/final-liga-betplay-2026-junior-vs-nacional-fpc-401187</t>
         </is>
       </c>
     </row>
@@ -1298,7 +1298,7 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 10:04 p. m.</t>
+          <t>01/06/2026 06:29 p. m.</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -1313,19 +1313,19 @@
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Asesinato de la patrullera Karen Pajoy: así fue la captura de los disidentes que cometieron el crimen</t>
+          <t>MinDefensa le responde al New York Times y niega haber pedido sanciones contra el oro colombiano</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/orden-publico/policia-captura-disidentes-asesinato-patrullera-karen-pajoy-huila-401177</t>
+          <t>https://www.lafm.com.co/orden-publico/mindefensa-respuesta-niega-pedir-sanciones-contra-oro-colombiano-401194</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 06:29 p. m.</t>
+          <t>01/06/2026 02:00 p. m.</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1340,12 +1340,12 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>MinDefensa le responde al New York Times y niega haber pedido sanciones contra el oro colombiano</t>
+          <t>De la Espriella pedirá a EE. UU. investigar presunto plan del petrismo para compra de votos</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/orden-publico/mindefensa-respuesta-niega-pedir-sanciones-contra-oro-colombiano-401194</t>
+          <t>https://www.lafm.com.co/politica/de-la-espriella-pedira-a-ee-uu-investigar-presunto-plan-del-petrismo-para-compra-de-votos-401207</t>
         </is>
       </c>
     </row>
@@ -1379,7 +1379,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>20/05/2026 02:29 p. m.</t>
+          <t>06/05/2026 12:08 a. m.</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1394,19 +1394,19 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>“Los votos no son de dirigentes, son de ciudadanos libres”: Fajardo dice que entregará decálogo con sus propuestas</t>
+          <t>Caso Lili Pink: Fiscalía anunció imputación de cargos contra ocho personas</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/sergio-fajardo-mensaje-de-la-espriella-ivan-cepeda-propuestas-segunda-vuelta-presidencial-401180</t>
+          <t>https://www.lafm.com.co/orden-publico/lili-pink-imputados-delitos-contrabando-robo-401188</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>06/05/2026 12:08 a. m.</t>
+          <t>10/02/2026 06:47 p. m.</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
@@ -1421,19 +1421,19 @@
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>Caso Lili Pink: Fiscalía anunció imputación de cargos contra ocho personas</t>
+          <t>“Parece una masacre”: Defensora del Pueblo sobre muerte de 11 menores en Guaviare</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/orden-publico/lili-pink-imputados-delitos-contrabando-robo-401188</t>
+          <t>https://www.lafm.com.co/orden-publico/parece-una-masacre-defensora-del-pueblo-sobre-muerte-de-11-menores-en-guaviare-401200</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>28/02/2026 12:08 p. m.</t>
+          <t>10/02/2026 03:03 p. m.</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1448,12 +1448,12 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Presidente Petro responde ante "respaldo" de Trump a De la Espriella</t>
+          <t>Denuncian desplazamiento de decenas de campesinos en El Tarra, Norte de Santander</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/presidente-petro-responde-ante-respaldo-de-trump-a-de-la-espriella-401205</t>
+          <t>https://www.lafm.com.co/orden-publico/denuncian-desplazamiento-de-decenas-de-campesinos-en-el-tarra-norte-de-santander-401202</t>
         </is>
       </c>
     </row>
@@ -1498,12 +1498,12 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Experto advierte que denuncias de Petro sobre supuesto fraude podrían favorecer a Abelardo de la Espriella</t>
+          <t>Un militar muerto y otro herido tras ataque con dron en el Catatumbo</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/petro-denuncia-fraude-electoral-favorece-aberlado-de-la-espriella-segunda-vuelta-401203</t>
+          <t>https://www.lafm.com.co/orden-publico/un-militar-muerto-y-otro-herido-tras-ataque-con-dron-en-el-catatumbo-401206</t>
         </is>
       </c>
     </row>
@@ -1521,12 +1521,12 @@
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>“Parece una masacre”: Defensora del Pueblo sobre muerte de 11 menores en Guaviare</t>
+          <t>Presidente Petro responde ante "respaldo" de Trump a De la Espriella</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/orden-publico/parece-una-masacre-defensora-del-pueblo-sobre-muerte-de-11-menores-en-guaviare-401200</t>
+          <t>https://www.lafm.com.co/politica/presidente-petro-responde-ante-respaldo-de-trump-a-de-la-espriella-401205</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 02:00 a. m.</t>
+          <t>03/06/2026 07:29 a. m.</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -1589,24 +1589,24 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>La OCDE advierte de que algunas economías entrarán en recesión si el bloqueo del estrecho de Ormuz se prolonga</t>
+          <t>Bus de la Selección Colombia quedó rodeado por manifestantes en marcha en Bogotá</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/economia/2026-06-03/la-ocde-advierte-de-que-algunas-economias-entraran-en-recesion-si-el-bloqueo-del-estrecho-de-ormuz-se-prolonga.html</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/02/bus-de-la-seleccion-colombia-quedo-rodeado-por-manifestantes-en-marcha-en-bogota/</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 01:49 a. m.</t>
+          <t>03/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
@@ -1616,24 +1616,24 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>El centenar de vecinos desalojados por el incendio en un municipio de Murcia regresa a sus casas</t>
+          <t>Catastrófica deforestación en el Día Internacional de los Bosques</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/espana/2026-06-03/el-centenar-de-vecinos-desalojados-por-el-incendio-en-un-municipio-de-murcia-regresa-a-sus-casas.html</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/03/catastrofica-deforestacion-en-el-dia-internacional-de-los-bosques/</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 01:37 a. m.</t>
+          <t>03/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -1643,24 +1643,24 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Al menos siete muertos en un ataque de Ucrania contra un autobús en la zona ocupada por Rusia</t>
+          <t>Columnistas</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/internacional/2026-06-03/al-menos-siete-muertos-en-un-ataque-de-ucrania-contra-un-autobus-en-la-zona-ocupada-por-rusia.html</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 12:37 a. m.</t>
+          <t>03/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
@@ -1670,24 +1670,24 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>La guerra de Estados Unidos e Israel contra Irán, en directo | Irán y EE UU intercambian nuevos ataques mientras las negociaciones siguen estancadas</t>
+          <t>Cuando la fiesta termina en tragedia</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/internacional/2026-06-03/la-guerra-de-estados-unidos-e-israel-contra-iran-en-directo.html</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/03/cuando-la-fiesta-termina-en-tragedia/</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 12:25 a. m.</t>
+          <t>03/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -1697,24 +1697,24 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>He probado los mejores ventiladores de techo inteligentes para el hogar, y te presento mi elección para este verano</t>
+          <t>Cuando toca, ¡toca!</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/hemeroteca/2026-06-03/</t>
+          <t>https://www.vanguardia.com/opinion/caricaturas/2026/06/03/cuando-toca-toca/</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 11:41 p. m.</t>
+          <t>03/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
@@ -1724,24 +1724,24 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>Abelardo de la Espriella endurece su discurso contra la izquierda: “No creo que haya empalme con esos bandidos”</t>
+          <t>Caricaturas</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/america-colombia/elecciones-presidenciales/2026-06-03/abelardo-de-la-espriella-refuerza-su-bandera-contra-la-izquierda-no-creo-que-haya-empalme-con-esos-bandidos.html</t>
+          <t>https://www.vanguardia.com/opinion/caricaturas/</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 11:37 p. m.</t>
+          <t>03/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -1751,24 +1751,24 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Becerra y Hilton toman ventaja en la carrera por la gubernatura de California rumbo a una segunda vuelta</t>
+          <t>UIS: excelencia académica y liderazgo nacional, fruto de una apuesta por la formación integral</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/us/2026-06-03/becerra-y-hilton-toman-ventaja-en-la-carrera-por-la-gubernatura-de-california-rumbo-a-una-segunda-vuelta.html</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/03/uis-excelencia-academica-y-liderazgo-nacional-fruto-de-una-apuesta-por-la-formacion-integral/</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 11:00 p. m.</t>
+          <t>02/06/2026 10:30 p. m.</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
@@ -1778,24 +1778,24 @@
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>El cándido presidente candidato</t>
+          <t>Tragedia en Guaviare: 11 adolescentes asesinados en combates entre alias ‘Iván Mordisco’ y ‘Calarcá’</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/america-colombia/elecciones-presidenciales/2026-06-03/el-candido-presidente-candidato.html</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/02/tragedia-en-guaviare-11-adolescentes-asesinados-en-combates-entre-alias-ivan-mordisco-y-calarca/</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 11:00 p. m.</t>
+          <t>02/06/2026 10:30 p. m.</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -1805,24 +1805,24 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>En Perú la impunidad ya es ley</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/america/2026-06-03/en-peru-la-impunidad-ya-es-ley.html</t>
+          <t>https://www.vanguardia.com/colombia/</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 11:00 p. m.</t>
+          <t>02/06/2026 07:09 p. m.</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
@@ -1832,24 +1832,24 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>Andrea Repetto sobre la megarreforma de Kast: “Es cara, con costos claros y beneficios inciertos”</t>
+          <t>En directo: Petro entrega balance sobre la erradición de cultivos de coca durante su gobierno</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/chile/2026-06-03/andrea-repetto-sobre-la-megarreforma-de-kast-es-cara-con-costos-claros-y-beneficios-inciertos.html</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/02/en-directo-el-presidente-petro-habla-sobre-los-resultados-de-la-primera-vuelta/</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 11:00 p. m.</t>
+          <t>02/06/2026 05:14 p. m.</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -1859,24 +1859,24 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>El referente latinoamericano de justicia: el Acuerdo de Escazú</t>
+          <t>¿Renunciará Petro para hacer campaña? Esto respondió su jefe de gabinete</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/america-futura/2026-06-03/el-referente-latinoamericano-de-justicia-el-acuerdo-de-escazu.html</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/02/renunciara-petro-para-hacer-campana-esto-respondio-su-jefe-de-gabinete/</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 11:00 p. m.</t>
+          <t>02/06/2026 04:27 p. m.</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
@@ -1886,24 +1886,24 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>Cuando la ley no basta: objeción de conciencia y acceso al aborto en Chile</t>
+          <t>Derecho de preferencia notarial en Colombia: ¿Es aplicable sin ley?</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/chile/2026-06-03/cuando-la-ley-no-basta-objecion-de-conciencia-y-acceso-al-aborto-en-chile.html</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/02/derecho-de-preferencia-notarial-en-colombia-es-aplicable-sin-ley/</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 11:00 p. m.</t>
+          <t>02/06/2026 03:56 p. m.</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -1913,24 +1913,24 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>Quiénes son los beneficiados con el bono de 30.000 pesos por hijo anunciado por Kast</t>
+          <t>Ataques contra periodistas se dispararon 227 % durante las elecciones presidenciales</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/chile/2026-06-03/quienes-son-los-beneficiados-con-el-bono-de-30000-pesos-por-hijo-anunciado-por-kast.html</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/02/ataques-contra-periodistas-se-dispararon-227-durante-las-elecciones-presidenciales/</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 11:00 p. m.</t>
+          <t>02/06/2026 03:16 p. m.</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
@@ -1940,24 +1940,24 @@
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>Educación parvularia: el nivel (nuevamente) olvidado</t>
+          <t>Empresario arremete contra Abelardo De la Espriella: “lo vamos a fumigar”</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/chile/2026-06-03/educacion-parvularia-el-nivel-nuevamente-olvidado.html</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/02/empresario-arremete-contra-abelardo-de-la-espriella-lo-vamos-a-fumigar/</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 11:00 p. m.</t>
+          <t>02/06/2026 10:57 a. m.</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -1967,24 +1967,24 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>La Feira Preta de Brasil, un faro para los emprendedores negros de Latinoamérica</t>
+          <t>Mujer fue detenida en Cartagena por intentar sacar a su hijo con permiso falso</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/america-futura/2026-06-03/la-feira-preta-de-brasil-un-faro-para-los-emprendedores-negros-de-latinoamerica.html</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/02/mujer-fue-detenida-en-cartagena-por-intentar-sacar-a-su-hijo-con-permiso-falso/</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 11:00 p. m.</t>
+          <t>02/06/2026 10:22 a. m.</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
@@ -1994,26 +1994,22 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>El liderazgo opositor en el exilio empieza a volver a Venezuela</t>
+          <t>Procuraduría suspende a Alfredo Saade, embajador en Brasil, por mensajes políticos en campaña</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/america/2026-06-03/el-liderazgo-opositor-en-el-exilio-empieza-a-volver-a-venezuela.html</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/02/procuraduria-suspende-a-embajador-en-brasil-por-mensajes-politicos-en-campana/</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>02/06/2026 11:00 p. m.</t>
-        </is>
-      </c>
+      <c r="A58" s="2" t="inlineStr"/>
       <c r="B58" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2021,24 +2017,24 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Racistas a la cárcel: claves que colocan a Brasil a la vanguardia de la lucha contra la discriminación racial</t>
+          <t>Cerrejón suspende operaciones en La Guajira: más de 12.000 trabajadores afectados</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/america/2026-06-03/racistas-a-la-carcel-claves-que-colocan-a-brasil-a-la-vanguardia-de-la-lucha-contra-la-discriminacion-racial.html</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/01/cerrejon-suspende-operaciones-en-la-guajira-mas-de-12000-trabajadores-afectados/</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 11:00 p. m.</t>
+          <t>03/06/2026 04:03 a. m.</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
@@ -2053,19 +2049,19 @@
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>Colombia, más allá de víctimas y victimarios (I)</t>
+          <t>Al menos 21 muertos en un incendio en un hotel en la India, entre ellos varios extranjeros</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/america-colombia/elecciones-presidenciales/2026-06-03/colombia-mas-alla-de-victimas-y-victimarios-i.html</t>
+          <t>https://elpais.com/internacional/2026-06-03/al-menos-21-muertos-en-un-incendio-en-un-hotel-en-la-india-entre-ellos-varios-extranjeros.html</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 11:00 p. m.</t>
+          <t>03/06/2026 03:59 a. m.</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -2080,19 +2076,19 @@
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Cepeda, más allá de la frontera del petrismo</t>
+          <t>El que tenen en comú Kapwani Kiwanga i Joan Miró</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/america-colombia/elecciones-presidenciales/2026-06-03/cepeda-mas-alla-de-la-frontera-del-petrismo.html</t>
+          <t>https://elpais.com/quadern/art-i-arquitectura/2026-06-03/el-que-tenen-en-comu-kapwani-kiwanga-i-joan-miro.html</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 11:00 p. m.</t>
+          <t>03/06/2026 03:58 a. m.</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
@@ -2107,19 +2103,19 @@
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>La abstención y sus 17,5 millones de votantes que no fueron a las urnas envían un mensaje</t>
+          <t>Illa defiende en el Parlament la respuesta del partido ante las causas del PSOE: “Ojalá todos hicieran como nosotros”</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/america-colombia/elecciones-presidenciales/2026-06-03/la-abstencion-y-sus-175-millones-de-votantes-que-no-fueron-a-las-urnas-envian-un-mensaje.html</t>
+          <t>https://elpais.com/espana/catalunya/2026-06-03/illa-defiende-en-el-parlament-la-respuesta-del-partido-ante-las-causas-del-psoe-ojala-todos-hicieran-como-nosotros.html</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 10:48 p. m.</t>
+          <t>03/06/2026 03:53 a. m.</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -2134,19 +2130,19 @@
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Un sindicato policial apoya a la profesora “golpeada y humillada” en Valencia que sufrió una “violencia injustificada”</t>
+          <t>Kendall Jenner y Jacob Elordi, las pistas del romance del que todo Hollywood murmura</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/espana/comunidad-valenciana/2026-06-03/un-sindicato-policial-apoya-a-la-profesora-golpeada-y-humillada-en-valencia-que-que-sufrio-una-violencia-injustificada.html</t>
+          <t>https://elpais.com/gente/2026-06-03/kendall-jenner-y-jacob-elordi-las-pistas-del-romance-del-que-todo-hollywood-murmura.html</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 10:45 p. m.</t>
+          <t>03/06/2026 03:51 a. m.</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
@@ -2161,19 +2157,19 @@
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
-          <t>Inés Hernand sobre la polémica con Bad Bunny: “Se arma tanto revuelo porque es el lugar político de los más jóvenes”</t>
+          <t>Cinco agentes forales de Navarra mueren en un accidente de tráfico en Gipuzkoa</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/podcasts/hoy-en-el-pais/2026-06-03/ines-hernand-sobre-la-casita-de-bad-bunny-le-tenian-muchas-ganas.html</t>
+          <t>https://elpais.com/espana/2026-06-03/cinco-agentes-forales-de-navarra-mueren-en-un-accidente-de-trafico-en-gipuzkoa.html</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 10:30 p. m.</t>
+          <t>03/06/2026 03:44 a. m.</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -2188,19 +2184,19 @@
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>El Gobierno ve imposible la moción  de censura por el rechazo en Cataluña y Euskadi al PP y Vox</t>
+          <t>Raúl Rabadán rechazó dirigir el CNIO por la “politización” y la “falta de estabilidad” del organismo</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/espana/2026-06-03/el-gobierno-ve-imposible-la-mocion-de-censura-por-el-rechazo-en-cataluna-y-euskadi-al-pp-y-vox.html</t>
+          <t>https://elpais.com/ciencia/2026-06-03/raul-rabadan-rechazo-dirigir-el-cnio-por-la-politizacion-y-la-falta-de-estabilidad-del-organismo.html</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 10:30 p. m.</t>
+          <t>03/06/2026 03:38 a. m.</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
@@ -2215,19 +2211,19 @@
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>Rusia intensifica los ataques contra Ucrania y sus amenazas a Europa: “Su pacífico sueño ha terminado”</t>
+          <t>Meliá también cede ante la presión de Trump y abandona la gestión de 15 hoteles en Cuba</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/internacional/2026-06-03/rusia-intensifica-los-ataques-contra-ucrania-y-sus-amenazas-a-europa-su-pacifico-sueno-ha-terminado.html</t>
+          <t>https://elpais.com/economia/2026-06-03/melia-tambien-cede-ante-la-presion-de-trump-y-abandona-la-gestion-de-15-hoteles-en-cuba.html</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 10:30 p. m.</t>
+          <t>03/06/2026 03:35 a. m.</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -2242,19 +2238,19 @@
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Las prisas cambian de bando en Irán: Trump busca una salida a la guerra con el tiempo en su contra</t>
+          <t>La jueza investiga ahora si hay “terceras personas” involucradas en la muerte de Isak Andic</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/internacional/2026-06-03/las-prisas-cambian-de-bando-en-iran-trump-busca-una-salida-a-la-guerra-con-el-tiempo-en-su-contra.html</t>
+          <t>https://elpais.com/espana/catalunya/2026-06-03/la-jueza-investiga-ahora-si-hay-terceras-personas-involucradas-en-la-muerte-de-isak-andic.html</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 10:30 p. m.</t>
+          <t>03/06/2026 03:31 a. m.</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr">
@@ -2269,19 +2265,19 @@
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>Del ‘nanopinganillo’ a la grabación: así se caza a los copiones en la Selectividad</t>
+          <t>Manel del Castillo propone reformar el estado del bienestar para evitar su colapso</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/educacion/2026-06-03/del-nanopinganillo-a-la-grabacion-asi-se-caza-a-los-copiones-en-la-selectividad.html</t>
+          <t>https://elpais.com/espana/catalunya/2026-06-03/manel-del-castillo-propone-reformar-el-estado-del-bienestar-para-evitar-su-colapso.html</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 10:30 p. m.</t>
+          <t>03/06/2026 03:29 a. m.</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -2296,19 +2292,19 @@
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>Marc Giró: “No estamos para equidistancias, soy radicalmente de izquierdas y antifascista, ¿existe esta transparencia con otros presentadores?”</t>
+          <t>El juez pospone la citación de Begoña Gómez al 15 de junio</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/television/2026-06-03/marc-giro-no-estamos-para-equidistancias-soy-radicalmente-de-izquierdas-y-antifascista-existe-esta-transparencia-con-otros-presentadores.html</t>
+          <t>https://elpais.com/espana/2026-06-03/el-juez-pospone-la-citacion-de-begona-gomez-al-15-de-junio.html</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 10:30 p. m.</t>
+          <t>03/06/2026 03:27 a. m.</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
@@ -2323,19 +2319,19 @@
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>Nueva subasta de Diana de Gales: así son sus fotos y cartas inéditas antes de ser princesa</t>
+          <t>Los delitos de odio alcanzan niveles récord con los menores cada vez más implicados</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/gente/2026-06-03/nueva-subasta-de-diana-de-gales-asi-son-sus-fotos-y-cartas-ineditas-antes-de-ser-princesa.html</t>
+          <t>https://elpais.com/espana/2026-06-03/los-delitos-de-odio-alcanzan-el-punto-maximo-y-los-menores-cada-vez-estan-mas-implicados.html</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 10:15 p. m.</t>
+          <t>03/06/2026 03:22 a. m.</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -2350,19 +2346,19 @@
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>¿Cómo va a cambiar el tiempo este verano por el fenómeno de ‘El Niño’</t>
+          <t>Dos menores agreden sexualmente a tres niñas de 10 y 11 años en una piscina pública de Vallecas</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/clima-y-medio-ambiente/2026-06-03/como-va-a-cambiar-el-tiempo-este-verano-por-el-fenomeno-de-el-nino.html</t>
+          <t>https://elpais.com/espana/madrid/2026-06-03/dos-menores-agreden-sexualmente-a-tres-ninas-de-10-y-11-anos-en-una-piscina-publica-de-vallecas.html</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 07:00 p. m.</t>
+          <t>03/06/2026 03:14 a. m.</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr">
@@ -2377,19 +2373,19 @@
       </c>
       <c r="D71" s="6" t="inlineStr">
         <is>
-          <t>Los microbios de Ötzi, el hombre de los hielos, se despiertan miles de años después de su muerte</t>
+          <t>La pobreza se estanca en España: “Vivir en una casa sola con mis hijos sería imposible para mí”</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/ciencia/2026-06-03/los-microbios-de-otzi-el-hombre-de-los-hielos-se-despiertan-miles-de-anos-despues-de-su-muerte.html</t>
+          <t>https://elpais.com/sociedad/2026-06-03/la-pobreza-se-estanca-en-espana-vivir-en-una-casa-sola-con-mis-hijos-seria-imposible-para-mi.html</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 01:53 a. m.</t>
+          <t>03/06/2026 03:12 a. m.</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -2399,24 +2395,24 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>Gremios le cierran la puerta al diálogo con</t>
+          <t>La receta de Lalachus para que los invitados de la Casita de Bad Bunny aprendan a disfrutar: “Tenéis que dar demasiada vergüenza ajena”</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/03/gremios-le-cierran-la-puerta-al-dialogo-con/</t>
+          <t>https://elpais.com/television/2026-06-03/la-receta-de-lalachus-para-que-los-invitados-de-la-casita-de-bad-bunny-aprendan-a-disfrutar-teneis-que-dar-demasiada-verguenza-ajena.html</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 01:21 a. m.</t>
+          <t>03/06/2026 03:02 a. m.</t>
         </is>
       </c>
       <c r="B73" s="5" t="inlineStr">
@@ -2426,24 +2422,24 @@
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D73" s="6" t="inlineStr">
         <is>
-          <t>Día sin carro y sin moto en Pasto: estas son las excepciones para este 3 de junio</t>
+          <t>Un juzgado de Sevilla investiga la muerte por quemaduras de una bebé de 16 meses mientras la bañaba la pareja de la madre</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/03/dia-sin-carro-y-sin-moto-en-pasto-estas-son-las-excepciones-para-este-3-de-junio/</t>
+          <t>https://elpais.com/sociedad/2026-06-03/un-juzgado-de-sevilla-investiga-la-muerte-por-quemaduras-de-una-bebe-de-16-meses-mientras-la-banaba-la-expareja-de-la-madre.html</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 01:03 a. m.</t>
+          <t>03/06/2026 02:57 a. m.</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -2453,24 +2449,24 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>Del 1 al 7 de junio el Puerto de Tumaco conmemora la Semana de los Océanos</t>
+          <t>La abogada de Koldo entrega a la UCO documentación para desmentir que intentara sobornar a la empresaria Carmen Pano</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/03/del-1-al-7-de-junio-el-puerto-de-tumaco-conmemora-la-semana-de-los-oceanos/</t>
+          <t>https://elpais.com/espana/2026-06-03/la-abogada-de-koldo-entrega-a-la-uco-documentacion-para-intentar-desmentir-que-sobornara-a-la-empersaria-carmen-pano.html</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 12:01 a. m.</t>
+          <t>03/06/2026 02:55 a. m.</t>
         </is>
       </c>
       <c r="B75" s="5" t="inlineStr">
@@ -2480,24 +2476,24 @@
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr">
         <is>
-          <t>Un soldado muerto y dos más heridos deja ataque con drones contra militares en el Catatumbo</t>
+          <t>La justicia europea anula en parte la condición de Meta como guardián de mercado</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/03/un-soldado-muerto-y-dos-mas-heridos-deja-ataque-con-drones-contra-militares-en-el-catatumbo/</t>
+          <t>https://elpais.com/economia/2026-06-03/la-justicia-europea-anula-en-parte-la-condicion-de-meta-como-guardian-de-mercado.html</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 11:17 p. m.</t>
+          <t>03/06/2026 02:50 a. m.</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -2507,24 +2503,24 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>Italia celebró su Día Nacional en Colombia destacando la cooperación entre ambos países</t>
+          <t>Última hora de la actualidad política, en directo | Page considera que su partido debería querellarse con Leire Díez y con “todos los que están manchando el nombre del PSOE”</t>
         </is>
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/03/italia-celebro-su-dia-nacional-en-colombia-destacando-la-cooperacion-entre-ambos-paises/</t>
+          <t>https://elpais.com/espana/2026-06-03/ultima-hora-de-la-actualidad-politica-en-directo.html</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 09:48 p. m.</t>
+          <t>03/06/2026 02:21 a. m.</t>
         </is>
       </c>
       <c r="B77" s="5" t="inlineStr">
@@ -2534,24 +2530,24 @@
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D77" s="6" t="inlineStr">
         <is>
-          <t>Trabajadores independientes podrían pagar IVA: conozca si está obligado ante la DIAN</t>
+          <t>El PP y Vox alcanzan un acuerdo de gobierno en Castilla y León  que incluye la “prioridad nacional”</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/03/trabajadores-independientes-podrian-pagar-iva-conozca-si-esta-obligado-ante-la-dian/</t>
+          <t>https://elpais.com/espana/elecciones-castilla-y-leon/2026-06-03/el-pp-y-vox-alcanzan-un-acuerdo-en-castilla-y-leon-para-investir-a-manueco-que-incluye-la-prioridad-nacional.html</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 09:39 p. m.</t>
+          <t>03/06/2026 02:15 a. m.</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -2561,24 +2557,24 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>Petro tras apoyo de Trump a De la Espriella: cuando un país interviene en otro, muere la libertad</t>
+          <t>Atraco a las 21.00 en un centro comercial de Madrid: tres encapuchados con un arma semiautomática roban en una joyería</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/03/petro-tras-apoyo-de-trump-a-de-la-espriella-cuando-un-pais-interviene-en-otro-muere-la-liberad/</t>
+          <t>https://elpais.com/espana/madrid/2026-06-03/tres-encapuchados-con-vestimenta-militar-atracan-una-joyeria-en-un-centro-comercial-de-madrid.html</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 08:48 p. m.</t>
+          <t>03/06/2026 02:13 a. m.</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
@@ -2588,24 +2584,24 @@
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
         <is>
-          <t>Registraduría advierte difusión de E-14 manipulados con IA para impulsar narrativa de fraude</t>
+          <t>Rusia intensifica los ataques contra Ucrania y sus amenazas a Europa: “Su pacífico sueño ha terminado”</t>
         </is>
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/03/registraduria-advierte-difusion-de-e-14-manipulados-con-ia-para-impulsar-narrativa-de-fraude/</t>
+          <t>https://elpais.com/internacional/2026-06-03/rusia-intensifica-los-ataques-contra-ucrania-y-sus-amenazas-a-europa-su-pacifico-sueno-ha-terminado.html</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 08:33 p. m.</t>
+          <t>03/06/2026 02:06 a. m.</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -2615,24 +2611,24 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>Medicina Legal reveló que, entre los 48 cadáveres hallados en Guaviare, 11 eran menores</t>
+          <t>El cocinero de Chueca que dará de cenar a Bad Bunny esta noche en el Metropolitano</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/03/medicina-legal-revelo-que-entre-los-48-cadaveres-hallados-en-guaviare-11-eran-menores/</t>
+          <t>https://elpais.com/gastronomia/2026-06-03/el-cocinero-de-chueca-que-dara-de-cenar-a-bad-bunny-esta-noche-en-el-metropolitano.html</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 08:12 p. m.</t>
+          <t>02/06/2026 10:45 p. m.</t>
         </is>
       </c>
       <c r="B81" s="5" t="inlineStr">
@@ -2642,24 +2638,24 @@
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D81" s="6" t="inlineStr">
         <is>
-          <t>Registraduría pide a Petro evitar “interpretaciones imprecisas” sobre software y censo electoral</t>
+          <t>Inés Hernand sobre la polémica con Bad Bunny: “Se arma tanto revuelo porque es el lugar político de los más jóvenes”</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/03/registraduria-pide-a-petro-evitar-interpretaciones-imprecisas-sobre-software-y-censo-electoral/</t>
+          <t>https://elpais.com/podcasts/hoy-en-el-pais/2026-06-03/ines-hernand-sobre-la-casita-de-bad-bunny-le-tenian-muchas-ganas.html</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 07:59 p. m.</t>
+          <t>02/06/2026 10:30 p. m.</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -2669,24 +2665,24 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>¿Benedetti renunciará a su cargo de ministro para trabajar en la campaña de Iván Cepeda?</t>
+          <t>El Gobierno ve imposible la moción  de censura por el rechazo en Cataluña y Euskadi al PP y Vox</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/03/benedetti-renunciara-a-su-cargo-de-ministro-para-trabajar-en-la-campana-de-ivan-cepeda/</t>
+          <t>https://elpais.com/espana/2026-06-03/el-gobierno-ve-imposible-la-mocion-de-censura-por-el-rechazo-en-cataluna-y-euskadi-al-pp-y-vox.html</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 07:51 p. m.</t>
+          <t>02/06/2026 10:30 p. m.</t>
         </is>
       </c>
       <c r="B83" s="5" t="inlineStr">
@@ -2696,24 +2692,24 @@
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D83" s="6" t="inlineStr">
         <is>
-          <t>Petro aseguró que no ha roto cooperación con EEUU a pesar de que imponen política ante narcotráfico</t>
+          <t>Las prisas cambian de bando en Irán: Trump busca una salida a la guerra con el tiempo en su contra</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/03/petro-aseguro-que-no-ha-roto-cooperacion-con-eeuu-a-pesar-de-que-imponen-politica-ante-narcotrafico/</t>
+          <t>https://elpais.com/internacional/2026-06-03/las-prisas-cambian-de-bando-en-iran-trump-busca-una-salida-a-la-guerra-con-el-tiempo-en-su-contra.html</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 07:30 p. m.</t>
+          <t>02/06/2026 10:30 p. m.</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -2723,24 +2719,24 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>OPS pide reforzar medidas de respuesta al sarampión a días del Mundial de fútbol</t>
+          <t>Del ‘nanopinganillo’ a la grabación: así se caza a los copiones en la Selectividad</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/03/ops-pide-reforzar-medidas-de-respuesta-al-sarampion-a-dias-del-mundial-de-futbol/</t>
+          <t>https://elpais.com/educacion/2026-06-03/del-nanopinganillo-a-la-grabacion-asi-se-caza-a-los-copiones-en-la-selectividad.html</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 07:27 p. m.</t>
+          <t>02/06/2026 10:30 p. m.</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr">
@@ -2750,24 +2746,24 @@
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D85" s="6" t="inlineStr">
         <is>
-          <t>Resultados de la Lotería Cruz Roja, del Huila y MiLoto HOY 02 de junio: premios y último sorteo</t>
+          <t>Marc Giró: “No estamos para equidistancias, soy radicalmente de izquierdas y antifascista, ¿existe esta transparencia con otros presentadores?”</t>
         </is>
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/03/resultados-de-la-loteria-cruz-roja-del-huila-y-miloto-hoy-02-de-junio-premios-y-ultimo-sorteo/</t>
+          <t>https://elpais.com/television/2026-06-03/marc-giro-no-estamos-para-equidistancias-soy-radicalmente-de-izquierdas-y-antifascista-existe-esta-transparencia-con-otros-presentadores.html</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 07:21 p. m.</t>
+          <t>02/06/2026 10:30 p. m.</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -2777,24 +2773,24 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>Rechazaron tutela con la que la exembajadora de Haití pretendía tumbar suspensión de la Procuraduría</t>
+          <t>Nueva subasta de Diana de Gales: así son sus fotos y cartas inéditas antes de ser princesa</t>
         </is>
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/03/rechazaron-tutela-con-la-que-la-exembajadora-de-haiti-pretendia-tumbar-suspension-de-la-procuraduria/</t>
+          <t>https://elpais.com/gente/2026-06-03/nueva-subasta-de-diana-de-gales-asi-son-sus-fotos-y-cartas-ineditas-antes-de-ser-princesa.html</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 07:17 p. m.</t>
+          <t>02/06/2026 10:15 p. m.</t>
         </is>
       </c>
       <c r="B87" s="5" t="inlineStr">
@@ -2804,24 +2800,24 @@
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D87" s="6" t="inlineStr">
         <is>
-          <t>Defensoría del Pueblo reporta 784 personas desplazadas en Catatumbo, Norte de Santander</t>
+          <t>¿Cómo va a cambiar el tiempo este verano por el fenómeno de ‘El Niño’</t>
         </is>
       </c>
       <c r="E87" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/03/defensoria-del-pueblo-reporta-784-personas-desplazadas-en-catatumbo-norte-de-santander/</t>
+          <t>https://elpais.com/clima-y-medio-ambiente/2026-06-03/como-va-a-cambiar-el-tiempo-este-verano-por-el-fenomeno-de-el-nino.html</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 07:11 p. m.</t>
+          <t>02/06/2026 07:00 p. m.</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -2831,24 +2827,24 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>Reviva la alocución del presidente Gustavo Petro</t>
+          <t>Los microbios de Ötzi, el hombre de los hielos, se despiertan miles de años después de su muerte</t>
         </is>
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/03/en-vivo-alocucion-del-presidente-gustavo-petro/</t>
+          <t>https://elpais.com/ciencia/2026-06-03/los-microbios-de-otzi-el-hombre-de-los-hielos-se-despiertan-miles-de-anos-despues-de-su-muerte.html</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 07:10 p. m.</t>
+          <t>03/06/2026 03:11 a. m.</t>
         </is>
       </c>
       <c r="B89" s="5" t="inlineStr">
@@ -2863,19 +2859,19 @@
       </c>
       <c r="D89" s="6" t="inlineStr">
         <is>
-          <t>MinDefensa responde al New York Times y niega haber pedido sanciones al oro colombiano</t>
+          <t>La guerra en Oriente Medio disminuirá el crecimiento y aumentará la inflación en todo el mundo: OCDE</t>
         </is>
       </c>
       <c r="E89" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/03/mindefensa-responde-al-new-york-times-y-niega-haber-pedido-sanciones-al-oro-colombiano/</t>
+          <t>https://caracol.com.co/2026/06/03/la-guerra-en-oriente-medio-disminuira-el-crecimiento-y-aumentara-la-inflacion-en-todo-el-mundo-ocde/</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 06:53 p. m.</t>
+          <t>03/06/2026 01:53 a. m.</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -2890,19 +2886,19 @@
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>SENA inició Tercera Convocatoria Presencial 2026: Estos son las fechas y requisitos para inscribirse</t>
+          <t>Gremios le cierran la puerta al diálogo con quienes no reconocen resultados electorales</t>
         </is>
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/02/sena-inicia-tercera-convocatoria-presencial-2026-estos-son-las-fechas-y-requisitos-para-inscribirse/</t>
+          <t>https://caracol.com.co/2026/06/03/gremios-le-cierran-la-puerta-al-dialogo-con/</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 06:22 p. m.</t>
+          <t>03/06/2026 01:21 a. m.</t>
         </is>
       </c>
       <c r="B91" s="5" t="inlineStr">
@@ -2917,19 +2913,19 @@
       </c>
       <c r="D91" s="6" t="inlineStr">
         <is>
-          <t>Guerra en Irán causa aumento de tráfico por el Canal de Panamá</t>
+          <t>Día sin carro y sin moto en Pasto: estas son las excepciones para este 3 de junio</t>
         </is>
       </c>
       <c r="E91" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/02/guerra-en-iran-causa-aumento-de-trafico-por-el-canal-de-panama/</t>
+          <t>https://caracol.com.co/2026/06/03/dia-sin-carro-y-sin-moto-en-pasto-estas-son-las-excepciones-para-este-3-de-junio/</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 01:00 a. m.</t>
+          <t>03/06/2026 01:03 a. m.</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -2939,24 +2935,24 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>Catastrófica deforestación en el Día Internacional de los Bosques</t>
+          <t>Del 1 al 7 de junio el Puerto de Tumaco conmemora la Semana de los Océanos</t>
         </is>
       </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/03/catastrofica-deforestacion-en-el-dia-internacional-de-los-bosques/</t>
+          <t>https://caracol.com.co/2026/06/03/del-1-al-7-de-junio-el-puerto-de-tumaco-conmemora-la-semana-de-los-oceanos/</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 01:00 a. m.</t>
+          <t>03/06/2026 12:01 a. m.</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
@@ -2966,24 +2962,24 @@
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D93" s="6" t="inlineStr">
         <is>
-          <t>Columnistas</t>
+          <t>Un soldado muerto y dos más heridos deja ataque con drones contra militares en el Catatumbo</t>
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/</t>
+          <t>https://caracol.com.co/2026/06/03/un-soldado-muerto-y-dos-mas-heridos-deja-ataque-con-drones-contra-militares-en-el-catatumbo/</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 01:00 a. m.</t>
+          <t>02/06/2026 11:17 p. m.</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -2993,24 +2989,24 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>Cuando la fiesta termina en tragedia</t>
+          <t>Italia celebró su Día Nacional en Colombia destacando la cooperación entre ambos países</t>
         </is>
       </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/03/cuando-la-fiesta-termina-en-tragedia/</t>
+          <t>https://caracol.com.co/2026/06/03/italia-celebro-su-dia-nacional-en-colombia-destacando-la-cooperacion-entre-ambos-paises/</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 01:00 a. m.</t>
+          <t>02/06/2026 09:48 p. m.</t>
         </is>
       </c>
       <c r="B95" s="5" t="inlineStr">
@@ -3020,24 +3016,24 @@
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D95" s="6" t="inlineStr">
         <is>
-          <t>Cuando toca, ¡toca!</t>
+          <t>Trabajadores independientes podrían pagar IVA: conozca si está obligado ante la DIAN</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/caricaturas/2026/06/03/cuando-toca-toca/</t>
+          <t>https://caracol.com.co/2026/06/03/trabajadores-independientes-podrian-pagar-iva-conozca-si-esta-obligado-ante-la-dian/</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 01:00 a. m.</t>
+          <t>02/06/2026 09:39 p. m.</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -3047,24 +3043,24 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>Caricaturas</t>
+          <t>Petro tras apoyo de Trump a De la Espriella: cuando un país interviene en otro, muere la libertad</t>
         </is>
       </c>
       <c r="E96" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/caricaturas/</t>
+          <t>https://caracol.com.co/2026/06/03/petro-tras-apoyo-de-trump-a-de-la-espriella-cuando-un-pais-interviene-en-otro-muere-la-liberad/</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 01:00 a. m.</t>
+          <t>02/06/2026 08:48 p. m.</t>
         </is>
       </c>
       <c r="B97" s="5" t="inlineStr">
@@ -3074,24 +3070,24 @@
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D97" s="6" t="inlineStr">
         <is>
-          <t>UIS: excelencia académica y liderazgo nacional, fruto de una apuesta por la formación integral</t>
+          <t>Registraduría advierte difusión de E-14 manipulados con IA para impulsar narrativa de fraude</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/03/uis-excelencia-academica-y-liderazgo-nacional-fruto-de-una-apuesta-por-la-formacion-integral/</t>
+          <t>https://caracol.com.co/2026/06/03/registraduria-advierte-difusion-de-e-14-manipulados-con-ia-para-impulsar-narrativa-de-fraude/</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 10:30 p. m.</t>
+          <t>02/06/2026 08:33 p. m.</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -3101,24 +3097,24 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>Tragedia en Guaviare: 11 adolescentes asesinados en combates entre alias ‘Iván Mordisco’ y ‘Calarcá’</t>
+          <t>Medicina Legal reveló que, entre los 48 cadáveres hallados en Guaviare, 11 eran menores</t>
         </is>
       </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/02/tragedia-en-guaviare-11-adolescentes-asesinados-en-combates-entre-alias-ivan-mordisco-y-calarca/</t>
+          <t>https://caracol.com.co/2026/06/03/medicina-legal-revelo-que-entre-los-48-cadaveres-hallados-en-guaviare-11-eran-menores/</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 10:30 p. m.</t>
+          <t>02/06/2026 08:12 p. m.</t>
         </is>
       </c>
       <c r="B99" s="5" t="inlineStr">
@@ -3128,24 +3124,24 @@
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D99" s="6" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Registraduría pide a Petro evitar “interpretaciones imprecisas” sobre software y censo electoral</t>
         </is>
       </c>
       <c r="E99" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/</t>
+          <t>https://caracol.com.co/2026/06/03/registraduria-pide-a-petro-evitar-interpretaciones-imprecisas-sobre-software-y-censo-electoral/</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 07:09 p. m.</t>
+          <t>02/06/2026 07:59 p. m.</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -3155,24 +3151,24 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>En directo: Petro entrega balance sobre la erradición de cultivos de coca durante su gobierno</t>
+          <t>¿Benedetti renunciará a su cargo de ministro para trabajar en la campaña de Iván Cepeda?</t>
         </is>
       </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/02/en-directo-el-presidente-petro-habla-sobre-los-resultados-de-la-primera-vuelta/</t>
+          <t>https://caracol.com.co/2026/06/03/benedetti-renunciara-a-su-cargo-de-ministro-para-trabajar-en-la-campana-de-ivan-cepeda/</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 05:14 p. m.</t>
+          <t>02/06/2026 07:51 p. m.</t>
         </is>
       </c>
       <c r="B101" s="5" t="inlineStr">
@@ -3182,24 +3178,24 @@
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D101" s="6" t="inlineStr">
         <is>
-          <t>¿Renunciará Petro para hacer campaña? Esto respondió su jefe de gabinete</t>
+          <t>Petro aseguró que no ha roto cooperación con EEUU a pesar de que imponen política ante narcotráfico</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/02/renunciara-petro-para-hacer-campana-esto-respondio-su-jefe-de-gabinete/</t>
+          <t>https://caracol.com.co/2026/06/03/petro-aseguro-que-no-ha-roto-cooperacion-con-eeuu-a-pesar-de-que-imponen-politica-ante-narcotrafico/</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 04:27 p. m.</t>
+          <t>02/06/2026 07:47 p. m.</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -3209,24 +3205,24 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>Derecho de preferencia notarial en Colombia: ¿Es aplicable sin ley?</t>
+          <t>Presidente Donald Trump expresó “respaldo total” al candidato Abelardo de La Espriella</t>
         </is>
       </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/02/derecho-de-preferencia-notarial-en-colombia-es-aplicable-sin-ley/</t>
+          <t>https://caracol.com.co/2026/06/03/presidente-donald-trump-expreso-respaldo-total-al-candidato-abelardo-de-la-espriella/</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 03:56 p. m.</t>
+          <t>02/06/2026 07:30 p. m.</t>
         </is>
       </c>
       <c r="B103" s="5" t="inlineStr">
@@ -3236,24 +3232,24 @@
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D103" s="6" t="inlineStr">
         <is>
-          <t>Ataques contra periodistas se dispararon 227 % durante las elecciones presidenciales</t>
+          <t>OPS pide reforzar medidas de respuesta al sarampión a días del Mundial de fútbol</t>
         </is>
       </c>
       <c r="E103" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/02/ataques-contra-periodistas-se-dispararon-227-durante-las-elecciones-presidenciales/</t>
+          <t>https://caracol.com.co/2026/06/03/ops-pide-reforzar-medidas-de-respuesta-al-sarampion-a-dias-del-mundial-de-futbol/</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 03:16 p. m.</t>
+          <t>02/06/2026 07:27 p. m.</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
@@ -3263,24 +3259,24 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>Empresario arremete contra Abelardo De la Espriella: “lo vamos a fumigar”</t>
+          <t>Resultados de la Lotería Cruz Roja, del Huila y MiLoto HOY 02 de junio: premios y último sorteo</t>
         </is>
       </c>
       <c r="E104" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/02/empresario-arremete-contra-abelardo-de-la-espriella-lo-vamos-a-fumigar/</t>
+          <t>https://caracol.com.co/2026/06/03/resultados-de-la-loteria-cruz-roja-del-huila-y-miloto-hoy-02-de-junio-premios-y-ultimo-sorteo/</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 10:57 a. m.</t>
+          <t>02/06/2026 07:21 p. m.</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
@@ -3290,24 +3286,24 @@
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D105" s="6" t="inlineStr">
         <is>
-          <t>Mujer fue detenida en Cartagena por intentar sacar a su hijo con permiso falso</t>
+          <t>Rechazaron tutela con la que la exembajadora de Haití pretendía tumbar suspensión de la Procuraduría</t>
         </is>
       </c>
       <c r="E105" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/02/mujer-fue-detenida-en-cartagena-por-intentar-sacar-a-su-hijo-con-permiso-falso/</t>
+          <t>https://caracol.com.co/2026/06/03/rechazaron-tutela-con-la-que-la-exembajadora-de-haiti-pretendia-tumbar-suspension-de-la-procuraduria/</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 10:22 a. m.</t>
+          <t>02/06/2026 07:17 p. m.</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
@@ -3317,24 +3313,24 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D106" s="3" t="inlineStr">
         <is>
-          <t>Procuraduría suspende a Alfredo Saade, embajador en Brasil, por mensajes políticos en campaña</t>
+          <t>Defensoría del Pueblo reporta 784 personas desplazadas en Catatumbo, Norte de Santander</t>
         </is>
       </c>
       <c r="E106" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/02/procuraduria-suspende-a-embajador-en-brasil-por-mensajes-politicos-en-campana/</t>
+          <t>https://caracol.com.co/2026/06/03/defensoria-del-pueblo-reporta-784-personas-desplazadas-en-catatumbo-norte-de-santander/</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 07:29 a. m.</t>
+          <t>02/06/2026 07:11 p. m.</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
@@ -3344,22 +3340,26 @@
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D107" s="6" t="inlineStr">
         <is>
-          <t>Bus de la Selección Colombia quedó rodeado por manifestantes en marcha en Bogotá</t>
+          <t>Reviva la alocución del presidente Gustavo Petro</t>
         </is>
       </c>
       <c r="E107" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/02/bus-de-la-seleccion-colombia-quedo-rodeado-por-manifestantes-en-marcha-en-bogota/</t>
+          <t>https://caracol.com.co/2026/06/03/en-vivo-alocucion-del-presidente-gustavo-petro/</t>
         </is>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="inlineStr"/>
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>02/06/2026 07:10 p. m.</t>
+        </is>
+      </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3367,17 +3367,17 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D108" s="3" t="inlineStr">
         <is>
-          <t>Cerrejón suspende operaciones en La Guajira: más de 12.000 trabajadores afectados</t>
+          <t>MinDefensa responde al New York Times y niega haber pedido sanciones al oro colombiano</t>
         </is>
       </c>
       <c r="E108" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/01/cerrejon-suspende-operaciones-en-la-guajira-mas-de-12000-trabajadores-afectados/</t>
+          <t>https://caracol.com.co/2026/06/03/mindefensa-responde-al-new-york-times-y-niega-haber-pedido-sanciones-al-oro-colombiano/</t>
         </is>
       </c>
     </row>
@@ -4413,19 +4413,19 @@
       </c>
       <c r="D147" s="6" t="inlineStr">
         <is>
-          <t>De elección y Bad Bunny</t>
+          <t>Todos del mismo lado de la incertidumbre</t>
         </is>
       </c>
       <c r="E147" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/oscar-guardiola-rivera/de-eleccion-y-bad-bunny/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/sandra-vilardy/todos-del-mismo-lado-de-la-incertidumbre/</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 12:03 a. m.</t>
+          <t>03/06/2026 12:05 a. m.</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
@@ -4440,19 +4440,19 @@
       </c>
       <c r="D148" s="3" t="inlineStr">
         <is>
-          <t>La primera vuelta</t>
+          <t>Cayeron en la trampa</t>
         </is>
       </c>
       <c r="E148" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/gonzalo-mallarino/mi-decision-en-consecuencia-es-votar-en-blanco-en-segunda-vuelta/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/mario-morales/cayeron-en-la-trampa/</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 10:11 p. m.</t>
+          <t>03/06/2026 12:05 a. m.</t>
         </is>
       </c>
       <c r="B149" s="5" t="inlineStr">
@@ -4467,19 +4467,19 @@
       </c>
       <c r="D149" s="6" t="inlineStr">
         <is>
-          <t>Atlético Nacional vs. Junior: ¿Cuándo será el partido de vuelta de la final de Liga BetPlay?</t>
+          <t>Mirando la vuelta</t>
         </is>
       </c>
       <c r="E149" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/deportes/futbol-colombiano/atletico-nacional-vs-junior-cuando-sera-el-partido-de-vuelta-de-la-final-de-liga-betplay/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/pascual-gaviria/mirando-la-segunda-vuelta-elecciones-colombia-2026/</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 10:03 p. m.</t>
+          <t>03/06/2026 12:05 a. m.</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
@@ -4494,19 +4494,19 @@
       </c>
       <c r="D150" s="3" t="inlineStr">
         <is>
-          <t>Crimen de la periodista Silvia Duzán llega a la Corte IDH contra el Estado colombiano</t>
+          <t>De elección y Bad Bunny</t>
         </is>
       </c>
       <c r="E150" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/judicial/corte-idh-estudia-caso-por-la-masacre-de-silvia-duzan-y-lideres-campesinos-en-santander/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/oscar-guardiola-rivera/de-eleccion-y-bad-bunny/</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 10:00 p. m.</t>
+          <t>03/06/2026 12:05 a. m.</t>
         </is>
       </c>
       <c r="B151" s="5" t="inlineStr">
@@ -4521,19 +4521,19 @@
       </c>
       <c r="D151" s="6" t="inlineStr">
         <is>
-          <t>Venezuela aprobó abrir su sector eléctrico a privados por primera vez en casi 20 años</t>
+          <t>La amenaza del caos</t>
         </is>
       </c>
       <c r="E151" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/economia/macroeconomia/venezuela-aprobo-abrir-su-sector-electrico-a-privados-por-primera-vez-en-casi-20-anos-noticias-hoy/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/andres-hoyos/la-amenaza-del-caos/</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 09:46 p. m.</t>
+          <t>03/06/2026 12:05 a. m.</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
@@ -4548,19 +4548,19 @@
       </c>
       <c r="D152" s="3" t="inlineStr">
         <is>
-          <t>La Ley de la Música será una realidad: fue aprobada en último debate en el Congreso</t>
+          <t>El reto: resistir la mano negra de Petro</t>
         </is>
       </c>
       <c r="E152" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/el-magazin-cultural/la-ley-de-la-musica-sera-una-realidad-fue-aprobada-en-ultimo-debate-en-el-congreso/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/pablo-felipe-robledo/el-reto-resistir-la-mano-negra-de-petro/</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 09:45 p. m.</t>
+          <t>03/06/2026 12:00 a. m.</t>
         </is>
       </c>
       <c r="B153" s="5" t="inlineStr">
@@ -4570,24 +4570,24 @@
       </c>
       <c r="C153" s="5" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae Colombia</t>
         </is>
       </c>
       <c r="D153" s="6" t="inlineStr">
         <is>
-          <t>Junior goleó a Nacional en la ida de la final y quedó a un paso del título de Liga BetPlay</t>
+          <t>Identifican a soldado profesional muerto en ataque con drones del ELN en Teorama, Norte de Santander</t>
         </is>
       </c>
       <c r="E153" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/deportes/futbol-colombiano/junior-vs-nacional-en-vivo-siga-los-mejores-momentos-de-la-final-de-liga-betplay-formaciones-goles-video-noticias-hoy/</t>
+          <t>https://www.infobae.com/colombia/2026/06/03/identifican-a-soldado-profesional-muerto-en-ataque-con-drones-del-eln-en-teorama-norte-de-santander/</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 09:30 p. m.</t>
+          <t>03/06/2026 12:00 a. m.</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
@@ -4597,22 +4597,26 @@
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae Colombia</t>
         </is>
       </c>
       <c r="D154" s="3" t="inlineStr">
         <is>
-          <t>Nace en EE. UU. una cría del caballo de Przewalski, una especie en peligro de extinción</t>
+          <t>Bogotá registra aumento en empleo turístico y conectividad aérea durante 2026</t>
         </is>
       </c>
       <c r="E154" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/ambiente/nace-en-ee-uu-una-cria-del-caballo-de-przewalski-una-especie-en-peligro-de-extincion/</t>
+          <t>https://www.infobae.com/colombia/2026/06/03/bogota-registra-aumento-en-empleo-turistico-y-conectividad-aerea-durante-2026/</t>
         </is>
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="5" t="inlineStr"/>
+      <c r="A155" s="5" t="inlineStr">
+        <is>
+          <t>03/06/2026 12:00 a. m.</t>
+        </is>
+      </c>
       <c r="B155" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4620,17 +4624,17 @@
       </c>
       <c r="C155" s="5" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae Colombia</t>
         </is>
       </c>
       <c r="D155" s="6" t="inlineStr">
         <is>
-          <t>De la Espriella e Iván Cepeda: estas son las cuentas de sus campañas en primera vuelta</t>
+          <t>Clima en Colombia: temperatura y probabilidad de lluvia para Barranquilla este 3 de junio</t>
         </is>
       </c>
       <c r="E155" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/investigacion/abelardo-de-la-espriella-e-ivan-cepeda-estas-son-las-cuentas-de-sus-campanas-en-primera-vuelta/</t>
+          <t>https://www.infobae.com/colombia/2026/06/03/clima-en-colombia-temperatura-y-probabilidad-de-lluvia-para-barranquilla-este-3-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4652,12 +4656,12 @@
       </c>
       <c r="D156" s="3" t="inlineStr">
         <is>
-          <t>“Las EPS tendrán máximo ocho horas”: Daniel Quintero anuncia nuevas medidas obligatorias para garantizar atención médica a menores</t>
+          <t>Pronóstico del clima: las temperaturas que se esperan en Bogotá este 3 de junio</t>
         </is>
       </c>
       <c r="E156" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/03/las-eps-tendran-maximo-ocho-horas-daniel-quintero-anuncia-nuevas-medidas-obligatorias-para-garantizar-atencion-medica-a-menores/</t>
+          <t>https://www.infobae.com/colombia/2026/06/03/pronostico-del-clima-las-temperaturas-que-se-esperan-en-bogota-este-3-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4679,12 +4683,12 @@
       </c>
       <c r="D157" s="6" t="inlineStr">
         <is>
-          <t>Pico y Placa en Bogotá: restricciones vehiculares para este miércoles 3 de junio</t>
+          <t>Pronóstico del estado del tiempo: las temperaturas que se esperan en Cali este 3 de junio</t>
         </is>
       </c>
       <c r="E157" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/03/pico-y-placa-en-bogota-restricciones-vehiculares-para-este-miercoles-3-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/03/pronostico-del-estado-del-tiempo-las-temperaturas-que-se-esperan-en-cali-este-3-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4706,12 +4710,12 @@
       </c>
       <c r="D158" s="3" t="inlineStr">
         <is>
-          <t>Abelardo de la Espriella agradece respaldo de Donald Trump: “Haremos una llave como nunca antes la ha tenido Colombia”</t>
+          <t>Previsión del clima en Medellín para antes de salir de casa este 3 de junio</t>
         </is>
       </c>
       <c r="E158" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/03/abelardo-de-la-espriella-agradece-respaldo-de-donald-trump-haremos-una-llave-como-nunca-antes-la-ha-tenido-colombia/</t>
+          <t>https://www.infobae.com/colombia/2026/06/03/prevision-del-clima-en-medellin-para-antes-de-salir-de-casa-este-3-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4733,12 +4737,12 @@
       </c>
       <c r="D159" s="6" t="inlineStr">
         <is>
-          <t>Embargos en Colombia 2026: estos son los casos en los que una cuenta bancaria no puede ser retenida por orden judicial</t>
+          <t>Colombia: las predicciones del tiempo en Cartagena de Indias este 3 de junio</t>
         </is>
       </c>
       <c r="E159" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/03/embargos-en-colombia-2026-estos-son-los-casos-en-los-que-una-cuenta-bancaria-no-puede-ser-retenida-por-orden-judicial/</t>
+          <t>https://www.infobae.com/colombia/2026/06/03/colombia-las-predicciones-del-tiempo-en-cartagena-de-indias-este-3-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4760,12 +4764,12 @@
       </c>
       <c r="D160" s="3" t="inlineStr">
         <is>
-          <t>Ni la goleada evitó los disturbios: enfrentamientos entre hinchas opacaron la final entre Junior y Atlético Nacional</t>
+          <t>Consejo Gremial lanza advertencia: no dialogará con quienes desconozcan resultados electorales en Colombia</t>
         </is>
       </c>
       <c r="E160" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/06/03/ni-la-goleada-evito-los-disturbios-enfrentamientos-entre-hinchas-opacaron-la-final-entre-junior-y-atletico-nacional/</t>
+          <t>https://www.infobae.com/colombia/2026/06/03/consejo-gremial-lanza-advertencia-no-dialogara-con-quienes-desconozcan-resultados-electorales-en-colombia/</t>
         </is>
       </c>
     </row>
@@ -4787,12 +4791,12 @@
       </c>
       <c r="D161" s="6" t="inlineStr">
         <is>
-          <t>“Te voy a derrotar y te voy a castigar”: Abelardo de la Espriella responde a Benedetti y escala la confrontación política</t>
+          <t>Centro Carter pide respetar los resultados de las elecciones presidenciales y destaca transparencia del proceso en Colombia</t>
         </is>
       </c>
       <c r="E161" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/03/te-voy-a-derrotar-y-te-voy-a-castigar-abelardo-de-la-espriella-responde-a-benedetti-y-escala-la-confrontacion-politica/</t>
+          <t>https://www.infobae.com/colombia/2026/06/03/centro-carter-pide-respetar-los-resultados-de-las-elecciones-presidenciales-y-destaca-transparencia-del-proceso-en-colombia/</t>
         </is>
       </c>
     </row>
@@ -4814,12 +4818,12 @@
       </c>
       <c r="D162" s="3" t="inlineStr">
         <is>
-          <t>“No me pidan buenas maneras con Petro”: Abelardo de la Espriella endurece su discurso y acusa al presidente de querer desconocer las elecciones</t>
+          <t>Petro rechaza respaldo de Trump a Abelardo de la Espriella: “Cuando un país interviene en las decisiones de otro, muere la libertad”</t>
         </is>
       </c>
       <c r="E162" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/03/no-me-pidan-buenas-maneras-con-petro-abelardo-de-la-espriella-endurece-su-discurso-y-acusa-al-presidente-de-querer-desconocer-las-elecciones/</t>
+          <t>https://www.infobae.com/colombia/2026/06/03/petro-rechaza-respaldo-de-trump-a-abelardo-de-la-espriella-cuando-un-pais-interviene-en-las-decisiones-de-otro-muere-la-libertad/</t>
         </is>
       </c>
     </row>
@@ -4841,12 +4845,12 @@
       </c>
       <c r="D163" s="6" t="inlineStr">
         <is>
-          <t>“He desbloqueado su cuenta”: Iván Cepeda respondió a Teleantioquia tras polémica por bloqueo en X</t>
+          <t>“Las EPS tendrán máximo ocho horas”: Daniel Quintero anuncia nuevas medidas obligatorias para garantizar atención médica a menores</t>
         </is>
       </c>
       <c r="E163" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/03/he-desbloqueado-su-cuenta-ivan-cepeda-respondio-a-teleantioquia-tras-polemica-por-bloqueo-en-x/</t>
+          <t>https://www.infobae.com/colombia/2026/06/03/las-eps-tendran-maximo-ocho-horas-daniel-quintero-anuncia-nuevas-medidas-obligatorias-para-garantizar-atencion-medica-a-menores/</t>
         </is>
       </c>
     </row>
@@ -4868,12 +4872,12 @@
       </c>
       <c r="D164" s="3" t="inlineStr">
         <is>
-          <t>Colombia activa una agenda ambiental para salvar sus océanos y costas en 2026</t>
+          <t>Pico y Placa en Bogotá: restricciones vehiculares para este miércoles 3 de junio</t>
         </is>
       </c>
       <c r="E164" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/03/colombia-activa-una-agenda-ambiental-para-salvar-sus-oceanos-y-costas-en-2026/</t>
+          <t>https://www.infobae.com/colombia/2026/06/03/pico-y-placa-en-bogota-restricciones-vehiculares-para-este-miercoles-3-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4895,12 +4899,12 @@
       </c>
       <c r="D165" s="6" t="inlineStr">
         <is>
-          <t>Resultado Super Astro Luna HOY: número ganador del martes 2 de junio</t>
+          <t>Abelardo de la Espriella agradece respaldo de Donald Trump: “Haremos una llave como nunca antes la ha tenido Colombia”</t>
         </is>
       </c>
       <c r="E165" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/03/resultado-super-astro-luna-hoy-numero-ganador-del-martes-2-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/03/abelardo-de-la-espriella-agradece-respaldo-de-donald-trump-haremos-una-llave-como-nunca-antes-la-ha-tenido-colombia/</t>
         </is>
       </c>
     </row>
@@ -4922,12 +4926,12 @@
       </c>
       <c r="D166" s="3" t="inlineStr">
         <is>
-          <t>Colombia modernizará su sistema de donación y trasplante de órganos: proyecto de Paloma Valencia fue aprobado en último debate</t>
+          <t>Embargos en Colombia 2026: estos son los casos en los que una cuenta bancaria no puede ser retenida por orden judicial</t>
         </is>
       </c>
       <c r="E166" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/03/colombia-modernizara-su-sistema-de-donacion-y-trasplante-de-organos-proyecto-de-paloma-valencia-fue-aprobado-en-ultimo-debate/</t>
+          <t>https://www.infobae.com/colombia/2026/06/03/embargos-en-colombia-2026-estos-son-los-casos-en-los-que-una-cuenta-bancaria-no-puede-ser-retenida-por-orden-judicial/</t>
         </is>
       </c>
     </row>
@@ -4949,12 +4953,12 @@
       </c>
       <c r="D167" s="6" t="inlineStr">
         <is>
-          <t>Pico y Placa en Cali: restricciones vehiculares para evitar multas este miércoles 3 de junio</t>
+          <t>Ni la goleada evitó los disturbios: enfrentamientos entre hinchas opacaron la final entre Junior y Atlético Nacional</t>
         </is>
       </c>
       <c r="E167" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/03/pico-y-placa-en-cali-restricciones-vehiculares-para-evitar-multas-este-miercoles-3-de-junio/</t>
+          <t>https://www.infobae.com/colombia/deportes/2026/06/03/ni-la-goleada-evito-los-disturbios-enfrentamientos-entre-hinchas-opacaron-la-final-entre-junior-y-atletico-nacional/</t>
         </is>
       </c>
     </row>
@@ -4976,12 +4980,12 @@
       </c>
       <c r="D168" s="3" t="inlineStr">
         <is>
-          <t>Pico y Placa en Villavicencio: qué vehículos descansan este miércoles 3 de junio</t>
+          <t>“Te voy a derrotar y te voy a castigar”: Abelardo de la Espriella responde a Benedetti y escala la confrontación política</t>
         </is>
       </c>
       <c r="E168" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/03/pico-y-placa-en-villavicencio-que-vehiculos-descansan-este-miercoles-3-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/03/te-voy-a-derrotar-y-te-voy-a-castigar-abelardo-de-la-espriella-responde-a-benedetti-y-escala-la-confrontacion-politica/</t>
         </is>
       </c>
     </row>
@@ -5003,12 +5007,12 @@
       </c>
       <c r="D169" s="6" t="inlineStr">
         <is>
-          <t>Pico y Placa en Cartagena: qué vehículos descansan este miércoles 3 de junio</t>
+          <t>“No me pidan buenas maneras con Petro”: Abelardo de la Espriella endurece su discurso y acusa al presidente de querer desconocer las elecciones</t>
         </is>
       </c>
       <c r="E169" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/03/pico-y-placa-en-cartagena-que-vehiculos-descansan-este-miercoles-3-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/03/no-me-pidan-buenas-maneras-con-petro-abelardo-de-la-espriella-endurece-su-discurso-y-acusa-al-presidente-de-querer-desconocer-las-elecciones/</t>
         </is>
       </c>
     </row>
@@ -5030,12 +5034,12 @@
       </c>
       <c r="D170" s="3" t="inlineStr">
         <is>
-          <t>Resultado Sinuano Noche hoy 2 de junio</t>
+          <t>“He desbloqueado su cuenta”: Iván Cepeda respondió a Teleantioquia tras polémica por bloqueo en X</t>
         </is>
       </c>
       <c r="E170" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/03/resultado-sinuano-noche-hoy-2-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/03/he-desbloqueado-su-cuenta-ivan-cepeda-respondio-a-teleantioquia-tras-polemica-por-bloqueo-en-x/</t>
         </is>
       </c>
     </row>
@@ -5057,12 +5061,12 @@
       </c>
       <c r="D171" s="6" t="inlineStr">
         <is>
-          <t>Cortes de agua en Bogotá, hoy 3 de junio</t>
+          <t>Colombia activa una agenda ambiental para salvar sus océanos y costas en 2026</t>
         </is>
       </c>
       <c r="E171" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/03/cortes-de-agua-en-bogota-hoy-3-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/03/colombia-activa-una-agenda-ambiental-para-salvar-sus-oceanos-y-costas-en-2026/</t>
         </is>
       </c>
     </row>
@@ -5084,19 +5088,19 @@
       </c>
       <c r="D172" s="3" t="inlineStr">
         <is>
-          <t>Pico y Placa Medellín: evita multas este miércoles 3 de junio</t>
+          <t>Resultado Super Astro Luna HOY: número ganador del martes 2 de junio</t>
         </is>
       </c>
       <c r="E172" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/03/pico-y-placa-medellin-evita-multas-este-miercoles-3-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/03/resultado-super-astro-luna-hoy-numero-ganador-del-martes-2-de-junio/</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 12:00 a. m.</t>
+          <t>02/06/2026 06:23 p. m.</t>
         </is>
       </c>
       <c r="B173" s="5" t="inlineStr">
@@ -5106,24 +5110,24 @@
       </c>
       <c r="C173" s="5" t="inlineStr">
         <is>
-          <t>Infobae Colombia</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D173" s="6" t="inlineStr">
         <is>
-          <t>Ataque con dron en El Tarra deja un muerto y agrava crisis humanitaria en Catatumbo: Defensoría alerta 784 desplazados</t>
+          <t>Juzgado ordena a Abelardo de la Espriella retractarse por comentarios a periodista por foto de su entrepierna</t>
         </is>
       </c>
       <c r="E173" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/03/ataque-con-dron-en-el-tarra-deja-un-muerto-y-agrava-crisis-humanitaria-en-catatumbo-defensoria-alerta-784-desplazados/</t>
+          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/juzgado-ordena-a-abelardo-de-la-espriella-retractarse-por-comentarios-a-periodista-por-foto-de-su-entrepierna</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 12:00 a. m.</t>
+          <t>02/06/2026 05:41 p. m.</t>
         </is>
       </c>
       <c r="B174" s="2" t="inlineStr">
@@ -5133,24 +5137,24 @@
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>Infobae Colombia</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D174" s="3" t="inlineStr">
         <is>
-          <t>Camiseta de la selección Colombia, otra vez en el centro del debate: creadora de contenido hizo su versión rococó del atuendo oficial</t>
+          <t>Fitch Ratings mantiene preocupaciones por la situación fiscal que heredará el próximo presidente. ¿Qué alertas hay?</t>
         </is>
       </c>
       <c r="E174" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/03/camiseta-de-la-seleccion-colombia-otra-vez-en-el-centro-del-debate-creadora-de-contenido-hizo-su-version-rococo-del-atuendo-oficial/</t>
+          <t>https://cambiocolombia.com/economia/articulo/2026/6/fitch-ratings-mantiene-preocupaciones-por-la-situacion-fiscal-que-heredara-el-proximo-presidente-que-alertas-hay</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 12:00 a. m.</t>
+          <t>02/06/2026 05:30 p. m.</t>
         </is>
       </c>
       <c r="B175" s="5" t="inlineStr">
@@ -5160,24 +5164,24 @@
       </c>
       <c r="C175" s="5" t="inlineStr">
         <is>
-          <t>Infobae Colombia</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D175" s="6" t="inlineStr">
         <is>
-          <t>Caribeña Noche: resultados ganadores del sorteo del lunes 1 de junio</t>
+          <t>Rama Judicial: "El escrutinio electoral se adelanta con independencia y rigor"</t>
         </is>
       </c>
       <c r="E175" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/03/caribena-noche-resultado-del-ultimo-sorteo-hoy-miercoles-3-de-junio/</t>
+          <t>https://cambiocolombia.com/poder/articulo/2026/6/rama-judicial-el-escrutinio-electoral-se-adelanta-con-independencia-y-rigor</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 06:23 p. m.</t>
+          <t>02/06/2026 04:00 p. m.</t>
         </is>
       </c>
       <c r="B176" s="2" t="inlineStr">
@@ -5192,19 +5196,19 @@
       </c>
       <c r="D176" s="3" t="inlineStr">
         <is>
-          <t>Juzgado ordena a Abelardo de la Espriella retractarse por comentarios a periodista por foto de su entrepierna</t>
+          <t>Procuraduría suspendió a Carlos Carrillo, director de la UNGRD, por presunta participación en política</t>
         </is>
       </c>
       <c r="E176" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/juzgado-ordena-a-abelardo-de-la-espriella-retractarse-por-comentarios-a-periodista-por-foto-de-su-entrepierna</t>
+          <t>https://cambiocolombia.com/poder/articulo/2026/6/procuraduria-suspendio-a-carlos-carrillo-director-de-la-ungrd-por-presunta-participacion-en-politica</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 05:41 p. m.</t>
+          <t>02/06/2026 01:45 p. m.</t>
         </is>
       </c>
       <c r="B177" s="5" t="inlineStr">
@@ -5219,19 +5223,19 @@
       </c>
       <c r="D177" s="6" t="inlineStr">
         <is>
-          <t>Fitch Ratings mantiene preocupaciones por la situación fiscal que heredará el próximo presidente. ¿Qué alertas hay?</t>
+          <t>Las fallas que la SIC vio en Tiendas Ara que estarían afectando a sus usuarios</t>
         </is>
       </c>
       <c r="E177" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/economia/articulo/2026/6/fitch-ratings-mantiene-preocupaciones-por-la-situacion-fiscal-que-heredara-el-proximo-presidente-que-alertas-hay</t>
+          <t>https://cambiocolombia.com/empresas/articulo/2026/6/las-fallas-que-la-sic-vio-en-tiendas-ara-que-estarian-afectando-a-sus-usuarios</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 05:30 p. m.</t>
+          <t>02/06/2026 11:15 a. m.</t>
         </is>
       </c>
       <c r="B178" s="2" t="inlineStr">
@@ -5246,19 +5250,19 @@
       </c>
       <c r="D178" s="3" t="inlineStr">
         <is>
-          <t>Rama Judicial: "El escrutinio electoral se adelanta con independencia y rigor"</t>
+          <t>Escrutinio coincide en 99,94 por ciento con el preconteo de la primera vuelta presidencial de 2026: Registraduría</t>
         </is>
       </c>
       <c r="E178" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/poder/articulo/2026/6/rama-judicial-el-escrutinio-electoral-se-adelanta-con-independencia-y-rigor</t>
+          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/escrutinio-coincide-en-9994-por-ciento-con-el-preconteo-de-la-primera-vuelta-presidencial-de-2026-registraduria</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 04:00 p. m.</t>
+          <t>02/06/2026 10:00 a. m.</t>
         </is>
       </c>
       <c r="B179" s="5" t="inlineStr">
@@ -5273,19 +5277,19 @@
       </c>
       <c r="D179" s="6" t="inlineStr">
         <is>
-          <t>Procuraduría suspendió a Carlos Carrillo, director de la UNGRD, por presunta participación en política</t>
+          <t>Petro insiste en el fraude pese a que Iván Cepeda se apartó de esa idea: ¿qué dijo el presidente?</t>
         </is>
       </c>
       <c r="E179" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/poder/articulo/2026/6/procuraduria-suspendio-a-carlos-carrillo-director-de-la-ungrd-por-presunta-participacion-en-politica</t>
+          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/petro-insiste-en-el-fraude-pese-a-que-ivan-cepeda-se-aparto-de-esa-idea-que-dijo-el-presidente</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 01:45 p. m.</t>
+          <t>02/06/2026 07:00 a. m.</t>
         </is>
       </c>
       <c r="B180" s="2" t="inlineStr">
@@ -5300,19 +5304,19 @@
       </c>
       <c r="D180" s="3" t="inlineStr">
         <is>
-          <t>Las fallas que la SIC vio en Tiendas Ara que estarían afectando a sus usuarios</t>
+          <t>Suspenden a Alfredo Saade por participación en política: el pastor le había pedido a Petro renunciar a su cargo</t>
         </is>
       </c>
       <c r="E180" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/empresas/articulo/2026/6/las-fallas-que-la-sic-vio-en-tiendas-ara-que-estarian-afectando-a-sus-usuarios</t>
+          <t>https://cambiocolombia.com/poder/articulo/2026/6/suspenden-a-alfredo-saade-por-participacion-en-politica-el-pastor-le-habia-pedido-a-petro-renunciar-a-su-cargo</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 11:15 a. m.</t>
+          <t>02/06/2026 06:00 a. m.</t>
         </is>
       </c>
       <c r="B181" s="5" t="inlineStr">
@@ -5327,19 +5331,19 @@
       </c>
       <c r="D181" s="6" t="inlineStr">
         <is>
-          <t>Escrutinio coincide en 99,94 por ciento con el preconteo de la primera vuelta presidencial de 2026: Registraduría</t>
+          <t>Murió el rector de la Universidad Militar, el general retirado Javier Ayala</t>
         </is>
       </c>
       <c r="E181" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/escrutinio-coincide-en-9994-por-ciento-con-el-preconteo-de-la-primera-vuelta-presidencial-de-2026-registraduria</t>
+          <t>https://cambiocolombia.com/pais/articulo/2026/6/murio-el-rector-de-la-universidad-militar-el-general-retirado-javier-ayala</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 10:00 a. m.</t>
+          <t>01/06/2026 05:30 p. m.</t>
         </is>
       </c>
       <c r="B182" s="2" t="inlineStr">
@@ -5354,19 +5358,19 @@
       </c>
       <c r="D182" s="3" t="inlineStr">
         <is>
-          <t>Petro insiste en el fraude pese a que Iván Cepeda se apartó de esa idea: ¿qué dijo el presidente?</t>
+          <t>La tierna carta de un niño para despedir a su padre, enviado al Sinaí para continuar su carrera militar</t>
         </is>
       </c>
       <c r="E182" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/petro-insiste-en-el-fraude-pese-a-que-ivan-cepeda-se-aparto-de-esa-idea-que-dijo-el-presidente</t>
+          <t>https://cambiocolombia.com/pais/articulo/2026/6/la-tierna-carta-de-un-nino-para-despedir-a-su-padre-enviado-al-sinai-para-continuar-su-carrera-militar</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="5" t="inlineStr">
         <is>
-          <t>02/06/2026 07:00 a. m.</t>
+          <t>01/06/2026 04:30 p. m.</t>
         </is>
       </c>
       <c r="B183" s="5" t="inlineStr">
@@ -5381,19 +5385,19 @@
       </c>
       <c r="D183" s="6" t="inlineStr">
         <is>
-          <t>Suspenden a Alfredo Saade por participación en política: el pastor le había pedido a Petro renunciar a su cargo</t>
+          <t>La FCF responde a Cepeda: no puede impedir uso electoral de la camiseta de la selección, pero piden evitarlo</t>
         </is>
       </c>
       <c r="E183" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/poder/articulo/2026/6/suspenden-a-alfredo-saade-por-participacion-en-politica-el-pastor-le-habia-pedido-a-petro-renunciar-a-su-cargo</t>
+          <t>https://cambiocolombia.com/pais/articulo/2026/6/la-fcf-responde-a-cepeda-no-puede-impedir-uso-electoral-de-la-camiseta-de-la-seleccion-pero-piden-evitarlo</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 06:00 a. m.</t>
+          <t>01/06/2026 03:30 p. m.</t>
         </is>
       </c>
       <c r="B184" s="2" t="inlineStr">
@@ -5408,19 +5412,19 @@
       </c>
       <c r="D184" s="3" t="inlineStr">
         <is>
-          <t>Murió el rector de la Universidad Militar, el general retirado Javier Ayala</t>
+          <t>Ministerio de Salud elimina Mipres para medicamentos UPC: ¿qué cambió?</t>
         </is>
       </c>
       <c r="E184" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/pais/articulo/2026/6/murio-el-rector-de-la-universidad-militar-el-general-retirado-javier-ayala</t>
+          <t>https://cambiocolombia.com/salud-y-bienestar/articulo/2026/6/ministerio-de-salud-elimina-mipres-para-medicamentos-upc-que-cambio</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 05:30 p. m.</t>
+          <t>01/06/2026 02:46 p. m.</t>
         </is>
       </c>
       <c r="B185" s="5" t="inlineStr">
@@ -5435,19 +5439,19 @@
       </c>
       <c r="D185" s="6" t="inlineStr">
         <is>
-          <t>La tierna carta de un niño para despedir a su padre, enviado al Sinaí para continuar su carrera militar</t>
+          <t>Las sanciones que enfrentaría el operador de la lancha donde murió Alexander Avendaño en Guatapé</t>
         </is>
       </c>
       <c r="E185" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/pais/articulo/2026/6/la-tierna-carta-de-un-nino-para-despedir-a-su-padre-enviado-al-sinai-para-continuar-su-carrera-militar</t>
+          <t>https://cambiocolombia.com/pais/articulo/2026/6/las-sanciones-que-enfrentaria-el-operador-de-la-lancha-donde-murio-alexander-avendano-en-guatape</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 04:30 p. m.</t>
+          <t>01/06/2026 02:00 p. m.</t>
         </is>
       </c>
       <c r="B186" s="2" t="inlineStr">
@@ -5462,21 +5466,17 @@
       </c>
       <c r="D186" s="3" t="inlineStr">
         <is>
-          <t>La FCF responde a Cepeda: no puede impedir uso electoral de la camiseta de la selección, pero piden evitarlo</t>
+          <t>Cuatro personas murieron en un accidente de avioneta en la ruta Villavicencio – La Macarena</t>
         </is>
       </c>
       <c r="E186" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/pais/articulo/2026/6/la-fcf-responde-a-cepeda-no-puede-impedir-uso-electoral-de-la-camiseta-de-la-seleccion-pero-piden-evitarlo</t>
+          <t>https://cambiocolombia.com/pais/articulo/2026/6/cuatro-personas-murieron-en-un-accidente-de-avioneta-en-la-ruta-villavicencio-la-macarena</t>
         </is>
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="5" t="inlineStr">
-        <is>
-          <t>01/06/2026 03:30 p. m.</t>
-        </is>
-      </c>
+      <c r="A187" s="5" t="inlineStr"/>
       <c r="B187" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5484,26 +5484,22 @@
       </c>
       <c r="C187" s="5" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D187" s="6" t="inlineStr">
         <is>
-          <t>Ministerio de Salud elimina Mipres para medicamentos UPC: ¿qué cambió?</t>
+          <t>“Es un honor brindarle mi respaldo total”: Donald Trump felicitó a Abelardo de la Espriella tras imponerse en la primera vuelta</t>
         </is>
       </c>
       <c r="E187" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/salud-y-bienestar/articulo/2026/6/ministerio-de-salud-elimina-mipres-para-medicamentos-upc-que-cambio</t>
+          <t>https://www.elcolombiano.com/colombia/respaldo-total-donald-trump-abelardo-de-la-espriella-elecciones-colombia-2026-PP37291680</t>
         </is>
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="2" t="inlineStr">
-        <is>
-          <t>01/06/2026 02:46 p. m.</t>
-        </is>
-      </c>
+      <c r="A188" s="2" t="inlineStr"/>
       <c r="B188" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5511,26 +5507,22 @@
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D188" s="3" t="inlineStr">
         <is>
-          <t>Las sanciones que enfrentaría el operador de la lancha donde murió Alexander Avendaño en Guatapé</t>
+          <t>Como en 2004, Nacional tocó fondo en la ida de la final ante Junior y el Atanasio espera una remontada épica por la estrella 19</t>
         </is>
       </c>
       <c r="E188" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/pais/articulo/2026/6/las-sanciones-que-enfrentaria-el-operador-de-la-lancha-donde-murio-alexander-avendano-en-guatape</t>
+          <t>https://www.elcolombiano.com/deportes/futbol/nacional-junior-en-vivo-ida-final-liga-betplay-minuto-a-minuto-online-television-nominas-PO37286696</t>
         </is>
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="5" t="inlineStr">
-        <is>
-          <t>01/06/2026 02:00 p. m.</t>
-        </is>
-      </c>
+      <c r="A189" s="5" t="inlineStr"/>
       <c r="B189" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5538,17 +5530,17 @@
       </c>
       <c r="C189" s="5" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D189" s="6" t="inlineStr">
         <is>
-          <t>Cuatro personas murieron en un accidente de avioneta en la ruta Villavicencio – La Macarena</t>
+          <t>Encuesta AtlasIntel: Abelardo de la Espriella lidera la segunda vuelta con 50,3 % de intención de voto ante Iván Cepeda con 42,6 %</t>
         </is>
       </c>
       <c r="E189" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/pais/articulo/2026/6/cuatro-personas-murieron-en-un-accidente-de-avioneta-en-la-ruta-villavicencio-la-macarena</t>
+          <t>https://www.elcolombiano.com/colombia/encuesta-atlasintel-abelardo-de-la-espriella-lidera-segunda-vuelta-ivan-cepeda-DO37287994</t>
         </is>
       </c>
     </row>
@@ -5566,12 +5558,12 @@
       </c>
       <c r="D190" s="3" t="inlineStr">
         <is>
-          <t>“Es un honor brindarle mi respaldo total”: Donald Trump felicitó a Abelardo de la Espriella tras imponerse en la primera vuelta</t>
+          <t>Identificaron a 43 de los 48 cuerpos del enfrentamiento de disidencias en Guaviare; 11 eran menores de edad</t>
         </is>
       </c>
       <c r="E190" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/respaldo-total-donald-trump-abelardo-de-la-espriella-elecciones-colombia-2026-PP37291680</t>
+          <t>https://www.elcolombiano.com/colombia/medicina-legal-identifica-43-cuerpos-san-jose-del-guaviare-11-menores-edad-MP37293852</t>
         </is>
       </c>
     </row>
@@ -5589,12 +5581,12 @@
       </c>
       <c r="D191" s="6" t="inlineStr">
         <is>
-          <t>Como en 2004, Nacional tocó fondo en la ida de la final ante Junior y el Atanasio espera una remontada épica por la estrella 19</t>
+          <t>Elecciones 2026: Centro Carter pidió respetar resultados y elogió sistema electoral</t>
         </is>
       </c>
       <c r="E191" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/deportes/futbol/nacional-junior-en-vivo-ida-final-liga-betplay-minuto-a-minuto-online-television-nominas-PO37286696</t>
+          <t>https://www.elcolombiano.com/colombia/politica/elecciones-2026-centro-carter-pidio-respetar-resultados-elogio-sistema-electoral-PO37288564</t>
         </is>
       </c>
     </row>
@@ -5612,12 +5604,12 @@
       </c>
       <c r="D192" s="3" t="inlineStr">
         <is>
-          <t>Encuesta AtlasIntel: Abelardo de la Espriella lidera la segunda vuelta con 50,3 % de intención de voto ante Iván Cepeda con 42,6 %</t>
+          <t>Iván Cepeda desbloqueó a Teleantioquia en X tras denuncias de censura del canal</t>
         </is>
       </c>
       <c r="E192" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/encuesta-atlasintel-abelardo-de-la-espriella-lidera-segunda-vuelta-ivan-cepeda-DO37287994</t>
+          <t>https://www.elcolombiano.com/antioquia/teleantioquia-denuncia-censura-ivan-cepeda-bloqueo-redes-sociales-EB37270523</t>
         </is>
       </c>
     </row>
@@ -5635,12 +5627,12 @@
       </c>
       <c r="D193" s="6" t="inlineStr">
         <is>
-          <t>Identificaron a 43 de los 48 cuerpos del enfrentamiento de disidencias en Guaviare; 11 eran menores de edad</t>
+          <t>Juzgado le ordena a De la Espriella retractarse y ofrecer disculpas a periodista por comentarios misóginos en una entrevista</t>
         </is>
       </c>
       <c r="E193" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/medicina-legal-identifica-43-cuerpos-san-jose-del-guaviare-11-menores-edad-MP37293852</t>
+          <t>https://www.elcolombiano.com/colombia/abelardo-de-la-espriella-juzgado-retractarse-ofrecer-disculpas-periodista-comentarios-misoginos-entrevista-PO37285578</t>
         </is>
       </c>
     </row>
@@ -5658,12 +5650,12 @@
       </c>
       <c r="D194" s="3" t="inlineStr">
         <is>
-          <t>Elecciones 2026: Centro Carter pidió respetar resultados y elogió sistema electoral</t>
+          <t>Van 7 altos funcionarios, incluido Petro, suspendidos o investigados por presunta participación en política</t>
         </is>
       </c>
       <c r="E194" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/politica/elecciones-2026-centro-carter-pidio-respetar-resultados-elogio-sistema-electoral-PO37288564</t>
+          <t>https://www.elcolombiano.com/especiales/elecciones-2026/elecciones-2026-gustavo-petro-procuraduria-suspension-saade-carrillo-GB37271315</t>
         </is>
       </c>
     </row>
@@ -5681,12 +5673,12 @@
       </c>
       <c r="D195" s="6" t="inlineStr">
         <is>
-          <t>Iván Cepeda desbloqueó a Teleantioquia en X tras denuncias de censura del canal</t>
+          <t>Operativo destapa helicóptero con pasado oscuro y motor Rolls-Royce</t>
         </is>
       </c>
       <c r="E195" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/antioquia/teleantioquia-denuncia-censura-ivan-cepeda-bloqueo-redes-sociales-EB37270523</t>
+          <t>https://www.elcolombiano.com/colombia/ejercito-incauta-helicoptero-de-la-mafia-NG33717192</t>
         </is>
       </c>
     </row>
@@ -5704,12 +5696,12 @@
       </c>
       <c r="D196" s="3" t="inlineStr">
         <is>
-          <t>Juzgado le ordena a De la Espriella retractarse y ofrecer disculpas a periodista por comentarios misóginos en una entrevista</t>
+          <t>De la alegría al desconsuelo: así se vivió la final de ida entre Nacional y Junior en las calles de Medellín</t>
         </is>
       </c>
       <c r="E196" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/abelardo-de-la-espriella-juzgado-retractarse-ofrecer-disculpas-periodista-comentarios-misoginos-entrevista-PO37285578</t>
+          <t>https://www.elcolombiano.com/deportes/futbol/final-nacional-vs-junior-liga-betplay-2026-como-se-vivio-en-medellin-FP37295541</t>
         </is>
       </c>
     </row>
@@ -5727,12 +5719,12 @@
       </c>
       <c r="D197" s="6" t="inlineStr">
         <is>
-          <t>Van 7 altos funcionarios, incluido Petro, suspendidos o investigados por presunta participación en política</t>
+          <t>Tras estudios, árbol centenario de Ciudad Bolívar fue talado ¿Por qué?</t>
         </is>
       </c>
       <c r="E197" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/elecciones-2026/elecciones-2026-gustavo-petro-procuraduria-suspension-saade-carrillo-GB37271315</t>
+          <t>https://www.elcolombiano.com/antioquia/talan-arbol-centenario-ciudad-bolivar-antioquia-CP37292055</t>
         </is>
       </c>
     </row>
@@ -5750,12 +5742,12 @@
       </c>
       <c r="D198" s="3" t="inlineStr">
         <is>
-          <t>Operativo destapa helicóptero con pasado oscuro y motor Rolls-Royce</t>
+          <t>La ciencia explica por qué hay más mujeres ansiosas y depresivas que hombres, ¿cómo actuar?</t>
         </is>
       </c>
       <c r="E198" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/ejercito-incauta-helicoptero-de-la-mafia-NG33717192</t>
+          <t>https://www.elcolombiano.com/tendencias/ansiedad-depresion-mujeres-por-que-FO37288629</t>
         </is>
       </c>
     </row>
@@ -5773,12 +5765,12 @@
       </c>
       <c r="D199" s="6" t="inlineStr">
         <is>
-          <t>De la alegría al desconsuelo: así se vivió la final de ida entre Nacional y Junior en las calles de Medellín</t>
+          <t>Estos son los elegidos de Uzbekistán para jugar el Mundial, el país que no existía hace 32 años contra el que debutará Colombia</t>
         </is>
       </c>
       <c r="E199" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/deportes/futbol/final-nacional-vs-junior-liga-betplay-2026-como-se-vivio-en-medellin-FP37295541</t>
+          <t>https://www.elcolombiano.com/deportes/futbol/convocados-seleccion-uzbekistan-mundial-norteamerica-2026-debut-vs-colombia-estadio-azteca-mexico-BO37285675</t>
         </is>
       </c>
     </row>
@@ -5796,12 +5788,12 @@
       </c>
       <c r="D200" s="3" t="inlineStr">
         <is>
-          <t>Tras estudios, árbol centenario de Ciudad Bolívar fue talado ¿Por qué?</t>
+          <t>Video | La justificación de la Policía por uso de fuerza contra músico callejero tras denuncias en Parque La Colina en Bogotá</t>
         </is>
       </c>
       <c r="E200" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/antioquia/talan-arbol-centenario-ciudad-bolivar-antioquia-CP37292055</t>
+          <t>https://www.elcolombiano.com/colombia/video-policia-justifica-uso-fuerza-musico-callejero-denunciasruido-bogota-AO37286161</t>
         </is>
       </c>
     </row>
@@ -5819,12 +5811,12 @@
       </c>
       <c r="D201" s="6" t="inlineStr">
         <is>
-          <t>La ciencia explica por qué hay más mujeres ansiosas y depresivas que hombres, ¿cómo actuar?</t>
+          <t>Concejo de Medellín inicia sesiones ordinarias, ¿por qué la revisión del POT será esencial?</t>
         </is>
       </c>
       <c r="E201" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/tendencias/ansiedad-depresion-mujeres-por-que-FO37288629</t>
+          <t>https://www.elcolombiano.com/medellin/inicio-sesiones-concejo-medellin-discusion-pot-MO37286864</t>
         </is>
       </c>
     </row>
@@ -5842,12 +5834,12 @@
       </c>
       <c r="D202" s="3" t="inlineStr">
         <is>
-          <t>Estos son los elegidos de Uzbekistán para jugar el Mundial, el país que no existía hace 32 años contra el que debutará Colombia</t>
+          <t>Mundial 2026: Un total de 289 futbolistas no portarán la camiseta del país donde nacieron, ¿qué selección tiene 25 nacionalizados?</t>
         </is>
       </c>
       <c r="E202" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/deportes/futbol/convocados-seleccion-uzbekistan-mundial-norteamerica-2026-debut-vs-colombia-estadio-azteca-mexico-BO37285675</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/mundial-2026-jugadores-nacionalizados-de-40-selecciones-olise-hakimi-DO37285161</t>
         </is>
       </c>
     </row>
@@ -5865,12 +5857,12 @@
       </c>
       <c r="D203" s="6" t="inlineStr">
         <is>
-          <t>Video | La justificación de la Policía por uso de fuerza contra músico callejero tras denuncias en Parque La Colina en Bogotá</t>
+          <t>Talento y juventud: las nuevas figuras que se estrenarán en el Mundial de Norteamérica 2026</t>
         </is>
       </c>
       <c r="E203" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/video-policia-justifica-uso-fuerza-musico-callejero-denunciasruido-bogota-AO37286161</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/nuevas-figuras-que-se-estrenaran-mundial-norteamerica-2026-IB37274972</t>
         </is>
       </c>
     </row>
@@ -5888,12 +5880,12 @@
       </c>
       <c r="D204" s="3" t="inlineStr">
         <is>
-          <t>Concejo de Medellín inicia sesiones ordinarias, ¿por qué la revisión del POT será esencial?</t>
+          <t>Tesla instala en Medellín la primera estación de sus “supercargadores” en Colombia ¿Dónde estará?</t>
         </is>
       </c>
       <c r="E204" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/medellin/inicio-sesiones-concejo-medellin-discusion-pot-MO37286864</t>
+          <t>https://www.elcolombiano.com/medellin/supercargadores-tesla-medellin-unicentro-CO37284710</t>
         </is>
       </c>
     </row>
@@ -5911,12 +5903,12 @@
       </c>
       <c r="D205" s="6" t="inlineStr">
         <is>
-          <t>Mundial 2026: Un total de 289 futbolistas no portarán la camiseta del país donde nacieron, ¿qué selección tiene 25 nacionalizados?</t>
+          <t>Forbes revela el ranking de los clubes más ricos del planeta y Real Madrid arrasa</t>
         </is>
       </c>
       <c r="E205" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/mundial-2026/mundial-2026-jugadores-nacionalizados-de-40-selecciones-olise-hakimi-DO37285161</t>
+          <t>https://www.elcolombiano.com/deportes/futbol/ranking-clubes-mas-ricos-mundo-revista-forbes-2026-PO37284290</t>
         </is>
       </c>
     </row>
@@ -5934,12 +5926,12 @@
       </c>
       <c r="D206" s="3" t="inlineStr">
         <is>
-          <t>Talento y juventud: las nuevas figuras que se estrenarán en el Mundial de Norteamérica 2026</t>
+          <t>Bombazo en Nacional: Franco Armani tiene vía libre para regresar</t>
         </is>
       </c>
       <c r="E206" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/mundial-2026/nuevas-figuras-que-se-estrenaran-mundial-norteamerica-2026-IB37274972</t>
+          <t>https://www.elcolombiano.com/deportes/futbol/regresa-franco-armani-a-atletico-nacional-IO37280109</t>
         </is>
       </c>
     </row>
@@ -5957,12 +5949,12 @@
       </c>
       <c r="D207" s="6" t="inlineStr">
         <is>
-          <t>Tesla instala en Medellín la primera estación de sus “supercargadores” en Colombia ¿Dónde estará?</t>
+          <t>¿Machismo en “La casita” de Bad Bunny? Hay polémica por las mujeres elegidas</t>
         </is>
       </c>
       <c r="E207" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/medellin/supercargadores-tesla-medellin-unicentro-CO37284710</t>
+          <t>https://www.elcolombiano.com/tendencias/machismo-casita-bad-bunny-polemica-mujeres-seleccionadas-EB37276736</t>
         </is>
       </c>
     </row>
@@ -5980,12 +5972,12 @@
       </c>
       <c r="D208" s="3" t="inlineStr">
         <is>
-          <t>Forbes revela el ranking de los clubes más ricos del planeta y Real Madrid arrasa</t>
+          <t>DIM venció a Cúcuta en Ditaires y clasificó a octavos de final de la Copa BetPlay: terminó el semestre con rendimiento de 39,3%</t>
         </is>
       </c>
       <c r="E208" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/deportes/futbol/ranking-clubes-mas-ricos-mundo-revista-forbes-2026-PO37284290</t>
+          <t>https://www.elcolombiano.com/deportes/futbol/dim-vs-cucuta-deportivo-copa-betplay-2026-fase-de-grupos-EO37283887</t>
         </is>
       </c>
     </row>
@@ -6003,12 +5995,12 @@
       </c>
       <c r="D209" s="6" t="inlineStr">
         <is>
-          <t>Bombazo en Nacional: Franco Armani tiene vía libre para regresar</t>
+          <t>Colombia está en el podio de las selecciones más “longevas” del Mundial 2026, ¿cuáles son las más veteranas y las más jóvenes?</t>
         </is>
       </c>
       <c r="E209" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/deportes/futbol/regresa-franco-armani-a-atletico-nacional-IO37280109</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/ranking-selecciones-mas-veteranas-mundial-norteamerica-2026-seleccion-colombia-BO37280607</t>
         </is>
       </c>
     </row>
@@ -6026,12 +6018,12 @@
       </c>
       <c r="D210" s="3" t="inlineStr">
         <is>
-          <t>¿Machismo en “La casita” de Bad Bunny? Hay polémica por las mujeres elegidas</t>
+          <t>Quintero resucitó a cuestionado exdirector del Hospital General de Medellín como interventor de Asmet Salud</t>
         </is>
       </c>
       <c r="E210" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/tendencias/machismo-casita-bad-bunny-polemica-mujeres-seleccionadas-EB37276736</t>
+          <t>https://www.elcolombiano.com/medellin/daniel-quintero-nombra-a-exgerente-del-hospital-general-en-asmet-salud-PO37282782</t>
         </is>
       </c>
     </row>
@@ -6049,12 +6041,12 @@
       </c>
       <c r="D211" s="6" t="inlineStr">
         <is>
-          <t>DIM venció a Cúcuta en Ditaires y clasificó a octavos de final de la Copa BetPlay: terminó el semestre con rendimiento de 39,3%</t>
+          <t>Colombia ya tiene dorsales para el Mundial 2026: James seguirá con el 10 y Luis Díaz lucirá el 7</t>
         </is>
       </c>
       <c r="E211" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/deportes/futbol/dim-vs-cucuta-deportivo-copa-betplay-2026-fase-de-grupos-EO37283887</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/dorsales-numeros-camisetas-jugadores-seleccion-colombia-mundial-2026-FO37281455</t>
         </is>
       </c>
     </row>
@@ -6072,12 +6064,12 @@
       </c>
       <c r="D212" s="3" t="inlineStr">
         <is>
-          <t>Colombia está en el podio de las selecciones más “longevas” del Mundial 2026, ¿cuáles son las más veteranas y las más jóvenes?</t>
+          <t>Ni tan caros ni tan contaminantes: estudio del MIT reveló que los carros eléctricos son incluso más asequibles que los de gasolina</t>
         </is>
       </c>
       <c r="E212" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/mundial-2026/ranking-selecciones-mas-veteranas-mundial-norteamerica-2026-seleccion-colombia-BO37280607</t>
+          <t>https://www.elcolombiano.com/negocios/mit-carros-electricos-mas-baratos-gasolina-estudio-PA37266854</t>
         </is>
       </c>
     </row>
@@ -6095,12 +6087,12 @@
       </c>
       <c r="D213" s="6" t="inlineStr">
         <is>
-          <t>Quintero resucitó a cuestionado exdirector del Hospital General de Medellín como interventor de Asmet Salud</t>
+          <t>Medellín busca que el tango haga parte del Patrimonio Cultural Inmaterial Distrital, ¿qué significa eso?</t>
         </is>
       </c>
       <c r="E213" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/medellin/daniel-quintero-nombra-a-exgerente-del-hospital-general-en-asmet-salud-PO37282782</t>
+          <t>https://www.elcolombiano.com/cultura/tango-patrimonio-cultural-medellin-festival-manrique-BB37276610</t>
         </is>
       </c>
     </row>
@@ -6118,12 +6110,12 @@
       </c>
       <c r="D214" s="3" t="inlineStr">
         <is>
-          <t>Colombia ya tiene dorsales para el Mundial 2026: James seguirá con el 10 y Luis Díaz lucirá el 7</t>
+          <t>Paloma invitó a café a Oviedo, López y Fajardo: “Colombia está al borde del abismo”</t>
         </is>
       </c>
       <c r="E214" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/mundial-2026/dorsales-numeros-camisetas-jugadores-seleccion-colombia-mundial-2026-FO37281455</t>
+          <t>https://www.elcolombiano.com/colombia/politica/paloma-valencia-invita-cafe-juan-daniel-oviedo-claudia-lopez-sergio-fajardo-HB37275174</t>
         </is>
       </c>
     </row>
@@ -6141,12 +6133,12 @@
       </c>
       <c r="D215" s="6" t="inlineStr">
         <is>
-          <t>Ni tan caros ni tan contaminantes: estudio del MIT reveló que los carros eléctricos son incluso más asequibles que los de gasolina</t>
+          <t>El artículo de The Economist que ve como ganador a De la Espriella frente al continuismo de Petro</t>
         </is>
       </c>
       <c r="E215" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/negocios/mit-carros-electricos-mas-baratos-gasolina-estudio-PA37266854</t>
+          <t>https://www.elcolombiano.com/colombia/the-economist-ve-ganador-abelardo-de-la-espriella-elecciones-presidenciales-2026-HO37285299</t>
         </is>
       </c>
     </row>
@@ -6164,12 +6156,12 @@
       </c>
       <c r="D216" s="3" t="inlineStr">
         <is>
-          <t>Medellín busca que el tango haga parte del Patrimonio Cultural Inmaterial Distrital, ¿qué significa eso?</t>
+          <t>Ante la polémica de la primera vuelta, Alcaldía de Medellín pidió reubicar puesto de votación del C.C. Sandiego ¿Para dónde?</t>
         </is>
       </c>
       <c r="E216" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/cultura/tango-patrimonio-cultural-medellin-festival-manrique-BB37276610</t>
+          <t>https://www.elcolombiano.com/medellin/alcaldia-de-medellin-pidio-traslado-mesa-de-votacion-centro-comercial-san-diego-HO37288825</t>
         </is>
       </c>
     </row>
@@ -6182,17 +6174,17 @@
       </c>
       <c r="C217" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D217" s="6" t="inlineStr">
         <is>
-          <t>Paloma invitó a café a Oviedo, López y Fajardo: “Colombia está al borde del abismo”</t>
+          <t>Primera entrevista de Abelardo De La Espriella tras la primera vuelta</t>
         </is>
       </c>
       <c r="E217" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/politica/paloma-valencia-invita-cafe-juan-daniel-oviedo-claudia-lopez-sergio-fajardo-HB37275174</t>
+          <t>https://www.semana.com/semana-tv/semana-noticias/articulo/en-vivo-primera-entrevista-de-abelardo-de-la-espriella-tras-la-primera-vuelta/202648/</t>
         </is>
       </c>
     </row>
@@ -6205,17 +6197,17 @@
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D218" s="3" t="inlineStr">
         <is>
-          <t>El artículo de The Economist que ve como ganador a De la Espriella frente al continuismo de Petro</t>
+          <t>SEMANA logra audiencia récord con entrevista a Abelardo de la Espriella: más de 1,6 millones de personas se conectaron</t>
         </is>
       </c>
       <c r="E218" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/the-economist-ve-ganador-abelardo-de-la-espriella-elecciones-presidenciales-2026-HO37285299</t>
+          <t>https://www.semana.com/confidenciales/articulo/semana-logra-audiencia-record-con-entrevista-a-abelardo-de-la-espriella-mas-de-16-millones-de-personas-se-conectaron/202644/</t>
         </is>
       </c>
     </row>
@@ -6228,17 +6220,17 @@
       </c>
       <c r="C219" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D219" s="6" t="inlineStr">
         <is>
-          <t>Ante la polémica de la primera vuelta, Alcaldía de Medellín pidió reubicar puesto de votación del C.C. Sandiego ¿Para dónde?</t>
+          <t>Abelardo de la Espriella hace graves señalamientos contra Armando Benedetti y revela para qué lo quieren en la campaña de Iván Cepeda</t>
         </is>
       </c>
       <c r="E219" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/medellin/alcaldia-de-medellin-pidio-traslado-mesa-de-votacion-centro-comercial-san-diego-HO37288825</t>
+          <t>https://www.semana.com/confidenciales/articulo/abelardo-de-la-espriella-hace-graves-senalamientos-contra-armando-benedetti-y-revela-para-que-lo-quieren-en-la-campana-de-ivan-cepeda/202657/</t>
         </is>
       </c>
     </row>
@@ -6256,12 +6248,12 @@
       </c>
       <c r="D220" s="3" t="inlineStr">
         <is>
-          <t>Primera entrevista de Abelardo De La Espriella tras la primera vuelta</t>
+          <t>Abelardo de la Espriella deja claras las intenciones de Gustavo Petro: “Se quiere robar las elecciones”</t>
         </is>
       </c>
       <c r="E220" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/semana-tv/semana-noticias/articulo/en-vivo-primera-entrevista-de-abelardo-de-la-espriella-tras-la-primera-vuelta/202648/</t>
+          <t>https://www.semana.com/politica/articulo/abelardo-de-la-espriella-deja-claras-las-intenciones-de-gustavo-petro-se-quiere-robar-las-elecciones/202619/</t>
         </is>
       </c>
     </row>
@@ -6279,12 +6271,12 @@
       </c>
       <c r="D221" s="6" t="inlineStr">
         <is>
-          <t>SEMANA logra audiencia récord con entrevista a Abelardo de la Espriella: más de 1,6 millones de personas se conectaron</t>
+          <t>Abelardo de la Espriella reacciona en SEMANA al respaldo de Donald Trump a su candidatura: “Compartimos valores y principios”</t>
         </is>
       </c>
       <c r="E221" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/confidenciales/articulo/semana-logra-audiencia-record-con-entrevista-a-abelardo-de-la-espriella-mas-de-16-millones-de-personas-se-conectaron/202644/</t>
+          <t>https://www.semana.com/politica/articulo/abelardo-de-la-espriella-reacciona-en-semana-al-respaldo-de-donald-trump-a-su-candidatura-compartimos-valores-y-principios/202608/</t>
         </is>
       </c>
     </row>
@@ -6302,12 +6294,12 @@
       </c>
       <c r="D222" s="3" t="inlineStr">
         <is>
-          <t>Abelardo de la Espriella hace graves señalamientos contra Armando Benedetti y revela para qué lo quieren en la campaña de Iván Cepeda</t>
+          <t>Presidente Gustavo Petro reaccionó al apoyo de Donald Trump a Abelardo de la Espriella: “Muere la libertad”</t>
         </is>
       </c>
       <c r="E222" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/confidenciales/articulo/abelardo-de-la-espriella-hace-graves-senalamientos-contra-armando-benedetti-y-revela-para-que-lo-quieren-en-la-campana-de-ivan-cepeda/202657/</t>
+          <t>https://www.semana.com/politica/articulo/presidente-gustavo-petro-reacciono-al-apoyo-de-donald-trump-a-abelardo-de-la-espriella-muere-la-libertad/202606/</t>
         </is>
       </c>
     </row>
@@ -6325,12 +6317,12 @@
       </c>
       <c r="D223" s="6" t="inlineStr">
         <is>
-          <t>Abelardo de la Espriella deja claras las intenciones de Gustavo Petro: “Se quiere robar las elecciones”</t>
+          <t>Abelardo de la Espriella alerta a los colombianos sobre “plan de Petro”: habla de lo que hay detrás del supuesto fraude del que habla el presidente</t>
         </is>
       </c>
       <c r="E223" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/abelardo-de-la-espriella-deja-claras-las-intenciones-de-gustavo-petro-se-quiere-robar-las-elecciones/202619/</t>
+          <t>https://www.semana.com/politica/articulo/abelardo-de-la-espriella-alerta-a-los-colombianos-sobre-plan-de-petro-dice-que-hay-detras-del-supuesto-fraude-del-que-habla-el-presidente/202651/</t>
         </is>
       </c>
     </row>
@@ -6348,12 +6340,12 @@
       </c>
       <c r="D224" s="3" t="inlineStr">
         <is>
-          <t>Abelardo de la Espriella reacciona en SEMANA al respaldo de Donald Trump a su candidatura: “Compartimos valores y principios”</t>
+          <t>“Lo de Petro es una vergüenza, sigue siendo un guerrillero, un bandido”: Abelardo de la Espriella se va con todo contra Gustavo Petro</t>
         </is>
       </c>
       <c r="E224" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/abelardo-de-la-espriella-reacciona-en-semana-al-respaldo-de-donald-trump-a-su-candidatura-compartimos-valores-y-principios/202608/</t>
+          <t>https://www.semana.com/politica/articulo/lo-de-petro-es-una-verguenza-sigue-siendo-un-guerrillero-un-bandido-abelardo-de-la-espriella-se-va-con-todo-contra-gustavo-petro/202645/</t>
         </is>
       </c>
     </row>
@@ -6371,12 +6363,12 @@
       </c>
       <c r="D225" s="6" t="inlineStr">
         <is>
-          <t>Presidente Gustavo Petro reaccionó al apoyo de Donald Trump a Abelardo de la Espriella: “Muere la libertad”</t>
+          <t>Ataques con drones y explosivos en el Catatumbo dejan este martes un soldado y un adulto mayor muertos y dos personas heridas</t>
         </is>
       </c>
       <c r="E225" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/presidente-gustavo-petro-reacciono-al-apoyo-de-donald-trump-a-abelardo-de-la-espriella-muere-la-libertad/202606/</t>
+          <t>https://www.semana.com/nacion/cucuta/articulo/ataques-con-drones-y-explosivos-en-el-catatumbo-dejan-este-martes-un-soldado-y-un-adulto-mayor-muertos-y-dos-personas-heridas/202649/</t>
         </is>
       </c>
     </row>
@@ -6394,12 +6386,12 @@
       </c>
       <c r="D226" s="3" t="inlineStr">
         <is>
-          <t>Abelardo de la Espriella alerta a los colombianos sobre “plan de Petro”: habla de lo que hay detrás del supuesto fraude del que habla el presidente</t>
+          <t>Junior se paseó a Nacional en la final de ida de la Liga BetPlay: el verde buscará el milagro en Medellín</t>
         </is>
       </c>
       <c r="E226" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/abelardo-de-la-espriella-alerta-a-los-colombianos-sobre-plan-de-petro-dice-que-hay-detras-del-supuesto-fraude-del-que-habla-el-presidente/202651/</t>
+          <t>https://www.semana.com/deportes/articulo/junior-se-paseo-a-nacional-en-la-final-de-ida-de-la-liga-betplay-el-verde-buscara-el-milagro-en-medellin/202632/</t>
         </is>
       </c>
     </row>
@@ -6417,12 +6409,12 @@
       </c>
       <c r="D227" s="6" t="inlineStr">
         <is>
-          <t>“Lo de Petro es una vergüenza, sigue siendo un guerrillero, un bandido”: Abelardo de la Espriella se va con todo contra Gustavo Petro</t>
+          <t>Sergio Fajardo da pistas de sus movimientos para la segunda vuelta presidencial: “El espíritu del millón de votos”</t>
         </is>
       </c>
       <c r="E227" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/lo-de-petro-es-una-verguenza-sigue-siendo-un-guerrillero-un-bandido-abelardo-de-la-espriella-se-va-con-todo-contra-gustavo-petro/202645/</t>
+          <t>https://www.semana.com/politica/articulo/sergio-fajardo-da-pistas-de-sus-movimientos-para-la-segunda-vuelta-presidencial-el-espiritu-del-millon-de-votos/202648/</t>
         </is>
       </c>
     </row>
@@ -6440,12 +6432,12 @@
       </c>
       <c r="D228" s="3" t="inlineStr">
         <is>
-          <t>Ataques con drones y explosivos en el Catatumbo dejan este martes un soldado y un adulto mayor muertos y dos personas heridas</t>
+          <t>Medicina Legal confirmó que entre los 48 muertos de San José de Guaviare hay 11 menores: esta es la lista de nombres de los cuerpos identificados</t>
         </is>
       </c>
       <c r="E228" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/cucuta/articulo/ataques-con-drones-y-explosivos-en-el-catatumbo-dejan-este-martes-un-soldado-y-un-adulto-mayor-muertos-y-dos-personas-heridas/202649/</t>
+          <t>https://www.semana.com/nacion/florencia/articulo/medicina-legal-confirmo-que-entre-los-48-muertos-de-san-jose-de-guaviare-hay-11-menores-esta-es-la-lista-de-nombres-de-los-cuerpos-identificados/202622/</t>
         </is>
       </c>
     </row>
@@ -6463,12 +6455,12 @@
       </c>
       <c r="D229" s="6" t="inlineStr">
         <is>
-          <t>Junior se paseó a Nacional en la final de ida de la Liga BetPlay: el verde buscará el milagro en Medellín</t>
+          <t>Punto por punto, la Registraduría desmiente a Gustavo Petro y evidencia por qué no es cierto el supuesto fraude electoral</t>
         </is>
       </c>
       <c r="E229" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/junior-se-paseo-a-nacional-en-la-final-de-ida-de-la-liga-betplay-el-verde-buscara-el-milagro-en-medellin/202632/</t>
+          <t>https://www.semana.com/politica/articulo/punto-por-punto-la-registraduria-desmiente-a-gustavo-petro-y-evidencia-por-que-no-es-cierto-el-supuesto-fraude-electoral/202628/</t>
         </is>
       </c>
     </row>
@@ -6486,12 +6478,12 @@
       </c>
       <c r="D230" s="3" t="inlineStr">
         <is>
-          <t>Sergio Fajardo da pistas de sus movimientos para la segunda vuelta presidencial: “El espíritu del millón de votos”</t>
+          <t>Por “insultos” del congresista Santiago Osorio, WestCol cancelaría transmisión en vivo con Iván Cepeda</t>
         </is>
       </c>
       <c r="E230" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/sergio-fajardo-da-pistas-de-sus-movimientos-para-la-segunda-vuelta-presidencial-el-espiritu-del-millon-de-votos/202648/</t>
+          <t>https://www.semana.com/politica/articulo/por-insultos-del-congresista-santiago-osorio-westcol-cancelaria-transmision-en-vivo-con-ivan-cepeda/202631/</t>
         </is>
       </c>
     </row>
@@ -6509,12 +6501,12 @@
       </c>
       <c r="D231" s="6" t="inlineStr">
         <is>
-          <t>Medicina Legal confirmó que entre los 48 muertos de San José de Guaviare hay 11 menores: esta es la lista de nombres de los cuerpos identificados</t>
+          <t>Carlos Carrillo, suspendido del cargo por participación en política, asegura ser víctima de una medida “desproporcionada”</t>
         </is>
       </c>
       <c r="E231" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/florencia/articulo/medicina-legal-confirmo-que-entre-los-48-muertos-de-san-jose-de-guaviare-hay-11-menores-esta-es-la-lista-de-nombres-de-los-cuerpos-identificados/202622/</t>
+          <t>https://www.semana.com/politica/articulo/carlos-carrillo-suspendido-del-cargo-por-participacion-en-politica-asegura-ser-victima-de-una-medida-desproporcionada/202636/</t>
         </is>
       </c>
     </row>
@@ -6532,12 +6524,12 @@
       </c>
       <c r="D232" s="3" t="inlineStr">
         <is>
-          <t>Punto por punto, la Registraduría desmiente a Gustavo Petro y evidencia por qué no es cierto el supuesto fraude electoral</t>
+          <t>Final Junior vs. Nacional, empañada por desmanes en el estadio Romelio Martínez: videos de lo ocurrido</t>
         </is>
       </c>
       <c r="E232" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/punto-por-punto-la-registraduria-desmiente-a-gustavo-petro-y-evidencia-por-que-no-es-cierto-el-supuesto-fraude-electoral/202628/</t>
+          <t>https://www.semana.com/deportes/articulo/final-junior-vs-nacional-empanada-por-desmanes-en-el-estadio-romelio-martinez-videos-de-lo-ocurrido/202611/</t>
         </is>
       </c>
     </row>
@@ -6555,12 +6547,12 @@
       </c>
       <c r="D233" s="6" t="inlineStr">
         <is>
-          <t>Por “insultos” del congresista Santiago Osorio, WestCol cancelaría transmisión en vivo con Iván Cepeda</t>
+          <t>La hora cero de Juan Daniel Oviedo: este miércoles anunciará su decisión frente a la segunda vuelta. Estos son sus tres escenarios</t>
         </is>
       </c>
       <c r="E233" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/por-insultos-del-congresista-santiago-osorio-westcol-cancelaria-transmision-en-vivo-con-ivan-cepeda/202631/</t>
+          <t>https://www.semana.com/politica/articulo/la-hora-cero-de-juan-daniel-oviedo-este-miercoles-anunciara-su-decision-frente-a-la-segunda-vuelta-estos-son-sus-tres-escenarios/202621/</t>
         </is>
       </c>
     </row>
@@ -6578,12 +6570,12 @@
       </c>
       <c r="D234" s="3" t="inlineStr">
         <is>
-          <t>Carlos Carrillo, suspendido del cargo por participación en política, asegura ser víctima de una medida “desproporcionada”</t>
+          <t>¿Angustia en la campaña de Iván Cepeda? En la izquierda y el progresismo llueven consejeros que lanzan recomendaciones al candidato para enderezar su rumbo</t>
         </is>
       </c>
       <c r="E234" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/carlos-carrillo-suspendido-del-cargo-por-participacion-en-politica-asegura-ser-victima-de-una-medida-desproporcionada/202636/</t>
+          <t>https://www.semana.com/politica/articulo/angustia-en-la-campana-de-ivan-cepeda-en-la-izquierda-y-el-progresismo-llueven-consejeros-que-lanzan-recomendaciones-al-candidato-para-enderezar-su-rumbo/202622/</t>
         </is>
       </c>
     </row>
@@ -6601,12 +6593,12 @@
       </c>
       <c r="D235" s="6" t="inlineStr">
         <is>
-          <t>Final Junior vs. Nacional, empañada por desmanes en el estadio Romelio Martínez: videos de lo ocurrido</t>
+          <t>El mensaje de Violeta Bergonzi sobre “la mujer del proceso” que exalta a la esposa de Abelardo de la Espriella</t>
         </is>
       </c>
       <c r="E235" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/final-junior-vs-nacional-empanada-por-desmanes-en-el-estadio-romelio-martinez-videos-de-lo-ocurrido/202611/</t>
+          <t>https://www.semana.com/gente/articulo/el-mensaje-de-violeta-bergonzi-sobre-la-mujer-del-proceso-que-exalta-a-la-esposa-de-abelardo-de-la-espriella/202602/</t>
         </is>
       </c>
     </row>
@@ -6624,12 +6616,12 @@
       </c>
       <c r="D236" s="3" t="inlineStr">
         <is>
-          <t>La hora cero de Juan Daniel Oviedo: este miércoles anunciará su decisión frente a la segunda vuelta. Estos son sus tres escenarios</t>
+          <t>Lionel Scaloni no pierde de vista a Colombia y la coloca como favorita al Mundial 2026: inesperadas palabras</t>
         </is>
       </c>
       <c r="E236" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/la-hora-cero-de-juan-daniel-oviedo-este-miercoles-anunciara-su-decision-frente-a-la-segunda-vuelta-estos-son-sus-tres-escenarios/202621/</t>
+          <t>https://www.semana.com/deportes/articulo/lionel-scaloni-no-pierde-de-vista-a-colombia-y-la-coloca-como-favorita-al-mundial-2026-inesperadas-palabras/202611/</t>
         </is>
       </c>
     </row>
@@ -6647,12 +6639,12 @@
       </c>
       <c r="D237" s="6" t="inlineStr">
         <is>
-          <t>¿Angustia en la campaña de Iván Cepeda? En la izquierda y el progresismo llueven consejeros que lanzan recomendaciones al candidato para enderezar su rumbo</t>
+          <t>Alcalde Galán envió mensaje a los ciudadanos que van a viajar al Mundial: “Una buena defensa hace la diferencia”</t>
         </is>
       </c>
       <c r="E237" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/angustia-en-la-campana-de-ivan-cepeda-en-la-izquierda-y-el-progresismo-llueven-consejeros-que-lanzan-recomendaciones-al-candidato-para-enderezar-su-rumbo/202622/</t>
+          <t>https://www.semana.com/nacion/bogota/articulo/alcalde-galan-envio-mensaje-a-los-ciudadanos-que-van-a-viajar-al-mundial-una-buena-defensa-hace-la-diferencia/202634/</t>
         </is>
       </c>
     </row>
@@ -6670,12 +6662,12 @@
       </c>
       <c r="D238" s="3" t="inlineStr">
         <is>
-          <t>El mensaje de Violeta Bergonzi sobre “la mujer del proceso” que exalta a la esposa de Abelardo de la Espriella</t>
+          <t>Los goles con los que Bélgica venció Croacia: Lukaku apareció sobre la hora</t>
         </is>
       </c>
       <c r="E238" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/gente/articulo/el-mensaje-de-violeta-bergonzi-sobre-la-mujer-del-proceso-que-exalta-a-la-esposa-de-abelardo-de-la-espriella/202602/</t>
+          <t>https://www.semana.com/deportes/articulo/los-goles-con-los-que-belgica-vencio-croacia-lukaku-aparecio-sobre-la-hora/202641/</t>
         </is>
       </c>
     </row>
@@ -6693,12 +6685,12 @@
       </c>
       <c r="D239" s="6" t="inlineStr">
         <is>
-          <t>Lionel Scaloni no pierde de vista a Colombia y la coloca como favorita al Mundial 2026: inesperadas palabras</t>
+          <t>Cancelan partido de RD Congo, rival de Colombia en el Mundial, a causa del ébola: “No se autoriza”</t>
         </is>
       </c>
       <c r="E239" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/lionel-scaloni-no-pierde-de-vista-a-colombia-y-la-coloca-como-favorita-al-mundial-2026-inesperadas-palabras/202611/</t>
+          <t>https://www.semana.com/deportes/articulo/cancelan-partido-de-rd-congo-rival-de-colombia-en-el-mundial-a-causa-del-ebola-no-se-autoriza/202658/</t>
         </is>
       </c>
     </row>
@@ -6716,12 +6708,12 @@
       </c>
       <c r="D240" s="3" t="inlineStr">
         <is>
-          <t>Alcalde Galán envió mensaje a los ciudadanos que van a viajar al Mundial: “Una buena defensa hace la diferencia”</t>
+          <t>Fifa le ordenó tres cambios a Colombia: anuncio oficial para la fase de grupos del Mundial 2026</t>
         </is>
       </c>
       <c r="E240" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/bogota/articulo/alcalde-galan-envio-mensaje-a-los-ciudadanos-que-van-a-viajar-al-mundial-una-buena-defensa-hace-la-diferencia/202634/</t>
+          <t>https://www.semana.com/deportes/articulo/fifa-le-ordeno-tres-cambios-a-colombia-anuncio-oficial-para-la-fase-de-grupos-del-mundial-2026/202656/</t>
         </is>
       </c>
     </row>
@@ -6739,12 +6731,12 @@
       </c>
       <c r="D241" s="6" t="inlineStr">
         <is>
-          <t>Los goles con los que Bélgica venció Croacia: Lukaku apareció sobre la hora</t>
+          <t>Abelardo de la Espriella sobre un posible empalme con el Gobierno Petro: “Hay que estar muy atentos a la destrucción de documentos”</t>
         </is>
       </c>
       <c r="E241" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/los-goles-con-los-que-belgica-vencio-croacia-lukaku-aparecio-sobre-la-hora/202641/</t>
+          <t>https://www.semana.com/politica/articulo/abelardo-de-la-espriella-sobre-un-posible-empalme-con-el-gobierno-petro-hay-que-estar-muy-atentos-a-la-destruccion-de-documentos/202657/</t>
         </is>
       </c>
     </row>
@@ -6762,12 +6754,12 @@
       </c>
       <c r="D242" s="3" t="inlineStr">
         <is>
-          <t>Cancelan partido de RD Congo, rival de Colombia en el Mundial, a causa del ébola: “No se autoriza”</t>
+          <t>Abelardo de la Espriella reveló cuáles son las mentiras que han dicho de sus propuestas: subsidios, salario mínimo y pensiones</t>
         </is>
       </c>
       <c r="E242" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/cancelan-partido-de-rd-congo-rival-de-colombia-en-el-mundial-a-causa-del-ebola-no-se-autoriza/202658/</t>
+          <t>https://www.semana.com/politica/articulo/abelardo-de-la-espriella-revelo-cuales-son-las-mentiras-que-han-dicho-de-sus-propuestas-subsidios-salario-minimo-y-pensiones/202619/</t>
         </is>
       </c>
     </row>
@@ -6785,12 +6777,12 @@
       </c>
       <c r="D243" s="6" t="inlineStr">
         <is>
-          <t>Fifa le ordenó tres cambios a Colombia: anuncio oficial para la fase de grupos del Mundial 2026</t>
+          <t>Gustavo Petro tuvo que rectificar señalamientos contra empresarios que hizo durante un consejo de ministros</t>
         </is>
       </c>
       <c r="E243" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/fifa-le-ordeno-tres-cambios-a-colombia-anuncio-oficial-para-la-fase-de-grupos-del-mundial-2026/202656/</t>
+          <t>https://www.semana.com/politica/articulo/gustavo-petro-tuvo-que-rectificar-senalamientos-contra-empresarios-que-hizo-durante-un-consejo-de-ministros/202618/</t>
         </is>
       </c>
     </row>
@@ -6808,12 +6800,12 @@
       </c>
       <c r="D244" s="3" t="inlineStr">
         <is>
-          <t>Abelardo de la Espriella sobre un posible empalme con el Gobierno Petro: “Hay que estar muy atentos a la destrucción de documentos”</t>
+          <t>Andrea Padilla advierte que 15 ejemplares de caimán llanero han muerto; el Gobierno conocía su crítica situación</t>
         </is>
       </c>
       <c r="E244" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/abelardo-de-la-espriella-sobre-un-posible-empalme-con-el-gobierno-petro-hay-que-estar-muy-atentos-a-la-destruccion-de-documentos/202657/</t>
+          <t>https://www.semana.com/politica/articulo/andrea-padilla-advierte-que-15-ejemplares-de-caiman-llanero-han-muerto-el-gobierno-conocia-su-critica-situacion/202627/</t>
         </is>
       </c>
     </row>
@@ -6831,12 +6823,12 @@
       </c>
       <c r="D245" s="6" t="inlineStr">
         <is>
-          <t>Abelardo de la Espriella reveló cuáles son las mentiras que han dicho de sus propuestas: subsidios, salario mínimo y pensiones</t>
+          <t>Menor de edad murió junto a su madre tras ser arrollados por un SITP: esto dijo TransMilenio</t>
         </is>
       </c>
       <c r="E245" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/abelardo-de-la-espriella-revelo-cuales-son-las-mentiras-que-han-dicho-de-sus-propuestas-subsidios-salario-minimo-y-pensiones/202619/</t>
+          <t>https://www.semana.com/nacion/bogota/articulo/menor-de-edad-murio-junto-a-su-madre-tras-ser-arrollados-por-un-sitp-esto-dijo-transmilenio/202613/</t>
         </is>
       </c>
     </row>
@@ -6854,12 +6846,12 @@
       </c>
       <c r="D246" s="3" t="inlineStr">
         <is>
-          <t>Gustavo Petro tuvo que rectificar señalamientos contra empresarios que hizo durante un consejo de ministros</t>
+          <t>Salió a trabajar y apareció muerta en un lote en Cali: el desgarrador clamor de la familia de Jenniffer Guevara</t>
         </is>
       </c>
       <c r="E246" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/gustavo-petro-tuvo-que-rectificar-senalamientos-contra-empresarios-que-hizo-durante-un-consejo-de-ministros/202618/</t>
+          <t>https://www.semana.com/nacion/cali/articulo/salio-a-trabajar-y-aparecio-muerta-en-un-lote-en-cali-el-desgarrador-clamor-de-la-familia-de-jenniffer-guevara/202616/</t>
         </is>
       </c>
     </row>
@@ -6872,17 +6864,17 @@
       </c>
       <c r="C247" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D247" s="6" t="inlineStr">
         <is>
-          <t>Andrea Padilla advierte que 15 ejemplares de caimán llanero han muerto; el Gobierno conocía su crítica situación</t>
+          <t>Fraude digital en Colombia: 1 de cada 3 personas ha sido víctima, según expertos</t>
         </is>
       </c>
       <c r="E247" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/andrea-padilla-advierte-que-15-ejemplares-de-caiman-llanero-han-muerto-el-gobierno-conocia-su-critica-situacion/202627/</t>
+          <t>https://canaltrece.com.co/noticias/fraude-digital-en-colombia-victimas-suplantacion-identidad/</t>
         </is>
       </c>
     </row>
@@ -6895,17 +6887,17 @@
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D248" s="3" t="inlineStr">
         <is>
-          <t>Menor de edad murió junto a su madre tras ser arrollados por un SITP: esto dijo TransMilenio</t>
+          <t>Juan Valdez y James Rodríguez lanzan edición especial de café inspirada en el fútbol</t>
         </is>
       </c>
       <c r="E248" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/bogota/articulo/menor-de-edad-murio-junto-a-su-madre-tras-ser-arrollados-por-un-sitp-esto-dijo-transmilenio/202613/</t>
+          <t>https://canaltrece.com.co/noticias/juan-valdez-y-james-rodriguez-edicion-especial-cafe/</t>
         </is>
       </c>
     </row>
@@ -6918,17 +6910,17 @@
       </c>
       <c r="C249" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D249" s="6" t="inlineStr">
         <is>
-          <t>Salió a trabajar y apareció muerta en un lote en Cali: el desgarrador clamor de la familia de Jenniffer Guevara</t>
+          <t>Fito Páez regresa a Colombia con Sale el Sol y celebra los 40 años de Giros</t>
         </is>
       </c>
       <c r="E249" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/cali/articulo/salio-a-trabajar-y-aparecio-muerta-en-un-lote-en-cali-el-desgarrador-clamor-de-la-familia-de-jenniffer-guevara/202616/</t>
+          <t>https://canaltrece.com.co/noticias/fito-paez-regresa-a-colombia-sale-el-sol-gira-2026/</t>
         </is>
       </c>
     </row>
@@ -6946,12 +6938,12 @@
       </c>
       <c r="D250" s="3" t="inlineStr">
         <is>
-          <t>Fraude digital en Colombia: 1 de cada 3 personas ha sido víctima, según expertos</t>
+          <t>Natalia Bedoya Romance Teatro Santander: el concierto que llega a Bucaramanga</t>
         </is>
       </c>
       <c r="E250" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/fraude-digital-en-colombia-victimas-suplantacion-identidad/</t>
+          <t>https://canaltrece.com.co/noticias/natalia-bedoya-romance-teatro-santander/</t>
         </is>
       </c>
     </row>
@@ -6969,12 +6961,12 @@
       </c>
       <c r="D251" s="6" t="inlineStr">
         <is>
-          <t>Juan Valdez y James Rodríguez lanzan edición especial de café inspirada en el fútbol</t>
+          <t>Dago García Creatividad y Escritura: el libro que revela cómo nacen las grandes historias</t>
         </is>
       </c>
       <c r="E251" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/juan-valdez-y-james-rodriguez-edicion-especial-cafe/</t>
+          <t>https://canaltrece.com.co/noticias/dago-garcia-creatividad-y-escritura/</t>
         </is>
       </c>
     </row>
@@ -6992,12 +6984,12 @@
       </c>
       <c r="D252" s="3" t="inlineStr">
         <is>
-          <t>Fito Páez regresa a Colombia con Sale el Sol y celebra los 40 años de Giros</t>
+          <t>Slayer vuelve a Colombia para celebrar 40 años de Reign in Blood</t>
         </is>
       </c>
       <c r="E252" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/fito-paez-regresa-a-colombia-sale-el-sol-gira-2026/</t>
+          <t>https://canaltrece.com.co/noticias/slayer-vuelve-a-colombia-para-celebrar-40-anos-de-reign-in-blood/</t>
         </is>
       </c>
     </row>
@@ -7015,12 +7007,12 @@
       </c>
       <c r="D253" s="6" t="inlineStr">
         <is>
-          <t>Natalia Bedoya Romance Teatro Santander: el concierto que llega a Bucaramanga</t>
+          <t>Álex Ubago regresa a Colombia con su gira “¿Qué Pides Tú?”</t>
         </is>
       </c>
       <c r="E253" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/natalia-bedoya-romance-teatro-santander/</t>
+          <t>https://canaltrece.com.co/noticias/alex-ubago-regresa-a-colombia-con-su-gira-que-pides-tu/</t>
         </is>
       </c>
     </row>
@@ -7038,12 +7030,12 @@
       </c>
       <c r="D254" s="3" t="inlineStr">
         <is>
-          <t>Dago García Creatividad y Escritura: el libro que revela cómo nacen las grandes historias</t>
+          <t>Mito &amp; Didier fusionan jazz y corrido en su nuevo sencillo</t>
         </is>
       </c>
       <c r="E254" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/dago-garcia-creatividad-y-escritura/</t>
+          <t>https://canaltrece.com.co/noticias/mito-didier-fusionan-jazz-y-corrido-en-su-nuevo-sencillo/</t>
         </is>
       </c>
     </row>
@@ -7061,12 +7053,12 @@
       </c>
       <c r="D255" s="6" t="inlineStr">
         <is>
-          <t>Slayer vuelve a Colombia para celebrar 40 años de Reign in Blood</t>
+          <t>Prótesis deportivas impulsan el regreso al deporte en Colombia</t>
         </is>
       </c>
       <c r="E255" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/slayer-vuelve-a-colombia-para-celebrar-40-anos-de-reign-in-blood/</t>
+          <t>https://canaltrece.com.co/noticias/protesis-deportivas-impulsan-el-regreso-al-deporte-en-colombia/</t>
         </is>
       </c>
     </row>
@@ -7084,12 +7076,12 @@
       </c>
       <c r="D256" s="3" t="inlineStr">
         <is>
-          <t>Álex Ubago regresa a Colombia con su gira “¿Qué Pides Tú?”</t>
+          <t>Belinda visitó Bogotá y sorprendió con show en Sala de Despecho</t>
         </is>
       </c>
       <c r="E256" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/alex-ubago-regresa-a-colombia-con-su-gira-que-pides-tu/</t>
+          <t>https://canaltrece.com.co/noticias/belinda-visito-bogota-y-sorprendio-con-show-en-sala-de-despecho/</t>
         </is>
       </c>
     </row>
@@ -7107,12 +7099,12 @@
       </c>
       <c r="D257" s="6" t="inlineStr">
         <is>
-          <t>Mito &amp; Didier fusionan jazz y corrido en su nuevo sencillo</t>
+          <t>La nariñense María Fuell canta junto a Carlos Vives en El Campín para despedir a la Selección Colombia</t>
         </is>
       </c>
       <c r="E257" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/mito-didier-fusionan-jazz-y-corrido-en-su-nuevo-sencillo/</t>
+          <t>https://canaltrece.com.co/noticias/la-narinense-maria-fuell-canta-junto-a-carlos-vives-en-el-campin-para-despedir-a-la-seleccion-colombia/</t>
         </is>
       </c>
     </row>
@@ -7130,12 +7122,12 @@
       </c>
       <c r="D258" s="3" t="inlineStr">
         <is>
-          <t>Prótesis deportivas impulsan el regreso al deporte en Colombia</t>
+          <t>La ciencia de la precisión: Colombia se convierte en mercado clave para la dermocosmética personalizada</t>
         </is>
       </c>
       <c r="E258" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/protesis-deportivas-impulsan-el-regreso-al-deporte-en-colombia/</t>
+          <t>https://canaltrece.com.co/noticias/la-ciencia-de-la-precision-colombia-se-convierte-en-mercado-clave-para-la-dermocosmetica-personalizada/</t>
         </is>
       </c>
     </row>
@@ -7153,12 +7145,12 @@
       </c>
       <c r="D259" s="6" t="inlineStr">
         <is>
-          <t>Belinda visitó Bogotá y sorprendió con show en Sala de Despecho</t>
+          <t>CHAOPELOS proyecta crecer un 35% en 2026 impulsado por la revolución del autocuidado en Colombia</t>
         </is>
       </c>
       <c r="E259" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/belinda-visito-bogota-y-sorprendio-con-show-en-sala-de-despecho/</t>
+          <t>https://canaltrece.com.co/noticias/chaopelos-proyecta-crecer-un-35-en-2026-impulsado-por-la-revolucion-del-autocuidado-en-colombia/</t>
         </is>
       </c>
     </row>
@@ -7176,12 +7168,12 @@
       </c>
       <c r="D260" s="3" t="inlineStr">
         <is>
-          <t>La nariñense María Fuell canta junto a Carlos Vives en El Campín para despedir a la Selección Colombia</t>
+          <t>Jessi Uribe y Paola Jara conquistan Europa y consagran el ‘regional colombiano’ con su gira “Despecho a 2 Voces”</t>
         </is>
       </c>
       <c r="E260" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/la-narinense-maria-fuell-canta-junto-a-carlos-vives-en-el-campin-para-despedir-a-la-seleccion-colombia/</t>
+          <t>https://canaltrece.com.co/noticias/jessi-uribe-y-paola-jara-conquistan-europa-y-consagran-el-regional-colombiano-con-su-gira-despecho-a-2-voces/</t>
         </is>
       </c>
     </row>
@@ -7199,12 +7191,12 @@
       </c>
       <c r="D261" s="6" t="inlineStr">
         <is>
-          <t>La ciencia de la precisión: Colombia se convierte en mercado clave para la dermocosmética personalizada</t>
+          <t>“Quiero a mi País”: Una canción de unión que revive el legado social de Michel Arnau</t>
         </is>
       </c>
       <c r="E261" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/la-ciencia-de-la-precision-colombia-se-convierte-en-mercado-clave-para-la-dermocosmetica-personalizada/</t>
+          <t>https://canaltrece.com.co/noticias/quiero-a-mi-pais-una-cancion-de-union-que-revive-el-legado-social-de-michel-arnau/</t>
         </is>
       </c>
     </row>
@@ -7222,12 +7214,12 @@
       </c>
       <c r="D262" s="3" t="inlineStr">
         <is>
-          <t>CHAOPELOS proyecta crecer un 35% en 2026 impulsado por la revolución del autocuidado en Colombia</t>
+          <t>Mesa Franca rinde homenaje a la tradición colombiana con su nueva experiencia ‘La Olla Dominical’</t>
         </is>
       </c>
       <c r="E262" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/chaopelos-proyecta-crecer-un-35-en-2026-impulsado-por-la-revolucion-del-autocuidado-en-colombia/</t>
+          <t>https://canaltrece.com.co/noticias/mesa-franca-rinde-homenaje-a-la-tradicion-colombiana-con-su-nueva-experiencia-la-olla-dominical/</t>
         </is>
       </c>
     </row>
@@ -7245,12 +7237,12 @@
       </c>
       <c r="D263" s="6" t="inlineStr">
         <is>
-          <t>Jessi Uribe y Paola Jara conquistan Europa y consagran el ‘regional colombiano’ con su gira “Despecho a 2 Voces”</t>
+          <t>Camilo regresa a Bogotá con el cierre de su gira mundial en 2026</t>
         </is>
       </c>
       <c r="E263" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/jessi-uribe-y-paola-jara-conquistan-europa-y-consagran-el-regional-colombiano-con-su-gira-despecho-a-2-voces/</t>
+          <t>https://canaltrece.com.co/noticias/camilo-regresa-a-bogota-con-el-cierre-de-su-gira-mundial-en-2026/</t>
         </is>
       </c>
     </row>
@@ -7268,12 +7260,12 @@
       </c>
       <c r="D264" s="3" t="inlineStr">
         <is>
-          <t>“Quiero a mi País”: Una canción de unión que revive el legado social de Michel Arnau</t>
+          <t>Hamilton: El ‘pelaito de CTG’ que exporta el orgullo y el sonido cartagenero al mundo</t>
         </is>
       </c>
       <c r="E264" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/quiero-a-mi-pais-una-cancion-de-union-que-revive-el-legado-social-de-michel-arnau/</t>
+          <t>https://canaltrece.com.co/noticias/hamilton-el-pelaito-de-ctg-que-exporta-el-orgullo-y-el-sonido-cartagenero-al-mundo/</t>
         </is>
       </c>
     </row>
@@ -7291,12 +7283,12 @@
       </c>
       <c r="D265" s="6" t="inlineStr">
         <is>
-          <t>Mesa Franca rinde homenaje a la tradición colombiana con su nueva experiencia ‘La Olla Dominical’</t>
+          <t>El Parque de Usaquén será el epicentro del ‘street dance’: Llega la Final Nacional de Red Bull Dance Your Style 2026</t>
         </is>
       </c>
       <c r="E265" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/mesa-franca-rinde-homenaje-a-la-tradicion-colombiana-con-su-nueva-experiencia-la-olla-dominical/</t>
+          <t>https://canaltrece.com.co/noticias/el-parque-de-usaquen-sera-el-epicentro-del-street-dance-llega-la-final-nacional-de-red-bull-dance-your-style-2026/</t>
         </is>
       </c>
     </row>
@@ -7314,12 +7306,12 @@
       </c>
       <c r="D266" s="3" t="inlineStr">
         <is>
-          <t>Camilo regresa a Bogotá con el cierre de su gira mundial en 2026</t>
+          <t>Niña Pastori rinde homenaje a la salsa con su álbum «Color Fania»</t>
         </is>
       </c>
       <c r="E266" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/camilo-regresa-a-bogota-con-el-cierre-de-su-gira-mundial-en-2026/</t>
+          <t>https://canaltrece.com.co/noticias/nina-pastori-rinde-homenaje-a-la-salsa-con-su-album-color-fania/</t>
         </is>
       </c>
     </row>
@@ -7337,12 +7329,12 @@
       </c>
       <c r="D267" s="6" t="inlineStr">
         <is>
-          <t>Hamilton: El ‘pelaito de CTG’ que exporta el orgullo y el sonido cartagenero al mundo</t>
+          <t>Colombia 5.0 Magdalena reunió a más de 1.150 asistentes en Santa Marta</t>
         </is>
       </c>
       <c r="E267" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/hamilton-el-pelaito-de-ctg-que-exporta-el-orgullo-y-el-sonido-cartagenero-al-mundo/</t>
+          <t>https://canaltrece.com.co/noticias/colombia-5-0-magdalena-reunio-a-mas-de-1-150-asistentes-en-santa-marta/</t>
         </is>
       </c>
     </row>
@@ -7360,12 +7352,12 @@
       </c>
       <c r="D268" s="3" t="inlineStr">
         <is>
-          <t>El Parque de Usaquén será el epicentro del ‘street dance’: Llega la Final Nacional de Red Bull Dance Your Style 2026</t>
+          <t>Bogotá estrena el Teatro Nancy Kotal de Cortés: Un nuevo templo para el arte, el bilingüismo y la cultura</t>
         </is>
       </c>
       <c r="E268" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/el-parque-de-usaquen-sera-el-epicentro-del-street-dance-llega-la-final-nacional-de-red-bull-dance-your-style-2026/</t>
+          <t>https://canaltrece.com.co/noticias/bogota-estrena-el-teatro-nancy-kotal-de-cortes-un-nuevo-templo-para-el-arte-el-bilinguismo-y-la-cultura/</t>
         </is>
       </c>
     </row>
@@ -7383,12 +7375,12 @@
       </c>
       <c r="D269" s="6" t="inlineStr">
         <is>
-          <t>Niña Pastori rinde homenaje a la salsa con su álbum «Color Fania»</t>
+          <t>Pantallas gigantes y alta tecnología: El Mundial de Fútbol dispara la venta de televisores en Colombia</t>
         </is>
       </c>
       <c r="E269" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/nina-pastori-rinde-homenaje-a-la-salsa-con-su-album-color-fania/</t>
+          <t>https://canaltrece.com.co/noticias/pantallas-gigantes-y-alta-tecnologia-el-mundial-de-futbol-dispara-la-venta-de-televisores-en-colombia/</t>
         </is>
       </c>
     </row>
@@ -7406,12 +7398,12 @@
       </c>
       <c r="D270" s="3" t="inlineStr">
         <is>
-          <t>Colombia 5.0 Magdalena reunió a más de 1.150 asistentes en Santa Marta</t>
+          <t>Nico González: El productor y director musical colombiano que revoluciona el pop latino desde Miami</t>
         </is>
       </c>
       <c r="E270" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/colombia-5-0-magdalena-reunio-a-mas-de-1-150-asistentes-en-santa-marta/</t>
+          <t>https://canaltrece.com.co/noticias/nico-gonzalez-el-productor-y-director-musical-colombiano-que-revoluciona-el-pop-latino-desde-miami/</t>
         </is>
       </c>
     </row>
@@ -7429,12 +7421,12 @@
       </c>
       <c r="D271" s="6" t="inlineStr">
         <is>
-          <t>Bogotá estrena el Teatro Nancy Kotal de Cortés: Un nuevo templo para el arte, el bilingüismo y la cultura</t>
+          <t>Claptone regresa a Medellín con su experiencia ‘Claptone &amp; Friends’</t>
         </is>
       </c>
       <c r="E271" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/bogota-estrena-el-teatro-nancy-kotal-de-cortes-un-nuevo-templo-para-el-arte-el-bilinguismo-y-la-cultura/</t>
+          <t>https://canaltrece.com.co/noticias/claptone-regresa-a-medellin-con-su-experiencia-claptone-friends/</t>
         </is>
       </c>
     </row>
@@ -7452,12 +7444,12 @@
       </c>
       <c r="D272" s="3" t="inlineStr">
         <is>
-          <t>Pantallas gigantes y alta tecnología: El Mundial de Fútbol dispara la venta de televisores en Colombia</t>
+          <t>El restaurante Inquebrantable de Bogotá recibe el ‘Sello M’: Primer reconocimiento a la cocina mexicana auténtica en Colombia</t>
         </is>
       </c>
       <c r="E272" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/pantallas-gigantes-y-alta-tecnologia-el-mundial-de-futbol-dispara-la-venta-de-televisores-en-colombia/</t>
+          <t>https://canaltrece.com.co/noticias/el-restaurante-inquebrantable-de-bogota-recibe-el-sello-m-primer-reconocimiento-a-la-cocina-mexicana-autentica-en-colombia/</t>
         </is>
       </c>
     </row>
@@ -7475,12 +7467,12 @@
       </c>
       <c r="D273" s="6" t="inlineStr">
         <is>
-          <t>Nico González: El productor y director musical colombiano que revoluciona el pop latino desde Miami</t>
+          <t>Mau y Ricky estrenan ‘Ricky y Mau’: Su álbum más íntimo, libre y colaborativo hasta la fecha</t>
         </is>
       </c>
       <c r="E273" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/nico-gonzalez-el-productor-y-director-musical-colombiano-que-revoluciona-el-pop-latino-desde-miami/</t>
+          <t>https://canaltrece.com.co/noticias/mau-y-ricky-estrenan-ricky-y-mau-su-album-mas-intimo-libre-y-colaborativo-hasta-la-fecha/</t>
         </is>
       </c>
     </row>
@@ -7498,12 +7490,12 @@
       </c>
       <c r="D274" s="3" t="inlineStr">
         <is>
-          <t>Claptone regresa a Medellín con su experiencia ‘Claptone &amp; Friends’</t>
+          <t>Alejandro Saavedra estrena su EP ‘El Malo Soy Yo x Tener Corazón’: La nueva era del merenguetón y el pop urbano</t>
         </is>
       </c>
       <c r="E274" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/claptone-regresa-a-medellin-con-su-experiencia-claptone-friends/</t>
+          <t>https://canaltrece.com.co/noticias/alejandro-saavedra-estrena-su-ep-el-malo-soy-yo-x-tener-corazon-la-nueva-era-del-merengueton-y-el-pop-urbano/</t>
         </is>
       </c>
     </row>
@@ -7521,12 +7513,12 @@
       </c>
       <c r="D275" s="6" t="inlineStr">
         <is>
-          <t>El restaurante Inquebrantable de Bogotá recibe el ‘Sello M’: Primer reconocimiento a la cocina mexicana auténtica en Colombia</t>
+          <t>Así son Ana Lucía Pineda y Pilar Rueda, las mujeres que aspiran a la Casa de Nariño</t>
         </is>
       </c>
       <c r="E275" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/el-restaurante-inquebrantable-de-bogota-recibe-el-sello-m-primer-reconocimiento-a-la-cocina-mexicana-autentica-en-colombia/</t>
+          <t>https://canaltrece.com.co/noticias/asi-son-ana-lucia-pineda-y-pilar-rueda-las-mujeres-que-aspiran-a-la-casa-de-narino/</t>
         </is>
       </c>
     </row>
@@ -7544,86 +7536,17 @@
       </c>
       <c r="D276" s="3" t="inlineStr">
         <is>
-          <t>Mau y Ricky estrenan ‘Ricky y Mau’: Su álbum más íntimo, libre y colaborativo hasta la fecha</t>
+          <t>Abelardo de la Espriella responde desde un buque blindado: «No permitiremos que Petro y Cepeda se roben las elecciones»</t>
         </is>
       </c>
       <c r="E276" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/mau-y-ricky-estrenan-ricky-y-mau-su-album-mas-intimo-libre-y-colaborativo-hasta-la-fecha/</t>
-        </is>
-      </c>
-    </row>
-    <row r="277">
-      <c r="A277" s="5" t="inlineStr"/>
-      <c r="B277" s="5" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C277" s="5" t="inlineStr">
-        <is>
-          <t>Canal Trece</t>
-        </is>
-      </c>
-      <c r="D277" s="6" t="inlineStr">
-        <is>
-          <t>Alejandro Saavedra estrena su EP ‘El Malo Soy Yo x Tener Corazón’: La nueva era del merenguetón y el pop urbano</t>
-        </is>
-      </c>
-      <c r="E277" s="7" t="inlineStr">
-        <is>
-          <t>https://canaltrece.com.co/noticias/alejandro-saavedra-estrena-su-ep-el-malo-soy-yo-x-tener-corazon-la-nueva-era-del-merengueton-y-el-pop-urbano/</t>
-        </is>
-      </c>
-    </row>
-    <row r="278">
-      <c r="A278" s="2" t="inlineStr"/>
-      <c r="B278" s="2" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C278" s="2" t="inlineStr">
-        <is>
-          <t>Canal Trece</t>
-        </is>
-      </c>
-      <c r="D278" s="3" t="inlineStr">
-        <is>
-          <t>Así son Ana Lucía Pineda y Pilar Rueda, las mujeres que aspiran a la Casa de Nariño</t>
-        </is>
-      </c>
-      <c r="E278" s="4" t="inlineStr">
-        <is>
-          <t>https://canaltrece.com.co/noticias/asi-son-ana-lucia-pineda-y-pilar-rueda-las-mujeres-que-aspiran-a-la-casa-de-narino/</t>
-        </is>
-      </c>
-    </row>
-    <row r="279">
-      <c r="A279" s="5" t="inlineStr"/>
-      <c r="B279" s="5" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C279" s="5" t="inlineStr">
-        <is>
-          <t>Canal Trece</t>
-        </is>
-      </c>
-      <c r="D279" s="6" t="inlineStr">
-        <is>
-          <t>Abelardo de la Espriella responde desde un buque blindado: «No permitiremos que Petro y Cepeda se roben las elecciones»</t>
-        </is>
-      </c>
-      <c r="E279" s="7" t="inlineStr">
-        <is>
           <t>https://canaltrece.com.co/noticias/abelardo-de-la-espriella-responde-desde-un-buque-blindado-no-permitiremos-que-petro-y-cepeda-se-roben-las-elecciones/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E279"/>
+  <autoFilter ref="A1:E276"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
@@ -7900,9 +7823,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E274" r:id="rId273"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E275" r:id="rId274"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E276" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E277" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E278" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E279" r:id="rId278"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Noticias actualizadas 04/06/2026 08:48
</commit_message>
<xml_diff>
--- a/docs/ultimahora.xlsx
+++ b/docs/ultimahora.xlsx
@@ -515,7 +515,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 01:29 a. m.</t>
+          <t>04/06/2026 03:04 a. m.</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -530,19 +530,19 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Senadora Andrea Padilla anunció que Fiscalía y Procuraduría abrieron investigación por crisis de 317 caimanes sin comida: 'Ya fueron alimentados'</t>
+          <t>Expolicía ecuatoriano aseguró que agentes y altos mandos sabían del atentado contra el candidato Fernando Villavicencio antes de ser asesinado en 2023</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/vida/medio-ambiente/senadora-andrea-padilla-anuncio-que-fiscalia-y-procuraduria-abrieron-investigacion-por-crisis-de-317-caimanes-sin-comida-ya-fueron-alimentados-3561989</t>
+          <t>https://www.eltiempo.com/mundo/latinoamerica/expolicia-ecuatoriano-aseguro-que-agentes-y-altos-mandos-sabian-del-atentado-contra-el-candidato-fernando-villavicencio-antes-de-ser-asesinado-en-3561991</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 12:37 a. m.</t>
+          <t>04/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -557,19 +557,19 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>Estas son las nuevas preguntas que podrían hacerle en su proceso de green card en Estados Unidos: miles colombianos se verían afectados</t>
+          <t>¡Ojo con las restricciones! Pico y placa en Pereira para el jueves 4 de junio de 2026</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/estas-son-las-nuevas-preguntas-que-podrian-hacerle-en-su-proceso-de-green-card-en-estados-unidos-miles-colombianos-se-verian-afectados-3561940</t>
+          <t>https://www.eltiempo.com/colombia/otras-ciudades/ojo-con-las-restricciones-pico-y-placa-en-pereira-para-el-jueves-4-de-junio-de-3561984</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 12:10 a. m.</t>
+          <t>04/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -584,19 +584,19 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Nueva ofensiva arancelaria de Trump podría golpear a Colombia: propuesta de EE. UU. elevaría al 12,5 % la tarifa sobre exportaciones nacionales</t>
+          <t>¡Ojo, conductor! Pico y placa en Medellín para el jueves 4 de junio de 2026: consulte las restricciones</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/nueva-ofensiva-arancelaria-de-trump-podria-golpear-a-colombia-propuesta-de-ee-uu-elevaria-al-12-5-la-tarifa-sobre-exportaciones-nacionales-3561904</t>
+          <t>https://www.eltiempo.com/colombia/medellin/ojo-conductor-pico-y-placa-en-medellin-para-el-jueves-4-de-junio-de-2026-consulte-las-restricciones-3561983</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 11:24 p. m.</t>
+          <t>04/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -611,19 +611,19 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Presidente Gustavo Petro ordenó bombardeo en Guaviare tras captura de alias Mona, presunta cabecilla de las disidencias de 'Iván Mordisco'</t>
+          <t>Así opera el pico y placa en Bucaramanga para el jueves 4 de junio de 2026</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/politica/gobierno/presidente-gustavo-petro-ordeno-bombardeo-en-guaviare-tras-captura-de-alias-mona-presunta-cabecilla-de-las-disidencias-de-ivan-mordisco-3561988</t>
+          <t>https://www.eltiempo.com/colombia/santander/asi-opera-el-pico-y-placa-en-bucaramanga-para-el-jueves-4-de-junio-de-3561982</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 11:17 p. m.</t>
+          <t>04/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -638,19 +638,19 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Identificaron a familiar de los hermanos Mucutuy entre los 11 menores fallecidos por combates de las disidencias en Guaviare: era prima de los niños</t>
+          <t>¡Evite multas! Pico y placa en Cali para el jueves 4 de junio de 2026: así opera la medida</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/justicia/conflicto-y-narcotrafico/identificaron-a-familiar-de-los-hermanos-mucutuy-entre-los-11-menores-fallecidos-por-combates-entre-disidencias-en-guaviare-era-prima-de-los-ninos-3561987</t>
+          <t>https://www.eltiempo.com/colombia/cali/evite-multas-pico-y-placa-en-cali-para-el-jueves-4-de-junio-de-2026-asi-opera-la-medida-3561981</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 11:08 p. m.</t>
+          <t>04/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -665,19 +665,19 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Senadora María Elvira Salazar pidió sanciones para quien realice fraude en segunda vuelta presidencial de Colombia: lista OFAC y cancelación de visas</t>
+          <t>¡Pilas en las vías! Pico y placa en Bogotá para el jueves 4 de junio de 2026</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/senadora-maria-elvira-salazar-pidio-incluir-en-la-lista-ofac-a-quien-realice-fraude-electoral-en-la-segunda-vuelta-presidencial-de-colombia-3561985</t>
+          <t>https://www.eltiempo.com/bogota/pilas-en-las-vias-pico-y-placa-en-bogota-para-el-jueves-4-de-junio-de-3561858</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 11:05 p. m.</t>
+          <t>04/06/2026 01:29 a. m.</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -692,19 +692,19 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Revelan las supuestas amenazas del anestesiólogo 'Leo' cuando Yulixa Toloza todavía tenía signos vitales tras procedimiento estético: 'Sacó un arma'</t>
+          <t>Senadora Andrea Padilla anunció que la Fiscalía y Procuraduría abrieron investigación por crisis de 317 caimanes sin comida: 'Ya fueron alimentados'</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/bogota/revelan-las-supuestas-amenazas-de-anestesiologo-leo-cuando-yulixa-toloza-todavia-tenia-signos-vitales-tras-procedimiento-estetico-saco-un-arma-3561986</t>
+          <t>https://www.eltiempo.com/vida/medio-ambiente/senadora-andrea-padilla-anuncio-que-fiscalia-y-procuraduria-abrieron-investigacion-por-crisis-de-317-caimanes-sin-comida-ya-fueron-alimentados-3561989</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 11:03 p. m.</t>
+          <t>04/06/2026 12:37 a. m.</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -719,19 +719,19 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Alertan por estafas migratorias en Estados Unidos: usan inteligencia artificial para suplantar abogados y ofrecer trámites falsos</t>
+          <t>Estas son las nuevas preguntas que podrían hacerle en su proceso de green card en Estados Unidos: miles colombianos se verían afectados</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/alertan-por-estafas-migratorias-en-estados-unidos-usan-inteligencia-artificial-para-suplantar-abogados-y-ofrecer-tramites-migratorios-falsos-3561967</t>
+          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/estas-son-las-nuevas-preguntas-que-podrian-hacerle-en-su-proceso-de-green-card-en-estados-unidos-miles-colombianos-se-verian-afectados-3561940</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 10:47 p. m.</t>
+          <t>04/06/2026 12:10 a. m.</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -746,19 +746,19 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Junior vs. Nacional: Alfredo Arias y sus tres lecciones a Diego Arias en final de ida de la Liga BetPlay</t>
+          <t>Nueva ofensiva arancelaria de Trump podría golpear a Colombia: propuesta de EE. UU. elevaría al 12,5 % la tarifa sobre exportaciones nacionales</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-colombiano/junior-vs-nacional-alfredo-arias-y-sus-tres-lecciones-a-diego-arias-en-final-de-ida-de-la-liga-betplay-3561972</t>
+          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/nueva-ofensiva-arancelaria-de-trump-podria-golpear-a-colombia-propuesta-de-ee-uu-elevaria-al-12-5-la-tarifa-sobre-exportaciones-nacionales-3561904</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 10:28 p. m.</t>
+          <t>03/06/2026 11:24 p. m.</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -773,19 +773,19 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>'Es hora de que el Gobierno Nacional fije sus ojos en la región': esto es lo que el sector productivo del Valle del Cauca le pide al nuevo presidente</t>
+          <t>Presidente Gustavo Petro ordenó bombardeo en Guaviare tras captura de alias Mona, presunta cabecilla de las disidencias de 'Iván Mordisco'</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/cali/es-hora-de-que-el-gobierno-nacional-fije-sus-ojos-en-la-region-esto-es-lo-que-el-sector-productivo-del-valle-del-cauca-le-pide-al-nuevo-presidente-3561979</t>
+          <t>https://www.eltiempo.com/politica/gobierno/presidente-gustavo-petro-ordeno-bombardeo-en-guaviare-tras-captura-de-alias-mona-presunta-cabecilla-de-las-disidencias-de-ivan-mordisco-3561988</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 10:09 p. m.</t>
+          <t>03/06/2026 11:17 p. m.</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -800,19 +800,19 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>El actor estadounidense Tyler Hoechlin será uno de los invitados centrales de la Comic Con Bogotá</t>
+          <t>Identificaron a familiar de los hermanos Mucutuy entre los 11 menores fallecidos por combates de las disidencias en Guaviare: era prima de los niños</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/cultura/cine-y-tv/el-actor-estadounidense-tyler-hoechlin-sera-uno-de-los-invitados-centrales-de-la-comic-con-bogota-3561980</t>
+          <t>https://www.eltiempo.com/justicia/conflicto-y-narcotrafico/identificaron-a-familiar-de-los-hermanos-mucutuy-entre-los-11-menores-fallecidos-por-combates-entre-disidencias-en-guaviare-era-prima-de-los-ninos-3561987</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 10:01 p. m.</t>
+          <t>03/06/2026 11:08 p. m.</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -827,19 +827,19 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>'Enemigo público': alcalde de Soacha hace denuncia por video que revelaría a empleados de la empresa de aseo Urbaser arrojando basura en las calles</t>
+          <t>Senadora María Elvira Salazar pidió sanciones para quien realice fraude en segunda vuelta presidencial de Colombia: lista OFAC y cancelación de visas</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/bogota/enemigo-publico-alcalde-de-soacha-hace-denuncia-por-video-que-revelaria-a-empleados-de-la-empresa-de-aseo-urbaser-arrojando-basura-en-las-calles-3561975</t>
+          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/senadora-maria-elvira-salazar-pidio-incluir-en-la-lista-ofac-a-quien-realice-fraude-electoral-en-la-segunda-vuelta-presidencial-de-colombia-3561985</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 10:01 p. m.</t>
+          <t>03/06/2026 11:05 p. m.</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -854,19 +854,19 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Tristeza total</t>
+          <t>Revelan las supuestas amenazas del anestesiólogo 'Leo' cuando Yulixa Toloza todavía tenía signos vitales tras procedimiento estético: 'Sacó un arma'</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/caricaturas/tristeza-total-3561947</t>
+          <t>https://www.eltiempo.com/bogota/revelan-las-supuestas-amenazas-de-anestesiologo-leo-cuando-yulixa-toloza-todavia-tenia-signos-vitales-tras-procedimiento-estetico-saco-un-arma-3561986</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 10:01 p. m.</t>
+          <t>03/06/2026 11:03 p. m.</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -881,19 +881,19 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Trump saludó</t>
+          <t>Alertan por estafas migratorias en Estados Unidos: usan inteligencia artificial para suplantar abogados y ofrecer trámites falsos</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/caricaturas/trump-saludo-3561946</t>
+          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/alertan-por-estafas-migratorias-en-estados-unidos-usan-inteligencia-artificial-para-suplantar-abogados-y-ofrecer-tramites-migratorios-falsos-3561967</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 10:01 p. m.</t>
+          <t>03/06/2026 10:47 p. m.</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -908,19 +908,19 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Cuidar la taza</t>
+          <t>Junior vs. Nacional: Alfredo Arias y sus tres lecciones a Diego Arias en final de ida de la Liga BetPlay</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/editorial/cuidar-la-taza-3561943</t>
+          <t>https://www.eltiempo.com/deportes/futbol-colombiano/junior-vs-nacional-alfredo-arias-y-sus-tres-lecciones-a-diego-arias-en-final-de-ida-de-la-liga-betplay-3561972</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 10:01 p. m.</t>
+          <t>03/06/2026 10:28 p. m.</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -935,19 +935,19 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>La iniciativa, esa magia del poder y la política</t>
+          <t>'Es hora de que el Gobierno Nacional fije sus ojos en la región': esto es lo que el sector productivo del Valle del Cauca le pide al nuevo presidente</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/columnistas/la-iniciativa-esa-magia-del-poder-y-la-politica-3561942</t>
+          <t>https://www.eltiempo.com/colombia/cali/es-hora-de-que-el-gobierno-nacional-fije-sus-ojos-en-la-region-esto-es-lo-que-el-sector-productivo-del-valle-del-cauca-le-pide-al-nuevo-presidente-3561979</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 10:01 p. m.</t>
+          <t>03/06/2026 10:09 p. m.</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -962,12 +962,12 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>‘Es falso que vamos a acabar con la matrícula cero, con los subsidios, con los programas sociales’: entrevista con José Manuel Restrepo</t>
+          <t>El actor estadounidense Tyler Hoechlin será uno de los invitados centrales de la Comic Con Bogotá</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/es-falso-que-vamos-a-acabar-con-la-matricula-cero-con-los-subsidios-con-los-programas-sociales-entrevista-con-jose-manuel-restrepo-3561927</t>
+          <t>https://www.eltiempo.com/cultura/cine-y-tv/el-actor-estadounidense-tyler-hoechlin-sera-uno-de-los-invitados-centrales-de-la-comic-con-bogota-3561980</t>
         </is>
       </c>
     </row>
@@ -989,12 +989,12 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>No es el más indicado</t>
+          <t>'Enemigo público': alcalde de Soacha hace denuncia por video que revelaría a empleados de la empresa de aseo Urbaser arrojando basura en las calles</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/cartas/no-es-el-mas-indicado-3561923</t>
+          <t>https://www.eltiempo.com/bogota/enemigo-publico-alcalde-de-soacha-hace-denuncia-por-video-que-revelaria-a-empleados-de-la-empresa-de-aseo-urbaser-arrojando-basura-en-las-calles-3561975</t>
         </is>
       </c>
     </row>
@@ -1016,12 +1016,12 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Universos para lelos</t>
+          <t>Tristeza total</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/columnistas/universos-para-lelos-3561911</t>
+          <t>https://www.eltiempo.com/opinion/caricaturas/tristeza-total-3561947</t>
         </is>
       </c>
     </row>
@@ -1043,19 +1043,19 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>El gran reto del nuevo tribunal para Ucrania: investigar el crimen de agresión</t>
+          <t>Trump saludó</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/columnistas/el-gran-reto-del-nuevo-tribunal-para-ucrania-investigar-el-crimen-de-agresion-3561883</t>
+          <t>https://www.eltiempo.com/opinion/caricaturas/trump-saludo-3561946</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 06:22 a. m.</t>
+          <t>04/06/2026 07:05 a. m.</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1070,19 +1070,19 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Fiscalía imputará cargos a ocho implicados en red de contrabando ligada a Lili Pink</t>
+          <t>Petro califica de intervencionista el respaldo de Trump a de La Espriella</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/03/fiscalia-imputara-cargos-a-ocho-implicados-en-red-de-contrabando-ligada-a-lili-pink/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/03/petro-califica-de-intervencionista-el-respaldo-de-trump-a-de-la-espriella/</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 01:00 a. m.</t>
+          <t>04/06/2026 06:22 a. m.</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -1097,12 +1097,12 @@
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>José Francisco Socarrás Colina</t>
+          <t>Fiscalía imputará cargos a ocho implicados en red de contrabando ligada a Lili Pink</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/04/jose-francisco-socarras-colina/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/03/fiscalia-imputara-cargos-a-ocho-implicados-en-red-de-contrabando-ligada-a-lili-pink/</t>
         </is>
       </c>
     </row>
@@ -1124,12 +1124,12 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Columnistas</t>
+          <t>José Francisco Socarrás Colina</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/04/jose-francisco-socarras-colina/</t>
         </is>
       </c>
     </row>
@@ -1151,12 +1151,12 @@
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>El Museo del Nunca Jamás</t>
+          <t>Columnistas</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/04/el-museo-del-nunca-jamas/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/</t>
         </is>
       </c>
     </row>
@@ -1178,19 +1178,19 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>En Santander las escuelas no salen a marchar</t>
+          <t>El Museo del Nunca Jamás</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/04/en-santander-las-escuelas-no-salen-a-marchar/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/04/el-museo-del-nunca-jamas/</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 06:08 p. m.</t>
+          <t>04/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -1205,12 +1205,12 @@
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>Piden llamar a indagatoria a Petro: los hallazgos que complican el caso de su campaña en 2022</t>
+          <t>En Santander las escuelas no salen a marchar</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/03/piden-llamar-a-indagatoria-a-petro-los-hallazgos-que-complican-el-caso-de-su-campana-en-2022/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/04/en-santander-las-escuelas-no-salen-a-marchar/</t>
         </is>
       </c>
     </row>
@@ -1232,19 +1232,19 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Piden llamar a indagatoria a Petro: los hallazgos que complican el caso de su campaña en 2022</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/03/piden-llamar-a-indagatoria-a-petro-los-hallazgos-que-complican-el-caso-de-su-campana-en-2022/</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 02:59 p. m.</t>
+          <t>03/06/2026 06:08 p. m.</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -1259,19 +1259,19 @@
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>Prima de los hermanos Mucutuy murió en combates tras ser reclutada por disidencias</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/03/prima-de-los-hermanos-mucutuy-murio-en-combates-tras-ser-reclutada-por-disidencias/</t>
+          <t>https://www.vanguardia.com/colombia/</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 02:18 p. m.</t>
+          <t>03/06/2026 02:59 p. m.</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1286,19 +1286,19 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Masacre de 11 menores en medio de combates expone la crisis por reclutamiento de niños</t>
+          <t>Prima de los hermanos Mucutuy murió en combates tras ser reclutada por disidencias</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/03/masacre-de-11-menores-en-combates-de-guaviare-expone-crisis-por-reclutamiento-de-ninos/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/03/prima-de-los-hermanos-mucutuy-murio-en-combates-tras-ser-reclutada-por-disidencias/</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 10:57 a. m.</t>
+          <t>03/06/2026 02:18 p. m.</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -1313,19 +1313,19 @@
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Orden judicial obligó a Petro a aclarar que los hermanos Moreno no fueron condenados</t>
+          <t>Masacre de 11 menores en medio de combates expone la crisis por reclutamiento de niños</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/politica/2026/06/03/orden-judicial-obligo-a-petro-a-aclarar-que-los-hermanos-moreno-no-fueron-condenados/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/03/masacre-de-11-menores-en-combates-de-guaviare-expone-crisis-por-reclutamiento-de-ninos/</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 09:24 a. m.</t>
+          <t>03/06/2026 10:57 a. m.</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1340,19 +1340,19 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>La justificación de la Policía por uso de fuerza contra músico callejero tras denuncias en Parque La Colina en Bogotá</t>
+          <t>Orden judicial obligó a Petro a aclarar que los hermanos Moreno no fueron condenados</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/03/la-justificacion-de-la-policia-por-uso-de-fuerza-contra-musico-callejero-tras-denuncias-en-parque-la-colina-en-bogota/</t>
+          <t>https://www.vanguardia.com/politica/2026/06/03/orden-judicial-obligo-a-petro-a-aclarar-que-los-hermanos-moreno-no-fueron-condenados/</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 07:05 a. m.</t>
+          <t>03/06/2026 09:24 a. m.</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
@@ -1367,12 +1367,12 @@
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>Petro califica de intervencionista el respaldo de Trump a de La Espriella</t>
+          <t>La justificación de la Policía por uso de fuerza contra músico callejero tras denuncias en Parque La Colina en Bogotá</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/03/petro-califica-de-intervencionista-el-respaldo-de-trump-a-de-la-espriella/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/03/la-justificacion-de-la-policia-por-uso-de-fuerza-contra-musico-callejero-tras-denuncias-en-parque-la-colina-en-bogota/</t>
         </is>
       </c>
     </row>
@@ -1448,7 +1448,7 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 02:57 a. m.</t>
+          <t>04/06/2026 03:21 a. m.</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
@@ -1458,24 +1458,24 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>Último sorteo Lotería de Manizales: resultado premio mayor hoy 3 de junio</t>
+          <t>Israel y Líbano acuerdan un alto el fuego mediado por Estados Unidos</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/sociedad/ultimo-sorteo-loteria-de-manizales-resultado-premio-mayor-hoy-3-de-junio-401332</t>
+          <t>https://caracol.com.co/2026/06/04/israel-y-libano-acuerdan-un-alto-el-fuego-mediado-por-estados-unidos/</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 02:14 a. m.</t>
+          <t>04/06/2026 01:13 a. m.</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -1485,24 +1485,24 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Un telescopio a 1,5 millones de kilómetros de la Tierra reveló algo que llevaba décadas oculto</t>
+          <t>Petro ordena bombardear campamento de ‘Mordisco’ tras confrontación entre disidencias en el Guaviare</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/sociedad/telescopio-revela-misterio-universo-oculto-decadas-cientificos-nasa-401328</t>
+          <t>https://caracol.com.co/2026/06/04/petro-ordena-bombardear-campamento-de-mordisco-tras-confrontacion-entre-disidencias-en-el-guaviare/</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 01:42 a. m.</t>
+          <t>03/06/2026 11:49 p. m.</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
@@ -1512,24 +1512,24 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>Claudia López se aleja de De la Espriella, reconoce la decencia de Cepeda y rechaza endosar sus votos</t>
+          <t>Aída Quilcué acepta stream con Westcol en el Cauca: “eres bienvenido a nuestra comunidad”</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/claudia-lopez-desconfianza-abelardo-de-la-espriella-respaldo-cepeda-401327</t>
+          <t>https://caracol.com.co/2026/06/04/aida-quilcue-acepta-invitacion-de-westcol-y-se-confirma-streaming-desde-el-cauca/</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 12:51 a. m.</t>
+          <t>03/06/2026 11:04 p. m.</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -1539,24 +1539,24 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Matemático alemán que acertó el campeón de los últimos tres mundiales, predijo quién ganará en 2026</t>
+          <t>Más de 800 estudiantes participaron en simulacro de emergencia volcánica en Pasto</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/deportes/copa-mundial-fifa-2026-prediccion-aleman-acerto-campeon-2014-2018-2022-401316</t>
+          <t>https://caracol.com.co/2026/06/04/mas-de-800-estudiantes-participaron-en-simulacro-de-emergencia-volcanica-en-pasto/</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 12:49 a. m.</t>
+          <t>03/06/2026 09:58 p. m.</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
@@ -1566,24 +1566,24 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>Capturan docente de Ética señalado de abusar de una niña en Cali: fue detenido mientras era jurado de votación</t>
+          <t>Llegada del fenómeno de El Niño se intensifica, según alerta de la OMM: esta es la última proyección</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/actualidad/abuso-menor-cali-capturan-docente-etica-senalado-jurado-votacion-401322</t>
+          <t>https://caracol.com.co/2026/06/04/llegada-del-fenomeno-de-el-nino-se-intensifica-segun-alerta-de-la-omm-esta-es-la-ultima-proyeccion/</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 11:59 p. m.</t>
+          <t>03/06/2026 09:52 p. m.</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -1593,24 +1593,24 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>El avión del papa: así será la operación de Iberia para mover a León XIV en su visita a España</t>
+          <t>Elecciones segunda vuelta: ¿Personas que fueron jurados de votación repiten el 21 de junio?</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/internacional/papa-leon-xiv-iberia-traslado-pontifice-espana-401317</t>
+          <t>https://caracol.com.co/2026/06/04/elecciones-segunda-vuelta-personas-que-fueron-jurados-de-votacion-repiten-el-21-de-junio/</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 11:45 p. m.</t>
+          <t>03/06/2026 09:50 p. m.</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
@@ -1620,24 +1620,24 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>El misterio de los "cazatesoros" que fueron grabados saliendo de alcantarillas en Nueva York</t>
+          <t>Capturan a la ‘Mona’, cabecilla de disidencias, señalada de trasladar menores entre Cauca y Guaviare</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/actualidad/policia-nueva-york-investiga-hombres-401311</t>
+          <t>https://caracol.com.co/2026/06/04/capturan-a-la-mona-cabecilla-de-disidencias-senalada-de-trasladar-menores-reclutados-entre-cauca/</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 11:17 p. m.</t>
+          <t>03/06/2026 09:36 p. m.</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -1647,24 +1647,24 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Graves emergencias en Andes, Antioquia, por las lluvias</t>
+          <t>¿Cuánto gana el vicepresidente de Colombia en 2026? Este sería el salario de Quilcué o Restrepo</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/sociedad/emergencias-lluvias-andes-antioquia-avenida-torrencial-401312</t>
+          <t>https://caracol.com.co/2026/06/04/cuanto-gana-el-vicepresidente-de-colombia-en-2026-este-seria-el-salario-de-quilcue-o-restrepo/</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 11:34 a. m.</t>
+          <t>03/06/2026 09:22 p. m.</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
@@ -1674,24 +1674,24 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>Abelardo de la Espriella no acepta apoyo del Partido Liberal: “es un apéndice de Petro y Cepeda”</t>
+          <t>Quinto ciclo Colombia Mayor: Prosperidad Social confirma fechas y canales para reclamar el subsidio</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/abelardo-de-la-espriella-no-acepta-apoyo-partido-liberal-apendice-de-petro-y-cepeda-401325</t>
+          <t>https://caracol.com.co/2026/06/04/quinto-ciclo-colombia-mayor-prosperidad-social-confirma-fechas-y-canales-para-reclamar-el-subsidio/</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 09:56 p. m.</t>
+          <t>03/06/2026 08:35 p. m.</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -1701,24 +1701,24 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Sin salida a la vista: continúa el cierre total de la Transversal del Sisga</t>
+          <t>Abelardo de la Espriella rechaza respaldo del Partido Liberal: “Es un apéndice de Petro y Cepeda”</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/actualidad/transversal-sisga-colombia-cerrada-deslizamiento-401320</t>
+          <t>https://caracol.com.co/2026/06/04/abelardo-de-la-espriella-rechaza-respaldo-liberal-es-un-apendice-de-petro-y-cepeda/</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 02:31 p. m.</t>
+          <t>03/06/2026 07:48 p. m.</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
@@ -1728,24 +1728,24 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>Aida Quilcué abre las puertas de su comunidad a Westcol y lleva la campaña presidencial al mundo del streaming</t>
+          <t>Fiscalía capturó a la madre de Mía Cataleya en El Espinal</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/aida-quilcue-abre-puertas-comunidad-westcol-401319</t>
+          <t>https://caracol.com.co/2026/06/04/fiscalia-capturo-a-la-madre-de-mia-cataleya-en-el-espinal/</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>31/05/2026 03:32 p. m.</t>
+          <t>03/06/2026 07:46 p. m.</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -1755,24 +1755,24 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>"El centro político está destinado a desaparecer": representante a la Cámara lanza advertencia tras la primera vuelta presidencial</t>
+          <t>Resultados Lotería del Valle, Manizales, Meta y Baloto HOY 03 de junio, 2026: último sorteo y premio</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/centro-politico-colombia-crisis-segunda-vuelta-2026-401335</t>
+          <t>https://caracol.com.co/2026/06/04/resultados-loteria-del-valle-manizales-meta-y-baloto-hoy-03-de-junio-2026-ultimo-sorteo-y-premio/</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>31/05/2026 12:32 p. m.</t>
+          <t>03/06/2026 07:24 p. m.</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
@@ -1782,22 +1782,26 @@
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>Petro ordenó bombardear zona del Guaviare donde se enfrentaron disidencias</t>
+          <t>Centro Democrático en Antioquia anuncia respaldo a Abelardo de la Espriella para la segunda vuelta</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/orden-publico/petro-ordeno-bombardear-zona-del-guaviare-donde-se-enfrentaron-disidencias-401336</t>
+          <t>https://caracol.com.co/2026/06/04/centro-democratico-en-antioquia-anuncia-respaldo-a-abelardo-de-la-espriella-para-la-segunda-vuelta/</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr"/>
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 07:12 p. m.</t>
+        </is>
+      </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1805,22 +1809,26 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>Los cuatro episodios que le recuerdan a Petro tras criticar apoyo de Trump a De la Espriella</t>
+          <t>Felipe Harman, director de la ANT sale del Gobierno para apoyar la campaña de Iván Cepeda</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/petro-opino-elecciones-extranjeras-cuatro-casos-401331</t>
+          <t>https://caracol.com.co/2026/06/04/felipe-harman-director-de-la-ant-sale-del-gobierno-para-apoyar-la-campana-de-ivan-cepeda/</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="5" t="inlineStr"/>
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>03/06/2026 07:01 p. m.</t>
+        </is>
+      </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1828,22 +1836,26 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>“Petro está reconociendo que su candidato no funcionó”; cuestionan protagonismo del presidente en la campaña de Cepeda</t>
+          <t>Petro pide al CNE atender su denuncia sobre presunto fraude, pese a aclaración de la Registraduría</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/gustavo-petro-ivan-cepeda-campana-pacto-historico-elecciones-presidenciales-2026-401330</t>
+          <t>https://caracol.com.co/2026/06/04/petro-pide-al-cne-atender-su-denuncia-sobre-presunto-fraude-pese-a-aclaracion-de-la-registraduria/</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr"/>
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 06:48 p. m.</t>
+        </is>
+      </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1851,22 +1863,26 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Movida clave en el gobierno Petro: Felipe Harman dejaría la ANT para aterrizar en la campaña de Iván Cepeda</t>
+          <t>Abren cupos para el Servicio Social para la Paz: certifica el servicio militar y entrega auxilio</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/agencia-nacional-de-tierras-felipe-harman-campana-ivan-cepeda-segunda-vuelta-401326</t>
+          <t>https://caracol.com.co/2026/06/03/abren-cupos-para-el-servicio-social-para-la-paz-certifica-el-servicio-militar-y-entrega-auxilio/</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="5" t="inlineStr"/>
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>03/06/2026 06:41 p. m.</t>
+        </is>
+      </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1874,22 +1890,26 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>Capturan a la mamá de la bebé que murió tras ser víctima de abuso en El Espinal, Tolima</t>
+          <t>Petro cuestiona solicitud de indagatoria: “Ya amenazaron con encarcelarme sin cometer un delito”</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/actualidad/capturan-mama-de-bebe-que-murio-en-el-espinal-tolima-401324</t>
+          <t>https://caracol.com.co/2026/06/03/petro-tras-solicitud-de-indagatoria-ya-amenazaron-con-encarcelarme-sin-cometer-un-delito/</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr"/>
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 06:41 p. m.</t>
+        </is>
+      </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1897,22 +1917,26 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>Entró en vigencia la ‘Ley Sara Sofía’, que crea un sistema de alerta para encontrar niños desaparecidos</t>
+          <t>OEA pide a grupos armados no interferir en segunda vuelta y a candidatos recibir resultados en paz</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/ley-sara-sofia-entra-en-vigencia-sistema-alerta-encontrar-ninos-desaparecidos-colombia-401321</t>
+          <t>https://caracol.com.co/2026/06/03/oea-pide-a-grupos-armados-no-interferir-en-segunda-vuelta-y-a-candidatos-recibir-resultados-en-paz/</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="5" t="inlineStr"/>
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>03/06/2026 06:23 p. m.</t>
+        </is>
+      </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1920,22 +1944,26 @@
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>Atención conductores: licencia de conducción cambia en 2026 para estas personas; estos son los nuevos exámenes y costos</t>
+          <t>Elecciones y Mundial: ¿Habrá inscripción de cédulas en sedes de Colombia? Esto dice la Registraduría</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/actualidad/licencia-conduccion-cambia-2026-nuevos-examenes-y-costos-401318</t>
+          <t>https://caracol.com.co/2026/06/03/elecciones-y-mundial-habra-inscripcion-de-cedulas-en-sedes-de-colombia-esto-dice-la-registraduria/</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr"/>
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 06:04 p. m.</t>
+        </is>
+      </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1943,24 +1971,24 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Colpensiones explica cómo reclamar el dinero de los aportes si no logra pensionarse</t>
+          <t>Procuraduría inhabilitó por 5 años a cónsul honorario en Italia por cobro ilegal</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/economia/colpensiones-devolucion-diniero-sin-semanas-y-requisitos-401307</t>
+          <t>https://caracol.com.co/2026/06/03/procuraduria-inhabilito-por-5-anos-a-consul-honorario-en-italia-por-cobro-ilegal/</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 01:36 a. m.</t>
+          <t>04/06/2026 02:57 a. m.</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
@@ -1970,24 +1998,24 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>"Estado no puede convertirse en maquinaria electoral", advierte campaña de Abelardo De La Espriella</t>
+          <t>Último sorteo Lotería de Manizales: resultado premio mayor hoy 3 de junio</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion/elecciones/estado-no-puede-convertirse-en-maquinaria-electoral-advierte-campana-de-abelardo-de-la-espriella-rg10</t>
+          <t>https://www.lafm.com.co/sociedad/ultimo-sorteo-loteria-de-manizales-resultado-premio-mayor-hoy-3-de-junio-401332</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 01:24 a. m.</t>
+          <t>04/06/2026 02:14 a. m.</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -1997,24 +2025,24 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Gobierno confirma tres muertos en bombardeo contra círculo cercano de ‘Iván Mordisco’ en Guaviare</t>
+          <t>Un telescopio a 1,5 millones de kilómetros de la Tierra reveló algo que llevaba décadas oculto</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion/paz/gobierno-confirma-tres-muertos-en-bombardeo-contra-circulo-cercano-de-ivan-mordisco-en-guaviare-rg10</t>
+          <t>https://www.lafm.com.co/sociedad/telescopio-revela-misterio-universo-oculto-decadas-cientificos-nasa-401328</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 10:47 p. m.</t>
+          <t>04/06/2026 01:42 a. m.</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
@@ -2024,24 +2052,24 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>Abelardo De La Espriella exige a Petro y Cepeda aceptar resultados tras rectificación electoral</t>
+          <t>Claudia López se aleja de De la Espriella, reconoce la decencia de Cepeda y rechaza endosar sus votos</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion/elecciones/abelardo-de-la-espriella-exige-a-petro-y-cepeda-aceptar-resultados-tras-rectificacion-electoral-rg10</t>
+          <t>https://www.lafm.com.co/politica/claudia-lopez-desconfianza-abelardo-de-la-espriella-respaldo-cepeda-401327</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 10:34 p. m.</t>
+          <t>04/06/2026 12:51 a. m.</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -2051,24 +2079,24 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Cepeda pide a jóvenes defender el cambio y cuestiona financiación de campaña de De La Espriella</t>
+          <t>Matemático alemán que acertó el campeón de los últimos tres mundiales, predijo quién ganará en 2026</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion/elecciones/cepeda-pide-a-jovenes-defender-el-cambio-y-cuestiona-financiacion-de-campana-de-de-la-espriella-rg10</t>
+          <t>https://www.lafm.com.co/deportes/copa-mundial-fifa-2026-prediccion-aleman-acerto-campeon-2014-2018-2022-401316</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 10:25 p. m.</t>
+          <t>04/06/2026 12:49 a. m.</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
@@ -2078,24 +2106,24 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>Excandidatos definen apoyos a Cepeda o De La Espriella: Recap - programa completo 3 de junio de 2026</t>
+          <t>Capturan docente de Ética señalado de abusar de una niña en Cali: fue detenido mientras era jurado de votación</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/recap/excandidatos-definen-apoyos-a-cepeda-o-de-la-espriella-recap-programa-completo-3-de-junio-de-2026-pr30</t>
+          <t>https://www.lafm.com.co/actualidad/abuso-menor-cali-capturan-docente-etica-senalado-jurado-votacion-401322</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 10:19 p. m.</t>
+          <t>03/06/2026 11:59 p. m.</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -2105,24 +2133,24 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>El Ibagué Festival 2026 no se realizará: esto dice su organizador, la Fundación Salvi</t>
+          <t>El avión del papa: así será la operación de Iberia para mover a León XIV en su visita a España</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/sociedad/cultura/el-ibague-festival-2026-no-se-realizara-esto-dice-su-organizador-la-fundacion-salvi-rg10</t>
+          <t>https://www.lafm.com.co/internacional/papa-leon-xiv-iberia-traslado-pontifice-espana-401317</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 09:51 p. m.</t>
+          <t>03/06/2026 11:45 p. m.</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
@@ -2132,24 +2160,24 @@
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
-          <t>Loterías de Manizales, Valle, Meta y Baloto: resultados hoy miércoles 3 de junio de 2026</t>
+          <t>El misterio de los "cazatesoros" que fueron grabados saliendo de alcantarillas en Nueva York</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/economia/juegos-de-azar/loterias-de-manizales-valle-meta-y-baloto-resultados-hoy-miercoles-3-de-junio-de-2026-so35</t>
+          <t>https://www.lafm.com.co/actualidad/policia-nueva-york-investiga-hombres-401311</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 09:51 p. m.</t>
+          <t>03/06/2026 11:17 p. m.</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -2159,24 +2187,24 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Baloto y Revancha, resultado del último sorteo hoy miércoles 3 de junio de 2026</t>
+          <t>Graves emergencias en Andes, Antioquia, por las lluvias</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/economia/juegos-de-azar/baloto-y-revancha-resultado-del-ultimo-sorteo-hoy-miercoles-3-de-junio-de-2026-so35</t>
+          <t>https://www.lafm.com.co/sociedad/emergencias-lluvias-andes-antioquia-avenida-torrencial-401312</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 09:50 p. m.</t>
+          <t>03/06/2026 11:34 a. m.</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
@@ -2186,24 +2214,24 @@
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>Familiares de Dilan, niño herido en zona rural de Suárez, realizaron velatón en el sur de Cali</t>
+          <t>Abelardo de la Espriella no acepta apoyo del Partido Liberal: “es un apéndice de Petro y Cepeda”</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/regiones/pacifico/familiares-de-dilan-nino-herido-en-zona-rural-de-suarez-realizaron-velaton-en-el-sur-de-cali-rg10</t>
+          <t>https://www.lafm.com.co/politica/abelardo-de-la-espriella-no-acepta-apoyo-partido-liberal-apendice-de-petro-y-cepeda-401325</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 09:50 p. m.</t>
+          <t>01/06/2026 09:56 p. m.</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -2213,24 +2241,24 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Lotería del Meta, resultados del último sorteo hoy miércoles 3 de junio de 2026</t>
+          <t>Sin salida a la vista: continúa el cierre total de la Transversal del Sisga</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/economia/juegos-de-azar/loteria-del-meta-resultados-del-ultimo-sorteo-hoy-miercoles-3-de-junio-de-2026-so35</t>
+          <t>https://www.lafm.com.co/actualidad/transversal-sisga-colombia-cerrada-deslizamiento-401320</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 09:49 p. m.</t>
+          <t>01/06/2026 02:31 p. m.</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr">
@@ -2240,24 +2268,24 @@
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>Lotería del Valle, resultados del último sorteo hoy miércoles 3 de junio de 2026</t>
+          <t>Aida Quilcué abre las puertas de su comunidad a Westcol y lleva la campaña presidencial al mundo del streaming</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/economia/juegos-de-azar/loteria-del-valle-resultados-del-ultimo-sorteo-hoy-miercoles-3-de-junio-de-2026-so35</t>
+          <t>https://www.lafm.com.co/politica/aida-quilcue-abre-puertas-comunidad-westcol-401319</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 09:49 p. m.</t>
+          <t>31/05/2026 03:32 p. m.</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -2267,24 +2295,24 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>Lotería de Manizales, resultados del último sorteo hoy miércoles 3 de junio de 2026</t>
+          <t>"El centro político está destinado a desaparecer": representante a la Cámara lanza advertencia tras la primera vuelta presidencial</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/economia/juegos-de-azar/loteria-de-manizales-resultados-del-ultimo-sorteo-hoy-miercoles-3-de-junio-de-2026-so35</t>
+          <t>https://www.lafm.com.co/politica/centro-politico-colombia-crisis-segunda-vuelta-2026-401335</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 01:13 a. m.</t>
+          <t>31/05/2026 12:32 p. m.</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
@@ -2294,26 +2322,22 @@
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>Petro ordena bombardear campamento de ‘Mordisco’ tras confrontación entre disidencias en el Guaviare</t>
+          <t>Petro ordenó bombardear zona del Guaviare donde se enfrentaron disidencias</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/petro-ordena-bombardear-campamento-de-mordisco-tras-confrontacion-entre-disidencias-en-el-guaviare/</t>
+          <t>https://www.lafm.com.co/orden-publico/petro-ordeno-bombardear-zona-del-guaviare-donde-se-enfrentaron-disidencias-401336</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="inlineStr">
-        <is>
-          <t>03/06/2026 11:49 p. m.</t>
-        </is>
-      </c>
+      <c r="A70" s="2" t="inlineStr"/>
       <c r="B70" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2321,26 +2345,22 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>Aída Quilcué acepta invitación de Westcol y se confirma streaming desde el Cauca</t>
+          <t>Los cuatro episodios que le recuerdan a Petro tras criticar apoyo de Trump a De la Espriella</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/aida-quilcue-acepta-invitacion-de-westcol-y-se-confirma-streaming-desde-el-cauca/</t>
+          <t>https://www.lafm.com.co/politica/petro-opino-elecciones-extranjeras-cuatro-casos-401331</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="5" t="inlineStr">
-        <is>
-          <t>03/06/2026 11:04 p. m.</t>
-        </is>
-      </c>
+      <c r="A71" s="5" t="inlineStr"/>
       <c r="B71" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2348,26 +2368,22 @@
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D71" s="6" t="inlineStr">
         <is>
-          <t>Más de 800 estudiantes participaron en simulacro de emergencia volcánica en Pasto</t>
+          <t>“Petro está reconociendo que su candidato no funcionó”; cuestionan protagonismo del presidente en la campaña de Cepeda</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/mas-de-800-estudiantes-participaron-en-simulacro-de-emergencia-volcanica-en-pasto/</t>
+          <t>https://www.lafm.com.co/politica/gustavo-petro-ivan-cepeda-campana-pacto-historico-elecciones-presidenciales-2026-401330</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="inlineStr">
-        <is>
-          <t>03/06/2026 09:58 p. m.</t>
-        </is>
-      </c>
+      <c r="A72" s="2" t="inlineStr"/>
       <c r="B72" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2375,26 +2391,22 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>Llegada del fenómeno de El Niño se intensifica, según alerta de la OMM: esta es la última proyección</t>
+          <t>Movida clave en el gobierno Petro: Felipe Harman dejaría la ANT para aterrizar en la campaña de Iván Cepeda</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/llegada-del-fenomeno-de-el-nino-se-intensifica-segun-alerta-de-la-omm-esta-es-la-ultima-proyeccion/</t>
+          <t>https://www.lafm.com.co/politica/agencia-nacional-de-tierras-felipe-harman-campana-ivan-cepeda-segunda-vuelta-401326</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="5" t="inlineStr">
-        <is>
-          <t>03/06/2026 09:52 p. m.</t>
-        </is>
-      </c>
+      <c r="A73" s="5" t="inlineStr"/>
       <c r="B73" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2402,26 +2414,22 @@
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D73" s="6" t="inlineStr">
         <is>
-          <t>Elecciones segunda vuelta: ¿Personas que fueron jurados de votación repiten el 21 de junio?</t>
+          <t>Capturan a la mamá de la bebé que murió tras ser víctima de abuso en El Espinal, Tolima</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/elecciones-segunda-vuelta-personas-que-fueron-jurados-de-votacion-repiten-el-21-de-junio/</t>
+          <t>https://www.lafm.com.co/actualidad/capturan-mama-de-bebe-que-murio-en-el-espinal-tolima-401324</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="inlineStr">
-        <is>
-          <t>03/06/2026 09:50 p. m.</t>
-        </is>
-      </c>
+      <c r="A74" s="2" t="inlineStr"/>
       <c r="B74" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2429,26 +2437,22 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>Capturan a la ‘Mona’, cabecilla de disidencias, señalada de trasladar menores entre Cauca y Guaviare</t>
+          <t>Entró en vigencia la ‘Ley Sara Sofía’, que crea un sistema de alerta para encontrar niños desaparecidos</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/capturan-a-la-mona-cabecilla-de-disidencias-senalada-de-trasladar-menores-reclutados-entre-cauca/</t>
+          <t>https://www.lafm.com.co/politica/ley-sara-sofia-entra-en-vigencia-sistema-alerta-encontrar-ninos-desaparecidos-colombia-401321</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="5" t="inlineStr">
-        <is>
-          <t>03/06/2026 09:36 p. m.</t>
-        </is>
-      </c>
+      <c r="A75" s="5" t="inlineStr"/>
       <c r="B75" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2456,26 +2460,22 @@
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr">
         <is>
-          <t>¿Cuánto gana el vicepresidente de Colombia en 2026? Este sería el salario de Quilcué o Restrepo</t>
+          <t>Atención conductores: licencia de conducción cambia en 2026 para estas personas; estos son los nuevos exámenes y costos</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/cuanto-gana-el-vicepresidente-de-colombia-en-2026-este-seria-el-salario-de-quilcue-o-restrepo/</t>
+          <t>https://www.lafm.com.co/actualidad/licencia-conduccion-cambia-2026-nuevos-examenes-y-costos-401318</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="inlineStr">
-        <is>
-          <t>03/06/2026 09:22 p. m.</t>
-        </is>
-      </c>
+      <c r="A76" s="2" t="inlineStr"/>
       <c r="B76" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2483,24 +2483,24 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>Quinto ciclo Colombia Mayor: Prosperidad Social confirma fechas y canales para reclamar el subsidio</t>
+          <t>Colpensiones explica cómo reclamar el dinero de los aportes si no logra pensionarse</t>
         </is>
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/quinto-ciclo-colombia-mayor-prosperidad-social-confirma-fechas-y-canales-para-reclamar-el-subsidio/</t>
+          <t>https://www.lafm.com.co/economia/colpensiones-devolucion-diniero-sin-semanas-y-requisitos-401307</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 08:35 p. m.</t>
+          <t>04/06/2026 01:36 a. m.</t>
         </is>
       </c>
       <c r="B77" s="5" t="inlineStr">
@@ -2510,24 +2510,24 @@
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D77" s="6" t="inlineStr">
         <is>
-          <t>Abelardo de la Espriella rechaza respaldo del Partido Liberal: “Es un apéndice de Petro y Cepeda”</t>
+          <t>"Estado no puede convertirse en maquinaria electoral", advierte campaña de Abelardo De La Espriella</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/abelardo-de-la-espriella-rechaza-respaldo-liberal-es-un-apendice-de-petro-y-cepeda/</t>
+          <t>https://www.bluradio.com/nacion/elecciones/estado-no-puede-convertirse-en-maquinaria-electoral-advierte-campana-de-abelardo-de-la-espriella-rg10</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 07:48 p. m.</t>
+          <t>04/06/2026 01:24 a. m.</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -2537,24 +2537,24 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>Fiscalía capturó a la madre de Mía Cataleya en El Espinal</t>
+          <t>Gobierno confirma tres muertos en bombardeo contra círculo cercano de ‘Iván Mordisco’ en Guaviare</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/fiscalia-capturo-a-la-madre-de-mia-cataleya-en-el-espinal/</t>
+          <t>https://www.bluradio.com/nacion/paz/gobierno-confirma-tres-muertos-en-bombardeo-contra-circulo-cercano-de-ivan-mordisco-en-guaviare-rg10</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 07:46 p. m.</t>
+          <t>03/06/2026 10:47 p. m.</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
@@ -2564,24 +2564,24 @@
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
         <is>
-          <t>Resultados Lotería del Valle, Manizales, Meta y Baloto HOY 03 de junio, 2026: último sorteo y premio</t>
+          <t>Abelardo De La Espriella exige a Petro y Cepeda aceptar resultados tras rectificación electoral</t>
         </is>
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/resultados-loteria-del-valle-manizales-meta-y-baloto-hoy-03-de-junio-2026-ultimo-sorteo-y-premio/</t>
+          <t>https://www.bluradio.com/nacion/elecciones/abelardo-de-la-espriella-exige-a-petro-y-cepeda-aceptar-resultados-tras-rectificacion-electoral-rg10</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 07:24 p. m.</t>
+          <t>03/06/2026 10:34 p. m.</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -2591,24 +2591,24 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>Centro Democrático en Antioquia anuncia respaldo a Abelardo de la Espriella para la segunda vuelta</t>
+          <t>Cepeda pide a jóvenes defender el cambio y cuestiona financiación de campaña de De La Espriella</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/centro-democratico-en-antioquia-anuncia-respaldo-a-abelardo-de-la-espriella-para-la-segunda-vuelta/</t>
+          <t>https://www.bluradio.com/nacion/elecciones/cepeda-pide-a-jovenes-defender-el-cambio-y-cuestiona-financiacion-de-campana-de-de-la-espriella-rg10</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 07:12 p. m.</t>
+          <t>03/06/2026 10:25 p. m.</t>
         </is>
       </c>
       <c r="B81" s="5" t="inlineStr">
@@ -2618,24 +2618,24 @@
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D81" s="6" t="inlineStr">
         <is>
-          <t>Felipe Harman, director de la ANT sale del Gobierno para apoyar la campaña de Iván Cepeda</t>
+          <t>Excandidatos definen apoyos a Cepeda o De La Espriella: Recap - programa completo 3 de junio de 2026</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/felipe-harman-director-de-la-ant-sale-del-gobierno-para-apoyar-la-campana-de-ivan-cepeda/</t>
+          <t>https://www.bluradio.com/recap/excandidatos-definen-apoyos-a-cepeda-o-de-la-espriella-recap-programa-completo-3-de-junio-de-2026-pr30</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 07:01 p. m.</t>
+          <t>03/06/2026 10:19 p. m.</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -2645,24 +2645,24 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>Petro pide al CNE atender su denuncia sobre presunto fraude, pese a aclaración de la Registraduría</t>
+          <t>El Ibagué Festival 2026 no se realizará: esto dice su organizador, la Fundación Salvi</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/petro-pide-al-cne-atender-su-denuncia-sobre-presunto-fraude-pese-a-aclaracion-de-la-registraduria/</t>
+          <t>https://www.bluradio.com/sociedad/cultura/el-ibague-festival-2026-no-se-realizara-esto-dice-su-organizador-la-fundacion-salvi-rg10</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 06:48 p. m.</t>
+          <t>03/06/2026 09:51 p. m.</t>
         </is>
       </c>
       <c r="B83" s="5" t="inlineStr">
@@ -2672,24 +2672,24 @@
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D83" s="6" t="inlineStr">
         <is>
-          <t>Abren cupos para el Servicio Social para la Paz: certifica el servicio militar y entrega auxilio</t>
+          <t>Loterías de Manizales, Valle, Meta y Baloto: resultados hoy miércoles 3 de junio de 2026</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/03/abren-cupos-para-el-servicio-social-para-la-paz-certifica-el-servicio-militar-y-entrega-auxilio/</t>
+          <t>https://www.bluradio.com/economia/juegos-de-azar/loterias-de-manizales-valle-meta-y-baloto-resultados-hoy-miercoles-3-de-junio-de-2026-so35</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 06:41 p. m.</t>
+          <t>03/06/2026 09:51 p. m.</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -2699,24 +2699,24 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>Petro cuestiona solicitud de indagatoria: “Ya amenazaron con encarcelarme sin cometer un delito”</t>
+          <t>Baloto y Revancha, resultado del último sorteo hoy miércoles 3 de junio de 2026</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/03/petro-tras-solicitud-de-indagatoria-ya-amenazaron-con-encarcelarme-sin-cometer-un-delito/</t>
+          <t>https://www.bluradio.com/economia/juegos-de-azar/baloto-y-revancha-resultado-del-ultimo-sorteo-hoy-miercoles-3-de-junio-de-2026-so35</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 06:41 p. m.</t>
+          <t>03/06/2026 09:50 p. m.</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr">
@@ -2726,24 +2726,24 @@
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D85" s="6" t="inlineStr">
         <is>
-          <t>OEA pide a grupos armados no interferir en segunda vuelta y a candidatos recibir resultados en paz</t>
+          <t>Familiares de Dilan, niño herido en zona rural de Suárez, realizaron velatón en el sur de Cali</t>
         </is>
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/03/oea-pide-a-grupos-armados-no-interferir-en-segunda-vuelta-y-a-candidatos-recibir-resultados-en-paz/</t>
+          <t>https://www.bluradio.com/regiones/pacifico/familiares-de-dilan-nino-herido-en-zona-rural-de-suarez-realizaron-velaton-en-el-sur-de-cali-rg10</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 06:23 p. m.</t>
+          <t>03/06/2026 09:50 p. m.</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -2753,24 +2753,24 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>Elecciones y Mundial: ¿Habrá inscripción de cédulas en sedes de Colombia? Esto dice la Registraduría</t>
+          <t>Lotería del Meta, resultados del último sorteo hoy miércoles 3 de junio de 2026</t>
         </is>
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/03/elecciones-y-mundial-habra-inscripcion-de-cedulas-en-sedes-de-colombia-esto-dice-la-registraduria/</t>
+          <t>https://www.bluradio.com/economia/juegos-de-azar/loteria-del-meta-resultados-del-ultimo-sorteo-hoy-miercoles-3-de-junio-de-2026-so35</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 06:04 p. m.</t>
+          <t>03/06/2026 09:49 p. m.</t>
         </is>
       </c>
       <c r="B87" s="5" t="inlineStr">
@@ -2780,24 +2780,24 @@
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D87" s="6" t="inlineStr">
         <is>
-          <t>Procuraduría inhabilitó por 5 años a cónsul honorario en Italia por cobro ilegal</t>
+          <t>Lotería del Valle, resultados del último sorteo hoy miércoles 3 de junio de 2026</t>
         </is>
       </c>
       <c r="E87" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/03/procuraduria-inhabilito-por-5-anos-a-consul-honorario-en-italia-por-cobro-ilegal/</t>
+          <t>https://www.bluradio.com/economia/juegos-de-azar/loteria-del-valle-resultados-del-ultimo-sorteo-hoy-miercoles-3-de-junio-de-2026-so35</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 06:00 p. m.</t>
+          <t>03/06/2026 09:49 p. m.</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -2807,24 +2807,24 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>Trump participará en la cumbre de la OTAN del 7 y 8 de julio en Turquía</t>
+          <t>Lotería de Manizales, resultados del último sorteo hoy miércoles 3 de junio de 2026</t>
         </is>
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/03/trump-participara-en-la-cumbre-de-la-otan-del-7-y-8-de-julio-en-turquia/</t>
+          <t>https://www.bluradio.com/economia/juegos-de-azar/loteria-de-manizales-resultados-del-ultimo-sorteo-hoy-miercoles-3-de-junio-de-2026-so35</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 12:33 a. m.</t>
+          <t>04/06/2026 12:48 a. m.</t>
         </is>
       </c>
       <c r="B89" s="5" t="inlineStr">
@@ -2834,26 +2834,22 @@
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D89" s="6" t="inlineStr">
         <is>
-          <t>Corte Constitucional tumba polémicas restricciones a encuestas electorales</t>
+          <t>El regreso deloutsider: Trump no inventó la nueva derecha latinoamericana</t>
         </is>
       </c>
       <c r="E89" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/colombia/2026/06/04/corte-constitucional-tumba-polemicas-restricciones-a-encuestas-electorales/</t>
+          <t>https://www.elcolombiano.com/internacional/el-regreso-del-outsider-trump-no-invento-la-nueva-derecha-latinoamericana-DC37353110</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="inlineStr">
-        <is>
-          <t>04/06/2026 12:33 a. m.</t>
-        </is>
-      </c>
+      <c r="A90" s="2" t="inlineStr"/>
       <c r="B90" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2861,26 +2857,22 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>El “salvador” Benedetti no llegaría a la campaña de Iván Cepeda y otros detalles inéditos</t>
         </is>
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/colombia/</t>
+          <t>https://www.elcolombiano.com/especiales/elecciones-2026/armando-benedetti-no-llegaria-campana-ivan-cepeda-detalles-ineditos-elecciones-2026-IC37352596</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="5" t="inlineStr">
-        <is>
-          <t>03/06/2026 11:42 p. m.</t>
-        </is>
-      </c>
+      <c r="A91" s="5" t="inlineStr"/>
       <c r="B91" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2888,26 +2880,22 @@
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D91" s="6" t="inlineStr">
         <is>
-          <t>Israel y Líbano sellan acuerdo que podría cambiar el conflicto</t>
+          <t>“Pueden tener el apoyo de Petro, pero no pueden violar la ley”: alcalde Federico Gutiérrez sobre desmanes en la UdeA</t>
         </is>
       </c>
       <c r="E91" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/mundo/2026/06/03/israel-y-libano-sellan-acuerdo-que-podria-cambiar-el-conflicto/</t>
+          <t>https://www.elcolombiano.com/medellin/federico-gutierrez-rechaza-disturbios-en-la-universidad-de-antioquia-DE37337598</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="2" t="inlineStr">
-        <is>
-          <t>03/06/2026 11:28 p. m.</t>
-        </is>
-      </c>
+      <c r="A92" s="2" t="inlineStr"/>
       <c r="B92" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2915,26 +2903,22 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>NBA: los New York Knicks golpean primero en las Finales y sorprenden a Spurs</t>
+          <t>Creciente de quebrada en Andes obligó a evacuación preventiva del corregimiento Santa Inés</t>
         </is>
       </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/deportes/2026/06/03/nba-los-new-york-knicks-golpean-primero-en-las-finales-y-sorprenden-a-spurs/</t>
+          <t>https://www.elcolombiano.com/antioquia/emergencia-creciente-quebrada-corregimiento-santa-ines-andes-LD37348535</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="5" t="inlineStr">
-        <is>
-          <t>03/06/2026 11:28 p. m.</t>
-        </is>
-      </c>
+      <c r="A93" s="5" t="inlineStr"/>
       <c r="B93" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2942,26 +2926,22 @@
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D93" s="6" t="inlineStr">
         <is>
-          <t>Deportes</t>
+          <t>Así estarían presionando las disidencias a comunidades de Nariño para votar por Cepeda</t>
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/deportes/</t>
+          <t>https://www.elcolombiano.com/especiales/elecciones-2026/denuncian-presiones-grupos-armados-elecciones-por-ivan-cepeda-OG37314138</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="2" t="inlineStr">
-        <is>
-          <t>03/06/2026 10:09 p. m.</t>
-        </is>
-      </c>
+      <c r="A94" s="2" t="inlineStr"/>
       <c r="B94" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2969,26 +2949,22 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>Segunda vuelta: así se mueven los apoyos a Cepeda y De La Espriella</t>
+          <t>Colombia, entre los seis países con peor desempeño laboral de la Ocde</t>
         </is>
       </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/colombia/2026/06/03/segunda-vuelta-asi-se-mueven-los-apoyos-a-cepeda-y-de-la-espriella/</t>
+          <t>https://www.elcolombiano.com/negocios/colombia-peor-desempeno-laboral-ocde-desempleo-IF37326097</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="5" t="inlineStr">
-        <is>
-          <t>03/06/2026 10:07 p. m.</t>
-        </is>
-      </c>
+      <c r="A95" s="5" t="inlineStr"/>
       <c r="B95" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2996,26 +2972,22 @@
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D95" s="6" t="inlineStr">
         <is>
-          <t>Exportaciones: esta es la aduana líder en estas operaciones en Colombia</t>
+          <t>Quien fuera: Alcalde de Sincelejo pidió un mes de permiso para ir a ver el Mundial ¡y se lo dieron!</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/economica/2026/06/03/exportaciones-esta-es-la-aduana-lider-en-estas-operaciones-en-colombia/</t>
+          <t>https://www.elcolombiano.com/colombia/alcalde-sincelejo-permiso-mes-mundial-2026-CF37323724</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="2" t="inlineStr">
-        <is>
-          <t>03/06/2026 10:07 p. m.</t>
-        </is>
-      </c>
+      <c r="A96" s="2" t="inlineStr"/>
       <c r="B96" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3023,26 +2995,22 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>Económica</t>
+          <t>Atención: Estación San Germán del Metro de la 80 será la primera subterránea del sistema y de Colombia</t>
         </is>
       </c>
       <c r="E96" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/economica/</t>
+          <t>https://www.elcolombiano.com/medellin/estacion-san-german-subterranea-metro-medellin-NG37314081</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="5" t="inlineStr">
-        <is>
-          <t>03/06/2026 09:57 p. m.</t>
-        </is>
-      </c>
+      <c r="A97" s="5" t="inlineStr"/>
       <c r="B97" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3050,26 +3018,22 @@
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D97" s="6" t="inlineStr">
         <is>
-          <t>¡Aberrate! Alias ‘Curra’ habría realizado tocamiento a una menor de 14 años</t>
+          <t>Registraduría desmontó, uno por uno, los señalamientos de Petro de supuesto fraude electoral</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/sucesos/2026/06/03/aberrate-alias-curra-habria-cometido-actos-a-una-menor-de-14-anos-en-cartagena/</t>
+          <t>https://www.elcolombiano.com/especiales/elecciones-2026/gustavo-petro-resultados-elecciones-registraduria-desmiente-senalamientos-fraude-IP37297870</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="inlineStr">
-        <is>
-          <t>03/06/2026 09:23 p. m.</t>
-        </is>
-      </c>
+      <c r="A98" s="2" t="inlineStr"/>
       <c r="B98" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3077,26 +3041,22 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>Sicarios irrumpieron en una calle de La Campiña y dejaron a un joven herido</t>
+          <t>Operativo destapa helicóptero con pasado oscuro y motor Rolls-Royce</t>
         </is>
       </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/sucesos/2026/06/03/sicarios-irrumpieron-en-una-calle-de-la-campina-y-dejaron-a-un-joven-herido/</t>
+          <t>https://www.elcolombiano.com/colombia/ejercito-incauta-helicoptero-de-la-mafia-NG33717192</t>
         </is>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="5" t="inlineStr">
-        <is>
-          <t>03/06/2026 09:00 p. m.</t>
-        </is>
-      </c>
+      <c r="A99" s="5" t="inlineStr"/>
       <c r="B99" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3104,26 +3064,22 @@
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D99" s="6" t="inlineStr">
         <is>
-          <t>Claudia López ya tomó una decisión para la segunda vuelta: ¿De la Espriella o Cepeda?</t>
+          <t>Así se mueven los 5 clanes en la Costa que según De la Espriella hacen parte de una operación de compra de votos a favor de Cepeda</t>
         </is>
       </c>
       <c r="E99" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/politica/2026/06/03/claudia-lopez-ya-tomo-una-decision-para-la-segunda-vuelta-de-la-espriella-o-cepeda/</t>
+          <t>https://www.elcolombiano.com/colombia/de-la-espriella-estas-son-las-familias-denunciados-de-compra-de-votos-GC37352433</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="inlineStr">
-        <is>
-          <t>03/06/2026 09:00 p. m.</t>
-        </is>
-      </c>
+      <c r="A100" s="2" t="inlineStr"/>
       <c r="B100" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3131,26 +3087,22 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>Política</t>
+          <t>Daniel Muñoz publicó emotivo video sobre su preparación para disputar su primer Mundial</t>
         </is>
       </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/politica/</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/daniel-munoz-publico-video-con-su-preparacion-y-recuperacion-con-miras-al-mundial-de-norteamerica-CD37348820</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="5" t="inlineStr">
-        <is>
-          <t>03/06/2026 08:32 p. m.</t>
-        </is>
-      </c>
+      <c r="A101" s="5" t="inlineStr"/>
       <c r="B101" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3158,26 +3110,22 @@
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D101" s="6" t="inlineStr">
         <is>
-          <t>A ‘César’ y ‘Anuar’ los pillaron vendiendo droga: acumulan más de 20 anotaciones</t>
+          <t>Corte tumbó estas dos reglas clave de la “Ley de Encuestas”: tienen que ver con los tiempos de publicación y microdatos</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/sucesos/2026/06/03/a-cesar-y-anuar-los-pillaron-vendiendo-droga-acumulan-mas-de-20-anotaciones/</t>
+          <t>https://www.elcolombiano.com/colombia/corte-constitucional-tumba-dos-articulos-de-ley-de-encuestas-esto-se-sabe-KD37348354</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="2" t="inlineStr">
-        <is>
-          <t>03/06/2026 08:23 p. m.</t>
-        </is>
-      </c>
+      <c r="A102" s="2" t="inlineStr"/>
       <c r="B102" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3185,26 +3133,22 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>Jerau se pone modo mundialista y le canta a la paz con sabor caribeño y africano</t>
+          <t>Así se jugará la primera fecha de la Liga BetPlay 2: la Dimayor oficializó el calendario del segundo semestre</t>
         </is>
       </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/farandula/2026/06/03/jerau-se-pone-modo-mundialista-y-le-canta-a-la-paz-con-sabor-caribeno-y-africano/</t>
+          <t>https://www.elcolombiano.com/deportes/futbol/asi-se-jugara-la-primera-fecha-de-la-liga-betplay-2-LD37343448</t>
         </is>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="5" t="inlineStr">
-        <is>
-          <t>03/06/2026 08:23 p. m.</t>
-        </is>
-      </c>
+      <c r="A103" s="5" t="inlineStr"/>
       <c r="B103" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3212,26 +3156,22 @@
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D103" s="6" t="inlineStr">
         <is>
-          <t>Farándula</t>
+          <t>“Todos tenemos que empujar a Nacional para la remontada”: Luis Fernando “Chonto” Herrera</t>
         </is>
       </c>
       <c r="E103" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/farandula/</t>
+          <t>https://www.elcolombiano.com/multimedia/videos/todos-tenemos-que-empujar-a-nacional-para-la-remontada-luis-fernando-chonto-herrera-ND37344922</t>
         </is>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="2" t="inlineStr">
-        <is>
-          <t>03/06/2026 08:08 p. m.</t>
-        </is>
-      </c>
+      <c r="A104" s="2" t="inlineStr"/>
       <c r="B104" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3239,26 +3179,22 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>Temblor de magnitud 5.08 sacude a California</t>
+          <t>Corrupción en Área Metropolitana: representante de firma investigada ofrece información sobre presunta red</t>
         </is>
       </c>
       <c r="E104" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/mundo/2026/06/03/temblor-de-magnitud-508-sacude-a-california/</t>
+          <t>https://www.elcolombiano.com/medellin/corrupcion-area-metropolitana-parque-de-las-aguas-medellin-DD37341525</t>
         </is>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="5" t="inlineStr">
-        <is>
-          <t>03/06/2026 07:35 p. m.</t>
-        </is>
-      </c>
+      <c r="A105" s="5" t="inlineStr"/>
       <c r="B105" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3266,26 +3202,22 @@
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D105" s="6" t="inlineStr">
         <is>
-          <t>MinTrabajo y Avianca impulsan empleos para personas con discapacidad</t>
+          <t>La Selección Colombia emprende el viaje para el Mundial este jueves: ¿a qué horas y cuál es su itinerario?</t>
         </is>
       </c>
       <c r="E105" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/colombia/2026/06/03/mintrabajo-y-avianca-impulsan-empleos-para-personas-con-discapacidad/</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/seleccion-colombia-viaje-mundial-itinerario-jueves-san-diego-amistoso-jordania-LD37343787</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="2" t="inlineStr">
-        <is>
-          <t>03/06/2026 06:52 p. m.</t>
-        </is>
-      </c>
+      <c r="A106" s="2" t="inlineStr"/>
       <c r="B106" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3293,26 +3225,22 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D106" s="3" t="inlineStr">
         <is>
-          <t>Mataron  a Deison Morales mientras compartía con su familia: había recibido amenazas</t>
+          <t>Mundial: Bayern Múnich y Manchester City son los equipos que más futbolistas tendrán en Norteamérica 2026</t>
         </is>
       </c>
       <c r="E106" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/sucesos/2026/06/03/acabaron-con-deison-morales-mientras-compartia-con-su-familia-habia-recibido-amenazas/</t>
+          <t>https://www.elcolombiano.com/deportes/futbol/mundial-2026-equipos-que-mas-jugadores-aportan-bayern-munich-manchester-city-2026-CE37333625</t>
         </is>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="5" t="inlineStr">
-        <is>
-          <t>03/06/2026 06:02 p. m.</t>
-        </is>
-      </c>
+      <c r="A107" s="5" t="inlineStr"/>
       <c r="B107" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3320,26 +3248,22 @@
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D107" s="6" t="inlineStr">
         <is>
-          <t>A la cárcel dos hombres señalados de agredir a un niño de 3 años y a una mujer</t>
+          <t>Video | Pasajero intentó abrir una puerta y obligó a desviar el avión a Miami</t>
         </is>
       </c>
       <c r="E107" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/sucesos/2026/06/03/a-la-carcel-dos-hombres-senalados-de-agredir-a-un-nino-de-3-anos-y-a-una-mujer/</t>
+          <t>https://www.elcolombiano.com/internacional/pasajero-intenta-abrir-puerta-avion-desviar-avion-a-miami-AE37331427</t>
         </is>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="inlineStr">
-        <is>
-          <t>03/06/2026 04:00 p. m.</t>
-        </is>
-      </c>
+      <c r="A108" s="2" t="inlineStr"/>
       <c r="B108" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3347,17 +3271,17 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D108" s="3" t="inlineStr">
         <is>
-          <t>Cartagena espera a J Balvin: crece la expectativa por sus invitados sorpresa</t>
+          <t>Este es el decálogo de Fajardo: no a la Constituyente, fin de “paz total” y ordenar la salud</t>
         </is>
       </c>
       <c r="E108" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/farandula/2026/06/03/cartagena-espera-a-j-balvin-crece-la-expectativa-por-sus-invitados-sorpresa/</t>
+          <t>https://www.elcolombiano.com/colombia/politica/elecciones-2026-decalogo-sergio-fajardo-constituyente-paz-total-sistema-salud-DF37328092</t>
         </is>
       </c>
     </row>
@@ -3370,17 +3294,17 @@
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D109" s="6" t="inlineStr">
         <is>
-          <t>Así puedes ganar entradas dobles para ver a J Balvin en Cartagena</t>
+          <t>Seis universidades colombianas entran al ranking de las 2.000 mejores del mundo: la Nacional lidera el listado</t>
         </is>
       </c>
       <c r="E109" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/cartagena/2026/06/02/asi-puedes-ganar-entradas-dobles-para-ver-a-jbalvin-en-cartagena/</t>
+          <t>https://www.elcolombiano.com/colombia/educacion/mejores-universidades-colombia-ranking-cwur-NF37328630</t>
         </is>
       </c>
     </row>
@@ -3393,17 +3317,17 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D110" s="3" t="inlineStr">
         <is>
-          <t>Cartagena</t>
+          <t>Pese a ataques violentos, Antioquia sigue bajando cifra de homicidios ¿Cuánto redujeron?</t>
         </is>
       </c>
       <c r="E110" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/cartagena/</t>
+          <t>https://www.elcolombiano.com/antioquia/homicidios-antioquia-reduccion-2026-GE37333566</t>
         </is>
       </c>
     </row>
@@ -3416,17 +3340,17 @@
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D111" s="6" t="inlineStr">
         <is>
-          <t>Dumek Turbay y Hamilton se reconcilian: “No quería estar lejos de su ciudad”</t>
+          <t>Ponencia pide abrir investigación y llamar a indagatoria a Petro por financiación de campaña</t>
         </is>
       </c>
       <c r="E111" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/farandula/2026/06/02/dumek-turbay-y-hamilton-se-reconcilian-no-queria-estar-lejos-de-su-ciudad/</t>
+          <t>https://www.elcolombiano.com/colombia/petro-comision-de-acusacion-analizara-llamado-a-indagatoria-a-petro-LE37333549</t>
         </is>
       </c>
     </row>
@@ -3439,17 +3363,17 @@
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D112" s="3" t="inlineStr">
         <is>
-          <t>Luister La Voz celebra a Cartagena: detalles del concierto de este 1 de junio</t>
+          <t>Prima de los hermanos Mucutuy murió en combates entre disidencias de las Farc en Guaviare</t>
         </is>
       </c>
       <c r="E112" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/farandula/2026/06/01/luister-la-voz-celebra-a-cartagena-detalles-del-concierto-de-este-1-de-junio/</t>
+          <t>https://www.elcolombiano.com/colombia/prima-hermanos-mucutuy-murio-combates-disidencias-farc-guaviare-MF37328501</t>
         </is>
       </c>
     </row>
@@ -3462,26 +3386,22 @@
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D113" s="6" t="inlineStr">
         <is>
-          <t>Ser cartagenero lejos de Cartagena: ¿qué es lo que más extrañan quienes dejan la ciudad?</t>
+          <t>Nacional no baja los brazos: estas son las remontadas que alimentan la esperanza verde ante Junior</t>
         </is>
       </c>
       <c r="E113" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/cartagena/2026/06/01/ser-cartagenero-lejos-de-cartagena-que-es-lo-que-mas-extranan-quienes-dejan-la-ciudad/</t>
+          <t>https://www.elcolombiano.com/deportes/futbol/atletico-nacional-remontadas-historicas-final-junior-vuelta-liga-betplay-atanasio-girardot-OE37331870</t>
         </is>
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="2" t="inlineStr">
-        <is>
-          <t>04/06/2026 12:06 a. m.</t>
-        </is>
-      </c>
+      <c r="A114" s="2" t="inlineStr"/>
       <c r="B114" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3489,26 +3409,22 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D114" s="3" t="inlineStr">
         <is>
-          <t>La mejor campaña era hacer un buen gobierno</t>
+          <t>Medellín explica las inversiones por casi $3 billones para tener un aire más limpio</t>
         </is>
       </c>
       <c r="E114" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/blancainesduran/la-mejor-campana-era-hacer-un-buen-gobierno/</t>
+          <t>https://www.elcolombiano.com/medellin/medellin-inversion-reducir-contaminacion-calidad-aire-GF37329593</t>
         </is>
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="5" t="inlineStr">
-        <is>
-          <t>04/06/2026 12:05 a. m.</t>
-        </is>
-      </c>
+      <c r="A115" s="5" t="inlineStr"/>
       <c r="B115" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3516,26 +3432,22 @@
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D115" s="6" t="inlineStr">
         <is>
-          <t>De Santa Marta a Tuvalu: cultivar la frágil esperanza</t>
+          <t>Parrandas de Jhon Jáder Durán tienen desesperados a sus vecinos en Llanogrande: “No nos dejan dormir”</t>
         </is>
       </c>
       <c r="E115" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/german-i-andrade-/de-santa-marta-a-tuvalu-cultivar-la-fragil-esperanza/</t>
+          <t>https://www.elcolombiano.com/antioquia/quejas-fiestas-jhon-jader-duran-finca-rionegro-antioquia-FG37316715</t>
         </is>
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="2" t="inlineStr">
-        <is>
-          <t>04/06/2026 12:05 a. m.</t>
-        </is>
-      </c>
+      <c r="A116" s="2" t="inlineStr"/>
       <c r="B116" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3543,26 +3455,22 @@
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D116" s="3" t="inlineStr">
         <is>
-          <t>¿Verde + rosa = blanco?</t>
+          <t>¿Clint Eastwood se retira a los 96 años? Lo que se sabe de las declaraciones de su hijo</t>
         </is>
       </c>
       <c r="E116" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/brigitte-lg-baptiste/verde-rosa-blanco/</t>
+          <t>https://www.elcolombiano.com/cultura/cine/clint-eastwood-retiro-jubilacion-hijos-verdad-mentira-96-OF37325029</t>
         </is>
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="5" t="inlineStr">
-        <is>
-          <t>04/06/2026 12:05 a. m.</t>
-        </is>
-      </c>
+      <c r="A117" s="5" t="inlineStr"/>
       <c r="B117" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3570,26 +3478,22 @@
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D117" s="6" t="inlineStr">
         <is>
-          <t>Sobre Mozart y la inteligencia artificial</t>
+          <t>Aída Quilcué aceptó la invitación de Westcol para un streaming</t>
         </is>
       </c>
       <c r="E117" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/manuel-drezner/sobre-mozart-y-la-inteligencia-artificial/</t>
+          <t>https://www.elcolombiano.com/colombia/aida-quilcue-acepta-hacer-streaming-con-westcol-ND37348371</t>
         </is>
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="2" t="inlineStr">
-        <is>
-          <t>04/06/2026 12:05 a. m.</t>
-        </is>
-      </c>
+      <c r="A118" s="2" t="inlineStr"/>
       <c r="B118" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3597,24 +3501,24 @@
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D118" s="3" t="inlineStr">
         <is>
-          <t>Más allá del voto en blanco</t>
+          <t>Denuncian a Gustavo Petro ante la MOE por hacer “intervención política” y poner en riesgo la contienda electoral</t>
         </is>
       </c>
       <c r="E118" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/cristinacarrizosa/mas-alla-del-voto-en-blanco/</t>
+          <t>https://www.elcolombiano.com/colombia/denuncian-petro-moe-declaraciones-elecciones-uso-recursos-campana-MG37315339</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 12:05 a. m.</t>
+          <t>04/06/2026 12:33 a. m.</t>
         </is>
       </c>
       <c r="B119" s="5" t="inlineStr">
@@ -3624,24 +3528,24 @@
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D119" s="6" t="inlineStr">
         <is>
-          <t>Líder del equipo digital de De la Espriella denunciado por violencia sexual</t>
+          <t>Corte Constitucional tumba polémicas restricciones a encuestas electorales</t>
         </is>
       </c>
       <c r="E119" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/catalina-ruiz-navarro/lider-del-equipo-digital-de-de-la-espriella-denunciado-por-violencia-sexual/</t>
+          <t>https://www.eluniversal.com.co/colombia/2026/06/04/corte-constitucional-tumba-polemicas-restricciones-a-encuestas-electorales/</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 12:05 a. m.</t>
+          <t>04/06/2026 12:33 a. m.</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
@@ -3651,24 +3555,24 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D120" s="3" t="inlineStr">
         <is>
-          <t>Los votos están ahí</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E120" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/javier-ortiz/los-votos-estan-ahi/</t>
+          <t>https://www.eluniversal.com.co/colombia/</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 12:04 a. m.</t>
+          <t>03/06/2026 11:42 p. m.</t>
         </is>
       </c>
       <c r="B121" s="5" t="inlineStr">
@@ -3678,24 +3582,24 @@
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D121" s="6" t="inlineStr">
         <is>
-          <t>Gurropín, corrupto dictador venerado por la izquierda populista</t>
+          <t>Israel y Líbano sellan acuerdo que podría cambiar el conflicto</t>
         </is>
       </c>
       <c r="E121" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/mauricio-rubio/gurropin-corrupto-dictador-venerado-por-la-izquierda-populista/</t>
+          <t>https://www.eluniversal.com.co/mundo/2026/06/03/israel-y-libano-sellan-acuerdo-que-podria-cambiar-el-conflicto/</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 12:04 a. m.</t>
+          <t>03/06/2026 11:28 p. m.</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
@@ -3705,24 +3609,24 @@
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D122" s="3" t="inlineStr">
         <is>
-          <t>Quiero hablar con las flores</t>
+          <t>NBA: los New York Knicks golpean primero en las Finales y sorprenden a Spurs</t>
         </is>
       </c>
       <c r="E122" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/juan-david-zuloaga-d-/quiero-hablar-con-las-flores/</t>
+          <t>https://www.eluniversal.com.co/deportes/2026/06/03/nba-los-new-york-knicks-golpean-primero-en-las-finales-y-sorprenden-a-spurs/</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 12:00 a. m.</t>
+          <t>03/06/2026 11:28 p. m.</t>
         </is>
       </c>
       <c r="B123" s="5" t="inlineStr">
@@ -3732,24 +3636,24 @@
       </c>
       <c r="C123" s="5" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D123" s="6" t="inlineStr">
         <is>
-          <t>Atrapados entre la espada, la pared y la improvisación</t>
+          <t>Deportes</t>
         </is>
       </c>
       <c r="E123" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/lectores/cartas/atrapados-entre-la-espada-la-pared-y-la-improvisacion/</t>
+          <t>https://www.eluniversal.com.co/deportes/</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 12:04 a. m.</t>
+          <t>03/06/2026 10:09 p. m.</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
@@ -3759,22 +3663,26 @@
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D124" s="3" t="inlineStr">
         <is>
-          <t>El regreso deloutsider: Trump no inventó la nueva derecha latinoamericana</t>
+          <t>Segunda vuelta: así se mueven los apoyos a Cepeda y De La Espriella</t>
         </is>
       </c>
       <c r="E124" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/internacional/el-regreso-del-outsider-trump-no-invento-la-nueva-derecha-latinoamericana-DC37353110</t>
+          <t>https://www.eluniversal.com.co/colombia/2026/06/03/segunda-vuelta-asi-se-mueven-los-apoyos-a-cepeda-y-de-la-espriella/</t>
         </is>
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="5" t="inlineStr"/>
+      <c r="A125" s="5" t="inlineStr">
+        <is>
+          <t>03/06/2026 10:07 p. m.</t>
+        </is>
+      </c>
       <c r="B125" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3782,22 +3690,26 @@
       </c>
       <c r="C125" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D125" s="6" t="inlineStr">
         <is>
-          <t>El “salvador” Benedetti no llegaría a la campaña de Iván Cepeda y otros detalles inéditos</t>
+          <t>Exportaciones: esta es la aduana líder en estas operaciones en Colombia</t>
         </is>
       </c>
       <c r="E125" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/elecciones-2026/armando-benedetti-no-llegaria-campana-ivan-cepeda-detalles-ineditos-elecciones-2026-IC37352596</t>
+          <t>https://www.eluniversal.com.co/economica/2026/06/03/exportaciones-esta-es-la-aduana-lider-en-estas-operaciones-en-colombia/</t>
         </is>
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="2" t="inlineStr"/>
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 10:07 p. m.</t>
+        </is>
+      </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3805,22 +3717,26 @@
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D126" s="3" t="inlineStr">
         <is>
-          <t>“Pueden tener el apoyo de Petro, pero no pueden violar la ley”: alcalde Federico Gutiérrez sobre desmanes en la UdeA</t>
+          <t>Económica</t>
         </is>
       </c>
       <c r="E126" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/medellin/federico-gutierrez-rechaza-disturbios-en-la-universidad-de-antioquia-DE37337598</t>
+          <t>https://www.eluniversal.com.co/economica/</t>
         </is>
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="5" t="inlineStr"/>
+      <c r="A127" s="5" t="inlineStr">
+        <is>
+          <t>03/06/2026 09:57 p. m.</t>
+        </is>
+      </c>
       <c r="B127" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3828,22 +3744,26 @@
       </c>
       <c r="C127" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D127" s="6" t="inlineStr">
         <is>
-          <t>Creciente de quebrada en Andes obligó a evacuación preventiva del corregimiento Santa Inés</t>
+          <t>¡Aberrate! Alias ‘Curra’ habría realizado tocamiento a una menor de 14 años</t>
         </is>
       </c>
       <c r="E127" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/antioquia/emergencia-creciente-quebrada-corregimiento-santa-ines-andes-LD37348535</t>
+          <t>https://www.eluniversal.com.co/sucesos/2026/06/03/aberrate-alias-curra-habria-cometido-actos-a-una-menor-de-14-anos-en-cartagena/</t>
         </is>
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="2" t="inlineStr"/>
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 09:23 p. m.</t>
+        </is>
+      </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3851,22 +3771,26 @@
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D128" s="3" t="inlineStr">
         <is>
-          <t>Así estarían presionando las disidencias a comunidades de Nariño para votar por Cepeda</t>
+          <t>Sicarios irrumpieron en una calle de La Campiña y dejaron a un joven herido</t>
         </is>
       </c>
       <c r="E128" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/elecciones-2026/denuncian-presiones-grupos-armados-elecciones-por-ivan-cepeda-OG37314138</t>
+          <t>https://www.eluniversal.com.co/sucesos/2026/06/03/sicarios-irrumpieron-en-una-calle-de-la-campina-y-dejaron-a-un-joven-herido/</t>
         </is>
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="5" t="inlineStr"/>
+      <c r="A129" s="5" t="inlineStr">
+        <is>
+          <t>03/06/2026 09:00 p. m.</t>
+        </is>
+      </c>
       <c r="B129" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3874,22 +3798,26 @@
       </c>
       <c r="C129" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D129" s="6" t="inlineStr">
         <is>
-          <t>Colombia, entre los seis países con peor desempeño laboral de la Ocde</t>
+          <t>Claudia López ya tomó una decisión para la segunda vuelta: ¿De la Espriella o Cepeda?</t>
         </is>
       </c>
       <c r="E129" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/negocios/colombia-peor-desempeno-laboral-ocde-desempleo-IF37326097</t>
+          <t>https://www.eluniversal.com.co/politica/2026/06/03/claudia-lopez-ya-tomo-una-decision-para-la-segunda-vuelta-de-la-espriella-o-cepeda/</t>
         </is>
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="2" t="inlineStr"/>
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 09:00 p. m.</t>
+        </is>
+      </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3897,22 +3825,26 @@
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D130" s="3" t="inlineStr">
         <is>
-          <t>Quien fuera: Alcalde de Sincelejo pidió un mes de permiso para ir a ver el Mundial ¡y se lo dieron!</t>
+          <t>Política</t>
         </is>
       </c>
       <c r="E130" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/alcalde-sincelejo-permiso-mes-mundial-2026-CF37323724</t>
+          <t>https://www.eluniversal.com.co/politica/</t>
         </is>
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="5" t="inlineStr"/>
+      <c r="A131" s="5" t="inlineStr">
+        <is>
+          <t>03/06/2026 08:32 p. m.</t>
+        </is>
+      </c>
       <c r="B131" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3920,22 +3852,26 @@
       </c>
       <c r="C131" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D131" s="6" t="inlineStr">
         <is>
-          <t>Atención: Estación San Germán del Metro de la 80 será la primera subterránea del sistema y de Colombia</t>
+          <t>A ‘César’ y ‘Anuar’ los pillaron vendiendo droga: acumulan más de 20 anotaciones</t>
         </is>
       </c>
       <c r="E131" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/medellin/estacion-san-german-subterranea-metro-medellin-NG37314081</t>
+          <t>https://www.eluniversal.com.co/sucesos/2026/06/03/a-cesar-y-anuar-los-pillaron-vendiendo-droga-acumulan-mas-de-20-anotaciones/</t>
         </is>
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="2" t="inlineStr"/>
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 08:23 p. m.</t>
+        </is>
+      </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3943,22 +3879,26 @@
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D132" s="3" t="inlineStr">
         <is>
-          <t>Registraduría desmontó, uno por uno, los señalamientos de Petro de supuesto fraude electoral</t>
+          <t>Jerau se pone modo mundialista y le canta a la paz con sabor caribeño y africano</t>
         </is>
       </c>
       <c r="E132" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/elecciones-2026/gustavo-petro-resultados-elecciones-registraduria-desmiente-senalamientos-fraude-IP37297870</t>
+          <t>https://www.eluniversal.com.co/farandula/2026/06/03/jerau-se-pone-modo-mundialista-y-le-canta-a-la-paz-con-sabor-caribeno-y-africano/</t>
         </is>
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="5" t="inlineStr"/>
+      <c r="A133" s="5" t="inlineStr">
+        <is>
+          <t>03/06/2026 08:23 p. m.</t>
+        </is>
+      </c>
       <c r="B133" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3966,22 +3906,26 @@
       </c>
       <c r="C133" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D133" s="6" t="inlineStr">
         <is>
-          <t>Operativo destapa helicóptero con pasado oscuro y motor Rolls-Royce</t>
+          <t>Farándula</t>
         </is>
       </c>
       <c r="E133" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/ejercito-incauta-helicoptero-de-la-mafia-NG33717192</t>
+          <t>https://www.eluniversal.com.co/farandula/</t>
         </is>
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="2" t="inlineStr"/>
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 08:08 p. m.</t>
+        </is>
+      </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3989,22 +3933,26 @@
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D134" s="3" t="inlineStr">
         <is>
-          <t>Así se mueven los 5 clanes en la Costa que según De la Espriella hacen parte de una operación de compra de votos a favor de Cepeda</t>
+          <t>Temblor de magnitud 5.08 sacude a California</t>
         </is>
       </c>
       <c r="E134" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/de-la-espriella-estas-son-las-familias-denunciados-de-compra-de-votos-GC37352433</t>
+          <t>https://www.eluniversal.com.co/mundo/2026/06/03/temblor-de-magnitud-508-sacude-a-california/</t>
         </is>
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="5" t="inlineStr"/>
+      <c r="A135" s="5" t="inlineStr">
+        <is>
+          <t>03/06/2026 07:35 p. m.</t>
+        </is>
+      </c>
       <c r="B135" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4012,22 +3960,26 @@
       </c>
       <c r="C135" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D135" s="6" t="inlineStr">
         <is>
-          <t>Daniel Muñoz publicó emotivo video sobre su preparación para disputar su primer Mundial</t>
+          <t>MinTrabajo y Avianca impulsan empleos para personas con discapacidad</t>
         </is>
       </c>
       <c r="E135" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/mundial-2026/daniel-munoz-publico-video-con-su-preparacion-y-recuperacion-con-miras-al-mundial-de-norteamerica-CD37348820</t>
+          <t>https://www.eluniversal.com.co/colombia/2026/06/03/mintrabajo-y-avianca-impulsan-empleos-para-personas-con-discapacidad/</t>
         </is>
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="2" t="inlineStr"/>
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 06:52 p. m.</t>
+        </is>
+      </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4035,22 +3987,26 @@
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D136" s="3" t="inlineStr">
         <is>
-          <t>Corte tumbó estas dos reglas clave de la “Ley de Encuestas”: tienen que ver con los tiempos de publicación y microdatos</t>
+          <t>Mataron  a Deison Morales mientras compartía con su familia: había recibido amenazas</t>
         </is>
       </c>
       <c r="E136" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/corte-constitucional-tumba-dos-articulos-de-ley-de-encuestas-esto-se-sabe-KD37348354</t>
+          <t>https://www.eluniversal.com.co/sucesos/2026/06/03/acabaron-con-deison-morales-mientras-compartia-con-su-familia-habia-recibido-amenazas/</t>
         </is>
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="5" t="inlineStr"/>
+      <c r="A137" s="5" t="inlineStr">
+        <is>
+          <t>03/06/2026 06:02 p. m.</t>
+        </is>
+      </c>
       <c r="B137" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4058,22 +4014,26 @@
       </c>
       <c r="C137" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D137" s="6" t="inlineStr">
         <is>
-          <t>Así se jugará la primera fecha de la Liga BetPlay 2: la Dimayor oficializó el calendario del segundo semestre</t>
+          <t>A la cárcel dos hombres señalados de agredir a un niño de 3 años y a una mujer</t>
         </is>
       </c>
       <c r="E137" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/deportes/futbol/asi-se-jugara-la-primera-fecha-de-la-liga-betplay-2-LD37343448</t>
+          <t>https://www.eluniversal.com.co/sucesos/2026/06/03/a-la-carcel-dos-hombres-senalados-de-agredir-a-un-nino-de-3-anos-y-a-una-mujer/</t>
         </is>
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="2" t="inlineStr"/>
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 04:00 p. m.</t>
+        </is>
+      </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4081,17 +4041,17 @@
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D138" s="3" t="inlineStr">
         <is>
-          <t>“Todos tenemos que empujar a Nacional para la remontada”: Luis Fernando “Chonto” Herrera</t>
+          <t>Cartagena espera a J Balvin: crece la expectativa por sus invitados sorpresa</t>
         </is>
       </c>
       <c r="E138" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/multimedia/videos/todos-tenemos-que-empujar-a-nacional-para-la-remontada-luis-fernando-chonto-herrera-ND37344922</t>
+          <t>https://www.eluniversal.com.co/farandula/2026/06/03/cartagena-espera-a-j-balvin-crece-la-expectativa-por-sus-invitados-sorpresa/</t>
         </is>
       </c>
     </row>
@@ -4104,17 +4064,17 @@
       </c>
       <c r="C139" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D139" s="6" t="inlineStr">
         <is>
-          <t>Corrupción en Área Metropolitana: representante de firma investigada ofrece información sobre presunta red</t>
+          <t>Así puedes ganar entradas dobles para ver a J Balvin en Cartagena</t>
         </is>
       </c>
       <c r="E139" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/medellin/corrupcion-area-metropolitana-parque-de-las-aguas-medellin-DD37341525</t>
+          <t>https://www.eluniversal.com.co/cartagena/2026/06/02/asi-puedes-ganar-entradas-dobles-para-ver-a-jbalvin-en-cartagena/</t>
         </is>
       </c>
     </row>
@@ -4127,17 +4087,17 @@
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D140" s="3" t="inlineStr">
         <is>
-          <t>La Selección Colombia emprende el viaje para el Mundial este jueves: ¿a qué horas y cuál es su itinerario?</t>
+          <t>Cartagena</t>
         </is>
       </c>
       <c r="E140" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/mundial-2026/seleccion-colombia-viaje-mundial-itinerario-jueves-san-diego-amistoso-jordania-LD37343787</t>
+          <t>https://www.eluniversal.com.co/cartagena/</t>
         </is>
       </c>
     </row>
@@ -4150,17 +4110,17 @@
       </c>
       <c r="C141" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D141" s="6" t="inlineStr">
         <is>
-          <t>Mundial: Bayern Múnich y Manchester City son los equipos que más futbolistas tendrán en Norteamérica 2026</t>
+          <t>Dumek Turbay y Hamilton se reconcilian: “No quería estar lejos de su ciudad”</t>
         </is>
       </c>
       <c r="E141" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/deportes/futbol/mundial-2026-equipos-que-mas-jugadores-aportan-bayern-munich-manchester-city-2026-CE37333625</t>
+          <t>https://www.eluniversal.com.co/farandula/2026/06/02/dumek-turbay-y-hamilton-se-reconcilian-no-queria-estar-lejos-de-su-ciudad/</t>
         </is>
       </c>
     </row>
@@ -4173,17 +4133,17 @@
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D142" s="3" t="inlineStr">
         <is>
-          <t>Video | Pasajero intentó abrir una puerta y obligó a desviar el avión a Miami</t>
+          <t>Luister La Voz celebra a Cartagena: detalles del concierto de este 1 de junio</t>
         </is>
       </c>
       <c r="E142" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/internacional/pasajero-intenta-abrir-puerta-avion-desviar-avion-a-miami-AE37331427</t>
+          <t>https://www.eluniversal.com.co/farandula/2026/06/01/luister-la-voz-celebra-a-cartagena-detalles-del-concierto-de-este-1-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4196,22 +4156,26 @@
       </c>
       <c r="C143" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D143" s="6" t="inlineStr">
         <is>
-          <t>Este es el decálogo de Fajardo: no a la Constituyente, fin de “paz total” y ordenar la salud</t>
+          <t>Ser cartagenero lejos de Cartagena: ¿qué es lo que más extrañan quienes dejan la ciudad?</t>
         </is>
       </c>
       <c r="E143" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/politica/elecciones-2026-decalogo-sergio-fajardo-constituyente-paz-total-sistema-salud-DF37328092</t>
+          <t>https://www.eluniversal.com.co/cartagena/2026/06/01/ser-cartagenero-lejos-de-cartagena-que-es-lo-que-mas-extranan-quienes-dejan-la-ciudad/</t>
         </is>
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="2" t="inlineStr"/>
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>04/06/2026 12:06 a. m.</t>
+        </is>
+      </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4219,22 +4183,26 @@
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D144" s="3" t="inlineStr">
         <is>
-          <t>Seis universidades colombianas entran al ranking de las 2.000 mejores del mundo: la Nacional lidera el listado</t>
+          <t>La mejor campaña era hacer un buen gobierno</t>
         </is>
       </c>
       <c r="E144" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/educacion/mejores-universidades-colombia-ranking-cwur-NF37328630</t>
+          <t>https://www.elespectador.com/opinion/columnistas/blancainesduran/la-mejor-campana-era-hacer-un-buen-gobierno/</t>
         </is>
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="5" t="inlineStr"/>
+      <c r="A145" s="5" t="inlineStr">
+        <is>
+          <t>04/06/2026 12:05 a. m.</t>
+        </is>
+      </c>
       <c r="B145" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4242,22 +4210,26 @@
       </c>
       <c r="C145" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D145" s="6" t="inlineStr">
         <is>
-          <t>Pese a ataques violentos, Antioquia sigue bajando cifra de homicidios ¿Cuánto redujeron?</t>
+          <t>De Santa Marta a Tuvalu: cultivar la frágil esperanza</t>
         </is>
       </c>
       <c r="E145" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/antioquia/homicidios-antioquia-reduccion-2026-GE37333566</t>
+          <t>https://www.elespectador.com/opinion/columnistas/german-i-andrade-/de-santa-marta-a-tuvalu-cultivar-la-fragil-esperanza/</t>
         </is>
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="2" t="inlineStr"/>
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>04/06/2026 12:05 a. m.</t>
+        </is>
+      </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4265,22 +4237,26 @@
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D146" s="3" t="inlineStr">
         <is>
-          <t>Ponencia pide abrir investigación y llamar a indagatoria a Petro por financiación de campaña</t>
+          <t>¿Verde + rosa = blanco?</t>
         </is>
       </c>
       <c r="E146" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/petro-comision-de-acusacion-analizara-llamado-a-indagatoria-a-petro-LE37333549</t>
+          <t>https://www.elespectador.com/opinion/columnistas/brigitte-lg-baptiste/verde-rosa-blanco/</t>
         </is>
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="5" t="inlineStr"/>
+      <c r="A147" s="5" t="inlineStr">
+        <is>
+          <t>04/06/2026 12:05 a. m.</t>
+        </is>
+      </c>
       <c r="B147" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4288,22 +4264,26 @@
       </c>
       <c r="C147" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D147" s="6" t="inlineStr">
         <is>
-          <t>Prima de los hermanos Mucutuy murió en combates entre disidencias de las Farc en Guaviare</t>
+          <t>Sobre Mozart y la inteligencia artificial</t>
         </is>
       </c>
       <c r="E147" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/prima-hermanos-mucutuy-murio-combates-disidencias-farc-guaviare-MF37328501</t>
+          <t>https://www.elespectador.com/opinion/columnistas/manuel-drezner/sobre-mozart-y-la-inteligencia-artificial/</t>
         </is>
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="2" t="inlineStr"/>
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>04/06/2026 12:05 a. m.</t>
+        </is>
+      </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4311,22 +4291,26 @@
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D148" s="3" t="inlineStr">
         <is>
-          <t>Nacional no baja los brazos: estas son las remontadas que alimentan la esperanza verde ante Junior</t>
+          <t>Más allá del voto en blanco</t>
         </is>
       </c>
       <c r="E148" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/deportes/futbol/atletico-nacional-remontadas-historicas-final-junior-vuelta-liga-betplay-atanasio-girardot-OE37331870</t>
+          <t>https://www.elespectador.com/opinion/columnistas/cristinacarrizosa/mas-alla-del-voto-en-blanco/</t>
         </is>
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="5" t="inlineStr"/>
+      <c r="A149" s="5" t="inlineStr">
+        <is>
+          <t>04/06/2026 12:05 a. m.</t>
+        </is>
+      </c>
       <c r="B149" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4334,22 +4318,26 @@
       </c>
       <c r="C149" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D149" s="6" t="inlineStr">
         <is>
-          <t>Medellín explica las inversiones por casi $3 billones para tener un aire más limpio</t>
+          <t>Los votos están ahí</t>
         </is>
       </c>
       <c r="E149" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/medellin/medellin-inversion-reducir-contaminacion-calidad-aire-GF37329593</t>
+          <t>https://www.elespectador.com/opinion/columnistas/javier-ortiz/los-votos-estan-ahi/</t>
         </is>
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="2" t="inlineStr"/>
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>04/06/2026 12:05 a. m.</t>
+        </is>
+      </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4357,22 +4345,26 @@
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D150" s="3" t="inlineStr">
         <is>
-          <t>Parrandas de Jhon Jáder Durán tienen desesperados a sus vecinos en Llanogrande: “No nos dejan dormir”</t>
+          <t>Líder del equipo digital de De la Espriella denunciado por violencia sexual</t>
         </is>
       </c>
       <c r="E150" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/antioquia/quejas-fiestas-jhon-jader-duran-finca-rionegro-antioquia-FG37316715</t>
+          <t>https://www.elespectador.com/opinion/columnistas/catalina-ruiz-navarro/lider-del-equipo-digital-de-de-la-espriella-denunciado-por-violencia-sexual/</t>
         </is>
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="5" t="inlineStr"/>
+      <c r="A151" s="5" t="inlineStr">
+        <is>
+          <t>04/06/2026 12:04 a. m.</t>
+        </is>
+      </c>
       <c r="B151" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4380,22 +4372,26 @@
       </c>
       <c r="C151" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D151" s="6" t="inlineStr">
         <is>
-          <t>¿Clint Eastwood se retira a los 96 años? Lo que se sabe de las declaraciones de su hijo</t>
+          <t>Gurropín, corrupto dictador venerado por la izquierda populista</t>
         </is>
       </c>
       <c r="E151" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/cultura/cine/clint-eastwood-retiro-jubilacion-hijos-verdad-mentira-96-OF37325029</t>
+          <t>https://www.elespectador.com/opinion/columnistas/mauricio-rubio/gurropin-corrupto-dictador-venerado-por-la-izquierda-populista/</t>
         </is>
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="2" t="inlineStr"/>
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>04/06/2026 12:04 a. m.</t>
+        </is>
+      </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4403,22 +4399,26 @@
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D152" s="3" t="inlineStr">
         <is>
-          <t>Aída Quilcué aceptó la invitación de Westcol para un streaming</t>
+          <t>Quiero hablar con las flores</t>
         </is>
       </c>
       <c r="E152" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/aida-quilcue-acepta-hacer-streaming-con-westcol-ND37348371</t>
+          <t>https://www.elespectador.com/opinion/columnistas/juan-david-zuloaga-d-/quiero-hablar-con-las-flores/</t>
         </is>
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="5" t="inlineStr"/>
+      <c r="A153" s="5" t="inlineStr">
+        <is>
+          <t>04/06/2026 12:00 a. m.</t>
+        </is>
+      </c>
       <c r="B153" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4426,17 +4426,17 @@
       </c>
       <c r="C153" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D153" s="6" t="inlineStr">
         <is>
-          <t>Denuncian a Gustavo Petro ante la MOE por hacer “intervención política” y poner en riesgo la contienda electoral</t>
+          <t>Atrapados entre la espada, la pared y la improvisación</t>
         </is>
       </c>
       <c r="E153" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/denuncian-petro-moe-declaraciones-elecciones-uso-recursos-campana-MG37315339</t>
+          <t>https://www.elespectador.com/opinion/lectores/cartas/atrapados-entre-la-espada-la-pared-y-la-improvisacion/</t>
         </is>
       </c>
     </row>
@@ -4458,12 +4458,12 @@
       </c>
       <c r="D154" s="3" t="inlineStr">
         <is>
-          <t>Nequi suspenderá temporalmente los pagos por PSE durante una jornada de mantenimiento: conozca cuándo será la interrupción</t>
+          <t>¿Cómo estará el clima en Medellín?</t>
         </is>
       </c>
       <c r="E154" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/nequi-suspendera-temporalmente-los-pagos-por-pse-durante-una-jornada-de-mantenimiento-conozca-cuando-sera-la-interrupcion/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/como-estara-el-clima-en-medellin/</t>
         </is>
       </c>
     </row>
@@ -4485,12 +4485,12 @@
       </c>
       <c r="D155" s="6" t="inlineStr">
         <is>
-          <t>Avenida torrencial en Andes arrasó puentes y obligó a evacuar al menos a 150 personas en Santa Inés, Antioquia</t>
+          <t>Las últimas previsiones para Bogotá: temperatura, lluvias y viento</t>
         </is>
       </c>
       <c r="E155" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/avenida-torrencial-en-andes-arraso-puentes-y-obligo-a-evacuar-al-menos-a-150-personas-en-santa-ines-antioquia/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/las-ultimas-previsiones-para-bogota-temperatura-lluvias-y-viento/</t>
         </is>
       </c>
     </row>
@@ -4512,12 +4512,12 @@
       </c>
       <c r="D156" s="3" t="inlineStr">
         <is>
-          <t>Pico y Placa Bogotá: evita multas este jueves 4 de junio</t>
+          <t>Clima en Cartagena de Indias: la predicción para este 4 de junio</t>
         </is>
       </c>
       <c r="E156" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/pico-y-placa-bogota-evita-multas-este-jueves-4-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/clima-en-cartagena-de-indias-la-prediccion-para-este-4-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4539,12 +4539,12 @@
       </c>
       <c r="D157" s="6" t="inlineStr">
         <is>
-          <t>Denuncian que lanzaron objetos desde un edificio contra manifestantes de Iván Cepeda en Medellín: un niño resultó herido</t>
+          <t>Pronóstico del clima en Cali este 4 de junio: temperatura, lluvias y viento</t>
         </is>
       </c>
       <c r="E157" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/denuncian-que-lanzaron-objetos-desde-un-edificio-contra-manifestantes-de-ivan-cepeda-en-medellin-un-nino-resulto-herido/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/pronostico-del-clima-en-cali-este-4-de-junio-temperatura-lluvias-y-viento/</t>
         </is>
       </c>
     </row>
@@ -4566,12 +4566,12 @@
       </c>
       <c r="D158" s="3" t="inlineStr">
         <is>
-          <t>Resultados Baloto y Revancha, último sorteo del miércoles 3 de junio</t>
+          <t>Las últimas previsiones para Barranquilla: temperatura, lluvias y viento</t>
         </is>
       </c>
       <c r="E158" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/resultados-baloto-y-revancha-ultimo-sorteo-del-miercoles-3-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/las-ultimas-previsiones-para-barranquilla-temperatura-lluvias-y-viento/</t>
         </is>
       </c>
     </row>
@@ -4593,12 +4593,12 @@
       </c>
       <c r="D159" s="6" t="inlineStr">
         <is>
-          <t>Resultado Baloto y Revancha hoy 3 de junio</t>
+          <t>“Haber traído a Álvaro Uribe Vélez como ministro de Defensa espantó al centro”: Juan Daniel Oviedo analiza caída de Paloma Valencia</t>
         </is>
       </c>
       <c r="E159" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/resultado-baloto-y-revancha-hoy-3-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/haber-traido-a-alvaro-uribe-velez-como-ministro-de-defensa-espanto-al-centro-juan-daniel-oviedo-analiza-caida-de-paloma-valencia/</t>
         </is>
       </c>
     </row>
@@ -4620,12 +4620,12 @@
       </c>
       <c r="D160" s="3" t="inlineStr">
         <is>
-          <t>MOE responde a denuncias de fraude: explica las 885.000 cédulas, las mesas adicionales y los puestos de votación en la primera vuelta</t>
+          <t>Felipe Harman dejaría la ANT para unirse a la campaña de Iván Cepeda y coordinar la recta final electoral</t>
         </is>
       </c>
       <c r="E160" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/moe-responde-a-denuncias-de-fraude-explica-las-885000-cedulas-las-mesas-adicionales-y-los-puestos-de-votacion-en-la-primera-vuelta/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/felipe-harman-dejaria-la-ant-para-unirse-a-la-campana-de-ivan-cepeda-y-coordinar-la-recta-final-electoral/</t>
         </is>
       </c>
     </row>
@@ -4647,12 +4647,12 @@
       </c>
       <c r="D161" s="6" t="inlineStr">
         <is>
-          <t>Lotería de Manizales resultados miércoles 3 de junio: quién ganó el premio mayor de $2.600 millones</t>
+          <t>Nequi suspenderá temporalmente los pagos por PSE durante una jornada de mantenimiento: conozca cuándo será la interrupción</t>
         </is>
       </c>
       <c r="E161" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/loteria-de-manizales-resultados-miercoles-3-de-junio-quien-gano-el-premio-mayor-de-2600-millones/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/nequi-suspendera-temporalmente-los-pagos-por-pse-durante-una-jornada-de-mantenimiento-conozca-cuando-sera-la-interrupcion/</t>
         </is>
       </c>
     </row>
@@ -4674,12 +4674,12 @@
       </c>
       <c r="D162" s="3" t="inlineStr">
         <is>
-          <t>Resultados de la Lotería del Valle miércoles 3 de junio de 2026: todos los secos millonarios</t>
+          <t>Avenida torrencial en Andes arrasó puentes y obligó a evacuar al menos a 150 personas en Santa Inés, Antioquia</t>
         </is>
       </c>
       <c r="E162" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/resultados-de-la-loteria-del-valle-miercoles-3-de-junio-de-2026-todos-los-secos-millonarios/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/avenida-torrencial-en-andes-arraso-puentes-y-obligo-a-evacuar-al-menos-a-150-personas-en-santa-ines-antioquia/</t>
         </is>
       </c>
     </row>
@@ -4701,12 +4701,12 @@
       </c>
       <c r="D163" s="6" t="inlineStr">
         <is>
-          <t>Resultados Lotería del Valle miércoles 3 de junio de 2026: quién ganó el premio mayor de $9.000 millones</t>
+          <t>Pico y Placa Bogotá: evita multas este jueves 4 de junio</t>
         </is>
       </c>
       <c r="E163" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/resultados-loteria-del-valle-miercoles-3-de-junio-de-2026-quien-gano-el-premio-mayor-de-9000-millones/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/pico-y-placa-bogota-evita-multas-este-jueves-4-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4728,12 +4728,12 @@
       </c>
       <c r="D164" s="3" t="inlineStr">
         <is>
-          <t>“No son estudiantes, son terroristas”: Federico Gutiérrez se pronuncia tras disturbios de encapuchados en la Universidad de Antioquia</t>
+          <t>Denuncian que lanzaron objetos desde un edificio contra manifestantes de Iván Cepeda en Medellín: un niño resultó herido</t>
         </is>
       </c>
       <c r="E164" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/no-son-estudiantes-son-terroristas-federico-gutierrez-se-pronuncia-tras-disturbios-de-encapuchados-en-la-universidad-de-antioquia/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/denuncian-que-lanzaron-objetos-desde-un-edificio-contra-manifestantes-de-ivan-cepeda-en-medellin-un-nino-resulto-herido/</t>
         </is>
       </c>
     </row>
@@ -4755,12 +4755,12 @@
       </c>
       <c r="D165" s="6" t="inlineStr">
         <is>
-          <t>“Jamás debieron vincular a su guerra”: ICBF condena la muerte de 11 menores en combates entre disidencias en Guaviare</t>
+          <t>Resultados Baloto y Revancha, último sorteo del miércoles 3 de junio</t>
         </is>
       </c>
       <c r="E165" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/jamas-debieron-vincular-a-su-guerra-icbf-condena-la-muerte-de-11-menores-en-combates-entre-disidencias-en-guaviare/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/resultados-baloto-y-revancha-ultimo-sorteo-del-miercoles-3-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4782,12 +4782,12 @@
       </c>
       <c r="D166" s="3" t="inlineStr">
         <is>
-          <t>Baloto y Revancha: números ganadores del lunes 1 de junio</t>
+          <t>Resultado Baloto y Revancha hoy 3 de junio</t>
         </is>
       </c>
       <c r="E166" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/baloto-y-revancha-numeros-ganadores-del-lunes-1-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/resultado-baloto-y-revancha-hoy-3-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4809,12 +4809,12 @@
       </c>
       <c r="D167" s="6" t="inlineStr">
         <is>
-          <t>Resultado Super Astro Luna HOY: número ganador del miércoles 3 de junio</t>
+          <t>MOE responde a denuncias de fraude: explica las 885.000 cédulas, las mesas adicionales y los puestos de votación en la primera vuelta</t>
         </is>
       </c>
       <c r="E167" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/resultado-super-astro-luna-hoy-numero-ganador-del-miercoles-3-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/moe-responde-a-denuncias-de-fraude-explica-las-885000-cedulas-las-mesas-adicionales-y-los-puestos-de-votacion-en-la-primera-vuelta/</t>
         </is>
       </c>
     </row>
@@ -4836,12 +4836,12 @@
       </c>
       <c r="D168" s="3" t="inlineStr">
         <is>
-          <t>Lotería del Meta resultados 3 de junio: números ganadores del premio mayor de $1.800 millones</t>
+          <t>Lotería de Manizales resultados miércoles 3 de junio: quién ganó el premio mayor de $2.600 millones</t>
         </is>
       </c>
       <c r="E168" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/loteria-de-meta-resultados-3-de-junio-numeros-ganadores-del-premio-mayor-de-1800-millones/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/loteria-de-manizales-resultados-miercoles-3-de-junio-quien-gano-el-premio-mayor-de-2600-millones/</t>
         </is>
       </c>
     </row>
@@ -4863,12 +4863,12 @@
       </c>
       <c r="D169" s="6" t="inlineStr">
         <is>
-          <t>Procuraduría inhabilita por cinco años a cónsul honorario de Colombia en Italia por cobro indebido a una ciudadana</t>
+          <t>Resultados de la Lotería del Valle miércoles 3 de junio de 2026: todos los secos millonarios</t>
         </is>
       </c>
       <c r="E169" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/procuraduria-inhabilita-por-cinco-anos-a-consul-honorario-de-colombia-en-italia-por-cobro-indebido-a-una-ciudadana/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/resultados-de-la-loteria-del-valle-miercoles-3-de-junio-de-2026-todos-los-secos-millonarios/</t>
         </is>
       </c>
     </row>
@@ -4890,12 +4890,12 @@
       </c>
       <c r="D170" s="3" t="inlineStr">
         <is>
-          <t>Pilas: Así rotará el Pico y Placa en Cali este jueves 4 de junio</t>
+          <t>Resultados Lotería del Valle miércoles 3 de junio de 2026: quién ganó el premio mayor de $9.000 millones</t>
         </is>
       </c>
       <c r="E170" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/pilas-asi-rotara-el-pico-y-placa-en-cali-este-jueves-4-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/resultados-loteria-del-valle-miercoles-3-de-junio-de-2026-quien-gano-el-premio-mayor-de-9000-millones/</t>
         </is>
       </c>
     </row>
@@ -4917,12 +4917,12 @@
       </c>
       <c r="D171" s="6" t="inlineStr">
         <is>
-          <t>Pico y Placa: qué vehículos no circulan en Villavicencio este jueves 4 de junio</t>
+          <t>“No son estudiantes, son terroristas”: Federico Gutiérrez se pronuncia tras disturbios de encapuchados en la Universidad de Antioquia</t>
         </is>
       </c>
       <c r="E171" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/pico-y-placa-que-vehiculos-no-circulan-en-villavicencio-este-jueves-4-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/no-son-estudiantes-son-terroristas-federico-gutierrez-se-pronuncia-tras-disturbios-de-encapuchados-en-la-universidad-de-antioquia/</t>
         </is>
       </c>
     </row>
@@ -4944,12 +4944,12 @@
       </c>
       <c r="D172" s="3" t="inlineStr">
         <is>
-          <t>Pico y Placa: qué autos descansan en Cartagena este jueves 4 de junio</t>
+          <t>“Jamás debieron vincular a su guerra”: ICBF condena la muerte de 11 menores en combates entre disidencias en Guaviare</t>
         </is>
       </c>
       <c r="E172" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/pico-y-placa-que-autos-descansan-en-cartagena-este-jueves-4-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/jamas-debieron-vincular-a-su-guerra-icbf-condena-la-muerte-de-11-menores-en-combates-entre-disidencias-en-guaviare/</t>
         </is>
       </c>
     </row>
@@ -4971,12 +4971,12 @@
       </c>
       <c r="D173" s="6" t="inlineStr">
         <is>
-          <t>Peajes de Autopistas del Café bajarán a $700 para vehículos beneficiarios tras anuncio de Gustavo Petro</t>
+          <t>Baloto y Revancha: números ganadores del lunes 1 de junio</t>
         </is>
       </c>
       <c r="E173" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/peajes-de-autopistas-del-cafe-bajaran-a-700-para-vehiculos-beneficiarios-tras-anuncio-de-gustavo-petro/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/baloto-y-revancha-numeros-ganadores-del-lunes-1-de-junio/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 Noticias actualizadas 04/06/2026 10:22
</commit_message>
<xml_diff>
--- a/docs/ultimahora.xlsx
+++ b/docs/ultimahora.xlsx
@@ -515,7 +515,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 03:04 a. m.</t>
+          <t>04/06/2026 05:15 a. m.</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -530,19 +530,19 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Expolicía ecuatoriano aseguró que agentes y altos mandos sabían del atentado contra el candidato Fernando Villavicencio antes de ser asesinado en 2023</t>
+          <t>Ranking: Estas son las empresas con más cortes de energía eléctrica y que dejan más horas sin luz a los colombianos</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/latinoamerica/expolicia-ecuatoriano-aseguro-que-agentes-y-altos-mandos-sabian-del-atentado-contra-el-candidato-fernando-villavicencio-antes-de-ser-asesinado-en-3561991</t>
+          <t>https://www.eltiempo.com/economia/sectores/ranking-estas-son-las-empresas-con-mas-cortes-de-energia-electrica-y-que-dejan-mas-horas-sin-luz-a-los-colombianos-3561936</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 02:30 a. m.</t>
+          <t>04/06/2026 04:43 a. m.</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -557,19 +557,19 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>¡Ojo con las restricciones! Pico y placa en Pereira para el jueves 4 de junio de 2026</t>
+          <t>Murió Marjane Satrapi, autora de 'Persepolis', a los 56 años: había enviudado un año antes</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/otras-ciudades/ojo-con-las-restricciones-pico-y-placa-en-pereira-para-el-jueves-4-de-junio-de-3561984</t>
+          <t>https://www.eltiempo.com/cultura/entretenimiento/murio-marjane-satrapi-autora-de-persepolis-a-los-56-anos-habia-enviudado-un-ano-antes-3561994</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 02:30 a. m.</t>
+          <t>04/06/2026 04:31 a. m.</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -584,19 +584,19 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>¡Ojo, conductor! Pico y placa en Medellín para el jueves 4 de junio de 2026: consulte las restricciones</t>
+          <t>Tuits y participación en política: la red social como plataforma y también como trampa</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/medellin/ojo-conductor-pico-y-placa-en-medellin-para-el-jueves-4-de-junio-de-2026-consulte-las-restricciones-3561983</t>
+          <t>https://www.eltiempo.com/podcast/el-cafe-de-hoy/tuits-y-participacion-en-politica-la-red-social-como-plataforma-y-tambien-como-trampa-3561993</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 02:30 a. m.</t>
+          <t>04/06/2026 04:30 a. m.</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -611,19 +611,19 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Así opera el pico y placa en Bucaramanga para el jueves 4 de junio de 2026</t>
+          <t>Movilidad en Bogotá jueves 04 de junio: conozca acá el pico y placa en la ciudad</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/santander/asi-opera-el-pico-y-placa-en-bucaramanga-para-el-jueves-4-de-junio-de-3561982</t>
+          <t>https://www.eltiempo.com/bogota/movilidad-en-bogota-jueves-04-de-junio-conozca-aca-el-pico-y-placa-en-la-ciudad-3561992</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 02:30 a. m.</t>
+          <t>04/06/2026 03:04 a. m.</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -638,12 +638,12 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>¡Evite multas! Pico y placa en Cali para el jueves 4 de junio de 2026: así opera la medida</t>
+          <t>Expolicía ecuatoriano aseguró que agentes y altos mandos sabían del atentado contra el candidato Fernando Villavicencio antes de ser asesinado en 2023</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/cali/evite-multas-pico-y-placa-en-cali-para-el-jueves-4-de-junio-de-2026-asi-opera-la-medida-3561981</t>
+          <t>https://www.eltiempo.com/mundo/latinoamerica/expolicia-ecuatoriano-aseguro-que-agentes-y-altos-mandos-sabian-del-atentado-contra-el-candidato-fernando-villavicencio-antes-de-ser-asesinado-en-3561991</t>
         </is>
       </c>
     </row>
@@ -665,19 +665,19 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>¡Pilas en las vías! Pico y placa en Bogotá para el jueves 4 de junio de 2026</t>
+          <t>¡Ojo con las restricciones! Pico y placa en Pereira para el jueves 4 de junio de 2026</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/bogota/pilas-en-las-vias-pico-y-placa-en-bogota-para-el-jueves-4-de-junio-de-3561858</t>
+          <t>https://www.eltiempo.com/colombia/otras-ciudades/ojo-con-las-restricciones-pico-y-placa-en-pereira-para-el-jueves-4-de-junio-de-3561984</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 01:29 a. m.</t>
+          <t>04/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -692,19 +692,19 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Senadora Andrea Padilla anunció que la Fiscalía y Procuraduría abrieron investigación por crisis de 317 caimanes sin comida: 'Ya fueron alimentados'</t>
+          <t>¡Ojo, conductor! Pico y placa en Medellín para el jueves 4 de junio de 2026: consulte las restricciones</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/vida/medio-ambiente/senadora-andrea-padilla-anuncio-que-fiscalia-y-procuraduria-abrieron-investigacion-por-crisis-de-317-caimanes-sin-comida-ya-fueron-alimentados-3561989</t>
+          <t>https://www.eltiempo.com/colombia/medellin/ojo-conductor-pico-y-placa-en-medellin-para-el-jueves-4-de-junio-de-2026-consulte-las-restricciones-3561983</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 12:37 a. m.</t>
+          <t>04/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -719,19 +719,19 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Estas son las nuevas preguntas que podrían hacerle en su proceso de green card en Estados Unidos: miles colombianos se verían afectados</t>
+          <t>Así opera el pico y placa en Bucaramanga para el jueves 4 de junio de 2026</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/estas-son-las-nuevas-preguntas-que-podrian-hacerle-en-su-proceso-de-green-card-en-estados-unidos-miles-colombianos-se-verian-afectados-3561940</t>
+          <t>https://www.eltiempo.com/colombia/santander/asi-opera-el-pico-y-placa-en-bucaramanga-para-el-jueves-4-de-junio-de-3561982</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 12:10 a. m.</t>
+          <t>04/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -746,19 +746,19 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Nueva ofensiva arancelaria de Trump podría golpear a Colombia: propuesta de EE. UU. elevaría al 12,5 % la tarifa sobre exportaciones nacionales</t>
+          <t>¡Evite multas! Pico y placa en Cali para el jueves 4 de junio de 2026: así opera la medida</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/nueva-ofensiva-arancelaria-de-trump-podria-golpear-a-colombia-propuesta-de-ee-uu-elevaria-al-12-5-la-tarifa-sobre-exportaciones-nacionales-3561904</t>
+          <t>https://www.eltiempo.com/colombia/cali/evite-multas-pico-y-placa-en-cali-para-el-jueves-4-de-junio-de-2026-asi-opera-la-medida-3561981</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 11:24 p. m.</t>
+          <t>04/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -773,19 +773,19 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Presidente Gustavo Petro ordenó bombardeo en Guaviare tras captura de alias Mona, presunta cabecilla de las disidencias de 'Iván Mordisco'</t>
+          <t>¡Pilas en las vías! Pico y placa en Bogotá para el jueves 4 de junio de 2026</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/politica/gobierno/presidente-gustavo-petro-ordeno-bombardeo-en-guaviare-tras-captura-de-alias-mona-presunta-cabecilla-de-las-disidencias-de-ivan-mordisco-3561988</t>
+          <t>https://www.eltiempo.com/bogota/pilas-en-las-vias-pico-y-placa-en-bogota-para-el-jueves-4-de-junio-de-3561858</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 11:17 p. m.</t>
+          <t>04/06/2026 01:29 a. m.</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -800,19 +800,19 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Identificaron a familiar de los hermanos Mucutuy entre los 11 menores fallecidos por combates de las disidencias en Guaviare: era prima de los niños</t>
+          <t>Senadora Andrea Padilla anunció que la Fiscalía y Procuraduría abrieron investigación por crisis de 317 caimanes sin comida: 'Ya fueron alimentados'</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/justicia/conflicto-y-narcotrafico/identificaron-a-familiar-de-los-hermanos-mucutuy-entre-los-11-menores-fallecidos-por-combates-entre-disidencias-en-guaviare-era-prima-de-los-ninos-3561987</t>
+          <t>https://www.eltiempo.com/vida/medio-ambiente/senadora-andrea-padilla-anuncio-que-fiscalia-y-procuraduria-abrieron-investigacion-por-crisis-de-317-caimanes-sin-comida-ya-fueron-alimentados-3561989</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 11:08 p. m.</t>
+          <t>04/06/2026 12:37 a. m.</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -827,19 +827,19 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Senadora María Elvira Salazar pidió sanciones para quien realice fraude en segunda vuelta presidencial de Colombia: lista OFAC y cancelación de visas</t>
+          <t>Estas son las nuevas preguntas que podrían hacerle en su proceso de green card en Estados Unidos: miles colombianos se verían afectados</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/senadora-maria-elvira-salazar-pidio-incluir-en-la-lista-ofac-a-quien-realice-fraude-electoral-en-la-segunda-vuelta-presidencial-de-colombia-3561985</t>
+          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/estas-son-las-nuevas-preguntas-que-podrian-hacerle-en-su-proceso-de-green-card-en-estados-unidos-miles-colombianos-se-verian-afectados-3561940</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 11:05 p. m.</t>
+          <t>04/06/2026 12:10 a. m.</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -854,19 +854,19 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Revelan las supuestas amenazas del anestesiólogo 'Leo' cuando Yulixa Toloza todavía tenía signos vitales tras procedimiento estético: 'Sacó un arma'</t>
+          <t>Nueva ofensiva arancelaria de Trump podría golpear a Colombia: propuesta de EE. UU. elevaría al 12,5 % la tarifa sobre exportaciones nacionales</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/bogota/revelan-las-supuestas-amenazas-de-anestesiologo-leo-cuando-yulixa-toloza-todavia-tenia-signos-vitales-tras-procedimiento-estetico-saco-un-arma-3561986</t>
+          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/nueva-ofensiva-arancelaria-de-trump-podria-golpear-a-colombia-propuesta-de-ee-uu-elevaria-al-12-5-la-tarifa-sobre-exportaciones-nacionales-3561904</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 11:03 p. m.</t>
+          <t>03/06/2026 11:24 p. m.</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -881,19 +881,19 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Alertan por estafas migratorias en Estados Unidos: usan inteligencia artificial para suplantar abogados y ofrecer trámites falsos</t>
+          <t>Presidente Gustavo Petro ordenó bombardeo en Guaviare tras captura de alias Mona, presunta cabecilla de las disidencias de 'Iván Mordisco'</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/alertan-por-estafas-migratorias-en-estados-unidos-usan-inteligencia-artificial-para-suplantar-abogados-y-ofrecer-tramites-migratorios-falsos-3561967</t>
+          <t>https://www.eltiempo.com/politica/gobierno/presidente-gustavo-petro-ordeno-bombardeo-en-guaviare-tras-captura-de-alias-mona-presunta-cabecilla-de-las-disidencias-de-ivan-mordisco-3561988</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 10:47 p. m.</t>
+          <t>03/06/2026 11:17 p. m.</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -908,19 +908,19 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Junior vs. Nacional: Alfredo Arias y sus tres lecciones a Diego Arias en final de ida de la Liga BetPlay</t>
+          <t>Identificaron a familiar de los hermanos Mucutuy entre los 11 menores fallecidos por combates de las disidencias en Guaviare: era prima de los niños</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-colombiano/junior-vs-nacional-alfredo-arias-y-sus-tres-lecciones-a-diego-arias-en-final-de-ida-de-la-liga-betplay-3561972</t>
+          <t>https://www.eltiempo.com/justicia/conflicto-y-narcotrafico/identificaron-a-familiar-de-los-hermanos-mucutuy-entre-los-11-menores-fallecidos-por-combates-entre-disidencias-en-guaviare-era-prima-de-los-ninos-3561987</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 10:28 p. m.</t>
+          <t>03/06/2026 11:08 p. m.</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -935,19 +935,19 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>'Es hora de que el Gobierno Nacional fije sus ojos en la región': esto es lo que el sector productivo del Valle del Cauca le pide al nuevo presidente</t>
+          <t>Senadora María Elvira Salazar pidió sanciones para quien realice fraude en segunda vuelta presidencial de Colombia: lista OFAC y cancelación de visas</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/cali/es-hora-de-que-el-gobierno-nacional-fije-sus-ojos-en-la-region-esto-es-lo-que-el-sector-productivo-del-valle-del-cauca-le-pide-al-nuevo-presidente-3561979</t>
+          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/senadora-maria-elvira-salazar-pidio-incluir-en-la-lista-ofac-a-quien-realice-fraude-electoral-en-la-segunda-vuelta-presidencial-de-colombia-3561985</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 10:09 p. m.</t>
+          <t>03/06/2026 11:05 p. m.</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -962,19 +962,19 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>El actor estadounidense Tyler Hoechlin será uno de los invitados centrales de la Comic Con Bogotá</t>
+          <t>Revelan las supuestas amenazas del anestesiólogo 'Leo' cuando Yulixa Toloza todavía tenía signos vitales tras procedimiento estético: 'Sacó un arma'</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/cultura/cine-y-tv/el-actor-estadounidense-tyler-hoechlin-sera-uno-de-los-invitados-centrales-de-la-comic-con-bogota-3561980</t>
+          <t>https://www.eltiempo.com/bogota/revelan-las-supuestas-amenazas-de-anestesiologo-leo-cuando-yulixa-toloza-todavia-tenia-signos-vitales-tras-procedimiento-estetico-saco-un-arma-3561986</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 10:01 p. m.</t>
+          <t>03/06/2026 11:03 p. m.</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -989,19 +989,19 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>'Enemigo público': alcalde de Soacha hace denuncia por video que revelaría a empleados de la empresa de aseo Urbaser arrojando basura en las calles</t>
+          <t>Alertan por estafas migratorias en Estados Unidos: usan inteligencia artificial para suplantar abogados y ofrecer trámites falsos</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/bogota/enemigo-publico-alcalde-de-soacha-hace-denuncia-por-video-que-revelaria-a-empleados-de-la-empresa-de-aseo-urbaser-arrojando-basura-en-las-calles-3561975</t>
+          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/alertan-por-estafas-migratorias-en-estados-unidos-usan-inteligencia-artificial-para-suplantar-abogados-y-ofrecer-tramites-migratorios-falsos-3561967</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 10:01 p. m.</t>
+          <t>03/06/2026 10:47 p. m.</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1016,19 +1016,19 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Tristeza total</t>
+          <t>Junior vs. Nacional: Alfredo Arias y sus tres lecciones a Diego Arias en final de ida de la Liga BetPlay</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/caricaturas/tristeza-total-3561947</t>
+          <t>https://www.eltiempo.com/deportes/futbol-colombiano/junior-vs-nacional-alfredo-arias-y-sus-tres-lecciones-a-diego-arias-en-final-de-ida-de-la-liga-betplay-3561972</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 10:01 p. m.</t>
+          <t>03/06/2026 10:28 p. m.</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
@@ -1043,19 +1043,19 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Trump saludó</t>
+          <t>'Es hora de que el Gobierno Nacional fije sus ojos en la región': esto es lo que el sector productivo del Valle del Cauca le pide al nuevo presidente</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/caricaturas/trump-saludo-3561946</t>
+          <t>https://www.eltiempo.com/colombia/cali/es-hora-de-que-el-gobierno-nacional-fije-sus-ojos-en-la-region-esto-es-lo-que-el-sector-productivo-del-valle-del-cauca-le-pide-al-nuevo-presidente-3561979</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 07:05 a. m.</t>
+          <t>04/06/2026 10:13 a. m.</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1065,24 +1065,24 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Petro califica de intervencionista el respaldo de Trump a de La Espriella</t>
+          <t>Jóvenes respaldan a Iván Cepeda en movilización por la vida y la educación en Bogotá</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/03/petro-califica-de-intervencionista-el-respaldo-de-trump-a-de-la-espriella/</t>
+          <t>https://www.lafm.com.co/actualidad/jovenes-respaldan-a-ivan-cepeda-en-movilizacion-por-la-vida-y-la-educacion-en-bogota-401337</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 06:22 a. m.</t>
+          <t>04/06/2026 02:23 a. m.</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -1092,24 +1092,24 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Fiscalía imputará cargos a ocho implicados en red de contrabando ligada a Lili Pink</t>
+          <t>“Petro está reconociendo que su candidato no funcionó”; cuestionan protagonismo del presidente en la campaña de Cepeda</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/03/fiscalia-imputara-cargos-a-ocho-implicados-en-red-de-contrabando-ligada-a-lili-pink/</t>
+          <t>https://www.lafm.com.co/politica/gustavo-petro-ivan-cepeda-campana-pacto-historico-elecciones-presidenciales-2026-401330</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 01:00 a. m.</t>
+          <t>04/06/2026 02:14 a. m.</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1119,24 +1119,24 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>José Francisco Socarrás Colina</t>
+          <t>Un telescopio a 1,5 millones de kilómetros de la Tierra reveló algo que llevaba décadas oculto</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/04/jose-francisco-socarras-colina/</t>
+          <t>https://www.lafm.com.co/sociedad/telescopio-revela-misterio-universo-oculto-decadas-cientificos-nasa-401328</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 01:00 a. m.</t>
+          <t>04/06/2026 01:42 a. m.</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
@@ -1146,24 +1146,24 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Columnistas</t>
+          <t>Claudia López se aleja de De la Espriella, reconoce la decencia de Cepeda y rechaza endosar sus votos</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/</t>
+          <t>https://www.lafm.com.co/politica/claudia-lopez-desconfianza-abelardo-de-la-espriella-respaldo-cepeda-401327</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 01:00 a. m.</t>
+          <t>04/06/2026 12:51 a. m.</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1173,24 +1173,24 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>El Museo del Nunca Jamás</t>
+          <t>Matemático alemán que acertó el campeón de los últimos tres mundiales, predijo quién ganará en 2026</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/04/el-museo-del-nunca-jamas/</t>
+          <t>https://www.lafm.com.co/deportes/copa-mundial-fifa-2026-prediccion-aleman-acerto-campeon-2014-2018-2022-401316</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 01:00 a. m.</t>
+          <t>04/06/2026 12:49 a. m.</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -1200,24 +1200,24 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>En Santander las escuelas no salen a marchar</t>
+          <t>Capturan docente de Ética señalado de abusar de una niña en Cali: fue detenido mientras era jurado de votación</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/04/en-santander-las-escuelas-no-salen-a-marchar/</t>
+          <t>https://www.lafm.com.co/actualidad/abuso-menor-cali-capturan-docente-etica-senalado-jurado-votacion-401322</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 06:08 p. m.</t>
+          <t>03/06/2026 11:59 p. m.</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1227,24 +1227,24 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Piden llamar a indagatoria a Petro: los hallazgos que complican el caso de su campaña en 2022</t>
+          <t>El avión del papa: así será la operación de Iberia para mover a León XIV en su visita a España</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/03/piden-llamar-a-indagatoria-a-petro-los-hallazgos-que-complican-el-caso-de-su-campana-en-2022/</t>
+          <t>https://www.lafm.com.co/internacional/papa-leon-xiv-iberia-traslado-pontifice-espana-401317</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 06:08 p. m.</t>
+          <t>03/06/2026 11:34 a. m.</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -1254,24 +1254,24 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Abelardo de la Espriella no acepta apoyo del Partido Liberal: “es un apéndice de Petro y Cepeda”</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/</t>
+          <t>https://www.lafm.com.co/politica/abelardo-de-la-espriella-no-acepta-apoyo-partido-liberal-apendice-de-petro-y-cepeda-401325</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 02:59 p. m.</t>
+          <t>01/06/2026 09:56 p. m.</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1281,24 +1281,24 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Prima de los hermanos Mucutuy murió en combates tras ser reclutada por disidencias</t>
+          <t>Sin salida a la vista: continúa el cierre total de la Transversal del Sisga</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/03/prima-de-los-hermanos-mucutuy-murio-en-combates-tras-ser-reclutada-por-disidencias/</t>
+          <t>https://www.lafm.com.co/actualidad/transversal-sisga-colombia-cerrada-deslizamiento-401320</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 02:18 p. m.</t>
+          <t>01/06/2026 02:31 p. m.</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -1308,24 +1308,24 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Masacre de 11 menores en medio de combates expone la crisis por reclutamiento de niños</t>
+          <t>Aida Quilcué abre las puertas de su comunidad a Westcol y lleva la campaña presidencial al mundo del streaming</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/03/masacre-de-11-menores-en-combates-de-guaviare-expone-crisis-por-reclutamiento-de-ninos/</t>
+          <t>https://www.lafm.com.co/politica/aida-quilcue-abre-puertas-comunidad-westcol-401319</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 10:57 a. m.</t>
+          <t>31/05/2026 12:32 p. m.</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1335,24 +1335,24 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Orden judicial obligó a Petro a aclarar que los hermanos Moreno no fueron condenados</t>
+          <t>Petro ordenó bombardear zona del Guaviare donde se enfrentaron disidencias</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/politica/2026/06/03/orden-judicial-obligo-a-petro-a-aclarar-que-los-hermanos-moreno-no-fueron-condenados/</t>
+          <t>https://www.lafm.com.co/orden-publico/petro-ordeno-bombardear-zona-del-guaviare-donde-se-enfrentaron-disidencias-401336</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 09:24 a. m.</t>
+          <t>19/05/2026 10:14 a. m.</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
@@ -1362,22 +1362,26 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>La justificación de la Policía por uso de fuerza contra músico callejero tras denuncias en Parque La Colina en Bogotá</t>
+          <t>Masacre deja cuatro víctimas en Mondomo, Cauca</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/03/la-justificacion-de-la-policia-por-uso-de-fuerza-contra-musico-callejero-tras-denuncias-en-parque-la-colina-en-bogota/</t>
+          <t>https://www.lafm.com.co/orden-publico/masacre-deja-cuatro-victimas-en-mondomo-cauca-401338</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr"/>
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>08/05/2026 05:05 p. m.</t>
+        </is>
+      </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1385,17 +1389,17 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Tragedia en Guaviare: 11 adolescentes asesinados en combates entre alias ‘Iván Mordisco’ y ‘Calarcá’</t>
+          <t>Los cuatro episodios que le recuerdan a Petro tras criticar apoyo de Trump a De la Espriella</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/02/tragedia-en-guaviare-11-adolescentes-asesinados-en-combates-entre-alias-ivan-mordisco-y-calarca/</t>
+          <t>https://www.lafm.com.co/politica/petro-opino-elecciones-extranjeras-cuatro-casos-401331</t>
         </is>
       </c>
     </row>
@@ -1408,17 +1412,17 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>En directo: Petro entrega balance sobre la erradición de cultivos de coca durante su gobierno</t>
+          <t>"El centro político está destinado a desaparecer": representante a la Cámara lanza advertencia tras la primera vuelta presidencial</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/02/en-directo-el-presidente-petro-habla-sobre-los-resultados-de-la-primera-vuelta/</t>
+          <t>https://www.lafm.com.co/politica/centro-politico-colombia-crisis-segunda-vuelta-2026-401335</t>
         </is>
       </c>
     </row>
@@ -1431,26 +1435,22 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>¿Renunciará Petro para hacer campaña? Esto respondió su jefe de gabinete</t>
+          <t>Último sorteo Lotería de Manizales: resultado premio mayor hoy 3 de junio</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/02/renunciara-petro-para-hacer-campana-esto-respondio-su-jefe-de-gabinete/</t>
+          <t>https://www.lafm.com.co/sociedad/ultimo-sorteo-loteria-de-manizales-resultado-premio-mayor-hoy-3-de-junio-401332</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>04/06/2026 03:21 a. m.</t>
-        </is>
-      </c>
+      <c r="A37" s="5" t="inlineStr"/>
       <c r="B37" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1458,26 +1458,22 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>Israel y Líbano acuerdan un alto el fuego mediado por Estados Unidos</t>
+          <t>Movida clave en el gobierno Petro: Felipe Harman dejaría la ANT para aterrizar en la campaña de Iván Cepeda</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/israel-y-libano-acuerdan-un-alto-el-fuego-mediado-por-estados-unidos/</t>
+          <t>https://www.lafm.com.co/politica/agencia-nacional-de-tierras-felipe-harman-campana-ivan-cepeda-segunda-vuelta-401326</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>04/06/2026 01:13 a. m.</t>
-        </is>
-      </c>
+      <c r="A38" s="2" t="inlineStr"/>
       <c r="B38" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1485,26 +1481,22 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Petro ordena bombardear campamento de ‘Mordisco’ tras confrontación entre disidencias en el Guaviare</t>
+          <t>Capturan a la mamá de la bebé que murió tras ser víctima de abuso en El Espinal, Tolima</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/petro-ordena-bombardear-campamento-de-mordisco-tras-confrontacion-entre-disidencias-en-el-guaviare/</t>
+          <t>https://www.lafm.com.co/actualidad/capturan-mama-de-bebe-que-murio-en-el-espinal-tolima-401324</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="inlineStr">
-        <is>
-          <t>03/06/2026 11:49 p. m.</t>
-        </is>
-      </c>
+      <c r="A39" s="5" t="inlineStr"/>
       <c r="B39" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1512,26 +1504,22 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>Aída Quilcué acepta stream con Westcol en el Cauca: “eres bienvenido a nuestra comunidad”</t>
+          <t>Entró en vigencia la ‘Ley Sara Sofía’, que crea un sistema de alerta para encontrar niños desaparecidos</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/aida-quilcue-acepta-invitacion-de-westcol-y-se-confirma-streaming-desde-el-cauca/</t>
+          <t>https://www.lafm.com.co/politica/ley-sara-sofia-entra-en-vigencia-sistema-alerta-encontrar-ninos-desaparecidos-colombia-401321</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>03/06/2026 11:04 p. m.</t>
-        </is>
-      </c>
+      <c r="A40" s="2" t="inlineStr"/>
       <c r="B40" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1539,26 +1527,22 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Más de 800 estudiantes participaron en simulacro de emergencia volcánica en Pasto</t>
+          <t>Atención conductores: licencia de conducción cambia en 2026 para estas personas; estos son los nuevos exámenes y costos</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/mas-de-800-estudiantes-participaron-en-simulacro-de-emergencia-volcanica-en-pasto/</t>
+          <t>https://www.lafm.com.co/actualidad/licencia-conduccion-cambia-2026-nuevos-examenes-y-costos-401318</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="inlineStr">
-        <is>
-          <t>03/06/2026 09:58 p. m.</t>
-        </is>
-      </c>
+      <c r="A41" s="5" t="inlineStr"/>
       <c r="B41" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1566,24 +1550,24 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>Llegada del fenómeno de El Niño se intensifica, según alerta de la OMM: esta es la última proyección</t>
+          <t>Colpensiones explica cómo reclamar el dinero de los aportes si no logra pensionarse</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/llegada-del-fenomeno-de-el-nino-se-intensifica-segun-alerta-de-la-omm-esta-es-la-ultima-proyeccion/</t>
+          <t>https://www.lafm.com.co/economia/colpensiones-devolucion-diniero-sin-semanas-y-requisitos-401307</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 09:52 p. m.</t>
+          <t>04/06/2026 09:24 a. m.</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -1593,24 +1577,24 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>Elecciones segunda vuelta: ¿Personas que fueron jurados de votación repiten el 21 de junio?</t>
+          <t>La justificación de la Policía por uso de fuerza contra músico callejero tras denuncias en Parque La Colina en Bogotá</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/elecciones-segunda-vuelta-personas-que-fueron-jurados-de-votacion-repiten-el-21-de-junio/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/03/la-justificacion-de-la-policia-por-uso-de-fuerza-contra-musico-callejero-tras-denuncias-en-parque-la-colina-en-bogota/</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 09:50 p. m.</t>
+          <t>04/06/2026 07:05 a. m.</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
@@ -1620,24 +1604,24 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>Capturan a la ‘Mona’, cabecilla de disidencias, señalada de trasladar menores entre Cauca y Guaviare</t>
+          <t>Petro califica de intervencionista el respaldo de Trump a de La Espriella</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/capturan-a-la-mona-cabecilla-de-disidencias-senalada-de-trasladar-menores-reclutados-entre-cauca/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/03/petro-califica-de-intervencionista-el-respaldo-de-trump-a-de-la-espriella/</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 09:36 p. m.</t>
+          <t>04/06/2026 06:22 a. m.</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -1647,24 +1631,24 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>¿Cuánto gana el vicepresidente de Colombia en 2026? Este sería el salario de Quilcué o Restrepo</t>
+          <t>Fiscalía imputará cargos a ocho implicados en red de contrabando ligada a Lili Pink</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/cuanto-gana-el-vicepresidente-de-colombia-en-2026-este-seria-el-salario-de-quilcue-o-restrepo/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/03/fiscalia-imputara-cargos-a-ocho-implicados-en-red-de-contrabando-ligada-a-lili-pink/</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 09:22 p. m.</t>
+          <t>04/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
@@ -1674,24 +1658,24 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>Quinto ciclo Colombia Mayor: Prosperidad Social confirma fechas y canales para reclamar el subsidio</t>
+          <t>José Francisco Socarrás Colina</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/quinto-ciclo-colombia-mayor-prosperidad-social-confirma-fechas-y-canales-para-reclamar-el-subsidio/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/04/jose-francisco-socarras-colina/</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 08:35 p. m.</t>
+          <t>04/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -1701,24 +1685,24 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Abelardo de la Espriella rechaza respaldo del Partido Liberal: “Es un apéndice de Petro y Cepeda”</t>
+          <t>Columnistas</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/abelardo-de-la-espriella-rechaza-respaldo-liberal-es-un-apendice-de-petro-y-cepeda/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 07:48 p. m.</t>
+          <t>04/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
@@ -1728,24 +1712,24 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>Fiscalía capturó a la madre de Mía Cataleya en El Espinal</t>
+          <t>El Museo del Nunca Jamás</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/fiscalia-capturo-a-la-madre-de-mia-cataleya-en-el-espinal/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/04/el-museo-del-nunca-jamas/</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 07:46 p. m.</t>
+          <t>04/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -1755,24 +1739,24 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Resultados Lotería del Valle, Manizales, Meta y Baloto HOY 03 de junio, 2026: último sorteo y premio</t>
+          <t>En Santander las escuelas no salen a marchar</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/resultados-loteria-del-valle-manizales-meta-y-baloto-hoy-03-de-junio-2026-ultimo-sorteo-y-premio/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/04/en-santander-las-escuelas-no-salen-a-marchar/</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 07:24 p. m.</t>
+          <t>03/06/2026 06:08 p. m.</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
@@ -1782,24 +1766,24 @@
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>Centro Democrático en Antioquia anuncia respaldo a Abelardo de la Espriella para la segunda vuelta</t>
+          <t>Piden llamar a indagatoria a Petro: los hallazgos que complican el caso de su campaña en 2022</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/centro-democratico-en-antioquia-anuncia-respaldo-a-abelardo-de-la-espriella-para-la-segunda-vuelta/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/03/piden-llamar-a-indagatoria-a-petro-los-hallazgos-que-complican-el-caso-de-su-campana-en-2022/</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 07:12 p. m.</t>
+          <t>03/06/2026 06:08 p. m.</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -1809,24 +1793,24 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>Felipe Harman, director de la ANT sale del Gobierno para apoyar la campaña de Iván Cepeda</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/felipe-harman-director-de-la-ant-sale-del-gobierno-para-apoyar-la-campana-de-ivan-cepeda/</t>
+          <t>https://www.vanguardia.com/colombia/</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 07:01 p. m.</t>
+          <t>03/06/2026 02:59 p. m.</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
@@ -1836,24 +1820,24 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>Petro pide al CNE atender su denuncia sobre presunto fraude, pese a aclaración de la Registraduría</t>
+          <t>Prima de los hermanos Mucutuy murió en combates tras ser reclutada por disidencias</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/petro-pide-al-cne-atender-su-denuncia-sobre-presunto-fraude-pese-a-aclaracion-de-la-registraduria/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/03/prima-de-los-hermanos-mucutuy-murio-en-combates-tras-ser-reclutada-por-disidencias/</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 06:48 p. m.</t>
+          <t>03/06/2026 02:18 p. m.</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -1863,24 +1847,24 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Abren cupos para el Servicio Social para la Paz: certifica el servicio militar y entrega auxilio</t>
+          <t>Masacre de 11 menores en medio de combates expone la crisis por reclutamiento de niños</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/03/abren-cupos-para-el-servicio-social-para-la-paz-certifica-el-servicio-militar-y-entrega-auxilio/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/03/masacre-de-11-menores-en-combates-de-guaviare-expone-crisis-por-reclutamiento-de-ninos/</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 06:41 p. m.</t>
+          <t>03/06/2026 10:57 a. m.</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
@@ -1890,26 +1874,22 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>Petro cuestiona solicitud de indagatoria: “Ya amenazaron con encarcelarme sin cometer un delito”</t>
+          <t>Orden judicial obligó a Petro a aclarar que los hermanos Moreno no fueron condenados</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/03/petro-tras-solicitud-de-indagatoria-ya-amenazaron-con-encarcelarme-sin-cometer-un-delito/</t>
+          <t>https://www.vanguardia.com/politica/2026/06/03/orden-judicial-obligo-a-petro-a-aclarar-que-los-hermanos-moreno-no-fueron-condenados/</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>03/06/2026 06:41 p. m.</t>
-        </is>
-      </c>
+      <c r="A54" s="2" t="inlineStr"/>
       <c r="B54" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1917,26 +1897,22 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>OEA pide a grupos armados no interferir en segunda vuelta y a candidatos recibir resultados en paz</t>
+          <t>Tragedia en Guaviare: 11 adolescentes asesinados en combates entre alias ‘Iván Mordisco’ y ‘Calarcá’</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/03/oea-pide-a-grupos-armados-no-interferir-en-segunda-vuelta-y-a-candidatos-recibir-resultados-en-paz/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/02/tragedia-en-guaviare-11-adolescentes-asesinados-en-combates-entre-alias-ivan-mordisco-y-calarca/</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="5" t="inlineStr">
-        <is>
-          <t>03/06/2026 06:23 p. m.</t>
-        </is>
-      </c>
+      <c r="A55" s="5" t="inlineStr"/>
       <c r="B55" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1944,26 +1920,22 @@
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>Elecciones y Mundial: ¿Habrá inscripción de cédulas en sedes de Colombia? Esto dice la Registraduría</t>
+          <t>En directo: Petro entrega balance sobre la erradición de cultivos de coca durante su gobierno</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/03/elecciones-y-mundial-habra-inscripcion-de-cedulas-en-sedes-de-colombia-esto-dice-la-registraduria/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/02/en-directo-el-presidente-petro-habla-sobre-los-resultados-de-la-primera-vuelta/</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>03/06/2026 06:04 p. m.</t>
-        </is>
-      </c>
+      <c r="A56" s="2" t="inlineStr"/>
       <c r="B56" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1971,24 +1943,24 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Procuraduría inhabilitó por 5 años a cónsul honorario en Italia por cobro ilegal</t>
+          <t>¿Renunciará Petro para hacer campaña? Esto respondió su jefe de gabinete</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/03/procuraduria-inhabilito-por-5-anos-a-consul-honorario-en-italia-por-cobro-ilegal/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/02/renunciara-petro-para-hacer-campana-esto-respondio-su-jefe-de-gabinete/</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 02:57 a. m.</t>
+          <t>04/06/2026 04:06 a. m.</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
@@ -1998,24 +1970,24 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>Último sorteo Lotería de Manizales: resultado premio mayor hoy 3 de junio</t>
+          <t>Estados Unidos ataca otra lancha en el Pacífico y mata a dos tripulantes</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/sociedad/ultimo-sorteo-loteria-de-manizales-resultado-premio-mayor-hoy-3-de-junio-401332</t>
+          <t>https://caracol.com.co/2026/06/04/estados-unidos-ataca-otra-lancha-en-el-pacifico-y-mata-a-dos-tripulantes/</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 02:14 a. m.</t>
+          <t>04/06/2026 03:21 a. m.</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -2025,24 +1997,24 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Un telescopio a 1,5 millones de kilómetros de la Tierra reveló algo que llevaba décadas oculto</t>
+          <t>Israel y Líbano acuerdan un alto el fuego mediado por Estados Unidos</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/sociedad/telescopio-revela-misterio-universo-oculto-decadas-cientificos-nasa-401328</t>
+          <t>https://caracol.com.co/2026/06/04/israel-y-libano-acuerdan-un-alto-el-fuego-mediado-por-estados-unidos/</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 01:42 a. m.</t>
+          <t>04/06/2026 01:13 a. m.</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
@@ -2052,24 +2024,24 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>Claudia López se aleja de De la Espriella, reconoce la decencia de Cepeda y rechaza endosar sus votos</t>
+          <t>Petro ordena bombardear campamento de ‘Mordisco’ tras confrontación entre disidencias en el Guaviare</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/claudia-lopez-desconfianza-abelardo-de-la-espriella-respaldo-cepeda-401327</t>
+          <t>https://caracol.com.co/2026/06/04/petro-ordena-bombardear-campamento-de-mordisco-tras-confrontacion-entre-disidencias-en-el-guaviare/</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 12:51 a. m.</t>
+          <t>03/06/2026 11:49 p. m.</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -2079,24 +2051,24 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Matemático alemán que acertó el campeón de los últimos tres mundiales, predijo quién ganará en 2026</t>
+          <t>Aída Quilcué acepta stream con Westcol en el Cauca: “eres bienvenido a nuestra comunidad”</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/deportes/copa-mundial-fifa-2026-prediccion-aleman-acerto-campeon-2014-2018-2022-401316</t>
+          <t>https://caracol.com.co/2026/06/04/aida-quilcue-acepta-invitacion-de-westcol-y-se-confirma-streaming-desde-el-cauca/</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 12:49 a. m.</t>
+          <t>03/06/2026 11:04 p. m.</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
@@ -2106,24 +2078,24 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>Capturan docente de Ética señalado de abusar de una niña en Cali: fue detenido mientras era jurado de votación</t>
+          <t>Más de 800 estudiantes participaron en simulacro de emergencia volcánica en Pasto</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/actualidad/abuso-menor-cali-capturan-docente-etica-senalado-jurado-votacion-401322</t>
+          <t>https://caracol.com.co/2026/06/04/mas-de-800-estudiantes-participaron-en-simulacro-de-emergencia-volcanica-en-pasto/</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 11:59 p. m.</t>
+          <t>03/06/2026 09:58 p. m.</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -2133,24 +2105,24 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>El avión del papa: así será la operación de Iberia para mover a León XIV en su visita a España</t>
+          <t>Llegada del fenómeno de El Niño se intensifica, según alerta de la OMM: esta es la última proyección</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/internacional/papa-leon-xiv-iberia-traslado-pontifice-espana-401317</t>
+          <t>https://caracol.com.co/2026/06/04/llegada-del-fenomeno-de-el-nino-se-intensifica-segun-alerta-de-la-omm-esta-es-la-ultima-proyeccion/</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 11:45 p. m.</t>
+          <t>03/06/2026 09:52 p. m.</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
@@ -2160,24 +2132,24 @@
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
-          <t>El misterio de los "cazatesoros" que fueron grabados saliendo de alcantarillas en Nueva York</t>
+          <t>Elecciones segunda vuelta: ¿Personas que fueron jurados de votación repiten el 21 de junio?</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/actualidad/policia-nueva-york-investiga-hombres-401311</t>
+          <t>https://caracol.com.co/2026/06/04/elecciones-segunda-vuelta-personas-que-fueron-jurados-de-votacion-repiten-el-21-de-junio/</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 11:17 p. m.</t>
+          <t>03/06/2026 09:50 p. m.</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -2187,24 +2159,24 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Graves emergencias en Andes, Antioquia, por las lluvias</t>
+          <t>Capturan a la ‘Mona’, cabecilla de disidencias, señalada de trasladar menores entre Cauca y Guaviare</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/sociedad/emergencias-lluvias-andes-antioquia-avenida-torrencial-401312</t>
+          <t>https://caracol.com.co/2026/06/04/capturan-a-la-mona-cabecilla-de-disidencias-senalada-de-trasladar-menores-reclutados-entre-cauca/</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 11:34 a. m.</t>
+          <t>03/06/2026 09:36 p. m.</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
@@ -2214,24 +2186,24 @@
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>Abelardo de la Espriella no acepta apoyo del Partido Liberal: “es un apéndice de Petro y Cepeda”</t>
+          <t>¿Cuánto gana el vicepresidente de Colombia en 2026? Este sería el salario de Quilcué o Restrepo</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/abelardo-de-la-espriella-no-acepta-apoyo-partido-liberal-apendice-de-petro-y-cepeda-401325</t>
+          <t>https://caracol.com.co/2026/06/04/cuanto-gana-el-vicepresidente-de-colombia-en-2026-este-seria-el-salario-de-quilcue-o-restrepo/</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 09:56 p. m.</t>
+          <t>03/06/2026 09:22 p. m.</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -2241,24 +2213,24 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Sin salida a la vista: continúa el cierre total de la Transversal del Sisga</t>
+          <t>Quinto ciclo Colombia Mayor: Prosperidad Social confirma fechas y canales para reclamar el subsidio</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/actualidad/transversal-sisga-colombia-cerrada-deslizamiento-401320</t>
+          <t>https://caracol.com.co/2026/06/04/quinto-ciclo-colombia-mayor-prosperidad-social-confirma-fechas-y-canales-para-reclamar-el-subsidio/</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>01/06/2026 02:31 p. m.</t>
+          <t>03/06/2026 08:35 p. m.</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr">
@@ -2268,24 +2240,24 @@
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>Aida Quilcué abre las puertas de su comunidad a Westcol y lleva la campaña presidencial al mundo del streaming</t>
+          <t>Abelardo de la Espriella rechaza respaldo del Partido Liberal: “Es un apéndice de Petro y Cepeda”</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/aida-quilcue-abre-puertas-comunidad-westcol-401319</t>
+          <t>https://caracol.com.co/2026/06/04/abelardo-de-la-espriella-rechaza-respaldo-liberal-es-un-apendice-de-petro-y-cepeda/</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>31/05/2026 03:32 p. m.</t>
+          <t>03/06/2026 07:48 p. m.</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -2295,24 +2267,24 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>"El centro político está destinado a desaparecer": representante a la Cámara lanza advertencia tras la primera vuelta presidencial</t>
+          <t>Fiscalía capturó a la madre de Mía Cataleya en El Espinal</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/centro-politico-colombia-crisis-segunda-vuelta-2026-401335</t>
+          <t>https://caracol.com.co/2026/06/04/fiscalia-capturo-a-la-madre-de-mia-cataleya-en-el-espinal/</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>31/05/2026 12:32 p. m.</t>
+          <t>03/06/2026 07:46 p. m.</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
@@ -2322,22 +2294,26 @@
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>Petro ordenó bombardear zona del Guaviare donde se enfrentaron disidencias</t>
+          <t>Resultados Lotería del Valle, Manizales, Meta y Baloto HOY 03 de junio, 2026: último sorteo y premio</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/orden-publico/petro-ordeno-bombardear-zona-del-guaviare-donde-se-enfrentaron-disidencias-401336</t>
+          <t>https://caracol.com.co/2026/06/04/resultados-loteria-del-valle-manizales-meta-y-baloto-hoy-03-de-junio-2026-ultimo-sorteo-y-premio/</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="inlineStr"/>
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 07:24 p. m.</t>
+        </is>
+      </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2345,22 +2321,26 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>Los cuatro episodios que le recuerdan a Petro tras criticar apoyo de Trump a De la Espriella</t>
+          <t>Centro Democrático en Antioquia anuncia respaldo a Abelardo de la Espriella para la segunda vuelta</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/petro-opino-elecciones-extranjeras-cuatro-casos-401331</t>
+          <t>https://caracol.com.co/2026/06/04/centro-democratico-en-antioquia-anuncia-respaldo-a-abelardo-de-la-espriella-para-la-segunda-vuelta/</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="5" t="inlineStr"/>
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t>03/06/2026 07:12 p. m.</t>
+        </is>
+      </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2368,22 +2348,26 @@
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D71" s="6" t="inlineStr">
         <is>
-          <t>“Petro está reconociendo que su candidato no funcionó”; cuestionan protagonismo del presidente en la campaña de Cepeda</t>
+          <t>Felipe Harman, director de la ANT sale del Gobierno para apoyar la campaña de Iván Cepeda</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/gustavo-petro-ivan-cepeda-campana-pacto-historico-elecciones-presidenciales-2026-401330</t>
+          <t>https://caracol.com.co/2026/06/04/felipe-harman-director-de-la-ant-sale-del-gobierno-para-apoyar-la-campana-de-ivan-cepeda/</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="inlineStr"/>
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 07:01 p. m.</t>
+        </is>
+      </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2391,22 +2375,26 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>Movida clave en el gobierno Petro: Felipe Harman dejaría la ANT para aterrizar en la campaña de Iván Cepeda</t>
+          <t>Petro pide al CNE atender su denuncia sobre presunto fraude, pese a aclaración de la Registraduría</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/agencia-nacional-de-tierras-felipe-harman-campana-ivan-cepeda-segunda-vuelta-401326</t>
+          <t>https://caracol.com.co/2026/06/04/petro-pide-al-cne-atender-su-denuncia-sobre-presunto-fraude-pese-a-aclaracion-de-la-registraduria/</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="5" t="inlineStr"/>
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>03/06/2026 06:48 p. m.</t>
+        </is>
+      </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2414,22 +2402,26 @@
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D73" s="6" t="inlineStr">
         <is>
-          <t>Capturan a la mamá de la bebé que murió tras ser víctima de abuso en El Espinal, Tolima</t>
+          <t>Abren cupos para el Servicio Social para la Paz: certifica el servicio militar y entrega auxilio</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/actualidad/capturan-mama-de-bebe-que-murio-en-el-espinal-tolima-401324</t>
+          <t>https://caracol.com.co/2026/06/03/abren-cupos-para-el-servicio-social-para-la-paz-certifica-el-servicio-militar-y-entrega-auxilio/</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="inlineStr"/>
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 06:41 p. m.</t>
+        </is>
+      </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2437,22 +2429,26 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>Entró en vigencia la ‘Ley Sara Sofía’, que crea un sistema de alerta para encontrar niños desaparecidos</t>
+          <t>Petro cuestiona solicitud de indagatoria: “Ya amenazaron con encarcelarme sin cometer un delito”</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/ley-sara-sofia-entra-en-vigencia-sistema-alerta-encontrar-ninos-desaparecidos-colombia-401321</t>
+          <t>https://caracol.com.co/2026/06/03/petro-tras-solicitud-de-indagatoria-ya-amenazaron-con-encarcelarme-sin-cometer-un-delito/</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="5" t="inlineStr"/>
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t>03/06/2026 06:41 p. m.</t>
+        </is>
+      </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2460,22 +2456,26 @@
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr">
         <is>
-          <t>Atención conductores: licencia de conducción cambia en 2026 para estas personas; estos son los nuevos exámenes y costos</t>
+          <t>OEA pide a grupos armados no interferir en segunda vuelta y a candidatos recibir resultados en paz</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/actualidad/licencia-conduccion-cambia-2026-nuevos-examenes-y-costos-401318</t>
+          <t>https://caracol.com.co/2026/06/03/oea-pide-a-grupos-armados-no-interferir-en-segunda-vuelta-y-a-candidatos-recibir-resultados-en-paz/</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="inlineStr"/>
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 06:23 p. m.</t>
+        </is>
+      </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2483,17 +2483,17 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>Colpensiones explica cómo reclamar el dinero de los aportes si no logra pensionarse</t>
+          <t>Elecciones y Mundial: ¿Habrá inscripción de cédulas en sedes de Colombia? Esto dice la Registraduría</t>
         </is>
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/economia/colpensiones-devolucion-diniero-sin-semanas-y-requisitos-401307</t>
+          <t>https://caracol.com.co/2026/06/03/elecciones-y-mundial-habra-inscripcion-de-cedulas-en-sedes-de-colombia-esto-dice-la-registraduria/</t>
         </is>
       </c>
     </row>
@@ -2824,7 +2824,7 @@
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 12:48 a. m.</t>
+          <t>04/06/2026 01:22 a. m.</t>
         </is>
       </c>
       <c r="B89" s="5" t="inlineStr">
@@ -4173,7 +4173,7 @@
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 12:06 a. m.</t>
+          <t>04/06/2026 12:00 a. m.</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
@@ -4183,24 +4183,24 @@
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae Colombia</t>
         </is>
       </c>
       <c r="D144" s="3" t="inlineStr">
         <is>
-          <t>La mejor campaña era hacer un buen gobierno</t>
+          <t>“Jamás debieron vincular a su guerra”: ICBF condena la muerte de 11 menores en combates entre disidencias en Guaviare</t>
         </is>
       </c>
       <c r="E144" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/blancainesduran/la-mejor-campana-era-hacer-un-buen-gobierno/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/jamas-debieron-vincular-a-su-guerra-icbf-condena-la-muerte-de-11-menores-en-combates-entre-disidencias-en-guaviare/</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 12:05 a. m.</t>
+          <t>04/06/2026 12:00 a. m.</t>
         </is>
       </c>
       <c r="B145" s="5" t="inlineStr">
@@ -4210,24 +4210,24 @@
       </c>
       <c r="C145" s="5" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae Colombia</t>
         </is>
       </c>
       <c r="D145" s="6" t="inlineStr">
         <is>
-          <t>De Santa Marta a Tuvalu: cultivar la frágil esperanza</t>
+          <t>Peajes de Autopistas del Café bajarán a $700 para vehículos beneficiarios tras anuncio de Gustavo Petro</t>
         </is>
       </c>
       <c r="E145" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/german-i-andrade-/de-santa-marta-a-tuvalu-cultivar-la-fragil-esperanza/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/peajes-de-autopistas-del-cafe-bajaran-a-700-para-vehiculos-beneficiarios-tras-anuncio-de-gustavo-petro/</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 12:05 a. m.</t>
+          <t>04/06/2026 12:00 a. m.</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
@@ -4237,24 +4237,24 @@
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae Colombia</t>
         </is>
       </c>
       <c r="D146" s="3" t="inlineStr">
         <is>
-          <t>¿Verde + rosa = blanco?</t>
+          <t>“No son estudiantes, son terroristas”: Federico Gutiérrez se pronuncia tras disturbios de encapuchados en la Universidad de Antioquia</t>
         </is>
       </c>
       <c r="E146" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/brigitte-lg-baptiste/verde-rosa-blanco/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/no-son-estudiantes-son-terroristas-federico-gutierrez-se-pronuncia-tras-disturbios-de-encapuchados-en-la-universidad-de-antioquia/</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 12:05 a. m.</t>
+          <t>04/06/2026 12:00 a. m.</t>
         </is>
       </c>
       <c r="B147" s="5" t="inlineStr">
@@ -4264,24 +4264,24 @@
       </c>
       <c r="C147" s="5" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae Colombia</t>
         </is>
       </c>
       <c r="D147" s="6" t="inlineStr">
         <is>
-          <t>Sobre Mozart y la inteligencia artificial</t>
+          <t>Procuraduría inhabilita por cinco años a cónsul honorario de Colombia en Italia por cobro indebido a una ciudadana</t>
         </is>
       </c>
       <c r="E147" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/manuel-drezner/sobre-mozart-y-la-inteligencia-artificial/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/procuraduria-inhabilita-por-cinco-anos-a-consul-honorario-de-colombia-en-italia-por-cobro-indebido-a-una-ciudadana/</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 12:05 a. m.</t>
+          <t>04/06/2026 12:00 a. m.</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
@@ -4291,24 +4291,24 @@
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae Colombia</t>
         </is>
       </c>
       <c r="D148" s="3" t="inlineStr">
         <is>
-          <t>Más allá del voto en blanco</t>
+          <t>Asesinan a cobradiario en Barranquilla que había sobrevivido a un atentado; ya son tres casos en menos de 48 horas</t>
         </is>
       </c>
       <c r="E148" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/cristinacarrizosa/mas-alla-del-voto-en-blanco/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/asesinan-a-cobradiario-en-barranquilla-que-habia-sobrevivido-a-un-atentado-ya-son-tres-casos-en-menos-de-48-horas/</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 12:05 a. m.</t>
+          <t>04/06/2026 12:00 a. m.</t>
         </is>
       </c>
       <c r="B149" s="5" t="inlineStr">
@@ -4318,24 +4318,24 @@
       </c>
       <c r="C149" s="5" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae Colombia</t>
         </is>
       </c>
       <c r="D149" s="6" t="inlineStr">
         <is>
-          <t>Los votos están ahí</t>
+          <t>Luis Gilberto Murillo rechaza injerencia extranjera y pide unidad nacional: “Nuestra soberanía, democracia y voto se respetan”</t>
         </is>
       </c>
       <c r="E149" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/javier-ortiz/los-votos-estan-ahi/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/luis-gilberto-murillo-rechaza-injerencia-extranjera-y-pide-unidad-nacional-nuestra-soberania-democracia-y-voto-se-respetan/</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 12:05 a. m.</t>
+          <t>04/06/2026 12:00 a. m.</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
@@ -4345,24 +4345,24 @@
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae Colombia</t>
         </is>
       </c>
       <c r="D150" s="3" t="inlineStr">
         <is>
-          <t>Líder del equipo digital de De la Espriella denunciado por violencia sexual</t>
+          <t>Dos niños terminan en UCI tras ingerir raticida en Atlántico; autoridades hacen llamado urgente a los padres</t>
         </is>
       </c>
       <c r="E150" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/catalina-ruiz-navarro/lider-del-equipo-digital-de-de-la-espriella-denunciado-por-violencia-sexual/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/dos-ninos-terminan-en-uci-tras-ingerir-raticida-en-atlantico-autoridades-hacen-llamado-urgente-a-los-padres/</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 12:04 a. m.</t>
+          <t>04/06/2026 12:00 a. m.</t>
         </is>
       </c>
       <c r="B151" s="5" t="inlineStr">
@@ -4372,24 +4372,24 @@
       </c>
       <c r="C151" s="5" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae Colombia</t>
         </is>
       </c>
       <c r="D151" s="6" t="inlineStr">
         <is>
-          <t>Gurropín, corrupto dictador venerado por la izquierda populista</t>
+          <t>Colombia podría enfrentar arancel de 12,5% en EE. UU. por nueva estrategia comercial impulsada por Trump</t>
         </is>
       </c>
       <c r="E151" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/mauricio-rubio/gurropin-corrupto-dictador-venerado-por-la-izquierda-populista/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/colombia-podria-enfrentar-arancel-de-125-en-ee-uu-por-nueva-estrategia-comercial-impulsada-por-trump/</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 12:04 a. m.</t>
+          <t>04/06/2026 12:00 a. m.</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
@@ -4399,17 +4399,17 @@
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae Colombia</t>
         </is>
       </c>
       <c r="D152" s="3" t="inlineStr">
         <is>
-          <t>Quiero hablar con las flores</t>
+          <t>¿Cómo estará el clima en Medellín?</t>
         </is>
       </c>
       <c r="E152" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/juan-david-zuloaga-d-/quiero-hablar-con-las-flores/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/como-estara-el-clima-en-medellin/</t>
         </is>
       </c>
     </row>
@@ -4426,17 +4426,17 @@
       </c>
       <c r="C153" s="5" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>Infobae Colombia</t>
         </is>
       </c>
       <c r="D153" s="6" t="inlineStr">
         <is>
-          <t>Atrapados entre la espada, la pared y la improvisación</t>
+          <t>Las últimas previsiones para Bogotá: temperatura, lluvias y viento</t>
         </is>
       </c>
       <c r="E153" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/lectores/cartas/atrapados-entre-la-espada-la-pared-y-la-improvisacion/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/las-ultimas-previsiones-para-bogota-temperatura-lluvias-y-viento/</t>
         </is>
       </c>
     </row>
@@ -4458,12 +4458,12 @@
       </c>
       <c r="D154" s="3" t="inlineStr">
         <is>
-          <t>¿Cómo estará el clima en Medellín?</t>
+          <t>Clima en Cartagena de Indias: la predicción para este 4 de junio</t>
         </is>
       </c>
       <c r="E154" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/como-estara-el-clima-en-medellin/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/clima-en-cartagena-de-indias-la-prediccion-para-este-4-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4485,12 +4485,12 @@
       </c>
       <c r="D155" s="6" t="inlineStr">
         <is>
-          <t>Las últimas previsiones para Bogotá: temperatura, lluvias y viento</t>
+          <t>Pronóstico del clima en Cali este 4 de junio: temperatura, lluvias y viento</t>
         </is>
       </c>
       <c r="E155" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/las-ultimas-previsiones-para-bogota-temperatura-lluvias-y-viento/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/pronostico-del-clima-en-cali-este-4-de-junio-temperatura-lluvias-y-viento/</t>
         </is>
       </c>
     </row>
@@ -4512,12 +4512,12 @@
       </c>
       <c r="D156" s="3" t="inlineStr">
         <is>
-          <t>Clima en Cartagena de Indias: la predicción para este 4 de junio</t>
+          <t>Las últimas previsiones para Barranquilla: temperatura, lluvias y viento</t>
         </is>
       </c>
       <c r="E156" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/clima-en-cartagena-de-indias-la-prediccion-para-este-4-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/las-ultimas-previsiones-para-barranquilla-temperatura-lluvias-y-viento/</t>
         </is>
       </c>
     </row>
@@ -4539,12 +4539,12 @@
       </c>
       <c r="D157" s="6" t="inlineStr">
         <is>
-          <t>Pronóstico del clima en Cali este 4 de junio: temperatura, lluvias y viento</t>
+          <t>“Haber traído a Álvaro Uribe Vélez como ministro de Defensa espantó al centro”: Juan Daniel Oviedo analiza caída de Paloma Valencia</t>
         </is>
       </c>
       <c r="E157" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/pronostico-del-clima-en-cali-este-4-de-junio-temperatura-lluvias-y-viento/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/haber-traido-a-alvaro-uribe-velez-como-ministro-de-defensa-espanto-al-centro-juan-daniel-oviedo-analiza-caida-de-paloma-valencia/</t>
         </is>
       </c>
     </row>
@@ -4566,12 +4566,12 @@
       </c>
       <c r="D158" s="3" t="inlineStr">
         <is>
-          <t>Las últimas previsiones para Barranquilla: temperatura, lluvias y viento</t>
+          <t>Felipe Harman dejaría la ANT para unirse a la campaña de Iván Cepeda y coordinar la recta final electoral</t>
         </is>
       </c>
       <c r="E158" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/las-ultimas-previsiones-para-barranquilla-temperatura-lluvias-y-viento/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/felipe-harman-dejaria-la-ant-para-unirse-a-la-campana-de-ivan-cepeda-y-coordinar-la-recta-final-electoral/</t>
         </is>
       </c>
     </row>
@@ -4593,12 +4593,12 @@
       </c>
       <c r="D159" s="6" t="inlineStr">
         <is>
-          <t>“Haber traído a Álvaro Uribe Vélez como ministro de Defensa espantó al centro”: Juan Daniel Oviedo analiza caída de Paloma Valencia</t>
+          <t>Nequi suspenderá temporalmente los pagos por PSE durante una jornada de mantenimiento: conozca cuándo será la interrupción</t>
         </is>
       </c>
       <c r="E159" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/haber-traido-a-alvaro-uribe-velez-como-ministro-de-defensa-espanto-al-centro-juan-daniel-oviedo-analiza-caida-de-paloma-valencia/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/nequi-suspendera-temporalmente-los-pagos-por-pse-durante-una-jornada-de-mantenimiento-conozca-cuando-sera-la-interrupcion/</t>
         </is>
       </c>
     </row>
@@ -4620,12 +4620,12 @@
       </c>
       <c r="D160" s="3" t="inlineStr">
         <is>
-          <t>Felipe Harman dejaría la ANT para unirse a la campaña de Iván Cepeda y coordinar la recta final electoral</t>
+          <t>Avenida torrencial en Andes arrasó puentes y obligó a evacuar al menos a 150 personas en Santa Inés, Antioquia</t>
         </is>
       </c>
       <c r="E160" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/felipe-harman-dejaria-la-ant-para-unirse-a-la-campana-de-ivan-cepeda-y-coordinar-la-recta-final-electoral/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/avenida-torrencial-en-andes-arraso-puentes-y-obligo-a-evacuar-al-menos-a-150-personas-en-santa-ines-antioquia/</t>
         </is>
       </c>
     </row>
@@ -4647,12 +4647,12 @@
       </c>
       <c r="D161" s="6" t="inlineStr">
         <is>
-          <t>Nequi suspenderá temporalmente los pagos por PSE durante una jornada de mantenimiento: conozca cuándo será la interrupción</t>
+          <t>Pico y Placa Bogotá: evita multas este jueves 4 de junio</t>
         </is>
       </c>
       <c r="E161" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/nequi-suspendera-temporalmente-los-pagos-por-pse-durante-una-jornada-de-mantenimiento-conozca-cuando-sera-la-interrupcion/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/pico-y-placa-bogota-evita-multas-este-jueves-4-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4674,12 +4674,12 @@
       </c>
       <c r="D162" s="3" t="inlineStr">
         <is>
-          <t>Avenida torrencial en Andes arrasó puentes y obligó a evacuar al menos a 150 personas en Santa Inés, Antioquia</t>
+          <t>Denuncian que lanzaron objetos desde un edificio contra manifestantes de Iván Cepeda en Medellín: un niño resultó herido</t>
         </is>
       </c>
       <c r="E162" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/avenida-torrencial-en-andes-arraso-puentes-y-obligo-a-evacuar-al-menos-a-150-personas-en-santa-ines-antioquia/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/denuncian-que-lanzaron-objetos-desde-un-edificio-contra-manifestantes-de-ivan-cepeda-en-medellin-un-nino-resulto-herido/</t>
         </is>
       </c>
     </row>
@@ -4701,19 +4701,19 @@
       </c>
       <c r="D163" s="6" t="inlineStr">
         <is>
-          <t>Pico y Placa Bogotá: evita multas este jueves 4 de junio</t>
+          <t>Resultados Baloto y Revancha, último sorteo del miércoles 3 de junio</t>
         </is>
       </c>
       <c r="E163" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/pico-y-placa-bogota-evita-multas-este-jueves-4-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/04/resultados-baloto-y-revancha-ultimo-sorteo-del-miercoles-3-de-junio/</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 12:00 a. m.</t>
+          <t>03/06/2026 07:45 p. m.</t>
         </is>
       </c>
       <c r="B164" s="2" t="inlineStr">
@@ -4723,24 +4723,24 @@
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>Infobae Colombia</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D164" s="3" t="inlineStr">
         <is>
-          <t>Denuncian que lanzaron objetos desde un edificio contra manifestantes de Iván Cepeda en Medellín: un niño resultó herido</t>
+          <t>Registraduría confirma cierre del escrutinio: reclamaciones no superaron el 0,7 por ciento de las mesas</t>
         </is>
       </c>
       <c r="E164" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/denuncian-que-lanzaron-objetos-desde-un-edificio-contra-manifestantes-de-ivan-cepeda-en-medellin-un-nino-resulto-herido/</t>
+          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/registraduria-confirma-cierre-del-escrutinio-reclamaciones-no-superaron-el-07-por-ciento-de-las-mesas</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 12:00 a. m.</t>
+          <t>03/06/2026 06:25 p. m.</t>
         </is>
       </c>
       <c r="B165" s="5" t="inlineStr">
@@ -4750,24 +4750,24 @@
       </c>
       <c r="C165" s="5" t="inlineStr">
         <is>
-          <t>Infobae Colombia</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D165" s="6" t="inlineStr">
         <is>
-          <t>Resultados Baloto y Revancha, último sorteo del miércoles 3 de junio</t>
+          <t>Denuncian que ataque con explosivos en El Bagre, Antioquia, afectó a animales de comunidades campesinas</t>
         </is>
       </c>
       <c r="E165" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/resultados-baloto-y-revancha-ultimo-sorteo-del-miercoles-3-de-junio/</t>
+          <t>https://cambiocolombia.com/conflicto-armado-en-colombia/articulo/2026/6/denuncian-que-ataque-con-explosivos-en-el-bagre-antioquia-afecto-a-animales-de-comunidades-campesinas</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 12:00 a. m.</t>
+          <t>03/06/2026 06:00 p. m.</t>
         </is>
       </c>
       <c r="B166" s="2" t="inlineStr">
@@ -4777,24 +4777,24 @@
       </c>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>Infobae Colombia</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D166" s="3" t="inlineStr">
         <is>
-          <t>Resultado Baloto y Revancha hoy 3 de junio</t>
+          <t>Caso Zulma Guzmán: ¿qué encontraron los investigadores en su locker en el Club El Nogal?</t>
         </is>
       </c>
       <c r="E166" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/resultado-baloto-y-revancha-hoy-3-de-junio/</t>
+          <t>https://cambiocolombia.com/pais/articulo/2026/6/caso-zulma-guzman-que-encontraron-los-investigadores-en-su-locker-en-el-club-el-nogal</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 12:00 a. m.</t>
+          <t>03/06/2026 06:00 p. m.</t>
         </is>
       </c>
       <c r="B167" s="5" t="inlineStr">
@@ -4804,24 +4804,24 @@
       </c>
       <c r="C167" s="5" t="inlineStr">
         <is>
-          <t>Infobae Colombia</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D167" s="6" t="inlineStr">
         <is>
-          <t>MOE responde a denuncias de fraude: explica las 885.000 cédulas, las mesas adicionales y los puestos de votación en la primera vuelta</t>
+          <t>Registraduría solicita al Gobierno recursos para la segunda vuelta presidencial del 21 de junio</t>
         </is>
       </c>
       <c r="E167" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/moe-responde-a-denuncias-de-fraude-explica-las-885000-cedulas-las-mesas-adicionales-y-los-puestos-de-votacion-en-la-primera-vuelta/</t>
+          <t>https://cambiocolombia.com/pais/articulo/2026/6/registraduria-solicita-al-gobierno-recursos-para-la-segunda-vuelta-presidencial-del-21-de-junio</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 12:00 a. m.</t>
+          <t>03/06/2026 05:00 p. m.</t>
         </is>
       </c>
       <c r="B168" s="2" t="inlineStr">
@@ -4831,24 +4831,24 @@
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>Infobae Colombia</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D168" s="3" t="inlineStr">
         <is>
-          <t>Lotería de Manizales resultados miércoles 3 de junio: quién ganó el premio mayor de $2.600 millones</t>
+          <t>Cambio de Frente: el newsletter de CAMBIO que cuenta el Mundial como se debe</t>
         </is>
       </c>
       <c r="E168" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/loteria-de-manizales-resultados-miercoles-3-de-junio-quien-gano-el-premio-mayor-de-2600-millones/</t>
+          <t>https://cambiocolombia.com/deportes/articulo/2026/6/cambio-de-frente-el-newsletter-de-cambio-que-cuenta-el-mundial-como-se-debe</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 12:00 a. m.</t>
+          <t>03/06/2026 04:45 p. m.</t>
         </is>
       </c>
       <c r="B169" s="5" t="inlineStr">
@@ -4858,24 +4858,24 @@
       </c>
       <c r="C169" s="5" t="inlineStr">
         <is>
-          <t>Infobae Colombia</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D169" s="6" t="inlineStr">
         <is>
-          <t>Resultados de la Lotería del Valle miércoles 3 de junio de 2026: todos los secos millonarios</t>
+          <t>Marco Rubio pide establecer “lo antes posible” las condiciones para elecciones en Venezuela y pide una nueva comisión electoral</t>
         </is>
       </c>
       <c r="E169" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/resultados-de-la-loteria-del-valle-miercoles-3-de-junio-de-2026-todos-los-secos-millonarios/</t>
+          <t>https://cambiocolombia.com/internacional/articulo/2026/6/marco-rubio-pide-establecer-lo-antes-posible-las-condiciones-para-elecciones-en-venezuela-y-pide-una-nueva-comision-electoral</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 12:00 a. m.</t>
+          <t>03/06/2026 03:10 p. m.</t>
         </is>
       </c>
       <c r="B170" s="2" t="inlineStr">
@@ -4885,24 +4885,24 @@
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>Infobae Colombia</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D170" s="3" t="inlineStr">
         <is>
-          <t>Resultados Lotería del Valle miércoles 3 de junio de 2026: quién ganó el premio mayor de $9.000 millones</t>
+          <t>Los mensajes de apoyo entre Trump y De la Espriella que desataron la reacción de Petro</t>
         </is>
       </c>
       <c r="E170" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/resultados-loteria-del-valle-miercoles-3-de-junio-de-2026-quien-gano-el-premio-mayor-de-9000-millones/</t>
+          <t>https://cambiocolombia.com/poder/articulo/2026/6/los-mensajes-de-apoyo-entre-trump-y-de-la-espriella-que-desataron-la-reaccion-de-petro</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 12:00 a. m.</t>
+          <t>03/06/2026 12:45 p. m.</t>
         </is>
       </c>
       <c r="B171" s="5" t="inlineStr">
@@ -4912,24 +4912,24 @@
       </c>
       <c r="C171" s="5" t="inlineStr">
         <is>
-          <t>Infobae Colombia</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D171" s="6" t="inlineStr">
         <is>
-          <t>“No son estudiantes, son terroristas”: Federico Gutiérrez se pronuncia tras disturbios de encapuchados en la Universidad de Antioquia</t>
+          <t>“Los niños y adolescentes no le pertenecen a la guerra”: Procurador exige acciones tras muerte de 11 menores en el Guaviare</t>
         </is>
       </c>
       <c r="E171" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/no-son-estudiantes-son-terroristas-federico-gutierrez-se-pronuncia-tras-disturbios-de-encapuchados-en-la-universidad-de-antioquia/</t>
+          <t>https://cambiocolombia.com/conflicto-armado-en-colombia/articulo/2026/6/los-ninos-y-adolescentes-no-le-pertenecen-a-la-guerra-procurador-exige-acciones-tras-muerte-de-11-menores-en-el-guaviare</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 12:00 a. m.</t>
+          <t>03/06/2026 12:00 p. m.</t>
         </is>
       </c>
       <c r="B172" s="2" t="inlineStr">
@@ -4939,24 +4939,24 @@
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>Infobae Colombia</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D172" s="3" t="inlineStr">
         <is>
-          <t>“Jamás debieron vincular a su guerra”: ICBF condena la muerte de 11 menores en combates entre disidencias en Guaviare</t>
+          <t>Registraduría le respondió a Petro por denuncia en 5.300 mesas: no encontraron irregularidades</t>
         </is>
       </c>
       <c r="E172" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/jamas-debieron-vincular-a-su-guerra-icbf-condena-la-muerte-de-11-menores-en-combates-entre-disidencias-en-guaviare/</t>
+          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/registraduria-le-respondio-a-petro-por-denuncia-en-5300-mesas-no-encontraron-irregularidades</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 12:00 a. m.</t>
+          <t>03/06/2026 11:45 a. m.</t>
         </is>
       </c>
       <c r="B173" s="5" t="inlineStr">
@@ -4966,24 +4966,24 @@
       </c>
       <c r="C173" s="5" t="inlineStr">
         <is>
-          <t>Infobae Colombia</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D173" s="6" t="inlineStr">
         <is>
-          <t>Baloto y Revancha: números ganadores del lunes 1 de junio</t>
+          <t>Leonardo Huerta, exfórmula de Claudia López, se une a la campaña de Abelardo de la Espriella</t>
         </is>
       </c>
       <c r="E173" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/04/baloto-y-revancha-numeros-ganadores-del-lunes-1-de-junio/</t>
+          <t>https://cambiocolombia.com/poder/articulo/2026/6/leonardo-huerta-exformula-de-claudia-lopez-se-une-a-la-campana-de-abelardo-de-la-espriella</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 07:45 p. m.</t>
+          <t>03/06/2026 11:00 a. m.</t>
         </is>
       </c>
       <c r="B174" s="2" t="inlineStr">
@@ -4998,19 +4998,19 @@
       </c>
       <c r="D174" s="3" t="inlineStr">
         <is>
-          <t>Registraduría confirma cierre del escrutinio: reclamaciones no superaron el 0,7 por ciento de las mesas</t>
+          <t>Corte Suprema condenó a exgobernador Arauca</t>
         </is>
       </c>
       <c r="E174" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/registraduria-confirma-cierre-del-escrutinio-reclamaciones-no-superaron-el-07-por-ciento-de-las-mesas</t>
+          <t>https://cambiocolombia.com/pais/articulo/2026/6/corte-suprema-condeno-a-exgobernador-arauca</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 06:25 p. m.</t>
+          <t>03/06/2026 10:45 a. m.</t>
         </is>
       </c>
       <c r="B175" s="5" t="inlineStr">
@@ -5025,19 +5025,19 @@
       </c>
       <c r="D175" s="6" t="inlineStr">
         <is>
-          <t>Denuncian que ataque con explosivos en El Bagre, Antioquia, afectó a animales de comunidades campesinas</t>
+          <t>El documento de Petro sobre fraude proviene de la Registraduría, pero modificado por alguien externo</t>
         </is>
       </c>
       <c r="E175" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/conflicto-armado-en-colombia/articulo/2026/6/denuncian-que-ataque-con-explosivos-en-el-bagre-antioquia-afecto-a-animales-de-comunidades-campesinas</t>
+          <t>https://cambiocolombia.com/poder/articulo/2026/6/el-documento-de-petro-sobre-fraude-proviene-de-la-registraduria-pero-modificado-por-alguien-externo</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 06:00 p. m.</t>
+          <t>03/06/2026 10:00 a. m.</t>
         </is>
       </c>
       <c r="B176" s="2" t="inlineStr">
@@ -5052,19 +5052,19 @@
       </c>
       <c r="D176" s="3" t="inlineStr">
         <is>
-          <t>Caso Zulma Guzmán: ¿qué encontraron los investigadores en su locker en el Club El Nogal?</t>
+          <t>"No más cafés, más debates": Juan Daniel Oviedo evita apoyar a Iván Cepeda o a Abelardo de la Espriella</t>
         </is>
       </c>
       <c r="E176" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/pais/articulo/2026/6/caso-zulma-guzman-que-encontraron-los-investigadores-en-su-locker-en-el-club-el-nogal</t>
+          <t>https://cambiocolombia.com/poder/articulo/2026/6/no-mas-cafes-mas-debates-juan-daniel-oviedo-evita-apoyar-a-ivan-cepeda-o-a-abelardo-de-la-espriella</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 06:00 p. m.</t>
+          <t>03/06/2026 08:02 a. m.</t>
         </is>
       </c>
       <c r="B177" s="5" t="inlineStr">
@@ -5079,19 +5079,19 @@
       </c>
       <c r="D177" s="6" t="inlineStr">
         <is>
-          <t>Registraduría solicita al Gobierno recursos para la segunda vuelta presidencial del 21 de junio</t>
+          <t>Registraduría defiende la legalidad del proceso electoral frente a críticas de Gustavo Petro</t>
         </is>
       </c>
       <c r="E177" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/pais/articulo/2026/6/registraduria-solicita-al-gobierno-recursos-para-la-segunda-vuelta-presidencial-del-21-de-junio</t>
+          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/registraduria-defiende-la-legalidad-del-proceso-electoral-frente-a-criticas-de-gustavo-petro</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 05:00 p. m.</t>
+          <t>03/06/2026 07:20 a. m.</t>
         </is>
       </c>
       <c r="B178" s="2" t="inlineStr">
@@ -5106,21 +5106,17 @@
       </c>
       <c r="D178" s="3" t="inlineStr">
         <is>
-          <t>Cambio de Frente: el newsletter de CAMBIO que cuenta el Mundial como se debe</t>
+          <t>Minambiente anuncia plan de acción para el caimán llanero tras denuncias de meses sin alimentación y muertes</t>
         </is>
       </c>
       <c r="E178" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/deportes/articulo/2026/6/cambio-de-frente-el-newsletter-de-cambio-que-cuenta-el-mundial-como-se-debe</t>
+          <t>https://cambiocolombia.com/medio-ambiente/articulo/2026/6/minambiente-anuncia-plan-de-accion-para-el-caiman-llanero-tras-denuncias-de-meses-sin-alimentacion-y-muertes</t>
         </is>
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="5" t="inlineStr">
-        <is>
-          <t>03/06/2026 04:45 p. m.</t>
-        </is>
-      </c>
+      <c r="A179" s="5" t="inlineStr"/>
       <c r="B179" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5128,26 +5124,22 @@
       </c>
       <c r="C179" s="5" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D179" s="6" t="inlineStr">
         <is>
-          <t>Marco Rubio pide establecer “lo antes posible” las condiciones para elecciones en Venezuela y pide una nueva comisión electoral</t>
+          <t>La mejor campaña era hacer un buen gobierno</t>
         </is>
       </c>
       <c r="E179" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/internacional/articulo/2026/6/marco-rubio-pide-establecer-lo-antes-posible-las-condiciones-para-elecciones-en-venezuela-y-pide-una-nueva-comision-electoral</t>
+          <t>https://www.elespectador.com/opinion/columnistas/blancainesduran/la-mejor-campana-era-hacer-un-buen-gobierno/</t>
         </is>
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="2" t="inlineStr">
-        <is>
-          <t>03/06/2026 03:10 p. m.</t>
-        </is>
-      </c>
+      <c r="A180" s="2" t="inlineStr"/>
       <c r="B180" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5155,26 +5147,22 @@
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D180" s="3" t="inlineStr">
         <is>
-          <t>Los mensajes de apoyo entre Trump y De la Espriella que desataron la reacción de Petro</t>
+          <t>De Santa Marta a Tuvalu: cultivar la frágil esperanza</t>
         </is>
       </c>
       <c r="E180" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/poder/articulo/2026/6/los-mensajes-de-apoyo-entre-trump-y-de-la-espriella-que-desataron-la-reaccion-de-petro</t>
+          <t>https://www.elespectador.com/opinion/columnistas/german-i-andrade-/de-santa-marta-a-tuvalu-cultivar-la-fragil-esperanza/</t>
         </is>
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="5" t="inlineStr">
-        <is>
-          <t>03/06/2026 12:45 p. m.</t>
-        </is>
-      </c>
+      <c r="A181" s="5" t="inlineStr"/>
       <c r="B181" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5182,26 +5170,22 @@
       </c>
       <c r="C181" s="5" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D181" s="6" t="inlineStr">
         <is>
-          <t>“Los niños y adolescentes no le pertenecen a la guerra”: Procurador exige acciones tras muerte de 11 menores en el Guaviare</t>
+          <t>¿Verde + rosa = blanco?</t>
         </is>
       </c>
       <c r="E181" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/conflicto-armado-en-colombia/articulo/2026/6/los-ninos-y-adolescentes-no-le-pertenecen-a-la-guerra-procurador-exige-acciones-tras-muerte-de-11-menores-en-el-guaviare</t>
+          <t>https://www.elespectador.com/opinion/columnistas/brigitte-lg-baptiste/verde-rosa-blanco/</t>
         </is>
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="2" t="inlineStr">
-        <is>
-          <t>03/06/2026 12:00 p. m.</t>
-        </is>
-      </c>
+      <c r="A182" s="2" t="inlineStr"/>
       <c r="B182" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5209,26 +5193,22 @@
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D182" s="3" t="inlineStr">
         <is>
-          <t>Registraduría le respondió a Petro por denuncia en 5.300 mesas: no encontraron irregularidades</t>
+          <t>Sobre Mozart y la inteligencia artificial</t>
         </is>
       </c>
       <c r="E182" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/registraduria-le-respondio-a-petro-por-denuncia-en-5300-mesas-no-encontraron-irregularidades</t>
+          <t>https://www.elespectador.com/opinion/columnistas/manuel-drezner/sobre-mozart-y-la-inteligencia-artificial/</t>
         </is>
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="5" t="inlineStr">
-        <is>
-          <t>03/06/2026 11:45 a. m.</t>
-        </is>
-      </c>
+      <c r="A183" s="5" t="inlineStr"/>
       <c r="B183" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5236,26 +5216,22 @@
       </c>
       <c r="C183" s="5" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D183" s="6" t="inlineStr">
         <is>
-          <t>Leonardo Huerta, exfórmula de Claudia López, se une a la campaña de Abelardo de la Espriella</t>
+          <t>Más allá del voto en blanco</t>
         </is>
       </c>
       <c r="E183" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/poder/articulo/2026/6/leonardo-huerta-exformula-de-claudia-lopez-se-une-a-la-campana-de-abelardo-de-la-espriella</t>
+          <t>https://www.elespectador.com/opinion/columnistas/cristinacarrizosa/mas-alla-del-voto-en-blanco/</t>
         </is>
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="2" t="inlineStr">
-        <is>
-          <t>03/06/2026 11:00 a. m.</t>
-        </is>
-      </c>
+      <c r="A184" s="2" t="inlineStr"/>
       <c r="B184" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5263,26 +5239,22 @@
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D184" s="3" t="inlineStr">
         <is>
-          <t>Corte Suprema condenó a exgobernador Arauca</t>
+          <t>Los votos están ahí</t>
         </is>
       </c>
       <c r="E184" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/pais/articulo/2026/6/corte-suprema-condeno-a-exgobernador-arauca</t>
+          <t>https://www.elespectador.com/opinion/columnistas/javier-ortiz/los-votos-estan-ahi/</t>
         </is>
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="5" t="inlineStr">
-        <is>
-          <t>03/06/2026 10:45 a. m.</t>
-        </is>
-      </c>
+      <c r="A185" s="5" t="inlineStr"/>
       <c r="B185" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5290,26 +5262,22 @@
       </c>
       <c r="C185" s="5" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D185" s="6" t="inlineStr">
         <is>
-          <t>El documento de Petro sobre fraude proviene de la Registraduría, pero modificado por alguien externo</t>
+          <t>Líder del equipo digital de De la Espriella denunciado por violencia sexual</t>
         </is>
       </c>
       <c r="E185" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/poder/articulo/2026/6/el-documento-de-petro-sobre-fraude-proviene-de-la-registraduria-pero-modificado-por-alguien-externo</t>
+          <t>https://www.elespectador.com/opinion/columnistas/catalina-ruiz-navarro/lider-del-equipo-digital-de-de-la-espriella-denunciado-por-violencia-sexual/</t>
         </is>
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="2" t="inlineStr">
-        <is>
-          <t>03/06/2026 10:00 a. m.</t>
-        </is>
-      </c>
+      <c r="A186" s="2" t="inlineStr"/>
       <c r="B186" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5317,26 +5285,22 @@
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D186" s="3" t="inlineStr">
         <is>
-          <t>"No más cafés, más debates": Juan Daniel Oviedo evita apoyar a Iván Cepeda o a Abelardo de la Espriella</t>
+          <t>Gurropín, corrupto dictador venerado por la izquierda populista</t>
         </is>
       </c>
       <c r="E186" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/poder/articulo/2026/6/no-mas-cafes-mas-debates-juan-daniel-oviedo-evita-apoyar-a-ivan-cepeda-o-a-abelardo-de-la-espriella</t>
+          <t>https://www.elespectador.com/opinion/columnistas/mauricio-rubio/gurropin-corrupto-dictador-venerado-por-la-izquierda-populista/</t>
         </is>
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="5" t="inlineStr">
-        <is>
-          <t>03/06/2026 08:02 a. m.</t>
-        </is>
-      </c>
+      <c r="A187" s="5" t="inlineStr"/>
       <c r="B187" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5344,26 +5308,22 @@
       </c>
       <c r="C187" s="5" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D187" s="6" t="inlineStr">
         <is>
-          <t>Registraduría defiende la legalidad del proceso electoral frente a críticas de Gustavo Petro</t>
+          <t>Quiero hablar con las flores</t>
         </is>
       </c>
       <c r="E187" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/registraduria-defiende-la-legalidad-del-proceso-electoral-frente-a-criticas-de-gustavo-petro</t>
+          <t>https://www.elespectador.com/opinion/columnistas/juan-david-zuloaga-d-/quiero-hablar-con-las-flores/</t>
         </is>
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="2" t="inlineStr">
-        <is>
-          <t>03/06/2026 07:20 a. m.</t>
-        </is>
-      </c>
+      <c r="A188" s="2" t="inlineStr"/>
       <c r="B188" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5371,17 +5331,17 @@
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D188" s="3" t="inlineStr">
         <is>
-          <t>Minambiente anuncia plan de acción para el caimán llanero tras denuncias de meses sin alimentación y muertes</t>
+          <t>Atrapados entre la espada, la pared y la improvisación</t>
         </is>
       </c>
       <c r="E188" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/medio-ambiente/articulo/2026/6/minambiente-anuncia-plan-de-accion-para-el-caiman-llanero-tras-denuncias-de-meses-sin-alimentacion-y-muertes</t>
+          <t>https://www.elespectador.com/opinion/lectores/cartas/atrapados-entre-la-espada-la-pared-y-la-improvisacion/</t>
         </is>
       </c>
     </row>
@@ -5394,17 +5354,17 @@
       </c>
       <c r="C189" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D189" s="6" t="inlineStr">
         <is>
-          <t>Claudia López anunció que no votará por Iván Cepeda, calificó su campaña como “arrogante” y habló de “disonancia” entre el candidato y Gustavo Petro</t>
+          <t>Amazonas colombiano: qué hacer, cómo viajar y cuánto cuesta</t>
         </is>
       </c>
       <c r="E189" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/claudia-lopez-anuncio-que-no-votara-por-ivan-cepeda-califico-su-campana-como-arrogante-y-hablo-de-disonancia-entre-el-candidato-y-gustavo-petro/202642/</t>
+          <t>https://canaltrece.com.co/regiones/amazonas/amazonas-colombiano-que-hacer-como-viajar-y-cuanto-cuesta/</t>
         </is>
       </c>
     </row>
@@ -5417,17 +5377,17 @@
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D190" s="3" t="inlineStr">
         <is>
-          <t>Abelardo de la Espriella le responde al Partido Liberal y no acepta su respaldo: “Son apéndice de Petro y Cepeda”</t>
+          <t>Cómo saber si soy jurado de votación en 2026: paso a paso</t>
         </is>
       </c>
       <c r="E190" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/abelardo-de-la-espriella-le-responde-al-partido-liberal-y-no-acepta-su-respaldo-son-apendice-de-petro-y-cepeda/202631/</t>
+          <t>https://canaltrece.com.co/noticias/como-saber-si-soy-jurado-de-votacion-en-2026-paso-a-paso/</t>
         </is>
       </c>
     </row>
@@ -5440,17 +5400,17 @@
       </c>
       <c r="C191" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D191" s="6" t="inlineStr">
         <is>
-          <t>Desde EE. UU. le dan una mala noticia a Gustavo Petro a pocos meses de salir de la Casa de Nariño: “No lo van a quitar”</t>
+          <t>Pueblos de Cundinamarca cerca de Bogotá para un fin de semana</t>
         </is>
       </c>
       <c r="E191" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/mundo/articulo/desde-eeuu-le-dan-una-mala-noticia-a-gustavo-petro-a-pocos-meses-de-salir-de-la-casa-de-narino-no-lo-van-a-quitar/202600/</t>
+          <t>https://canaltrece.com.co/noticias/pueblos-de-cundinamarca-cerca-de-bogota-para-un-fin-de-semana/</t>
         </is>
       </c>
     </row>
@@ -5463,17 +5423,17 @@
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D192" s="3" t="inlineStr">
         <is>
-          <t>Alcalde Federico Gutiérrez hace duro pronunciamiento ante las protestas de encapuchados en la Universidad de Antioquia: “No son estudiantes”</t>
+          <t>¿Puedo cambiar mi puesto de votación para segunda vuelta?</t>
         </is>
       </c>
       <c r="E192" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/alcalde-federico-gutierrez-hace-duro-pronunciamiento-ante-las-protestas-de-encapuchados-en-la-universidad-de-antioquia-no-son-estudiantes/202654/</t>
+          <t>https://canaltrece.com.co/noticias/puedo-cambiar-mi-puesto-de-votacion-para-segunda-vuelta/</t>
         </is>
       </c>
     </row>
@@ -5486,17 +5446,17 @@
       </c>
       <c r="C193" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D193" s="6" t="inlineStr">
         <is>
-          <t>Video | Así fue la campaña de mentiras sobre Abelardo de la Espriella: “A los abuelos les decimos eso y caen”</t>
+          <t>Calendario de Colombia Mundial 2026: fechas, horarios y rivales</t>
         </is>
       </c>
       <c r="E193" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/video-asi-fue-la-campana-de-mentiras-sobre-abelardo-de-la-espriella-a-los-abuelos-les-decimos-eso-y-caen/202627/</t>
+          <t>https://canaltrece.com.co/noticias/calendario-de-colombia-mundial-2026-fechas-horarios-y-rivales/</t>
         </is>
       </c>
     </row>
@@ -5509,17 +5469,17 @@
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D194" s="3" t="inlineStr">
         <is>
-          <t>Fin a las especulaciones: SEMANA conoció la decisión de Armando Benedetti sobre su supuesta llegada a la campaña de Iván Cepeda</t>
+          <t>Día del Padre 2026 en Colombia: fecha y planes para celebrar</t>
         </is>
       </c>
       <c r="E194" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/fin-a-las-especulaciones-semana-conocio-la-decision-de-armando-benedetti-sobre-su-supuesta-llegada-a-la-campana-de-ivan-cepeda/202604/</t>
+          <t>https://canaltrece.com.co/noticias/dia-del-padre-2026-en-colombia-fecha-y-planes-para-celebrar/</t>
         </is>
       </c>
     </row>
@@ -5532,17 +5492,17 @@
       </c>
       <c r="C195" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D195" s="6" t="inlineStr">
         <is>
-          <t>Abelardo de la Espriella le hace una propuesta audaz a Elon Musk: “Una alianza de conectividad y que conozca a Colombia”</t>
+          <t>Dónde me toca votar en Colombia 2026: consulte su puesto</t>
         </is>
       </c>
       <c r="E195" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/confidenciales/articulo/abelardo-de-la-espriella-le-hace-una-propuesta-audaz-a-elon-musk-una-alianza-de-conectividad-y-que-conozca-a-colombia/202601/</t>
+          <t>https://canaltrece.com.co/noticias/donde-me-toca-votar-en-colombia-2026-consulte-su-puesto/</t>
         </is>
       </c>
     </row>
@@ -5555,17 +5515,17 @@
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D196" s="3" t="inlineStr">
         <is>
-          <t>“Amenazaron”: Gustavo Petro reaccionó a petición de congresistas de la Comisión de Acusación de llamarlo a indagatoria por irregularidades en su campaña</t>
+          <t>Dónde ver los partidos de Colombia en el Mundial 2026</t>
         </is>
       </c>
       <c r="E196" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/amenazaron-gustavo-petro-reacciono-a-peticion-de-congresistas-de-la-comision-de-acusacion-de-llamarlo-a-indagatoria-por-irregularidades-en-su-campana/202652/</t>
+          <t>https://canaltrece.com.co/noticias/donde-ver-los-partidos-de-colombia-en-el-mundial-2026/</t>
         </is>
       </c>
     </row>
@@ -5578,17 +5538,17 @@
       </c>
       <c r="C197" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D197" s="6" t="inlineStr">
         <is>
-          <t>Nuevo ataque del Ejército de EE. UU. a una narcolancha en el Pacífico deja 2 muertos</t>
+          <t>Día del Padre asado en casa: cómo elegir los mejores elementos para una celebración perfecta</t>
         </is>
       </c>
       <c r="E197" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/mundo/articulo/nuevo-ataque-del-ejercito-de-ee-uu-a-una-narcolancha-en-el-pacifico-deja-2-muertos/202624/</t>
+          <t>https://canaltrece.com.co/noticias/dia-del-padre-asado-en-casa-elementos-parrilla/</t>
         </is>
       </c>
     </row>
@@ -5601,17 +5561,17 @@
       </c>
       <c r="C198" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D198" s="3" t="inlineStr">
         <is>
-          <t>Sofía Petro sorprende a los empresarios y toma decisión para que voten por Iván Cepeda; Margarita Rosa no se quedó callada</t>
+          <t>Qué hacer en Villavicencio: planes, cultura, comida y naturaleza</t>
         </is>
       </c>
       <c r="E198" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/gente/articulo/sofia-petro-sorprende-a-los-empresarios-y-toma-decision-para-que-voten-por-ivan-cepeda-margarita-rosa-no-se-quedo-callada/202634/</t>
+          <t>https://canaltrece.com.co/regiones/meta/que-hacer-en-villavicencio-planes-cultura-comida-y-naturaleza/</t>
         </is>
       </c>
     </row>
@@ -5624,17 +5584,17 @@
       </c>
       <c r="C199" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D199" s="6" t="inlineStr">
         <is>
-          <t>Caso talio: los detalles de la audiencia clave en el proceso contra Zulma Guzmán</t>
+          <t>Festival Afro de Santa Fe 2026: música, gastronomía y cultura afro en el centro de Bogotá</t>
         </is>
       </c>
       <c r="E199" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/caso-talio-los-detalles-de-la-audiencia-clave-en-el-proceso-contra-zulma-guzman/202620/</t>
+          <t>https://canaltrece.com.co/editorial/festival-afro-de-santa-fe-2026-bogota/</t>
         </is>
       </c>
     </row>
@@ -5647,17 +5607,17 @@
       </c>
       <c r="C200" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D200" s="3" t="inlineStr">
         <is>
-          <t>Manifestantes se congregaron en inmediaciones de la Universidad Distrital, en el Tintal, para expresar su apoyo a Iván Cepeda</t>
+          <t>Feria Belleza y Bienestar Farmatodo 2026 regresa a Bogotá con más de 100 marcas y entrada gratuita</t>
         </is>
       </c>
       <c r="E200" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/bogota/articulo/manifestantes-se-toman-las-inmediaciones-de-la-universidad-distrital-en-el-tintal-para-expresar-su-apoyo-a-ivan-cepeda/202608/</t>
+          <t>https://canaltrece.com.co/noticias/feria-belleza-y-bienestar-farmatodo-2026-bogota/</t>
         </is>
       </c>
     </row>
@@ -5670,17 +5630,17 @@
       </c>
       <c r="C201" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D201" s="6" t="inlineStr">
         <is>
-          <t>José Manuel Restrepo invitó a debatir a Aída Quilcué en un ‘terreno neutral’: “la democracia se nutre en la discusión”</t>
+          <t>Conciertos en Colombia junio 2026: fechas, artistas y boletas</t>
         </is>
       </c>
       <c r="E201" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/jose-manuel-restrepo-invito-a-debatir-a-aida-quilcue-en-un-terreno-neutral-la-democracia-se-nutre-en-la-discusion/202609/</t>
+          <t>https://canaltrece.com.co/noticias/conciertos-en-colombia-junio-2026-fechas-artistas-y-boletas/</t>
         </is>
       </c>
     </row>
@@ -5693,17 +5653,17 @@
       </c>
       <c r="C202" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D202" s="3" t="inlineStr">
         <is>
-          <t>Aída Quilcué le abrió las puertas a Westcol: la candidata vicepresidencial aceptó invitación para transmitir en vivo desde territorio indígena</t>
+          <t>Alix y Bobby Sierra Agua: la canción que habla de amores imposibles y nostalgia</t>
         </is>
       </c>
       <c r="E202" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/aida-quilcue-le-abrio-las-puertas-a-westcol-candidata-vicepresidencial-acepto-invitacion-para-transmitir-en-vivo-desde-territorio-indigena/202610/</t>
+          <t>https://canaltrece.com.co/noticias/alix-y-bobby-sierra-agua/</t>
         </is>
       </c>
     </row>
@@ -5716,17 +5676,17 @@
       </c>
       <c r="C203" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D203" s="6" t="inlineStr">
         <is>
-          <t>Juan Daniel Oviedo habla de la segunda vuelta: “No soy un actor influyente para mover votos como si los votantes fueran cabezas de ganado”</t>
+          <t>Ritvales 2026 regresa a Medellín para celebrar más de una década de historia electrónica</t>
         </is>
       </c>
       <c r="E203" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/juan-daniel-oviedo-habla-de-la-segunda-vuelta-no-soy-un-actor-influyente-para-mover-votos-como-si-los-votantes-fueran-cabezas-de-ganado/202646/</t>
+          <t>https://canaltrece.com.co/noticias/ritvales-2026-medellin/</t>
         </is>
       </c>
     </row>
@@ -5739,17 +5699,17 @@
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D204" s="3" t="inlineStr">
         <is>
-          <t>🔴 Simulador del Mundial 2026 |Arme el fixture completo y defina a su campeón</t>
+          <t>Hamilton YouTube Foundry 2026: el colombiano elegido por YouTube</t>
         </is>
       </c>
       <c r="E204" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/especiales-multimedia/articulo/mundial-2026-el-simulador-con-el-que-usted-puede-jugar-y-atinar-hasta-que-haya-campeon/202529/</t>
+          <t>https://canaltrece.com.co/noticias/hamilton-youtube-foundry-2026/</t>
         </is>
       </c>
     </row>
@@ -5762,17 +5722,17 @@
       </c>
       <c r="C205" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D205" s="6" t="inlineStr">
         <is>
-          <t>Abelardo de la Espriella, con el 82 % de posibilidades de ganar la Presidencia, según Polymarket; Ivan Cepeda, con el 19 %</t>
+          <t>Planes memorables para celebrar a papá en su día: Opciones para todos los gustos</t>
         </is>
       </c>
       <c r="E205" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/abelardo-de-la-espriella-con-el-82-de-posibilidades-de-ganar-la-presidencia-segun-polymarket-ivan-cepeda-con-el-19/202629/</t>
+          <t>https://canaltrece.com.co/noticias/planes-memorables-para-celebrar-a-papa-en-su-dia-opciones-para-todos-los-gustos/</t>
         </is>
       </c>
     </row>
@@ -5785,17 +5745,17 @@
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D206" s="3" t="inlineStr">
         <is>
-          <t>“No tengo vida social”: Shakira habla de su realidad en la soltería y sus exigentes planes</t>
+          <t>¿Se adelanta el Día del Padre? Proponen mover la fecha en Colombia por las elecciones de segunda vuelta</t>
         </is>
       </c>
       <c r="E206" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/gente/articulo/no-tengo-vida-social-shakira-habla-de-su-realidad-en-la-solteria-y-sus-exigentes-planes/202624/</t>
+          <t>https://canaltrece.com.co/noticias/se-adelanta-el-dia-del-padre-proponen-mover-la-fecha-en-colombia-por-las-elecciones-de-segunda-vuelta/</t>
         </is>
       </c>
     </row>
@@ -5808,17 +5768,17 @@
       </c>
       <c r="C207" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D207" s="6" t="inlineStr">
         <is>
-          <t>Fechas y horarios para Independiente Medellín, Santa Fe y Tolima en la Copa Libertadores y Sudamericana</t>
+          <t>Trabajo sí hay: Bogotá ofrece más de 5.000 vacantes de empleo en Teatron este jueves</t>
         </is>
       </c>
       <c r="E207" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/fechas-y-horarios-para-independiente-medellin-santa-fe-y-tolima-en-la-copa-libertadores-y-sudamericana/202632/</t>
+          <t>https://canaltrece.com.co/noticias/trabajo-si-hay-bogota-ofrece-mas-de-5-000-vacantes-de-empleo-en-teatron-este-jueves/</t>
         </is>
       </c>
     </row>
@@ -5831,17 +5791,17 @@
       </c>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D208" s="3" t="inlineStr">
         <is>
-          <t>Rival de Colombia en el Mundial 2026 tiene serios problemas: está dispuesto a jugar a puerta cerrada</t>
+          <t>Alerta en Bogotá: Ojo con la nueva estafa de códigos QR en falsos comparendos</t>
         </is>
       </c>
       <c r="E208" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/rival-de-colombia-en-el-mundial-2026-tiene-serios-problemas-esta-dispuesto-a-jugar-a-puerta-cerrada/202650/</t>
+          <t>https://canaltrece.com.co/noticias/alerta-en-bogota-ojo-con-la-nueva-estafa-de-codigos-qr-en-falsos-comparendos/</t>
         </is>
       </c>
     </row>
@@ -5854,17 +5814,17 @@
       </c>
       <c r="C209" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D209" s="6" t="inlineStr">
         <is>
-          <t>RD Congo sorprende a Dinamarca y avisa a la Selección Colombia: no se escondió en amistoso</t>
+          <t>Bogotá celebra el Día Mundial de la Bicicleta en 2026 ratificándose como la Capital Mundial de la Bici</t>
         </is>
       </c>
       <c r="E209" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/rd-congo-sorprende-a-dinamarca-y-avisa-a-la-seleccion-colombia-no-se-escondio-en-amistoso/202640/</t>
+          <t>https://canaltrece.com.co/noticias/bogota-celebra-el-dia-mundial-de-la-bicicleta-en-2026-ratificandose-como-la-capital-mundial-de-la-bici/</t>
         </is>
       </c>
     </row>
@@ -5877,17 +5837,17 @@
       </c>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D210" s="3" t="inlineStr">
         <is>
-          <t>Usuarios de Roku, la aplicación se actualiza para el Mundial 2026, así se verán los partidos en Colombia</t>
+          <t>Aída Quilcué Vivas: La voz inquebrantable de la dignidad y la resistencia indígena en Colombia</t>
         </is>
       </c>
       <c r="E210" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/tecnologia/articulo/usuarios-de-roku-la-aplicacion-se-actualiza-para-el-mundial-2026-asi-se-veran-los-partidos-en-colombia/202604/</t>
+          <t>https://canaltrece.com.co/noticias/aida-quilcue-vivas-la-voz-inquebrantable-de-la-dignidad-y-la-resistencia-indigena-en-colombia/</t>
         </is>
       </c>
     </row>
@@ -5900,17 +5860,17 @@
       </c>
       <c r="C211" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D211" s="6" t="inlineStr">
         <is>
-          <t>¿Es ilegal? Lo que dice la ley sobre hacer una ‘polla’ del Mundial en la oficina</t>
+          <t>José Manuel Restrepo Abondano: El economista y educador que lidera la academia en Colombia</t>
         </is>
       </c>
       <c r="E211" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/economia/empresas/articulo/es-ilegal-lo-que-dice-la-ley-sobre-hacer-una-polla-del-mundial-en-la-oficina/202639/</t>
+          <t>https://canaltrece.com.co/noticias/jose-manuel-restrepo-abondano-el-economista-y-educador-que-lidera-la-academia-en-colombia/</t>
         </is>
       </c>
     </row>
@@ -5923,17 +5883,17 @@
       </c>
       <c r="C212" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D212" s="3" t="inlineStr">
         <is>
-          <t>Miércoles negro para Petro en la Comisión de Acusación: radican solicitud para investigarlo formalmente por su campaña; piden llamarlo a indagatoria</t>
+          <t>Del diseño al arte: El realismo se consolida como la tendencia de tatuaje más importante de 2026</t>
         </is>
       </c>
       <c r="E212" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/miercoles-negro-para-petro-en-la-comision-de-acusacion-radicada-solicitud-de-investigarlo-formalmente-por-su-campana-piden-llamarlo-a-indagatoria/202625/</t>
+          <t>https://canaltrece.com.co/noticias/del-diseno-al-arte-el-realismo-se-consolida-como-la-tendencia-de-tatuaje-mas-importante-de-2026/</t>
         </is>
       </c>
     </row>
@@ -5946,17 +5906,17 @@
       </c>
       <c r="C213" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D213" s="6" t="inlineStr">
         <is>
-          <t>Gustavo Petro choca con Abelardo de la Espriella por el aumento del salario mínimo y destapó el verdadero “problema”</t>
+          <t>Lactancia y autonomía: Cómo la tecnología wearable le devuelve el tiempo a las madres</t>
         </is>
       </c>
       <c r="E213" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/gustavo-petro-choca-con-abelardo-de-la-espriella-por-el-aumento-del-salario-minimo-y-destapo-el-verdadero-problema/202619/</t>
+          <t>https://canaltrece.com.co/noticias/lactancia-y-autonomia-como-la-tecnologia-wearable-le-devuelve-el-tiempo-a-las-madres/</t>
         </is>
       </c>
     </row>
@@ -5969,17 +5929,17 @@
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D214" s="3" t="inlineStr">
         <is>
-          <t>A Iván Cepeda no le gustó el apoyo de Donald Trump a Abelardo de la Espriella y aseguró que hay un “tinte injerencista”</t>
+          <t>Fraude digital en Colombia: 1 de cada 3 personas ha sido víctima, según expertos</t>
         </is>
       </c>
       <c r="E214" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/a-ivan-cepeda-no-le-gusto-el-apoyo-de-donald-trump-a-abelardo-de-la-espriella-y-aseguro-que-hay-un-tinte-injerencista/202606/</t>
+          <t>https://canaltrece.com.co/noticias/fraude-digital-en-colombia-victimas-suplantacion-identidad/</t>
         </is>
       </c>
     </row>
@@ -5992,17 +5952,17 @@
       </c>
       <c r="C215" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D215" s="6" t="inlineStr">
         <is>
-          <t>Wilson Ruiz pidió medidas cautelares para que se prohíba a Gustavo Petro emitir mensajes a favor del candidato Iván Cepeda</t>
+          <t>Juan Valdez y James Rodríguez lanzan edición especial de café inspirada en el fútbol</t>
         </is>
       </c>
       <c r="E215" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/wilson-ruiz-pidio-medidas-cautelares-para-que-se-prohiba-a-gustavo-petro-emitir-mensajes-a-favor-del-candidato-ivan-cepeda/202633/</t>
+          <t>https://canaltrece.com.co/noticias/juan-valdez-y-james-rodriguez-edicion-especial-cafe/</t>
         </is>
       </c>
     </row>
@@ -6015,17 +5975,17 @@
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D216" s="3" t="inlineStr">
         <is>
-          <t>Misterioso hallazgo en el locker de Zulma Guzmán en exclusivo club social desata nuevas preguntas en el caso</t>
+          <t>Fito Páez regresa a Colombia con Sale el Sol y celebra los 40 años de Giros</t>
         </is>
       </c>
       <c r="E216" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/misterioso-hallazgo-en-el-locker-de-zulma-guzman-en-exclusivo-club-social-desata-nuevas-preguntas-en-el-caso/202639/</t>
+          <t>https://canaltrece.com.co/noticias/fito-paez-regresa-a-colombia-sale-el-sol-gira-2026/</t>
         </is>
       </c>
     </row>
@@ -6038,17 +5998,17 @@
       </c>
       <c r="C217" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D217" s="6" t="inlineStr">
         <is>
-          <t>Golpe millonario al ELN: destruyen megalaboratorio capaz de producir dos toneladas de cocaína al mes</t>
+          <t>Natalia Bedoya Romance Teatro Santander: el concierto que llega a Bucaramanga</t>
         </is>
       </c>
       <c r="E217" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/golpe-millonario-al-eln-destruyen-megalaboratorio-capaz-de-producir-dos-toneladas-de-cocaina-al-mes/202624/</t>
+          <t>https://canaltrece.com.co/noticias/natalia-bedoya-romance-teatro-santander/</t>
         </is>
       </c>
     </row>
@@ -6061,17 +6021,17 @@
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D218" s="3" t="inlineStr">
         <is>
-          <t>Estudiantes protagonizaron marchas en Bogotá en rechazo a los resultados de la primera vuelta presidencial</t>
+          <t>Dago García Creatividad y Escritura: el libro que revela cómo nacen las grandes historias</t>
         </is>
       </c>
       <c r="E218" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/bogota/articulo/estudiantes-protagonizaron-marchas-en-bogota-en-rechazo-a-los-resultados-de-la-primera-vuelta-presidencial/202610/</t>
+          <t>https://canaltrece.com.co/noticias/dago-garcia-creatividad-y-escritura/</t>
         </is>
       </c>
     </row>
@@ -6084,17 +6044,17 @@
       </c>
       <c r="C219" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D219" s="6" t="inlineStr">
         <is>
-          <t>Amazonas colombiano: qué hacer, cómo viajar y cuánto cuesta</t>
+          <t>Claudia López anunció que no votará por Iván Cepeda, calificó su campaña como “arrogante” y habló de “disonancia” entre el candidato y Gustavo Petro</t>
         </is>
       </c>
       <c r="E219" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/regiones/amazonas/amazonas-colombiano-que-hacer-como-viajar-y-cuanto-cuesta/</t>
+          <t>https://www.semana.com/politica/articulo/claudia-lopez-anuncio-que-no-votara-por-ivan-cepeda-califico-su-campana-como-arrogante-y-hablo-de-disonancia-entre-el-candidato-y-gustavo-petro/202642/</t>
         </is>
       </c>
     </row>
@@ -6107,17 +6067,17 @@
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D220" s="3" t="inlineStr">
         <is>
-          <t>Cómo saber si soy jurado de votación en 2026: paso a paso</t>
+          <t>Abelardo de la Espriella le responde al Partido Liberal y no acepta su respaldo: “Son apéndice de Petro y Cepeda”</t>
         </is>
       </c>
       <c r="E220" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/como-saber-si-soy-jurado-de-votacion-en-2026-paso-a-paso/</t>
+          <t>https://www.semana.com/politica/articulo/abelardo-de-la-espriella-le-responde-al-partido-liberal-y-no-acepta-su-respaldo-son-apendice-de-petro-y-cepeda/202631/</t>
         </is>
       </c>
     </row>
@@ -6130,17 +6090,17 @@
       </c>
       <c r="C221" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D221" s="6" t="inlineStr">
         <is>
-          <t>Pueblos de Cundinamarca cerca de Bogotá para un fin de semana</t>
+          <t>Desde EE. UU. le dan una mala noticia a Gustavo Petro a pocos meses de salir de la Casa de Nariño: “No lo van a quitar”</t>
         </is>
       </c>
       <c r="E221" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/pueblos-de-cundinamarca-cerca-de-bogota-para-un-fin-de-semana/</t>
+          <t>https://www.semana.com/mundo/articulo/desde-eeuu-le-dan-una-mala-noticia-a-gustavo-petro-a-pocos-meses-de-salir-de-la-casa-de-narino-no-lo-van-a-quitar/202600/</t>
         </is>
       </c>
     </row>
@@ -6153,17 +6113,17 @@
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D222" s="3" t="inlineStr">
         <is>
-          <t>¿Puedo cambiar mi puesto de votación para segunda vuelta?</t>
+          <t>Alcalde Federico Gutiérrez hace duro pronunciamiento ante las protestas de encapuchados en la Universidad de Antioquia: “No son estudiantes”</t>
         </is>
       </c>
       <c r="E222" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/puedo-cambiar-mi-puesto-de-votacion-para-segunda-vuelta/</t>
+          <t>https://www.semana.com/nacion/articulo/alcalde-federico-gutierrez-hace-duro-pronunciamiento-ante-las-protestas-de-encapuchados-en-la-universidad-de-antioquia-no-son-estudiantes/202654/</t>
         </is>
       </c>
     </row>
@@ -6176,17 +6136,17 @@
       </c>
       <c r="C223" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D223" s="6" t="inlineStr">
         <is>
-          <t>Calendario de Colombia Mundial 2026: fechas, horarios y rivales</t>
+          <t>Video | Así fue la campaña de mentiras sobre Abelardo de la Espriella: “A los abuelos les decimos eso y caen”</t>
         </is>
       </c>
       <c r="E223" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/calendario-de-colombia-mundial-2026-fechas-horarios-y-rivales/</t>
+          <t>https://www.semana.com/politica/articulo/video-asi-fue-la-campana-de-mentiras-sobre-abelardo-de-la-espriella-a-los-abuelos-les-decimos-eso-y-caen/202627/</t>
         </is>
       </c>
     </row>
@@ -6199,17 +6159,17 @@
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D224" s="3" t="inlineStr">
         <is>
-          <t>Día del Padre 2026 en Colombia: fecha y planes para celebrar</t>
+          <t>Fin a las especulaciones: SEMANA conoció la decisión de Armando Benedetti sobre su supuesta llegada a la campaña de Iván Cepeda</t>
         </is>
       </c>
       <c r="E224" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/dia-del-padre-2026-en-colombia-fecha-y-planes-para-celebrar/</t>
+          <t>https://www.semana.com/politica/articulo/fin-a-las-especulaciones-semana-conocio-la-decision-de-armando-benedetti-sobre-su-supuesta-llegada-a-la-campana-de-ivan-cepeda/202604/</t>
         </is>
       </c>
     </row>
@@ -6222,17 +6182,17 @@
       </c>
       <c r="C225" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D225" s="6" t="inlineStr">
         <is>
-          <t>Dónde me toca votar en Colombia 2026: consulte su puesto</t>
+          <t>Abelardo de la Espriella le hace una propuesta audaz a Elon Musk: “Una alianza de conectividad y que conozca a Colombia”</t>
         </is>
       </c>
       <c r="E225" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/donde-me-toca-votar-en-colombia-2026-consulte-su-puesto/</t>
+          <t>https://www.semana.com/confidenciales/articulo/abelardo-de-la-espriella-le-hace-una-propuesta-audaz-a-elon-musk-una-alianza-de-conectividad-y-que-conozca-a-colombia/202601/</t>
         </is>
       </c>
     </row>
@@ -6245,17 +6205,17 @@
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D226" s="3" t="inlineStr">
         <is>
-          <t>Dónde ver los partidos de Colombia en el Mundial 2026</t>
+          <t>“Amenazaron”: Gustavo Petro reaccionó a petición de congresistas de la Comisión de Acusación de llamarlo a indagatoria por irregularidades en su campaña</t>
         </is>
       </c>
       <c r="E226" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/donde-ver-los-partidos-de-colombia-en-el-mundial-2026/</t>
+          <t>https://www.semana.com/politica/articulo/amenazaron-gustavo-petro-reacciono-a-peticion-de-congresistas-de-la-comision-de-acusacion-de-llamarlo-a-indagatoria-por-irregularidades-en-su-campana/202652/</t>
         </is>
       </c>
     </row>
@@ -6268,17 +6228,17 @@
       </c>
       <c r="C227" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D227" s="6" t="inlineStr">
         <is>
-          <t>Día del Padre asado en casa: cómo elegir los mejores elementos para una celebración perfecta</t>
+          <t>Nuevo ataque del Ejército de EE. UU. a una narcolancha en el Pacífico deja 2 muertos</t>
         </is>
       </c>
       <c r="E227" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/dia-del-padre-asado-en-casa-elementos-parrilla/</t>
+          <t>https://www.semana.com/mundo/articulo/nuevo-ataque-del-ejercito-de-ee-uu-a-una-narcolancha-en-el-pacifico-deja-2-muertos/202624/</t>
         </is>
       </c>
     </row>
@@ -6291,17 +6251,17 @@
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D228" s="3" t="inlineStr">
         <is>
-          <t>Qué hacer en Villavicencio: planes, cultura, comida y naturaleza</t>
+          <t>Sofía Petro sorprende a los empresarios y toma decisión para que voten por Iván Cepeda; Margarita Rosa no se quedó callada</t>
         </is>
       </c>
       <c r="E228" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/regiones/meta/que-hacer-en-villavicencio-planes-cultura-comida-y-naturaleza/</t>
+          <t>https://www.semana.com/gente/articulo/sofia-petro-sorprende-a-los-empresarios-y-toma-decision-para-que-voten-por-ivan-cepeda-margarita-rosa-no-se-quedo-callada/202634/</t>
         </is>
       </c>
     </row>
@@ -6314,17 +6274,17 @@
       </c>
       <c r="C229" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D229" s="6" t="inlineStr">
         <is>
-          <t>Festival Afro de Santa Fe 2026: música, gastronomía y cultura afro en el centro de Bogotá</t>
+          <t>Caso talio: los detalles de la audiencia clave en el proceso contra Zulma Guzmán</t>
         </is>
       </c>
       <c r="E229" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/editorial/festival-afro-de-santa-fe-2026-bogota/</t>
+          <t>https://www.semana.com/nacion/articulo/caso-talio-los-detalles-de-la-audiencia-clave-en-el-proceso-contra-zulma-guzman/202620/</t>
         </is>
       </c>
     </row>
@@ -6337,17 +6297,17 @@
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D230" s="3" t="inlineStr">
         <is>
-          <t>Feria Belleza y Bienestar Farmatodo 2026 regresa a Bogotá con más de 100 marcas y entrada gratuita</t>
+          <t>Manifestantes se congregaron en inmediaciones de la Universidad Distrital, en el Tintal, para expresar su apoyo a Iván Cepeda</t>
         </is>
       </c>
       <c r="E230" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/feria-belleza-y-bienestar-farmatodo-2026-bogota/</t>
+          <t>https://www.semana.com/nacion/bogota/articulo/manifestantes-se-toman-las-inmediaciones-de-la-universidad-distrital-en-el-tintal-para-expresar-su-apoyo-a-ivan-cepeda/202608/</t>
         </is>
       </c>
     </row>
@@ -6360,17 +6320,17 @@
       </c>
       <c r="C231" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D231" s="6" t="inlineStr">
         <is>
-          <t>Conciertos en Colombia junio 2026: fechas, artistas y boletas</t>
+          <t>José Manuel Restrepo invitó a debatir a Aída Quilcué en un ‘terreno neutral’: “la democracia se nutre en la discusión”</t>
         </is>
       </c>
       <c r="E231" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/conciertos-en-colombia-junio-2026-fechas-artistas-y-boletas/</t>
+          <t>https://www.semana.com/politica/articulo/jose-manuel-restrepo-invito-a-debatir-a-aida-quilcue-en-un-terreno-neutral-la-democracia-se-nutre-en-la-discusion/202609/</t>
         </is>
       </c>
     </row>
@@ -6383,17 +6343,17 @@
       </c>
       <c r="C232" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D232" s="3" t="inlineStr">
         <is>
-          <t>Alix y Bobby Sierra Agua: la canción que habla de amores imposibles y nostalgia</t>
+          <t>Aída Quilcué le abrió las puertas a Westcol: la candidata vicepresidencial aceptó invitación para transmitir en vivo desde territorio indígena</t>
         </is>
       </c>
       <c r="E232" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/alix-y-bobby-sierra-agua/</t>
+          <t>https://www.semana.com/politica/articulo/aida-quilcue-le-abrio-las-puertas-a-westcol-candidata-vicepresidencial-acepto-invitacion-para-transmitir-en-vivo-desde-territorio-indigena/202610/</t>
         </is>
       </c>
     </row>
@@ -6406,17 +6366,17 @@
       </c>
       <c r="C233" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D233" s="6" t="inlineStr">
         <is>
-          <t>Ritvales 2026 regresa a Medellín para celebrar más de una década de historia electrónica</t>
+          <t>Juan Daniel Oviedo habla de la segunda vuelta: “No soy un actor influyente para mover votos como si los votantes fueran cabezas de ganado”</t>
         </is>
       </c>
       <c r="E233" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/ritvales-2026-medellin/</t>
+          <t>https://www.semana.com/politica/articulo/juan-daniel-oviedo-habla-de-la-segunda-vuelta-no-soy-un-actor-influyente-para-mover-votos-como-si-los-votantes-fueran-cabezas-de-ganado/202646/</t>
         </is>
       </c>
     </row>
@@ -6429,17 +6389,17 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D234" s="3" t="inlineStr">
         <is>
-          <t>Hamilton YouTube Foundry 2026: el colombiano elegido por YouTube</t>
+          <t>🔴 Simulador del Mundial 2026 |Arme el fixture completo y defina a su campeón</t>
         </is>
       </c>
       <c r="E234" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/hamilton-youtube-foundry-2026/</t>
+          <t>https://www.semana.com/deportes/especiales-multimedia/articulo/mundial-2026-el-simulador-con-el-que-usted-puede-jugar-y-atinar-hasta-que-haya-campeon/202529/</t>
         </is>
       </c>
     </row>
@@ -6452,17 +6412,17 @@
       </c>
       <c r="C235" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D235" s="6" t="inlineStr">
         <is>
-          <t>Planes memorables para celebrar a papá en su día: Opciones para todos los gustos</t>
+          <t>Abelardo de la Espriella, con el 82 % de posibilidades de ganar la Presidencia, según Polymarket; Ivan Cepeda, con el 19 %</t>
         </is>
       </c>
       <c r="E235" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/planes-memorables-para-celebrar-a-papa-en-su-dia-opciones-para-todos-los-gustos/</t>
+          <t>https://www.semana.com/politica/articulo/abelardo-de-la-espriella-con-el-82-de-posibilidades-de-ganar-la-presidencia-segun-polymarket-ivan-cepeda-con-el-19/202629/</t>
         </is>
       </c>
     </row>
@@ -6475,17 +6435,17 @@
       </c>
       <c r="C236" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D236" s="3" t="inlineStr">
         <is>
-          <t>¿Se adelanta el Día del Padre? Proponen mover la fecha en Colombia por las elecciones de segunda vuelta</t>
+          <t>“No tengo vida social”: Shakira habla de su realidad en la soltería y sus exigentes planes</t>
         </is>
       </c>
       <c r="E236" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/se-adelanta-el-dia-del-padre-proponen-mover-la-fecha-en-colombia-por-las-elecciones-de-segunda-vuelta/</t>
+          <t>https://www.semana.com/gente/articulo/no-tengo-vida-social-shakira-habla-de-su-realidad-en-la-solteria-y-sus-exigentes-planes/202624/</t>
         </is>
       </c>
     </row>
@@ -6498,17 +6458,17 @@
       </c>
       <c r="C237" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D237" s="6" t="inlineStr">
         <is>
-          <t>Trabajo sí hay: Bogotá ofrece más de 5.000 vacantes de empleo en Teatron este jueves</t>
+          <t>Fechas y horarios para Independiente Medellín, Santa Fe y Tolima en la Copa Libertadores y Sudamericana</t>
         </is>
       </c>
       <c r="E237" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/trabajo-si-hay-bogota-ofrece-mas-de-5-000-vacantes-de-empleo-en-teatron-este-jueves/</t>
+          <t>https://www.semana.com/deportes/articulo/fechas-y-horarios-para-independiente-medellin-santa-fe-y-tolima-en-la-copa-libertadores-y-sudamericana/202632/</t>
         </is>
       </c>
     </row>
@@ -6521,17 +6481,17 @@
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D238" s="3" t="inlineStr">
         <is>
-          <t>Alerta en Bogotá: Ojo con la nueva estafa de códigos QR en falsos comparendos</t>
+          <t>Rival de Colombia en el Mundial 2026 tiene serios problemas: está dispuesto a jugar a puerta cerrada</t>
         </is>
       </c>
       <c r="E238" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/alerta-en-bogota-ojo-con-la-nueva-estafa-de-codigos-qr-en-falsos-comparendos/</t>
+          <t>https://www.semana.com/deportes/articulo/rival-de-colombia-en-el-mundial-2026-tiene-serios-problemas-esta-dispuesto-a-jugar-a-puerta-cerrada/202650/</t>
         </is>
       </c>
     </row>
@@ -6544,17 +6504,17 @@
       </c>
       <c r="C239" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D239" s="6" t="inlineStr">
         <is>
-          <t>Bogotá celebra el Día Mundial de la Bicicleta en 2026 ratificándose como la Capital Mundial de la Bici</t>
+          <t>RD Congo sorprende a Dinamarca y avisa a la Selección Colombia: no se escondió en amistoso</t>
         </is>
       </c>
       <c r="E239" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/bogota-celebra-el-dia-mundial-de-la-bicicleta-en-2026-ratificandose-como-la-capital-mundial-de-la-bici/</t>
+          <t>https://www.semana.com/deportes/articulo/rd-congo-sorprende-a-dinamarca-y-avisa-a-la-seleccion-colombia-no-se-escondio-en-amistoso/202640/</t>
         </is>
       </c>
     </row>
@@ -6567,17 +6527,17 @@
       </c>
       <c r="C240" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D240" s="3" t="inlineStr">
         <is>
-          <t>Aída Quilcué Vivas: La voz inquebrantable de la dignidad y la resistencia indígena en Colombia</t>
+          <t>Usuarios de Roku, la aplicación se actualiza para el Mundial 2026, así se verán los partidos en Colombia</t>
         </is>
       </c>
       <c r="E240" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/aida-quilcue-vivas-la-voz-inquebrantable-de-la-dignidad-y-la-resistencia-indigena-en-colombia/</t>
+          <t>https://www.semana.com/tecnologia/articulo/usuarios-de-roku-la-aplicacion-se-actualiza-para-el-mundial-2026-asi-se-veran-los-partidos-en-colombia/202604/</t>
         </is>
       </c>
     </row>
@@ -6590,17 +6550,17 @@
       </c>
       <c r="C241" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D241" s="6" t="inlineStr">
         <is>
-          <t>José Manuel Restrepo Abondano: El economista y educador que lidera la academia en Colombia</t>
+          <t>¿Es ilegal? Lo que dice la ley sobre hacer una ‘polla’ del Mundial en la oficina</t>
         </is>
       </c>
       <c r="E241" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/jose-manuel-restrepo-abondano-el-economista-y-educador-que-lidera-la-academia-en-colombia/</t>
+          <t>https://www.semana.com/economia/empresas/articulo/es-ilegal-lo-que-dice-la-ley-sobre-hacer-una-polla-del-mundial-en-la-oficina/202639/</t>
         </is>
       </c>
     </row>
@@ -6613,17 +6573,17 @@
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D242" s="3" t="inlineStr">
         <is>
-          <t>Del diseño al arte: El realismo se consolida como la tendencia de tatuaje más importante de 2026</t>
+          <t>Miércoles negro para Petro en la Comisión de Acusación: radican solicitud para investigarlo formalmente por su campaña; piden llamarlo a indagatoria</t>
         </is>
       </c>
       <c r="E242" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/del-diseno-al-arte-el-realismo-se-consolida-como-la-tendencia-de-tatuaje-mas-importante-de-2026/</t>
+          <t>https://www.semana.com/politica/articulo/miercoles-negro-para-petro-en-la-comision-de-acusacion-radicada-solicitud-de-investigarlo-formalmente-por-su-campana-piden-llamarlo-a-indagatoria/202625/</t>
         </is>
       </c>
     </row>
@@ -6636,17 +6596,17 @@
       </c>
       <c r="C243" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D243" s="6" t="inlineStr">
         <is>
-          <t>Lactancia y autonomía: Cómo la tecnología wearable le devuelve el tiempo a las madres</t>
+          <t>Gustavo Petro choca con Abelardo de la Espriella por el aumento del salario mínimo y destapó el verdadero “problema”</t>
         </is>
       </c>
       <c r="E243" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/lactancia-y-autonomia-como-la-tecnologia-wearable-le-devuelve-el-tiempo-a-las-madres/</t>
+          <t>https://www.semana.com/politica/articulo/gustavo-petro-choca-con-abelardo-de-la-espriella-por-el-aumento-del-salario-minimo-y-destapo-el-verdadero-problema/202619/</t>
         </is>
       </c>
     </row>
@@ -6659,17 +6619,17 @@
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D244" s="3" t="inlineStr">
         <is>
-          <t>Fraude digital en Colombia: 1 de cada 3 personas ha sido víctima, según expertos</t>
+          <t>A Iván Cepeda no le gustó el apoyo de Donald Trump a Abelardo de la Espriella y aseguró que hay un “tinte injerencista”</t>
         </is>
       </c>
       <c r="E244" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/fraude-digital-en-colombia-victimas-suplantacion-identidad/</t>
+          <t>https://www.semana.com/politica/articulo/a-ivan-cepeda-no-le-gusto-el-apoyo-de-donald-trump-a-abelardo-de-la-espriella-y-aseguro-que-hay-un-tinte-injerencista/202606/</t>
         </is>
       </c>
     </row>
@@ -6682,17 +6642,17 @@
       </c>
       <c r="C245" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D245" s="6" t="inlineStr">
         <is>
-          <t>Juan Valdez y James Rodríguez lanzan edición especial de café inspirada en el fútbol</t>
+          <t>Wilson Ruiz pidió medidas cautelares para que se prohíba a Gustavo Petro emitir mensajes a favor del candidato Iván Cepeda</t>
         </is>
       </c>
       <c r="E245" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/juan-valdez-y-james-rodriguez-edicion-especial-cafe/</t>
+          <t>https://www.semana.com/politica/articulo/wilson-ruiz-pidio-medidas-cautelares-para-que-se-prohiba-a-gustavo-petro-emitir-mensajes-a-favor-del-candidato-ivan-cepeda/202633/</t>
         </is>
       </c>
     </row>
@@ -6705,17 +6665,17 @@
       </c>
       <c r="C246" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D246" s="3" t="inlineStr">
         <is>
-          <t>Fito Páez regresa a Colombia con Sale el Sol y celebra los 40 años de Giros</t>
+          <t>Misterioso hallazgo en el locker de Zulma Guzmán en exclusivo club social desata nuevas preguntas en el caso</t>
         </is>
       </c>
       <c r="E246" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/fito-paez-regresa-a-colombia-sale-el-sol-gira-2026/</t>
+          <t>https://www.semana.com/nacion/articulo/misterioso-hallazgo-en-el-locker-de-zulma-guzman-en-exclusivo-club-social-desata-nuevas-preguntas-en-el-caso/202639/</t>
         </is>
       </c>
     </row>
@@ -6728,17 +6688,17 @@
       </c>
       <c r="C247" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D247" s="6" t="inlineStr">
         <is>
-          <t>Natalia Bedoya Romance Teatro Santander: el concierto que llega a Bucaramanga</t>
+          <t>Golpe millonario al ELN: destruyen megalaboratorio capaz de producir dos toneladas de cocaína al mes</t>
         </is>
       </c>
       <c r="E247" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/natalia-bedoya-romance-teatro-santander/</t>
+          <t>https://www.semana.com/nacion/articulo/golpe-millonario-al-eln-destruyen-megalaboratorio-capaz-de-producir-dos-toneladas-de-cocaina-al-mes/202624/</t>
         </is>
       </c>
     </row>
@@ -6751,17 +6711,17 @@
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D248" s="3" t="inlineStr">
         <is>
-          <t>Dago García Creatividad y Escritura: el libro que revela cómo nacen las grandes historias</t>
+          <t>Estudiantes protagonizaron marchas en Bogotá en rechazo a los resultados de la primera vuelta presidencial</t>
         </is>
       </c>
       <c r="E248" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/dago-garcia-creatividad-y-escritura/</t>
+          <t>https://www.semana.com/nacion/bogota/articulo/estudiantes-protagonizaron-marchas-en-bogota-en-rechazo-a-los-resultados-de-la-primera-vuelta-presidencial/202610/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 Noticias actualizadas 05/06/2026 09:16
</commit_message>
<xml_diff>
--- a/docs/ultimahora.xlsx
+++ b/docs/ultimahora.xlsx
@@ -529,7 +529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>05/06/2026 02:30 a. m.</t>
+          <t>05/06/2026 04:05 a. m.</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -544,19 +544,19 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>¡Atención conductores! Pico y placa en Medellín para el viernes 5 de junio de 2026: así funcionará la medida</t>
+          <t>Los diez mandamientos de la parrilla, según el argentino Emiliano Yulita, chef de uno de los templos para comer carne en Buenos Aires</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/medellin/atencion-conductores-pico-y-placa-en-medellin-para-el-viernes-5-de-junio-de-2026-asi-funcionara-la-medida-3562151</t>
+          <t>https://www.eltiempo.com/cultura/gastronomia/los-diez-mandamientos-de-la-parrilla-segun-el-argentino-emiliano-yulita-chef-de-uno-de-los-templos-para-comer-carne-en-buenos-aires-3562227</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>05/06/2026 02:30 a. m.</t>
+          <t>05/06/2026 04:01 a. m.</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -571,19 +571,19 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>¡Evite sanciones! Pico y placa en Bucaramanga para el viernes 5 de junio de 2026: consulte las restricciones</t>
+          <t>Movilidad en Bogotá viernes 05 de junio: conozca acá el pico y placa en la ciudad</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/santander/evite-sanciones-pico-y-placa-en-bucaramanga-para-el-viernes-5-de-junio-de-2026-consulte-las-restricciones-3562147</t>
+          <t>https://www.eltiempo.com/bogota/movilidad-en-bogota-viernes-05-de-junio-conozca-aca-el-pico-y-placa-en-la-ciudad-3562274</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>05/06/2026 02:30 a. m.</t>
+          <t>05/06/2026 03:25 a. m.</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -598,19 +598,19 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>¡Ojo, conductores! Pico y placa en Pereira para el viernes 5 de junio de 2026: consulte las restricciones</t>
+          <t>¿Qué pasa si su certificado electoral no tiene la firma del jurado? La Registraduría Nacional del Estado Civil respondió</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/otras-ciudades/ojo-conductores-pico-y-placa-en-pereira-para-el-viernes-5-de-junio-de-2026-consulte-las-restricciones-3562145</t>
+          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/que-pasa-si-su-certificado-electoral-no-tiene-la-firma-del-jurado-la-registraduria-nacional-del-estado-civil-respondio-3562279</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>05/06/2026 02:30 a. m.</t>
+          <t>05/06/2026 02:37 a. m.</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -625,12 +625,12 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>¡Ojo, conductor! Pico y placa en Cali para el viernes 5 de junio de 2026: consulte las restricciones</t>
+          <t>Fito Páez, una de las 'joyas' del rock en español, se alista para empezar en Cali su gira de conciertos 'Sale el sol'</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/cali/ojo-conductor-pico-y-placa-en-cali-para-el-viernes-5-de-junio-de-2026-consulte-las-restricciones-3562140</t>
+          <t>https://www.eltiempo.com/colombia/cali/fito-paez-una-de-las-joyas-del-rock-en-espanol-se-alista-para-empezar-en-cali-su-gira-de-conciertos-sale-el-sol-3562278</t>
         </is>
       </c>
     </row>
@@ -652,19 +652,19 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>¡Atención conductores! Pico y placa en Bogotá para el viernes 5 de junio de 2026: así funcionará la medida</t>
+          <t>¡Atención conductores! Pico y placa en Medellín para el viernes 5 de junio de 2026: así funcionará la medida</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/bogota/atencion-conductores-pico-y-placa-en-bogota-para-el-viernes-5-de-junio-de-2026-asi-funcionara-la-medida-3562139</t>
+          <t>https://www.eltiempo.com/colombia/medellin/atencion-conductores-pico-y-placa-en-medellin-para-el-viernes-5-de-junio-de-2026-asi-funcionara-la-medida-3562151</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>05/06/2026 12:58 a. m.</t>
+          <t>05/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -679,19 +679,19 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Gobierno cambió las reglas de seguridad para expresidentes y exvicepresidentes: incluyó a la Dirección Nacional de Inteligencia</t>
+          <t>¡Evite sanciones! Pico y placa en Bucaramanga para el viernes 5 de junio de 2026: consulte las restricciones</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/politica/gobierno/gobierno-cambio-las-reglas-de-seguridad-para-expresidentes-y-exvicepresidentes-incluyo-a-la-direccion-nacional-de-inteligencia-3562273</t>
+          <t>https://www.eltiempo.com/colombia/santander/evite-sanciones-pico-y-placa-en-bucaramanga-para-el-viernes-5-de-junio-de-2026-consulte-las-restricciones-3562147</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>05/06/2026 12:15 a. m.</t>
+          <t>05/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -706,19 +706,19 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Senador de origen colombiano abre una batalla contra Trump por la ‘green card’: ¿podrá detener la medida que preocupa a millones de inmigrantes?</t>
+          <t>¡Ojo, conductores! Pico y placa en Pereira para el viernes 5 de junio de 2026: consulte las restricciones</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/senador-de-origen-colombiano-abre-una-batalla-contra-trump-por-la-green-card-podra-detener-la-medida-que-preocupa-a-millones-de-inmigrantes-3562054</t>
+          <t>https://www.eltiempo.com/colombia/otras-ciudades/ojo-conductores-pico-y-placa-en-pereira-para-el-viernes-5-de-junio-de-2026-consulte-las-restricciones-3562145</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>05/06/2026 12:14 a. m.</t>
+          <t>05/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -733,19 +733,19 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>La elección más tensa de los últimos años: lo que viene para Colombia</t>
+          <t>¡Ojo, conductor! Pico y placa en Cali para el viernes 5 de junio de 2026: consulte las restricciones</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/podcast/sala-de-redaccion-citytv/la-eleccion-mas-tensa-de-los-ultimos-anos-lo-que-viene-para-colombia-3562272</t>
+          <t>https://www.eltiempo.com/colombia/cali/ojo-conductor-pico-y-placa-en-cali-para-el-viernes-5-de-junio-de-2026-consulte-las-restricciones-3562140</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>05/06/2026 12:09 a. m.</t>
+          <t>05/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -760,19 +760,19 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Tribunal Administrativo del Cesar ordenó al Hospital Eduardo Arredondo Daza pagar $1.300 millones por presuntas fallas médicas en Valledupar</t>
+          <t>¡Atención conductores! Pico y placa en Bogotá para el viernes 5 de junio de 2026: así funcionará la medida</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/otras-ciudades/tribunal-administrativo-del-cesar-ordeno-al-hospital-eduardo-arredondo-daza-pagar-1-300-millones-por-presuntas-fallas-medicas-en-valledupar-3562258</t>
+          <t>https://www.eltiempo.com/bogota/atencion-conductores-pico-y-placa-en-bogota-para-el-viernes-5-de-junio-de-2026-asi-funcionara-la-medida-3562139</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>05/06/2026 12:08 a. m.</t>
+          <t>05/06/2026 12:58 a. m.</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -787,19 +787,19 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>¿El tarot es brujería?: Una experta explica cómo puede transformar su vida</t>
+          <t>Gobierno cambió las reglas de seguridad para expresidentes y exvicepresidentes: incluyó a la Dirección Nacional de Inteligencia</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/podcast/entre-vivos-y-muertos/el-tarot-es-brujeria-una-experta-explica-como-puede-transformar-su-vida-3562271</t>
+          <t>https://www.eltiempo.com/politica/gobierno/gobierno-cambio-las-reglas-de-seguridad-para-expresidentes-y-exvicepresidentes-incluyo-a-la-direccion-nacional-de-inteligencia-3562273</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>05/06/2026 12:05 a. m.</t>
+          <t>05/06/2026 12:15 a. m.</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -814,19 +814,19 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>#ElFiltro: circula imagen falsa con estilos de EL TIEMPO que difunde una supuesta propuesta de Abelardo de la Espriella sobre entidades sociales</t>
+          <t>Senador de origen colombiano abre una batalla contra Trump por la ‘green card’: ¿podrá detener la medida que preocupa a millones de inmigrantes?</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/elfiltro-circula-imagen-falsa-con-estilos-de-el-tiempo-que-difunde-una-supuesta-propuesta-de-abelardo-de-la-espriella-sobre-entidades-sociales-3562270</t>
+          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/senador-de-origen-colombiano-abre-una-batalla-contra-trump-por-la-green-card-podra-detener-la-medida-que-preocupa-a-millones-de-inmigrantes-3562054</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 11:56 p. m.</t>
+          <t>05/06/2026 12:14 a. m.</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -841,19 +841,19 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Dago García, de grabar bautizos y fiestas, a ser el rey del cine, el teatro y la televisión</t>
+          <t>La elección más tensa de los últimos años: lo que viene para Colombia</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/podcast/la-habitacion-invisible/dago-garcia-de-grabar-bautizos-y-fiestas-a-ser-el-rey-del-cine-el-teatro-y-la-television-3562269</t>
+          <t>https://www.eltiempo.com/podcast/sala-de-redaccion-citytv/la-eleccion-mas-tensa-de-los-ultimos-anos-lo-que-viene-para-colombia-3562272</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38 p. m.</t>
+          <t>05/06/2026 12:09 a. m.</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -868,19 +868,19 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Con doble calzada y drenajes, Yumbo busca solucionar problemas históricos en su conexión con Cali</t>
+          <t>Tribunal Administrativo del Cesar ordenó al Hospital Eduardo Arredondo Daza pagar $1.300 millones por presuntas fallas médicas en Valledupar</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/cali/con-doble-calzada-y-drenajes-yumbo-busca-solucionar-problemas-historicos-en-su-conexion-con-cali-3562267</t>
+          <t>https://www.eltiempo.com/colombia/otras-ciudades/tribunal-administrativo-del-cesar-ordeno-al-hospital-eduardo-arredondo-daza-pagar-1-300-millones-por-presuntas-fallas-medicas-en-valledupar-3562258</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38 p. m.</t>
+          <t>05/06/2026 12:08 a. m.</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -895,19 +895,19 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>El PGA Tour Américas vuelve a Colombia: fue presentada la nueva edición del Inter Rapidísimo Golf Championship</t>
+          <t>¿El tarot es brujería?: Una experta explica cómo puede transformar su vida</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/otros-deportes/el-pga-tour-americas-vuelve-a-colombia-fue-presentada-la-nueva-edicion-del-inter-rapidisimo-golf-championship-3562268</t>
+          <t>https://www.eltiempo.com/podcast/entre-vivos-y-muertos/el-tarot-es-brujeria-una-experta-explica-como-puede-transformar-su-vida-3562271</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 11:10 p. m.</t>
+          <t>05/06/2026 12:05 a. m.</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -922,19 +922,19 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Fotos | Selección Colombia viajó rumbo al Mundial 2026: presidente Gustavo Petro entregó la bandera del país en emotiva despedida en Catam</t>
+          <t>#ElFiltro: circula imagen falsa con estilos de EL TIEMPO que difunde una supuesta propuesta de Abelardo de la Espriella sobre entidades sociales</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-colombiano/fotos-seleccion-colombia-emprendio-viaje-al-mundial-2026-presidente-gustavo-petro-entrego-la-bandera-del-pais-en-emotiva-despedida-en-catam-3562257</t>
+          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/elfiltro-circula-imagen-falsa-con-estilos-de-el-tiempo-que-difunde-una-supuesta-propuesta-de-abelardo-de-la-espriella-sobre-entidades-sociales-3562270</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 11:03 p. m.</t>
+          <t>04/06/2026 11:56 p. m.</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -949,19 +949,19 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>La Selección Colombia Femenina busca contra Uruguay el cupo directo al Mundial 2027 y seguir peleando por ganar la Liga de Naciones: hora y TV</t>
+          <t>Dago García, de grabar bautizos y fiestas, a ser el rey del cine, el teatro y la televisión</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/la-seleccion-colombia-femenina-busca-contra-uruguay-el-cupo-directo-al-mundial-2027-y-seguir-peleando-por-ganar-la-liga-de-naciones-hora-y-tv-3562266</t>
+          <t>https://www.eltiempo.com/podcast/la-habitacion-invisible/dago-garcia-de-grabar-bautizos-y-fiestas-a-ser-el-rey-del-cine-el-teatro-y-la-television-3562269</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 11:01 p. m.</t>
+          <t>04/06/2026 11:38 p. m.</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -976,19 +976,19 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>'Juan Daniel, ¿qué pasó el domingo?' / Entrevista de María Isabel Rueda</t>
+          <t>Con doble calzada y drenajes, Yumbo busca solucionar problemas históricos en su conexión con Cali</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/juan-daniel-que-paso-el-domingo-entrevista-de-maria-isabel-rueda-3562243</t>
+          <t>https://www.eltiempo.com/colombia/cali/con-doble-calzada-y-drenajes-yumbo-busca-solucionar-problemas-historicos-en-su-conexion-con-cali-3562267</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 10:59 p. m.</t>
+          <t>04/06/2026 11:38 p. m.</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -1003,19 +1003,19 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Presidente Gustavo Petro aseguró que 'Estados Unidos se alió con narcotraficantes' tras respaldo de Donald Trump a campaña de Abelardo de la Espriella</t>
+          <t>El PGA Tour Américas vuelve a Colombia: fue presentada la nueva edición del Inter Rapidísimo Golf Championship</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/presidente-gustavo-petro-aseguro-que-estados-unidos-se-alio-con-narcotraficantes-tras-respaldo-de-donald-trump-a-campana-de-abelardo-de-la-espriella-3562265</t>
+          <t>https://www.eltiempo.com/deportes/otros-deportes/el-pga-tour-americas-vuelve-a-colombia-fue-presentada-la-nueva-edicion-del-inter-rapidisimo-golf-championship-3562268</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 10:46 p. m.</t>
+          <t>04/06/2026 11:10 p. m.</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1030,19 +1030,19 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Buenaventura, la joya del Pacífico que lidera la apuesta turística del Valle por captar 500 mil visitantes durante los tres puentes festivos de junio</t>
+          <t>Fotos | Selección Colombia viajó rumbo al Mundial 2026: presidente Gustavo Petro entregó la bandera del país en emotiva despedida en Catam</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/cali/buenaventura-la-joya-del-pacifico-que-lidera-la-apuesta-turistica-del-valle-por-captar-500-mil-visitantes-durante-los-tres-puentes-festivos-de-junio-3562259</t>
+          <t>https://www.eltiempo.com/deportes/futbol-colombiano/fotos-seleccion-colombia-emprendio-viaje-al-mundial-2026-presidente-gustavo-petro-entrego-la-bandera-del-pais-en-emotiva-despedida-en-catam-3562257</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 10:30 p. m.</t>
+          <t>04/06/2026 11:03 p. m.</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
@@ -1057,19 +1057,19 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Personería de Bogotá llega a un acuerdo con EPS e IPS para 'humanizar la atención a los pacientes' tras recibir cerca de 12.000 quejas</t>
+          <t>La Selección Colombia Femenina busca contra Uruguay el cupo directo al Mundial 2027 y seguir peleando por ganar la Liga de Naciones: hora y TV</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/bogota/personeria-de-bogota-llega-a-un-acuerdo-con-eps-e-ips-para-humanizar-la-atencion-a-los-pacientes-tras-recibir-cerca-de-12-000-quejas-3561954</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/la-seleccion-colombia-femenina-busca-contra-uruguay-el-cupo-directo-al-mundial-2027-y-seguir-peleando-por-ganar-la-liga-de-naciones-hora-y-tv-3562266</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>05/06/2026 03:57 a. m.</t>
+          <t>05/06/2026 08:37 a. m.</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1079,24 +1079,24 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Un joven herido dejó ataque contra seguidores de Abelardo de la Espriella en Bogotá</t>
+          <t>¡Es hoy! Cartagena celebra sus 493 años con una gran fiesta y concierto gratuito</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/orden-publico/un-joven-herido-dejo-ataque-contra-seguidores-de-abelardo-de-la-espriella-en-bogota-401463</t>
+          <t>https://www.eluniversal.com.co/farandula/2026/06/04/es-hoy-cartagena-celebra-sus-493-anos-con-una-gran-fiesta-y-concierto-gratuito/</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>05/06/2026 03:45 a. m.</t>
+          <t>05/06/2026 08:37 a. m.</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -1106,24 +1106,24 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>"La situación es dramática": Gobernación del Valle declara emergencia humanitaria por crisis en la salud</t>
+          <t>Farándula</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/actualidad/declaran-emergencia-humanitaria-por-crisis-en-la-salud-en-el-valle-del-cauca-401462</t>
+          <t>https://www.eluniversal.com.co/farandula/</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>05/06/2026 02:41 a. m.</t>
+          <t>05/06/2026 12:23 a. m.</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1133,24 +1133,24 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Último sorteo Lotería de Bogotá: resultado premio mayor hoy 4 de junio de 2026</t>
+          <t>Abogada de Sean ‘Diddy’ Combs entra al equipo legal de Nicolás Maduro</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/sociedad/ultimo-sorteo-loteria-de-bogota-resultado-premio-mayor-hoy-4-de-junio-de-2026-401461</t>
+          <t>https://www.eluniversal.com.co/mundo/2026/06/05/abogada-de-sean-diddy-combs-entra-al-equipo-legal-de-nicolas-maduro/</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>05/06/2026 01:37 a. m.</t>
+          <t>05/06/2026 12:00 a. m.</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
@@ -1160,24 +1160,24 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>¿Maldición en el Mundial? El inquietante historial que persigue al número 1 del ranking FIFA</t>
+          <t>Dimar anuncia investigación tras explosión de barcaza que dejó 4 muertos en Cartagena</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/deportes/mundial-2026-historial-negativo-persigue-numero-1-ranking-fifa-401453</t>
+          <t>https://www.eluniversal.com.co/cartagena/2026/06/05/dimar-anuncia-investigacion-tras-explosion-de-barcaza-que-dejo-4-fallecidos-en-cartagena/</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>05/06/2026 01:34 a. m.</t>
+          <t>05/06/2026 12:00 a. m.</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1187,24 +1187,24 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>"Yo sí creo, con todo respeto, que el candidato no es Iván Cepeda; el candidato es Gustavo Petro"</t>
+          <t>Cartagena</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/constituyente-bandera-politica-petro-impulso-campana-ivan-cepeda-401456</t>
+          <t>https://www.eluniversal.com.co/cartagena/</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 11:42 p. m.</t>
+          <t>04/06/2026 10:31 p. m.</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -1214,24 +1214,24 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>Petro se enfrenta a Tomás Uribe tras ratificación de condena contra su tío Santiago Uribe</t>
+          <t>Predial en Cartagena: Distrito ya recaudó más del 70% de la meta de 2026</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/santiago-uribe-gustavo-petro-responde-tomas-uribe-ratificacion-condena-401450</t>
+          <t>https://www.eluniversal.com.co/economica/2026/06/04/predial-en-cartagena-distrito-ya-recaudo-mas-del-70-de-la-meta-de-2026/</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 11:00 p. m.</t>
+          <t>04/06/2026 10:31 p. m.</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1241,24 +1241,24 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>De la Espriella responde a medida cautelar sobre camiseta de la Selección: “pretenden restringir libertades y desconocer derechos ciudadanos”</t>
+          <t>Económica</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/abelardo-de-la-espriella-responde-polemica-camiseta-seleccion-colombia-cuestiona-restricciones-durante-campana-401444</t>
+          <t>https://www.eluniversal.com.co/economica/</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 10:37 p. m.</t>
+          <t>04/06/2026 09:45 p. m.</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -1268,24 +1268,24 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>Los dos fichajes que prometió Florentino Pérez si logra la reelección en el Real Madrid</t>
+          <t>Video: Manifestantes rodearon sede de campaña de Abelardo De la Espriella en Bogotá</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/internacional/real-madrid-florentino-perez-fichajes-reeleccion-mourinho-401442</t>
+          <t>https://www.eluniversal.com.co/colombia/2026/06/04/video-manifestantes-rodearon-sede-de-campana-de-abelardo-de-la-espriella-en-bogota/</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 10:27 p. m.</t>
+          <t>04/06/2026 09:45 p. m.</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1295,24 +1295,24 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>‘Hombres a la Plancha’ vuelve a Bogotá con una temporada renovada llena de nostalgia y grandes éxitos</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/entretenimiento/hombres-plancha-bogota-temporada-renovada-nostalgia-401438</t>
+          <t>https://www.eluniversal.com.co/colombia/</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 10:25 p. m.</t>
+          <t>04/06/2026 09:45 p. m.</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -1322,24 +1322,24 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Tragedia en Cartagena: confirman que explosión en astillero dejó cuatro muertos y 11 heridos</t>
+          <t>¿Dónde está José Luis Márquez? Desapareció luego de la explosión en Pasacaballos</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/sociedad/tragedia-en-cartagena-confirman-que-explosion-en-astillero-dejo-cuatro-muertos-y-11-heridos-401437</t>
+          <t>https://www.eluniversal.com.co/sucesos/2026/06/04/donde-esta-jose-luis-marquez-desaparecio-luego-de-la-explosion-en-pasacaballos/</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 10:07 p. m.</t>
+          <t>04/06/2026 09:19 p. m.</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1349,24 +1349,24 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Registraduría aseguró que los softwares y censo electoral no fueron modificados tras realizar auditorías técnicas</t>
+          <t>Abelardo de la Espriella desafía fallo sobre camiseta de Colombia: esto dijo</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/softwares-y-censo-electoral-no-fueron-modificados-401443</t>
+          <t>https://www.eluniversal.com.co/colombia/2026/06/04/abelardo-de-la-espriella-desafia-fallo-sobre-camiseta-de-colombia-esto-dijo/</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>03/06/2026 01:14 p. m.</t>
+          <t>04/06/2026 09:13 p. m.</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
@@ -1376,24 +1376,24 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>“Es una decisión muy injusta”: Álvaro Uribe tras condena a su hermano Santiago</t>
+          <t>A la cárcel por la muerte de su hija, Mía Khataleya, una bebé de seis meses</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/actualidad/alvaro-uribe-injunto-fallo-santiago-uribe-12-apostoles-401447</t>
+          <t>https://www.eluniversal.com.co/sucesos/2026/06/04/a-la-carcel-por-la-muerte-de-su-hija-mia-khataleya-una-bebe-de-seis-meses/</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>22/04/2026 12:04 p. m.</t>
+          <t>04/06/2026 08:16 p. m.</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1403,24 +1403,24 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Gobierno cambió requisito para recibir dinero extra para la pensión: ya es oficial</t>
+          <t>4 víctimas fatales dejó una masacre: grupos armados estarían  detrás del ataque</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/economia/dinero-extra-pension-2026-nuevo-requisito-401451</t>
+          <t>https://www.eluniversal.com.co/sucesos/2026/06/04/cuatro-victimas-fatales-dejo-una-masacre-grupos-ilegales-estarian-detras-del-crimen/</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>26/11/2025 12:27 p. m.</t>
+          <t>04/06/2026 07:55 p. m.</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
@@ -1430,24 +1430,24 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>Abogados de Santiago Uribe califican de injusta la condena ratificada por la Corte Suprema</t>
+          <t>Estados Unidos incluye en lista Clinton a Miguel Díaz-Canel y al hijo de Raúl Castro</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/abogados-santiago-uribe-califican-injusta-condena-401439</t>
+          <t>https://www.eluniversal.com.co/mundo/2026/06/04/estados-unidos-incluye-en-lista-clinton-a-miguel-diaz-canel-y-al-hijo-de-raul-castro/</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>25/11/2025 04:53 p. m.</t>
+          <t>04/06/2026 07:31 p. m.</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1457,22 +1457,26 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>¿Qué viene ahora para Santiago Uribe tras quedar en firme su condena por homicidio y concierto para delinquir?</t>
+          <t>¡Le frenan el negocio! Recuperan 13 reses robadas y capturan a un hombre en Magangué</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/actualidad/santiago-uribe-condena-paramilitarismo-que-viene-ahora-401440</t>
+          <t>https://www.eluniversal.com.co/sucesos/2026/06/04/le-frenan-el-negocio-recuperan-13-reses-robadas-y-capturan-a-un-hombre-en-magangue/</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="inlineStr"/>
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>04/06/2026 07:06 p. m.</t>
+        </is>
+      </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1480,22 +1484,26 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>Top de los países con más festivos del mundo: ¿en qué posición quedó Colombia?</t>
+          <t>Armando Castro, el cobradiario ultimado mientras estaba en una estación de gasolina</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/actualidad/festivos-colombia-top-paises-con-mas-dias-feriados-2026-401457</t>
+          <t>https://www.eluniversal.com.co/sucesos/2026/06/04/armando-castro-el-cobradiario-ultimado-mientras-estaba-en-una-estacion-de-gasolina/</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr"/>
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>04/06/2026 07:00 p. m.</t>
+        </is>
+      </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1503,22 +1511,26 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>“La camiseta de la Selección es de todos”; juristas critican decisión contra De la Espriella</t>
+          <t>Racionamiento de agua en Cartagena seguirá una semana más: este es el cronograma</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/camiseta-seleccion-colombia-juristas-cuestionamiento-fallo-abelardo-de-la-espriella-401454</t>
+          <t>https://www.eluniversal.com.co/cartagena/2026/06/04/racionamientos-de-agua-en-cartagena-seguiran-una-semana-mas-este-es-el-cronograma/</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="inlineStr"/>
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>04/06/2026 05:42 p. m.</t>
+        </is>
+      </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1526,22 +1538,26 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>Prima para empleados públicos en 2026: cuándo deben recibir el pago y cómo se liquida</t>
+          <t>Alcaldía de Cartagena reabrió las puertas del Parque Apolo: Así quedó</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/economia/prima-empleados-publicos-2026-fecha-pago-y-monto-401455</t>
+          <t>https://www.eluniversal.com.co/cartagena/2026/06/04/alcaldia-de-cartagena-reabrio-las-puertas-del-parque-apolo-asi-quedo/</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr"/>
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>04/06/2026 05:18 p. m.</t>
+        </is>
+      </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1549,22 +1565,26 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Andi pide a la CIDH medidas cautelares por riesgos en elecciones de 2026</t>
+          <t>Video: Explosión de cisternas de gas en México provocó evacuación masiva de personas</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/economia/solicitan-medidas-cautelares-cidh-riesgos-elecciones-colombia-2026-401446</t>
+          <t>https://www.eluniversal.com.co/mundo/2026/06/04/video-explosion-de-cisternas-de-gas-en-mexico-provoco-evacuacion-masiva-de-personas/</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="inlineStr"/>
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>04/06/2026 05:09 p. m.</t>
+        </is>
+      </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1572,24 +1592,24 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>Conmoción en Cali por el asesinato de dos adolescentes en establecimiento de comidas</t>
+          <t>A sus 17 años, ‘Papucho’ habría sembrado terror con más de 20 crímenes</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/orden-publico/conmocin-en-cali-por-el-asesinato-de-dos-adolescentes-en-establecimiento-de-comidas-401445</t>
+          <t>https://www.eluniversal.com.co/sucesos/2026/06/04/a-sus-17-anos-papucho-habria-sembrado-terror-con-mas-de-20-crimenes/</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>05/06/2026 01:00 a. m.</t>
+          <t>04/06/2026 05:03 p. m.</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -1599,26 +1619,22 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>El Rugido del Tigre</t>
+          <t>Erick Poveda viajó a Ecuador buscando un mejor futuro y sicarios le quitaron la vida</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/05/el-rugido-del-tigre/</t>
+          <t>https://www.eluniversal.com.co/sucesos/2026/06/04/erick-poveda-viajo-a-ecuador-buscando-un-mejor-futuro-y-sicarios-le-quitaron-la-vida/</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="inlineStr">
-        <is>
-          <t>05/06/2026 01:00 a. m.</t>
-        </is>
-      </c>
+      <c r="A43" s="5" t="inlineStr"/>
       <c r="B43" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1626,26 +1642,22 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>Columnistas</t>
+          <t>Cartagena espera a J Balvin: crece la expectativa por sus invitados sorpresa</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/</t>
+          <t>https://www.eluniversal.com.co/farandula/2026/06/03/cartagena-espera-a-j-balvin-crece-la-expectativa-por-sus-invitados-sorpresa/</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>05/06/2026 01:00 a. m.</t>
-        </is>
-      </c>
+      <c r="A44" s="2" t="inlineStr"/>
       <c r="B44" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1653,26 +1665,22 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Un nuevo festivo en Colombia</t>
+          <t>Así puedes ganar entradas dobles para ver a J Balvin en Cartagena</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/05/un-nuevo-festivo-en-colombia/</t>
+          <t>https://www.eluniversal.com.co/cartagena/2026/06/02/asi-puedes-ganar-entradas-dobles-para-ver-a-jbalvin-en-cartagena/</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="5" t="inlineStr">
-        <is>
-          <t>05/06/2026 01:00 a. m.</t>
-        </is>
-      </c>
+      <c r="A45" s="5" t="inlineStr"/>
       <c r="B45" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1680,26 +1688,22 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>Saturados</t>
+          <t>Dumek Turbay y Hamilton se reconcilian: “No quería estar lejos de su ciudad”</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/caricaturas/2026/06/05/saturados/</t>
+          <t>https://www.eluniversal.com.co/farandula/2026/06/02/dumek-turbay-y-hamilton-se-reconcilian-no-queria-estar-lejos-de-su-ciudad/</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>05/06/2026 01:00 a. m.</t>
-        </is>
-      </c>
+      <c r="A46" s="2" t="inlineStr"/>
       <c r="B46" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -1707,24 +1711,24 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Caricaturas</t>
+          <t>Luister La Voz celebra a Cartagena: detalles del concierto de este 1 de junio</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/caricaturas/</t>
+          <t>https://www.eluniversal.com.co/farandula/2026/06/01/luister-la-voz-celebra-a-cartagena-detalles-del-concierto-de-este-1-de-junio/</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>05/06/2026 01:00 a. m.</t>
+          <t>05/06/2026 03:57 a. m.</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
@@ -1734,24 +1738,24 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>Después de Uribe</t>
+          <t>Un joven herido dejó ataque contra seguidores de Abelardo de la Espriella en Bogotá</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/05/despues-de-uribe/</t>
+          <t>https://www.lafm.com.co/orden-publico/un-joven-herido-dejo-ataque-contra-seguidores-de-abelardo-de-la-espriella-en-bogota-401463</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 11:30 p. m.</t>
+          <t>05/06/2026 03:45 a. m.</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -1761,24 +1765,24 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Polémica en redes por el supuesto desplante de James Rodríguez a la hija de Petro</t>
+          <t>"La situación es dramática": Gobernación del Valle declara emergencia humanitaria por crisis en la salud</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/04/polemica-en-redes-por-el-supuesto-desplante-de-james-rodriguez-a-la-hija-de-petro/</t>
+          <t>https://www.lafm.com.co/actualidad/declaran-emergencia-humanitaria-por-crisis-en-la-salud-en-el-valle-del-cauca-401462</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 11:30 p. m.</t>
+          <t>05/06/2026 02:41 a. m.</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
@@ -1788,24 +1792,24 @@
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Último sorteo Lotería de Bogotá: resultado premio mayor hoy 4 de junio de 2026</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/</t>
+          <t>https://www.lafm.com.co/sociedad/ultimo-sorteo-loteria-de-bogota-resultado-premio-mayor-hoy-4-de-junio-de-2026-401461</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 10:57 p. m.</t>
+          <t>05/06/2026 01:37 a. m.</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -1815,24 +1819,24 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>Cancillería denuncia una página web falsa que estafa con citas para el pasaporte</t>
+          <t>¿Maldición en el Mundial? El inquietante historial que persigue al número 1 del ranking FIFA</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/04/cancilleria-denuncia-una-pagina-web-falsa-que-estafa-con-citas-para-el-pasaporte/</t>
+          <t>https://www.lafm.com.co/deportes/mundial-2026-historial-negativo-persigue-numero-1-ranking-fifa-401453</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 10:26 p. m.</t>
+          <t>05/06/2026 01:34 a. m.</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
@@ -1842,24 +1846,24 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>Intentó sacar dos ardillas ocultas en sus partes íntimas desde Cartagena a República Dominicana: una murió</t>
+          <t>"Yo sí creo, con todo respeto, que el candidato no es Iván Cepeda; el candidato es Gustavo Petro"</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/04/intento-sacar-dos-ardillas-ocultas-en-sus-partes-intimas-desde-cartagena-a-republica-dominicana-una-murio/</t>
+          <t>https://www.lafm.com.co/politica/constituyente-bandera-politica-petro-impulso-campana-ivan-cepeda-401456</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 10:06 p. m.</t>
+          <t>04/06/2026 11:42 p. m.</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -1869,24 +1873,24 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Caso ‘Los 12 apóstoles’: Corte Suprema ratifica condena contra Santiago Uribe</t>
+          <t>Petro se enfrenta a Tomás Uribe tras ratificación de condena contra su tío Santiago Uribe</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/04/corte-suprema-ratifica-condena-contra-santiago-uribe-y-le-cierra-la-puerta-a-la-absolucion-por-el-homicidio-de-camilo-barrientos/</t>
+          <t>https://www.lafm.com.co/politica/santiago-uribe-gustavo-petro-responde-tomas-uribe-ratificacion-condena-401450</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 08:42 p. m.</t>
+          <t>04/06/2026 11:00 p. m.</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
@@ -1896,24 +1900,24 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>“Es muy injusto”: Álvaro Uribe reacciona tras ratificación de condena contra su hermano Santiago Uribe</t>
+          <t>De la Espriella responde a medida cautelar sobre camiseta de la Selección: “pretenden restringir libertades y desconocer derechos ciudadanos”</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/04/es-muy-injusto-alvaro-uribe-reacciona-tras-ratificacion-de-condena-contra-su-hermano-santiago-uribe/</t>
+          <t>https://www.lafm.com.co/politica/abelardo-de-la-espriella-responde-polemica-camiseta-seleccion-colombia-cuestiona-restricciones-durante-campana-401444</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 04:59 p. m.</t>
+          <t>04/06/2026 10:37 p. m.</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -1923,24 +1927,24 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>Nueva explosión en mina de carbón en zona rural de Sutatausa: habría trabajadores atrapados</t>
+          <t>Los dos fichajes que prometió Florentino Pérez si logra la reelección en el Real Madrid</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/04/nueva-explosion-en-mina-de-carbon-en-zona-rural-de-sutatausa-se-temen-trabajadores-atrapados/</t>
+          <t>https://www.lafm.com.co/internacional/real-madrid-florentino-perez-fichajes-reeleccion-mourinho-401442</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 03:48 p. m.</t>
+          <t>04/06/2026 10:27 p. m.</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
@@ -1950,24 +1954,24 @@
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>General Erick Rodríguez pasa a polémico retiro tras denunciar carnetización en Meta y Guaviare por disidencias</t>
+          <t>‘Hombres a la Plancha’ vuelve a Bogotá con una temporada renovada llena de nostalgia y grandes éxitos</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/04/general-erick-rodriguez-pasa-a-retiro-de-manera-polemica-tras-denunciar-carnetizacion-en-meta-y-guaviare-por-las-disidencias/</t>
+          <t>https://www.lafm.com.co/entretenimiento/hombres-plancha-bogota-temporada-renovada-nostalgia-401438</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 02:49 p. m.</t>
+          <t>04/06/2026 10:25 p. m.</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -1977,24 +1981,24 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Presidente luce camiseta de Colombia en la despedida de la Selección rumbo al Mundial</t>
+          <t>Tragedia en Cartagena: confirman que explosión en astillero dejó cuatro muertos y 11 heridos</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/04/presidente-luce-camiseta-de-colombia-en-la-despedida-de-la-seleccion-rumbo-al-mundial/</t>
+          <t>https://www.lafm.com.co/sociedad/tragedia-en-cartagena-confirman-que-explosion-en-astillero-dejo-cuatro-muertos-y-11-heridos-401437</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 01:19 p. m.</t>
+          <t>03/06/2026 10:07 p. m.</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
@@ -2004,24 +2008,24 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>Gobierno confirma nuevo día festivo en Colombia para conmemorar el Día de la Virgen de Chiquinquirá</t>
+          <t>Registraduría aseguró que los softwares y censo electoral no fueron modificados tras realizar auditorías técnicas</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/04/gobierno-confirma-nuevo-dia-festivo-en-colombia-par-conmemorar-el-dia-de-la-virgen-de-chiquinquira/</t>
+          <t>https://www.lafm.com.co/politica/softwares-y-censo-electoral-no-fueron-modificados-401443</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 12:06 p. m.</t>
+          <t>03/06/2026 01:14 p. m.</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -2031,24 +2035,24 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>“El país necesita certezas”: Empresarios desconfían del anuncio del Gobierno de desistir de la Constituyente</t>
+          <t>“Es una decisión muy injusta”: Álvaro Uribe tras condena a su hermano Santiago</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/politica/elecciones/2026/06/04/el-pais-necesita-certezas-empresarios-desconfian-del-anuncio-del-gobierno-de-desistir-de-la-constituyente/</t>
+          <t>https://www.lafm.com.co/actualidad/alvaro-uribe-injunto-fallo-santiago-uribe-12-apostoles-401447</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 12:06 p. m.</t>
+          <t>22/04/2026 12:04 p. m.</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
@@ -2058,24 +2062,24 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>Elecciones</t>
+          <t>Gobierno cambió requisito para recibir dinero extra para la pensión: ya es oficial</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/politica/elecciones/</t>
+          <t>https://www.lafm.com.co/economia/dinero-extra-pension-2026-nuevo-requisito-401451</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>05/06/2026 12:48 a. m.</t>
+          <t>26/11/2025 12:27 p. m.</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -2085,24 +2089,24 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Presidente Petro llamó a ‘atemperar’ los ánimos de las campañas presidenciales para evitar desmanes</t>
+          <t>Abogados de Santiago Uribe califican de injusta la condena ratificada por la Corte Suprema</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/05/presidente-petro-llamo-a-atemperar-los-animos-de-las-campanas-presidenciales-para-evitar-desmanes/</t>
+          <t>https://www.lafm.com.co/politica/abogados-santiago-uribe-califican-injusta-condena-401439</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 11:42 p. m.</t>
+          <t>25/11/2025 04:53 p. m.</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
@@ -2112,26 +2116,22 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>Álvaro Uribe calificó de “injusta” condena contra su hermano: “Mi familia está muy abatida”</t>
+          <t>¿Qué viene ahora para Santiago Uribe tras quedar en firme su condena por homicidio y concierto para delinquir?</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/05/uribe-califico-de-injusta-condena-contra-su-hermano-mi-familia-esta-muy-abatida/</t>
+          <t>https://www.lafm.com.co/actualidad/santiago-uribe-condena-paramilitarismo-que-viene-ahora-401440</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>04/06/2026 10:26 p. m.</t>
-        </is>
-      </c>
+      <c r="A62" s="2" t="inlineStr"/>
       <c r="B62" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2139,26 +2139,22 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Fernando Carrillo lanza “Colombia 2050”, un libro que reúne 65 voces para pensar el futuro del país</t>
+          <t>Top de los países con más festivos del mundo: ¿en qué posición quedó Colombia?</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/05/fernando-carrillo-lanza-colombia-2050-un-libro-que-reune-65-voces-para-pensar-el-futuro-del-pais/</t>
+          <t>https://www.lafm.com.co/actualidad/festivos-colombia-top-paises-con-mas-dias-feriados-2026-401457</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="5" t="inlineStr">
-        <is>
-          <t>04/06/2026 09:34 p. m.</t>
-        </is>
-      </c>
+      <c r="A63" s="5" t="inlineStr"/>
       <c r="B63" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2166,26 +2162,22 @@
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
-          <t>Así queda el calendario OFICIAL en lo que queda de 2026: ¿cuál es el nuevo festivo? Esto dice la ley</t>
+          <t>“La camiseta de la Selección es de todos”; juristas critican decisión contra De la Espriella</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/05/asi-queda-el-calendario-oficial-en-lo-que-queda-de-2026-cual-es-el-nuevo-festivo-esto-dice-la-ley/</t>
+          <t>https://www.lafm.com.co/politica/camiseta-seleccion-colombia-juristas-cuestionamiento-fallo-abelardo-de-la-espriella-401454</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>04/06/2026 09:12 p. m.</t>
-        </is>
-      </c>
+      <c r="A64" s="2" t="inlineStr"/>
       <c r="B64" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2193,26 +2185,22 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Pilotos y viajeros, atentos: cambiará el operador del parqueadero del Puente Aéreo en El Dorado</t>
+          <t>Prima para empleados públicos en 2026: cuándo deben recibir el pago y cómo se liquida</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/05/pilotos-y-viajeros-atentos-cambiara-el-operador-del-parqueadero-del-puente-aereo-en-el-dorado/</t>
+          <t>https://www.lafm.com.co/economia/prima-empleados-publicos-2026-fecha-pago-y-monto-401455</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="5" t="inlineStr">
-        <is>
-          <t>04/06/2026 08:55 p. m.</t>
-        </is>
-      </c>
+      <c r="A65" s="5" t="inlineStr"/>
       <c r="B65" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2220,26 +2208,22 @@
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>Registraduría presentó evidencia a partidos políticos de que no habría sido modificado software</t>
+          <t>Andi pide a la CIDH medidas cautelares por riesgos en elecciones de 2026</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/05/registraduria-presento-evidencia-a-partidos-politicos-de-que-no-habria-sido-modificado-software/</t>
+          <t>https://www.lafm.com.co/economia/solicitan-medidas-cautelares-cidh-riesgos-elecciones-colombia-2026-401446</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>04/06/2026 08:17 p. m.</t>
-        </is>
-      </c>
+      <c r="A66" s="2" t="inlineStr"/>
       <c r="B66" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2247,24 +2231,24 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Caracol Radio</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Andi y Fundación Estado de Derecho solicitan medidas cautelares para el presidente Petro ante CIDH</t>
+          <t>Conmoción en Cali por el asesinato de dos adolescentes en establecimiento de comidas</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/05/andi-y-fundacion-estado-de-derecho-solicita-medidas-cautelares-para-el-presidente-petro-ante-cidh/</t>
+          <t>https://www.lafm.com.co/orden-publico/conmocin-en-cali-por-el-asesinato-de-dos-adolescentes-en-establecimiento-de-comidas-401445</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 07:38 p. m.</t>
+          <t>05/06/2026 03:47 a. m.</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr">
@@ -2279,19 +2263,19 @@
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>“Hay que exigirle a la JEP que realmente le cumpla a las víctimas”: José Manuel Restrepo</t>
+          <t>Shakira y Burna Boy presentarán ‘Dai Dai’ en la inauguración del Mundial</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/05/hay-que-exigirle-a-la-jep-que-realmente-le-cumpla-a-las-victimas-jose-manuel-restrepo/</t>
+          <t>https://caracol.com.co/2026/06/05/shakira-y-burna-boy-presentaran-dai-dai-en-la-inauguracion-del-mundial/</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 07:28 p. m.</t>
+          <t>05/06/2026 12:48 a. m.</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -2306,19 +2290,19 @@
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>JEP: Ninguno de los 40 generales llamados por falsos positivos había respondido ante la justicia</t>
+          <t>Presidente Petro llamó a ‘atemperar’ los ánimos de las campañas presidenciales para evitar desmanes</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/05/jep-ninguno-de-los-40-militares-llamados-por-falsos-positivos-habia-respondido-ante-la-justicia/</t>
+          <t>https://caracol.com.co/2026/06/05/presidente-petro-llamo-a-atemperar-los-animos-de-las-campanas-presidenciales-para-evitar-desmanes/</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 07:10 p. m.</t>
+          <t>04/06/2026 11:42 p. m.</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
@@ -2333,19 +2317,19 @@
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>ATENCIÓN: Ataque armado contra la seguridad del Buque Hospital Benkos Biohó en Chocó</t>
+          <t>Álvaro Uribe calificó de “injusta” condena contra su hermano: “Mi familia está muy abatida”</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/05/atencion-ataque-armado-contra-la-seguridad-del-buque-hospital-benkos-bioho-en-choco/</t>
+          <t>https://caracol.com.co/2026/06/05/uribe-califico-de-injusta-condena-contra-su-hermano-mi-familia-esta-muy-abatida/</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 06:56 p. m.</t>
+          <t>04/06/2026 10:26 p. m.</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -2360,19 +2344,19 @@
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>Candidatos presidenciales peruanos cierran campaña en Lima</t>
+          <t>Fernando Carrillo lanza “Colombia 2050”, un libro que reúne 65 voces para pensar el futuro del país</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/candidatos-presidenciales-peruanos-cierran-campana-en-lima/</t>
+          <t>https://caracol.com.co/2026/06/05/fernando-carrillo-lanza-colombia-2050-un-libro-que-reune-65-voces-para-pensar-el-futuro-del-pais/</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 06:08 p. m.</t>
+          <t>04/06/2026 09:34 p. m.</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr">
@@ -2387,19 +2371,19 @@
       </c>
       <c r="D71" s="6" t="inlineStr">
         <is>
-          <t>¿Qué se debe conectar primero, el celular o el cargador?: esto dicen los expertos para evitar daños</t>
+          <t>Así queda el calendario OFICIAL en lo que queda de 2026: ¿cuál es el nuevo festivo? Esto dice la ley</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/que-se-debe-conectar-primero-el-celular-o-el-cargador-esto-dicen-los-expertos-para-evitar-danos/</t>
+          <t>https://caracol.com.co/2026/06/05/asi-queda-el-calendario-oficial-en-lo-que-queda-de-2026-cual-es-el-nuevo-festivo-esto-dice-la-ley/</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 06:04 p. m.</t>
+          <t>04/06/2026 09:12 p. m.</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -2414,19 +2398,19 @@
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>“Seguiremos portando la camiseta”: Abelardo de la Espriella pese a decisión judicial</t>
+          <t>Pilotos y viajeros, atentos: cambiará el operador del parqueadero del Puente Aéreo en El Dorado</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/seguiremos-portando-la-camiseta-abelardo-de-la-espriella-pese-a-decision-judicial/</t>
+          <t>https://caracol.com.co/2026/06/05/pilotos-y-viajeros-atentos-cambiara-el-operador-del-parqueadero-del-puente-aereo-en-el-dorado/</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 05:50 p. m.</t>
+          <t>04/06/2026 08:55 p. m.</t>
         </is>
       </c>
       <c r="B73" s="5" t="inlineStr">
@@ -2441,19 +2425,19 @@
       </c>
       <c r="D73" s="6" t="inlineStr">
         <is>
-          <t>Alianza Verde aprobó estudio de escisión de Catherine Juvinao y abre paso a nuevo proyecto político</t>
+          <t>Registraduría presentó evidencia a partidos políticos de que no habría sido modificado software</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/alianza-verde-aprobo-escision-de-catherine-juvinao-y-abre-paso-a-nuevo-proyecto-politico/</t>
+          <t>https://caracol.com.co/2026/06/05/registraduria-presento-evidencia-a-partidos-politicos-de-que-no-habria-sido-modificado-software/</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 05:36 p. m.</t>
+          <t>04/06/2026 08:17 p. m.</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -2468,19 +2452,19 @@
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>Fenómeno de ‘El Niño’ podría causar muerte de corales a nivel global</t>
+          <t>Andi y Fundación Estado de Derecho solicitan medidas cautelares para el presidente Petro ante CIDH</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/fenomeno-de-el-nino-podria-causar-muerte-de-corales-a-nivel-global/</t>
+          <t>https://caracol.com.co/2026/06/05/andi-y-fundacion-estado-de-derecho-solicita-medidas-cautelares-para-el-presidente-petro-ante-cidh/</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 05:27 p. m.</t>
+          <t>04/06/2026 07:38 p. m.</t>
         </is>
       </c>
       <c r="B75" s="5" t="inlineStr">
@@ -2495,19 +2479,19 @@
       </c>
       <c r="D75" s="6" t="inlineStr">
         <is>
-          <t>Congreso aprobó proyecto para castigar la zoofilia como delito: estas serían las penas</t>
+          <t>“Hay que exigirle a la JEP que realmente le cumpla a las víctimas”: José Manuel Restrepo</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/congreso-aprobo-proyecto-para-castigar-la-zoofilia-como-delito-estas-serian-las-penas/</t>
+          <t>https://caracol.com.co/2026/06/05/hay-que-exigirle-a-la-jep-que-realmente-le-cumpla-a-las-victimas-jose-manuel-restrepo/</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 05:03 p. m.</t>
+          <t>04/06/2026 07:28 p. m.</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -2522,19 +2506,19 @@
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>FMI y Venezuela registran progreso en negociaciones sobre monitoreo y asistencia monetaria</t>
+          <t>JEP: Ninguno de los 40 generales llamados por falsos positivos había respondido ante la justicia</t>
         </is>
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/fmi-y-venezuela-registran-progreso-en-negociaciones-sobre-monitoreo-y-asistencia-monetaria/</t>
+          <t>https://caracol.com.co/2026/06/05/jep-ninguno-de-los-40-militares-llamados-por-falsos-positivos-habia-respondido-ante-la-justicia/</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 05:00 p. m.</t>
+          <t>04/06/2026 07:10 p. m.</t>
         </is>
       </c>
       <c r="B77" s="5" t="inlineStr">
@@ -2549,19 +2533,19 @@
       </c>
       <c r="D77" s="6" t="inlineStr">
         <is>
-          <t>CTI capturó a uno de los presuntos implicados en crimen de estudiante en la estación Minuto de Dios</t>
+          <t>ATENCIÓN: Ataque armado contra la seguridad del Buque Hospital Benkos Biohó en Chocó</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/cti-capturo-a-uno-de-los-presuntos-implicados-en-crimen-de-estudiante-en-la-estacion-minuto-de-dios/</t>
+          <t>https://caracol.com.co/2026/06/05/atencion-ataque-armado-contra-la-seguridad-del-buque-hospital-benkos-bioho-en-choco/</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 04:58 p. m.</t>
+          <t>04/06/2026 06:56 p. m.</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -2576,19 +2560,19 @@
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>“Esto se llama censura de prensa”: presidente Petro por investigación a Hollman Morris</t>
+          <t>Candidatos presidenciales peruanos cierran campaña en Lima</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/esto-se-llama-censura-de-prensa-presidente-petro-por-investigacion-a-hollman-morris/</t>
+          <t>https://caracol.com.co/2026/06/04/candidatos-presidenciales-peruanos-cierran-campana-en-lima/</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 04:54 p. m.</t>
+          <t>04/06/2026 06:08 p. m.</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
@@ -2603,19 +2587,19 @@
       </c>
       <c r="D79" s="6" t="inlineStr">
         <is>
-          <t>Abogado Jaime Granados acata fallo de la Corte: insiste en que condena de Santiago Uribe es injusta</t>
+          <t>¿Qué se debe conectar primero, el celular o el cargador?: esto dicen los expertos para evitar daños</t>
         </is>
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/04/abogado-jaime-granados-acata-fallo-de-la-corte-insiste-en-que-condena-de-santiago-uribe-es-injusta/</t>
+          <t>https://caracol.com.co/2026/06/04/que-se-debe-conectar-primero-el-celular-o-el-cargador-esto-dicen-los-expertos-para-evitar-danos/</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>05/06/2026 12:23 a. m.</t>
+          <t>04/06/2026 06:04 p. m.</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -2625,24 +2609,24 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>Abogada de Sean ‘Diddy’ Combs entra al equipo legal de Nicolás Maduro</t>
+          <t>“Seguiremos portando la camiseta”: Abelardo de la Espriella pese a decisión judicial</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/mundo/2026/06/05/abogada-de-sean-diddy-combs-entra-al-equipo-legal-de-nicolas-maduro/</t>
+          <t>https://caracol.com.co/2026/06/04/seguiremos-portando-la-camiseta-abelardo-de-la-espriella-pese-a-decision-judicial/</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>05/06/2026 12:00 a. m.</t>
+          <t>04/06/2026 05:50 p. m.</t>
         </is>
       </c>
       <c r="B81" s="5" t="inlineStr">
@@ -2652,24 +2636,24 @@
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D81" s="6" t="inlineStr">
         <is>
-          <t>Dimar anuncia investigación tras explosión de barcaza que dejó 4 muertos en Cartagena</t>
+          <t>Alianza Verde aprobó estudio de escisión de Catherine Juvinao y abre paso a nuevo proyecto político</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/cartagena/2026/06/05/dimar-anuncia-investigacion-tras-explosion-de-barcaza-que-dejo-4-fallecidos-en-cartagena/</t>
+          <t>https://caracol.com.co/2026/06/04/alianza-verde-aprobo-escision-de-catherine-juvinao-y-abre-paso-a-nuevo-proyecto-politico/</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>05/06/2026 12:00 a. m.</t>
+          <t>04/06/2026 05:36 p. m.</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -2679,24 +2663,24 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>Cartagena</t>
+          <t>Fenómeno de ‘El Niño’ podría causar muerte de corales a nivel global</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/cartagena/</t>
+          <t>https://caracol.com.co/2026/06/04/fenomeno-de-el-nino-podria-causar-muerte-de-corales-a-nivel-global/</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 10:31 p. m.</t>
+          <t>04/06/2026 05:27 p. m.</t>
         </is>
       </c>
       <c r="B83" s="5" t="inlineStr">
@@ -2706,24 +2690,24 @@
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D83" s="6" t="inlineStr">
         <is>
-          <t>Predial en Cartagena: Distrito ya recaudó más del 70% de la meta de 2026</t>
+          <t>Congreso aprobó proyecto para castigar la zoofilia como delito: estas serían las penas</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/economica/2026/06/04/predial-en-cartagena-distrito-ya-recaudo-mas-del-70-de-la-meta-de-2026/</t>
+          <t>https://caracol.com.co/2026/06/04/congreso-aprobo-proyecto-para-castigar-la-zoofilia-como-delito-estas-serian-las-penas/</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 10:31 p. m.</t>
+          <t>04/06/2026 05:03 p. m.</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -2733,24 +2717,24 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>Económica</t>
+          <t>FMI y Venezuela registran progreso en negociaciones sobre monitoreo y asistencia monetaria</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/economica/</t>
+          <t>https://caracol.com.co/2026/06/04/fmi-y-venezuela-registran-progreso-en-negociaciones-sobre-monitoreo-y-asistencia-monetaria/</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 09:45 p. m.</t>
+          <t>04/06/2026 05:00 p. m.</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr">
@@ -2760,24 +2744,24 @@
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D85" s="6" t="inlineStr">
         <is>
-          <t>Video: Manifestantes rodearon sede de campaña de Abelardo De la Espriella en Bogotá</t>
+          <t>CTI capturó a uno de los presuntos implicados en crimen de estudiante en la estación Minuto de Dios</t>
         </is>
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/colombia/2026/06/04/video-manifestantes-rodearon-sede-de-campana-de-abelardo-de-la-espriella-en-bogota/</t>
+          <t>https://caracol.com.co/2026/06/04/cti-capturo-a-uno-de-los-presuntos-implicados-en-crimen-de-estudiante-en-la-estacion-minuto-de-dios/</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 09:45 p. m.</t>
+          <t>04/06/2026 04:58 p. m.</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -2787,24 +2771,24 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>Caracol Radio</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>“Esto se llama censura de prensa”: presidente Petro por investigación a Hollman Morris</t>
         </is>
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/colombia/</t>
+          <t>https://caracol.com.co/2026/06/04/esto-se-llama-censura-de-prensa-presidente-petro-por-investigacion-a-hollman-morris/</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 09:45 p. m.</t>
+          <t>05/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B87" s="5" t="inlineStr">
@@ -2814,24 +2798,24 @@
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D87" s="6" t="inlineStr">
         <is>
-          <t>¿Dónde está José Luis Márquez? Desapareció luego de la explosión en Pasacaballos</t>
+          <t>El Rugido del Tigre</t>
         </is>
       </c>
       <c r="E87" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/sucesos/2026/06/04/donde-esta-jose-luis-marquez-desaparecio-luego-de-la-explosion-en-pasacaballos/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/05/el-rugido-del-tigre/</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 09:19 p. m.</t>
+          <t>05/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -2841,24 +2825,24 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>Abelardo de la Espriella desafía fallo sobre camiseta de Colombia: esto dijo</t>
+          <t>Columnistas</t>
         </is>
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/colombia/2026/06/04/abelardo-de-la-espriella-desafia-fallo-sobre-camiseta-de-colombia-esto-dijo/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 09:13 p. m.</t>
+          <t>05/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B89" s="5" t="inlineStr">
@@ -2868,24 +2852,24 @@
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D89" s="6" t="inlineStr">
         <is>
-          <t>A la cárcel por la muerte de su hija, Mía Khataleya, una bebé de seis meses</t>
+          <t>Un nuevo festivo en Colombia</t>
         </is>
       </c>
       <c r="E89" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/sucesos/2026/06/04/a-la-carcel-por-la-muerte-de-su-hija-mia-khataleya-una-bebe-de-seis-meses/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/05/un-nuevo-festivo-en-colombia/</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 08:16 p. m.</t>
+          <t>05/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -2895,24 +2879,24 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>4 víctimas fatales dejó una masacre: grupos armados estarían  detrás del ataque</t>
+          <t>Saturados</t>
         </is>
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/sucesos/2026/06/04/cuatro-victimas-fatales-dejo-una-masacre-grupos-ilegales-estarian-detras-del-crimen/</t>
+          <t>https://www.vanguardia.com/opinion/caricaturas/2026/06/05/saturados/</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 07:55 p. m.</t>
+          <t>05/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B91" s="5" t="inlineStr">
@@ -2922,24 +2906,24 @@
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D91" s="6" t="inlineStr">
         <is>
-          <t>Estados Unidos incluye en lista Clinton a Miguel Díaz-Canel y al hijo de Raúl Castro</t>
+          <t>Caricaturas</t>
         </is>
       </c>
       <c r="E91" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/mundo/2026/06/04/estados-unidos-incluye-en-lista-clinton-a-miguel-diaz-canel-y-al-hijo-de-raul-castro/</t>
+          <t>https://www.vanguardia.com/opinion/caricaturas/</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 07:31 p. m.</t>
+          <t>05/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -2949,24 +2933,24 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>¡Le frenan el negocio! Recuperan 13 reses robadas y capturan a un hombre en Magangué</t>
+          <t>Después de Uribe</t>
         </is>
       </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/sucesos/2026/06/04/le-frenan-el-negocio-recuperan-13-reses-robadas-y-capturan-a-un-hombre-en-magangue/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/05/despues-de-uribe/</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 07:06 p. m.</t>
+          <t>04/06/2026 11:30 p. m.</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
@@ -2976,24 +2960,24 @@
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D93" s="6" t="inlineStr">
         <is>
-          <t>Armando Castro, el cobradiario ultimado mientras estaba en una estación de gasolina</t>
+          <t>Polémica en redes por el supuesto desplante de James Rodríguez a la hija de Petro</t>
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/sucesos/2026/06/04/armando-castro-el-cobradiario-ultimado-mientras-estaba-en-una-estacion-de-gasolina/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/04/polemica-en-redes-por-el-supuesto-desplante-de-james-rodriguez-a-la-hija-de-petro/</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 07:00 p. m.</t>
+          <t>04/06/2026 11:30 p. m.</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -3003,24 +2987,24 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>Racionamiento de agua en Cartagena seguirá una semana más: este es el cronograma</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/cartagena/2026/06/04/racionamientos-de-agua-en-cartagena-seguiran-una-semana-mas-este-es-el-cronograma/</t>
+          <t>https://www.vanguardia.com/colombia/</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 05:42 p. m.</t>
+          <t>04/06/2026 10:57 p. m.</t>
         </is>
       </c>
       <c r="B95" s="5" t="inlineStr">
@@ -3030,24 +3014,24 @@
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D95" s="6" t="inlineStr">
         <is>
-          <t>Alcaldía de Cartagena reabrió las puertas del Parque Apolo: Así quedó</t>
+          <t>Cancillería denuncia una página web falsa que estafa con citas para el pasaporte</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/cartagena/2026/06/04/alcaldia-de-cartagena-reabrio-las-puertas-del-parque-apolo-asi-quedo/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/04/cancilleria-denuncia-una-pagina-web-falsa-que-estafa-con-citas-para-el-pasaporte/</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 05:18 p. m.</t>
+          <t>04/06/2026 10:26 p. m.</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -3057,24 +3041,24 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>Video: Explosión de cisternas de gas en México provocó evacuación masiva de personas</t>
+          <t>Intentó sacar dos ardillas ocultas en sus partes íntimas desde Cartagena a República Dominicana: una murió</t>
         </is>
       </c>
       <c r="E96" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/mundo/2026/06/04/video-explosion-de-cisternas-de-gas-en-mexico-provoco-evacuacion-masiva-de-personas/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/04/intento-sacar-dos-ardillas-ocultas-en-sus-partes-intimas-desde-cartagena-a-republica-dominicana-una-murio/</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 05:09 p. m.</t>
+          <t>04/06/2026 10:06 p. m.</t>
         </is>
       </c>
       <c r="B97" s="5" t="inlineStr">
@@ -3084,24 +3068,24 @@
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D97" s="6" t="inlineStr">
         <is>
-          <t>A sus 17 años, ‘Papucho’ habría sembrado terror con más de 20 crímenes</t>
+          <t>Caso ‘Los 12 apóstoles’: Corte Suprema ratifica condena contra Santiago Uribe</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/sucesos/2026/06/04/a-sus-17-anos-papucho-habria-sembrado-terror-con-mas-de-20-crimenes/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/04/corte-suprema-ratifica-condena-contra-santiago-uribe-y-le-cierra-la-puerta-a-la-absolucion-por-el-homicidio-de-camilo-barrientos/</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 05:03 p. m.</t>
+          <t>04/06/2026 08:42 p. m.</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -3111,24 +3095,24 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>Erick Poveda viajó a Ecuador buscando un mejor futuro y sicarios le quitaron la vida</t>
+          <t>“Es muy injusto”: Álvaro Uribe reacciona tras ratificación de condena contra su hermano Santiago Uribe</t>
         </is>
       </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/sucesos/2026/06/04/erick-poveda-viajo-a-ecuador-buscando-un-mejor-futuro-y-sicarios-le-quitaron-la-vida/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/04/es-muy-injusto-alvaro-uribe-reacciona-tras-ratificacion-de-condena-contra-su-hermano-santiago-uribe/</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 08:37 a. m.</t>
+          <t>04/06/2026 04:59 p. m.</t>
         </is>
       </c>
       <c r="B99" s="5" t="inlineStr">
@@ -3138,24 +3122,24 @@
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D99" s="6" t="inlineStr">
         <is>
-          <t>¡Es hoy! Cartagena celebra sus 493 años con una gran fiesta y concierto gratuito</t>
+          <t>Nueva explosión en mina de carbón en zona rural de Sutatausa: habría trabajadores atrapados</t>
         </is>
       </c>
       <c r="E99" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/farandula/2026/06/04/es-hoy-cartagena-celebra-sus-493-anos-con-una-gran-fiesta-y-concierto-gratuito/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/04/nueva-explosion-en-mina-de-carbon-en-zona-rural-de-sutatausa-se-temen-trabajadores-atrapados/</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 08:37 a. m.</t>
+          <t>04/06/2026 03:48 p. m.</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -3165,22 +3149,26 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>Farándula</t>
+          <t>General Erick Rodríguez pasa a polémico retiro tras denunciar carnetización en Meta y Guaviare por disidencias</t>
         </is>
       </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/farandula/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/04/general-erick-rodriguez-pasa-a-retiro-de-manera-polemica-tras-denunciar-carnetizacion-en-meta-y-guaviare-por-las-disidencias/</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="5" t="inlineStr"/>
+      <c r="A101" s="5" t="inlineStr">
+        <is>
+          <t>04/06/2026 02:49 p. m.</t>
+        </is>
+      </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3188,22 +3176,26 @@
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D101" s="6" t="inlineStr">
         <is>
-          <t>Cartagena espera a J Balvin: crece la expectativa por sus invitados sorpresa</t>
+          <t>Presidente luce camiseta de Colombia en la despedida de la Selección rumbo al Mundial</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/farandula/2026/06/03/cartagena-espera-a-j-balvin-crece-la-expectativa-por-sus-invitados-sorpresa/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/04/presidente-luce-camiseta-de-colombia-en-la-despedida-de-la-seleccion-rumbo-al-mundial/</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="2" t="inlineStr"/>
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>04/06/2026 01:19 p. m.</t>
+        </is>
+      </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3211,22 +3203,26 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>Así puedes ganar entradas dobles para ver a J Balvin en Cartagena</t>
+          <t>Gobierno confirma nuevo día festivo en Colombia para conmemorar el Día de la Virgen de Chiquinquirá</t>
         </is>
       </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/cartagena/2026/06/02/asi-puedes-ganar-entradas-dobles-para-ver-a-jbalvin-en-cartagena/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/04/gobierno-confirma-nuevo-dia-festivo-en-colombia-par-conmemorar-el-dia-de-la-virgen-de-chiquinquira/</t>
         </is>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="5" t="inlineStr"/>
+      <c r="A103" s="5" t="inlineStr">
+        <is>
+          <t>04/06/2026 12:06 p. m.</t>
+        </is>
+      </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3234,22 +3230,26 @@
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D103" s="6" t="inlineStr">
         <is>
-          <t>Dumek Turbay y Hamilton se reconcilian: “No quería estar lejos de su ciudad”</t>
+          <t>“El país necesita certezas”: Empresarios desconfían del anuncio del Gobierno de desistir de la Constituyente</t>
         </is>
       </c>
       <c r="E103" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/farandula/2026/06/02/dumek-turbay-y-hamilton-se-reconcilian-no-queria-estar-lejos-de-su-ciudad/</t>
+          <t>https://www.vanguardia.com/politica/elecciones/2026/06/04/el-pais-necesita-certezas-empresarios-desconfian-del-anuncio-del-gobierno-de-desistir-de-la-constituyente/</t>
         </is>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="2" t="inlineStr"/>
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>04/06/2026 12:06 p. m.</t>
+        </is>
+      </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3257,24 +3257,24 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>Luister La Voz celebra a Cartagena: detalles del concierto de este 1 de junio</t>
+          <t>Elecciones</t>
         </is>
       </c>
       <c r="E104" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/farandula/2026/06/01/luister-la-voz-celebra-a-cartagena-detalles-del-concierto-de-este-1-de-junio/</t>
+          <t>https://www.vanguardia.com/politica/elecciones/</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>05/06/2026 12:01 a. m.</t>
+          <t>05/06/2026 12:05 a. m.</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
@@ -3289,19 +3289,19 @@
       </c>
       <c r="D105" s="6" t="inlineStr">
         <is>
-          <t>De la Espriella ofrece a Colombia un plan que no funcionó en El Salvador</t>
+          <t>‘Backrooms’: El laberinto liminal de Kane Parsons no logra despegar</t>
         </is>
       </c>
       <c r="E105" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/allison-benson-hernandez/de-la-espriella-ofrece-a-colombia-un-plan-que-no-funciono-en-el-salvador/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/criticadecine/backrooms-el-laberinto-liminal-de-kane-parsons-no-logra-despegar/</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>05/06/2026 12:00 a. m.</t>
+          <t>05/06/2026 12:05 a. m.</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
@@ -3316,19 +3316,19 @@
       </c>
       <c r="D106" s="3" t="inlineStr">
         <is>
-          <t>¡Que ruede la pecosa!</t>
+          <t>China 1999-2026: de Belgrado a Trump</t>
         </is>
       </c>
       <c r="E106" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/madame-papita/que-ruede-la-pecosa/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/fernando-barbosa/china-1999-2026-de-belgrado-a-trump/</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>05/06/2026 12:00 a. m.</t>
+          <t>05/06/2026 12:05 a. m.</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
@@ -3343,19 +3343,19 @@
       </c>
       <c r="D107" s="6" t="inlineStr">
         <is>
-          <t>Un aire nuevo y desconocido</t>
+          <t>Una decisión importante</t>
         </is>
       </c>
       <c r="E107" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/arturo-guerrero/un-aire-nuevo-y-desconocido/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/francisco-gutierrez-sanin/una-decision-importante/</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>05/06/2026 12:00 a. m.</t>
+          <t>05/06/2026 12:05 a. m.</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
@@ -3370,19 +3370,19 @@
       </c>
       <c r="D108" s="3" t="inlineStr">
         <is>
-          <t>Palabras armadas</t>
+          <t>¿Cesó la horrible noche para el Valle?</t>
         </is>
       </c>
       <c r="E108" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/augusto-trujillo-munoz/palabras-armadas/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/mario-fernando-prado/ceso-la-horrible-noche-para-el-valle/</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 10:00 p. m.</t>
+          <t>05/06/2026 12:01 a. m.</t>
         </is>
       </c>
       <c r="B109" s="5" t="inlineStr">
@@ -3397,19 +3397,19 @@
       </c>
       <c r="D109" s="6" t="inlineStr">
         <is>
-          <t>Google quiere liberar 64 millones de mosquitos infectados con bacterias, ¿por qué?</t>
+          <t>De la Espriella ofrece a Colombia un plan que no funcionó en El Salvador</t>
         </is>
       </c>
       <c r="E109" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/ambiente/google-quiere-liberar-64-millones-de-mosquitos-infectados-con-bacterias-por-que/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/allison-benson-hernandez/de-la-espriella-ofrece-a-colombia-un-plan-que-no-funciono-en-el-salvador/</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 09:55 p. m.</t>
+          <t>05/06/2026 12:00 a. m.</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
@@ -3424,17 +3424,21 @@
       </c>
       <c r="D110" s="3" t="inlineStr">
         <is>
-          <t>Fiscalía imputará a Blessd por presunto secuestro extorsivo contra el mánager de su doble</t>
+          <t>No estamos para constituyentes</t>
         </is>
       </c>
       <c r="E110" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/judicial/fiscalia-imputara-a-blessd-por-presunto-secuestro-extorsivo-contra-el-manager-de-su-doble/</t>
+          <t>https://www.elespectador.com/opinion/editorial/no-estamos-para-constituyentes/</t>
         </is>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="5" t="inlineStr"/>
+      <c r="A111" s="5" t="inlineStr">
+        <is>
+          <t>05/06/2026 12:00 a. m.</t>
+        </is>
+      </c>
       <c r="B111" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3447,17 +3451,21 @@
       </c>
       <c r="D111" s="6" t="inlineStr">
         <is>
-          <t>Los cinco puntos claves de la condena contra Santiago Uribe por “Los 12 Apóstoles”</t>
+          <t>¡Que ruede la pecosa!</t>
         </is>
       </c>
       <c r="E111" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/judicial/santiago-uribe-velez-los-cinco-puntos-claves-de-la-condena-de-la-corte-suprema-por-el-caso-de-los-12-apostoles/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/madame-papita/que-ruede-la-pecosa/</t>
         </is>
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="2" t="inlineStr"/>
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>05/06/2026 12:00 a. m.</t>
+        </is>
+      </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3470,17 +3478,21 @@
       </c>
       <c r="D112" s="3" t="inlineStr">
         <is>
-          <t>Nuevo festivo llega en julio de 2026: esto deben saber las empresas sobre sus obligaciones</t>
+          <t>Palabras armadas</t>
         </is>
       </c>
       <c r="E112" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/economia/empresas/nuevo-festivo-llega-en-julio-de-2026-esto-deben-saber-las-empresas-sobre-sus-obligaciones-noticias-colombia/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/augusto-trujillo-munoz/palabras-armadas/</t>
         </is>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="5" t="inlineStr"/>
+      <c r="A113" s="5" t="inlineStr">
+        <is>
+          <t>05/06/2026 12:00 a. m.</t>
+        </is>
+      </c>
       <c r="B113" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3493,12 +3505,12 @@
       </c>
       <c r="D113" s="6" t="inlineStr">
         <is>
-          <t>Accidente minero en Sutatausa deja una víctima fatal y cuatro operarios atrapados</t>
+          <t>Un aire nuevo y desconocido</t>
         </is>
       </c>
       <c r="E113" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/bogota/accidente-minero-en-sutatausa-deja-una-victima-fatal-y-cuatro-operarios-atrapados/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/arturo-guerrero/un-aire-nuevo-y-desconocido/</t>
         </is>
       </c>
     </row>
@@ -3516,12 +3528,12 @@
       </c>
       <c r="D114" s="3" t="inlineStr">
         <is>
-          <t>Así se aplicaron ajustes “duros” en las campañas presidenciales de De la Espriella y Cepeda</t>
+          <t>Google quiere liberar 64 millones de mosquitos infectados con bacterias, ¿por qué?</t>
         </is>
       </c>
       <c r="E114" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/politica/elecciones-colombia-2026/abelardo-de-la-espriella-se-afianzo-en-la-derecha-global-mientras-que-ivan-cepeda-se-bajo-del-bus-constituyente-noticias-hoy/</t>
+          <t>https://www.elespectador.com/ambiente/google-quiere-liberar-64-millones-de-mosquitos-infectados-con-bacterias-por-que/</t>
         </is>
       </c>
     </row>
@@ -3570,12 +3582,12 @@
       </c>
       <c r="D116" s="3" t="inlineStr">
         <is>
-          <t>Resultados de la Lotería de Bogotá jueves 4 de junio: números ganadores del premio mayor y los 50 secos millonarios</t>
+          <t>Hombre murió electrocutado en Medellín mientras huía tras una riña entre vecinos en Moravia</t>
         </is>
       </c>
       <c r="E116" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/05/resultados-de-la-loteria-de-bogota-jueves-4-de-junio-numeros-ganadores-del-premio-mayor-y-los-50-secos-millonarios/</t>
+          <t>https://www.infobae.com/colombia/2026/06/05/hombre-murio-electrocutado-en-medellin-mientras-huia-tras-una-rina-entre-vecinos-en-moravia/</t>
         </is>
       </c>
     </row>
@@ -3597,12 +3609,12 @@
       </c>
       <c r="D117" s="6" t="inlineStr">
         <is>
-          <t>Pilas: Así rotará el pico y placa en Bogotá este 5 de junio</t>
+          <t>Valle del Cauca declara emergencia humanitaria en salud por crisis en hospitales y servicios médicos</t>
         </is>
       </c>
       <c r="E117" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/05/pilas-asi-rotara-el-pico-y-placa-en-bogota-este-5-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/05/valle-del-cauca-declara-emergencia-humanitaria-en-salud-por-crisis-en-hospitales-y-servicios-medicos/</t>
         </is>
       </c>
     </row>
@@ -3624,12 +3636,12 @@
       </c>
       <c r="D118" s="3" t="inlineStr">
         <is>
-          <t>Resultado Super Astro Luna HOY: número ganador del jueves 4 de junio</t>
+          <t>Falsos policías asesinaron a joven de 19 años durante asalto en Palmira; dos personas más resultaron heridas</t>
         </is>
       </c>
       <c r="E118" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/05/resultado-super-astro-luna-hoy-numero-ganador-del-jueves-4-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/05/falsos-policias-asesinaron-a-joven-de-19-anos-durante-asalto-en-palmira-dos-personas-mas-resultaron-heridas/</t>
         </is>
       </c>
     </row>
@@ -3651,12 +3663,12 @@
       </c>
       <c r="D119" s="6" t="inlineStr">
         <is>
-          <t>Sinuano Día y Noche hoy jueves 4 de junio, revise aquí los números ganadores de esta lotería</t>
+          <t>¿Cuál es la temperatura promedio en Medellín?</t>
         </is>
       </c>
       <c r="E119" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/05/resultado-sinuano-noche-hoy-3-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/05/cual-es-la-temperatura-promedio-en-medellin/</t>
         </is>
       </c>
     </row>
@@ -3678,12 +3690,12 @@
       </c>
       <c r="D120" s="3" t="inlineStr">
         <is>
-          <t>Pico y Placa: qué vehículos descansan en Cartagena este viernes 5 de junio</t>
+          <t>¿Cómo estará el clima en Barranquilla?</t>
         </is>
       </c>
       <c r="E120" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/05/pico-y-placa-que-vehiculos-descansan-en-cartagena-este-viernes-5-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/05/como-estara-el-clima-en-barranquilla/</t>
         </is>
       </c>
     </row>
@@ -3705,12 +3717,12 @@
       </c>
       <c r="D121" s="6" t="inlineStr">
         <is>
-          <t>Pico y Placa: ¿Puedes manejar en Villavicencio sin infringir la ley?</t>
+          <t>Pronóstico del clima en Cartagena de Indias para este 5 de junio</t>
         </is>
       </c>
       <c r="E121" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/05/pico-y-placa-puedes-manejar-en-villavicencio-sin-infringir-la-ley/</t>
+          <t>https://www.infobae.com/colombia/2026/06/05/pronostico-del-clima-en-cartagena-de-indias-para-este-5-de-junio/</t>
         </is>
       </c>
     </row>
@@ -3732,12 +3744,12 @@
       </c>
       <c r="D122" s="3" t="inlineStr">
         <is>
-          <t>El Pico y Placa en Cali para este viernes 5 de junio</t>
+          <t>Colombia: las predicciones del tiempo en Bogotá este 5 de junio</t>
         </is>
       </c>
       <c r="E122" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/05/el-pico-y-placa-en-cali-para-este-viernes-5-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/05/colombia-las-predicciones-del-tiempo-en-bogota-este-5-de-junio/</t>
         </is>
       </c>
     </row>
@@ -3759,12 +3771,12 @@
       </c>
       <c r="D123" s="6" t="inlineStr">
         <is>
-          <t>Caribeña Noche, resultados ganadores del último sorteo de hoy jueves 4 de junio</t>
+          <t>Cali: la predicción del tiempo para este 5 de junio</t>
         </is>
       </c>
       <c r="E123" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/05/caribena-noche-resultados-ganadores-del-ultimo-sorteo-de-hoy-jueves-4-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/05/cali-la-prediccion-del-tiempo-para-este-5-de-junio/</t>
         </is>
       </c>
     </row>
@@ -3786,12 +3798,12 @@
       </c>
       <c r="D124" s="3" t="inlineStr">
         <is>
-          <t>Este es el Pico y Placa en Medellín para este viernes 5 de junio</t>
+          <t>Resultados de la Lotería de Bogotá jueves 4 de junio: números ganadores del premio mayor y los 50 secos millonarios</t>
         </is>
       </c>
       <c r="E124" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/05/este-es-el-pico-y-placa-en-medellin-para-este-viernes-5-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/05/resultados-de-la-loteria-de-bogota-jueves-4-de-junio-numeros-ganadores-del-premio-mayor-y-los-50-secos-millonarios/</t>
         </is>
       </c>
     </row>
@@ -3813,12 +3825,12 @@
       </c>
       <c r="D125" s="6" t="inlineStr">
         <is>
-          <t>Qué necesita Colombia para clasificar al Mundial femenino de Brasil 2027: cuentas, tabla y programación completa</t>
+          <t>Pilas: Así rotará el pico y placa en Bogotá este 5 de junio</t>
         </is>
       </c>
       <c r="E125" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/06/05/que-necesita-colombia-para-clasificar-al-mundial-femenino-de-brasil-2027-cuentas-tabla-y-programacion-completa/</t>
+          <t>https://www.infobae.com/colombia/2026/06/05/pilas-asi-rotara-el-pico-y-placa-en-bogota-este-5-de-junio/</t>
         </is>
       </c>
     </row>
@@ -3840,12 +3852,12 @@
       </c>
       <c r="D126" s="3" t="inlineStr">
         <is>
-          <t>Sismo hoy: se registró un temblor en El Tocuyo, Venezuela con magnitud 4.8</t>
+          <t>Resultado Super Astro Luna HOY: número ganador del jueves 4 de junio</t>
         </is>
       </c>
       <c r="E126" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/05/sismo-hoy-se-registro-un-temblor-en-el-tocuyo-venezuela-con-magnitud-48/</t>
+          <t>https://www.infobae.com/colombia/2026/06/05/resultado-super-astro-luna-hoy-numero-ganador-del-jueves-4-de-junio/</t>
         </is>
       </c>
     </row>
@@ -3867,12 +3879,12 @@
       </c>
       <c r="D127" s="6" t="inlineStr">
         <is>
-          <t>El polémico gesto de James Rodríguez con Antonella Petro desató la defensa de Nicolás Alcocer: “Ese no es el ejemplo”</t>
+          <t>Sinuano Día y Noche hoy jueves 4 de junio, revise aquí los números ganadores de esta lotería</t>
         </is>
       </c>
       <c r="E127" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/05/el-polemico-gesto-de-james-rodriguez-con-antonella-petro-desato-la-defensa-de-nicolas-alcocer-ese-no-es-el-ejemplo/</t>
+          <t>https://www.infobae.com/colombia/2026/06/05/resultado-sinuano-noche-hoy-3-de-junio/</t>
         </is>
       </c>
     </row>
@@ -3894,12 +3906,12 @@
       </c>
       <c r="D128" s="3" t="inlineStr">
         <is>
-          <t>Resultado Súper Chontico Millonario Noche hoy jueves 4 de junio</t>
+          <t>Pico y Placa: qué vehículos descansan en Cartagena este viernes 5 de junio</t>
         </is>
       </c>
       <c r="E128" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/05/resultado-super-chontico-millonario-noche-hoy-jueves-4-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/05/pico-y-placa-que-vehiculos-descansan-en-cartagena-este-viernes-5-de-junio/</t>
         </is>
       </c>
     </row>
@@ -3921,12 +3933,12 @@
       </c>
       <c r="D129" s="6" t="inlineStr">
         <is>
-          <t>La Fiscalía citó a imputación con medida de aseguramiento a Blessd y a su mánager por presunto secuestro extorsivo</t>
+          <t>Pico y Placa: ¿Puedes manejar en Villavicencio sin infringir la ley?</t>
         </is>
       </c>
       <c r="E129" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/05/la-fiscalia-cito-a-imputacion-con-medida-de-aseguramiento-a-blessd-y-a-su-manager-por-presunto-secuestro-extorsivo/</t>
+          <t>https://www.infobae.com/colombia/2026/06/05/pico-y-placa-puedes-manejar-en-villavicencio-sin-infringir-la-ley/</t>
         </is>
       </c>
     </row>
@@ -3948,12 +3960,12 @@
       </c>
       <c r="D130" s="3" t="inlineStr">
         <is>
-          <t>El Gobierno nacional destinó más de $700.000 millones para modernizar 30 universidades públicas en Colombia: reveló las zonas beneficiadas</t>
+          <t>El Pico y Placa en Cali para este viernes 5 de junio</t>
         </is>
       </c>
       <c r="E130" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/05/el-gobierno-nacional-destino-mas-de-700000-millones-para-modernizar-30-universidades-publicas-en-colombia-revelo-las-zonas-beneficiadas/</t>
+          <t>https://www.infobae.com/colombia/2026/06/05/el-pico-y-placa-en-cali-para-este-viernes-5-de-junio/</t>
         </is>
       </c>
     </row>
@@ -3975,12 +3987,12 @@
       </c>
       <c r="D131" s="6" t="inlineStr">
         <is>
-          <t>Los 10 jugadores más valiosos de la Liga BetPlay en el mercado de fichajes, según un reciente estudio</t>
+          <t>Caribeña Noche, resultados ganadores del último sorteo de hoy jueves 4 de junio</t>
         </is>
       </c>
       <c r="E131" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/06/05/los-10-jugadores-mas-valiosos-de-la-liga-betplay-en-el-mercado-de-fichajes-segun-un-reciente-estudio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/05/caribena-noche-resultados-ganadores-del-ultimo-sorteo-de-hoy-jueves-4-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4002,12 +4014,12 @@
       </c>
       <c r="D132" s="3" t="inlineStr">
         <is>
-          <t>Exesposa de Santiago Botero cuestionó denuncia de violencia intrafamiliar interpuesta por Manuela Echeverri: “Nunca me levantó la mano”</t>
+          <t>Este es el Pico y Placa en Medellín para este viernes 5 de junio</t>
         </is>
       </c>
       <c r="E132" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/05/exesposa-de-santiago-botero-cuestiono-denuncia-de-violencia-intrafamiliar-interpuesta-por-manuela-echeverri-nunca-me-levanto-la-mano/</t>
+          <t>https://www.infobae.com/colombia/2026/06/05/este-es-el-pico-y-placa-en-medellin-para-este-viernes-5-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4029,12 +4041,12 @@
       </c>
       <c r="D133" s="6" t="inlineStr">
         <is>
-          <t>Alcaldía de Medellín declaró alerta naranja para atender emergencias por el fenómeno de El Niño</t>
+          <t>Qué necesita Colombia para clasificar al Mundial femenino de Brasil 2027: cuentas, tabla y programación completa</t>
         </is>
       </c>
       <c r="E133" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/05/alcaldia-de-medellin-declaro-alerta-naranja-para-atender-emergencias-por-el-fenomeno-de-el-nino/</t>
+          <t>https://www.infobae.com/colombia/deportes/2026/06/05/que-necesita-colombia-para-clasificar-al-mundial-femenino-de-brasil-2027-cuentas-tabla-y-programacion-completa/</t>
         </is>
       </c>
     </row>
@@ -4056,12 +4068,12 @@
       </c>
       <c r="D134" s="3" t="inlineStr">
         <is>
-          <t>Este es el equipo de Antonella Petro, la hija de Gustavo Petro que protagonizó un momento viral con James Rodríguez</t>
+          <t>Sismo hoy: se registró un temblor en El Tocuyo, Venezuela con magnitud 4.8</t>
         </is>
       </c>
       <c r="E134" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/05/este-es-el-equipo-de-antonella-petro-la-hija-de-gustavo-petro-que-protagonizo-un-momento-viral-con-james-rodriguez/</t>
+          <t>https://www.infobae.com/colombia/2026/06/05/sismo-hoy-se-registro-un-temblor-en-el-tocuyo-venezuela-con-magnitud-48/</t>
         </is>
       </c>
     </row>
@@ -4083,12 +4095,12 @@
       </c>
       <c r="D135" s="6" t="inlineStr">
         <is>
-          <t>Sede de Abelardo de la Espriella en Bogotá fue blanco de hostigamientos: protagonistas de los incidentes serían seguidores de Iván Cepeda</t>
+          <t>El polémico gesto de James Rodríguez con Antonella Petro desató la defensa de Nicolás Alcocer: “Ese no es el ejemplo”</t>
         </is>
       </c>
       <c r="E135" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/05/sede-de-abelardo-de-la-espriella-en-bogota-fue-blanco-de-hostigamientos-protagonistas-de-los-incidentes-serian-seguidores-de-ivan-cepeda/</t>
+          <t>https://www.infobae.com/colombia/2026/06/05/el-polemico-gesto-de-james-rodriguez-con-antonella-petro-desato-la-defensa-de-nicolas-alcocer-ese-no-es-el-ejemplo/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 Noticias actualizadas 11/06/2026 09:02
</commit_message>
<xml_diff>
--- a/docs/ultimahora.xlsx
+++ b/docs/ultimahora.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Todas las noticias" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Todas las noticias'!$A$1:$E$284</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Todas las noticias'!$A$1:$E$282</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -38,7 +38,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -58,16 +58,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFEF5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F5FBFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EAF2FB"/>
       </patternFill>
     </fill>
   </fills>
@@ -97,7 +87,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -118,24 +108,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -503,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E284"/>
+  <dimension ref="A1:E282"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -543,7 +515,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 02:06 a. m.</t>
+          <t>11/06/2026 03:30 a. m.</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -558,19 +530,19 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Irán afirmó que convertirá Oriente Medio en un 'infierno' para Estados Unidos</t>
+          <t>Elecciones presidenciales de Colombia 2026: fecha, candidatos, fórmulas vicepresidenciales y todo sobre la segunda vuelta electoral</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/medio-oriente/iran-afirmo-que-convertira-oriente-medio-en-un-infierno-para-estados-unidos-3563532</t>
+          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/elecciones-presidenciales-de-colombia-2026-fecha-candidatos-formulas-vicepresidenciales-y-todo-sobre-la-segunda-vuelta-electoral-3563537</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>11/06/2026 01:30 a. m.</t>
+          <t>11/06/2026 02:57 a. m.</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -585,19 +557,19 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>Inauguración del Mundial 2026: Show inaugural, artistas, horario y todas las presentaciones en la Ciudad de México</t>
+          <t>México vs Sudáfrica: siga el minuto a minuto del partido inaugural del grupo A en el Mundial 2026</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/inauguracion-del-mundial-2026-show-inaugural-artistas-horario-y-todas-las-presentaciones-en-la-ciudad-de-mexico-3563530</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/mexico-vs-sudafrica-siga-el-minuto-a-minuto-del-partido-inaugural-del-grupo-a-en-el-mundial-3563536</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 01:01 a. m.</t>
+          <t>11/06/2026 02:55 a. m.</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -612,19 +584,19 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>A cinco meses de la caída de Maduro, el chavismo se reorganiza, afianza el autoritarismo y frena la democracia en Venezuela: ¿se agotó la transición?</t>
+          <t>Video | Así quedó el vehículo que fue impactado por un artefacto explosivo cuando pasaba por Univalle: 'Mi niñita venía en este carro'</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/venezuela/a-cinco-meses-de-la-caida-de-maduro-el-chavismo-se-reorganiza-afianza-el-autoritarismo-y-frena-la-democracia-en-venezuela-se-agoto-la-transicion-3563051</t>
+          <t>https://www.eltiempo.com/colombia/cali/video-asi-quedo-el-vehiculo-que-fue-impactado-por-un-artefacto-explosivo-cuando-pasaba-por-univalle-mi-ninita-venia-en-este-carro-3563535</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>11/06/2026 12:01 a. m.</t>
+          <t>11/06/2026 02:37 a. m.</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -639,19 +611,19 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>El recrudecimiento de la violencia vuelve a golpear a Colombia: el país cae en Índice Global de Paz y se mantiene como el menos pacífico de Sudamérica</t>
+          <t>Familias de desaparecidos en México desafían cerco del Mundial a horas de la inauguración: 'La pelota regresa a casa, ¿nuestros desaparecidos cuándo?'</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/latinoamerica/el-recrudecimiento-de-la-violencia-vuelve-a-golpear-a-colombia-el-pais-cae-en-indice-global-de-paz-y-se-mantiene-como-el-menos-pacifico-de-sudamerica-3563436</t>
+          <t>https://www.eltiempo.com/mundo/mexico/familias-de-desaparecidos-en-mexico-desafian-cerco-del-mundial-a-horas-de-la-inauguracion-la-pelota-regresa-a-casa-nuestros-desaparecidos-cuando-3563534</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 11:32 p. m.</t>
+          <t>11/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -666,19 +638,19 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Con la mayor remontada de la historia de las finales, New York Knicks quedó a un triunfo del campeonato de la NBA</t>
+          <t>¡Atención, conductores! Pico y placa en Pereira para el jueves 11 de junio de 2026: así regirá la medida</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/otros-deportes/con-la-mayor-remontada-de-la-historia-de-las-finales-new-york-knicks-quedo-a-un-triunfo-del-campeonato-de-la-nba-3563531</t>
+          <t>https://www.eltiempo.com/colombia/otras-ciudades/atencion-conductores-pico-y-placa-en-pereira-para-el-jueves-11-de-junio-de-2026-asi-regira-la-medida-3563385</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>10/06/2026 11:18 p. m.</t>
+          <t>11/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -693,19 +665,19 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Comienza el Inter Rapidísimo Golf Championship: siete colombianos, por la victoria en el club El Rincón</t>
+          <t>¡Evite contratiempos! Pico y placa en Bucaramanga para el jueves 11 de junio de 2026</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/otros-deportes/comienza-el-inter-rapidisimo-golf-championship-siete-colombianos-por-la-victoria-en-el-club-el-rincon-3563529</t>
+          <t>https://www.eltiempo.com/colombia/santander/evite-contratiempos-pico-y-placa-en-bucaramanga-para-el-jueves-11-de-junio-de-3563383</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 11:11 p. m.</t>
+          <t>11/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -720,19 +692,19 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Alertan que señalados asesinos de Sara Millerey en Bello, Antioquia, podrían quedar en libertad: esto denunció la familia de la víctima</t>
+          <t>¡Siga la medida de movilidad! Pico y placa en Medellín para el jueves 11 de junio de 2026: así funciona la restricción</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/medellin/alertan-que-senalados-asesinos-de-sara-millerey-en-antioquia-podrian-quedar-en-libertad-esto-dijo-la-familia-de-la-victima-3563528</t>
+          <t>https://www.eltiempo.com/colombia/medellin/siga-la-medida-de-movilidad-pico-y-placa-en-medellin-para-el-jueves-11-de-junio-de-2026-asi-funciona-la-restriccion-3563381</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>10/06/2026 10:55 p. m.</t>
+          <t>11/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -747,19 +719,19 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Esta sería la causa de muerte de empresario costarricense que había sido reportado como desaparecido en Bogotá: familia habló tras hallazgo del cuerpo</t>
+          <t>¡Pilas en las vías! Pico y placa en Bogotá para el jueves 11 de junio de 2026</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/bogota/esta-seria-la-causa-de-muerte-de-empresario-costarricense-que-habia-sido-reportado-como-desaparecido-en-bogota-familia-hablo-tras-hallazgo-del-cuerpo-3563461</t>
+          <t>https://www.eltiempo.com/bogota/pilas-en-las-vias-pico-y-placa-en-bogota-para-el-jueves-11-de-junio-de-3563376</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 10:50 p. m.</t>
+          <t>11/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -774,19 +746,19 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Mario Mendoza, el ‘rock star’de la literatura colombiana</t>
+          <t>¡Evite multas! Pico y placa en Cali para el jueves 11 de junio de 2026: así opera la medida</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/cultura/musica-y-libros/mario-mendoza-el-rock-star-de-la-literatura-colombiana-3563521</t>
+          <t>https://www.eltiempo.com/colombia/cali/evite-multas-pico-y-placa-en-cali-para-el-jueves-11-de-junio-de-2026-asi-opera-la-medida-3563374</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>10/06/2026 10:43 p. m.</t>
+          <t>11/06/2026 02:06 a. m.</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -801,19 +773,19 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Gianni Infantino, presidente de Fifa, y la insólita historia del periodista que se acreditó para el Mundial y está en prisión: 'Hay una plaza libre'</t>
+          <t>Irán afirmó que convertirá Oriente Medio en un 'infierno' para Estados Unidos</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/gianni-infantino-presidente-de-fifa-y-la-insolita-historia-del-periodista-que-se-acredito-para-el-mundial-y-esta-en-prision-hay-una-plaza-libre-3563527</t>
+          <t>https://www.eltiempo.com/mundo/medio-oriente/iran-afirmo-que-convertira-oriente-medio-en-un-infierno-para-estados-unidos-3563532</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 10:42 p. m.</t>
+          <t>11/06/2026 01:30 a. m.</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -828,19 +800,19 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Motociclista atropelló a un agente de tránsito cuando intentaba escapar de un puesto de control en Bogotá; video captó el momento exacto del accidente</t>
+          <t>Inauguración del Mundial 2026: Show inaugural, artistas, horario y todas las presentaciones en la Ciudad de México</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/bogota/motociclista-atropello-a-un-agente-de-transito-luego-de-evadir-un-puesto-de-control-en-bogota-el-conductor-cayo-al-piso-metros-despues-3563522</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/inauguracion-del-mundial-2026-show-inaugural-artistas-horario-y-todas-las-presentaciones-en-la-ciudad-de-mexico-3563530</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>10/06/2026 10:33 p. m.</t>
+          <t>11/06/2026 01:01 a. m.</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -855,19 +827,19 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Terremoto en Filipinas y México: La ciencia detrás del Cinturón de Fuego</t>
+          <t>A cinco meses de la caída de Maduro, el chavismo se reorganiza, afianza el autoritarismo y frena la democracia en Venezuela: ¿se agotó la transición?</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/vida/ciencia/terremoto-en-filipinas-y-mexico-la-ciencia-detras-del-cinturon-de-fuego-3563526</t>
+          <t>https://www.eltiempo.com/mundo/venezuela/a-cinco-meses-de-la-caida-de-maduro-el-chavismo-se-reorganiza-afianza-el-autoritarismo-y-frena-la-democracia-en-venezuela-se-agoto-la-transicion-3563051</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 10:31 p. m.</t>
+          <t>11/06/2026 12:01 a. m.</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -882,19 +854,19 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Los cinco duelos imperdibles que marcarán la fase de grupos del Mundial 2026: prográmese y disfrute</t>
+          <t>El recrudecimiento de la violencia vuelve a golpear a Colombia: el país cae en Índice Global de Paz y se mantiene como el menos pacífico de Sudamérica</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/los-cinco-duelos-imperdibles-que-marcaran-la-fase-de-grupos-del-mundial-2026-programese-y-disfrute-3563525</t>
+          <t>https://www.eltiempo.com/mundo/latinoamerica/el-recrudecimiento-de-la-violencia-vuelve-a-golpear-a-colombia-el-pais-cae-en-indice-global-de-paz-y-se-mantiene-como-el-menos-pacifico-de-sudamerica-3563436</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>10/06/2026 10:30 p. m.</t>
+          <t>10/06/2026 11:32 p. m.</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -909,19 +881,19 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Alcaldía de Bogotá anuncia horarios de ley seca para el fin de semana de la segunda vuelta presidencial: comenzará en la tarde del viernes 19 de junio</t>
+          <t>Con la mayor remontada de la historia de las finales, New York Knicks quedó a un triunfo del campeonato de la NBA</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/alcaldia-de-bogota-anuncia-horarios-de-ley-seca-para-el-fin-de-semana-de-la-segunda-vuelta-presidencial-comenzara-en-la-tarde-del-viernes-19-de-junio-3563523</t>
+          <t>https://www.eltiempo.com/deportes/otros-deportes/con-la-mayor-remontada-de-la-historia-de-las-finales-new-york-knicks-quedo-a-un-triunfo-del-campeonato-de-la-nba-3563531</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 10:30 p. m.</t>
+          <t>10/06/2026 11:18 p. m.</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -936,19 +908,19 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Estos son los diez países más pacíficos del mundo, según el Índice Global de Paz 2026; la gran mayoría pertenece a la misma región</t>
+          <t>Comienza el Inter Rapidísimo Golf Championship: siete colombianos, por la victoria en el club El Rincón</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/mas-regiones/estos-son-los-diez-paises-mas-pacificos-del-mundo-segun-el-indice-global-de-paz-2026-la-gran-mayoria-pertenece-a-la-misma-region-3563402</t>
+          <t>https://www.eltiempo.com/deportes/otros-deportes/comienza-el-inter-rapidisimo-golf-championship-siete-colombianos-por-la-victoria-en-el-club-el-rincon-3563529</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>10/06/2026 10:30 p. m.</t>
+          <t>10/06/2026 11:11 p. m.</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -963,19 +935,19 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>Ni estudiantes ni profesionales: proyecto republicano endurece acceso a residencia para migrantes legales a EE. UU. y afectaría a miles de colombianos</t>
+          <t>Alertan que señalados asesinos de Sara Millerey en Bello, Antioquia, podrían quedar en libertad: esto denunció la familia de la víctima</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/ni-estudiantes-ni-profesionales-proyecto-republicano-endurece-acceso-a-residencia-para-migrantes-legales-a-ee-uu-y-afectaria-a-miles-de-colombianos-3563272</t>
+          <t>https://www.eltiempo.com/colombia/medellin/alertan-que-senalados-asesinos-de-sara-millerey-en-antioquia-podrian-quedar-en-libertad-esto-dijo-la-familia-de-la-victima-3563528</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 10:20 p. m.</t>
+          <t>10/06/2026 10:55 p. m.</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -990,19 +962,19 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Ana Guzmán, la heroína de la Selección Colombia campeona de la Liga de Naciones de la Conmebol</t>
+          <t>Esta sería la causa de muerte de empresario costarricense que había sido reportado como desaparecido en Bogotá: familia habló tras hallazgo del cuerpo</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/ana-guzman-la-heroina-de-la-seleccion-colombia-campeona-de-la-liga-de-naciones-de-la-conmebol-3563524</t>
+          <t>https://www.eltiempo.com/bogota/esta-seria-la-causa-de-muerte-de-empresario-costarricense-que-habia-sido-reportado-como-desaparecido-en-bogota-familia-hablo-tras-hallazgo-del-cuerpo-3563461</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>10/06/2026 10:15 p. m.</t>
+          <t>10/06/2026 10:50 p. m.</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -1017,19 +989,19 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Mundial de la Fifa 2026: estos son los precios por asiento más caros que tendrá la Copa del Mundo; un partido de Colombia hace parte de la lista</t>
+          <t>Mario Mendoza, el ‘rock star’de la literatura colombiana</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/mundial-de-la-fifa-2026-estos-son-los-precios-por-asiento-mas-caros-que-tendra-la-copa-del-mundo-un-partido-de-colombia-hace-parte-de-la-lista-3563324</t>
+          <t>https://www.eltiempo.com/cultura/musica-y-libros/mario-mendoza-el-rock-star-de-la-literatura-colombiana-3563521</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 10:01 p. m.</t>
+          <t>10/06/2026 10:43 p. m.</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1044,19 +1016,19 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Llegó el Mundial</t>
+          <t>Gianni Infantino, presidente de Fifa, y la insólita historia del periodista que se acreditó para el Mundial y está en prisión: 'Hay una plaza libre'</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/caricaturas/llego-el-mundial-3563505</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/gianni-infantino-presidente-de-fifa-y-la-insolita-historia-del-periodista-que-se-acredito-para-el-mundial-y-esta-en-prision-hay-una-plaza-libre-3563527</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>10/06/2026 10:01 p. m.</t>
+          <t>10/06/2026 10:42 p. m.</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
@@ -1071,12 +1043,12 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Infraestructura vial</t>
+          <t>Motociclista atropelló a un agente de tránsito cuando intentaba escapar de un puesto de control en Bogotá; video captó el momento exacto del accidente</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/caricaturas/infraestructura-vial-3563504</t>
+          <t>https://www.eltiempo.com/bogota/motociclista-atropello-a-un-agente-de-transito-luego-de-evadir-un-puesto-de-control-en-bogota-el-conductor-cayo-al-piso-metros-despues-3563522</t>
         </is>
       </c>
     </row>
@@ -1623,7 +1595,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 06:43 a. m.</t>
+          <t>11/06/2026 07:54 a. m.</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -1638,19 +1610,19 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>Santiago Uribe se entregó a la Policía tras quedar en firme su condena por ‘Los doce apóstoles’</t>
+          <t>Petro regresa a Nueva York tras la polémica que desató tensiones con Estados Unidos</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/10/santiago-uribe-se-entrego-a-la-policia-tras-quedar-en-firme-su-condena-por-los-doce-apostoles/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/10/petro-regresa-a-nueva-york-tras-la-polemica-que-desato-tensiones-con-estados-unidos/</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>11/06/2026 01:00 a. m.</t>
+          <t>11/06/2026 07:35 a. m.</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
@@ -1665,19 +1637,19 @@
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>La reflexión de Obaldía</t>
+          <t>Temblor en Santander: sismo sacudió Los Santos este miércoles</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/11/la-reflexion-de-obaldia/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/10/temblor-en-santander-sismo-sacudio-los-santos-este-miercoles/</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 01:00 a. m.</t>
+          <t>11/06/2026 06:43 a. m.</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -1692,12 +1664,12 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Columnistas</t>
+          <t>Santiago Uribe se entregó a la Policía tras quedar en firme su condena por ‘Los doce apóstoles’</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/10/santiago-uribe-se-entrego-a-la-policia-tras-quedar-en-firme-su-condena-por-los-doce-apostoles/</t>
         </is>
       </c>
     </row>
@@ -1719,12 +1691,12 @@
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>¿Qué hay detrás del intento de suspender a Petro?</t>
+          <t>La reflexión de Obaldía</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/editorial/2026/06/11/que-hay-detras-del-intento-de-suspender-a-petro/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/11/la-reflexion-de-obaldia/</t>
         </is>
       </c>
     </row>
@@ -1746,12 +1718,12 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Editorial</t>
+          <t>Columnistas</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/editorial/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/</t>
         </is>
       </c>
     </row>
@@ -1773,12 +1745,12 @@
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>El orgullo también es nuestro</t>
+          <t>¿Qué hay detrás del intento de suspender a Petro?</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/11/el-orgullo-tambien-es-nuestro/</t>
+          <t>https://www.vanguardia.com/opinion/editorial/2026/06/11/que-hay-detras-del-intento-de-suspender-a-petro/</t>
         </is>
       </c>
     </row>
@@ -1800,19 +1772,19 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Todos necesitamos una cancha</t>
+          <t>Editorial</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/11/todos-necesitamos-una-cancha/</t>
+          <t>https://www.vanguardia.com/opinion/editorial/</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>10/06/2026 09:15 p. m.</t>
+          <t>11/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
@@ -1827,19 +1799,19 @@
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>ONU pide a Colombia garantizar justicia y reparación a personas afectadas por lepra</t>
+          <t>El orgullo también es nuestro</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/10/onu-pide-a-colombia-garantizar-justicia-y-reparacion-a-personas-afectadas-por-lepra/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/11/el-orgullo-tambien-es-nuestro/</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 09:15 p. m.</t>
+          <t>11/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -1854,19 +1826,19 @@
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Todos necesitamos una cancha</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/11/todos-necesitamos-una-cancha/</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>10/06/2026 08:45 p. m.</t>
+          <t>10/06/2026 09:15 p. m.</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
@@ -1881,19 +1853,19 @@
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>Encuesta de AtlasIntel muestra  intención de voto para segunda vuelta</t>
+          <t>ONU pide a Colombia garantizar justicia y reparación a personas afectadas por lepra</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/10/encuesta-de-atlasintel-muestra-intencion-de-voto-para-segunda-vuelta/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/10/onu-pide-a-colombia-garantizar-justicia-y-reparacion-a-personas-afectadas-por-lepra/</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 06:23 p. m.</t>
+          <t>10/06/2026 09:15 p. m.</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -1908,19 +1880,19 @@
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Reportan explosivos contra vehículos cerca de la Universidad del Valle en Cali</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/10/reportan-explosivos-contra-vehiculos-cerca-de-la-universidad-del-valle-en-cali/</t>
+          <t>https://www.vanguardia.com/colombia/</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>10/06/2026 05:56 p. m.</t>
+          <t>10/06/2026 08:45 p. m.</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
@@ -1935,19 +1907,19 @@
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>Supersalud lanza advertencia por graves fallas en entrega de medicamentos en Pasto</t>
+          <t>Encuesta de AtlasIntel muestra  intención de voto para segunda vuelta</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/10/supersalud-lanza-advertencia-por-graves-fallas-en-entrega-de-medicamentos-en-pasto/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/10/encuesta-de-atlasintel-muestra-intencion-de-voto-para-segunda-vuelta/</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 10:00 a. m.</t>
+          <t>10/06/2026 06:23 p. m.</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -1962,19 +1934,19 @@
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>Gustavo Petro habla ante la ONU sobre conflictos internacionales y cambio climático</t>
+          <t>Reportan explosivos contra vehículos cerca de la Universidad del Valle en Cali</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/10/gustavo-petro-habla-ante-la-onu-sobre-conflictos-internacionales-y-cambio-climatico/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/10/reportan-explosivos-contra-vehiculos-cerca-de-la-universidad-del-valle-en-cali/</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>10/06/2026 09:42 a. m.</t>
+          <t>10/06/2026 05:56 p. m.</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
@@ -1989,19 +1961,19 @@
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>“Solo el Senado puede suspender al Presidente”: Benedetti a medida contra  Petro</t>
+          <t>Supersalud lanza advertencia por graves fallas en entrega de medicamentos en Pasto</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/politica/2026/06/10/solo-el-senado-puede-suspender-al-presidente-benedetti-a-medida-contra-petro/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/10/supersalud-lanza-advertencia-por-graves-fallas-en-entrega-de-medicamentos-en-pasto/</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 09:42 a. m.</t>
+          <t>10/06/2026 10:00 a. m.</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -2016,19 +1988,19 @@
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Política</t>
+          <t>Gustavo Petro habla ante la ONU sobre conflictos internacionales y cambio climático</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/politica/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/10/gustavo-petro-habla-ante-la-onu-sobre-conflictos-internacionales-y-cambio-climatico/</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>10/06/2026 09:05 a. m.</t>
+          <t>10/06/2026 09:42 a. m.</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
@@ -2043,19 +2015,19 @@
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>El pacífico colombiano recibirá más de ocho mil ballenas en temporada 2026</t>
+          <t>“Solo el Senado puede suspender al Presidente”: Benedetti a medida contra  Petro</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/10/el-pacifico-colombiano-recibira-mas-de-ocho-mil-ballenas-en-temporada-2026/</t>
+          <t>https://www.vanguardia.com/politica/2026/06/10/solo-el-senado-puede-suspender-al-presidente-benedetti-a-medida-contra-petro/</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 07:54 a. m.</t>
+          <t>10/06/2026 09:42 a. m.</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -2070,19 +2042,19 @@
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Petro regresa a Nueva York tras la polémica que desató tensiones con Estados Unidos</t>
+          <t>Política</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/10/petro-regresa-a-nueva-york-tras-la-polemica-que-desato-tensiones-con-estados-unidos/</t>
+          <t>https://www.vanguardia.com/politica/</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>10/06/2026 07:35 a. m.</t>
+          <t>10/06/2026 09:05 a. m.</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
@@ -2097,12 +2069,12 @@
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>Temblor en Santander: sismo sacudió Los Santos este miércoles</t>
+          <t>El pacífico colombiano recibirá más de ocho mil ballenas en temporada 2026</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/10/temblor-en-santander-sismo-sacudio-los-santos-este-miercoles/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/10/el-pacifico-colombiano-recibira-mas-de-ocho-mil-ballenas-en-temporada-2026/</t>
         </is>
       </c>
     </row>
@@ -2641,7 +2613,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 02:03 a. m.</t>
+          <t>11/06/2026 04:00 a. m.</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -2656,19 +2628,19 @@
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>Visita del papa León XIV, en directo | El Pontífice llega este jueves a las islas Canarias</t>
+          <t>Inauguración de la Copa Mundial de fútbol 2026: últimas noticias en directo</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/espana/2026-06-11/visita-del-papa-leon-xiv-en-directo.html</t>
+          <t>https://elpais.com/deportes/mundial-futbol/2026-06-11/inauguracion-de-la-copa-mundial-de-futbol-resumen-y-ultimas-noticias.html</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>11/06/2026 02:00 a. m.</t>
+          <t>11/06/2026 03:46 a. m.</t>
         </is>
       </c>
       <c r="B81" s="5" t="inlineStr">
@@ -2683,19 +2655,19 @@
       </c>
       <c r="D81" s="6" t="inlineStr">
         <is>
-          <t>Última hora de la Copa Mundial de fútbol en directo | Estados Unidos, México y Canadá se preparan para el inicio del torneo hoy jueves</t>
+          <t>Visita del papa León XIV, en directo | El Pontífice llega este jueves a las islas Canarias</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/deportes/mundial-futbol/2026-06-10/ultima-hora-de-la-copa-mundial-de-futbol.html</t>
+          <t>https://elpais.com/espana/2026-06-11/visita-del-papa-leon-xiv-en-directo.html</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 01:58 a. m.</t>
+          <t>11/06/2026 03:35 a. m.</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -2710,19 +2682,19 @@
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>Mueren dos personas en un incendio en un bloque de viviendas de Magaluf (Mallorca)</t>
+          <t>La revancha de Amy Adams: cómo la eterna nominada al Oscar intenta escapar de su “era de fracasos”</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/espana/2026-06-11/mueren-dos-personas-en-un-incendio-en-un-bloque-de-viviendas-de-magaluf-mallorca.html</t>
+          <t>https://elpais.com/smoda/famosos/2026-06-11/la-revancha-de-amy-adams-como-la-eterna-nominada-al-oscar-intenta-escapar-de-su-era-de-fracasos.html</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>11/06/2026 01:24 a. m.</t>
+          <t>11/06/2026 03:34 a. m.</t>
         </is>
       </c>
       <c r="B83" s="5" t="inlineStr">
@@ -2737,19 +2709,19 @@
       </c>
       <c r="D83" s="6" t="inlineStr">
         <is>
-          <t>Indignación entre los 600 cantantes expulsados de la Sagrada Familia: “Por tres o cuatro estelades, todos castigados”</t>
+          <t>Una escuela pública infantil del centro de Madrid lleva desde enero con una plaga de cucarachas: pidió ayuda al Gobierno sin éxito</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/espana/catalunya/2026-06-11/indignacion-entre-los-600-cantantes-expulsados-de-la-sagrada-familia-por-tres-o-cuatro-estelades-todos-castigados.html</t>
+          <t>https://elpais.com/espana/madrid/2026-06-11/una-escuela-publica-infantil-del-centro-de-madrid-lleva-desde-enero-con-una-plaga-de-cucarachas-pidio-ayuda-al-gobierno-sin-exito.html</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 12:25 a. m.</t>
+          <t>11/06/2026 03:17 a. m.</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -2764,19 +2736,19 @@
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>Analizamos cuatro camas refrescantes para perros</t>
+          <t>Una propuesta digital que concede privilegios únicos a los amantes del deporte</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/hemeroteca/2026-06-11/</t>
+          <t>https://elpais.com/sociedad/2026-06-11/una-propuesta-digital-que-concede-privilegios-unicos-a-los-amantes-del-deporte.html</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>11/06/2026 12:20 a. m.</t>
+          <t>11/06/2026 03:11 a. m.</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr">
@@ -2791,19 +2763,19 @@
       </c>
       <c r="D85" s="6" t="inlineStr">
         <is>
-          <t>Última hora de la guerra de Estados Unidos e Israel contra Irán, en directo | EE UU e Irán intercambian ataques por segundo día consecutivo</t>
+          <t>Juan Echanove sobre su salida de ‘Cuéntame’: “Eso no es un motivo argumental, eso es una putada”</t>
         </is>
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/internacional/2026-06-11/ultima-hora-de-la-guerra-de-estados-unidos-e-israel-contra-iran-en-directo.html</t>
+          <t>https://elpais.com/television/2026-06-11/juan-echanove-sobre-su-salida-de-cuentame-eso-no-es-un-motivo-argumental-eso-es-una-putada.html</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 12:00 a. m.</t>
+          <t>11/06/2026 03:02 a. m.</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -2818,19 +2790,19 @@
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>Alexandra Lange, Pulitzer de Crítica 2025: “Hemos hecho la infancia demasiado segura”</t>
+          <t>Hallada la mitad de un cuerpo humano en avanzado estado de descomposición en la playa de El Saler de Valencia</t>
         </is>
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/economia/formacion/2026-06-11/alexandra-lange-pulitzer-de-critica-2025-hemos-hecho-la-infancia-demasiado-segura.html</t>
+          <t>https://elpais.com/espana/comunidad-valenciana/2026-06-11/hallada-la-mitad-de-un-cuerpo-humano-en-avanzado-estado-de-descomposicion-en-la-playa-de-el-saler-de-valencia.html</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>11/06/2026 12:00 a. m.</t>
+          <t>11/06/2026 03:00 a. m.</t>
         </is>
       </c>
       <c r="B87" s="5" t="inlineStr">
@@ -2845,19 +2817,19 @@
       </c>
       <c r="D87" s="6" t="inlineStr">
         <is>
-          <t>Los seis destinos en África para ver este año con EL PAÍS Viajes</t>
+          <t>Vox advierte a Ayuso: “¿Sabe lo que tiene límite? Las mayorías absolutas”</t>
         </is>
       </c>
       <c r="E87" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/elviajero/viajes/2026-06-11/los-seis-destinos-en-africa-para-ver-este-ano-con-el-pais-viajes.html</t>
+          <t>https://elpais.com/espana/madrid/2026-06-11/ayuso-y-la-oposicion-ponen-a-prueba-en-la-asamblea-de-madrid-el-mensaje-que-dejo-el-papa.html</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 12:00 a. m.</t>
+          <t>11/06/2026 02:59 a. m.</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -2872,19 +2844,19 @@
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>Visita del Papa León XIV a Canarias: agenda del pontífice en su viaje por España</t>
+          <t>Taylor Swift, Timothée Chalamet y otros famosos que han vibrado con la remontada de los Knicks</t>
         </is>
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/espana/2026-06-11/visita-del-papa-leon-xiv-a-canarias-agenda-del-pontifice-en-su-viaje-por-espana.html</t>
+          <t>https://elpais.com/gente/2026-06-11/taylor-swift-timothee-chalamet-y-otros-famosos-que-han-vibrado-con-la-remontada-de-los-knicks.html</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>10/06/2026 11:56 p. m.</t>
+          <t>11/06/2026 02:47 a. m.</t>
         </is>
       </c>
       <c r="B89" s="5" t="inlineStr">
@@ -2899,19 +2871,19 @@
       </c>
       <c r="D89" s="6" t="inlineStr">
         <is>
-          <t>Los Knicks acarician el campeonato de la NBA frente a los Spurs tras la mayor remontada de la historia</t>
+          <t>Fallece un niño de dos años ahogado en una piscina hinchable en una vivienda de Almazán, Soria</t>
         </is>
       </c>
       <c r="E89" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/deportes/baloncesto/2026-06-11/los-knicks-acarician-el-campeonato-de-la-nba-frente-a-los-spurs-tras-la-mayor-remontada-de-la-historia.html</t>
+          <t>https://elpais.com/espana/2026-06-11/fallece-un-nino-de-dos-anos-ahogado-en-una-piscina-hinchable-en-una-vivienda-de-almazan-soria.html</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 11:45 p. m.</t>
+          <t>11/06/2026 02:07 a. m.</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -2926,19 +2898,19 @@
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>Un muro de policía para evitar que Jonathan, Olin, Ana o Mayra lleguen al Estadio Azteca</t>
+          <t>I el Papa va parlar en català</t>
         </is>
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/mexico/2026-06-11/un-muro-de-policia-para-evitar-que-jonathan-olin-ana-o-mayra-lleguen-al-estadio-azteca.html</t>
+          <t>https://elpais.com/quadern/2026-06-11/i-el-papa-va-parlar-en-catala.html</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>10/06/2026 11:15 p. m.</t>
+          <t>11/06/2026 01:58 a. m.</t>
         </is>
       </c>
       <c r="B91" s="5" t="inlineStr">
@@ -2953,19 +2925,19 @@
       </c>
       <c r="D91" s="6" t="inlineStr">
         <is>
-          <t>Fujimori se aferra al voto de los peruanos en el exterior en su remontada contra Sánchez</t>
+          <t>Mueren dos personas y una permanece grave tras un incendio en un edificio en Magaluf</t>
         </is>
       </c>
       <c r="E91" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/america/2026-06-11/fujimori-se-aferra-al-voto-de-los-peruanos-en-el-exterior-para-una-remontada-contra-sanchez.html</t>
+          <t>https://elpais.com/espana/2026-06-11/mueren-dos-personas-en-un-incendio-en-un-bloque-de-viviendas-de-magaluf-mallorca.html</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 11:09 p. m.</t>
+          <t>11/06/2026 01:24 a. m.</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -2980,19 +2952,19 @@
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>Bellver presenta su dimisión como director de Transparencia de la Generalitat tras ser imputado por su etapa como edil de Rita Barberá</t>
+          <t>Indignación entre los 600 cantantes expulsados de la Sagrada Familia: “Por tres o cuatro estelades, todos castigados”</t>
         </is>
       </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/espana/comunidad-valenciana/2026-06-11/bellver-anticipa-su-salida-como-director-de-transparencia-al-poner-su-cargo-a-disposicion-de-llorca-tras-su-imputacion.html</t>
+          <t>https://elpais.com/espana/catalunya/2026-06-11/indignacion-entre-los-600-cantantes-expulsados-de-la-sagrada-familia-por-tres-o-cuatro-estelades-todos-castigados.html</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>10/06/2026 11:00 p. m.</t>
+          <t>11/06/2026 12:25 a. m.</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
@@ -3007,19 +2979,19 @@
       </c>
       <c r="D93" s="6" t="inlineStr">
         <is>
-          <t>Los intercambios de fuego entre Estados Unidos e Irán abren una peligrosa nueva fase en la guerra</t>
+          <t>Analizamos cuatro camas refrescantes para perros</t>
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/internacional/2026-06-11/los-intercambios-de-fuego-entre-estados-unidos-e-iran-abren-una-peligrosa-nueva-fase-en-la-guerra.html</t>
+          <t>https://elpais.com/hemeroteca/2026-06-11/</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 11:00 p. m.</t>
+          <t>11/06/2026 12:20 a. m.</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -3034,19 +3006,19 @@
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>Radiografía de los rivales de México en el Grupo A: Sudáfrica, Corea del Sur y República Checa</t>
+          <t>Última hora de la guerra de Estados Unidos e Israel contra Irán, en directo | EE UU e Irán intercambian ataques por segundo día consecutivo</t>
         </is>
       </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/mexico/2026-06-11/radiografia-de-los-rivales-de-mexico-en-el-grupo-a-sudafrica-corea-del-sur-y-republica-checa.html</t>
+          <t>https://elpais.com/internacional/2026-06-11/ultima-hora-de-la-guerra-de-estados-unidos-e-israel-contra-iran-en-directo.html</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>10/06/2026 11:00 p. m.</t>
+          <t>11/06/2026 12:00 a. m.</t>
         </is>
       </c>
       <c r="B95" s="5" t="inlineStr">
@@ -3061,19 +3033,19 @@
       </c>
       <c r="D95" s="6" t="inlineStr">
         <is>
-          <t>La Agencia Europea de Derechos Fundamentales urge a los Veintisiete a abordar la crisis de la vivienda</t>
+          <t>Alexandra Lange, Pulitzer de Crítica 2025: “Hemos hecho la infancia demasiado segura”</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/economia/2026-06-11/la-agencia-europea-de-derechos-fundamentales-urge-a-los-veintisiete-a-abordar-la-crisis-de-la-vivienda.html</t>
+          <t>https://elpais.com/economia/formacion/2026-06-11/alexandra-lange-pulitzer-de-critica-2025-hemos-hecho-la-infancia-demasiado-segura.html</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 11:00 p. m.</t>
+          <t>11/06/2026 12:00 a. m.</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -3088,19 +3060,19 @@
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>Suspender al presidente, suspender las banderas: la campaña electoral se empantana en debates legales</t>
+          <t>Visita del Papa León XIV a Canarias: agenda del pontífice en su viaje por España</t>
         </is>
       </c>
       <c r="E96" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/america-colombia/elecciones-presidenciales/2026-06-11/suspender-al-presidente-suspender-las-banderas-la-campana-electoral-se-empantana-en-debates-legales.html</t>
+          <t>https://elpais.com/espana/2026-06-11/visita-del-papa-leon-xiv-a-canarias-agenda-del-pontifice-en-su-viaje-por-espana.html</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>10/06/2026 11:00 p. m.</t>
+          <t>11/06/2026 12:00 a. m.</t>
         </is>
       </c>
       <c r="B97" s="5" t="inlineStr">
@@ -3115,19 +3087,19 @@
       </c>
       <c r="D97" s="6" t="inlineStr">
         <is>
-          <t>“Los reos del crimen organizado se sienten en una playa en las cárceles chilenas”</t>
+          <t>Los seis destinos en África para ver este año con EL PAÍS Viajes</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/chile/2026-06-11/los-reos-del-crimen-organizado-se-sienten-en-una-playa-en-las-carceles-chilenas.html?autoplay=1</t>
+          <t>https://elpais.com/elviajero/viajes/2026-06-11/los-seis-destinos-en-africa-para-ver-este-ano-con-el-pais-viajes.html</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 11:00 p. m.</t>
+          <t>10/06/2026 11:56 p. m.</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -3142,19 +3114,19 @@
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>Trueque, reventa y colección virtual: la crisis no detiene el furor de los argentinos por el álbum del Mundial</t>
+          <t>Los Knicks acarician el campeonato de la NBA frente a los Spurs tras la mayor remontada de la historia</t>
         </is>
       </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/argentina/2026-06-11/trueque-reventa-y-coleccion-virtual-la-crisis-no-detiene-el-furor-de-los-argentinos-por-el-album-del-mundial.html</t>
+          <t>https://elpais.com/deportes/baloncesto/2026-06-11/los-knicks-acarician-el-campeonato-de-la-nba-frente-a-los-spurs-tras-la-mayor-remontada-de-la-historia.html</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="5" t="inlineStr">
         <is>
-          <t>10/06/2026 10:40 p. m.</t>
+          <t>10/06/2026 11:45 p. m.</t>
         </is>
       </c>
       <c r="B99" s="5" t="inlineStr">
@@ -3169,19 +3141,19 @@
       </c>
       <c r="D99" s="6" t="inlineStr">
         <is>
-          <t>¿Quién ganará el Mundial? Así arrancan nuestras predicciones</t>
+          <t>Un muro de policía para evitar que Jonathan, Olin, Ana o Mayra lleguen al Estadio Azteca</t>
         </is>
       </c>
       <c r="E99" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/deportes/mundial-futbol/2026-06-11/quien-ganara-el-mundial-asi-arrancan-nuestras-predicciones.html</t>
+          <t>https://elpais.com/mexico/2026-06-11/un-muro-de-policia-para-evitar-que-jonathan-olin-ana-o-mayra-lleguen-al-estadio-azteca.html</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 10:30 p. m.</t>
+          <t>10/06/2026 11:00 p. m.</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -3196,19 +3168,19 @@
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>Cómo la extrema derecha agita las calles contra la inmigración tras crímenes como el de Belfast o Southampton</t>
+          <t>Los intercambios de fuego entre Estados Unidos e Irán abren una peligrosa nueva fase en la guerra</t>
         </is>
       </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/internacional/2026-06-11/como-la-extrema-derecha-agita-las-calles-contra-la-inmigracion-tras-crimenes-como-el-de-belfast-o-southampton.html</t>
+          <t>https://elpais.com/internacional/2026-06-11/los-intercambios-de-fuego-entre-estados-unidos-e-iran-abren-una-peligrosa-nueva-fase-en-la-guerra.html</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>10/06/2026 10:30 p. m.</t>
+          <t>10/06/2026 10:40 p. m.</t>
         </is>
       </c>
       <c r="B101" s="5" t="inlineStr">
@@ -3223,12 +3195,12 @@
       </c>
       <c r="D101" s="6" t="inlineStr">
         <is>
-          <t>Las carreras universitarias con mejor sueldo y más salidas laborales, según esta calculadora con datos del INE</t>
+          <t>¿Quién ganará el Mundial? Así arrancan nuestras predicciones</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/educacion/2026-06-11/las-carreras-universitarias-con-mejor-sueldo-y-mas-salidas-laborales-segun-esta-calculadora-con-datos-del-ine.html</t>
+          <t>https://elpais.com/deportes/mundial-futbol/2026-06-11/quien-ganara-el-mundial-asi-arrancan-nuestras-predicciones.html</t>
         </is>
       </c>
     </row>
@@ -3250,12 +3222,12 @@
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>La productora del directivo investigado por agredir sexualmente a una reportera fue condenada por acoso laboral en 2024</t>
+          <t>Cómo la extrema derecha agita las calles contra la inmigración tras crímenes como el de Belfast o Southampton</t>
         </is>
       </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/sociedad/2026-06-11/la-productora-del-directivo-investigado-por-agredir-sexualmente-a-una-reportera-fue-condenada-por-acoso-laboral-en-2024.html</t>
+          <t>https://elpais.com/internacional/2026-06-11/como-la-extrema-derecha-agita-las-calles-contra-la-inmigracion-tras-crimenes-como-el-de-belfast-o-southampton.html</t>
         </is>
       </c>
     </row>
@@ -3277,12 +3249,12 @@
       </c>
       <c r="D103" s="6" t="inlineStr">
         <is>
-          <t>La revancha de Amy Adams: cómo la eterna nominada al Oscar intenta escapar de su “era de fracasos”</t>
+          <t>Las carreras universitarias con mejor sueldo y más salidas laborales, según esta calculadora con datos del INE</t>
         </is>
       </c>
       <c r="E103" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/smoda/famosos/2026-06-11/la-revancha-de-amy-adams-como-la-eterna-nominada-al-oscar-intenta-escapar-de-su-era-de-fracasos.html</t>
+          <t>https://elpais.com/educacion/2026-06-11/las-carreras-universitarias-con-mejor-sueldo-y-mas-salidas-laborales-segun-esta-calculadora-con-datos-del-ine.html</t>
         </is>
       </c>
     </row>
@@ -3304,12 +3276,12 @@
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>El mapa del precio real de la vivienda en España, calle a calle</t>
+          <t>La productora del directivo investigado por agredir sexualmente a una reportera fue condenada por acoso laboral en 2024</t>
         </is>
       </c>
       <c r="E104" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/economia/vivienda/2026-06-11/el-mapa-del-precio-real-de-la-vivienda-en-espana-calle-a-calle.html</t>
+          <t>https://elpais.com/sociedad/2026-06-11/la-productora-del-directivo-investigado-por-agredir-sexualmente-a-una-reportera-fue-condenada-por-acoso-laboral-en-2024.html</t>
         </is>
       </c>
     </row>
@@ -3331,12 +3303,12 @@
       </c>
       <c r="D105" s="6" t="inlineStr">
         <is>
-          <t>Vega, cantante: “Ya no sé cómo lidiar con discográficas. Si lo hiciese, sería insufrible”</t>
+          <t>El mapa del precio real de la vivienda en España, calle a calle</t>
         </is>
       </c>
       <c r="E105" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/cultura/2026-06-11/vega-cantante-ya-no-se-como-lidiar-con-discograficas-si-lo-hiciese-seria-insufrible.html</t>
+          <t>https://elpais.com/economia/vivienda/2026-06-11/el-mapa-del-precio-real-de-la-vivienda-en-espana-calle-a-calle.html</t>
         </is>
       </c>
     </row>
@@ -3358,12 +3330,12 @@
       </c>
       <c r="D106" s="3" t="inlineStr">
         <is>
-          <t>Arranca el Mundial de los extremos, el último que aún vibra con el duelo Messi-Cristiano</t>
+          <t>Vega, cantante: “Ya no sé cómo lidiar con discográficas. Si lo hiciese, sería insufrible”</t>
         </is>
       </c>
       <c r="E106" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/deportes/mundial-futbol/2026-06-11/arranca-el-mundial-de-los-extremos.html</t>
+          <t>https://elpais.com/cultura/2026-06-11/vega-cantante-ya-no-se-como-lidiar-con-discograficas-si-lo-hiciese-seria-insufrible.html</t>
         </is>
       </c>
     </row>
@@ -3385,19 +3357,19 @@
       </c>
       <c r="D107" s="6" t="inlineStr">
         <is>
-          <t>Pochettino: “Acepto la arrogancia española, argentina, inglesa... Pero en Estados Unidos hay un poco de confusión”</t>
+          <t>Arranca el Mundial de los extremos, el último que aún vibra con el duelo Messi-Cristiano</t>
         </is>
       </c>
       <c r="E107" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/deportes/mundial-futbol/2026-06-11/pochettino-acepto-la-arrogancia-espanola-argentina-inglesa-pero-en-estados-unidos-hay-un-poco-de-confusion.html</t>
+          <t>https://elpais.com/deportes/mundial-futbol/2026-06-11/arranca-el-mundial-de-los-extremos.html</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 10:30 p. m.</t>
+          <t>10/06/2026 10:30 p. m.</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
@@ -3412,12 +3384,12 @@
       </c>
       <c r="D108" s="3" t="inlineStr">
         <is>
-          <t>Cómo buscar un sitio perfecto para ver el eclipse total: tres apps y una web resuelven el dilema</t>
+          <t>Pochettino: “Acepto la arrogancia española, argentina, inglesa... Pero en Estados Unidos hay un poco de confusión”</t>
         </is>
       </c>
       <c r="E108" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/ciencia/2026-06-10/como-buscar-un-sitio-perfecto-para-ver-el-eclipse-total-tres-apps-y-una-web-resuelven-el-dilema.html</t>
+          <t>https://elpais.com/deportes/mundial-futbol/2026-06-11/pochettino-acepto-la-arrogancia-espanola-argentina-inglesa-pero-en-estados-unidos-hay-un-poco-de-confusion.html</t>
         </is>
       </c>
     </row>
@@ -4488,12 +4460,12 @@
       </c>
       <c r="D148" s="3" t="inlineStr">
         <is>
-          <t>Siempre es con los otros</t>
+          <t>¿Qué propuestas tienen De la Espriella y Cepeda para el sector de la Cultura?</t>
         </is>
       </c>
       <c r="E148" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/tatiana-duplat/siempre-es-con-los-otros/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/columnista-invitado-ee/que-propuestas-tienen-de-la-espriella-y-cepeda-para-el-sector-de-la-cultura/</t>
         </is>
       </c>
     </row>
@@ -4515,12 +4487,12 @@
       </c>
       <c r="D149" s="6" t="inlineStr">
         <is>
-          <t>Los periodistas en época electoral</t>
+          <t>Siempre es con los otros</t>
         </is>
       </c>
       <c r="E149" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/claudia-morales/los-periodistas-en-epoca-electoral/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/tatiana-duplat/siempre-es-con-los-otros/</t>
         </is>
       </c>
     </row>
@@ -4542,12 +4514,12 @@
       </c>
       <c r="D150" s="3" t="inlineStr">
         <is>
-          <t>¿Qué propuestas tienen De la Espriella y Cepeda para el sector de la Cultura?</t>
+          <t>Los periodistas en época electoral</t>
         </is>
       </c>
       <c r="E150" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/columnista-invitado-ee/que-propuestas-tienen-de-la-espriella-y-cepeda-para-el-sector-de-la-cultura/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/claudia-morales/los-periodistas-en-epoca-electoral/</t>
         </is>
       </c>
     </row>
@@ -4714,56 +4686,56 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="8" t="inlineStr">
-        <is>
-          <t>11/06/2026 12:35 a. m.</t>
-        </is>
-      </c>
-      <c r="B157" s="8" t="inlineStr">
-        <is>
-          <t>Entidad Oficial</t>
-        </is>
-      </c>
-      <c r="C157" s="8" t="inlineStr">
-        <is>
-          <t>Superintendencia Nacional de Salud</t>
-        </is>
-      </c>
-      <c r="D157" s="9" t="inlineStr">
-        <is>
-          <t>Supersalud intensifica inspecciones a dispensarios de medicamentos en Bogotá</t>
-        </is>
-      </c>
-      <c r="E157" s="10" t="inlineStr">
-        <is>
-          <t>https://wcmportal.supersalud.gov.co/portalweb/Comunicaciones/Lists/Noticias/Noticia.aspx?ID=2593</t>
+      <c r="A157" s="5" t="inlineStr">
+        <is>
+          <t>11/06/2026 12:00 a. m.</t>
+        </is>
+      </c>
+      <c r="B157" s="5" t="inlineStr">
+        <is>
+          <t>Medio de Comunicación</t>
+        </is>
+      </c>
+      <c r="C157" s="5" t="inlineStr">
+        <is>
+          <t>Infobae Colombia</t>
+        </is>
+      </c>
+      <c r="D157" s="6" t="inlineStr">
+        <is>
+          <t>Consejo Superior Universitario aplaza elección de rector de la Universidad de Antioquia hasta el 24 de junio</t>
+        </is>
+      </c>
+      <c r="E157" s="7" t="inlineStr">
+        <is>
+          <t>https://www.infobae.com/colombia/2026/06/11/consejo-superior-universitario-aplaza-eleccion-de-rector-de-la-universidad-de-antioquia-hasta-el-24-de-junio/</t>
         </is>
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="11" t="inlineStr">
-        <is>
-          <t>11/06/2026 12:25 a. m.</t>
-        </is>
-      </c>
-      <c r="B158" s="11" t="inlineStr">
-        <is>
-          <t>Entidad Oficial</t>
-        </is>
-      </c>
-      <c r="C158" s="11" t="inlineStr">
-        <is>
-          <t>Superintendencia Nacional de Salud</t>
-        </is>
-      </c>
-      <c r="D158" s="12" t="inlineStr">
-        <is>
-          <t>Por incumplir una medida cautelar, Supersalud ordena cierre de servicios en Clínica Láser Surgical</t>
-        </is>
-      </c>
-      <c r="E158" s="13" t="inlineStr">
-        <is>
-          <t>https://wcmportal.supersalud.gov.co/portalweb/Comunicaciones/Lists/Noticias/Noticia.aspx?ID=2589</t>
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>11/06/2026 12:00 a. m.</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>Medio de Comunicación</t>
+        </is>
+      </c>
+      <c r="C158" s="2" t="inlineStr">
+        <is>
+          <t>Infobae Colombia</t>
+        </is>
+      </c>
+      <c r="D158" s="3" t="inlineStr">
+        <is>
+          <t>Conoce el clima de este día en Bogotá</t>
+        </is>
+      </c>
+      <c r="E158" s="4" t="inlineStr">
+        <is>
+          <t>https://www.infobae.com/colombia/2026/06/11/conoce-el-clima-de-este-dia-en-bogota/</t>
         </is>
       </c>
     </row>
@@ -4785,12 +4757,12 @@
       </c>
       <c r="D159" s="6" t="inlineStr">
         <is>
-          <t>Ministerio de la Igualdad inicia su cierre: funcionarios reciben instrucciones ante posible liquidación el 20 de junio</t>
+          <t>Previsión meteorológica del clima en Cali para este 11 de junio</t>
         </is>
       </c>
       <c r="E159" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/11/ministerio-de-la-igualdad-inicia-su-cierre-funcionarios-reciben-instrucciones-ante-posible-liquidacion-el-20-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/11/prevision-meteorologica-del-clima-en-cali-para-este-11-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4812,12 +4784,12 @@
       </c>
       <c r="D160" s="3" t="inlineStr">
         <is>
-          <t>Pico y Placa en Bogotá: restricciones vehiculares para evitar multas este jueves 11 de junio</t>
+          <t>Adiós a la incertidumbre, conoce las condiciones climáticas en Cartagena de Indias</t>
         </is>
       </c>
       <c r="E160" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/11/pico-y-placa-en-bogota-restricciones-vehiculares-para-evitar-multas-este-jueves-11-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/11/adios-a-la-incertidumbre-conoce-las-condiciones-climaticas-en-cartagena-de-indias/</t>
         </is>
       </c>
     </row>
@@ -4839,12 +4811,12 @@
       </c>
       <c r="D161" s="6" t="inlineStr">
         <is>
-          <t>James Rodríguez se ilusiona con la final y Lorenzo promete “el mejor Mundial posible” tras llegada de Colombia a México</t>
+          <t>Colombia: el pronóstico del tiempo para Medellín este 11 de junio</t>
         </is>
       </c>
       <c r="E161" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/06/11/james-rodriguez-se-ilusiona-con-la-final-y-lorenzo-promete-el-mejor-mundial-posible-tras-llegada-de-colombia-a-mexico/</t>
+          <t>https://www.infobae.com/colombia/2026/06/11/colombia-el-pronostico-del-tiempo-para-medellin-este-11-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4866,12 +4838,12 @@
       </c>
       <c r="D162" s="3" t="inlineStr">
         <is>
-          <t>Baloto y Revancha: números ganadores del miércoles 10 de junio</t>
+          <t>Adiós a la incertidumbre, conoce las condiciones climáticas en Barranquilla</t>
         </is>
       </c>
       <c r="E162" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/11/baloto-y-revancha-numeros-ganadores-del-miercoles-10-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/11/adios-a-la-incertidumbre-conoce-las-condiciones-climaticas-en-barranquilla/</t>
         </is>
       </c>
     </row>
@@ -4893,12 +4865,12 @@
       </c>
       <c r="D163" s="6" t="inlineStr">
         <is>
-          <t>Sismo hoy: se registró un temblor en en el océano Pacífico sur con magnitud 4.9</t>
+          <t>Jefe de campaña de Abelardo de la Espriella controla clínica que recibe recursos públicos y empresas con demandas laborales</t>
         </is>
       </c>
       <c r="E163" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/11/sismo-hoy-se-registro-un-temblor-en-en-el-oceano-pacifico-sur-con-magnitud-49/</t>
+          <t>https://www.infobae.com/colombia/2026/06/11/jefe-de-campana-de-abelardo-de-la-espriella-controla-clinica-que-recibe-recursos-publicos-y-empresas-con-demandas-laborales/</t>
         </is>
       </c>
     </row>
@@ -4920,12 +4892,12 @@
       </c>
       <c r="D164" s="3" t="inlineStr">
         <is>
-          <t>Sismo hoy: se registró un temblor en Costa Rica con magnitud 5.1</t>
+          <t>Ministerio de la Igualdad inicia su cierre: funcionarios reciben instrucciones ante posible liquidación el 20 de junio</t>
         </is>
       </c>
       <c r="E164" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/11/sismo-hoy-se-registro-un-temblor-en-costa-rica-con-magnitud-51/</t>
+          <t>https://www.infobae.com/colombia/2026/06/11/ministerio-de-la-igualdad-inicia-su-cierre-funcionarios-reciben-instrucciones-ante-posible-liquidacion-el-20-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4947,12 +4919,12 @@
       </c>
       <c r="D165" s="6" t="inlineStr">
         <is>
-          <t>Resultados Lotería de Manizales miércoles 10 de junio de 2026: números ganadores del último sorteo</t>
+          <t>Pico y Placa en Bogotá: restricciones vehiculares para evitar multas este jueves 11 de junio</t>
         </is>
       </c>
       <c r="E165" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/11/resultados-loteria-de-manizales-miercoles-10-de-junio-de-2026-numeros-ganadores-del-ultimo-sorteo/</t>
+          <t>https://www.infobae.com/colombia/2026/06/11/pico-y-placa-en-bogota-restricciones-vehiculares-para-evitar-multas-este-jueves-11-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4974,12 +4946,12 @@
       </c>
       <c r="D166" s="3" t="inlineStr">
         <is>
-          <t>Habrá ley seca en Bogotá durante la segunda vuelta presidencial del 21 de junio: fechas, horarios y sanciones</t>
+          <t>James Rodríguez se ilusiona con la final y Lorenzo promete “el mejor Mundial posible” tras llegada de Colombia a México</t>
         </is>
       </c>
       <c r="E166" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/11/habra-ley-seca-en-bogota-durante-la-segunda-vuelta-presidencial-del-21-de-junio-fechas-horarios-y-sanciones/</t>
+          <t>https://www.infobae.com/colombia/deportes/2026/06/11/james-rodriguez-se-ilusiona-con-la-final-y-lorenzo-promete-el-mejor-mundial-posible-tras-llegada-de-colombia-a-mexico/</t>
         </is>
       </c>
     </row>
@@ -5001,12 +4973,12 @@
       </c>
       <c r="D167" s="6" t="inlineStr">
         <is>
-          <t>Se registró visita técnica en el Puerto de Tumaco para garantizar el abastecimiento de combustibles en el suroccidente del país</t>
+          <t>Baloto y Revancha: números ganadores del miércoles 10 de junio</t>
         </is>
       </c>
       <c r="E167" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/11/se-registro-visita-tecnica-en-el-puerto-de-tumaco-para-garantizar-el-abastecimiento-de-combustibles-en-el-suroccidente-del-pais/</t>
+          <t>https://www.infobae.com/colombia/2026/06/11/baloto-y-revancha-numeros-ganadores-del-miercoles-10-de-junio/</t>
         </is>
       </c>
     </row>
@@ -5028,12 +5000,12 @@
       </c>
       <c r="D168" s="3" t="inlineStr">
         <is>
-          <t>Resultados Lotería del Valle miércoles 10 de junio de 2026: números ganadores del premio mayor de $9.000 millones</t>
+          <t>Sismo hoy: se registró un temblor en en el océano Pacífico sur con magnitud 4.9</t>
         </is>
       </c>
       <c r="E168" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/11/resultados-loteria-del-valle-miercoles-10-de-junio-de-2026-numeros-ganadores-del-premio-mayor-de-9000-millones/</t>
+          <t>https://www.infobae.com/colombia/2026/06/11/sismo-hoy-se-registro-un-temblor-en-en-el-oceano-pacifico-sur-con-magnitud-49/</t>
         </is>
       </c>
     </row>
@@ -5055,12 +5027,12 @@
       </c>
       <c r="D169" s="6" t="inlineStr">
         <is>
-          <t>Resultados Baloto y Revancha, último sorteo del lunes 8 de junio</t>
+          <t>Sismo hoy: se registró un temblor en Costa Rica con magnitud 5.1</t>
         </is>
       </c>
       <c r="E169" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/11/resultados-baloto-y-revancha-ultimo-sorteo-del-lunes-8-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/11/sismo-hoy-se-registro-un-temblor-en-costa-rica-con-magnitud-51/</t>
         </is>
       </c>
     </row>
@@ -5082,12 +5054,12 @@
       </c>
       <c r="D170" s="3" t="inlineStr">
         <is>
-          <t>Resultado Super Astro Luna HOY: número ganador del miércoles 10 de junio</t>
+          <t>Resultados Lotería de Manizales miércoles 10 de junio de 2026: números ganadores del último sorteo</t>
         </is>
       </c>
       <c r="E170" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/11/resultado-super-astro-luna-hoy-numero-ganador-del-miercoles-10-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/11/resultados-loteria-de-manizales-miercoles-10-de-junio-de-2026-numeros-ganadores-del-ultimo-sorteo/</t>
         </is>
       </c>
     </row>
@@ -5109,12 +5081,12 @@
       </c>
       <c r="D171" s="6" t="inlineStr">
         <is>
-          <t>Este es el precio del oro en Colombia este miércoles 10 de junio</t>
+          <t>Habrá ley seca en Bogotá durante la segunda vuelta presidencial del 21 de junio: fechas, horarios y sanciones</t>
         </is>
       </c>
       <c r="E171" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/11/este-es-el-precio-del-oro-en-colombia-este-jueves-11-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/11/habra-ley-seca-en-bogota-durante-la-segunda-vuelta-presidencial-del-21-de-junio-fechas-horarios-y-sanciones/</t>
         </is>
       </c>
     </row>
@@ -5136,12 +5108,12 @@
       </c>
       <c r="D172" s="3" t="inlineStr">
         <is>
-          <t>Lotería de Meta resultados 10 de junio: números ganadores del premio mayor de $1.800 millones</t>
+          <t>Se registró visita técnica en el Puerto de Tumaco para garantizar el abastecimiento de combustibles en el suroccidente del país</t>
         </is>
       </c>
       <c r="E172" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/11/loteria-de-meta-resultados-10-de-junio-numeros-ganadores-del-premio-mayor-de-1800-millones/</t>
+          <t>https://www.infobae.com/colombia/2026/06/11/se-registro-visita-tecnica-en-el-puerto-de-tumaco-para-garantizar-el-abastecimiento-de-combustibles-en-el-suroccidente-del-pais/</t>
         </is>
       </c>
     </row>
@@ -5163,12 +5135,12 @@
       </c>
       <c r="D173" s="6" t="inlineStr">
         <is>
-          <t>Pico y placa en Cali hoy 11 de junio de 2026, así regirá la medida</t>
+          <t>Resultados Lotería del Valle miércoles 10 de junio de 2026: números ganadores del premio mayor de $9.000 millones</t>
         </is>
       </c>
       <c r="E173" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/11/pico-y-placa-en-cali-hoy-11-de-junio-de-2026-asi-regira-la-medida/</t>
+          <t>https://www.infobae.com/colombia/2026/06/11/resultados-loteria-del-valle-miercoles-10-de-junio-de-2026-numeros-ganadores-del-premio-mayor-de-9000-millones/</t>
         </is>
       </c>
     </row>
@@ -5190,12 +5162,12 @@
       </c>
       <c r="D174" s="3" t="inlineStr">
         <is>
-          <t>Pico y Placa: qué vehículos descansan en Villavicencio este jueves 11 de junio</t>
+          <t>Resultados Baloto y Revancha, último sorteo del lunes 8 de junio</t>
         </is>
       </c>
       <c r="E174" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/11/pico-y-placa-que-vehiculos-descansan-en-villavicencio-este-jueves-11-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/11/resultados-baloto-y-revancha-ultimo-sorteo-del-lunes-8-de-junio/</t>
         </is>
       </c>
     </row>
@@ -5217,12 +5189,12 @@
       </c>
       <c r="D175" s="6" t="inlineStr">
         <is>
-          <t>Resultado Sinuano Noche hoy 10 de junio</t>
+          <t>Resultado Super Astro Luna HOY: número ganador del miércoles 10 de junio</t>
         </is>
       </c>
       <c r="E175" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/11/resultado-sinuano-noche-hoy-9-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/11/resultado-super-astro-luna-hoy-numero-ganador-del-miercoles-10-de-junio/</t>
         </is>
       </c>
     </row>
@@ -5244,19 +5216,19 @@
       </c>
       <c r="D176" s="3" t="inlineStr">
         <is>
-          <t>Tenga en cuenta: Así regirá el pico y placa en Cartagena este jueves 11 de junio</t>
+          <t>Este es el precio del oro en Colombia este miércoles 10 de junio</t>
         </is>
       </c>
       <c r="E176" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/11/tenga-en-cuenta-asi-regira-el-pico-y-placa-en-cartagena-este-jueves/</t>
+          <t>https://www.infobae.com/colombia/2026/06/11/este-es-el-precio-del-oro-en-colombia-este-jueves-11-de-junio/</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="5" t="inlineStr">
         <is>
-          <t>11/06/2026 12:00 a. m.</t>
+          <t>10/06/2026 07:56 p. m.</t>
         </is>
       </c>
       <c r="B177" s="5" t="inlineStr">
@@ -5266,24 +5238,24 @@
       </c>
       <c r="C177" s="5" t="inlineStr">
         <is>
-          <t>Infobae Colombia</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D177" s="6" t="inlineStr">
         <is>
-          <t>Pico y Placa: qué autos no circulan en Medellín este jueves 11 de junio</t>
+          <t>Juristas y académicos advierten "insalvable conflicto de lealtades" en candidatura de Abelardo de la Espriella</t>
         </is>
       </c>
       <c r="E177" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/11/pico-y-placa-que-autos-no-circulan-en-medellin-este-jueves-11-de-junio/</t>
+          <t>https://cambiocolombia.com/poder/articulo/2026/6/juristas-y-academicos-advierten-insalvable-conflicto-de-lealtades-en-candidatura-de-abelardo-de-la-espriella</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 12:00 a. m.</t>
+          <t>10/06/2026 07:15 p. m.</t>
         </is>
       </c>
       <c r="B178" s="2" t="inlineStr">
@@ -5293,24 +5265,24 @@
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>Infobae Colombia</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D178" s="3" t="inlineStr">
         <is>
-          <t>Caribeña Noche, resultados ganadores del último sorteo de hoy miércoles 10 de junio</t>
+          <t>Comisión de Acusación inició investigación previa contra el presidente Petro por la compra de los aviones Gripen</t>
         </is>
       </c>
       <c r="E178" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/11/caribena-noche-resultados-ganadores-del-ultimo-sorteo-de-hoy-miercoles-10-de-junio/</t>
+          <t>https://cambiocolombia.com/poder/articulo/2026/6/comision-de-acusacion-inicio-investigacion-previa-contra-el-presidente-petro-por-la-compra-de-los-aviones-gripen</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="5" t="inlineStr">
         <is>
-          <t>10/06/2026 07:56 p. m.</t>
+          <t>10/06/2026 05:54 p. m.</t>
         </is>
       </c>
       <c r="B179" s="5" t="inlineStr">
@@ -5325,19 +5297,19 @@
       </c>
       <c r="D179" s="6" t="inlineStr">
         <is>
-          <t>Juristas y académicos advierten "insalvable conflicto de lealtades" en candidatura de Abelardo de la Espriella</t>
+          <t>Belfast arde: disturbios reflejan la creciente tensión migratoria en Europa</t>
         </is>
       </c>
       <c r="E179" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/poder/articulo/2026/6/juristas-y-academicos-advierten-insalvable-conflicto-de-lealtades-en-candidatura-de-abelardo-de-la-espriella</t>
+          <t>https://cambiocolombia.com/internacional/articulo/2026/6/belfast-arde-disturbios-reflejan-la-creciente-tension-migratoria-en-europa</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 07:15 p. m.</t>
+          <t>10/06/2026 05:30 p. m.</t>
         </is>
       </c>
       <c r="B180" s="2" t="inlineStr">
@@ -5352,19 +5324,19 @@
       </c>
       <c r="D180" s="3" t="inlineStr">
         <is>
-          <t>Comisión de Acusación inició investigación previa contra el presidente Petro por la compra de los aviones Gripen</t>
+          <t>¿Quién es Gloria Arizabaleta y cuál ha sido su trayectoria en la política y la justicia?</t>
         </is>
       </c>
       <c r="E180" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/poder/articulo/2026/6/comision-de-acusacion-inicio-investigacion-previa-contra-el-presidente-petro-por-la-compra-de-los-aviones-gripen</t>
+          <t>https://cambiocolombia.com/pais/articulo/2026/6/quien-es-gloria-arizabaleta-y-cual-ha-sido-su-trayectoria-en-la-politica-y-la-justicia</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="5" t="inlineStr">
         <is>
-          <t>10/06/2026 05:54 p. m.</t>
+          <t>10/06/2026 05:30 p. m.</t>
         </is>
       </c>
       <c r="B181" s="5" t="inlineStr">
@@ -5379,19 +5351,19 @@
       </c>
       <c r="D181" s="6" t="inlineStr">
         <is>
-          <t>Belfast arde: disturbios reflejan la creciente tensión migratoria en Europa</t>
+          <t>Congreso aprobó, al fin, el proyecto para prevenir y erradicar la mutilación genital femenina en Colombia: ¿qué cambiará?</t>
         </is>
       </c>
       <c r="E181" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/internacional/articulo/2026/6/belfast-arde-disturbios-reflejan-la-creciente-tension-migratoria-en-europa</t>
+          <t>https://cambiocolombia.com/pais/articulo/2026/6/congreso-aprobo-al-fin-el-proyecto-para-prevenir-y-erradicar-la-mutilacion-genital-femenina-en-colombia-que-cambiara</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 05:30 p. m.</t>
+          <t>10/06/2026 05:00 p. m.</t>
         </is>
       </c>
       <c r="B182" s="2" t="inlineStr">
@@ -5406,19 +5378,19 @@
       </c>
       <c r="D182" s="3" t="inlineStr">
         <is>
-          <t>¿Quién es Gloria Arizabaleta y cuál ha sido su trayectoria en la política y la justicia?</t>
+          <t>Donald Trump vuelve a respaldar a Abelardo de la Espriella y promete todo el apoyo de Estados Unidos si gana la Presidencia</t>
         </is>
       </c>
       <c r="E182" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/pais/articulo/2026/6/quien-es-gloria-arizabaleta-y-cual-ha-sido-su-trayectoria-en-la-politica-y-la-justicia</t>
+          <t>https://cambiocolombia.com/poder/articulo/2026/6/donald-trump-vuelve-a-respaldar-a-abelardo-de-la-espriella-y-promete-todo-el-apoyo-de-estados-unidos-si-gana-la-presidencia</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="5" t="inlineStr">
         <is>
-          <t>10/06/2026 05:30 p. m.</t>
+          <t>10/06/2026 04:00 p. m.</t>
         </is>
       </c>
       <c r="B183" s="5" t="inlineStr">
@@ -5433,19 +5405,19 @@
       </c>
       <c r="D183" s="6" t="inlineStr">
         <is>
-          <t>Congreso aprobó, al fin, el proyecto para prevenir y erradicar la mutilación genital femenina en Colombia: ¿qué cambiará?</t>
+          <t>Juan Carlos Florián renunció al Consulado de Colombia en Bruselas: ¿se unirá a la campaña de Iván Cepeda?</t>
         </is>
       </c>
       <c r="E183" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/pais/articulo/2026/6/congreso-aprobo-al-fin-el-proyecto-para-prevenir-y-erradicar-la-mutilacion-genital-femenina-en-colombia-que-cambiara</t>
+          <t>https://cambiocolombia.com/poder/articulo/2026/6/juan-carlos-florian-renuncio-al-consulado-de-colombia-en-bruselas-se-unira-a-la-campana-de-ivan-cepeda</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 05:00 p. m.</t>
+          <t>10/06/2026 01:45 p. m.</t>
         </is>
       </c>
       <c r="B184" s="2" t="inlineStr">
@@ -5460,19 +5432,19 @@
       </c>
       <c r="D184" s="3" t="inlineStr">
         <is>
-          <t>Donald Trump vuelve a respaldar a Abelardo de la Espriella y promete todo el apoyo de Estados Unidos si gana la Presidencia</t>
+          <t>¿Quiénes son los expertos económicos que acompañarán a Iván Cepeda si llega a la Presidencia?</t>
         </is>
       </c>
       <c r="E184" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/poder/articulo/2026/6/donald-trump-vuelve-a-respaldar-a-abelardo-de-la-espriella-y-promete-todo-el-apoyo-de-estados-unidos-si-gana-la-presidencia</t>
+          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/quienes-son-los-expertos-economicos-que-acompanaran-a-ivan-cepeda-si-llega-a-la-presidencia</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="5" t="inlineStr">
         <is>
-          <t>10/06/2026 04:00 p. m.</t>
+          <t>10/06/2026 01:25 p. m.</t>
         </is>
       </c>
       <c r="B185" s="5" t="inlineStr">
@@ -5487,19 +5459,19 @@
       </c>
       <c r="D185" s="6" t="inlineStr">
         <is>
-          <t>Juan Carlos Florián renunció al Consulado de Colombia en Bruselas: ¿se unirá a la campaña de Iván Cepeda?</t>
+          <t>¿Cómo operaban Los Náuticos, la red que contrabandeaba armas desde Estados Unidos para dárselas al Clan del Golfo?</t>
         </is>
       </c>
       <c r="E185" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/poder/articulo/2026/6/juan-carlos-florian-renuncio-al-consulado-de-colombia-en-bruselas-se-unira-a-la-campana-de-ivan-cepeda</t>
+          <t>https://cambiocolombia.com/pais/articulo/2026/6/como-operaban-los-nauticos-la-red-que-contrabandeaba-armas-desde-estados-unidos-para-darselas-al-clan-del-golfo</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 01:45 p. m.</t>
+          <t>10/06/2026 01:15 p. m.</t>
         </is>
       </c>
       <c r="B186" s="2" t="inlineStr">
@@ -5514,19 +5486,19 @@
       </c>
       <c r="D186" s="3" t="inlineStr">
         <is>
-          <t>¿Quiénes son los expertos económicos que acompañarán a Iván Cepeda si llega a la Presidencia?</t>
+          <t>Los detalles del proyecto que crearía un nuevo seguro obligatorio para conductores, diferente al Soat</t>
         </is>
       </c>
       <c r="E186" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/quienes-son-los-expertos-economicos-que-acompanaran-a-ivan-cepeda-si-llega-a-la-presidencia</t>
+          <t>https://cambiocolombia.com/pais/articulo/2026/6/los-detalles-del-proyecto-que-crearia-un-nuevo-seguro-obligatorio-para-conductores-diferente-al-soat</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="5" t="inlineStr">
         <is>
-          <t>10/06/2026 01:25 p. m.</t>
+          <t>10/06/2026 12:23 p. m.</t>
         </is>
       </c>
       <c r="B187" s="5" t="inlineStr">
@@ -5541,19 +5513,19 @@
       </c>
       <c r="D187" s="6" t="inlineStr">
         <is>
-          <t>¿Cómo operaban Los Náuticos, la red que contrabandeaba armas desde Estados Unidos para dárselas al Clan del Golfo?</t>
+          <t>Consejo de Estado niega demanda que pretendía la muerte política del presidente Gustavo Petro</t>
         </is>
       </c>
       <c r="E187" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/pais/articulo/2026/6/como-operaban-los-nauticos-la-red-que-contrabandeaba-armas-desde-estados-unidos-para-darselas-al-clan-del-golfo</t>
+          <t>https://cambiocolombia.com/justicia/articulo/2026/6/consejo-de-estado-niega-demanda-que-pretendia-la-muerte-politica-del-presidente-gustavo-petro</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 01:15 p. m.</t>
+          <t>10/06/2026 09:30 a. m.</t>
         </is>
       </c>
       <c r="B188" s="2" t="inlineStr">
@@ -5568,19 +5540,19 @@
       </c>
       <c r="D188" s="3" t="inlineStr">
         <is>
-          <t>Los detalles del proyecto que crearía un nuevo seguro obligatorio para conductores, diferente al Soat</t>
+          <t>“El único efecto que tendrá es político”: las reacciones al proyecto que propone suspender al presidente Petro</t>
         </is>
       </c>
       <c r="E188" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/pais/articulo/2026/6/los-detalles-del-proyecto-que-crearia-un-nuevo-seguro-obligatorio-para-conductores-diferente-al-soat</t>
+          <t>https://cambiocolombia.com/poder/articulo/2026/6/el-unico-efecto-que-tendra-es-politico-las-reacciones-al-proyecto-que-propone-suspender-al-presidente-petro</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="5" t="inlineStr">
         <is>
-          <t>10/06/2026 12:23 p. m.</t>
+          <t>10/06/2026 07:30 a. m.</t>
         </is>
       </c>
       <c r="B189" s="5" t="inlineStr">
@@ -5595,19 +5567,19 @@
       </c>
       <c r="D189" s="6" t="inlineStr">
         <is>
-          <t>Consejo de Estado niega demanda que pretendía la muerte política del presidente Gustavo Petro</t>
+          <t>Cuatro masacres en dos días dejan al menos 13 víctimas en tres departamentos del país: la cifra sube a 65 en lo que va del año</t>
         </is>
       </c>
       <c r="E189" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/justicia/articulo/2026/6/consejo-de-estado-niega-demanda-que-pretendia-la-muerte-politica-del-presidente-gustavo-petro</t>
+          <t>https://cambiocolombia.com/conflicto-armado-en-colombia/articulo/2026/6/cuatro-masacres-en-dos-dias-dejan-al-menos-13-victimas-en-tres-departamentos-del-pais-la-cifra-sube-a-65-en-lo-que-va-del-ano</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 09:30 a. m.</t>
+          <t>10/06/2026 06:45 a. m.</t>
         </is>
       </c>
       <c r="B190" s="2" t="inlineStr">
@@ -5622,19 +5594,19 @@
       </c>
       <c r="D190" s="3" t="inlineStr">
         <is>
-          <t>“El único efecto que tendrá es político”: las reacciones al proyecto que propone suspender al presidente Petro</t>
+          <t>Capturan al sicario y a dos cómplices del asesinato del periodista Cristian Herrera: "pretendían salir del país"</t>
         </is>
       </c>
       <c r="E190" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/poder/articulo/2026/6/el-unico-efecto-que-tendra-es-politico-las-reacciones-al-proyecto-que-propone-suspender-al-presidente-petro</t>
+          <t>https://cambiocolombia.com/pais/articulo/2026/6/capturan-al-sicario-y-a-dos-complices-del-asesinato-del-periodista-cristian-herrera-pretendian-salir-del-pais</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="5" t="inlineStr">
         <is>
-          <t>10/06/2026 07:30 a. m.</t>
+          <t>09/06/2026 08:00 p. m.</t>
         </is>
       </c>
       <c r="B191" s="5" t="inlineStr">
@@ -5649,19 +5621,19 @@
       </c>
       <c r="D191" s="6" t="inlineStr">
         <is>
-          <t>Cuatro masacres en dos días dejan al menos 13 víctimas en tres departamentos del país: la cifra sube a 65 en lo que va del año</t>
+          <t>Erick Rodríguez deja las Fuerzas Militares tras más de 35 años de carrera</t>
         </is>
       </c>
       <c r="E191" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/conflicto-armado-en-colombia/articulo/2026/6/cuatro-masacres-en-dos-dias-dejan-al-menos-13-victimas-en-tres-departamentos-del-pais-la-cifra-sube-a-65-en-lo-que-va-del-ano</t>
+          <t>https://cambiocolombia.com/pais/articulo/2026/6/erick-rodriguez-deja-las-fuerzas-militares-tras-mas-de-35-anos-de-carrera</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 06:45 a. m.</t>
+          <t>09/06/2026 01:53 p. m.</t>
         </is>
       </c>
       <c r="B192" s="2" t="inlineStr">
@@ -5676,21 +5648,17 @@
       </c>
       <c r="D192" s="3" t="inlineStr">
         <is>
-          <t>Capturan al sicario y a dos cómplices del asesinato del periodista Cristian Herrera: "pretendían salir del país"</t>
+          <t>Tribunal prohíbe la propaganda política con la expresión “firmes por la patria”</t>
         </is>
       </c>
       <c r="E192" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/pais/articulo/2026/6/capturan-al-sicario-y-a-dos-complices-del-asesinato-del-periodista-cristian-herrera-pretendian-salir-del-pais</t>
+          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/tribunal-prohibe-la-propaganda-politica-con-la-expresion-firmes-por-la-patria</t>
         </is>
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="5" t="inlineStr">
-        <is>
-          <t>09/06/2026 08:00 p. m.</t>
-        </is>
-      </c>
+      <c r="A193" s="5" t="inlineStr"/>
       <c r="B193" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5698,26 +5666,22 @@
       </c>
       <c r="C193" s="5" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D193" s="6" t="inlineStr">
         <is>
-          <t>Erick Rodríguez deja las Fuerzas Militares tras más de 35 años de carrera</t>
+          <t>Petro planeaba reunirse con el alcalde de Nueva York, pero el gobierno Trump amenazó con arrestarlo si realizaba actividades diferentes a su agenda en la ONU</t>
         </is>
       </c>
       <c r="E193" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/pais/articulo/2026/6/erick-rodriguez-deja-las-fuerzas-militares-tras-mas-de-35-anos-de-carrera</t>
+          <t>https://www.elcolombiano.com/colombia/departamento-de-estado-amenaza-arresto-gustavo-petro-reunion-alcalde-nueva-york-GG37571250</t>
         </is>
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="2" t="inlineStr">
-        <is>
-          <t>09/06/2026 01:53 p. m.</t>
-        </is>
-      </c>
+      <c r="A194" s="2" t="inlineStr"/>
       <c r="B194" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5725,17 +5689,17 @@
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D194" s="3" t="inlineStr">
         <is>
-          <t>Tribunal prohíbe la propaganda política con la expresión “firmes por la patria”</t>
+          <t>De la Espriella (52,6%) le saca 8 puntos a Cepeda (44,8%), según nueva encuesta de AtlasIntel: así va la tendencia</t>
         </is>
       </c>
       <c r="E194" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/tribunal-prohibe-la-propaganda-politica-con-la-expresion-firmes-por-la-patria</t>
+          <t>https://www.elcolombiano.com/especiales/elecciones-2026/encuestas-atlas-intel-de-la-espriella-ivan-cepeda-segunda-vuelta-intencion-voto-FG37570577</t>
         </is>
       </c>
     </row>
@@ -5753,12 +5717,12 @@
       </c>
       <c r="D195" s="6" t="inlineStr">
         <is>
-          <t>Petro planeaba reunirse con el alcalde de Nueva York, pero el gobierno Trump amenazó con arrestarlo si realizaba actividades diferentes a su agenda en la ONU</t>
+          <t>Colombia llegó a México a la Academia Atlas, “casa” de Camilo Vargas, donde se concentrará para el Mundial</t>
         </is>
       </c>
       <c r="E195" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/departamento-de-estado-amenaza-arresto-gustavo-petro-reunion-alcalde-nueva-york-GG37571250</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/seleccion-colombia-guadalajara-atlas-mexico-camilo-vargas-mundial-2026-concentracion-CH37568309</t>
         </is>
       </c>
     </row>
@@ -5776,12 +5740,12 @@
       </c>
       <c r="D196" s="3" t="inlineStr">
         <is>
-          <t>De la Espriella (52,6%) le saca 8 puntos a Cepeda (44,8%), según nueva encuesta de AtlasIntel: así va la tendencia</t>
+          <t>Aplazan elección de rector en la Universidad de Antioquia, ¿qué pasó?</t>
         </is>
       </c>
       <c r="E196" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/elecciones-2026/encuestas-atlas-intel-de-la-espriella-ivan-cepeda-segunda-vuelta-intencion-voto-FG37570577</t>
+          <t>https://www.elcolombiano.com/antioquia/universidad-de-antioquia-rector-eleccion-GH37564507</t>
         </is>
       </c>
     </row>
@@ -5799,12 +5763,12 @@
       </c>
       <c r="D197" s="6" t="inlineStr">
         <is>
-          <t>Colombia llegó a México a la Academia Atlas, “casa” de Camilo Vargas, donde se concentrará para el Mundial</t>
+          <t>Estos son los ocho congresistas que renunciaron para ir por alcaldías y gobernaciones, ¿podría haber más?</t>
         </is>
       </c>
       <c r="E197" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/mundial-2026/seleccion-colombia-guadalajara-atlas-mexico-camilo-vargas-mundial-2026-concentracion-CH37568309</t>
+          <t>https://www.elcolombiano.com/colombia/congresistas-renuncian-aspirar-gobernaciones-alcaldias-2027-GE37557098</t>
         </is>
       </c>
     </row>
@@ -5822,12 +5786,12 @@
       </c>
       <c r="D198" s="3" t="inlineStr">
         <is>
-          <t>Aplazan elección de rector en la Universidad de Antioquia, ¿qué pasó?</t>
+          <t>Denuncian amenazas de las disidencias a campesinos en Antioquia para voltear las elecciones</t>
         </is>
       </c>
       <c r="E198" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/antioquia/universidad-de-antioquia-rector-eleccion-GH37564507</t>
+          <t>https://www.elcolombiano.com/antioquia/disidencias-farc-amenazan-campesinos-elecciones-presidenciales-antioquia-CE37558486</t>
         </is>
       </c>
     </row>
@@ -5845,12 +5809,12 @@
       </c>
       <c r="D199" s="6" t="inlineStr">
         <is>
-          <t>Estos son los ocho congresistas que renunciaron para ir por alcaldías y gobernaciones, ¿podría haber más?</t>
+          <t>A Petro no le bastaron las redes sociales: Ahora amplificó sus polémicos trinos en el Consejo de Seguridad de la ONU</t>
         </is>
       </c>
       <c r="E199" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/congresistas-renuncian-aspirar-gobernaciones-alcaldias-2027-GE37557098</t>
+          <t>https://www.elcolombiano.com/colombia/gustavo-petro-preside-debate-onu-DF37545897</t>
         </is>
       </c>
     </row>
@@ -5868,12 +5832,12 @@
       </c>
       <c r="D200" s="3" t="inlineStr">
         <is>
-          <t>Denuncian amenazas de las disidencias a campesinos en Antioquia para voltear las elecciones</t>
+          <t>CIDH ordenó el cierre de El Helicoide, el temido centro de torturas del chavismo en Venezuela</t>
         </is>
       </c>
       <c r="E200" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/antioquia/disidencias-farc-amenazan-campesinos-elecciones-presidenciales-antioquia-CE37558486</t>
+          <t>https://www.elcolombiano.com/internacional/cidh-ordeno-cerrar-temido-centro-de-tortura-en-venezuela-FE37556131</t>
         </is>
       </c>
     </row>
@@ -5891,12 +5855,12 @@
       </c>
       <c r="D201" s="6" t="inlineStr">
         <is>
-          <t>A Petro no le bastaron las redes sociales: Ahora amplificó sus polémicos trinos en el Consejo de Seguridad de la ONU</t>
+          <t>Operativo destapa helicóptero con pasado oscuro y motor Rolls-Royce</t>
         </is>
       </c>
       <c r="E201" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/gustavo-petro-preside-debate-onu-DF37545897</t>
+          <t>https://www.elcolombiano.com/colombia/ejercito-incauta-helicoptero-de-la-mafia-NG33717192</t>
         </is>
       </c>
     </row>
@@ -5914,12 +5878,12 @@
       </c>
       <c r="D202" s="3" t="inlineStr">
         <is>
-          <t>CIDH ordenó el cierre de El Helicoide, el temido centro de torturas del chavismo en Venezuela</t>
+          <t>Irán acusó a EE. UU. de usar el Mundial para “humillar y discriminar” a otras naciones</t>
         </is>
       </c>
       <c r="E202" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/internacional/cidh-ordeno-cerrar-temido-centro-de-tortura-en-venezuela-FE37556131</t>
+          <t>https://www.elcolombiano.com/deportes/futbol/iran-acusa-ee-uu-usar-mundial-humillar-y-discriminar-otras-naciones-PG37574803</t>
         </is>
       </c>
     </row>
@@ -5937,12 +5901,12 @@
       </c>
       <c r="D203" s="6" t="inlineStr">
         <is>
-          <t>Operativo destapa helicóptero con pasado oscuro y motor Rolls-Royce</t>
+          <t>Consternación en La Ceja tras hallazgo del cadáver de mujer trans en un río</t>
         </is>
       </c>
       <c r="E203" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/ejercito-incauta-helicoptero-de-la-mafia-NG33717192</t>
+          <t>https://www.elcolombiano.com/antioquia/la-chapola-mujer-trans-hallada-muerta-en-la-ceja-antioquia-DG37575152</t>
         </is>
       </c>
     </row>
@@ -5960,12 +5924,12 @@
       </c>
       <c r="D204" s="3" t="inlineStr">
         <is>
-          <t>Irán acusó a EE. UU. de usar el Mundial para “humillar y discriminar” a otras naciones</t>
+          <t>Intentó atracar a un turista con un arma en El Poblado y lo capturó la Policía</t>
         </is>
       </c>
       <c r="E204" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/deportes/futbol/iran-acusa-ee-uu-usar-mundial-humillar-y-discriminar-otras-naciones-PG37574803</t>
+          <t>https://www.elcolombiano.com/medellin/captura-ladron-intento-robo-turista-extranjero-el-poblado-medellin-GG37574453</t>
         </is>
       </c>
     </row>
@@ -5983,12 +5947,12 @@
       </c>
       <c r="D205" s="6" t="inlineStr">
         <is>
-          <t>Consternación en La Ceja tras hallazgo del cadáver de mujer trans en un río</t>
+          <t>Comisión de Acusaciones abrió investigación contra Petro por compra de aviones Gripen; MinDefensa respondió</t>
         </is>
       </c>
       <c r="E205" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/antioquia/la-chapola-mujer-trans-hallada-muerta-en-la-ceja-antioquia-DG37575152</t>
+          <t>https://www.elcolombiano.com/colombia/comision-acusaciones-investigacion-petro-aviones-gripen-BG37573031</t>
         </is>
       </c>
     </row>
@@ -6006,12 +5970,12 @@
       </c>
       <c r="D206" s="3" t="inlineStr">
         <is>
-          <t>Intentó atracar a un turista con un arma en El Poblado y lo capturó la Policía</t>
+          <t>Trabajadores del Hospital La María que sacaron a un paciente a la calle fueron apartados de sus cargos</t>
         </is>
       </c>
       <c r="E206" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/medellin/captura-ladron-intento-robo-turista-extranjero-el-poblado-medellin-GG37574453</t>
+          <t>https://www.elcolombiano.com/antioquia/suspenden-trabajadores-hospital-la-maria-por-abandonar-paciente-en-la-calle-PG37572962</t>
         </is>
       </c>
     </row>
@@ -6029,12 +5993,12 @@
       </c>
       <c r="D207" s="6" t="inlineStr">
         <is>
-          <t>Comisión de Acusaciones abrió investigación contra Petro por compra de aviones Gripen; MinDefensa respondió</t>
+          <t>El día de la revelación llega a cines: ¿es la despedida de Spielberg?</t>
         </is>
       </c>
       <c r="E207" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/comision-acusaciones-investigacion-petro-aviones-gripen-BG37573031</t>
+          <t>https://www.elcolombiano.com/cultura/cine/spielberg-dia-revelacion-estreno-retiro-legado-ciencia-ficcion-2026-GG37570475</t>
         </is>
       </c>
     </row>
@@ -6052,12 +6016,12 @@
       </c>
       <c r="D208" s="3" t="inlineStr">
         <is>
-          <t>Trabajadores del Hospital La María que sacaron a un paciente a la calle fueron apartados de sus cargos</t>
+          <t>El registrador reveló si habrá cambios en el tarjetón tras fallo contra logo de De la Espriella</t>
         </is>
       </c>
       <c r="E208" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/antioquia/suspenden-trabajadores-hospital-la-maria-por-abandonar-paciente-en-la-calle-PG37572962</t>
+          <t>https://www.elcolombiano.com/colombia/registradoria-cambios-tarjeton-segunda-vuelta-fallo-abelardo-espriella-logo-OH37568204</t>
         </is>
       </c>
     </row>
@@ -6075,12 +6039,12 @@
       </c>
       <c r="D209" s="6" t="inlineStr">
         <is>
-          <t>El día de la revelación llega a cines: ¿es la despedida de Spielberg?</t>
+          <t>Andrey Estupiñán es el goleador de la Liga Betplay, ¿porqué le ganó el premio a Luis Muriel si ambos anotaron la misma cantidad de goles?</t>
         </is>
       </c>
       <c r="E209" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/cultura/cine/spielberg-dia-revelacion-estreno-retiro-legado-ciencia-ficcion-2026-GG37570475</t>
+          <t>https://www.elcolombiano.com/deportes/futbol/andrey-estupinan-goleador-liga-betplay-fpc-luis-muriel-BH37569923</t>
         </is>
       </c>
     </row>
@@ -6098,12 +6062,12 @@
       </c>
       <c r="D210" s="3" t="inlineStr">
         <is>
-          <t>El registrador reveló si habrá cambios en el tarjetón tras fallo contra logo de De la Espriella</t>
+          <t>Petroleras colombianas ya miran a Venezuela ante el freno de Petro a la exploración</t>
         </is>
       </c>
       <c r="E210" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/registradoria-cambios-tarjeton-segunda-vuelta-fallo-abelardo-espriella-logo-OH37568204</t>
+          <t>https://www.elcolombiano.com/negocios/empresas-petroleras-colombia-venezuela-exploracion-campetrol-CH37567317</t>
         </is>
       </c>
     </row>
@@ -6121,12 +6085,12 @@
       </c>
       <c r="D211" s="6" t="inlineStr">
         <is>
-          <t>Andrey Estupiñán es el goleador de la Liga Betplay, ¿porqué le ganó el premio a Luis Muriel si ambos anotaron la misma cantidad de goles?</t>
+          <t>Anthony Gordon lideró goleada de Inglaterra sobre Costa Rica en amistoso premundialista</t>
         </is>
       </c>
       <c r="E211" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/deportes/futbol/andrey-estupinan-goleador-liga-betplay-fpc-luis-muriel-BH37569923</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/inglaterra-goles-partido-costa-rica-mundial-norteamerica-2026-DG37570254</t>
         </is>
       </c>
     </row>
@@ -6144,12 +6108,12 @@
       </c>
       <c r="D212" s="3" t="inlineStr">
         <is>
-          <t>Petroleras colombianas ya miran a Venezuela ante el freno de Petro a la exploración</t>
+          <t>Tensión en Guantánamo: jefe del Pentágono frena el rearme de Cuba y advirtió que no tolerará amenazas EE. UU.</t>
         </is>
       </c>
       <c r="E212" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/negocios/empresas-petroleras-colombia-venezuela-exploracion-campetrol-CH37567317</t>
+          <t>https://www.elcolombiano.com/internacional/jefe-pentagono-pete-hegseth-compra-armas-cuba-advierte-amenazas-florida-LE37556739</t>
         </is>
       </c>
     </row>
@@ -6167,12 +6131,12 @@
       </c>
       <c r="D213" s="6" t="inlineStr">
         <is>
-          <t>Anthony Gordon lideró goleada de Inglaterra sobre Costa Rica en amistoso premundialista</t>
+          <t>Portugal sufrió en su último partido amistoso antes de enfrentar a Colombia en el Mundial: venció 2-1 a Nigeria</t>
         </is>
       </c>
       <c r="E213" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/mundial-2026/inglaterra-goles-partido-costa-rica-mundial-norteamerica-2026-DG37570254</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/portugal-partido-nigeria-amistoso-mundial-rival-colombia-cristiano-ronaldo-hoy-JH37564490</t>
         </is>
       </c>
     </row>
@@ -6190,12 +6154,12 @@
       </c>
       <c r="D214" s="3" t="inlineStr">
         <is>
-          <t>Tensión en Guantánamo: jefe del Pentágono frena el rearme de Cuba y advirtió que no tolerará amenazas EE. UU.</t>
+          <t>Si Nacional vende a Juan Manuel Rengifo, ¿quién ocuparía su lugar?</t>
         </is>
       </c>
       <c r="E214" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/internacional/jefe-pentagono-pete-hegseth-compra-armas-cuba-advierte-amenazas-florida-LE37556739</t>
+          <t>https://www.elcolombiano.com/deportes/futbol/atletico-nacional-interes-juan-manuel-rengifo-brasil-europa-equipos-reemplazo-valor-MH37569566</t>
         </is>
       </c>
     </row>
@@ -6213,12 +6177,12 @@
       </c>
       <c r="D215" s="6" t="inlineStr">
         <is>
-          <t>Portugal sufrió en su último partido amistoso antes de enfrentar a Colombia en el Mundial: venció 2-1 a Nigeria</t>
+          <t>¿Regresará Sebastián Pérez a Nacional?</t>
         </is>
       </c>
       <c r="E215" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/mundial-2026/portugal-partido-nigeria-amistoso-mundial-rival-colombia-cristiano-ronaldo-hoy-JH37564490</t>
+          <t>https://www.elcolombiano.com/multimedia/videos/regresara-sebastian-perez-a-nacional-OH37567966</t>
         </is>
       </c>
     </row>
@@ -6236,12 +6200,12 @@
       </c>
       <c r="D216" s="3" t="inlineStr">
         <is>
-          <t>Si Nacional vende a Juan Manuel Rengifo, ¿quién ocuparía su lugar?</t>
+          <t>Congreso aprueba nuevo Régimen Sancionatorio Aduanero y evita riesgo fiscal de $3,2 billones en Colombia</t>
         </is>
       </c>
       <c r="E216" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/deportes/futbol/atletico-nacional-interes-juan-manuel-rengifo-brasil-europa-equipos-reemplazo-valor-MH37569566</t>
+          <t>https://www.elcolombiano.com/negocios/colombia-aprueba-nuevo-regimen-sancionatorio-aduanero-evita-vacio-legal-GH37567133</t>
         </is>
       </c>
     </row>
@@ -6259,12 +6223,12 @@
       </c>
       <c r="D217" s="6" t="inlineStr">
         <is>
-          <t>¿Regresará Sebastián Pérez a Nacional?</t>
+          <t>General (r) José Pastor Ruiz Mahecha es excluido de la JEP por no aportar a la verdad sobre falsos positivos</t>
         </is>
       </c>
       <c r="E217" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/multimedia/videos/regresara-sebastian-perez-a-nacional-OH37567966</t>
+          <t>https://www.elcolombiano.com/colombia/falsos-positivos-jose-pastor-ruiz-mahecha-excluido-jep-no-aportar-verdad-DE37552010</t>
         </is>
       </c>
     </row>
@@ -6282,12 +6246,12 @@
       </c>
       <c r="D218" s="3" t="inlineStr">
         <is>
-          <t>Congreso aprueba nuevo Régimen Sancionatorio Aduanero y evita riesgo fiscal de $3,2 billones en Colombia</t>
+          <t>Bill Gates declaró en el Congreso de EE. UU. que Epstein lo chantajeaba para no revelar sus “infidelidades”</t>
         </is>
       </c>
       <c r="E218" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/negocios/colombia-aprueba-nuevo-regimen-sancionatorio-aduanero-evita-vacio-legal-GH37567133</t>
+          <t>https://www.elcolombiano.com/internacional/bill-gates-niega-conocer-delitos-sexuales-de-jeffrey-epstein-NH37561286</t>
         </is>
       </c>
     </row>
@@ -6305,12 +6269,12 @@
       </c>
       <c r="D219" s="6" t="inlineStr">
         <is>
-          <t>General (r) José Pastor Ruiz Mahecha es excluido de la JEP por no aportar a la verdad sobre falsos positivos</t>
+          <t>¿Otra vez? Militante de la campaña de Cepeda pide “dejar ese tema de la ética”</t>
         </is>
       </c>
       <c r="E219" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/falsos-positivos-jose-pastor-ruiz-mahecha-excluido-jep-no-aportar-verdad-DE37552010</t>
+          <t>https://www.elcolombiano.com/especiales/elecciones-2026/ivan-cepeda-campana-linea-etica-bolivar-GF37545605</t>
         </is>
       </c>
     </row>
@@ -6328,12 +6292,12 @@
       </c>
       <c r="D220" s="3" t="inlineStr">
         <is>
-          <t>Bill Gates declaró en el Congreso de EE. UU. que Epstein lo chantajeaba para no revelar sus “infidelidades”</t>
+          <t>Reforzarán esquemas de seguridad de candidatos en medio de acusaciones mutuas de autoatentados</t>
         </is>
       </c>
       <c r="E220" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/internacional/bill-gates-niega-conocer-delitos-sexuales-de-jeffrey-epstein-NH37561286</t>
+          <t>https://www.elcolombiano.com/especiales/elecciones-2026/campana-presidencial-reforzaran-esquemas-seguridad-candidatos-quejas-autoatentados-BC37537350</t>
         </is>
       </c>
     </row>
@@ -6351,12 +6315,12 @@
       </c>
       <c r="D221" s="6" t="inlineStr">
         <is>
-          <t>¿Otra vez? Militante de la campaña de Cepeda pide “dejar ese tema de la ética”</t>
+          <t>El puesto de votación en San Diego que desató polémica en Medellín tendrá modificaciones para la segunda vuelta</t>
         </is>
       </c>
       <c r="E221" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/elecciones-2026/ivan-cepeda-campana-linea-etica-bolivar-GF37545605</t>
+          <t>https://www.elcolombiano.com/medellin/puesto-de-votacion-medellin-centro-comercial-san-diego-cambio-OC37535281</t>
         </is>
       </c>
     </row>
@@ -6374,12 +6338,12 @@
       </c>
       <c r="D222" s="3" t="inlineStr">
         <is>
-          <t>Reforzarán esquemas de seguridad de candidatos en medio de acusaciones mutuas de autoatentados</t>
+          <t>¿El Pacto Histórico respetará los resultados de la segunda vuelta? La respuesta confusa de María Fernanda Carrascal</t>
         </is>
       </c>
       <c r="E222" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/elecciones-2026/campana-presidencial-reforzaran-esquemas-seguridad-candidatos-quejas-autoatentados-BC37537350</t>
+          <t>https://www.elcolombiano.com/especiales/elecciones-2026/ivan-cepeda-segunda-vuelta-maria-fernanda-carrascal-resultados-OD37529043</t>
         </is>
       </c>
     </row>
@@ -6392,17 +6356,17 @@
       </c>
       <c r="C223" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D223" s="6" t="inlineStr">
         <is>
-          <t>El puesto de votación en San Diego que desató polémica en Medellín tendrá modificaciones para la segunda vuelta</t>
+          <t>Abelardo de la Espriella (52,6 %) le saca casi 8 puntos de ventaja a Iván Cepeda (44,8 %), a 11 días de la segunda vuelta presidencial, según nueva encuesta de AtlasIntel</t>
         </is>
       </c>
       <c r="E223" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/medellin/puesto-de-votacion-medellin-centro-comercial-san-diego-cambio-OC37535281</t>
+          <t>https://www.semana.com/politica/articulo/abelardo-de-la-espriella-526-le-saca-casi-8-puntos-a-ivan-cepeda-448-a-11-dias-de-la-segunda-vuelta-presidencial-segun-nueva-encuesta-de-atlasintel/202602/</t>
         </is>
       </c>
     </row>
@@ -6415,17 +6379,17 @@
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D224" s="3" t="inlineStr">
         <is>
-          <t>¿El Pacto Histórico respetará los resultados de la segunda vuelta? La respuesta confusa de María Fernanda Carrascal</t>
+          <t>Fuerte reproche de Petro a Abelardo de la Espriella por no acatar prohibición de usar la frase “firmes por la patria”</t>
         </is>
       </c>
       <c r="E224" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/elecciones-2026/ivan-cepeda-segunda-vuelta-maria-fernanda-carrascal-resultados-OD37529043</t>
+          <t>https://www.semana.com/politica/articulo/fuerte-reproche-de-petro-a-abelardo-de-la-espriella-por-no-acatar-prohibicion-de-usar-la-frase-firmes-por-la-patria/202635/</t>
         </is>
       </c>
     </row>
@@ -6443,12 +6407,12 @@
       </c>
       <c r="D225" s="6" t="inlineStr">
         <is>
-          <t>Abelardo de la Espriella (52,6 %) le saca casi 8 puntos de ventaja a Iván Cepeda (44,8 %), a 11 días de la segunda vuelta presidencial, según nueva encuesta de AtlasIntel</t>
+          <t>Donald Trump envía nuevo respaldo a Abelardo de la Espriella, tras intervención de Gustavo Petro en la ONU</t>
         </is>
       </c>
       <c r="E225" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/abelardo-de-la-espriella-526-le-saca-casi-8-puntos-a-ivan-cepeda-448-a-11-dias-de-la-segunda-vuelta-presidencial-segun-nueva-encuesta-de-atlasintel/202602/</t>
+          <t>https://www.semana.com/mundo/articulo/donald-trump-envia-nuevo-respaldo-a-abelardo-de-la-espriella-tras-intervencion-de-gustavo-petro-en-la-onu/202619/</t>
         </is>
       </c>
     </row>
@@ -6466,12 +6430,12 @@
       </c>
       <c r="D226" s="3" t="inlineStr">
         <is>
-          <t>Fuerte reproche de Petro a Abelardo de la Espriella por no acatar prohibición de usar la frase “firmes por la patria”</t>
+          <t>Primeras imágenes de la llegada de la Selección Colombia a Guadalajara: se calienta el debut del Mundial 2026</t>
         </is>
       </c>
       <c r="E226" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/fuerte-reproche-de-petro-a-abelardo-de-la-espriella-por-no-acatar-prohibicion-de-usar-la-frase-firmes-por-la-patria/202635/</t>
+          <t>https://www.semana.com/deportes/articulo/primeras-imagenes-de-la-llegada-de-la-seleccion-colombia-a-guadalajara-se-calienta-el-debut-del-mundial-2026/202637/</t>
         </is>
       </c>
     </row>
@@ -6489,12 +6453,12 @@
       </c>
       <c r="D227" s="6" t="inlineStr">
         <is>
-          <t>Donald Trump envía nuevo respaldo a Abelardo de la Espriella, tras intervención de Gustavo Petro en la ONU</t>
+          <t>Esta es la millonaria indemnización que solicitaron los padres de Valeria Afanador al Gimnasio Los Laureles</t>
         </is>
       </c>
       <c r="E227" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/mundo/articulo/donald-trump-envia-nuevo-respaldo-a-abelardo-de-la-espriella-tras-intervencion-de-gustavo-petro-en-la-onu/202619/</t>
+          <t>https://www.semana.com/nacion/articulo/esta-es-la-millonaria-indemnizacion-que-solicitaron-los-padres-de-valeria-afanador-al-gimnasio-los-laureles/202635/</t>
         </is>
       </c>
     </row>
@@ -6512,12 +6476,12 @@
       </c>
       <c r="D228" s="3" t="inlineStr">
         <is>
-          <t>Primeras imágenes de la llegada de la Selección Colombia a Guadalajara: se calienta el debut del Mundial 2026</t>
+          <t>“Es un asilado político, no un prófugo”: Defensa de Carlos Ramón González rechazó calificativos de la Fiscalía</t>
         </is>
       </c>
       <c r="E228" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/primeras-imagenes-de-la-llegada-de-la-seleccion-colombia-a-guadalajara-se-calienta-el-debut-del-mundial-2026/202637/</t>
+          <t>https://www.semana.com/nacion/articulo/es-un-asilado-politico-no-un-profugo-defensa-de-carlos-ramon-gonzalez-rechazo-calificativos-de-la-fiscalia/202659/</t>
         </is>
       </c>
     </row>
@@ -6535,12 +6499,12 @@
       </c>
       <c r="D229" s="6" t="inlineStr">
         <is>
-          <t>Esta es la millonaria indemnización que solicitaron los padres de Valeria Afanador al Gimnasio Los Laureles</t>
+          <t>🔴 Simulador del Mundial 2026 | Arme el fixture completo y defina a su campeón</t>
         </is>
       </c>
       <c r="E229" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/esta-es-la-millonaria-indemnizacion-que-solicitaron-los-padres-de-valeria-afanador-al-gimnasio-los-laureles/202635/</t>
+          <t>https://www.semana.com/deportes/especiales-multimedia/articulo/mundial-2026-el-simulador-con-el-que-usted-puede-jugar-y-atinar-hasta-que-haya-campeon/202529/</t>
         </is>
       </c>
     </row>
@@ -6558,12 +6522,12 @@
       </c>
       <c r="D230" s="3" t="inlineStr">
         <is>
-          <t>“Es un asilado político, no un prófugo”: Defensa de Carlos Ramón González rechazó calificativos de la Fiscalía</t>
+          <t>Esposa de Cristian Herrera relata el angustiante momento y las últimas palabras del periodista asesinado en Cúcuta: “Me mataron”</t>
         </is>
       </c>
       <c r="E230" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/es-un-asilado-politico-no-un-profugo-defensa-de-carlos-ramon-gonzalez-rechazo-calificativos-de-la-fiscalia/202659/</t>
+          <t>https://www.semana.com/nacion/articulo/esposa-de-cristian-herrera-relata-el-angustiante-momento-y-las-ultimas-palabras-del-periodista-asesinado-en-cucuta-me-mataron/202615/</t>
         </is>
       </c>
     </row>
@@ -6581,12 +6545,12 @@
       </c>
       <c r="D231" s="6" t="inlineStr">
         <is>
-          <t>🔴 Simulador del Mundial 2026 | Arme el fixture completo y defina a su campeón</t>
+          <t>¿Qué partidos del Mundial 2026 se juegan este 11 de junio? Fecha, horario y canal de TV</t>
         </is>
       </c>
       <c r="E231" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/especiales-multimedia/articulo/mundial-2026-el-simulador-con-el-que-usted-puede-jugar-y-atinar-hasta-que-haya-campeon/202529/</t>
+          <t>https://www.semana.com/deportes/articulo/que-partidos-del-mundial-2026-se-juegan-este-11-de-junio-fecha-horario-y-canal-de-tv/202604/</t>
         </is>
       </c>
     </row>
@@ -6604,12 +6568,12 @@
       </c>
       <c r="D232" s="3" t="inlineStr">
         <is>
-          <t>Esposa de Cristian Herrera relata el angustiante momento y las últimas palabras del periodista asesinado en Cúcuta: “Me mataron”</t>
+          <t>Ranking FIFA para el Mundial 2026: así se ubica Colombia tras Jordania, Costa Rica y amistosos de Portugal e Inglaterra</t>
         </is>
       </c>
       <c r="E232" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/esposa-de-cristian-herrera-relata-el-angustiante-momento-y-las-ultimas-palabras-del-periodista-asesinado-en-cucuta-me-mataron/202615/</t>
+          <t>https://www.semana.com/deportes/articulo/ranking-fifa-para-el-mundial-2026-asi-se-ubica-colombia-tras-jordania-costa-rica-y-amistosos-de-portugal-e-inglaterra/202631/</t>
         </is>
       </c>
     </row>
@@ -6627,12 +6591,12 @@
       </c>
       <c r="D233" s="6" t="inlineStr">
         <is>
-          <t>¿Qué partidos del Mundial 2026 se juegan este 11 de junio? Fecha, horario y canal de TV</t>
+          <t>Ley seca en Bogotá para la segunda vuelta de las elecciones a Presidente: horarios, restricciones y multas</t>
         </is>
       </c>
       <c r="E233" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/que-partidos-del-mundial-2026-se-juegan-este-11-de-junio-fecha-horario-y-canal-de-tv/202604/</t>
+          <t>https://www.semana.com/nacion/bogota/articulo/ley-seca-en-bogota-para-la-segunda-vuelta-de-las-elecciones-a-presidente-horarios-restricciones-y-multas/202616/</t>
         </is>
       </c>
     </row>
@@ -6650,12 +6614,12 @@
       </c>
       <c r="D234" s="3" t="inlineStr">
         <is>
-          <t>Ranking FIFA para el Mundial 2026: así se ubica Colombia tras Jordania, Costa Rica y amistosos de Portugal e Inglaterra</t>
+          <t>¿Le robaron mientras moría? Amigas de Yulixa Toloza serán investigadas por presunta omisión de socorro</t>
         </is>
       </c>
       <c r="E234" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/ranking-fifa-para-el-mundial-2026-asi-se-ubica-colombia-tras-jordania-costa-rica-y-amistosos-de-portugal-e-inglaterra/202631/</t>
+          <t>https://www.semana.com/nacion/articulo/le-robaron-mientras-moria-amigas-de-yulixa-toloza-seran-investigadas-por-presunta-omision-de-socorro/202631/</t>
         </is>
       </c>
     </row>
@@ -6673,12 +6637,12 @@
       </c>
       <c r="D235" s="6" t="inlineStr">
         <is>
-          <t>Ley seca en Bogotá para la segunda vuelta de las elecciones a Presidente: horarios, restricciones y multas</t>
+          <t>Alcalde Galán promete recuperar estas zonas públicas que son utilizadas para delinquir</t>
         </is>
       </c>
       <c r="E235" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/bogota/articulo/ley-seca-en-bogota-para-la-segunda-vuelta-de-las-elecciones-a-presidente-horarios-restricciones-y-multas/202616/</t>
+          <t>https://www.semana.com/nacion/bogota/articulo/alcalde-galan-promete-recuperar-estas-zonas-publicas-que-son-utilizadas-para-delinquir/202634/</t>
         </is>
       </c>
     </row>
@@ -6696,12 +6660,12 @@
       </c>
       <c r="D236" s="3" t="inlineStr">
         <is>
-          <t>¿Le robaron mientras moría? Amigas de Yulixa Toloza serán investigadas por presunta omisión de socorro</t>
+          <t>Sergio Fajardo, sin candidato para la segunda vuelta, presenta nuevo listado de cualidades que debe cumplir el próximo presidente</t>
         </is>
       </c>
       <c r="E236" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/le-robaron-mientras-moria-amigas-de-yulixa-toloza-seran-investigadas-por-presunta-omision-de-socorro/202631/</t>
+          <t>https://www.semana.com/politica/articulo/sergio-fajardo-sin-candidato-para-la-segunda-vuelta-saca-nuevo-listado-de-cualidades-que-debe-cumplir-el-proximo-presidente/202640/</t>
         </is>
       </c>
     </row>
@@ -6719,12 +6683,12 @@
       </c>
       <c r="D237" s="6" t="inlineStr">
         <is>
-          <t>Alcalde Galán promete recuperar estas zonas públicas que son utilizadas para delinquir</t>
+          <t>EE. UU. dice que terminó nueva ola de ataques contra Irán y se refiere a presunto cierre del estrecho de Ormuz</t>
         </is>
       </c>
       <c r="E237" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/bogota/articulo/alcalde-galan-promete-recuperar-estas-zonas-publicas-que-son-utilizadas-para-delinquir/202634/</t>
+          <t>https://www.semana.com/mundo/articulo/ee-uu-dice-que-termino-nueva-ola-de-ataques-contra-iran-y-se-refiere-a-presunto-cierre-del-estrecho-de-ormuz/202614/</t>
         </is>
       </c>
     </row>
@@ -6742,12 +6706,12 @@
       </c>
       <c r="D238" s="3" t="inlineStr">
         <is>
-          <t>Sergio Fajardo, sin candidato para la segunda vuelta, presenta nuevo listado de cualidades que debe cumplir el próximo presidente</t>
+          <t>🔴 Shakira en la inauguración del Mundial 2026 EN VIVO: la colombiana está lista para el show. “Esto ya arrancó mi gente”, dijo</t>
         </is>
       </c>
       <c r="E238" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/sergio-fajardo-sin-candidato-para-la-segunda-vuelta-saca-nuevo-listado-de-cualidades-que-debe-cumplir-el-proximo-presidente/202640/</t>
+          <t>https://www.semana.com/gente/articulo/shakira-en-la-inauguracion-del-mundial-2026-en-vivo-siga-en-directo-el-show-ultimas-noticias-y-reacciones-de-la-ceremonia/202614/</t>
         </is>
       </c>
     </row>
@@ -6765,12 +6729,12 @@
       </c>
       <c r="D239" s="6" t="inlineStr">
         <is>
-          <t>EE. UU. dice que terminó nueva ola de ataques contra Irán y se refiere a presunto cierre del estrecho de Ormuz</t>
+          <t>“Si no fuera futbolista, me habría gustado ser músico”: la inesperada confesión de Luis Díaz a Ryan Castro</t>
         </is>
       </c>
       <c r="E239" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/mundo/articulo/ee-uu-dice-que-termino-nueva-ola-de-ataques-contra-iran-y-se-refiere-a-presunto-cierre-del-estrecho-de-ormuz/202614/</t>
+          <t>https://www.semana.com/gente/articulo/si-no-fuera-futbolista-me-habria-gustado-ser-musico-la-inesperada-confesion-de-luis-diaz-a-ryan-castro/202657/</t>
         </is>
       </c>
     </row>
@@ -6788,12 +6752,12 @@
       </c>
       <c r="D240" s="3" t="inlineStr">
         <is>
-          <t>🔴 Shakira en la inauguración del Mundial 2026 EN VIVO: la colombiana está lista para el show. “Esto ya arrancó mi gente”, dijo</t>
+          <t>Expertos advierten de un botón en los celulares: al presionarlo podrían robarlo en cuestión de segundos</t>
         </is>
       </c>
       <c r="E240" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/gente/articulo/shakira-en-la-inauguracion-del-mundial-2026-en-vivo-siga-en-directo-el-show-ultimas-noticias-y-reacciones-de-la-ceremonia/202614/</t>
+          <t>https://www.semana.com/tecnologia/articulo/expertos-advierten-de-un-boton-en-los-celulares-al-presionarlo-podrian-robarlo-en-cuestion-de-segundos/202628/</t>
         </is>
       </c>
     </row>
@@ -6811,12 +6775,12 @@
       </c>
       <c r="D241" s="6" t="inlineStr">
         <is>
-          <t>“Si no fuera futbolista, me habría gustado ser músico”: la inesperada confesión de Luis Díaz a Ryan Castro</t>
+          <t>“No son mi familia de sangre”: Aida Victoria Merlano confesó quiénes la criaron en su niñez y rindió homenaje a su nana</t>
         </is>
       </c>
       <c r="E241" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/gente/articulo/si-no-fuera-futbolista-me-habria-gustado-ser-musico-la-inesperada-confesion-de-luis-diaz-a-ryan-castro/202657/</t>
+          <t>https://www.semana.com/gente/articulo/no-son-mi-familia-de-sangre-aida-victoria-merlano-confeso-quienes-la-criaron-en-su-ninez-y-rindio-homenaje-a-su-nana/202610/</t>
         </is>
       </c>
     </row>
@@ -6834,12 +6798,12 @@
       </c>
       <c r="D242" s="3" t="inlineStr">
         <is>
-          <t>Expertos advierten de un botón en los celulares: al presionarlo podrían robarlo en cuestión de segundos</t>
+          <t>Filtran medida en Selección Colombia sobre Richard Ríos: tendría efecto de cara al debut ante Uzbekistán</t>
         </is>
       </c>
       <c r="E242" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/tecnologia/articulo/expertos-advierten-de-un-boton-en-los-celulares-al-presionarlo-podrian-robarlo-en-cuestion-de-segundos/202628/</t>
+          <t>https://www.semana.com/deportes/articulo/filtran-medida-en-seleccion-colombia-sobre-richard-rios-tendria-efecto-de-cara-al-debut-ante-uzbekistan/202652/</t>
         </is>
       </c>
     </row>
@@ -6857,12 +6821,12 @@
       </c>
       <c r="D243" s="6" t="inlineStr">
         <is>
-          <t>“No son mi familia de sangre”: Aida Victoria Merlano confesó quiénes la criaron en su niñez y rindió homenaje a su nana</t>
+          <t>Corea del Sur vs. República Checa: canal y hora para ver el segundo partido del Mundial 2026</t>
         </is>
       </c>
       <c r="E243" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/gente/articulo/no-son-mi-familia-de-sangre-aida-victoria-merlano-confeso-quienes-la-criaron-en-su-ninez-y-rindio-homenaje-a-su-nana/202610/</t>
+          <t>https://www.semana.com/deportes/articulo/corea-del-sur-vs-republica-checa-canal-y-hora-para-ver-el-segundo-partido-del-mundial-2026/202602/</t>
         </is>
       </c>
     </row>
@@ -6880,12 +6844,12 @@
       </c>
       <c r="D244" s="3" t="inlineStr">
         <is>
-          <t>Filtran medida en Selección Colombia sobre Richard Ríos: tendría efecto de cara al debut ante Uzbekistán</t>
+          <t>Fifa le llama la atención a la marca colombiana Saeta: Haití sufre cambios de última hora para el Mundial 2026</t>
         </is>
       </c>
       <c r="E244" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/filtran-medida-en-seleccion-colombia-sobre-richard-rios-tendria-efecto-de-cara-al-debut-ante-uzbekistan/202652/</t>
+          <t>https://www.semana.com/deportes/articulo/fifa-le-llama-la-atencion-a-la-marca-colombiana-saeta-haiti-sufre-cambios-de-ultima-hora-para-el-mundial-2026/202612/</t>
         </is>
       </c>
     </row>
@@ -6903,12 +6867,12 @@
       </c>
       <c r="D245" s="6" t="inlineStr">
         <is>
-          <t>Corea del Sur vs. República Checa: canal y hora para ver el segundo partido del Mundial 2026</t>
+          <t>¿Se podría suspender Colombia vs. Uzbekistán en el Mundial 2026? Esto dice el reglamento de la FIFA ante el caos en México</t>
         </is>
       </c>
       <c r="E245" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/corea-del-sur-vs-republica-checa-canal-y-hora-para-ver-el-segundo-partido-del-mundial-2026/202602/</t>
+          <t>https://www.semana.com/deportes/articulo/se-podria-suspender-colombia-vs-uzbekistan-en-el-mundial-2026-esto-dice-el-reglamento-de-la-fifa-ante-el-caos-en-mexico/202657/</t>
         </is>
       </c>
     </row>
@@ -6926,12 +6890,12 @@
       </c>
       <c r="D246" s="3" t="inlineStr">
         <is>
-          <t>Fifa le llama la atención a la marca colombiana Saeta: Haití sufre cambios de última hora para el Mundial 2026</t>
+          <t>Expresidente Uribe lanzó pulla a Iván Cepeda tras su visita a Medellín: “Usted no es capaz”</t>
         </is>
       </c>
       <c r="E246" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/fifa-le-llama-la-atencion-a-la-marca-colombiana-saeta-haiti-sufre-cambios-de-ultima-hora-para-el-mundial-2026/202612/</t>
+          <t>https://www.semana.com/politica/articulo/expresidente-uribe-lanzo-pulla-a-ivan-cepeda-tras-su-visita-a-medellin-usted-no-es-capaz/202623/</t>
         </is>
       </c>
     </row>
@@ -6949,12 +6913,12 @@
       </c>
       <c r="D247" s="6" t="inlineStr">
         <is>
-          <t>¿Se podría suspender Colombia vs. Uzbekistán en el Mundial 2026? Esto dice el reglamento de la FIFA ante el caos en México</t>
+          <t>Histórico paso en Colombia: aprueban la primera ley nuclear y crean autoridad para regular el sector</t>
         </is>
       </c>
       <c r="E247" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/se-podria-suspender-colombia-vs-uzbekistan-en-el-mundial-2026-esto-dice-el-reglamento-de-la-fifa-ante-el-caos-en-mexico/202657/</t>
+          <t>https://www.semana.com/politica/articulo/historico-paso-en-colombia-aprueban-la-primera-ley-nuclear-y-crean-autoridad-para-regular-el-sector/202619/</t>
         </is>
       </c>
     </row>
@@ -6972,12 +6936,12 @@
       </c>
       <c r="D248" s="3" t="inlineStr">
         <is>
-          <t>Expresidente Uribe lanzó pulla a Iván Cepeda tras su visita a Medellín: “Usted no es capaz”</t>
+          <t>¿Reversazo en la suspensión a Gustavo Petro? Congresista matizó el auto, pidió a la Sala Plena someter la decisión “a consulta” y remitió su postura al Senado</t>
         </is>
       </c>
       <c r="E248" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/expresidente-uribe-lanzo-pulla-a-ivan-cepeda-tras-su-visita-a-medellin-usted-no-es-capaz/202623/</t>
+          <t>https://www.semana.com/politica/articulo/reversazo-en-la-suspension-a-gustavo-petro-congresista-matizo-el-auto-pidio-a-la-sala-plena-someter-la-decision-a-consulta-y-remitio-su-postura-al-senado/202648/</t>
         </is>
       </c>
     </row>
@@ -6995,12 +6959,12 @@
       </c>
       <c r="D249" s="6" t="inlineStr">
         <is>
-          <t>Histórico paso en Colombia: aprueban la primera ley nuclear y crean autoridad para regular el sector</t>
+          <t>María Fernanda Cabal se despidió del Senado: “Me voy con el orgullo de ser la mujer más votada y orgullosamente de derecha”</t>
         </is>
       </c>
       <c r="E249" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/historico-paso-en-colombia-aprueban-la-primera-ley-nuclear-y-crean-autoridad-para-regular-el-sector/202619/</t>
+          <t>https://www.semana.com/politica/articulo/maria-fernanda-cabal-se-despidio-del-senado-me-voy-con-el-orgullo-de-ser-la-mujer-mas-votada-y-orgullosamente-de-derecha/202654/</t>
         </is>
       </c>
     </row>
@@ -7018,12 +6982,12 @@
       </c>
       <c r="D250" s="3" t="inlineStr">
         <is>
-          <t>¿Reversazo en la suspensión a Gustavo Petro? Congresista matizó el auto, pidió a la Sala Plena someter la decisión “a consulta” y remitió su postura al Senado</t>
+          <t>Operativo de recuperación de espacio público en Bogotá terminó en fuertes confrontaciones: esto dijeron las autoridades</t>
         </is>
       </c>
       <c r="E250" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/reversazo-en-la-suspension-a-gustavo-petro-congresista-matizo-el-auto-pidio-a-la-sala-plena-someter-la-decision-a-consulta-y-remitio-su-postura-al-senado/202648/</t>
+          <t>https://www.semana.com/nacion/bogota/articulo/operativo-de-recuperacion-de-espacio-publico-en-bogota-termino-en-fuertes-confrontaciones-esto-dijeron-las-autoridades/202647/</t>
         </is>
       </c>
     </row>
@@ -7041,12 +7005,12 @@
       </c>
       <c r="D251" s="6" t="inlineStr">
         <is>
-          <t>María Fernanda Cabal se despidió del Senado: “Me voy con el orgullo de ser la mujer más votada y orgullosamente de derecha”</t>
+          <t>¿Dónde está Mariana Candela? Buscan a menor que desapareció en Bogotá tras salir de su hogar; la última vez que la vieron no estaba sola</t>
         </is>
       </c>
       <c r="E251" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/maria-fernanda-cabal-se-despidio-del-senado-me-voy-con-el-orgullo-de-ser-la-mujer-mas-votada-y-orgullosamente-de-derecha/202654/</t>
+          <t>https://www.semana.com/nacion/articulo/donde-esta-mariana-candela-buscan-a-menor-que-desaparecio-en-bogota-tras-salir-de-su-hogar-la-ultima-vez-que-la-vieron-no-estaba-sola/202631/</t>
         </is>
       </c>
     </row>
@@ -7064,12 +7028,12 @@
       </c>
       <c r="D252" s="3" t="inlineStr">
         <is>
-          <t>Operativo de recuperación de espacio público en Bogotá terminó en fuertes confrontaciones: esto dijeron las autoridades</t>
+          <t>Niña de cuatro años fue brutalmente golpeada por su padrastro en Sibaté: Policía y Alcaldía hablaron</t>
         </is>
       </c>
       <c r="E252" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/bogota/articulo/operativo-de-recuperacion-de-espacio-publico-en-bogota-termino-en-fuertes-confrontaciones-esto-dijeron-las-autoridades/202647/</t>
+          <t>https://www.semana.com/nacion/articulo/nina-de-cuatro-anos-fue-brutalmente-golpeada-por-su-padrastro-en-sibate-policia-y-alcaldia-hablaron/202620/</t>
         </is>
       </c>
     </row>
@@ -7082,17 +7046,17 @@
       </c>
       <c r="C253" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D253" s="6" t="inlineStr">
         <is>
-          <t>¿Dónde está Mariana Candela? Buscan a menor que desapareció en Bogotá tras salir de su hogar; la última vez que la vieron no estaba sola</t>
+          <t>CDMX La Batalla 2.0 regresa a Bogotá: música mexicana y duelo en el Astor Plaza</t>
         </is>
       </c>
       <c r="E253" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/donde-esta-mariana-candela-buscan-a-menor-que-desaparecio-en-bogota-tras-salir-de-su-hogar-la-ultima-vez-que-la-vieron-no-estaba-sola/202631/</t>
+          <t>https://canaltrece.com.co/noticias/cdmx-la-batalla-2-bogota/</t>
         </is>
       </c>
     </row>
@@ -7105,17 +7069,17 @@
       </c>
       <c r="C254" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D254" s="3" t="inlineStr">
         <is>
-          <t>Niña de cuatro años fue brutalmente golpeada por su padrastro en Sibaté: Policía y Alcaldía hablaron</t>
+          <t>Nuevo formato Mundial 2026: así cambiará la Copa del Mundo para siempre</t>
         </is>
       </c>
       <c r="E254" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/nina-de-cuatro-anos-fue-brutalmente-golpeada-por-su-padrastro-en-sibate-policia-y-alcaldia-hablaron/202620/</t>
+          <t>https://canaltrece.com.co/noticias/nuevo-formato-mundial-2026/</t>
         </is>
       </c>
     </row>
@@ -7133,12 +7097,12 @@
       </c>
       <c r="D255" s="6" t="inlineStr">
         <is>
-          <t>CDMX La Batalla 2.0 regresa a Bogotá: música mexicana y duelo en el Astor Plaza</t>
+          <t>Mundial Amazónico 2026: deporte, cultura e integración en Leticia</t>
         </is>
       </c>
       <c r="E255" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/cdmx-la-batalla-2-bogota/</t>
+          <t>https://canaltrece.com.co/noticias/mundial-amazonico-2026-deporte-cultura-e-integracion-en-leticia/</t>
         </is>
       </c>
     </row>
@@ -7156,12 +7120,12 @@
       </c>
       <c r="D256" s="3" t="inlineStr">
         <is>
-          <t>Nuevo formato Mundial 2026: así cambiará la Copa del Mundo para siempre</t>
+          <t>Selecciones sorpresa Mundial 2026: los equipos que podrían cambiar la historia</t>
         </is>
       </c>
       <c r="E256" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/nuevo-formato-mundial-2026/</t>
+          <t>https://canaltrece.com.co/noticias/selecciones-sorpresa-mundial-2026/</t>
         </is>
       </c>
     </row>
@@ -7179,12 +7143,12 @@
       </c>
       <c r="D257" s="6" t="inlineStr">
         <is>
-          <t>Mundial Amazónico 2026: deporte, cultura e integración en Leticia</t>
+          <t>Ceremonia inauguración Mundial 2026: hora, artistas y cómo verla en vivo</t>
         </is>
       </c>
       <c r="E257" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/mundial-amazonico-2026-deporte-cultura-e-integracion-en-leticia/</t>
+          <t>https://canaltrece.com.co/noticias/ceremonia-inauguracion-mundial-2026/</t>
         </is>
       </c>
     </row>
@@ -7202,12 +7166,12 @@
       </c>
       <c r="D258" s="3" t="inlineStr">
         <is>
-          <t>Selecciones sorpresa Mundial 2026: los equipos que podrían cambiar la historia</t>
+          <t>Jugadores jóvenes Mundial 2026: las promesas que podrían convertirse en estrellas</t>
         </is>
       </c>
       <c r="E258" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/selecciones-sorpresa-mundial-2026/</t>
+          <t>https://canaltrece.com.co/noticias/jugadores-jovenes-mundial-2026/</t>
         </is>
       </c>
     </row>
@@ -7225,12 +7189,12 @@
       </c>
       <c r="D259" s="6" t="inlineStr">
         <is>
-          <t>Ceremonia inauguración Mundial 2026: hora, artistas y cómo verla en vivo</t>
+          <t>La fiebre del Mundial de la FIFA 2026: El salvavidas que impulsa la economía y el consumo en Colombia</t>
         </is>
       </c>
       <c r="E259" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/ceremonia-inauguracion-mundial-2026/</t>
+          <t>https://canaltrece.com.co/noticias/la-fiebre-del-mundial-de-la-fifa-2026-el-salvavidas-que-impulsa-la-economia-y-el-consumo-en-colombia/</t>
         </is>
       </c>
     </row>
@@ -7248,12 +7212,12 @@
       </c>
       <c r="D260" s="3" t="inlineStr">
         <is>
-          <t>Jugadores jóvenes Mundial 2026: las promesas que podrían convertirse en estrellas</t>
+          <t>Fuerte operativo de recuperación de espacio público en la glorieta de la Avenida Villavicencio deja desalojos y control policial permanente</t>
         </is>
       </c>
       <c r="E260" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/jugadores-jovenes-mundial-2026/</t>
+          <t>https://canaltrece.com.co/noticias/fuerte-operativo-de-recuperacion-de-espacio-publico-en-la-glorieta-de-la-avenida-villavicencio-deja-desalojos-y-control-policial-permanente/</t>
         </is>
       </c>
     </row>
@@ -7271,12 +7235,12 @@
       </c>
       <c r="D261" s="6" t="inlineStr">
         <is>
-          <t>La fiebre del Mundial de la FIFA 2026: El salvavidas que impulsa la economía y el consumo en Colombia</t>
+          <t>El termómetro del poder: Los presidentes con mayor y menor aprobación en América Latina</t>
         </is>
       </c>
       <c r="E261" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/la-fiebre-del-mundial-de-la-fifa-2026-el-salvavidas-que-impulsa-la-economia-y-el-consumo-en-colombia/</t>
+          <t>https://canaltrece.com.co/noticias/el-termometro-del-poder-los-presidentes-con-mayor-y-menor-aprobacion-en-america-latina/</t>
         </is>
       </c>
     </row>
@@ -7294,12 +7258,12 @@
       </c>
       <c r="D262" s="3" t="inlineStr">
         <is>
-          <t>Fuerte operativo de recuperación de espacio público en la glorieta de la Avenida Villavicencio deja desalojos y control policial permanente</t>
+          <t>Los efectos de la Reforma Laboral: Más de 8.000 empresas prefieren pagar cuota de monetización al SENA que contratar aprendices</t>
         </is>
       </c>
       <c r="E262" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/fuerte-operativo-de-recuperacion-de-espacio-publico-en-la-glorieta-de-la-avenida-villavicencio-deja-desalojos-y-control-policial-permanente/</t>
+          <t>https://canaltrece.com.co/noticias/los-efectos-de-la-reforma-laboral-mas-de-8-000-empresas-prefieren-pagar-cuota-de-monetizacion-al-sena-que-contratar-aprendices/</t>
         </is>
       </c>
     </row>
@@ -7317,12 +7281,12 @@
       </c>
       <c r="D263" s="6" t="inlineStr">
         <is>
-          <t>El termómetro del poder: Los presidentes con mayor y menor aprobación en América Latina</t>
+          <t>Histórico choque institucional: Presidenta de la Comisión de Acusaciones ordena suspender provisionalmente al presidente Gustavo Petro</t>
         </is>
       </c>
       <c r="E263" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/el-termometro-del-poder-los-presidentes-con-mayor-y-menor-aprobacion-en-america-latina/</t>
+          <t>https://canaltrece.com.co/noticias/historico-choque-institucional-presidenta-de-la-comision-de-acusaciones-ordena-suspender-provisionalmente-al-presidente-gustavo-petro/</t>
         </is>
       </c>
     </row>
@@ -7340,12 +7304,12 @@
       </c>
       <c r="D264" s="3" t="inlineStr">
         <is>
-          <t>Los efectos de la Reforma Laboral: Más de 8.000 empresas prefieren pagar cuota de monetización al SENA que contratar aprendices</t>
+          <t>Tania y Violeta Bergonzi lanzan colección inspirada en la autenticidad</t>
         </is>
       </c>
       <c r="E264" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/los-efectos-de-la-reforma-laboral-mas-de-8-000-empresas-prefieren-pagar-cuota-de-monetizacion-al-sena-que-contratar-aprendices/</t>
+          <t>https://canaltrece.com.co/noticias/tania-y-violeta-bergonzi-lanzan-coleccion-inspirada-en-la-autenticidad/</t>
         </is>
       </c>
     </row>
@@ -7363,12 +7327,12 @@
       </c>
       <c r="D265" s="6" t="inlineStr">
         <is>
-          <t>Histórico choque institucional: Presidenta de la Comisión de Acusaciones ordena suspender provisionalmente al presidente Gustavo Petro</t>
+          <t>Rizadas y El Mindo lanzan Papi-Q BBQ, una edición limitada</t>
         </is>
       </c>
       <c r="E265" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/historico-choque-institucional-presidenta-de-la-comision-de-acusaciones-ordena-suspender-provisionalmente-al-presidente-gustavo-petro/</t>
+          <t>https://canaltrece.com.co/noticias/rizadas-y-el-mindo-lanzan-papi-q-bbq-una-edicion-limitada/</t>
         </is>
       </c>
     </row>
@@ -7386,12 +7350,12 @@
       </c>
       <c r="D266" s="3" t="inlineStr">
         <is>
-          <t>Tania y Violeta Bergonzi lanzan colección inspirada en la autenticidad</t>
+          <t>“Tu Casa un Estadio”: fútbol, diseño y hogar</t>
         </is>
       </c>
       <c r="E266" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/tania-y-violeta-bergonzi-lanzan-coleccion-inspirada-en-la-autenticidad/</t>
+          <t>https://canaltrece.com.co/noticias/tu-casa-un-estadio-futbol-diseno-y-hogar/</t>
         </is>
       </c>
     </row>
@@ -7409,12 +7373,12 @@
       </c>
       <c r="D267" s="6" t="inlineStr">
         <is>
-          <t>Rizadas y El Mindo lanzan Papi-Q BBQ, una edición limitada</t>
+          <t>Dos Elegidos y El Pepo Show unen al Caribe en “Entera Completa”</t>
         </is>
       </c>
       <c r="E267" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/rizadas-y-el-mindo-lanzan-papi-q-bbq-una-edicion-limitada/</t>
+          <t>https://canaltrece.com.co/noticias/dos-elegidos-y-el-pepo-show-unen-al-caribe-en-entera-completa/</t>
         </is>
       </c>
     </row>
@@ -7432,12 +7396,12 @@
       </c>
       <c r="D268" s="3" t="inlineStr">
         <is>
-          <t>“Tu Casa un Estadio”: fútbol, diseño y hogar</t>
+          <t>Ryan Castro en Cali y Bucaramanga: boletas y prerregistro</t>
         </is>
       </c>
       <c r="E268" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/tu-casa-un-estadio-futbol-diseno-y-hogar/</t>
+          <t>https://canaltrece.com.co/noticias/ryan-castro-en-cali-y-bucaramanga-boletas-y-prerregistro/</t>
         </is>
       </c>
     </row>
@@ -7455,12 +7419,12 @@
       </c>
       <c r="D269" s="6" t="inlineStr">
         <is>
-          <t>Dos Elegidos y El Pepo Show unen al Caribe en “Entera Completa”</t>
+          <t>Festival Cordillera 2026 reveló su cartel: boletas, fechas y artistas</t>
         </is>
       </c>
       <c r="E269" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/dos-elegidos-y-el-pepo-show-unen-al-caribe-en-entera-completa/</t>
+          <t>https://canaltrece.com.co/noticias/festival-cordillera-2026-cartel-boletas-fechas-y-artistas/</t>
         </is>
       </c>
     </row>
@@ -7478,12 +7442,12 @@
       </c>
       <c r="D270" s="3" t="inlineStr">
         <is>
-          <t>Ryan Castro en Cali y Bucaramanga: boletas y prerregistro</t>
+          <t>Yidy’s presenta “Soñando Descalzos”, el nacimiento de GS Dynasty: Una historia de amor, familia y música</t>
         </is>
       </c>
       <c r="E270" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/ryan-castro-en-cali-y-bucaramanga-boletas-y-prerregistro/</t>
+          <t>https://canaltrece.com.co/noticias/yidys-presenta-sonando-descalzos-el-nacimiento-de-gs-dynasty-una-historia-de-amor-familia-y-musica/</t>
         </is>
       </c>
     </row>
@@ -7501,12 +7465,12 @@
       </c>
       <c r="D271" s="6" t="inlineStr">
         <is>
-          <t>Festival Cordillera 2026 reveló su cartel: boletas, fechas y artistas</t>
+          <t>Los Hitmen reviven la esencia del perreo clásico junto a Wisin y De La Ghetto en «La Culpable»</t>
         </is>
       </c>
       <c r="E271" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/festival-cordillera-2026-cartel-boletas-fechas-y-artistas/</t>
+          <t>https://canaltrece.com.co/noticias/los-hitmen-reviven-la-esencia-del-perreo-clasico-junto-a-wisin-y-de-la-ghetto-en-la-culpable/</t>
         </is>
       </c>
     </row>
@@ -7524,12 +7488,12 @@
       </c>
       <c r="D272" s="3" t="inlineStr">
         <is>
-          <t>Yidy’s presenta “Soñando Descalzos”, el nacimiento de GS Dynasty: Una historia de amor, familia y música</t>
+          <t>¿Dificultades para tener hijos? Mitos, cuándo consultar y las técnicas avanzadas que ofrece Profamilia</t>
         </is>
       </c>
       <c r="E272" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/yidys-presenta-sonando-descalzos-el-nacimiento-de-gs-dynasty-una-historia-de-amor-familia-y-musica/</t>
+          <t>https://canaltrece.com.co/noticias/dificultades-para-tener-hijos-mitos-cuando-consultar-y-las-tecnicas-avanzadas-que-ofrece-profamilia/</t>
         </is>
       </c>
     </row>
@@ -7547,12 +7511,12 @@
       </c>
       <c r="D273" s="6" t="inlineStr">
         <is>
-          <t>Los Hitmen reviven la esencia del perreo clásico junto a Wisin y De La Ghetto en «La Culpable»</t>
+          <t>Luis7Lunes presenta «V Sabor», un álbum que explora los distintos colores del rap desde la madurez y la identidad</t>
         </is>
       </c>
       <c r="E273" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/los-hitmen-reviven-la-esencia-del-perreo-clasico-junto-a-wisin-y-de-la-ghetto-en-la-culpable/</t>
+          <t>https://canaltrece.com.co/noticias/luis7lunes-presenta-v-sabor-un-album-que-explora-los-distintos-colores-del-rap-desde-la-madurez-y-la-identidad/</t>
         </is>
       </c>
     </row>
@@ -7570,12 +7534,12 @@
       </c>
       <c r="D274" s="3" t="inlineStr">
         <is>
-          <t>¿Dificultades para tener hijos? Mitos, cuándo consultar y las técnicas avanzadas que ofrece Profamilia</t>
+          <t>Danny Polo, el enfermero que conquista la música, lanza “Lo que no sabes tú”, el sencillo principal de su EP “Momento Zero”</t>
         </is>
       </c>
       <c r="E274" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/dificultades-para-tener-hijos-mitos-cuando-consultar-y-las-tecnicas-avanzadas-que-ofrece-profamilia/</t>
+          <t>https://canaltrece.com.co/noticias/danny-polo-el-enfermero-que-conquista-la-musica-lanza-lo-que-no-sabes-tu-el-sencillo-principal-de-su-ep-momento-zero/</t>
         </is>
       </c>
     </row>
@@ -7593,12 +7557,12 @@
       </c>
       <c r="D275" s="6" t="inlineStr">
         <is>
-          <t>Luis7Lunes presenta «V Sabor», un álbum que explora los distintos colores del rap desde la madurez y la identidad</t>
+          <t>Maisak se une nuevamente a Nicky Jam en “Con Amor”: Un himno que abraza la tusa desde la gratitud</t>
         </is>
       </c>
       <c r="E275" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/luis7lunes-presenta-v-sabor-un-album-que-explora-los-distintos-colores-del-rap-desde-la-madurez-y-la-identidad/</t>
+          <t>https://canaltrece.com.co/noticias/maisak-se-une-nuevamente-a-nicky-jam-en-con-amor-un-himno-que-abraza-la-tusa-desde-la-gratitud/</t>
         </is>
       </c>
     </row>
@@ -7616,12 +7580,12 @@
       </c>
       <c r="D276" s="3" t="inlineStr">
         <is>
-          <t>Danny Polo, el enfermero que conquista la música, lanza “Lo que no sabes tú”, el sencillo principal de su EP “Momento Zero”</t>
+          <t>Soley se une a Juan Duque en “Sorry”: Un dancehall con mucha actitud para dedicarle a los ‘casi algo’</t>
         </is>
       </c>
       <c r="E276" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/danny-polo-el-enfermero-que-conquista-la-musica-lanza-lo-que-no-sabes-tu-el-sencillo-principal-de-su-ep-momento-zero/</t>
+          <t>https://canaltrece.com.co/noticias/soley-se-une-a-juan-duque-en-sorry-un-dancehall-con-mucha-actitud-para-dedicarle-a-los-casi-algo/</t>
         </is>
       </c>
     </row>
@@ -7639,12 +7603,12 @@
       </c>
       <c r="D277" s="6" t="inlineStr">
         <is>
-          <t>Maisak se une nuevamente a Nicky Jam en “Con Amor”: Un himno que abraza la tusa desde la gratitud</t>
+          <t>Maca &amp; Gero presentan “Lo Que Queda En El Aire – Live Sessions”: Una íntima experiencia acústica</t>
         </is>
       </c>
       <c r="E277" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/maisak-se-une-nuevamente-a-nicky-jam-en-con-amor-un-himno-que-abraza-la-tusa-desde-la-gratitud/</t>
+          <t>https://canaltrece.com.co/noticias/maca-gero-presentan-lo-que-queda-en-el-aire-live-sessions-una-intima-experiencia-acustica/</t>
         </is>
       </c>
     </row>
@@ -7662,12 +7626,12 @@
       </c>
       <c r="D278" s="3" t="inlineStr">
         <is>
-          <t>Soley se une a Juan Duque en “Sorry”: Un dancehall con mucha actitud para dedicarle a los ‘casi algo’</t>
+          <t>Fer Ariza apuesta por el espíritu del mundial con “Somos Latinos”</t>
         </is>
       </c>
       <c r="E278" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/soley-se-une-a-juan-duque-en-sorry-un-dancehall-con-mucha-actitud-para-dedicarle-a-los-casi-algo/</t>
+          <t>https://canaltrece.com.co/noticias/fer-ariza-apuesta-por-el-espiritu-del-mundial-con-somos-latinos/</t>
         </is>
       </c>
     </row>
@@ -7685,12 +7649,12 @@
       </c>
       <c r="D279" s="6" t="inlineStr">
         <is>
-          <t>Maca &amp; Gero presentan “Lo Que Queda En El Aire – Live Sessions”: Una íntima experiencia acústica</t>
+          <t>“El Ritmo de Verdad”, el sencillo con el que Gaia sigue conquistando la música electrónica</t>
         </is>
       </c>
       <c r="E279" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/maca-gero-presentan-lo-que-queda-en-el-aire-live-sessions-una-intima-experiencia-acustica/</t>
+          <t>https://canaltrece.com.co/noticias/el-ritmo-de-verdad-el-sencillo-con-el-que-gaia-sigue-conquistando-la-musica-electronica/</t>
         </is>
       </c>
     </row>
@@ -7708,12 +7672,12 @@
       </c>
       <c r="D280" s="3" t="inlineStr">
         <is>
-          <t>Fer Ariza apuesta por el espíritu del mundial con “Somos Latinos”</t>
+          <t>Alexis Cortés presenta “Se Vino a Beber”: Una innovadora trifusión de despecho, fiesta y verdades sin filtro</t>
         </is>
       </c>
       <c r="E280" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/fer-ariza-apuesta-por-el-espiritu-del-mundial-con-somos-latinos/</t>
+          <t>https://canaltrece.com.co/noticias/alexis-cortes-presenta-se-vino-a-beber-una-innovadora-trifusion-de-despecho-fiesta-y-verdades-sin-filtro/</t>
         </is>
       </c>
     </row>
@@ -7731,12 +7695,12 @@
       </c>
       <c r="D281" s="6" t="inlineStr">
         <is>
-          <t>“El Ritmo de Verdad”, el sencillo con el que Gaia sigue conquistando la música electrónica</t>
+          <t>A qué hora juega Colombia en el Mundial 2026</t>
         </is>
       </c>
       <c r="E281" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/el-ritmo-de-verdad-el-sencillo-con-el-que-gaia-sigue-conquistando-la-musica-electronica/</t>
+          <t>https://canaltrece.com.co/noticias/a-que-hora-juega-colombia-en-el-mundial-2026/</t>
         </is>
       </c>
     </row>
@@ -7754,63 +7718,17 @@
       </c>
       <c r="D282" s="3" t="inlineStr">
         <is>
-          <t>Alexis Cortés presenta “Se Vino a Beber”: Una innovadora trifusión de despecho, fiesta y verdades sin filtro</t>
+          <t>Colombia en el Mundial 2026: calendario, rivales y dónde ver</t>
         </is>
       </c>
       <c r="E282" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/alexis-cortes-presenta-se-vino-a-beber-una-innovadora-trifusion-de-despecho-fiesta-y-verdades-sin-filtro/</t>
-        </is>
-      </c>
-    </row>
-    <row r="283">
-      <c r="A283" s="5" t="inlineStr"/>
-      <c r="B283" s="5" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C283" s="5" t="inlineStr">
-        <is>
-          <t>Canal Trece</t>
-        </is>
-      </c>
-      <c r="D283" s="6" t="inlineStr">
-        <is>
-          <t>A qué hora juega Colombia en el Mundial 2026</t>
-        </is>
-      </c>
-      <c r="E283" s="7" t="inlineStr">
-        <is>
-          <t>https://canaltrece.com.co/noticias/a-que-hora-juega-colombia-en-el-mundial-2026/</t>
-        </is>
-      </c>
-    </row>
-    <row r="284">
-      <c r="A284" s="2" t="inlineStr"/>
-      <c r="B284" s="2" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C284" s="2" t="inlineStr">
-        <is>
-          <t>Canal Trece</t>
-        </is>
-      </c>
-      <c r="D284" s="3" t="inlineStr">
-        <is>
-          <t>Colombia en el Mundial 2026: calendario, rivales y dónde ver</t>
-        </is>
-      </c>
-      <c r="E284" s="4" t="inlineStr">
-        <is>
           <t>https://canaltrece.com.co/noticias/colombia-mundial-2026-calendario-rivales-donde-ver/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E284"/>
+  <autoFilter ref="A1:E282"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
@@ -8093,8 +8011,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E280" r:id="rId279"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E281" r:id="rId280"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E282" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E283" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E284" r:id="rId283"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Noticias actualizadas 13/06/2026 09:39
</commit_message>
<xml_diff>
--- a/docs/ultimahora.xlsx
+++ b/docs/ultimahora.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Todas las noticias" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Todas las noticias'!$A$1:$E$280</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Todas las noticias'!$A$1:$E$300</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E280"/>
+  <dimension ref="A1:E300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -515,7 +515,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 03:01 a. m.</t>
+          <t>13/06/2026 04:30 a. m.</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -530,19 +530,19 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>'La producción petrolera está relegando la transición democrática en Venezuela': analista de la Universidad de Harvard</t>
+          <t>¿Placer con Culpa? / El Condimentario</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/venezuela/la-produccion-petrolera-esta-relegando-la-transicion-democratica-en-venezuela-analista-de-la-universidad-de-harvard-3564038</t>
+          <t>https://www.eltiempo.com/cultura/gastronomia/placer-con-culpa-el-condimentario-3564022</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 02:30 a. m.</t>
+          <t>13/06/2026 04:01 a. m.</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -557,19 +557,19 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>‘Eternos’, el disco que David Bisbal esperó diez años para grabar | Entrevista</t>
+          <t>De Roma a las misas en estadios: así ha cambiado la devoción hacia el papa</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/cultura/musica-y-libros/eternos-el-disco-que-david-bisbal-espero-diez-anos-para-grabar-entrevista-3563765</t>
+          <t>https://www.eltiempo.com/vida/religion/de-roma-a-las-misas-en-estadios-asi-ha-cambiado-la-devocion-hacia-el-papa-3564052</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 02:10 a. m.</t>
+          <t>13/06/2026 03:39 a. m.</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -584,19 +584,19 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Asambleas y circulares por WhatsApp: claves para evitar vacíos legales y financieros en su conjunto</t>
+          <t>Ataque de tiburón en Sídney, Australia: cierran famosas playas como Bondi y Coogee por 24 horas</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/economia/finanzas-personales/asambleas-y-circulares-por-whatsapp-claves-para-evitar-vacios-legales-y-financieros-en-su-conjunto-3564048</t>
+          <t>https://www.eltiempo.com/mundo/mas-regiones/ataque-de-tiburon-en-sidney-australia-cierran-famosas-playas-como-bondi-y-coogee-por-24-horas-3564100</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 02:05 a. m.</t>
+          <t>13/06/2026 03:33 a. m.</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -611,19 +611,19 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Irán afirma que el acuerdo con Estados Unidos se podría firmar en los 'próximos días'</t>
+          <t>¿Por qué Cali será la ciudad más vigilada del país el 21 de junio? Las claves del operativo de seguridad que anuncia el Gobierno Nacional</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/medio-oriente/iran-afirma-que-el-acuerdo-con-estados-unidos-se-podria-firmar-en-los-proximos-dias-3564097</t>
+          <t>https://www.eltiempo.com/colombia/cali/por-que-cali-sera-la-ciudad-mas-vigilada-del-pais-el-21-de-junio-las-claves-del-operativo-de-seguridad-que-anuncia-el-gobierno-nacional-3564099</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 12:40 a. m.</t>
+          <t>13/06/2026 03:30 a. m.</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -638,19 +638,19 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Mundial 2026: Estados Unidos ganó 4-1 contra Paraguay en Los Ángeles, California</t>
+          <t>Casa Landino: un café de lujo colombiano</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/mundial-2026-estados-unidos-gano-4-1-contra-paraguay-en-los-angeles-california-3564096</t>
+          <t>https://www.eltiempo.com/cultura/gastronomia/casa-landino-un-cafe-de-lujo-colombiano-3564012</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 11:53 p. m.</t>
+          <t>13/06/2026 03:11 a. m.</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -665,19 +665,19 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Endrick, la joven estrella que va por la gloria en el Mundial: 'Quiero volver con Brasil como campeón’</t>
+          <t>Elecciones Colombia 2026: última hora de la segunda vuelta entre Abelardo de la Espriella e Iván Cepeda este 21 de junio</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/endrick-la-joven-estrella-que-va-por-la-gloria-en-el-mundial-quiero-volver-con-brasil-como-campeon-3564094</t>
+          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/elecciones-colombia-2026-ultima-hora-de-la-segunda-vuelta-entre-abelardo-de-la-espriella-e-ivan-cepeda-este-21-de-junio-3564098</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 11:48 p. m.</t>
+          <t>13/06/2026 03:01 a. m.</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -692,19 +692,19 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>¿Hora de preocuparse por el '9' de la Selección Colombia? Así están las opciones antes del debut contra Uzbekistán</t>
+          <t>'La producción petrolera está relegando la transición democrática en Venezuela': analista de la Universidad de Harvard</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/hora-de-preocuparse-por-el-9-de-la-seleccion-colombia-asi-estan-las-opciones-antes-del-debut-contra-uzbekistan-3564093</t>
+          <t>https://www.eltiempo.com/mundo/venezuela/la-produccion-petrolera-esta-relegando-la-transicion-democratica-en-venezuela-analista-de-la-universidad-de-harvard-3564038</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 11:29 p. m.</t>
+          <t>13/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -719,19 +719,19 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Videos de la balacera y sicariato cerca de estación de TransMilenio en Bogotá que dejó dos muertos y un herido: así escaparon los responsables</t>
+          <t>‘Eternos’, el disco que David Bisbal esperó diez años para grabar | Entrevista</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/bogota/videos-de-la-balacera-y-sicariato-cerca-de-estacion-de-transmilenio-en-bogota-que-dejo-dos-muertos-y-un-herido-asi-escaparon-los-responsables-3564092</t>
+          <t>https://www.eltiempo.com/cultura/musica-y-libros/eternos-el-disco-que-david-bisbal-espero-diez-anos-para-grabar-entrevista-3563765</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 11:28 p. m.</t>
+          <t>13/06/2026 02:10 a. m.</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -746,19 +746,19 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Amor, gratitud y buena onda: la consigna de un joven llamado Martín Fonseca</t>
+          <t>Asambleas y circulares por WhatsApp: claves para evitar vacíos legales y financieros en su conjunto</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/vida/tendencias/amor-gratitud-y-buena-onda-la-consigna-de-un-joven-llamado-martin-fonseca-3564008</t>
+          <t>https://www.eltiempo.com/economia/finanzas-personales/asambleas-y-circulares-por-whatsapp-claves-para-evitar-vacios-legales-y-financieros-en-su-conjunto-3564048</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 11:15 p. m.</t>
+          <t>13/06/2026 02:05 a. m.</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -773,19 +773,19 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Sobreviviente entrega detalles del dramático accidente marítimo en San Andrés que dejó a madre e hija fallecidas: 'Ahí supe que también estaba muerta'</t>
+          <t>Irán afirma que el acuerdo con Estados Unidos se podría firmar en los 'próximos días'</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/otras-ciudades/sobreviviente-entrega-detalles-del-dramatico-accidente-maritimo-en-san-andres-que-dejo-a-madre-e-hija-fallecidas-ahi-supe-que-tambien-estaba-muerta-3564091</t>
+          <t>https://www.eltiempo.com/mundo/medio-oriente/iran-afirma-que-el-acuerdo-con-estados-unidos-se-podria-firmar-en-los-proximos-dias-3564097</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 11:04 p. m.</t>
+          <t>13/06/2026 12:40 a. m.</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -800,19 +800,19 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Colombia Mayor suspenderá los pagos de sus subsidios por tres días: así será el 'blindaje electoral' de cara a la segunda vuelta presidencial</t>
+          <t>Mundial 2026: roban las botas y los balones de la selección inglesa antes de su llegada a Kansas City</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/economia/finanzas-personales/colombia-mayor-suspendera-los-pagos-de-sus-subsidios-por-tres-dias-asi-sera-el-blindaje-electoral-de-cara-a-la-segunda-vuelta-presidencial-3563950</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/mundial-2026-estados-unidos-gano-4-1-contra-paraguay-en-los-angeles-california-3564096</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 11:01 p. m.</t>
+          <t>12/06/2026 11:53 p. m.</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -827,19 +827,19 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>¡Pilas! Bogotá iniciará desde el 1 de julio la transición del Sisbén al Registro Universal de Ingresos: el periodo de implementación será de dos años</t>
+          <t>Endrick, la joven estrella que va por la gloria en el Mundial: 'Quiero volver con Brasil como campeón’</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/bogota/pilas-bogota-iniciara-desde-el-1-de-julio-la-transicion-del-sisben-al-registro-universal-de-ingresos-el-periodo-de-implementacion-sera-de-dos-anos-3563972</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/endrick-la-joven-estrella-que-va-por-la-gloria-en-el-mundial-quiero-volver-con-brasil-como-campeon-3564094</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 11:01 p. m.</t>
+          <t>12/06/2026 11:48 p. m.</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -854,19 +854,19 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>FBI indaga a alias el Faraón, la pista para llegar a los asesinos del periodista Cristian Herrera y a sus cómplices políticos</t>
+          <t>¿Hora de preocuparse por el '9' de la Selección Colombia? Así están las opciones antes del debut contra Uzbekistán</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/unidad-investigativa/fbi-indaga-a-alias-el-faraon-la-pista-para-llegar-a-los-asesinos-del-periodista-cristian-herrera-y-a-sus-complices-y-a-sus-complices-politicos-3564053</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/hora-de-preocuparse-por-el-9-de-la-seleccion-colombia-asi-estan-las-opciones-antes-del-debut-contra-uzbekistan-3564093</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 11:01 p. m.</t>
+          <t>12/06/2026 11:29 p. m.</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -881,19 +881,19 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Las jugadas de Gloria Arizabaleta, la petrista que intentó suspender al presidente y estalló nuevo escándalo en el Gobierno</t>
+          <t>Videos de la balacera y sicariato cerca de estación de TransMilenio en Bogotá que dejó dos muertos y un herido: así escaparon los responsables</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/unidad-investigativa/las-jugadas-de-gloria-arizabaleta-la-petrista-que-intento-suspender-al-presidente-y-estallo-nuevo-escandalo-en-el-gobierno-3564044</t>
+          <t>https://www.eltiempo.com/bogota/videos-de-la-balacera-y-sicariato-cerca-de-estacion-de-transmilenio-en-bogota-que-dejo-dos-muertos-y-un-herido-asi-escaparon-los-responsables-3564092</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 10:54 p. m.</t>
+          <t>12/06/2026 11:28 p. m.</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -908,19 +908,19 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>La gasolina sigue en competencia</t>
+          <t>Amor, gratitud y buena onda: la consigna de un joven llamado Martín Fonseca</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/economia/sectores/la-gasolina-sigue-en-competencia-3564090</t>
+          <t>https://www.eltiempo.com/vida/tendencias/amor-gratitud-y-buena-onda-la-consigna-de-un-joven-llamado-martin-fonseca-3564008</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 10:51 p. m.</t>
+          <t>12/06/2026 11:15 p. m.</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -935,19 +935,19 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>Investigan extraña muerte de escolta de concejal de Bogotá: fue encontrado en delicado estado de salud 36 horas después de salir de su turno</t>
+          <t>Sobreviviente entrega detalles del dramático accidente marítimo en San Andrés que dejó a madre e hija fallecidas: 'Ahí supe que también estaba muerta'</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/bogota/concejo-de-bogota-lamento-la-muerte-de-escolta-del-concejal-fernando-lopez-el-hombre-fue-encontrado-en-delicado-estado-de-salud-36-horas-despues-3564083</t>
+          <t>https://www.eltiempo.com/colombia/otras-ciudades/sobreviviente-entrega-detalles-del-dramatico-accidente-maritimo-en-san-andres-que-dejo-a-madre-e-hija-fallecidas-ahi-supe-que-tambien-estaba-muerta-3564091</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 10:48 p. m.</t>
+          <t>12/06/2026 11:04 p. m.</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -962,19 +962,19 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Venezuela confirmó operación conjunta con Estados Unidos en la que fue abatido 'Niño Guerrero', jefe del Tren de Aragua: nuevos detalles del operativo</t>
+          <t>Colombia Mayor suspenderá los pagos de sus subsidios por tres días: así será el 'blindaje electoral' de cara a la segunda vuelta presidencial</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/venezuela/venezuela-confirmo-operacion-conjunta-con-estados-unidos-en-la-que-fue-abatido-nino-guerrero-jefe-del-tren-de-aragua-nuevos-detalles-del-operativo-3564089</t>
+          <t>https://www.eltiempo.com/economia/finanzas-personales/colombia-mayor-suspendera-los-pagos-de-sus-subsidios-por-tres-dias-asi-sera-el-blindaje-electoral-de-cara-a-la-segunda-vuelta-presidencial-3563950</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 10:40 p. m.</t>
+          <t>12/06/2026 11:01 p. m.</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -989,19 +989,19 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Visas negadas, veto de viajeros y protestas: los problemas extradeportivos que marcan el arranque del Mundial de Fútbol 2026</t>
+          <t>¡Pilas! Bogotá iniciará desde el 1 de julio la transición del Sisbén al Registro Universal de Ingresos: el periodo de implementación será de dos años</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/visas-negadas-veto-de-viajeros-y-protestas-los-problemas-extradeportivos-que-marcan-el-arranque-del-mundial-de-futbol-3563946</t>
+          <t>https://www.eltiempo.com/bogota/pilas-bogota-iniciara-desde-el-1-de-julio-la-transicion-del-sisben-al-registro-universal-de-ingresos-el-periodo-de-implementacion-sera-de-dos-anos-3563972</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 10:37 p. m.</t>
+          <t>12/06/2026 11:01 p. m.</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1016,19 +1016,19 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Campaña del candidato presidencial Abelardo de la Espriella emitió alerta por existencia de estafas a su nombre: 'Ninguna persona'</t>
+          <t>FBI indaga a alias el Faraón, la pista para llegar a los asesinos del periodista Cristian Herrera y a sus cómplices políticos</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/campana-presidencial-de-abelardo-de-la-espriella-emitio-una-alerta-urgente-en-la-que-denuncia-la-existencia-de-estafas-a-su-nombre-ninguna-persona-3564085</t>
+          <t>https://www.eltiempo.com/unidad-investigativa/fbi-indaga-a-alias-el-faraon-la-pista-para-llegar-a-los-asesinos-del-periodista-cristian-herrera-y-a-sus-complices-y-a-sus-complices-politicos-3564053</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 10:29 p. m.</t>
+          <t>12/06/2026 11:01 p. m.</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
@@ -1043,12 +1043,12 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Los más buscados del frente 4 de las disidencias de las Farc: esta es alias Samantha, la 'comunicadora' de la estructura en el Nordeste de Antioquia</t>
+          <t>Las jugadas de Gloria Arizabaleta, la petrista que intentó suspender al presidente y estalló nuevo escándalo en el Gobierno</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/medellin/los-mas-buscados-del-frente-4-de-las-disidencias-de-las-farc-esta-es-alias-samantha-la-comunicadora-de-la-estructura-en-el-nordeste-de-antioquia-3564070</t>
+          <t>https://www.eltiempo.com/unidad-investigativa/las-jugadas-de-gloria-arizabaleta-la-petrista-que-intento-suspender-al-presidente-y-estallo-nuevo-escandalo-en-el-gobierno-3564044</t>
         </is>
       </c>
     </row>
@@ -1637,12 +1637,12 @@
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>La seguridad en Colombia</t>
+          <t>Votar sin miedo</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/13/la-seguridad-en-colombia/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/13/votar-sin-miedo/</t>
         </is>
       </c>
     </row>
@@ -1691,12 +1691,12 @@
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>El espejismo de los extremos: constitución o continuismo</t>
+          <t>La seguridad en Colombia</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/13/el-espejismo-de-los-extremos-constitucion-o-continuismo/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/13/la-seguridad-en-colombia/</t>
         </is>
       </c>
     </row>
@@ -1718,12 +1718,12 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Los gobiernos cambian, las instituciones permanecen</t>
+          <t>El espejismo de los extremos: constitución o continuismo</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/13/los-gobiernos-cambian-las-instituciones-permanecen/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/13/el-espejismo-de-los-extremos-constitucion-o-continuismo/</t>
         </is>
       </c>
     </row>
@@ -1745,12 +1745,12 @@
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>El presidente de Colombia no debe tener doble nacionalidad</t>
+          <t>Los gobiernos cambian, las instituciones permanecen</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/13/el-presidente-de-colombia-no-debe-tener-doble-nacionalidad/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/13/los-gobiernos-cambian-las-instituciones-permanecen/</t>
         </is>
       </c>
     </row>
@@ -2266,7 +2266,7 @@
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 11:45 p. m.</t>
+          <t>12/06/2026 11:18 p. m.</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr">
@@ -2281,19 +2281,19 @@
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>Atención viajeros: Ideam pronostica lluvias para el puente festivo del 15 de junio en gran parte del país</t>
+          <t>Así son los Twin Otter, los nuevos aviones con los que Satena llegará a las zonas más remotas en medio de la selva</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/actualidad/clima-ideam-puente-festivo-13-14-15-junio-2026-llovera-regiones-colombia-402158</t>
+          <t>https://www.lafm.com.co/orden-publico/twinn-otter-nuevos-aviones-satena-llegar-zonas-apartadas-selva-402152</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 11:18 p. m.</t>
+          <t>12/06/2026 11:03 p. m.</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -2308,19 +2308,19 @@
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>Así son los Twin Otter, los nuevos aviones con los que Satena llegará a las zonas más remotas en medio de la selva</t>
+          <t>Agmeth Escaf responde tras la sanción por insultos a De La Espriella: "No me asustan y no me retracto"</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/orden-publico/twinn-otter-nuevos-aviones-satena-llegar-zonas-apartadas-selva-402152</t>
+          <t>https://www.lafm.com.co/politica/agmeth-escaf-insultos-abelardo-de-la-espriella-sancion-no-se-retracta-demanda-402157</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 11:03 p. m.</t>
+          <t>12/06/2026 10:41 p. m.</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
@@ -2335,19 +2335,19 @@
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>Agmeth Escaf responde tras la sanción por insultos a De La Espriella: "No me asustan y no me retracto"</t>
+          <t>Código de Policía: la sanción para los vecinos que actúan de buena fe</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/agmeth-escaf-insultos-abelardo-de-la-espriella-sancion-no-se-retracta-demanda-402157</t>
+          <t>https://www.lafm.com.co/sociedad/sancion-por-instalar-contenedores-de-basura-402155</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 10:41 p. m.</t>
+          <t>12/06/2026 10:11 p. m.</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -2362,19 +2362,19 @@
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>Código de Policía: la sanción para los vecinos que actúan de buena fe</t>
+          <t>Prima de mitad de año: qué pasa si un trabajador renuncia antes de recibirla</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/sociedad/sancion-por-instalar-contenedores-de-basura-402155</t>
+          <t>https://www.lafm.com.co/sociedad/prima-mitad-ano-2026-junio-renuncia-antes-del-pago-402149</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 10:11 p. m.</t>
+          <t>04/06/2026 02:23 a. m.</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr">
@@ -2389,19 +2389,19 @@
       </c>
       <c r="D71" s="6" t="inlineStr">
         <is>
-          <t>Prima de mitad de año: qué pasa si un trabajador renuncia antes de recibirla</t>
+          <t>En medio de denuncias de censura, el presidente Petro destacó la reducción histórica de la pobreza en su gobierno</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/sociedad/prima-mitad-ano-2026-junio-renuncia-antes-del-pago-402149</t>
+          <t>https://www.lafm.com.co/politica/petro-asegura-que-colombia-tiene-pobreza-mas-baja-siglo-censura-402165</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 09:40 p. m.</t>
+          <t>20/05/2026 10:25 p. m.</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -2416,19 +2416,19 @@
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>¿Por qué el Ministerio del Trabajo frenó diligencia en la Alcaldía de Santa Marta?</t>
+          <t>¿Quién ganó las elecciones en Perú? Último reporte tras alcanzarse el 98.32 % del escrutinio de la segunda vuelta</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/por-que-el-ministerio-trabajo-frena-diligencia-en-alcaldia-de-santa-marta-402116</t>
+          <t>https://www.lafm.com.co/internacional/elecciones-presidenciales-en-peru-ultimo-reporte-tras-alcanzarse-el-9392-del-escrutinio-de-la-segunda-vuelta-401695</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>04/06/2026 02:23 a. m.</t>
+          <t>20/04/2026 08:03 p. m.</t>
         </is>
       </c>
       <c r="B73" s="5" t="inlineStr">
@@ -2443,19 +2443,19 @@
       </c>
       <c r="D73" s="6" t="inlineStr">
         <is>
-          <t>En medio de denuncias de censura, el presidente Petro destacó la reducción histórica de la pobreza en su gobierno</t>
+          <t>Ofrecen $100 millones de recompensa por encapuchado que lanzó papa bomba a vehículo en Cali</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/petro-asegura-que-colombia-tiene-pobreza-mas-baja-siglo-censura-402165</t>
+          <t>https://www.lafm.com.co/actualidad/recompensa-por-responsable-de-lanzar-papa-bomba-en-medio-de-disturbios-en-cali-402160</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>20/05/2026 10:25 p. m.</t>
+          <t>04/11/2025 01:48 p. m.</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -2470,21 +2470,17 @@
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>¿Quién ganó las elecciones en Perú? Último reporte tras alcanzarse el 98.32 % del escrutinio de la segunda vuelta</t>
+          <t>Piden apartar de su cargo al vicepresidente de Ecopetrol</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/internacional/elecciones-presidenciales-en-peru-ultimo-reporte-tras-alcanzarse-el-9392-del-escrutinio-de-la-segunda-vuelta-401695</t>
+          <t>https://www.lafm.com.co/actualidad/piden-apartar-de-su-cargo-al-vicepresidente-de-ecopetrol-402172</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="5" t="inlineStr">
-        <is>
-          <t>20/04/2026 08:03 p. m.</t>
-        </is>
-      </c>
+      <c r="A75" s="5" t="inlineStr"/>
       <c r="B75" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2497,12 +2493,12 @@
       </c>
       <c r="D75" s="6" t="inlineStr">
         <is>
-          <t>Ofrecen $100 millones de recompensa por encapuchado que lanzó papa bomba a vehículo en Cali</t>
+          <t>Atención viajeros: Ideam pronostica lluvias para el puente festivo del 15 de junio en gran parte del país</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/actualidad/recompensa-por-responsable-de-lanzar-papa-bomba-en-medio-de-disturbios-en-cali-402160</t>
+          <t>https://www.lafm.com.co/actualidad/clima-ideam-puente-festivo-13-14-15-junio-2026-llovera-regiones-colombia-402158</t>
         </is>
       </c>
     </row>
@@ -2578,7 +2574,7 @@
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 03:09 a. m.</t>
+          <t>13/06/2026 04:24 a. m.</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
@@ -2588,24 +2584,24 @@
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
         <is>
-          <t>Piden a Estados Unidos que investigue e incluya en la Lista Clinton a Ricardo Roa, presidente de Ecopetrol, por transacciones en la campaña de Petro</t>
+          <t>Resultados de loterías de Medellín, Santander, Risaralda y MiLoto hoy 12 de junio de 2026</t>
         </is>
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/piden-a-estados-unidos-que-investigue-e-incluya-en-la-lista-clinton-a-ricardo-roa-presidente-de-ecopetrol-por-transacciones-en-la-campana-de-petro/202620/</t>
+          <t>https://www.bluradio.com/economia/juegos-de-azar/resultados-de-loterias-de-medellin-santander-risaralda-y-miloto-hoy-12-de-junio-de-2026-so35</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 03:08 a. m.</t>
+          <t>13/06/2026 04:21 a. m.</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -2615,24 +2611,24 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>¿Doble rasero? Mientras se retiró a un general sin investigaciones, otros con procesos de falsos positivos, concierto para delinquir y peculado son protegidos</t>
+          <t>Resultados de MiLoto hoy 12 de junio de 2026: números ganadores y nuevo acumulado de $300 millones</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/doble-rasero-mientras-se-retiro-a-un-general-sin-investigaciones-otros-con-procesos-de-falsos-positivos-concierto-para-delinquir-y-peculado-son-protegidos/202629/</t>
+          <t>https://www.bluradio.com/economia/juegos-de-azar/resultados-de-miloto-del-12-de-junio-de-2026-numeros-ganadores-y-nuevo-acumulado-so35</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 02:49 a. m.</t>
+          <t>13/06/2026 04:13 a. m.</t>
         </is>
       </c>
       <c r="B81" s="5" t="inlineStr">
@@ -2642,24 +2638,24 @@
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D81" s="6" t="inlineStr">
         <is>
-          <t>Max Henriquez lanza alerta por fenómeno del superniño en Colombia: “Es posible que haya racionamiento de agua y energía”</t>
+          <t>Resultados Lotería de Risaralda 12 de junio de 2026: premio mayor y números ganadores de secos</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/max-henriquez-lanza-alerta-por-fenomeno-del-supernino-en-colombia-es-posible-que-haya-racionamiento-de-agua-y-energia/202629/</t>
+          <t>https://www.bluradio.com/economia/juegos-de-azar/resultados-loteria-de-risaralda-12-de-junio-de-2026-premio-mayor-y-numeros-ganadores-de-secos-so35</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 02:41 a. m.</t>
+          <t>13/06/2026 04:09 a. m.</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -2669,24 +2665,24 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>Añorado regreso de la Selección Colombia: ocho años deseándolo y así llega a la gran cita de la Copa del Mundo</t>
+          <t>Resultado Lotería de Santander hoy 12 de junio, premio mayor y secos, resultados último sorteo</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/anorado-regreso-de-la-seleccion-colombia-ocho-anos-deseandolo-y-asi-llega-a-la-gran-cita-de-la-copa-del-mundo/202656/</t>
+          <t>https://www.bluradio.com/economia/juegos-de-azar/loteria-de-santander-12-de-junio-premio-mayor-y-secos-resultados-ultimo-sorteo-so35</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 02:39 a. m.</t>
+          <t>13/06/2026 03:59 a. m.</t>
         </is>
       </c>
       <c r="B83" s="5" t="inlineStr">
@@ -2696,24 +2692,24 @@
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D83" s="6" t="inlineStr">
         <is>
-          <t>Selección Colombia: SEMANA conversó con los familiares de los convocados al Mundial 2026. Historias de sacrificio, temple y mucho amor</t>
+          <t>Lotería de Medellín hoy 12 de junio, premio mayor y secos del último sorteo</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/seleccion-colombia-semana-converso-con-los-familiares-de-los-convocados-al-mundial-2026-historias-de-sacrificio-temple-y-mucho-amor/202621/</t>
+          <t>https://www.bluradio.com/economia/juegos-de-azar/resultado-loteria-de-medellin-12-de-junio-premio-mayor-y-secos-del-ultimo-sorteo-so35</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 02:25 a. m.</t>
+          <t>12/06/2026 11:56 p. m.</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -2723,24 +2719,24 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>¿Abelardo de la Espriella, presidente? El Tigre derrotaría a Iván Cepeda en la segunda vuelta, según la más reciente encuesta de AtlasIntel</t>
+          <t>Impactante choque: policía resulta herido en persecución tras chocar de frente contra un vehículo</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/abelardo-de-la-espriella-presidente-el-tigre-derrotaria-a-ivan-cepeda-en-la-segunda-vuelta-segun-la-mas-reciente-encuesta-de-atlasintel/202644/</t>
+          <t>https://www.bluradio.com/mundo/impactante-choque-policia-resulta-herido-en-persecucion-tras-chocar-de-frente-contra-un-vehiculo-so35</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 02:10 a. m.</t>
+          <t>12/06/2026 10:46 p. m.</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr">
@@ -2750,24 +2746,24 @@
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D85" s="6" t="inlineStr">
         <is>
-          <t>Habla Sofía Otero, la doctora de la mafia</t>
+          <t>Dos militares ecuatorianos heridos en enfrentamiento con civiles armados en frontera con Colombia</t>
         </is>
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/habla-sofia-otero-la-doctora-de-la-mafia/202636/</t>
+          <t>https://www.bluradio.com/mundo/dos-militares-ecuatorianos-heridos-en-enfrentamiento-con-civiles-armados-en-frontera-con-colombia-so35</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 02:10 a. m.</t>
+          <t>12/06/2026 09:13 p. m.</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -2777,24 +2773,24 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>Clara Elvira Ospina, periodista colombiana en Perú, habla en SEMANA y anticipa triunfo de Keiko Fujimori tras largas elecciones</t>
+          <t>¿Quién era el 'Niño Guerrero', el temido líder del  Tren de Aragua abatido por Estados Unidos?</t>
         </is>
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/mundo/articulo/clara-elvira-ospina-periodista-colombiana-en-peru-habla-en-semana-y-anticipa-triunfo-de-keiko-fujimori-tras-largas-elecciones/202652/</t>
+          <t>https://www.bluradio.com/venezuela/quien-era-nino-guerrero-el-temido-lider-del-tren-de-aragua-abatido-por-estados-unidos-so35</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 02:10 a. m.</t>
+          <t>12/06/2026 08:37 p. m.</t>
         </is>
       </c>
       <c r="B87" s="5" t="inlineStr">
@@ -2804,24 +2800,24 @@
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D87" s="6" t="inlineStr">
         <is>
-          <t>Toy Story 5: Kenna Harris y Lindsey Collins hablan con SEMANA sobre el futuro de Woody, Buzz y Jessie</t>
+          <t>Trump anuncia la muerte del 'Niño Guerrero', el líder de banda venezolana Tren de Aragua</t>
         </is>
       </c>
       <c r="E87" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/cultura/cine/articulo/toy-story-5-kenna-harris-y-lindsey-collins-hablan-con-semana-sobre-el-futuro-de-woody-buzz-y-jessie/202643/</t>
+          <t>https://www.bluradio.com/mundo/trump-anuncia-la-muerte-del-nino-guerrero-el-lider-de-banda-venezolana-tren-de-aragua-cb20</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 01:10 a. m.</t>
+          <t>12/06/2026 08:18 p. m.</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -2831,22 +2827,26 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>El mercado ya apostó por un cambio de Gobierno: Acciones al alza y dólar a la baja</t>
+          <t>"El gobierno reconoce el estado calamitoso en que entrega las finanzas": ANDI sobre nueva tributaria</t>
         </is>
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/economia/macroeconomia/articulo/el-mercado-ya-aposto-por-un-cambio-de-gobierno-acciones-al-alza-y-dolar-a-la-baja/202638/</t>
+          <t>https://www.bluradio.com/economia/el-gobierno-reconoce-el-estado-calamitoso-en-que-entrega-las-finanzas-andi-sobre-nueva-tributaria-so35</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="5" t="inlineStr"/>
+      <c r="A89" s="5" t="inlineStr">
+        <is>
+          <t>12/06/2026 08:11 p. m.</t>
+        </is>
+      </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2854,22 +2854,26 @@
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D89" s="6" t="inlineStr">
         <is>
-          <t>Donald Trump anuncia la muerte de alias Niño Guerrero, líder máximo del Tren de Aragua</t>
+          <t>Astro Luna, resultado del último sorteo hoy viernes 12  de junio de 2026</t>
         </is>
       </c>
       <c r="E89" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/mundo/articulo/donald-trump-anuncia-la-muerte-de-alias-nino-guerrero-lider-maximo-del-tren-de-aragua/202639/</t>
+          <t>https://www.bluradio.com/economia/juegos-de-azar/astro-luna-resultado-del-ultimo-sorteo-hoy-viernes-12-de-junio-de-2026-so35</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="inlineStr"/>
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>12/06/2026 08:11 p. m.</t>
+        </is>
+      </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2877,22 +2881,26 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>Gustavo Petro hizo un llamado para la segunda vuelta presidencial: “Intentemos hacer vacas para financiar”</t>
+          <t>Caribeña Noche, resultado del último sorteo hoy viernes 12 de junio de 2026</t>
         </is>
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/gustavo-petro-hizo-un-llamado-para-la-segunda-vuelta-presidencial-intentemos-hacer-vacas-para-financiar/202603/</t>
+          <t>https://www.bluradio.com/economia/juegos-de-azar/caribena-noche-resultado-del-ultimo-sorteo-hoy-viernes-12-de-junio-de-2026-so35</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="5" t="inlineStr"/>
+      <c r="A91" s="5" t="inlineStr">
+        <is>
+          <t>13/06/2026 04:21 a. m.</t>
+        </is>
+      </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2900,22 +2908,26 @@
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D91" s="6" t="inlineStr">
         <is>
-          <t>Este sería el video del ataque que acabó con la vida de alias Niño Guerrero, temido líder del Tren de Aragua</t>
+          <t>Trece detenidos en Barcelona en una operación policial contra el uso de armas de fuego</t>
         </is>
       </c>
       <c r="E91" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/mundo/articulo/este-seria-el-video-del-ataque-que-acabo-con-la-vida-de-alias-nino-guerrero-temido-lider-del-tren-de-aragua/202610/</t>
+          <t>https://elpais.com/espana/catalunya/2026-06-11/los-mossos-atribuyen-al-crimen-organizado-los-ultimos-seis-muertos-a-tiros-en-cataluna.html</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="2" t="inlineStr"/>
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>13/06/2026 04:06 a. m.</t>
+        </is>
+      </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2923,22 +2935,26 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>Estados Unidos baja de la nube a Paraguay: inesperado resultado sacude el grupo D del Mundial 2026</t>
+          <t>Última hora de la guerra de Estados Unidos e Israel contra Irán, en directo | Israel emite una orden de evacuación para 20 localidades en el sur de Líbano y reanuda los bombardeos</t>
         </is>
       </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/estados-unidos-baja-de-la-nube-a-paraguay-inesperado-resultado-sacude-el-grupo-d-del-mundial-2026/202657/</t>
+          <t>https://elpais.com/internacional/2026-06-13/ultima-hora-de-la-guerra-de-estados-unidos-e-israel-contra-iran-en-directo.html</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="5" t="inlineStr"/>
+      <c r="A93" s="5" t="inlineStr">
+        <is>
+          <t>13/06/2026 03:54 a. m.</t>
+        </is>
+      </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2946,22 +2962,26 @@
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D93" s="6" t="inlineStr">
         <is>
-          <t>Iván Cepeda vivió un tenso momento en Bucaramanga: recibió abucheos de algunas personas en el aeropuerto</t>
+          <t>Mundial 2026, ultimas noticias en directo | EEUU vence a Paraguay y Brasil y Marruecos preparan el primer choque entre selecciones candidatas</t>
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/confidenciales/articulo/ivan-cepeda-vivio-un-tenso-momento-en-bucaramanga-recibio-abucheos-de-algunas-personas-en-el-aeropuerto/202617/</t>
+          <t>https://elpais.com/deportes/mundial-futbol/2026-06-13/resumen-y-ultimas-noticias-de-la-copa-mundial-de-futbol.html</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="2" t="inlineStr"/>
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>13/06/2026 02:28 a. m.</t>
+        </is>
+      </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2969,22 +2989,26 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>La inesperada propuesta del oponente de Keiko Fujimori en pleno conteo de votos</t>
+          <t>Sarral, el Huntington y la Copa del Mundo</t>
         </is>
       </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/mundo/articulo/la-inesperada-propuesta-del-oponente-de-keiko-fujimori-en-pleno-conteo-de-votos/202651/</t>
+          <t>https://elpais.com/espana/catalunya/2026-06-13/sarral-el-huntington-y-la-copa-del-mundo.html</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="5" t="inlineStr"/>
+      <c r="A95" s="5" t="inlineStr">
+        <is>
+          <t>13/06/2026 02:03 a. m.</t>
+        </is>
+      </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2992,22 +3016,26 @@
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D95" s="6" t="inlineStr">
         <is>
-          <t>🔴 Simulador del Mundial 2026 | Arme el fixture completo y defina a su campeón</t>
+          <t>Lotería Nacional: sorteo del sábado 13 de junio</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/especiales-multimedia/articulo/mundial-2026-el-simulador-con-el-que-usted-puede-jugar-y-atinar-hasta-que-haya-campeon/202529/</t>
+          <t>https://elpais.com/sorteos/2026-06-13/loteria-nacional-sorteo-del-sabado-13-de-junio.html</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="2" t="inlineStr"/>
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>13/06/2026 12:39 a. m.</t>
+        </is>
+      </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3015,22 +3043,26 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>La lluvia de estrellas más intensa del 2026 está cerca; científicos piden prepararnos para el espectáculo más imponente de toda una década</t>
+          <t>Un tiro en un pie: salir del CIADI le puede salir caro a Colombia</t>
         </is>
       </c>
       <c r="E96" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/tecnologia/articulo/la-lluvia-de-estrellas-mas-intensa-del-2026-esta-cerca-cientificos-piden-prepararnos-para-el-espectaculo-mas-imponente-de-toda-una-decada/202617/</t>
+          <t>https://elpais.com/america-colombia/2026-06-13/un-tiro-en-un-pie-salir-del-ciadi-le-puede-salir-caro-a-colombia.html</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="5" t="inlineStr"/>
+      <c r="A97" s="5" t="inlineStr">
+        <is>
+          <t>13/06/2026 12:08 a. m.</t>
+        </is>
+      </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3038,22 +3070,26 @@
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D97" s="6" t="inlineStr">
         <is>
-          <t>Armando Benedetti ya no piensa en el Gobierno Petro y se va con toda contra la Fifa</t>
+          <t>Niño Guerrero, de una barriada de Venezuela a conquistar América Latina con el Tren de Aragua</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/confidenciales/articulo/armando-benedetti-ya-no-piensa-en-el-gobierno-petro-y-se-va-con-toda-contra-la-fifa/202633/</t>
+          <t>https://elpais.com/america/2026-06-13/nino-guerrero-de-una-barriada-de-venezuela-a-conquistar-america-latina-con-el-tren-de-aragua.html</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="inlineStr"/>
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>13/06/2026 12:05 a. m.</t>
+        </is>
+      </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3061,22 +3097,26 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>¿Qué partidos del Mundial 2026 se juegan este 13 de junio? Fecha, horario y canal de TV</t>
+          <t>Trump alaba al Tigre y reta a la izquierda, mientras Cepeda acude a la CPI</t>
         </is>
       </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/que-partidos-del-mundial-2026-se-juegan-este-13-de-junio-fecha-horario-y-canal-de-tv/202654/</t>
+          <t>https://elpais.com/america-colombia/elecciones-presidenciales/2026-06-13/trump-alaba-al-tigre-y-reta-a-la-izquierda-mientras-cepeda-acude-a-la-cpi.html</t>
         </is>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="5" t="inlineStr"/>
+      <c r="A99" s="5" t="inlineStr">
+        <is>
+          <t>13/06/2026 12:01 a. m.</t>
+        </is>
+      </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3084,22 +3124,26 @@
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D99" s="6" t="inlineStr">
         <is>
-          <t>Apostar al Mundial 2026: el boom que mueve billones, tributa más y preocupa a los expertos</t>
+          <t>Los creyentes progresistas que le disputan el voto religioso a Abelardo de la Espriella</t>
         </is>
       </c>
       <c r="E99" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/mundo/articulo/apostar-al-mundial-2026-el-boom-que-mueve-billones-tributa-mas-y-preocupa-a-los-expertos/202600/</t>
+          <t>https://elpais.com/america-colombia/2026-06-13/los-creyentes-progresistas-que-le-disputan-el-voto-religioso-a-abelardo-de-la-espriella.html</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="inlineStr"/>
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>13/06/2026 12:00 a. m.</t>
+        </is>
+      </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3107,22 +3151,26 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>Cámara captó el dolor que sufre Dibu Martínez: hay dudas en Argentina cerca del debut mundialista</t>
+          <t>Vinicius, tras la estela de Garrincha en Brasil</t>
         </is>
       </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/camara-capto-el-dolor-que-sufre-dibu-martinez-hay-dudas-en-argentina-cerca-del-debut-mundialista/202658/</t>
+          <t>https://elpais.com/deportes/mundial-futbol/2026-06-13/vinicius-tras-la-estela-de-garrincha-en-brasil.html</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="5" t="inlineStr"/>
+      <c r="A101" s="5" t="inlineStr">
+        <is>
+          <t>13/06/2026 12:00 a. m.</t>
+        </is>
+      </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3130,22 +3178,26 @@
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D101" s="6" t="inlineStr">
         <is>
-          <t>De norte a sur: así se está pintado el mapa político de América Latina que gira hacia la derecha</t>
+          <t>Pickleball: por qué todo el mundo está jugando (y qué necesitas para empezar)</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/de-norte-a-sur-asi-se-esta-pintado-el-mapa-politico-de-america-latina-que-gira-hacia-la-derecha/202631/</t>
+          <t>https://elpais.com/hemeroteca/2026-06-13/</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="2" t="inlineStr"/>
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>12/06/2026 11:55 p. m.</t>
+        </is>
+      </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3153,22 +3205,26 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>“No entregue un solo peso”: campaña de Abelardo De La Espriella lanza alerta por presuntas estafas con su nombre</t>
+          <t>Abelardo de la Espriella matiza sus propuestas ‘milagro’</t>
         </is>
       </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/no-entregue-un-solo-peso-campana-de-abelardo-de-la-espriella-lanza-alerta-por-presuntas-estafas-con-su-nombre/202615/</t>
+          <t>https://elpais.com/america-colombia/elecciones-presidenciales/2026-06-13/abelardo-de-la-espriella-matiza-sus-propuestas-milagro.html</t>
         </is>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="5" t="inlineStr"/>
+      <c r="A103" s="5" t="inlineStr">
+        <is>
+          <t>12/06/2026 11:52 p. m.</t>
+        </is>
+      </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3176,22 +3232,26 @@
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D103" s="6" t="inlineStr">
         <is>
-          <t>¿Es viable un mundial en Colombia como lo propone Iván Cepeda? Esta es la realidad</t>
+          <t>Sin constituyente y sin paz total: Iván Cepeda publica un plan de gobierno más moderado</t>
         </is>
       </c>
       <c r="E103" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/es-viable-un-mundial-en-colombia-como-lo-propone-ivan-cepeda-esta-es-la-realidad/202611/</t>
+          <t>https://elpais.com/america-colombia/elecciones-presidenciales/2026-06-13/sin-constituyente-y-sin-paz-total-ivan-cepeda-publica-un-plan-de-gobierno-mas-moderado.html</t>
         </is>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="2" t="inlineStr"/>
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>12/06/2026 11:13 p. m.</t>
+        </is>
+      </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3199,22 +3259,26 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>Petro envió audio a pocos días de la segunda vuelta presidencial: “En su voto está la posibilidad de ampliar este legado”</t>
+          <t>Pilar Rueda, esposa de Iván Cepeda: “En esta elección está en juego la libertad de ser”</t>
         </is>
       </c>
       <c r="E104" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/petro-envio-audio-a-pocos-dias-de-la-segunda-vuelta-presidencial-en-su-voto-esta-la-posibilidad-de-ampliar-este-legado/202626/</t>
+          <t>https://elpais.com/america-colombia/elecciones-presidenciales/2026-06-13/pilar-rueda-esposa-de-ivan-cepeda-en-esta-eleccion-esta-en-juego-la-libertad-de-ser.html</t>
         </is>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="5" t="inlineStr"/>
+      <c r="A105" s="5" t="inlineStr">
+        <is>
+          <t>12/06/2026 11:00 p. m.</t>
+        </is>
+      </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3222,22 +3286,26 @@
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D105" s="6" t="inlineStr">
         <is>
-          <t>Las víctimas que a nadie le duelen: así viven miles de campesinos bajo el yugo de grupos armados en zonas rurales de Colombia</t>
+          <t>Los últimos días de Alligator Alcatraz, el símbolo de la ofensiva migratoria de Trump</t>
         </is>
       </c>
       <c r="E105" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/cali/articulo/las-victimas-que-a-nadie-le-duelen-asi-viven-miles-de-campesinos-bajo-el-yugo-de-grupos-armados-en-zonas-rurales-de-colombia/202601/</t>
+          <t>https://elpais.com/us/migracion/2026-06-13/los-ultimos-dias-de-alligator-alcatraz-el-simbolo-de-la-ofensiva-migratoria-de-trump.html</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="2" t="inlineStr"/>
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>12/06/2026 11:00 p. m.</t>
+        </is>
+      </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3245,22 +3313,26 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D106" s="3" t="inlineStr">
         <is>
-          <t>Cuerpos embolsados: así se ha reconfigurado el mapa criminal de Bogotá y Soacha el último año</t>
+          <t>Morena en ebullición: más de 50 cuadros apuntan a una gubernatura en 2027</t>
         </is>
       </c>
       <c r="E106" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/bogota/articulo/cuerpos-embolsados-asi-se-ha-reconfigurado-el-mapa-criminal-de-bogota-y-soacha-el-ultimo-ano/202644/</t>
+          <t>https://elpais.com/mexico/2026-06-13/morena-en-ebullicion-mas-de-50-cuadros-apuntan-a-una-gubernatura-en-2027.html</t>
         </is>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="5" t="inlineStr"/>
+      <c r="A107" s="5" t="inlineStr">
+        <is>
+          <t>12/06/2026 11:00 p. m.</t>
+        </is>
+      </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3268,22 +3340,26 @@
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D107" s="6" t="inlineStr">
         <is>
-          <t>Video | Persecución de película quedó grabada: Policía detuvo a una mujer señalada de robo</t>
+          <t>La batalla por las actas impugnadas aboca a Perú a un escenario de máxima incertidumbre</t>
         </is>
       </c>
       <c r="E107" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/medellin/articulo/video-persecucion-de-pelicula-quedo-grabada-policia-detuvo-a-una-mujer-senalada-de-robo/202610/</t>
+          <t>https://elpais.com/america/2026-06-13/la-batalla-por-las-actas-impugnadas-aboca-a-peru-a-un-escenario-de-maxima-incertidumbre.html</t>
         </is>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="inlineStr"/>
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>12/06/2026 11:00 p. m.</t>
+        </is>
+      </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3291,24 +3367,24 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D108" s="3" t="inlineStr">
         <is>
-          <t>¿Qué pasó con la Chapola? Investigan la muerte de reconocida líder trans hallada sin vida en un río de Antioquia</t>
+          <t>Raúl ‘Tala’ Rangel toma el relevo del emblema Guillermo Ochoa en la portería de México</t>
         </is>
       </c>
       <c r="E108" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/que-paso-con-la-chapola-investigan-la-muerte-de-reconocida-lider-trans-hallada-sin-vida-en-un-rio-de-antioquia/202627/</t>
+          <t>https://elpais.com/mexico/2026-06-13/raul-tala-rangel-toma-el-relevo-del-emblema-guillermo-ochoa-en-la-porteria-de-mexico.html</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 02:48 a. m.</t>
+          <t>12/06/2026 10:45 p. m.</t>
         </is>
       </c>
       <c r="B109" s="5" t="inlineStr">
@@ -3323,19 +3399,19 @@
       </c>
       <c r="D109" s="6" t="inlineStr">
         <is>
-          <t>Última hora de la guerra de Estados Unidos e Israel contra Irán, en directo | El ejército estadounidense asegura que Irán ha lanzado ataques con drones en el estrecho de Ormuz</t>
+          <t>¿Puedes batir nuestra predicción? Juega a pronosticar el Mundial</t>
         </is>
       </c>
       <c r="E109" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/internacional/2026-06-13/ultima-hora-de-la-guerra-de-estados-unidos-e-israel-contra-iran-en-directo.html</t>
+          <t>https://elpais.com/deportes/mundial-futbol/2026-06-13/puedes-batir-nuestra-prediccion-juega-a-pronosticar-el-mundial.html</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 02:44 a. m.</t>
+          <t>12/06/2026 10:30 p. m.</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
@@ -3350,19 +3426,19 @@
       </c>
       <c r="D110" s="3" t="inlineStr">
         <is>
-          <t>Mundial 2026, ultimas noticias en directo | EEUU vence a Paraguay y Brasil y Marruecos preparan el primer choque entre selecciones candidatas</t>
+          <t>Viviendas, sanidad y otros servicios: los suizos se preguntan hasta dónde pueden crecer</t>
         </is>
       </c>
       <c r="E110" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/deportes/mundial-futbol/2026-06-13/resumen-y-ultimas-noticias-de-la-copa-mundial-de-futbol.html</t>
+          <t>https://elpais.com/internacional/2026-06-13/viviendas-sanidad-y-otros-servicios-los-suizos-se-preguntan-hasta-donde-pueden-crecer.html</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 02:28 a. m.</t>
+          <t>12/06/2026 10:30 p. m.</t>
         </is>
       </c>
       <c r="B111" s="5" t="inlineStr">
@@ -3377,19 +3453,19 @@
       </c>
       <c r="D111" s="6" t="inlineStr">
         <is>
-          <t>Sarral, el Huntington y la Copa del Mundo</t>
+          <t>Los excursionistas que auxiliaron a Jonathan Andic, el quebradero de cabeza de los Mossos</t>
         </is>
       </c>
       <c r="E111" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/espana/catalunya/2026-06-13/sarral-el-huntington-y-la-copa-del-mundo.html</t>
+          <t>https://elpais.com/espana/catalunya/2026-06-13/los-excursionistas-que-auxiliaron-a-jonathan-andic-el-quebradero-de-cabeza-de-los-mossos.html</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 02:03 a. m.</t>
+          <t>12/06/2026 10:30 p. m.</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
@@ -3404,19 +3480,19 @@
       </c>
       <c r="D112" s="3" t="inlineStr">
         <is>
-          <t>Lotería Nacional: sorteo del sábado 13 de junio</t>
+          <t>La investigación a Zapatero por posible delito fiscal con las joyas limita cualquier regularización ante Hacienda</t>
         </is>
       </c>
       <c r="E112" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/sorteos/2026-06-13/loteria-nacional-sorteo-del-sabado-13-de-junio.html</t>
+          <t>https://elpais.com/economia/2026-06-13/la-investigacion-a-zapatero-por-posible-delito-fiscal-con-las-joyas-limita-cualquier-regularizacion-ante-hacienda.html</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 12:39 a. m.</t>
+          <t>12/06/2026 10:30 p. m.</t>
         </is>
       </c>
       <c r="B113" s="5" t="inlineStr">
@@ -3431,19 +3507,19 @@
       </c>
       <c r="D113" s="6" t="inlineStr">
         <is>
-          <t>Un tiro en un pie: salir del CIADI le puede salir caro a Colombia</t>
+          <t>¿Está quemando Telecinco ‘Supervivientes’ y ‘La isla de las tentaciones’? La respuesta de los datos de audiencia</t>
         </is>
       </c>
       <c r="E113" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/america-colombia/2026-06-13/un-tiro-en-un-pie-salir-del-ciadi-le-puede-salir-caro-a-colombia.html</t>
+          <t>https://elpais.com/television/2026-06-13/esta-quemando-telecinco-supervivientes-y-la-isla-de-las-tentaciones-la-respuesta-de-los-datos-de-audiencia.html</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 12:08 a. m.</t>
+          <t>12/06/2026 10:30 p. m.</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
@@ -3458,19 +3534,19 @@
       </c>
       <c r="D114" s="3" t="inlineStr">
         <is>
-          <t>Niño Guerrero, de una barriada de Venezuela a conquistar América Latina con el Tren de Aragua</t>
+          <t>Los primeros estudiantes del grado de Matemáticas y Filosofía, único en España: “Hay que aprender a utilizar la IA con ética”</t>
         </is>
       </c>
       <c r="E114" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/america/2026-06-13/nino-guerrero-de-una-barriada-de-venezuela-a-conquistar-america-latina-con-el-tren-de-aragua.html</t>
+          <t>https://elpais.com/educacion/2026-06-13/los-primeros-estudiantes-del-grado-de-matematicas-y-filosofia-unico-en-espana-hay-que-aprender-a-utilizar-la-ia-con-etica.html</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 12:05 a. m.</t>
+          <t>12/06/2026 10:30 p. m.</t>
         </is>
       </c>
       <c r="B115" s="5" t="inlineStr">
@@ -3485,19 +3561,19 @@
       </c>
       <c r="D115" s="6" t="inlineStr">
         <is>
-          <t>Trump alaba al Tigre y reta a la izquierda, mientras Cepeda acude a la CPI</t>
+          <t>El paso al frente de Marruecos con su nuevo seleccionador Mohamed Ouahbi</t>
         </is>
       </c>
       <c r="E115" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/america-colombia/elecciones-presidenciales/2026-06-13/trump-alaba-al-tigre-y-reta-a-la-izquierda-mientras-cepeda-acude-a-la-cpi.html</t>
+          <t>https://elpais.com/deportes/mundial-futbol/2026-06-13/el-paso-al-frente-de-marruecos-con-su-nuevo-seleccionador-mohamed-ouahbi.html</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 12:01 a. m.</t>
+          <t>12/06/2026 10:30 p. m.</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
@@ -3512,19 +3588,19 @@
       </c>
       <c r="D116" s="3" t="inlineStr">
         <is>
-          <t>Los creyentes progresistas que le disputan el voto religioso a Abelardo de la Espriella</t>
+          <t>El vértigo de viajar solo en verano: “Llevo demasiado tiempo viviendo como si mi vida estuviera en pausa”</t>
         </is>
       </c>
       <c r="E116" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/america-colombia/2026-06-13/los-creyentes-progresistas-que-le-disputan-el-voto-religioso-a-abelardo-de-la-espriella.html</t>
+          <t>https://elpais.com/estilo-de-vida/2026-06-13/el-vertigo-de-viajar-solo-en-verano-llevo-demasiado-tiempo-viviendo-como-si-mi-vida-estuviera-en-pausa.html</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 12:00 a. m.</t>
+          <t>12/06/2026 08:15 p. m.</t>
         </is>
       </c>
       <c r="B117" s="5" t="inlineStr">
@@ -3539,19 +3615,19 @@
       </c>
       <c r="D117" s="6" t="inlineStr">
         <is>
-          <t>Vinicius, tras la estela de Garrincha en Brasil</t>
+          <t>Trump anuncia que el ejército de Estados Unidos ha matado en Venezuela al Niño Guerrero, líder del Tren de Aragua</t>
         </is>
       </c>
       <c r="E117" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/deportes/mundial-futbol/2026-06-13/vinicius-tras-la-estela-de-garrincha-en-brasil.html</t>
+          <t>https://elpais.com/america/2026-06-13/trump-anuncia-que-el-ejercito-de-estados-unidos-ha-matado-al-nino-guerrero-lider-del-tren-de-aragua.html</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 12:00 a. m.</t>
+          <t>12/06/2026 02:45 a. m.</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
@@ -3566,21 +3642,17 @@
       </c>
       <c r="D118" s="3" t="inlineStr">
         <is>
-          <t>Pickleball: por qué todo el mundo está jugando (y qué necesitas para empezar)</t>
+          <t>Maxi Iglesias: “Intento seguir mi vida sin hacer mucho caso al ruido que generan mis decisiones”</t>
         </is>
       </c>
       <c r="E118" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/hemeroteca/2026-06-13/</t>
+          <t>https://elpais.com/icon/2026-06-12/maxi-iglesias-intento-seguir-mi-vida-sin-hacer-mucho-caso-al-ruido-que-generan-mis-decisiones.html</t>
         </is>
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="5" t="inlineStr">
-        <is>
-          <t>12/06/2026 11:55 p. m.</t>
-        </is>
-      </c>
+      <c r="A119" s="5" t="inlineStr"/>
       <c r="B119" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3593,21 +3665,17 @@
       </c>
       <c r="D119" s="6" t="inlineStr">
         <is>
-          <t>Abelardo de la Espriella matiza sus propuestas ‘milagro’</t>
+          <t>Predicciones</t>
         </is>
       </c>
       <c r="E119" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/america-colombia/elecciones-presidenciales/2026-06-13/abelardo-de-la-espriella-matiza-sus-propuestas-milagro.html</t>
+          <t>https://elpais.com/deportes/mundial-futbol/2026-06-11/quien-ganara-el-mundial-asi-arrancan-nuestras-predicciones.html</t>
         </is>
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="2" t="inlineStr">
-        <is>
-          <t>12/06/2026 11:52 p. m.</t>
-        </is>
-      </c>
+      <c r="A120" s="2" t="inlineStr"/>
       <c r="B120" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3620,19 +3688,19 @@
       </c>
       <c r="D120" s="3" t="inlineStr">
         <is>
-          <t>Sin constituyente y sin paz total: Iván Cepeda publica un plan de gobierno más moderado</t>
+          <t>Selecciones</t>
         </is>
       </c>
       <c r="E120" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/america-colombia/elecciones-presidenciales/2026-06-13/sin-constituyente-y-sin-paz-total-ivan-cepeda-publica-un-plan-de-gobierno-mas-moderado.html</t>
+          <t>https://elpais.com/deportes/mundial-futbol/2026-06-05/todas-las-selecciones-del-mundial-de-estados-unidos-canada-y-mexico.html</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 11:13 p. m.</t>
+          <t>13/06/2026 03:39 a. m.</t>
         </is>
       </c>
       <c r="B121" s="5" t="inlineStr">
@@ -3642,24 +3710,24 @@
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D121" s="6" t="inlineStr">
         <is>
-          <t>Pilar Rueda, esposa de Iván Cepeda: “En esta elección está en juego la libertad de ser”</t>
+          <t>Horas de infarto en la Comisión de Acusación. Tras la suspensión de Gloria Arizabaleta, así se le despejará el camino a Petro en sus investigaciones</t>
         </is>
       </c>
       <c r="E121" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/america-colombia/elecciones-presidenciales/2026-06-13/pilar-rueda-esposa-de-ivan-cepeda-en-esta-eleccion-esta-en-juego-la-libertad-de-ser.html</t>
+          <t>https://www.semana.com/politica/articulo/horas-de-infarto-en-la-comision-de-acusacion-tras-la-suspension-de-gloria-arizabaleta-asi-se-le-despejara-el-camino-a-petro-en-sus-investigaciones/202616/</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 11:00 p. m.</t>
+          <t>13/06/2026 03:39 a. m.</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
@@ -3669,24 +3737,24 @@
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D122" s="3" t="inlineStr">
         <is>
-          <t>Manuel Adorni, un mapa de miserias</t>
+          <t>¿Doble rasero? Mientras se retiró a un general sin investigaciones, otros con procesos de falsos positivos, concierto para delinquir y peculado son protegidos</t>
         </is>
       </c>
       <c r="E122" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/argentina/2026-06-13/manuel-adorni-un-mapa-de-miserias.html</t>
+          <t>https://www.semana.com/nacion/articulo/doble-rasero-mientras-se-retiro-a-un-general-sin-investigaciones-otros-con-procesos-de-falsos-positivos-concierto-para-delinquir-y-peculado-son-protegidos/202629/</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 11:00 p. m.</t>
+          <t>13/06/2026 03:39 a. m.</t>
         </is>
       </c>
       <c r="B123" s="5" t="inlineStr">
@@ -3696,24 +3764,24 @@
       </c>
       <c r="C123" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D123" s="6" t="inlineStr">
         <is>
-          <t>La muerte de Julio Jung rescata la historia de cuando Superman vino a Chile a desafiar la dictadura de Pinochet</t>
+          <t>Magnicidio de Miguel Uribe Turbay: duros reparos a la Fiscalía por errores en la investigación. No logró demostrar que Iván Márquez es prófugo de la justicia</t>
         </is>
       </c>
       <c r="E123" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/chile/2026-06-13/la-muerte-de-julio-jung-rescata-la-historia-de-cuando-superman-vino-a-chile-a-desafiar-la-dictadura-de-pinochet.html</t>
+          <t>https://www.semana.com/nacion/articulo/magnicidio-de-miguel-uribe-turbay-duros-reparos-a-la-fiscalia-por-errores-en-la-investigacion-no-logro-demostrar-que-ivan-marquez-es-profugo-de-la-justicia/202601/</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 11:00 p. m.</t>
+          <t>13/06/2026 03:39 a. m.</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
@@ -3723,24 +3791,24 @@
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D124" s="3" t="inlineStr">
         <is>
-          <t>Cuba ensaya al borde del abismo su enésima apertura económica</t>
+          <t>Agustín Laje habló con SEMANA y rechazó la campaña del petrismo sobre Argentina y el supuesto fracaso de Milei. “No compren esa propaganda”</t>
         </is>
       </c>
       <c r="E124" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/us/2026-06-13/cuba-ensaya-al-borde-del-abismo-su-enesima-apertura-economica.html</t>
+          <t>https://www.semana.com/mundo/articulo/agustin-laje-hablo-con-semana-y-rechazo-la-campana-del-petrismo-sobre-argentina-y-el-supuesto-fracaso-de-milei-no-compren-esa-propaganda/202619/</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 11:00 p. m.</t>
+          <t>13/06/2026 03:39 a. m.</t>
         </is>
       </c>
       <c r="B125" s="5" t="inlineStr">
@@ -3750,24 +3818,24 @@
       </c>
       <c r="C125" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D125" s="6" t="inlineStr">
         <is>
-          <t>Morena en ebullición: más de 50 cuadros apuntan a una gubernatura en 2027</t>
+          <t>Selección Colombia: SEMANA conversó con los familiares de los convocados al Mundial 2026. Historias de sacrificio, temple y mucho amor</t>
         </is>
       </c>
       <c r="E125" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/mexico/2026-06-13/morena-en-ebullicion-mas-de-50-cuadros-apuntan-a-una-gubernatura-en-2027.html</t>
+          <t>https://www.semana.com/deportes/articulo/seleccion-colombia-semana-converso-con-los-familiares-de-los-convocados-al-mundial-2026-historias-de-sacrificio-temple-y-mucho-amor/202621/</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 11:00 p. m.</t>
+          <t>13/06/2026 03:39 a. m.</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
@@ -3777,24 +3845,24 @@
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D126" s="3" t="inlineStr">
         <is>
-          <t>Los últimos días de Alligator Alcatraz, el símbolo de la ofensiva migratoria de Trump</t>
+          <t>Max Henriquez lanza alerta por fenómeno del superniño en Colombia: “Es posible que haya racionamiento de agua y energía”</t>
         </is>
       </c>
       <c r="E126" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/us/migracion/2026-06-13/los-ultimos-dias-de-alligator-alcatraz-el-simbolo-de-la-ofensiva-migratoria-de-trump.html</t>
+          <t>https://www.semana.com/nacion/articulo/max-henriquez-lanza-alerta-por-fenomeno-del-supernino-en-colombia-es-posible-que-haya-racionamiento-de-agua-y-energia/202629/</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 10:45 p. m.</t>
+          <t>13/06/2026 03:39 a. m.</t>
         </is>
       </c>
       <c r="B127" s="5" t="inlineStr">
@@ -3804,24 +3872,24 @@
       </c>
       <c r="C127" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D127" s="6" t="inlineStr">
         <is>
-          <t>¿Puedes batir nuestra predicción? Juega a pronosticar el Mundial</t>
+          <t>Piden a Estados Unidos que investigue e incluya en la Lista Clinton a Ricardo Roa, presidente de Ecopetrol, por transacciones en la campaña de Petro</t>
         </is>
       </c>
       <c r="E127" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/deportes/mundial-futbol/2026-06-13/puedes-batir-nuestra-prediccion-juega-a-pronosticar-el-mundial.html</t>
+          <t>https://www.semana.com/nacion/articulo/piden-a-estados-unidos-que-investigue-e-incluya-en-la-lista-clinton-a-ricardo-roa-presidente-de-ecopetrol-por-transacciones-en-la-campana-de-petro/202620/</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 10:30 p. m.</t>
+          <t>13/06/2026 03:39 a. m.</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
@@ -3831,24 +3899,24 @@
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D128" s="3" t="inlineStr">
         <is>
-          <t>La investigación a Zapatero por posible delito fiscal con las joyas limita cualquier regularización ante Hacienda</t>
+          <t>Estos son los políticos cuestionados que apoyan la candidatura de Iván Cepeda: son señalados por presunta corrupción</t>
         </is>
       </c>
       <c r="E128" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/economia/2026-06-13/la-investigacion-a-zapatero-por-posible-delito-fiscal-con-las-joyas-limita-cualquier-regularizacion-ante-hacienda.html</t>
+          <t>https://www.semana.com/politica/articulo/estos-son-los-politicos-cuestionados-que-apoyan-la-candidatura-de-ivan-cepeda-son-senalados-por-presunta-corrupcion/202608/</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 10:30 p. m.</t>
+          <t>13/06/2026 03:39 a. m.</t>
         </is>
       </c>
       <c r="B129" s="5" t="inlineStr">
@@ -3858,24 +3926,24 @@
       </c>
       <c r="C129" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D129" s="6" t="inlineStr">
         <is>
-          <t>Los excursionistas que auxiliaron a Jonathan Andic, el quebradero de cabeza de los Mossos</t>
+          <t>Mauricio Vargas dice que Abelardo de la Espriella ganará la presidencia y que “Iván Cepeda y Gustavo Petro competirán por la oposición”</t>
         </is>
       </c>
       <c r="E129" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/espana/catalunya/2026-06-13/los-excursionistas-que-auxiliaron-a-jonathan-andic-el-quebradero-de-cabeza-de-los-mossos.html</t>
+          <t>https://www.semana.com/politica/articulo/mauricio-vargas-dice-que-abelardo-de-la-espriella-ganara-la-presidencia-y-que-ivan-cepeda-y-gustavo-petro-competiran-por-la-oposicion/202627/</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 10:30 p. m.</t>
+          <t>13/06/2026 03:39 a. m.</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
@@ -3885,24 +3953,24 @@
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D130" s="3" t="inlineStr">
         <is>
-          <t>¿Está quemando Telecinco ‘Supervivientes’ y ‘La isla de las tentaciones’? La respuesta de los datos de audiencia</t>
+          <t>Añorado regreso de la Selección Colombia: ocho años deseándolo y así llega a la gran cita de la Copa del Mundo</t>
         </is>
       </c>
       <c r="E130" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/television/2026-06-13/esta-quemando-telecinco-supervivientes-y-la-isla-de-las-tentaciones-la-respuesta-de-los-datos-de-audiencia.html</t>
+          <t>https://www.semana.com/deportes/articulo/anorado-regreso-de-la-seleccion-colombia-ocho-anos-deseandolo-y-asi-llega-a-la-gran-cita-de-la-copa-del-mundo/202656/</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 10:30 p. m.</t>
+          <t>13/06/2026 03:39 a. m.</t>
         </is>
       </c>
       <c r="B131" s="5" t="inlineStr">
@@ -3912,24 +3980,24 @@
       </c>
       <c r="C131" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D131" s="6" t="inlineStr">
         <is>
-          <t>Los primeros estudiantes del grado de Matemáticas y Filosofía, único en España: “Hay que aprender a utilizar la IA con ética”</t>
+          <t>SEMANA revela detalles de la investigación del asesinato del periodista Cristian Herrera en Cúcuta: cámaras de seguridad, una oficina de sicarios y la orden de un cabecilla desde la cárcel</t>
         </is>
       </c>
       <c r="E131" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/educacion/2026-06-13/los-primeros-estudiantes-del-grado-de-matematicas-y-filosofia-unico-en-espana-hay-que-aprender-a-utilizar-la-ia-con-etica.html</t>
+          <t>https://www.semana.com/nacion/articulo/semana-revela-detalles-de-la-investigacion-del-asesinato-del-periodista-cristian-herrera-en-cucuta-camaras-de-seguridad-una-oficina-de-sicarios-y-la-orden-de-un-cabecilla-desde-la-carcel/202625/</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 10:30 p. m.</t>
+          <t>13/06/2026 03:39 a. m.</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
@@ -3939,24 +4007,24 @@
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D132" s="3" t="inlineStr">
         <is>
-          <t>El paso al frente de Marruecos con su nuevo seleccionador Mohamed Ouahbi</t>
+          <t>¿Qué puede hacer Donald Trump en las elecciones en Colombia? ¿Puede quitar visas? El exembajador Kevin Whitaker lo explica</t>
         </is>
       </c>
       <c r="E132" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/deportes/mundial-futbol/2026-06-13/el-paso-al-frente-de-marruecos-con-su-nuevo-seleccionador-mohamed-ouahbi.html</t>
+          <t>https://www.semana.com/politica/articulo/que-puede-hacer-donald-trump-en-las-elecciones-en-colombia-puede-quitar-visas-el-exembajador-kevin-whitaker-lo-explica/202616/</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 10:30 p. m.</t>
+          <t>13/06/2026 03:39 a. m.</t>
         </is>
       </c>
       <c r="B133" s="5" t="inlineStr">
@@ -3966,24 +4034,24 @@
       </c>
       <c r="C133" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D133" s="6" t="inlineStr">
         <is>
-          <t>El vértigo de viajar solo en verano: “Llevo demasiado tiempo viviendo como si mi vida estuviera en pausa”</t>
+          <t>Salud Hernández-Mora recorrió el Guaviare y comprobó cómo alias Calarcá será un desafío para el próximo presidente</t>
         </is>
       </c>
       <c r="E133" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/estilo-de-vida/2026-06-13/el-vertigo-de-viajar-solo-en-verano-llevo-demasiado-tiempo-viviendo-como-si-mi-vida-estuviera-en-pausa.html</t>
+          <t>https://www.semana.com/nacion/articulo/salud-hernandez-mora-recorrio-el-guaviare-y-comprobo-como-alias-calarca-sera-un-desafio-para-el-proximo-presidente/202620/</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 08:15 p. m.</t>
+          <t>13/06/2026 02:39 a. m.</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
@@ -3993,24 +4061,24 @@
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D134" s="3" t="inlineStr">
         <is>
-          <t>Trump anuncia que el ejército de Estados Unidos ha matado en Venezuela al Niño Guerrero, líder del Tren de Aragua</t>
+          <t>Habla Sofía Otero, la doctora de la mafia</t>
         </is>
       </c>
       <c r="E134" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/america/2026-06-13/trump-anuncia-que-el-ejercito-de-estados-unidos-ha-matado-al-nino-guerrero-lider-del-tren-de-aragua.html</t>
+          <t>https://www.semana.com/nacion/articulo/habla-sofia-otero-la-doctora-de-la-mafia/202636/</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 11:04 a. m.</t>
+          <t>13/06/2026 02:39 a. m.</t>
         </is>
       </c>
       <c r="B135" s="5" t="inlineStr">
@@ -4020,24 +4088,24 @@
       </c>
       <c r="C135" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D135" s="6" t="inlineStr">
         <is>
-          <t>Los canarios valoran al Papa, pero la migración es otro cantar: “El problema está en África, no aquí”</t>
+          <t>¿Abelardo de la Espriella, presidente? El Tigre derrotaría a Iván Cepeda en la segunda vuelta, según la más reciente encuesta de AtlasIntel</t>
         </is>
       </c>
       <c r="E135" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/espana/2026-06-12/los-canarios-valoran-al-papa-pero-la-migracion-es-otro-cantar-el-problema-esta-en-africa-no-aqui.html</t>
+          <t>https://www.semana.com/politica/articulo/abelardo-de-la-espriella-presidente-el-tigre-derrotaria-a-ivan-cepeda-en-la-segunda-vuelta-segun-la-mas-reciente-encuesta-de-atlasintel/202644/</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 02:45 a. m.</t>
+          <t>13/06/2026 01:39 a. m.</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
@@ -4047,22 +4115,26 @@
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D136" s="3" t="inlineStr">
         <is>
-          <t>Maxi Iglesias: “Intento seguir mi vida sin hacer mucho caso al ruido que generan mis decisiones”</t>
+          <t>Toy Story 5: Kenna Harris y Lindsey Collins hablan con SEMANA sobre el futuro de Woody, Buzz y Jessie</t>
         </is>
       </c>
       <c r="E136" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/icon/2026-06-12/maxi-iglesias-intento-seguir-mi-vida-sin-hacer-mucho-caso-al-ruido-que-generan-mis-decisiones.html</t>
+          <t>https://www.semana.com/cultura/cine/articulo/toy-story-5-kenna-harris-y-lindsey-collins-hablan-con-semana-sobre-el-futuro-de-woody-buzz-y-jessie/202643/</t>
         </is>
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="5" t="inlineStr"/>
+      <c r="A137" s="5" t="inlineStr">
+        <is>
+          <t>13/06/2026 01:39 a. m.</t>
+        </is>
+      </c>
       <c r="B137" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4070,22 +4142,26 @@
       </c>
       <c r="C137" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D137" s="6" t="inlineStr">
         <is>
-          <t>Predicciones</t>
+          <t>El mercado ya apostó por un cambio de Gobierno: Acciones al alza y dólar a la baja</t>
         </is>
       </c>
       <c r="E137" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/deportes/mundial-futbol/2026-06-11/quien-ganara-el-mundial-asi-arrancan-nuestras-predicciones.html</t>
+          <t>https://www.semana.com/economia/macroeconomia/articulo/el-mercado-ya-aposto-por-un-cambio-de-gobierno-acciones-al-alza-y-dolar-a-la-baja/202638/</t>
         </is>
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="2" t="inlineStr"/>
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>13/06/2026 01:39 a. m.</t>
+        </is>
+      </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4093,26 +4169,22 @@
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D138" s="3" t="inlineStr">
         <is>
-          <t>Selecciones</t>
+          <t>Clara Elvira Ospina, periodista colombiana en Perú, habla en SEMANA y anticipa triunfo de Keiko Fujimori tras largas elecciones</t>
         </is>
       </c>
       <c r="E138" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/deportes/mundial-futbol/2026-06-05/todas-las-selecciones-del-mundial-de-estados-unidos-canada-y-mexico.html</t>
+          <t>https://www.semana.com/mundo/articulo/clara-elvira-ospina-periodista-colombiana-en-peru-habla-en-semana-y-anticipa-triunfo-de-keiko-fujimori-tras-largas-elecciones/202652/</t>
         </is>
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="5" t="inlineStr">
-        <is>
-          <t>13/06/2026 12:44 a. m.</t>
-        </is>
-      </c>
+      <c r="A139" s="5" t="inlineStr"/>
       <c r="B139" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4120,26 +4192,22 @@
       </c>
       <c r="C139" s="5" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D139" s="6" t="inlineStr">
         <is>
-          <t>Resultados de loterías de Medellín, Santander, Risaralda y MiLoto hoy 12 de junio de 2026</t>
+          <t>Dian insiste en que hay que introducir más impuestos mientras la evasión sigue en niveles críticos</t>
         </is>
       </c>
       <c r="E139" s="7" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/economia/juegos-de-azar/resultados-de-loterias-de-medellin-santander-risaralda-y-miloto-hoy-12-de-junio-de-2026-so35</t>
+          <t>https://www.semana.com/economia/articulo/dian-insiste-en-que-hay-que-introducir-mas-impuestos-mientras-la-evasion-sigue-en-niveles-criticos/202600/</t>
         </is>
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="2" t="inlineStr">
-        <is>
-          <t>12/06/2026 11:56 p. m.</t>
-        </is>
-      </c>
+      <c r="A140" s="2" t="inlineStr"/>
       <c r="B140" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4147,26 +4215,22 @@
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D140" s="3" t="inlineStr">
         <is>
-          <t>Impactante choque: policía resulta herido en persecución tras chocar de frente contra un vehículo</t>
+          <t>¿Qué partidos del Mundial 2026 se juegan este 13 de junio? Fecha, horario y canal de TV</t>
         </is>
       </c>
       <c r="E140" s="4" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/mundo/impactante-choque-policia-resulta-herido-en-persecucion-tras-chocar-de-frente-contra-un-vehiculo-so35</t>
+          <t>https://www.semana.com/deportes/articulo/que-partidos-del-mundial-2026-se-juegan-este-13-de-junio-fecha-horario-y-canal-de-tv/202654/</t>
         </is>
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="5" t="inlineStr">
-        <is>
-          <t>12/06/2026 10:46 p. m.</t>
-        </is>
-      </c>
+      <c r="A141" s="5" t="inlineStr"/>
       <c r="B141" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4174,26 +4238,22 @@
       </c>
       <c r="C141" s="5" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D141" s="6" t="inlineStr">
         <is>
-          <t>Dos militares ecuatorianos heridos en enfrentamiento con civiles armados en frontera con Colombia</t>
+          <t>Apostar al Mundial 2026: el boom que mueve billones, tributa más y preocupa a los expertos</t>
         </is>
       </c>
       <c r="E141" s="7" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/mundo/dos-militares-ecuatorianos-heridos-en-enfrentamiento-con-civiles-armados-en-frontera-con-colombia-so35</t>
+          <t>https://www.semana.com/mundo/articulo/apostar-al-mundial-2026-el-boom-que-mueve-billones-tributa-mas-y-preocupa-a-los-expertos/202600/</t>
         </is>
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="2" t="inlineStr">
-        <is>
-          <t>12/06/2026 09:52 p. m.</t>
-        </is>
-      </c>
+      <c r="A142" s="2" t="inlineStr"/>
       <c r="B142" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4201,26 +4261,22 @@
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D142" s="3" t="inlineStr">
         <is>
-          <t>Resultados de MiLoto del 12 de junio de 2026: números ganadores y nuevo acumulado</t>
+          <t>Cámara captó el dolor que sufre Dibu Martínez: hay dudas en Argentina cerca del debut mundialista</t>
         </is>
       </c>
       <c r="E142" s="4" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/economia/juegos-de-azar/resultados-de-miloto-del-12-de-junio-de-2026-numeros-ganadores-y-nuevo-acumulado-so35</t>
+          <t>https://www.semana.com/deportes/articulo/camara-capto-el-dolor-que-sufre-dibu-martinez-hay-dudas-en-argentina-cerca-del-debut-mundialista/202658/</t>
         </is>
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="5" t="inlineStr">
-        <is>
-          <t>12/06/2026 09:40 p. m.</t>
-        </is>
-      </c>
+      <c r="A143" s="5" t="inlineStr"/>
       <c r="B143" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4228,26 +4284,22 @@
       </c>
       <c r="C143" s="5" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D143" s="6" t="inlineStr">
         <is>
-          <t>Resultados Lotería de Risaralda 12 de junio de 2026: premio mayor y números ganadores de secos</t>
+          <t>Iván Cepeda vivió un tenso momento en Bucaramanga: recibió abucheos de algunas personas en el aeropuerto</t>
         </is>
       </c>
       <c r="E143" s="7" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/economia/juegos-de-azar/resultados-loteria-de-risaralda-12-de-junio-de-2026-premio-mayor-y-numeros-ganadores-de-secos-so35</t>
+          <t>https://www.semana.com/confidenciales/articulo/ivan-cepeda-vivio-un-tenso-momento-en-bucaramanga-recibio-abucheos-de-algunas-personas-en-el-aeropuerto/202617/</t>
         </is>
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="2" t="inlineStr">
-        <is>
-          <t>12/06/2026 09:34 p. m.</t>
-        </is>
-      </c>
+      <c r="A144" s="2" t="inlineStr"/>
       <c r="B144" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4255,26 +4307,22 @@
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D144" s="3" t="inlineStr">
         <is>
-          <t>Lotería de Santander 12 de junio, premio mayor y secos, resultados último sorteo</t>
+          <t>De norte a sur: así se está pintado el mapa político de América Latina que gira hacia la derecha</t>
         </is>
       </c>
       <c r="E144" s="4" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/economia/juegos-de-azar/loteria-de-santander-12-de-junio-premio-mayor-y-secos-resultados-ultimo-sorteo-so35</t>
+          <t>https://www.semana.com/politica/articulo/de-norte-a-sur-asi-se-esta-pintado-el-mapa-politico-de-america-latina-que-gira-hacia-la-derecha/202631/</t>
         </is>
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="5" t="inlineStr">
-        <is>
-          <t>12/06/2026 09:13 p. m.</t>
-        </is>
-      </c>
+      <c r="A145" s="5" t="inlineStr"/>
       <c r="B145" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4282,26 +4330,22 @@
       </c>
       <c r="C145" s="5" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D145" s="6" t="inlineStr">
         <is>
-          <t>¿Quién era el 'Niño Guerrero', el temido líder del  Tren de Aragua abatido por Estados Unidos?</t>
+          <t>“No entregue un solo peso”: campaña de Abelardo De La Espriella lanza alerta por presuntas estafas con su nombre</t>
         </is>
       </c>
       <c r="E145" s="7" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/venezuela/quien-era-nino-guerrero-el-temido-lider-del-tren-de-aragua-abatido-por-estados-unidos-so35</t>
+          <t>https://www.semana.com/politica/articulo/no-entregue-un-solo-peso-campana-de-abelardo-de-la-espriella-lanza-alerta-por-presuntas-estafas-con-su-nombre/202615/</t>
         </is>
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="2" t="inlineStr">
-        <is>
-          <t>12/06/2026 09:10 p. m.</t>
-        </is>
-      </c>
+      <c r="A146" s="2" t="inlineStr"/>
       <c r="B146" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4309,26 +4353,22 @@
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D146" s="3" t="inlineStr">
         <is>
-          <t>Resultado Lotería de Medellín 12 de junio, premio mayor y secos del último sorteo</t>
+          <t>¿Es viable un mundial en Colombia como lo propone Iván Cepeda? Esta es la realidad</t>
         </is>
       </c>
       <c r="E146" s="4" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/economia/juegos-de-azar/resultado-loteria-de-medellin-12-de-junio-premio-mayor-y-secos-del-ultimo-sorteo-so35</t>
+          <t>https://www.semana.com/politica/articulo/es-viable-un-mundial-en-colombia-como-lo-propone-ivan-cepeda-esta-es-la-realidad/202611/</t>
         </is>
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="5" t="inlineStr">
-        <is>
-          <t>12/06/2026 08:37 p. m.</t>
-        </is>
-      </c>
+      <c r="A147" s="5" t="inlineStr"/>
       <c r="B147" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4336,26 +4376,22 @@
       </c>
       <c r="C147" s="5" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D147" s="6" t="inlineStr">
         <is>
-          <t>Trump anuncia la muerte del 'Niño Guerrero', el líder de banda venezolana Tren de Aragua</t>
+          <t>Las víctimas que a nadie le duelen: así viven miles de campesinos bajo el yugo de grupos armados en zonas rurales de Colombia</t>
         </is>
       </c>
       <c r="E147" s="7" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/mundo/trump-anuncia-la-muerte-del-nino-guerrero-el-lider-de-banda-venezolana-tren-de-aragua-cb20</t>
+          <t>https://www.semana.com/nacion/cali/articulo/las-victimas-que-a-nadie-le-duelen-asi-viven-miles-de-campesinos-bajo-el-yugo-de-grupos-armados-en-zonas-rurales-de-colombia/202601/</t>
         </is>
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="2" t="inlineStr">
-        <is>
-          <t>12/06/2026 08:18 p. m.</t>
-        </is>
-      </c>
+      <c r="A148" s="2" t="inlineStr"/>
       <c r="B148" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4363,26 +4399,22 @@
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D148" s="3" t="inlineStr">
         <is>
-          <t>"El gobierno reconoce el estado calamitoso en que entrega las finanzas": ANDI sobre nueva tributaria</t>
+          <t>Cuerpos embolsados: así se ha reconfigurado el mapa criminal de Bogotá y Soacha el último año</t>
         </is>
       </c>
       <c r="E148" s="4" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/economia/el-gobierno-reconoce-el-estado-calamitoso-en-que-entrega-las-finanzas-andi-sobre-nueva-tributaria-so35</t>
+          <t>https://www.semana.com/nacion/bogota/articulo/cuerpos-embolsados-asi-se-ha-reconfigurado-el-mapa-criminal-de-bogota-y-soacha-el-ultimo-ano/202644/</t>
         </is>
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="5" t="inlineStr">
-        <is>
-          <t>12/06/2026 08:11 p. m.</t>
-        </is>
-      </c>
+      <c r="A149" s="5" t="inlineStr"/>
       <c r="B149" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4390,26 +4422,22 @@
       </c>
       <c r="C149" s="5" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D149" s="6" t="inlineStr">
         <is>
-          <t>Astro Luna, resultado del último sorteo hoy viernes 12  de junio de 2026</t>
+          <t>Video | Persecución de película quedó grabada: Policía detuvo a una mujer señalada de robo</t>
         </is>
       </c>
       <c r="E149" s="7" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/economia/juegos-de-azar/astro-luna-resultado-del-ultimo-sorteo-hoy-viernes-12-de-junio-de-2026-so35</t>
+          <t>https://www.semana.com/nacion/medellin/articulo/video-persecucion-de-pelicula-quedo-grabada-policia-detuvo-a-una-mujer-senalada-de-robo/202610/</t>
         </is>
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="2" t="inlineStr">
-        <is>
-          <t>12/06/2026 08:11 p. m.</t>
-        </is>
-      </c>
+      <c r="A150" s="2" t="inlineStr"/>
       <c r="B150" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4417,17 +4445,17 @@
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D150" s="3" t="inlineStr">
         <is>
-          <t>Caribeña Noche, resultado del último sorteo hoy viernes 12 de junio de 2026</t>
+          <t>¿Qué pasó con la Chapola? Investigan la muerte de reconocida líder trans hallada sin vida en un río de Antioquia</t>
         </is>
       </c>
       <c r="E150" s="4" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/economia/juegos-de-azar/caribena-noche-resultado-del-ultimo-sorteo-hoy-viernes-12-de-junio-de-2026-so35</t>
+          <t>https://www.semana.com/nacion/articulo/que-paso-con-la-chapola-investigan-la-muerte-de-reconocida-lider-trans-hallada-sin-vida-en-un-rio-de-antioquia/202627/</t>
         </is>
       </c>
     </row>
@@ -4675,11 +4703,7 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="2" t="inlineStr">
-        <is>
-          <t>12/06/2026 10:37 p. m.</t>
-        </is>
-      </c>
+      <c r="A160" s="2" t="inlineStr"/>
       <c r="B160" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -4704,7 +4728,7 @@
     <row r="161">
       <c r="A161" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 12:10 a. m.</t>
+          <t>13/06/2026 12:39 a. m.</t>
         </is>
       </c>
       <c r="B161" s="5" t="inlineStr">
@@ -4731,7 +4755,7 @@
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 12:10 a. m.</t>
+          <t>13/06/2026 12:39 a. m.</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
@@ -6092,12 +6116,12 @@
       </c>
       <c r="D216" s="3" t="inlineStr">
         <is>
-          <t>Resultado Sinuano Noche hoy 12 de junio</t>
+          <t>Ideam advierte que Colombia enfrentaría el fenómeno de El Niño más fuerte desde 1950 y que su pico llegaría a fin de año</t>
         </is>
       </c>
       <c r="E216" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/resultado-sinuano-noche-hoy-12-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/ideam-advierte-que-colombia-enfrentaria-el-fenomeno-de-el-nino-mas-fuerte-desde-1950-y-que-su-pico-llegaria-a-fin-de-ano/</t>
         </is>
       </c>
     </row>
@@ -6119,12 +6143,12 @@
       </c>
       <c r="D217" s="6" t="inlineStr">
         <is>
-          <t>Mindefensa alerta por posibles disturbios tras la segunda vuelta y anticipa medidas por información de inteligencia</t>
+          <t>Clima: las temperaturas que predominarán este 13 de junio en Barranquilla</t>
         </is>
       </c>
       <c r="E217" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/mindefensa-alerta-por-posibles-disturbios-tras-la-segunda-vuelta-y-anticipa-medidas-por-informacion-de-inteligencia/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/clima-las-temperaturas-que-predominaran-este-13-de-junio-en-barranquilla/</t>
         </is>
       </c>
     </row>
@@ -6146,12 +6170,12 @@
       </c>
       <c r="D218" s="3" t="inlineStr">
         <is>
-          <t>JEP ha identificado plenamente a 1.956 víctimas de falsos positivos y aún busca establecer quiénes son otras 418</t>
+          <t>Clima: las temperaturas que predominarán este 13 de junio en Bogotá</t>
         </is>
       </c>
       <c r="E218" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/jep-ha-identificado-plenamente-a-1956-victimas-de-falsos-positivos-y-aun-busca-establecer-quienes-son-otras-418/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/clima-las-temperaturas-que-predominaran-este-13-de-junio-en-bogota/</t>
         </is>
       </c>
     </row>
@@ -6173,12 +6197,12 @@
       </c>
       <c r="D219" s="6" t="inlineStr">
         <is>
-          <t>“Costó 30.000 pesos y hoy estoy pagando con todo este dolor”: influencer denuncia procedimiento estético que casi le cuesta la vida</t>
+          <t>¿Cuál es la temperatura promedio en Medellín?</t>
         </is>
       </c>
       <c r="E219" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/costo-30000-pesos-y-hoy-estoy-pagando-con-todo-este-dolor-influencer-denuncia-procedimiento-estetico-que-casi-le-cuesta-la-vida/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/cual-es-la-temperatura-promedio-en-medellin/</t>
         </is>
       </c>
     </row>
@@ -6200,12 +6224,12 @@
       </c>
       <c r="D220" s="3" t="inlineStr">
         <is>
-          <t>Resultados Lotería de Santander hoy 13 de junio: revise su billete y cobre el premio mayor</t>
+          <t>Clima hoy en Colombia: temperaturas para Cali este 13 de junio</t>
         </is>
       </c>
       <c r="E220" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/resultados-loteria-de-santander-hoy-13-de-junio-revise-su-billete-y-cobre-el-premio-mayor/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/clima-hoy-en-colombia-temperaturas-para-cali-este-13-de-junio/</t>
         </is>
       </c>
     </row>
@@ -6227,12 +6251,12 @@
       </c>
       <c r="D221" s="6" t="inlineStr">
         <is>
-          <t>Iván Cepeda firma pacto por el agua en Bucaramanga y busca sumar apoyos en Santander para la segunda vuelta</t>
+          <t>Clima hoy en Colombia: temperaturas para Cartagena de Indias este 13 de junio</t>
         </is>
       </c>
       <c r="E221" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/ivan-cepeda-firma-pacto-por-el-agua-en-bucaramanga-y-busca-sumar-apoyos-en-santander-para-la-segunda-vuelta/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/clima-hoy-en-colombia-temperaturas-para-cartagena-de-indias-este-13-de-junio/</t>
         </is>
       </c>
     </row>
@@ -6254,12 +6278,12 @@
       </c>
       <c r="D222" s="3" t="inlineStr">
         <is>
-          <t>Generadoras alertan que deuda de Air-e podría superar los $3 billones y ponen sobre la mesa riesgo por fenómeno de El Niño</t>
+          <t>Resultado Sinuano Noche hoy 12 de junio</t>
         </is>
       </c>
       <c r="E222" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/generadoras-alertan-que-deuda-de-air-e-podria-superar-los-3-billones-y-ponen-sobre-la-mesa-riesgo-por-fenomeno-de-el-nino/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/resultado-sinuano-noche-hoy-12-de-junio/</t>
         </is>
       </c>
     </row>
@@ -6281,12 +6305,12 @@
       </c>
       <c r="D223" s="6" t="inlineStr">
         <is>
-          <t>Resultado Chontico Noche: números ganadores del último sorteo hoy, viernes 12 de junio de 2026</t>
+          <t>Mindefensa alerta por posibles disturbios tras la segunda vuelta y anticipa medidas por información de inteligencia</t>
         </is>
       </c>
       <c r="E223" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/resultado-chontico-noche-numeros-ganadores-del-ultimo-sorteo-hoy-viernes-12-de-junio-de-2026/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/mindefensa-alerta-por-posibles-disturbios-tras-la-segunda-vuelta-y-anticipa-medidas-por-informacion-de-inteligencia/</t>
         </is>
       </c>
     </row>
@@ -6308,12 +6332,12 @@
       </c>
       <c r="D224" s="3" t="inlineStr">
         <is>
-          <t>Lotería de Risaralda: resultados ganadores del sábado 13 de junio</t>
+          <t>JEP ha identificado plenamente a 1.956 víctimas de falsos positivos y aún busca establecer quiénes son otras 418</t>
         </is>
       </c>
       <c r="E224" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/loteria-de-risaralda-resultados-ganadores-del-sabado-13-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/jep-ha-identificado-plenamente-a-1956-victimas-de-falsos-positivos-y-aun-busca-establecer-quienes-son-otras-418/</t>
         </is>
       </c>
     </row>
@@ -6335,12 +6359,12 @@
       </c>
       <c r="D225" s="6" t="inlineStr">
         <is>
-          <t>Resultados Lotería de Medellín 12 de junio: números ganadores del último sorteo</t>
+          <t>“Costó 30.000 pesos y hoy estoy pagando con todo este dolor”: influencer denuncia procedimiento estético que casi le cuesta la vida</t>
         </is>
       </c>
       <c r="E225" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/resultados-loteria-de-medellin-12-de-junio-numeros-ganadores-del-ultimo-sorteo/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/costo-30000-pesos-y-hoy-estoy-pagando-con-todo-este-dolor-influencer-denuncia-procedimiento-estetico-que-casi-le-cuesta-la-vida/</t>
         </is>
       </c>
     </row>
@@ -6362,12 +6386,12 @@
       </c>
       <c r="D226" s="3" t="inlineStr">
         <is>
-          <t>Resultado Super Astro Luna HOY: número ganador del viernes 12 de junio</t>
+          <t>Resultados Lotería de Santander hoy 13 de junio: revise su billete y cobre el premio mayor</t>
         </is>
       </c>
       <c r="E226" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/resultado-super-astro-luna-hoy-numero-ganador-del-viernes-12-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/resultados-loteria-de-santander-hoy-13-de-junio-revise-su-billete-y-cobre-el-premio-mayor/</t>
         </is>
       </c>
     </row>
@@ -6389,12 +6413,12 @@
       </c>
       <c r="D227" s="6" t="inlineStr">
         <is>
-          <t>Alias Samantha, la vocera de las disidencias de las Farc por la que ofrecen 100 millones de pesos de recompensa</t>
+          <t>Iván Cepeda firma pacto por el agua en Bucaramanga y busca sumar apoyos en Santander para la segunda vuelta</t>
         </is>
       </c>
       <c r="E227" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/alias-samantha-la-vocera-de-las-disidencias-de-las-farc-por-la-que-ofrecen-100-millones-de-pesos-de-recompensa/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/ivan-cepeda-firma-pacto-por-el-agua-en-bucaramanga-y-busca-sumar-apoyos-en-santander-para-la-segunda-vuelta/</t>
         </is>
       </c>
     </row>
@@ -6416,12 +6440,12 @@
       </c>
       <c r="D228" s="3" t="inlineStr">
         <is>
-          <t>Sebastián Montoya repite problemas en clasificación de la Fórmula 2: esta será su posición en el Gran Premio de Barcelona</t>
+          <t>Generadoras alertan que deuda de Air-e podría superar los $3 billones y ponen sobre la mesa riesgo por fenómeno de El Niño</t>
         </is>
       </c>
       <c r="E228" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/06/13/sebastian-montoya-repite-problemas-en-clasificacion-de-la-formula-2-esta-sera-su-posicion-en-el-gran-premio-de-barcelona/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/generadoras-alertan-que-deuda-de-air-e-podria-superar-los-3-billones-y-ponen-sobre-la-mesa-riesgo-por-fenomeno-de-el-nino/</t>
         </is>
       </c>
     </row>
@@ -6443,12 +6467,12 @@
       </c>
       <c r="D229" s="6" t="inlineStr">
         <is>
-          <t>Así le fue al rating de la televisión colombiana con la inauguración del Mundial 2026</t>
+          <t>Resultado Chontico Noche: números ganadores del último sorteo hoy, viernes 12 de junio de 2026</t>
         </is>
       </c>
       <c r="E229" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/asi-le-fue-al-rating-de-la-television-colombiana-con-la-inauguracion-del-mundial-2026/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/resultado-chontico-noche-numeros-ganadores-del-ultimo-sorteo-hoy-viernes-12-de-junio-de-2026/</t>
         </is>
       </c>
     </row>
@@ -6470,12 +6494,12 @@
       </c>
       <c r="D230" s="3" t="inlineStr">
         <is>
-          <t>Prepárese si va a salir en puente festivo por la vía al Llano: se registra bloqueo total por protestas</t>
+          <t>Lotería de Risaralda: resultados ganadores del sábado 13 de junio</t>
         </is>
       </c>
       <c r="E230" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/preparese-si-va-a-salir-en-puente-festivo-por-la-via-al-llano-se-registra-bloqueo-total-por-protestas/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/loteria-de-risaralda-resultados-ganadores-del-sabado-13-de-junio/</t>
         </is>
       </c>
     </row>
@@ -6497,12 +6521,12 @@
       </c>
       <c r="D231" s="6" t="inlineStr">
         <is>
-          <t>Periodistas españoles clasificaron las camisetas de las 48 selecciones del Mundial: así le fue a Colombia</t>
+          <t>Resultados Lotería de Medellín 12 de junio: números ganadores del último sorteo</t>
         </is>
       </c>
       <c r="E231" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/06/13/periodistas-espanoles-clasificaron-las-camisetas-de-las-48-selecciones-del-mundial-asi-le-fue-a-colombia/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/resultados-loteria-de-medellin-12-de-junio-numeros-ganadores-del-ultimo-sorteo/</t>
         </is>
       </c>
     </row>
@@ -6524,12 +6548,12 @@
       </c>
       <c r="D232" s="3" t="inlineStr">
         <is>
-          <t>Gustavo Bolívar recreó polémica entrevista de De la Espriella para hacerle campaña a Cepeda: “Unos votos bien bacanos del electorado femenino”</t>
+          <t>Resultado Super Astro Luna HOY: número ganador del viernes 12 de junio</t>
         </is>
       </c>
       <c r="E232" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/gustavo-bolivar-recreo-polemica-entrevista-de-de-la-espriella-para-hacerle-campana-a-cepeda-unos-votos-bien-bacanos-del-electorado-femenino/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/resultado-super-astro-luna-hoy-numero-ganador-del-viernes-12-de-junio/</t>
         </is>
       </c>
     </row>
@@ -6551,12 +6575,12 @@
       </c>
       <c r="D233" s="6" t="inlineStr">
         <is>
-          <t>Hombre se salvó de secuestro al lanzarse de un vehículo en movimiento en Medellín: hay dos capturados</t>
+          <t>Alias Samantha, la vocera de las disidencias de las Farc por la que ofrecen 100 millones de pesos de recompensa</t>
         </is>
       </c>
       <c r="E233" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/hombre-se-salvo-de-secuestro-al-lanzarse-de-un-vehiculo-en-movimiento-en-medellin-hay-dos-capturados/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/alias-samantha-la-vocera-de-las-disidencias-de-las-farc-por-la-que-ofrecen-100-millones-de-pesos-de-recompensa/</t>
         </is>
       </c>
     </row>
@@ -6578,12 +6602,12 @@
       </c>
       <c r="D234" s="3" t="inlineStr">
         <is>
-          <t>Abelardo de la Espriella se pronunció sobre caída de las acciones legales que perjudicaban su campaña: “No tenemos rabo de paja”</t>
+          <t>Sebastián Montoya repite problemas en clasificación de la Fórmula 2: esta será su posición en el Gran Premio de Barcelona</t>
         </is>
       </c>
       <c r="E234" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/abelardo-de-la-espriella-se-pronuncio-sobre-caida-de-las-acciones-legales-que-perjudicaban-su-campana-no-tenemos-rabo-de-paja/</t>
+          <t>https://www.infobae.com/colombia/deportes/2026/06/13/sebastian-montoya-repite-problemas-en-clasificacion-de-la-formula-2-esta-sera-su-posicion-en-el-gran-premio-de-barcelona/</t>
         </is>
       </c>
     </row>
@@ -7020,7 +7044,11 @@
       </c>
     </row>
     <row r="251">
-      <c r="A251" s="5" t="inlineStr"/>
+      <c r="A251" s="5" t="inlineStr">
+        <is>
+          <t>12/06/2026 05:19 p. m.</t>
+        </is>
+      </c>
       <c r="B251" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -7028,22 +7056,26 @@
       </c>
       <c r="C251" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>La Silla Vacía</t>
         </is>
       </c>
       <c r="D251" s="6" t="inlineStr">
         <is>
-          <t>La Especial Águila: el fichaje del año une cerveza y maní para la fiesta del fútbol</t>
+          <t>Petro vuelve a rayar la participación en política en canal de WhatsApp</t>
         </is>
       </c>
       <c r="E251" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/la-especial-aguila/</t>
+          <t>https://www.lasillavacia.com/en-vivo/petro-vuelve-a-rayar-la-participacion-en-politica-en-canal-de-whatsapp/</t>
         </is>
       </c>
     </row>
     <row r="252">
-      <c r="A252" s="2" t="inlineStr"/>
+      <c r="A252" s="2" t="inlineStr">
+        <is>
+          <t>12/06/2026 03:55 p. m.</t>
+        </is>
+      </c>
       <c r="B252" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -7051,22 +7083,26 @@
       </c>
       <c r="C252" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>La Silla Vacía</t>
         </is>
       </c>
       <c r="D252" s="3" t="inlineStr">
         <is>
-          <t>Natura tienda Andino: la marca fortalece su apuesta omnicanal en Colombia</t>
+          <t>El último Marco Fiscal espera cerrar 2026 con un mayor pago de intereses</t>
         </is>
       </c>
       <c r="E252" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/natura-tienda-andino/</t>
+          <t>https://www.lasillavacia.com/en-vivo/el-ultimo-marco-fiscal-espera-cerrar-2026-con-un-mayor-pago-de-intereses/</t>
         </is>
       </c>
     </row>
     <row r="253">
-      <c r="A253" s="5" t="inlineStr"/>
+      <c r="A253" s="5" t="inlineStr">
+        <is>
+          <t>12/06/2026 03:44 p. m.</t>
+        </is>
+      </c>
       <c r="B253" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -7074,22 +7110,26 @@
       </c>
       <c r="C253" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>La Silla Vacía</t>
         </is>
       </c>
       <c r="D253" s="6" t="inlineStr">
         <is>
-          <t>Grupo Firme Ibagué 2026: todo listo para La Última Peda Tour en la Ciudad Musical</t>
+          <t>USO convocó a intensificar movilizaciones en instalaciones de Ecopetrol</t>
         </is>
       </c>
       <c r="E253" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/grupo-firme-ibague-2026/</t>
+          <t>https://www.lasillavacia.com/en-vivo/uso-convoco-a-intensificar-movilizaciones-en-instalaciones-de-ecopetrol/</t>
         </is>
       </c>
     </row>
     <row r="254">
-      <c r="A254" s="2" t="inlineStr"/>
+      <c r="A254" s="2" t="inlineStr">
+        <is>
+          <t>12/06/2026 02:45 p. m.</t>
+        </is>
+      </c>
       <c r="B254" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -7097,22 +7137,26 @@
       </c>
       <c r="C254" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>La Silla Vacía</t>
         </is>
       </c>
       <c r="D254" s="3" t="inlineStr">
         <is>
-          <t>Roger Taylor Violence Insane In A Beautiful World: anuncia nuevo álbum solista</t>
+          <t>Dane reporta que pobreza monetaria de 2025 cayó al 28%</t>
         </is>
       </c>
       <c r="E254" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/roger-taylor-violence-insane-in-a-beautiful-world/</t>
+          <t>https://www.lasillavacia.com/en-vivo/dane-reporta-que-pobreza-monetaria-de-2025-cayo-al-28/</t>
         </is>
       </c>
     </row>
     <row r="255">
-      <c r="A255" s="5" t="inlineStr"/>
+      <c r="A255" s="5" t="inlineStr">
+        <is>
+          <t>12/06/2026 02:33 p. m.</t>
+        </is>
+      </c>
       <c r="B255" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -7120,22 +7164,26 @@
       </c>
       <c r="C255" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>La Silla Vacía</t>
         </is>
       </c>
       <c r="D255" s="6" t="inlineStr">
         <is>
-          <t>Christian Albarracín Maestro de Maestros: el artista colombiano fue reconocido por su trayectoria</t>
+          <t>Mindefensa advierte posibles disturbios violentos tras segunda vuelta</t>
         </is>
       </c>
       <c r="E255" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/christian-albarracin-maestro-de-maestros/</t>
+          <t>https://www.lasillavacia.com/en-vivo/mindefensa-advierte-posibles-disturbios-violentos-tras-segunda-vuelta/</t>
         </is>
       </c>
     </row>
     <row r="256">
-      <c r="A256" s="2" t="inlineStr"/>
+      <c r="A256" s="2" t="inlineStr">
+        <is>
+          <t>12/06/2026 01:39 p. m.</t>
+        </is>
+      </c>
       <c r="B256" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -7143,22 +7191,26 @@
       </c>
       <c r="C256" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>La Silla Vacía</t>
         </is>
       </c>
       <c r="D256" s="3" t="inlineStr">
         <is>
-          <t>Guía del Festival del Bambuco en San Juan y San Pedro: Historia, sedes, actividades y cómo se vive en Colombia</t>
+          <t>Diario de Campaña: programas, denuncias y viento a favor de De la Espriella</t>
         </is>
       </c>
       <c r="E256" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/guia-del-festival-del-bambuco-en-san-juan-y-san-pedro-historia-sedes-actividades-y-como-se-vive-en-colombia/</t>
+          <t>https://www.lasillavacia.com/en-vivo/diario-de-campana-programas-denuncias-y-viento-a-favor-de-de-la-espriella/</t>
         </is>
       </c>
     </row>
     <row r="257">
-      <c r="A257" s="5" t="inlineStr"/>
+      <c r="A257" s="5" t="inlineStr">
+        <is>
+          <t>12/06/2026 01:03 p. m.</t>
+        </is>
+      </c>
       <c r="B257" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -7166,22 +7218,26 @@
       </c>
       <c r="C257" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>La Silla Vacía</t>
         </is>
       </c>
       <c r="D257" s="6" t="inlineStr">
         <is>
-          <t>El descanso que viene: Estos son los próximos días festivos que le quedan a Colombia en 2026</t>
+          <t>Sin sorpresas, el Mais se adhiere a la campaña de Cepeda</t>
         </is>
       </c>
       <c r="E257" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/el-descanso-que-viene-estos-son-los-proximos-dias-festivos-que-le-quedan-a-colombia-en-2026/</t>
+          <t>https://www.lasillavacia.com/en-vivo/sin-sorpresas-el-mais-se-adhiere-a-la-campana-de-cepeda/</t>
         </is>
       </c>
     </row>
     <row r="258">
-      <c r="A258" s="2" t="inlineStr"/>
+      <c r="A258" s="2" t="inlineStr">
+        <is>
+          <t>12/06/2026 12:18 p. m.</t>
+        </is>
+      </c>
       <c r="B258" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -7189,22 +7245,26 @@
       </c>
       <c r="C258" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>La Silla Vacía</t>
         </is>
       </c>
       <c r="D258" s="3" t="inlineStr">
         <is>
-          <t>Fiestas temáticas e inolvidables: Guía de ideas creativas para celebrar un cumpleaños por lo alto</t>
+          <t>Corte Suprema frena orden que prohibía a Abelardo usar símbolos patrios</t>
         </is>
       </c>
       <c r="E258" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/fiestas-tematicas-e-inolvidables-guia-de-ideas-creativas-para-celebrar-un-cumpleanos-por-lo-alto/</t>
+          <t>https://www.lasillavacia.com/en-vivo/corte-suprema-frena-la-orden-que-prohibia-a-abelardo-usar-simbolos-patrios/</t>
         </is>
       </c>
     </row>
     <row r="259">
-      <c r="A259" s="5" t="inlineStr"/>
+      <c r="A259" s="5" t="inlineStr">
+        <is>
+          <t>12/06/2026 11:20 a. m.</t>
+        </is>
+      </c>
       <c r="B259" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -7212,22 +7272,26 @@
       </c>
       <c r="C259" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>La Silla Vacía</t>
         </is>
       </c>
       <c r="D259" s="6" t="inlineStr">
         <is>
-          <t>Travesía por el llano: Los pueblos más lindos y encantadores para visitar en el Meta y Casanare</t>
+          <t>Oviedo se reunió con Uribe, pero sigue sin apoyar a ningún candidato</t>
         </is>
       </c>
       <c r="E259" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/travesia-por-el-llano-los-pueblos-mas-lindos-y-encantadores-para-visitar-en-el-meta-y-casanare/</t>
+          <t>https://www.lasillavacia.com/en-vivo/oviedo-se-reunio-con-uribe-pero-sigue-sin-apoyar-a-ningun-candidato/</t>
         </is>
       </c>
     </row>
     <row r="260">
-      <c r="A260" s="2" t="inlineStr"/>
+      <c r="A260" s="2" t="inlineStr">
+        <is>
+          <t>12/06/2026 10:07 a. m.</t>
+        </is>
+      </c>
       <c r="B260" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -7235,22 +7299,26 @@
       </c>
       <c r="C260" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>La Silla Vacía</t>
         </is>
       </c>
       <c r="D260" s="3" t="inlineStr">
         <is>
-          <t>¡Evite estafas! Terminal de Transporte de Bogotá alerta sobre fraudes y suplantación en las Zonas de Parqueo Pago</t>
+          <t>Santander: artistas denuncian amenazas y exigencias para buscar votos</t>
         </is>
       </c>
       <c r="E260" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/evite-estafas-terminal-de-transporte-de-bogota-alerta-sobre-fraudes-y-suplantacion-en-las-zonas-de-parqueo-pago/</t>
+          <t>https://www.lasillavacia.com/en-vivo/santander-artistas-denuncian-amenazas-y-exigencias-para-buscar-votos/</t>
         </is>
       </c>
     </row>
     <row r="261">
-      <c r="A261" s="5" t="inlineStr"/>
+      <c r="A261" s="5" t="inlineStr">
+        <is>
+          <t>12/06/2026 09:21 a. m.</t>
+        </is>
+      </c>
       <c r="B261" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -7258,22 +7326,26 @@
       </c>
       <c r="C261" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>La Silla Vacía</t>
         </is>
       </c>
       <c r="D261" s="6" t="inlineStr">
         <is>
-          <t>El camino tricolor: El fixture, las sedes y las expectativas de la Selección Colombia en el Mundial 2026</t>
+          <t>Invamer no publicará encuestas presidenciales para segunda vuelta</t>
         </is>
       </c>
       <c r="E261" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/el-camino-tricolor-el-fixture-las-sedes-y-las-expectativas-de-la-seleccion-colombia-en-el-mundial-2026/</t>
+          <t>https://www.lasillavacia.com/en-vivo/invamer-no-publicara-encuestas-presidenciales-para-segunda-vuelta/</t>
         </is>
       </c>
     </row>
     <row r="262">
-      <c r="A262" s="2" t="inlineStr"/>
+      <c r="A262" s="2" t="inlineStr">
+        <is>
+          <t>12/06/2026 08:18 a. m.</t>
+        </is>
+      </c>
       <c r="B262" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -7281,22 +7353,26 @@
       </c>
       <c r="C262" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>La Silla Vacía</t>
         </is>
       </c>
       <c r="D262" s="3" t="inlineStr">
         <is>
-          <t>GYAL Festival 2026: Alexis y Fido junto a Baby Rasta &amp; Gringo revivirán el reggaetón de los 2000</t>
+          <t>Consejo de Estado deja en firme candidatura de Abelardo de la Espriella</t>
         </is>
       </c>
       <c r="E262" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/gyal-festival-2026/</t>
+          <t>https://www.lasillavacia.com/en-vivo/consejo-de-estado-deja-en-firme-candidatura-de-abelardo-de-la-espriella/</t>
         </is>
       </c>
     </row>
     <row r="263">
-      <c r="A263" s="5" t="inlineStr"/>
+      <c r="A263" s="5" t="inlineStr">
+        <is>
+          <t>12/06/2026 07:31 a. m.</t>
+        </is>
+      </c>
       <c r="B263" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -7304,22 +7380,26 @@
       </c>
       <c r="C263" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>La Silla Vacía</t>
         </is>
       </c>
       <c r="D263" s="6" t="inlineStr">
         <is>
-          <t>Medios comunitarios en Colombia: los retos que definirán su futuro</t>
+          <t>Desayune informado con las movidas de este 12 de junio de 2026</t>
         </is>
       </c>
       <c r="E263" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/medios-comunitarios-colombia/</t>
+          <t>https://www.lasillavacia.com/en-vivo/desayune-informado-con-las-movidas-de-este-12-de-junio-de-2026/</t>
         </is>
       </c>
     </row>
     <row r="264">
-      <c r="A264" s="2" t="inlineStr"/>
+      <c r="A264" s="2" t="inlineStr">
+        <is>
+          <t>11/06/2026 07:31 p. m.</t>
+        </is>
+      </c>
       <c r="B264" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -7327,22 +7407,26 @@
       </c>
       <c r="C264" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>La Silla Vacía</t>
         </is>
       </c>
       <c r="D264" s="3" t="inlineStr">
         <is>
-          <t>Última hora: Plenaria de la Cámara suspende a Gloria Arizabaleta tras ordenar la salida provisional de Gustavo Petro</t>
+          <t>Duerma informado con las movidas de este 11 de junio de 2026</t>
         </is>
       </c>
       <c r="E264" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/ultima-hora-plenaria-de-la-camara-suspende-a-gloria-arizabaleta-tras-ordenar-la-salida-provisional-de-gustavo-petro/</t>
+          <t>https://www.lasillavacia.com/en-vivo/duerma-informado-con-las-movidas-de-este-11-de-junio-de-2026-2/</t>
         </is>
       </c>
     </row>
     <row r="265">
-      <c r="A265" s="5" t="inlineStr"/>
+      <c r="A265" s="5" t="inlineStr">
+        <is>
+          <t>11/06/2026 07:19 p. m.</t>
+        </is>
+      </c>
       <c r="B265" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -7350,22 +7434,26 @@
       </c>
       <c r="C265" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>La Silla Vacía</t>
         </is>
       </c>
       <c r="D265" s="6" t="inlineStr">
         <is>
-          <t>¡Rueda el balón! Así se vivió la espectacular y emotiva inauguración del Mundial de la FIFA 2026 en el Estadio Azteca</t>
+          <t>Nairo, Borja y El Pibe: Abelardo suma adhesiones deportivas a su campaña</t>
         </is>
       </c>
       <c r="E265" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/rueda-el-balon-asi-se-vivio-la-espectacular-y-emotiva-inauguracion-del-mundial-de-la-fifa-2026-en-el-estadio-azteca/</t>
+          <t>https://www.lasillavacia.com/en-vivo/nairo-borja-y-el-pibe-abelardo-suma-adhesiones-deportivas-a-su-campana/</t>
         </is>
       </c>
     </row>
     <row r="266">
-      <c r="A266" s="2" t="inlineStr"/>
+      <c r="A266" s="2" t="inlineStr">
+        <is>
+          <t>11/06/2026 06:32 p. m.</t>
+        </is>
+      </c>
       <c r="B266" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -7373,22 +7461,26 @@
       </c>
       <c r="C266" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>La Silla Vacía</t>
         </is>
       </c>
       <c r="D266" s="3" t="inlineStr">
         <is>
-          <t>Desinformación en América Latina: el debate que marcará el Encuentro de Medios en Cartagena</t>
+          <t>El Niño llegó oficialmente a Colombia tres meses antes de lo previsto</t>
         </is>
       </c>
       <c r="E266" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/desinformacion-america-latina/</t>
+          <t>https://www.lasillavacia.com/en-vivo/el-nino-llego-oficialmente-a-colombia-tres-meses-antes-de-lo-previsto/</t>
         </is>
       </c>
     </row>
     <row r="267">
-      <c r="A267" s="5" t="inlineStr"/>
+      <c r="A267" s="5" t="inlineStr">
+        <is>
+          <t>11/06/2026 05:42 p. m.</t>
+        </is>
+      </c>
       <c r="B267" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -7396,22 +7488,26 @@
       </c>
       <c r="C267" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>La Silla Vacía</t>
         </is>
       </c>
       <c r="D267" s="6" t="inlineStr">
         <is>
-          <t>Premios Jaime Garzón 2026: el homenaje que marcará el Encuentro de Medios Alternativos</t>
+          <t>A diez días de la segunda vuelta, Cepeda publica su plan de gobierno</t>
         </is>
       </c>
       <c r="E267" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/premios-jaime-garzon-2026/</t>
+          <t>https://www.lasillavacia.com/en-vivo/a-diez-dias-para-la-segunda-vuelta-cepeda-publica-su-plan-de-gobierno/</t>
         </is>
       </c>
     </row>
     <row r="268">
-      <c r="A268" s="2" t="inlineStr"/>
+      <c r="A268" s="2" t="inlineStr">
+        <is>
+          <t>11/06/2026 04:59 p. m.</t>
+        </is>
+      </c>
       <c r="B268" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -7419,22 +7515,26 @@
       </c>
       <c r="C268" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>La Silla Vacía</t>
         </is>
       </c>
       <c r="D268" s="3" t="inlineStr">
         <is>
-          <t>Pink Floyd 8-Tracks: el nuevo recopilatorio revive la era dorada de la banda</t>
+          <t>Consejo de Estado deja en firme elección de Héctor Carvajal en la Corte</t>
         </is>
       </c>
       <c r="E268" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/pink-floyd-8-tracks/</t>
+          <t>https://www.lasillavacia.com/en-vivo/consejo-de-estado-deja-en-firme-eleccion-de-hector-carvajal-en-la-corte/</t>
         </is>
       </c>
     </row>
     <row r="269">
-      <c r="A269" s="5" t="inlineStr"/>
+      <c r="A269" s="5" t="inlineStr">
+        <is>
+          <t>11/06/2026 03:22 p. m.</t>
+        </is>
+      </c>
       <c r="B269" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -7442,22 +7542,26 @@
       </c>
       <c r="C269" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>La Silla Vacía</t>
         </is>
       </c>
       <c r="D269" s="6" t="inlineStr">
         <is>
-          <t>Morat Panini Mundial 2026: la banda colombiana hace historia rumbo a la Copa del Mundo</t>
+          <t>“Cortinas de humo”: Abelardo responde a denuncia de Cepeda en su contra</t>
         </is>
       </c>
       <c r="E269" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/morat-panini-mundial-2026/</t>
+          <t>https://www.lasillavacia.com/en-vivo/cortina-de-humo-abelardo-responde-a-denuncia-de-cepeda-en-su-contra/</t>
         </is>
       </c>
     </row>
     <row r="270">
-      <c r="A270" s="2" t="inlineStr"/>
+      <c r="A270" s="2" t="inlineStr">
+        <is>
+          <t>11/06/2026 02:31 p. m.</t>
+        </is>
+      </c>
       <c r="B270" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -7465,17 +7569,17 @@
       </c>
       <c r="C270" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>La Silla Vacía</t>
         </is>
       </c>
       <c r="D270" s="3" t="inlineStr">
         <is>
-          <t>Julián Daza La Diez: el nuevo himno de Ronaldinho que une fútbol y música</t>
+          <t>Abogado de Petro anunció denuncia contra Arizabaleta por prevaricato</t>
         </is>
       </c>
       <c r="E270" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/julian-daza-la-diez-ronaldinho/</t>
+          <t>https://www.lasillavacia.com/en-vivo/abogado-de-petro-anuncio-denuncia-contra-arizabaleta-por-prevaricato/</t>
         </is>
       </c>
     </row>
@@ -7493,12 +7597,12 @@
       </c>
       <c r="D271" s="6" t="inlineStr">
         <is>
-          <t>Encuentro de Medios Alternativos 2026 reunirá voces de América Latina en Cartagena</t>
+          <t>La Especial Águila: el fichaje del año une cerveza y maní para la fiesta del fútbol</t>
         </is>
       </c>
       <c r="E271" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/encuentro-medios-alternativos-2026/</t>
+          <t>https://canaltrece.com.co/noticias/la-especial-aguila/</t>
         </is>
       </c>
     </row>
@@ -7516,12 +7620,12 @@
       </c>
       <c r="D272" s="3" t="inlineStr">
         <is>
-          <t>CDMX La Batalla 2.0 regresa a Bogotá: música mexicana y duelo en el Astor Plaza</t>
+          <t>Natura tienda Andino: la marca fortalece su apuesta omnicanal en Colombia</t>
         </is>
       </c>
       <c r="E272" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/cdmx-la-batalla-2-bogota/</t>
+          <t>https://canaltrece.com.co/noticias/natura-tienda-andino/</t>
         </is>
       </c>
     </row>
@@ -7539,12 +7643,12 @@
       </c>
       <c r="D273" s="6" t="inlineStr">
         <is>
-          <t>Nuevo formato Mundial 2026: así cambiará la Copa del Mundo para siempre</t>
+          <t>Grupo Firme Ibagué 2026: todo listo para La Última Peda Tour en la Ciudad Musical</t>
         </is>
       </c>
       <c r="E273" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/nuevo-formato-mundial-2026/</t>
+          <t>https://canaltrece.com.co/noticias/grupo-firme-ibague-2026/</t>
         </is>
       </c>
     </row>
@@ -7562,12 +7666,12 @@
       </c>
       <c r="D274" s="3" t="inlineStr">
         <is>
-          <t>Mundial Amazónico 2026: deporte, cultura e integración en Leticia</t>
+          <t>Roger Taylor Violence Insane In A Beautiful World: anuncia nuevo álbum solista</t>
         </is>
       </c>
       <c r="E274" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/mundial-amazonico-2026-deporte-cultura-e-integracion-en-leticia/</t>
+          <t>https://canaltrece.com.co/noticias/roger-taylor-violence-insane-in-a-beautiful-world/</t>
         </is>
       </c>
     </row>
@@ -7585,12 +7689,12 @@
       </c>
       <c r="D275" s="6" t="inlineStr">
         <is>
-          <t>Selecciones sorpresa Mundial 2026: los equipos que podrían cambiar la historia</t>
+          <t>Christian Albarracín Maestro de Maestros: el artista colombiano fue reconocido por su trayectoria</t>
         </is>
       </c>
       <c r="E275" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/selecciones-sorpresa-mundial-2026/</t>
+          <t>https://canaltrece.com.co/noticias/christian-albarracin-maestro-de-maestros/</t>
         </is>
       </c>
     </row>
@@ -7608,12 +7712,12 @@
       </c>
       <c r="D276" s="3" t="inlineStr">
         <is>
-          <t>Ceremonia inauguración Mundial 2026: hora, artistas y cómo verla en vivo</t>
+          <t>Guía del Festival del Bambuco en San Juan y San Pedro: Historia, sedes, actividades y cómo se vive en Colombia</t>
         </is>
       </c>
       <c r="E276" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/ceremonia-inauguracion-mundial-2026/</t>
+          <t>https://canaltrece.com.co/noticias/guia-del-festival-del-bambuco-en-san-juan-y-san-pedro-historia-sedes-actividades-y-como-se-vive-en-colombia/</t>
         </is>
       </c>
     </row>
@@ -7631,12 +7735,12 @@
       </c>
       <c r="D277" s="6" t="inlineStr">
         <is>
-          <t>Jugadores jóvenes Mundial 2026: las promesas que podrían convertirse en estrellas</t>
+          <t>El descanso que viene: Estos son los próximos días festivos que le quedan a Colombia en 2026</t>
         </is>
       </c>
       <c r="E277" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/jugadores-jovenes-mundial-2026/</t>
+          <t>https://canaltrece.com.co/noticias/el-descanso-que-viene-estos-son-los-proximos-dias-festivos-que-le-quedan-a-colombia-en-2026/</t>
         </is>
       </c>
     </row>
@@ -7654,12 +7758,12 @@
       </c>
       <c r="D278" s="3" t="inlineStr">
         <is>
-          <t>La fiebre del Mundial de la FIFA 2026: El salvavidas que impulsa la economía y el consumo en Colombia</t>
+          <t>Fiestas temáticas e inolvidables: Guía de ideas creativas para celebrar un cumpleaños por lo alto</t>
         </is>
       </c>
       <c r="E278" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/la-fiebre-del-mundial-de-la-fifa-2026-el-salvavidas-que-impulsa-la-economia-y-el-consumo-en-colombia/</t>
+          <t>https://canaltrece.com.co/noticias/fiestas-tematicas-e-inolvidables-guia-de-ideas-creativas-para-celebrar-un-cumpleanos-por-lo-alto/</t>
         </is>
       </c>
     </row>
@@ -7677,12 +7781,12 @@
       </c>
       <c r="D279" s="6" t="inlineStr">
         <is>
-          <t>Fuerte operativo de recuperación de espacio público en la glorieta de la Avenida Villavicencio deja desalojos y control policial permanente</t>
+          <t>Travesía por el llano: Los pueblos más lindos y encantadores para visitar en el Meta y Casanare</t>
         </is>
       </c>
       <c r="E279" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/fuerte-operativo-de-recuperacion-de-espacio-publico-en-la-glorieta-de-la-avenida-villavicencio-deja-desalojos-y-control-policial-permanente/</t>
+          <t>https://canaltrece.com.co/noticias/travesia-por-el-llano-los-pueblos-mas-lindos-y-encantadores-para-visitar-en-el-meta-y-casanare/</t>
         </is>
       </c>
     </row>
@@ -7700,17 +7804,477 @@
       </c>
       <c r="D280" s="3" t="inlineStr">
         <is>
+          <t>¡Evite estafas! Terminal de Transporte de Bogotá alerta sobre fraudes y suplantación en las Zonas de Parqueo Pago</t>
+        </is>
+      </c>
+      <c r="E280" s="4" t="inlineStr">
+        <is>
+          <t>https://canaltrece.com.co/noticias/evite-estafas-terminal-de-transporte-de-bogota-alerta-sobre-fraudes-y-suplantacion-en-las-zonas-de-parqueo-pago/</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="5" t="inlineStr"/>
+      <c r="B281" s="5" t="inlineStr">
+        <is>
+          <t>Medio de Comunicación</t>
+        </is>
+      </c>
+      <c r="C281" s="5" t="inlineStr">
+        <is>
+          <t>Canal Trece</t>
+        </is>
+      </c>
+      <c r="D281" s="6" t="inlineStr">
+        <is>
+          <t>El camino tricolor: El fixture, las sedes y las expectativas de la Selección Colombia en el Mundial 2026</t>
+        </is>
+      </c>
+      <c r="E281" s="7" t="inlineStr">
+        <is>
+          <t>https://canaltrece.com.co/noticias/el-camino-tricolor-el-fixture-las-sedes-y-las-expectativas-de-la-seleccion-colombia-en-el-mundial-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="2" t="inlineStr"/>
+      <c r="B282" s="2" t="inlineStr">
+        <is>
+          <t>Medio de Comunicación</t>
+        </is>
+      </c>
+      <c r="C282" s="2" t="inlineStr">
+        <is>
+          <t>Canal Trece</t>
+        </is>
+      </c>
+      <c r="D282" s="3" t="inlineStr">
+        <is>
+          <t>GYAL Festival 2026: Alexis y Fido junto a Baby Rasta &amp; Gringo revivirán el reggaetón de los 2000</t>
+        </is>
+      </c>
+      <c r="E282" s="4" t="inlineStr">
+        <is>
+          <t>https://canaltrece.com.co/noticias/gyal-festival-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="5" t="inlineStr"/>
+      <c r="B283" s="5" t="inlineStr">
+        <is>
+          <t>Medio de Comunicación</t>
+        </is>
+      </c>
+      <c r="C283" s="5" t="inlineStr">
+        <is>
+          <t>Canal Trece</t>
+        </is>
+      </c>
+      <c r="D283" s="6" t="inlineStr">
+        <is>
+          <t>Medios comunitarios en Colombia: los retos que definirán su futuro</t>
+        </is>
+      </c>
+      <c r="E283" s="7" t="inlineStr">
+        <is>
+          <t>https://canaltrece.com.co/noticias/medios-comunitarios-colombia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="2" t="inlineStr"/>
+      <c r="B284" s="2" t="inlineStr">
+        <is>
+          <t>Medio de Comunicación</t>
+        </is>
+      </c>
+      <c r="C284" s="2" t="inlineStr">
+        <is>
+          <t>Canal Trece</t>
+        </is>
+      </c>
+      <c r="D284" s="3" t="inlineStr">
+        <is>
+          <t>Última hora: Plenaria de la Cámara suspende a Gloria Arizabaleta tras ordenar la salida provisional de Gustavo Petro</t>
+        </is>
+      </c>
+      <c r="E284" s="4" t="inlineStr">
+        <is>
+          <t>https://canaltrece.com.co/noticias/ultima-hora-plenaria-de-la-camara-suspende-a-gloria-arizabaleta-tras-ordenar-la-salida-provisional-de-gustavo-petro/</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="5" t="inlineStr"/>
+      <c r="B285" s="5" t="inlineStr">
+        <is>
+          <t>Medio de Comunicación</t>
+        </is>
+      </c>
+      <c r="C285" s="5" t="inlineStr">
+        <is>
+          <t>Canal Trece</t>
+        </is>
+      </c>
+      <c r="D285" s="6" t="inlineStr">
+        <is>
+          <t>¡Rueda el balón! Así se vivió la espectacular y emotiva inauguración del Mundial de la FIFA 2026 en el Estadio Azteca</t>
+        </is>
+      </c>
+      <c r="E285" s="7" t="inlineStr">
+        <is>
+          <t>https://canaltrece.com.co/noticias/rueda-el-balon-asi-se-vivio-la-espectacular-y-emotiva-inauguracion-del-mundial-de-la-fifa-2026-en-el-estadio-azteca/</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="2" t="inlineStr"/>
+      <c r="B286" s="2" t="inlineStr">
+        <is>
+          <t>Medio de Comunicación</t>
+        </is>
+      </c>
+      <c r="C286" s="2" t="inlineStr">
+        <is>
+          <t>Canal Trece</t>
+        </is>
+      </c>
+      <c r="D286" s="3" t="inlineStr">
+        <is>
+          <t>Desinformación en América Latina: el debate que marcará el Encuentro de Medios en Cartagena</t>
+        </is>
+      </c>
+      <c r="E286" s="4" t="inlineStr">
+        <is>
+          <t>https://canaltrece.com.co/noticias/desinformacion-america-latina/</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="5" t="inlineStr"/>
+      <c r="B287" s="5" t="inlineStr">
+        <is>
+          <t>Medio de Comunicación</t>
+        </is>
+      </c>
+      <c r="C287" s="5" t="inlineStr">
+        <is>
+          <t>Canal Trece</t>
+        </is>
+      </c>
+      <c r="D287" s="6" t="inlineStr">
+        <is>
+          <t>Premios Jaime Garzón 2026: el homenaje que marcará el Encuentro de Medios Alternativos</t>
+        </is>
+      </c>
+      <c r="E287" s="7" t="inlineStr">
+        <is>
+          <t>https://canaltrece.com.co/noticias/premios-jaime-garzon-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="2" t="inlineStr"/>
+      <c r="B288" s="2" t="inlineStr">
+        <is>
+          <t>Medio de Comunicación</t>
+        </is>
+      </c>
+      <c r="C288" s="2" t="inlineStr">
+        <is>
+          <t>Canal Trece</t>
+        </is>
+      </c>
+      <c r="D288" s="3" t="inlineStr">
+        <is>
+          <t>Pink Floyd 8-Tracks: el nuevo recopilatorio revive la era dorada de la banda</t>
+        </is>
+      </c>
+      <c r="E288" s="4" t="inlineStr">
+        <is>
+          <t>https://canaltrece.com.co/noticias/pink-floyd-8-tracks/</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="5" t="inlineStr"/>
+      <c r="B289" s="5" t="inlineStr">
+        <is>
+          <t>Medio de Comunicación</t>
+        </is>
+      </c>
+      <c r="C289" s="5" t="inlineStr">
+        <is>
+          <t>Canal Trece</t>
+        </is>
+      </c>
+      <c r="D289" s="6" t="inlineStr">
+        <is>
+          <t>Morat Panini Mundial 2026: la banda colombiana hace historia rumbo a la Copa del Mundo</t>
+        </is>
+      </c>
+      <c r="E289" s="7" t="inlineStr">
+        <is>
+          <t>https://canaltrece.com.co/noticias/morat-panini-mundial-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="2" t="inlineStr"/>
+      <c r="B290" s="2" t="inlineStr">
+        <is>
+          <t>Medio de Comunicación</t>
+        </is>
+      </c>
+      <c r="C290" s="2" t="inlineStr">
+        <is>
+          <t>Canal Trece</t>
+        </is>
+      </c>
+      <c r="D290" s="3" t="inlineStr">
+        <is>
+          <t>Julián Daza La Diez: el nuevo himno de Ronaldinho que une fútbol y música</t>
+        </is>
+      </c>
+      <c r="E290" s="4" t="inlineStr">
+        <is>
+          <t>https://canaltrece.com.co/noticias/julian-daza-la-diez-ronaldinho/</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="5" t="inlineStr"/>
+      <c r="B291" s="5" t="inlineStr">
+        <is>
+          <t>Medio de Comunicación</t>
+        </is>
+      </c>
+      <c r="C291" s="5" t="inlineStr">
+        <is>
+          <t>Canal Trece</t>
+        </is>
+      </c>
+      <c r="D291" s="6" t="inlineStr">
+        <is>
+          <t>Encuentro de Medios Alternativos 2026 reunirá voces de América Latina en Cartagena</t>
+        </is>
+      </c>
+      <c r="E291" s="7" t="inlineStr">
+        <is>
+          <t>https://canaltrece.com.co/noticias/encuentro-medios-alternativos-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="2" t="inlineStr"/>
+      <c r="B292" s="2" t="inlineStr">
+        <is>
+          <t>Medio de Comunicación</t>
+        </is>
+      </c>
+      <c r="C292" s="2" t="inlineStr">
+        <is>
+          <t>Canal Trece</t>
+        </is>
+      </c>
+      <c r="D292" s="3" t="inlineStr">
+        <is>
+          <t>CDMX La Batalla 2.0 regresa a Bogotá: música mexicana y duelo en el Astor Plaza</t>
+        </is>
+      </c>
+      <c r="E292" s="4" t="inlineStr">
+        <is>
+          <t>https://canaltrece.com.co/noticias/cdmx-la-batalla-2-bogota/</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="5" t="inlineStr"/>
+      <c r="B293" s="5" t="inlineStr">
+        <is>
+          <t>Medio de Comunicación</t>
+        </is>
+      </c>
+      <c r="C293" s="5" t="inlineStr">
+        <is>
+          <t>Canal Trece</t>
+        </is>
+      </c>
+      <c r="D293" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo formato Mundial 2026: así cambiará la Copa del Mundo para siempre</t>
+        </is>
+      </c>
+      <c r="E293" s="7" t="inlineStr">
+        <is>
+          <t>https://canaltrece.com.co/noticias/nuevo-formato-mundial-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="2" t="inlineStr"/>
+      <c r="B294" s="2" t="inlineStr">
+        <is>
+          <t>Medio de Comunicación</t>
+        </is>
+      </c>
+      <c r="C294" s="2" t="inlineStr">
+        <is>
+          <t>Canal Trece</t>
+        </is>
+      </c>
+      <c r="D294" s="3" t="inlineStr">
+        <is>
+          <t>Mundial Amazónico 2026: deporte, cultura e integración en Leticia</t>
+        </is>
+      </c>
+      <c r="E294" s="4" t="inlineStr">
+        <is>
+          <t>https://canaltrece.com.co/noticias/mundial-amazonico-2026-deporte-cultura-e-integracion-en-leticia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="5" t="inlineStr"/>
+      <c r="B295" s="5" t="inlineStr">
+        <is>
+          <t>Medio de Comunicación</t>
+        </is>
+      </c>
+      <c r="C295" s="5" t="inlineStr">
+        <is>
+          <t>Canal Trece</t>
+        </is>
+      </c>
+      <c r="D295" s="6" t="inlineStr">
+        <is>
+          <t>Selecciones sorpresa Mundial 2026: los equipos que podrían cambiar la historia</t>
+        </is>
+      </c>
+      <c r="E295" s="7" t="inlineStr">
+        <is>
+          <t>https://canaltrece.com.co/noticias/selecciones-sorpresa-mundial-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="2" t="inlineStr"/>
+      <c r="B296" s="2" t="inlineStr">
+        <is>
+          <t>Medio de Comunicación</t>
+        </is>
+      </c>
+      <c r="C296" s="2" t="inlineStr">
+        <is>
+          <t>Canal Trece</t>
+        </is>
+      </c>
+      <c r="D296" s="3" t="inlineStr">
+        <is>
+          <t>Ceremonia inauguración Mundial 2026: hora, artistas y cómo verla en vivo</t>
+        </is>
+      </c>
+      <c r="E296" s="4" t="inlineStr">
+        <is>
+          <t>https://canaltrece.com.co/noticias/ceremonia-inauguracion-mundial-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="5" t="inlineStr"/>
+      <c r="B297" s="5" t="inlineStr">
+        <is>
+          <t>Medio de Comunicación</t>
+        </is>
+      </c>
+      <c r="C297" s="5" t="inlineStr">
+        <is>
+          <t>Canal Trece</t>
+        </is>
+      </c>
+      <c r="D297" s="6" t="inlineStr">
+        <is>
+          <t>Jugadores jóvenes Mundial 2026: las promesas que podrían convertirse en estrellas</t>
+        </is>
+      </c>
+      <c r="E297" s="7" t="inlineStr">
+        <is>
+          <t>https://canaltrece.com.co/noticias/jugadores-jovenes-mundial-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="2" t="inlineStr"/>
+      <c r="B298" s="2" t="inlineStr">
+        <is>
+          <t>Medio de Comunicación</t>
+        </is>
+      </c>
+      <c r="C298" s="2" t="inlineStr">
+        <is>
+          <t>Canal Trece</t>
+        </is>
+      </c>
+      <c r="D298" s="3" t="inlineStr">
+        <is>
+          <t>La fiebre del Mundial de la FIFA 2026: El salvavidas que impulsa la economía y el consumo en Colombia</t>
+        </is>
+      </c>
+      <c r="E298" s="4" t="inlineStr">
+        <is>
+          <t>https://canaltrece.com.co/noticias/la-fiebre-del-mundial-de-la-fifa-2026-el-salvavidas-que-impulsa-la-economia-y-el-consumo-en-colombia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="5" t="inlineStr"/>
+      <c r="B299" s="5" t="inlineStr">
+        <is>
+          <t>Medio de Comunicación</t>
+        </is>
+      </c>
+      <c r="C299" s="5" t="inlineStr">
+        <is>
+          <t>Canal Trece</t>
+        </is>
+      </c>
+      <c r="D299" s="6" t="inlineStr">
+        <is>
+          <t>Fuerte operativo de recuperación de espacio público en la glorieta de la Avenida Villavicencio deja desalojos y control policial permanente</t>
+        </is>
+      </c>
+      <c r="E299" s="7" t="inlineStr">
+        <is>
+          <t>https://canaltrece.com.co/noticias/fuerte-operativo-de-recuperacion-de-espacio-publico-en-la-glorieta-de-la-avenida-villavicencio-deja-desalojos-y-control-policial-permanente/</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="2" t="inlineStr"/>
+      <c r="B300" s="2" t="inlineStr">
+        <is>
+          <t>Medio de Comunicación</t>
+        </is>
+      </c>
+      <c r="C300" s="2" t="inlineStr">
+        <is>
+          <t>Canal Trece</t>
+        </is>
+      </c>
+      <c r="D300" s="3" t="inlineStr">
+        <is>
           <t>El termómetro del poder: Los presidentes con mayor y menor aprobación en América Latina</t>
         </is>
       </c>
-      <c r="E280" s="4" t="inlineStr">
+      <c r="E300" s="4" t="inlineStr">
         <is>
           <t>https://canaltrece.com.co/noticias/el-termometro-del-poder-los-presidentes-con-mayor-y-menor-aprobacion-en-america-latina/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E280"/>
+  <autoFilter ref="A1:E300"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
@@ -7991,6 +8555,26 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E278" r:id="rId277"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E279" r:id="rId278"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E280" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E281" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E282" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E283" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E284" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E285" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E286" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E287" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E288" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E289" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E290" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E291" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E292" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E293" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E294" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E295" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E296" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E297" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E298" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E299" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E300" r:id="rId299"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Noticias actualizadas 13/06/2026 11:40
</commit_message>
<xml_diff>
--- a/docs/ultimahora.xlsx
+++ b/docs/ultimahora.xlsx
@@ -515,7 +515,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 05:45 a. m.</t>
+          <t>13/06/2026 06:30 a. m.</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -530,19 +530,19 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Roban los guayos y los balones de la selección inglesa antes de su llegada a Kansas City</t>
+          <t>La dieta occidentalizada es ‘tóxica’ para el organismo: este patrón dietético afecta la microbiota intestinal</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/roban-los-guayos-y-los-balones-de-la-seleccion-inglesa-antes-de-su-llegada-a-kansas-city-3564101</t>
+          <t>https://www.eltiempo.com/salud/la-dieta-occidentalizada-es-toxica-para-el-organismo-este-patron-dietetico-afecta-la-microbiota-intestinal-3564033</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 05:15 a. m.</t>
+          <t>13/06/2026 06:03 a. m.</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -557,19 +557,19 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>Más de 125.000 personas salieron de la pobreza monetaria en Bogotá en el último año: ¿a qué se debe esa reducción?</t>
+          <t>Perú procesa 100 % de las actas pero queda a la espera de resolver 1.550 observaciones en elecciones presidenciales</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/bogota/mas-de-125-000-personas-salieron-de-la-pobreza-monetaria-en-bogota-en-el-ultimo-ano-a-que-se-debe-esa-reduccion-3564088</t>
+          <t>https://www.eltiempo.com/mundo/latinoamerica/peru-procesa-100-de-las-actas-pero-queda-a-la-espera-de-resolver-1-550-observaciones-en-elecciones-presidenciales-3564102</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 05:03 a. m.</t>
+          <t>13/06/2026 06:01 a. m.</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -584,19 +584,19 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Encuesta final de Guarumo y Ecoanalítica para segunda vuelta presidencial: Abelardo De la Espriella, 52,6 %; Iván Cepeda, 45 %</t>
+          <t>Panamá necesita un plan concreto ante la rivalidad entre Estados Unidos y China</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/encuesta-final-de-guarumo-y-ecoanalitica-para-segunda-vuelta-presidencial-abelardo-de-la-espriella-52-6-ivan-cepeda-3564095</t>
+          <t>https://www.eltiempo.com/mundo/latinoamerica/panama-necesita-un-plan-concreto-ante-la-rivalidad-entre-estados-unidos-y-china-3564043</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 04:30 a. m.</t>
+          <t>13/06/2026 05:45 a. m.</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -611,19 +611,19 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>¿Placer con Culpa? / El Condimentario</t>
+          <t>Roban los guayos y los balones de la selección inglesa antes de su llegada a Kansas City</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/cultura/gastronomia/placer-con-culpa-el-condimentario-3564022</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/roban-los-guayos-y-los-balones-de-la-seleccion-inglesa-antes-de-su-llegada-a-kansas-city-3564101</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 04:01 a. m.</t>
+          <t>13/06/2026 05:15 a. m.</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -638,19 +638,19 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>De Roma a las misas en estadios: así ha cambiado la devoción hacia el papa</t>
+          <t>Más de 125.000 personas salieron de la pobreza monetaria en Bogotá en el último año: ¿a qué se debe esa reducción?</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/vida/religion/de-roma-a-las-misas-en-estadios-asi-ha-cambiado-la-devocion-hacia-el-papa-3564052</t>
+          <t>https://www.eltiempo.com/bogota/mas-de-125-000-personas-salieron-de-la-pobreza-monetaria-en-bogota-en-el-ultimo-ano-a-que-se-debe-esa-reduccion-3564088</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 03:39 a. m.</t>
+          <t>13/06/2026 05:03 a. m.</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -665,19 +665,19 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Ataque de tiburón en Sídney, Australia: cierran famosas playas como Bondi y Coogee por 24 horas</t>
+          <t>Encuesta final de Guarumo y Ecoanalítica para segunda vuelta presidencial: Abelardo De la Espriella, 52,6 %; Iván Cepeda, 45 %</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/mas-regiones/ataque-de-tiburon-en-sidney-australia-cierran-famosas-playas-como-bondi-y-coogee-por-24-horas-3564100</t>
+          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/encuesta-final-de-guarumo-y-ecoanalitica-para-segunda-vuelta-presidencial-abelardo-de-la-espriella-52-6-ivan-cepeda-3564095</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 03:33 a. m.</t>
+          <t>13/06/2026 04:30 a. m.</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -692,19 +692,19 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>¿Por qué Cali será la ciudad más vigilada del país el 21 de junio? Las claves del operativo de seguridad que anuncia el Gobierno Nacional</t>
+          <t>¿Placer con Culpa? / El Condimentario</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/cali/por-que-cali-sera-la-ciudad-mas-vigilada-del-pais-el-21-de-junio-las-claves-del-operativo-de-seguridad-que-anuncia-el-gobierno-nacional-3564099</t>
+          <t>https://www.eltiempo.com/cultura/gastronomia/placer-con-culpa-el-condimentario-3564022</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 03:30 a. m.</t>
+          <t>13/06/2026 04:01 a. m.</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -719,19 +719,19 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Casa Landino: un café de lujo colombiano</t>
+          <t>De Roma a las misas en estadios: así ha cambiado la devoción hacia el papa</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/cultura/gastronomia/casa-landino-un-cafe-de-lujo-colombiano-3564012</t>
+          <t>https://www.eltiempo.com/vida/religion/de-roma-a-las-misas-en-estadios-asi-ha-cambiado-la-devocion-hacia-el-papa-3564052</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 03:11 a. m.</t>
+          <t>13/06/2026 03:39 a. m.</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -746,19 +746,19 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Elecciones Colombia 2026: última hora de la segunda vuelta entre Abelardo de la Espriella e Iván Cepeda este 21 de junio</t>
+          <t>Ataque de tiburón en Sídney, Australia: cierran famosas playas como Bondi y Coogee por 24 horas</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/elecciones-colombia-2026-ultima-hora-de-la-segunda-vuelta-entre-abelardo-de-la-espriella-e-ivan-cepeda-este-21-de-junio-3564098</t>
+          <t>https://www.eltiempo.com/mundo/mas-regiones/ataque-de-tiburon-en-sidney-australia-cierran-famosas-playas-como-bondi-y-coogee-por-24-horas-3564100</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 03:01 a. m.</t>
+          <t>13/06/2026 03:33 a. m.</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -773,19 +773,19 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>'La producción petrolera está relegando la transición democrática en Venezuela': analista de la Universidad de Harvard</t>
+          <t>¿Por qué Cali será la ciudad más vigilada del país el 21 de junio? Las claves del operativo de seguridad que anuncia el Gobierno Nacional</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/venezuela/la-produccion-petrolera-esta-relegando-la-transicion-democratica-en-venezuela-analista-de-la-universidad-de-harvard-3564038</t>
+          <t>https://www.eltiempo.com/colombia/cali/por-que-cali-sera-la-ciudad-mas-vigilada-del-pais-el-21-de-junio-las-claves-del-operativo-de-seguridad-que-anuncia-el-gobierno-nacional-3564099</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 02:30 a. m.</t>
+          <t>13/06/2026 03:30 a. m.</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -800,19 +800,19 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>‘Eternos’, el disco que David Bisbal esperó diez años para grabar | Entrevista</t>
+          <t>Casa Landino: un café de lujo colombiano</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/cultura/musica-y-libros/eternos-el-disco-que-david-bisbal-espero-diez-anos-para-grabar-entrevista-3563765</t>
+          <t>https://www.eltiempo.com/cultura/gastronomia/casa-landino-un-cafe-de-lujo-colombiano-3564012</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 02:10 a. m.</t>
+          <t>13/06/2026 03:11 a. m.</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -827,19 +827,19 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Asambleas y circulares por WhatsApp: claves para evitar vacíos legales y financieros en su conjunto</t>
+          <t>Elecciones Colombia 2026: última hora de la segunda vuelta entre Abelardo de la Espriella e Iván Cepeda este 21 de junio</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/economia/finanzas-personales/asambleas-y-circulares-por-whatsapp-claves-para-evitar-vacios-legales-y-financieros-en-su-conjunto-3564048</t>
+          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/elecciones-colombia-2026-ultima-hora-de-la-segunda-vuelta-entre-abelardo-de-la-espriella-e-ivan-cepeda-este-21-de-junio-3564098</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 02:05 a. m.</t>
+          <t>13/06/2026 03:01 a. m.</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -854,19 +854,19 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Irán afirma que el acuerdo con Estados Unidos se podría firmar en los 'próximos días'</t>
+          <t>'La producción petrolera está relegando la transición democrática en Venezuela': analista de la Universidad de Harvard</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/medio-oriente/iran-afirma-que-el-acuerdo-con-estados-unidos-se-podria-firmar-en-los-proximos-dias-3564097</t>
+          <t>https://www.eltiempo.com/mundo/venezuela/la-produccion-petrolera-esta-relegando-la-transicion-democratica-en-venezuela-analista-de-la-universidad-de-harvard-3564038</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 12:40 a. m.</t>
+          <t>13/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -881,19 +881,19 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Mundial 2026: roban las botas y los balones de la selección inglesa antes de su llegada a Kansas City</t>
+          <t>‘Eternos’, el disco que David Bisbal esperó diez años para grabar | Entrevista</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/mundial-2026-estados-unidos-gano-4-1-contra-paraguay-en-los-angeles-california-3564096</t>
+          <t>https://www.eltiempo.com/cultura/musica-y-libros/eternos-el-disco-que-david-bisbal-espero-diez-anos-para-grabar-entrevista-3563765</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 11:53 p. m.</t>
+          <t>13/06/2026 02:10 a. m.</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -908,19 +908,19 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Endrick, la joven estrella que va por la gloria en el Mundial: 'Quiero volver con Brasil como campeón’</t>
+          <t>Asambleas y circulares por WhatsApp: claves para evitar vacíos legales y financieros en su conjunto</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/endrick-la-joven-estrella-que-va-por-la-gloria-en-el-mundial-quiero-volver-con-brasil-como-campeon-3564094</t>
+          <t>https://www.eltiempo.com/economia/finanzas-personales/asambleas-y-circulares-por-whatsapp-claves-para-evitar-vacios-legales-y-financieros-en-su-conjunto-3564048</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 11:48 p. m.</t>
+          <t>13/06/2026 02:05 a. m.</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -935,19 +935,19 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>¿Hora de preocuparse por el '9' de la Selección Colombia? Así están las opciones antes del debut contra Uzbekistán</t>
+          <t>Irán afirma que el acuerdo con Estados Unidos se podría firmar en los 'próximos días'</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/hora-de-preocuparse-por-el-9-de-la-seleccion-colombia-asi-estan-las-opciones-antes-del-debut-contra-uzbekistan-3564093</t>
+          <t>https://www.eltiempo.com/mundo/medio-oriente/iran-afirma-que-el-acuerdo-con-estados-unidos-se-podria-firmar-en-los-proximos-dias-3564097</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 11:29 p. m.</t>
+          <t>13/06/2026 12:40 a. m.</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -962,19 +962,19 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Videos de la balacera y sicariato cerca de estación de TransMilenio en Bogotá que dejó dos muertos y un herido: así escaparon los responsables</t>
+          <t>Mundial 2026: roban las botas y los balones de la selección inglesa antes de su llegada a Kansas City</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/bogota/videos-de-la-balacera-y-sicariato-cerca-de-estacion-de-transmilenio-en-bogota-que-dejo-dos-muertos-y-un-herido-asi-escaparon-los-responsables-3564092</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/mundial-2026-estados-unidos-gano-4-1-contra-paraguay-en-los-angeles-california-3564096</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 11:28 p. m.</t>
+          <t>12/06/2026 11:53 p. m.</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -989,19 +989,19 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Amor, gratitud y buena onda: la consigna de un joven llamado Martín Fonseca</t>
+          <t>Endrick, la joven estrella que va por la gloria en el Mundial: 'Quiero volver con Brasil como campeón’</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/vida/tendencias/amor-gratitud-y-buena-onda-la-consigna-de-un-joven-llamado-martin-fonseca-3564008</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/endrick-la-joven-estrella-que-va-por-la-gloria-en-el-mundial-quiero-volver-con-brasil-como-campeon-3564094</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 11:15 p. m.</t>
+          <t>12/06/2026 11:48 p. m.</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1016,19 +1016,19 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Sobreviviente entrega detalles del dramático accidente marítimo en San Andrés que dejó a madre e hija fallecidas: 'Ahí supe que también estaba muerta'</t>
+          <t>¿Hora de preocuparse por el '9' de la Selección Colombia? Así están las opciones antes del debut contra Uzbekistán</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/otras-ciudades/sobreviviente-entrega-detalles-del-dramatico-accidente-maritimo-en-san-andres-que-dejo-a-madre-e-hija-fallecidas-ahi-supe-que-tambien-estaba-muerta-3564091</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/hora-de-preocuparse-por-el-9-de-la-seleccion-colombia-asi-estan-las-opciones-antes-del-debut-contra-uzbekistan-3564093</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 11:04 p. m.</t>
+          <t>12/06/2026 11:29 p. m.</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
@@ -1043,12 +1043,12 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Colombia Mayor suspenderá los pagos de sus subsidios por tres días: así será el 'blindaje electoral' de cara a la segunda vuelta presidencial</t>
+          <t>Videos de la balacera y sicariato cerca de estación de TransMilenio en Bogotá que dejó dos muertos y un herido: así escaparon los responsables</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/economia/finanzas-personales/colombia-mayor-suspendera-los-pagos-de-sus-subsidios-por-tres-dias-asi-sera-el-blindaje-electoral-de-cara-a-la-segunda-vuelta-presidencial-3563950</t>
+          <t>https://www.eltiempo.com/bogota/videos-de-la-balacera-y-sicariato-cerca-de-estacion-de-transmilenio-en-bogota-que-dejo-dos-muertos-y-un-herido-asi-escaparon-los-responsables-3564092</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 10:52 p. m.</t>
+          <t>13/06/2026 06:22 a. m.</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -1097,19 +1097,19 @@
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>CRC negó alocución presidencial de Petro al no encontrar razones de urgencia y excepcionalidad</t>
+          <t>Israel bombardea el sur de Líbano tras emitir llamado de evacuación</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/13/crc-nego-alocucion-presidencial-de-petro-al-no-encontrar-razones-de-urgencia-y-excepcionalidad/</t>
+          <t>https://caracol.com.co/2026/06/13/israel-bombardea-el-sur-de-libano-tras-emitir-llamado-de-evacuacion/</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 10:51 p. m.</t>
+          <t>13/06/2026 06:19 a. m.</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1124,19 +1124,19 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Gobierno de Venezuela confirma que muerte de alias ‘Niño Guerrero’ fue en el sureste del país</t>
+          <t>Gobierno chileno califica de “golpe relevante” la muerte del líder del Tren de Aragua</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/13/gobierno-de-venezuela-confirma-que-muerte-de-alias-nino-guerrero-fue-en-el-sureste-del-pais/</t>
+          <t>https://caracol.com.co/2026/06/13/gobierno-chileno-califica-de-golpe-relevante-la-muerte-del-lider-del-tren-de-aragua/</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 10:03 p. m.</t>
+          <t>12/06/2026 10:52 p. m.</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
@@ -1151,19 +1151,19 @@
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Estados Unidos aplasta a Paraguay y arranca el Mundial con una contundente victoria</t>
+          <t>CRC negó alocución presidencial de Petro al no encontrar razones de urgencia y excepcionalidad</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/12/en-vivo-esados-unidos-vs-paraguay-siga-el-minuto-a-minuto-y-la-transmision-del-partido/</t>
+          <t>https://caracol.com.co/2026/06/13/crc-nego-alocucion-presidencial-de-petro-al-no-encontrar-razones-de-urgencia-y-excepcionalidad/</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 09:48 p. m.</t>
+          <t>12/06/2026 10:51 p. m.</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1178,19 +1178,19 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>VIDEO: Así fue el ataque militar de EEUU que dio de baja a ‘Niño Guerrero’, jefe del Tren de Aragua</t>
+          <t>Gobierno de Venezuela confirma que muerte de alias ‘Niño Guerrero’ fue en el sureste del país</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/13/video-asi-fue-el-ataque-militar-de-eeuu-que-dio-de-baja-a-nino-guerrero-jefe-del-tren-de-aragua/</t>
+          <t>https://caracol.com.co/2026/06/13/gobierno-de-venezuela-confirma-que-muerte-de-alias-nino-guerrero-fue-en-el-sureste-del-pais/</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 09:01 p. m.</t>
+          <t>12/06/2026 10:03 p. m.</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -1205,19 +1205,19 @@
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>Iván Cepeda publicó nuevo programa de gobierno 2026-2030: las “tres revoluciones” que propone</t>
+          <t>Estados Unidos aplasta a Paraguay y arranca el Mundial con una contundente victoria</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/13/ivan-cepeda-publico-nuevo-programa-de-gobierno-2026-2030-las-tres-revoluciones-que-propone/</t>
+          <t>https://caracol.com.co/2026/06/12/en-vivo-esados-unidos-vs-paraguay-siga-el-minuto-a-minuto-y-la-transmision-del-partido/</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 09:01 p. m.</t>
+          <t>12/06/2026 09:48 p. m.</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1232,19 +1232,19 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Rh nulo el tipo de sangre más raro del mundo: ¿Cuál es la mutación que lo provoca?</t>
+          <t>VIDEO: Así fue el ataque militar de EEUU que dio de baja a ‘Niño Guerrero’, jefe del Tren de Aragua</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/13/rh-nulo-el-tipo-de-sangre-mas-raro-del-mundo-cual-es-la-mutacion-que-lo-provoca/</t>
+          <t>https://caracol.com.co/2026/06/13/video-asi-fue-el-ataque-militar-de-eeuu-que-dio-de-baja-a-nino-guerrero-jefe-del-tren-de-aragua/</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 08:27 p. m.</t>
+          <t>12/06/2026 09:01 p. m.</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -1259,19 +1259,19 @@
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>Trump asegura que fuerzas estadounidenses dieron de baja a ‘Niño Guerrero’, jefe del Tren de Aragua</t>
+          <t>Iván Cepeda publicó nuevo programa de gobierno 2026-2030: las “tres revoluciones” que propone</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/13/trump-asegura-que-fuerzas-estadounidenses-dieron-de-baja-a-nino-guerrero-jefe-del-tren-de-aragua/</t>
+          <t>https://caracol.com.co/2026/06/13/ivan-cepeda-publico-nuevo-programa-de-gobierno-2026-2030-las-tres-revoluciones-que-propone/</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 07:40 p. m.</t>
+          <t>12/06/2026 09:01 p. m.</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1286,19 +1286,19 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Alcalde de Pasto demandará penalmente a la ministra de Transporte y su equipo</t>
+          <t>Rh nulo el tipo de sangre más raro del mundo: ¿Cuál es la mutación que lo provoca?</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/13/alcalde-de-pasto-demandara-penalmente-a-la-ministra-de-transporte-y-su-equipo/</t>
+          <t>https://caracol.com.co/2026/06/13/rh-nulo-el-tipo-de-sangre-mas-raro-del-mundo-cual-es-la-mutacion-que-lo-provoca/</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 07:12 p. m.</t>
+          <t>12/06/2026 08:27 p. m.</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -1313,19 +1313,19 @@
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>SuperSalud exigió a la Nueva EPS garantizar entrega de medicamentos en Nariño</t>
+          <t>Trump asegura que fuerzas estadounidenses dieron de baja a ‘Niño Guerrero’, jefe del Tren de Aragua</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/13/supersalud-exigio-a-la-nueva-eps-garantizar-entrega-de-medicamentos-en-narino/</t>
+          <t>https://caracol.com.co/2026/06/13/trump-asegura-que-fuerzas-estadounidenses-dieron-de-baja-a-nino-guerrero-jefe-del-tren-de-aragua/</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 06:59 p. m.</t>
+          <t>12/06/2026 07:40 p. m.</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1340,19 +1340,19 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>La ANDI advierte que la reforma tributaria para el 2027 será la mas grande de la historia</t>
+          <t>Alcalde de Pasto demandará penalmente a la ministra de Transporte y su equipo</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/12/la-andi-advierte-que-reforma-tributaria-para-el-2027-sera-la-mas-grande-de-la-historia/</t>
+          <t>https://caracol.com.co/2026/06/13/alcalde-de-pasto-demandara-penalmente-a-la-ministra-de-transporte-y-su-equipo/</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 06:59 p. m.</t>
+          <t>12/06/2026 07:12 p. m.</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
@@ -1367,19 +1367,19 @@
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>La CREG inspeccionó infraestructura del Puerto de Tumaco para abastecimiento de combustibles</t>
+          <t>SuperSalud exigió a la Nueva EPS garantizar entrega de medicamentos en Nariño</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/12/la-creg-inspecciono-infraestructura-del-puerto-de-tumaco-para-garantizar-abastecimiento-de-combustib/</t>
+          <t>https://caracol.com.co/2026/06/13/supersalud-exigio-a-la-nueva-eps-garantizar-entrega-de-medicamentos-en-narino/</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 06:47 p. m.</t>
+          <t>12/06/2026 06:59 p. m.</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1394,19 +1394,19 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Iván Cepeda propone que Colombia sea sede de una Copa Mundial de Fútbol</t>
+          <t>La ANDI advierte que la reforma tributaria para el 2027 será la mas grande de la historia</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/12/ivan-cepeda-propone-que-colombia-sea-sede-de-una-copa-mundial-de-futbol/</t>
+          <t>https://caracol.com.co/2026/06/12/la-andi-advierte-que-reforma-tributaria-para-el-2027-sera-la-mas-grande-de-la-historia/</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 06:28 p. m.</t>
+          <t>12/06/2026 06:59 p. m.</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
@@ -1421,19 +1421,19 @@
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>Siguen conversaciones entre Gobierno y cafeteros para definir futuro del contrato del Fondo del Café</t>
+          <t>La CREG inspeccionó infraestructura del Puerto de Tumaco para abastecimiento de combustibles</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/12/siguen-conversaciones-entre-gobierno-y-cafeteros-para-definir-futuro-del-contrato-del-fondo-del-cafe/</t>
+          <t>https://caracol.com.co/2026/06/12/la-creg-inspecciono-infraestructura-del-puerto-de-tumaco-para-garantizar-abastecimiento-de-combustib/</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 06:22 p. m.</t>
+          <t>12/06/2026 06:47 p. m.</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1448,19 +1448,19 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>UNAB marca un hito en Investigación Criminal y Ciencias Forenses con acreditación de alta calidad</t>
+          <t>Iván Cepeda propone que Colombia sea sede de una Copa Mundial de Fútbol</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/12/unab-marca-un-hito-en-investigacion-criminal-y-ciencias-forenses-con-acreditacion-de-alta-calidad/</t>
+          <t>https://caracol.com.co/2026/06/12/ivan-cepeda-propone-que-colombia-sea-sede-de-una-copa-mundial-de-futbol/</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 06:16 p. m.</t>
+          <t>12/06/2026 06:28 p. m.</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
@@ -1475,19 +1475,19 @@
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>Sincelejo la ciudad de Colombia donde menos roban a la gente</t>
+          <t>Siguen conversaciones entre Gobierno y cafeteros para definir futuro del contrato del Fondo del Café</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/12/sincelejo-la-ciudad-de-colombia-donde-menos-roban-a-la-gente/</t>
+          <t>https://caracol.com.co/2026/06/12/siguen-conversaciones-entre-gobierno-y-cafeteros-para-definir-futuro-del-contrato-del-fondo-del-cafe/</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 06:01 p. m.</t>
+          <t>12/06/2026 06:22 p. m.</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -1502,19 +1502,19 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Guerra en Ucrania ya ha durado más que la Primera Guerra Mundial</t>
+          <t>UNAB marca un hito en Investigación Criminal y Ciencias Forenses con acreditación de alta calidad</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/12/guerra-en-ucrania-ya-ha-durado-mas-que-la-primera-guerra-mundial/</t>
+          <t>https://caracol.com.co/2026/06/12/unab-marca-un-hito-en-investigacion-criminal-y-ciencias-forenses-con-acreditacion-de-alta-calidad/</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 05:55 p. m.</t>
+          <t>12/06/2026 06:16 p. m.</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
@@ -1529,19 +1529,19 @@
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>Así se vive la Feria Nacional e Internacional de la Ganadería en Córdoba: programación y más</t>
+          <t>Sincelejo la ciudad de Colombia donde menos roban a la gente</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/12/asi-se-vive-la-feria-nacional-e-internacional-de-la-ganaderia-en-cordoba-programacion-y-mas/</t>
+          <t>https://caracol.com.co/2026/06/12/sincelejo-la-ciudad-de-colombia-donde-menos-roban-a-la-gente/</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 05:46 p. m.</t>
+          <t>12/06/2026 06:01 p. m.</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -1556,19 +1556,19 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>El Decameron Galeón en Santa Marta: conozca el espacio natural entre playas y montañas</t>
+          <t>Guerra en Ucrania ya ha durado más que la Primera Guerra Mundial</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/12/el-decameron-galeon-en-santa-marta-conozca-el-espacio-natural-entre-playas-y-montanas/</t>
+          <t>https://caracol.com.co/2026/06/12/guerra-en-ucrania-ya-ha-durado-mas-que-la-primera-guerra-mundial/</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>12/06/2026 05:41 p. m.</t>
+          <t>12/06/2026 05:55 p. m.</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
@@ -1583,12 +1583,12 @@
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>San Andrés, de los destinos turísticos más visitados de Colombia: 5 hoteles icónicos ‘All inclusive’</t>
+          <t>Así se vive la Feria Nacional e Internacional de la Ganadería en Córdoba: programación y más</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/12/san-andres-de-los-destinos-turisticos-mas-visitados-de-colombia-5-hoteles-iconicos-all-inclusive/</t>
+          <t>https://caracol.com.co/2026/06/12/asi-se-vive-la-feria-nacional-e-internacional-de-la-ganaderia-en-cordoba-programacion-y-mas/</t>
         </is>
       </c>
     </row>
@@ -2050,7 +2050,7 @@
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 05:52 a. m.</t>
+          <t>13/06/2026 06:38 a. m.</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
@@ -2060,24 +2060,24 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>Hidroavión promete vuelo de 17 minutos entre Medellín y embalse de Guatapé: ¿cómo operaría?</t>
+          <t>Última hora de la guerra de Estados Unidos e Israel contra Irán, en directo | Israel emite una orden de evacuación para 20 localidades en el sur de Líbano y reanuda los bombardeos</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/antioquia/hidroavion-medellin-guatape-asi-operaria-FF37678739</t>
+          <t>https://elpais.com/internacional/2026-06-13/ultima-hora-de-la-guerra-de-estados-unidos-e-israel-contra-iran-en-directo.html</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 12:52 a. m.</t>
+          <t>13/06/2026 06:21 a. m.</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -2087,24 +2087,24 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Comiendo por Colombia: los 11 magníficos, segunda parte</t>
+          <t>Mañueco mantiene a buena parte de sus consejeros, cambia de área a su polémico titular de Medio Ambiente y Vox elige perfiles técnicos</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/cultura/gastronomia/platos-de-la-gastronomia-colombiana-alvaro-molina-sancocho-lechona-MK37682169</t>
+          <t>https://elpais.com/espana/elecciones-castilla-y-leon/2026-06-13/manueco-mantiene-a-buena-parte-de-sus-consejeros-cambia-de-area-a-su-polemico-titular-de-medio-ambiente-y-vox-elige-perfiles-tecnicos.html</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 12:52 a. m.</t>
+          <t>13/06/2026 06:07 a. m.</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
@@ -2114,22 +2114,26 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>“El nombramiento de Quintero nos hizo perder cientos de votos en Antioquia”: Carlos Carrillo</t>
+          <t>Ione Belarra anuncia que encabezará la candidatura de Podemos a la Comunidad de Madrid</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/carlos-carrillo-habla-de-daniel-quintero-gobierno-gustavo-petro-y-campana-ivan-cepeda-AK37681472</t>
+          <t>https://elpais.com/espana/2026-06-13/ione-belarra-anuncia-que-encabezara-la-candidatura-de-podemos-a-la-comunidad-de-madrid.html</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="inlineStr"/>
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>13/06/2026 05:50 a. m.</t>
+        </is>
+      </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2137,22 +2141,26 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Dos modelos de país muy distintos: ¿quién gobernaría mejor a Colombia entre De la Espriella y Cepeda?</t>
+          <t>Mundial 2026, ultimas noticias en directo | EEUU vence a Paraguay y Brasil y Marruecos preparan el primer choque entre selecciones candidatas</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/elecciones-2026/abelardo-cepeda-modelos-pais-distintos-gobernar-colombia-AK37682112</t>
+          <t>https://elpais.com/deportes/mundial-futbol/2026-06-13/resumen-y-ultimas-noticias-de-la-copa-mundial-de-futbol.html</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="5" t="inlineStr"/>
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>13/06/2026 05:27 a. m.</t>
+        </is>
+      </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2160,22 +2168,26 @@
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
-          <t>Buga y Bogotá, las plazas donde Abelardo y Cepeda libran su último pulso</t>
+          <t>El Kennedy Center cumple con la orden judicial de retirar el nombre de Donald Trump de su fachada</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/elecciones-2026/elecciones-2026-abelardo-cepeda-buga-bogota-pulso-campana-NK37681729</t>
+          <t>https://elpais.com/internacional/2026-06-13/el-kennedy-center-cumple-con-la-orden-judicial-de-retirar-el-nombre-de-donald-trump-de-su-fachada.html</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="inlineStr"/>
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>13/06/2026 05:17 a. m.</t>
+        </is>
+      </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2183,22 +2195,26 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Trump dice que Estados Unidos mató al ‘Niño Guerrero’, jefe del Tren de Aragua</t>
+          <t>Rodalies comienza el fin de semana con dos incidencias semana en la R3 y la R 11</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/internacional/estados-unidos-mato-nino-guerrero-jefe-del-tren-de-aragua-venezuela-KF37679407</t>
+          <t>https://elpais.com/espana/catalunya/2026-06-13/rodalies-comienza-el-fin-de-semana-con-dos-incidencias-semana-en-la-r3-y-la-r-11.html</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="5" t="inlineStr"/>
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>13/06/2026 04:34 a. m.</t>
+        </is>
+      </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2206,22 +2222,26 @@
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>¿Por qué le está fallando la estrategia a Cepeda?</t>
+          <t>Anthropic suspende el acceso a sus modelos más avanzados de inteligencia artificial por el veto de EE UU a los extranjeros</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/multimedia/videos/por-que-le-esta-fallando-la-estrategia-a-cepeda-JF37671787</t>
+          <t>https://elpais.com/economia/2026-06-13/anthropic-suspende-el-acceso-a-sus-modelos-mas-avanzados-de-inteligencia-artificial-por-el-veto-de-ee-uu-a-los-extranjeros.html</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="inlineStr"/>
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>13/06/2026 04:21 a. m.</t>
+        </is>
+      </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2229,22 +2249,26 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Contratista de Coljuegos pagó campaña del hijo de director al Congreso: es del Pacto</t>
+          <t>Trece detenidos en Barcelona en una operación policial contra el uso de armas de fuego</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/politica/contratista-coljuegos-pago-campana-hijo-director-congreso-pacto-historico-GF37670688</t>
+          <t>https://elpais.com/espana/catalunya/2026-06-11/los-mossos-atribuyen-al-crimen-organizado-los-ultimos-seis-muertos-a-tiros-en-cataluna.html</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="5" t="inlineStr"/>
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>13/06/2026 02:28 a. m.</t>
+        </is>
+      </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2252,22 +2276,26 @@
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>Precio del dólar se desploma a $3.475, nivel que no se veía desde el 2021</t>
+          <t>Sarral, el Huntington y la Copa del Mundo</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/negocios/dolar-precio-hoy-12-junio-colombia-cierre-desplome-PH37659215</t>
+          <t>https://elpais.com/espana/catalunya/2026-06-13/sarral-el-huntington-y-la-copa-del-mundo.html</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="inlineStr"/>
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>13/06/2026 02:03 a. m.</t>
+        </is>
+      </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2275,22 +2303,26 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>Es oficial: Atlético Nacional sacó a Diego Arias y ya piensa en su reemplazo</t>
+          <t>Lotería Nacional: sorteo del sábado 13 de junio</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/deportes/futbol/atletico-nacional-oficializo-salida-tecnico-diego-arias-busca-reemplazo-KE37663801</t>
+          <t>https://elpais.com/sorteos/2026-06-13/loteria-nacional-sorteo-del-sabado-13-de-junio.html</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="5" t="inlineStr"/>
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t>13/06/2026 12:39 a. m.</t>
+        </is>
+      </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2298,22 +2330,26 @@
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>Operativo destapa helicóptero con pasado oscuro y motor Rolls-Royce</t>
+          <t>Un tiro en un pie: salir del CIADI le puede salir caro a Colombia</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/ejercito-incauta-helicoptero-de-la-mafia-NG33717192</t>
+          <t>https://elpais.com/america-colombia/2026-06-13/un-tiro-en-un-pie-salir-del-ciadi-le-puede-salir-caro-a-colombia.html</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="inlineStr"/>
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>13/06/2026 12:08 a. m.</t>
+        </is>
+      </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2321,22 +2357,26 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>¿Va a viajar este puente? Así estará la movilidad en las vías de Antioquia y Medellín</t>
+          <t>Niño Guerrero, de una barriada de Venezuela a conquistar América Latina con el Tren de Aragua</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/antioquia/puente-festivo-cierres-restricciones-viales-antioquia-medellin-FK37681411</t>
+          <t>https://elpais.com/america/2026-06-13/nino-guerrero-de-una-barriada-de-venezuela-a-conquistar-america-latina-con-el-tren-de-aragua.html</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="5" t="inlineStr"/>
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t>13/06/2026 12:05 a. m.</t>
+        </is>
+      </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2344,22 +2384,26 @@
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D71" s="6" t="inlineStr">
         <is>
-          <t>¿El fin de la guerra? Irán anunció que el acuerdo de paz con EE. UU. está a solo días de firmarse</t>
+          <t>Trump alaba al Tigre y reta a la izquierda, mientras Cepeda acude a la CPI</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/internacional/iran-anuncia-acuerdo-paz-ee-uu-dias-firmar-fin-guerra-DF37675314</t>
+          <t>https://elpais.com/america-colombia/elecciones-presidenciales/2026-06-13/trump-alaba-al-tigre-y-reta-a-la-izquierda-mientras-cepeda-acude-a-la-cpi.html</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="inlineStr"/>
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>13/06/2026 12:01 a. m.</t>
+        </is>
+      </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2367,22 +2411,26 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>Julieta Venegas responde a polémica por “La niña futbolista”: ¿por qué la canción mundialista fue tan criticada?</t>
+          <t>Los creyentes progresistas que le disputan el voto religioso a Abelardo de la Espriella</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/cultura/musica/julieta-venegas-responde-polemica-nina-futbolista-cancion-criticas-HF37675002</t>
+          <t>https://elpais.com/america-colombia/2026-06-13/los-creyentes-progresistas-que-le-disputan-el-voto-religioso-a-abelardo-de-la-espriella.html</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="5" t="inlineStr"/>
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>13/06/2026 12:00 a. m.</t>
+        </is>
+      </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2390,22 +2438,26 @@
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D73" s="6" t="inlineStr">
         <is>
-          <t>Modelo webcam se fotografió semidesnuda en una iglesia de Guarne: ¿podría enfrentar sanciones?</t>
+          <t>Vinicius, tras la estela de Garrincha en Brasil</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/antioquia/modelo-webcam-iglesia-guarne-fotos-KF37676963</t>
+          <t>https://elpais.com/deportes/mundial-futbol/2026-06-13/vinicius-tras-la-estela-de-garrincha-en-brasil.html</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="inlineStr"/>
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>13/06/2026 12:00 a. m.</t>
+        </is>
+      </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2413,22 +2465,26 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>Luis7Lunes: rapero a tiempo completo</t>
+          <t>Pickleball: por qué todo el mundo está jugando (y qué necesitas para empezar)</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/cultura/luis7lunes-nuevo-disco-v-sabor-rap-afterclass-FF37675415</t>
+          <t>https://elpais.com/hemeroteca/2026-06-13/</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="5" t="inlineStr"/>
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t>12/06/2026 11:55 p. m.</t>
+        </is>
+      </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2436,22 +2492,26 @@
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr">
         <is>
-          <t>Colombia redujo su desigualdad en 2025; el nivel más bajo de los últimos seis años</t>
+          <t>Abelardo de la Espriella matiza sus propuestas ‘milagro’</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/negocios/desigualdad-colombia-cae-2025-nivel-bajo-dane-BF37675510</t>
+          <t>https://elpais.com/america-colombia/elecciones-presidenciales/2026-06-13/abelardo-de-la-espriella-matiza-sus-propuestas-milagro.html</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="inlineStr"/>
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>12/06/2026 11:52 p. m.</t>
+        </is>
+      </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2459,22 +2519,26 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>Cristiano Ronaldo respondió a las críticas antes del debut: “Estoy bien, ¿no has visto los partidos?”</t>
+          <t>Sin constituyente y sin paz total: Iván Cepeda publica un plan de gobierno más moderado</t>
         </is>
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/deportes/futbol/cristiano-ronaldo-responde-criticas-antes-debut-mundial-2026-portugal-IF37670945</t>
+          <t>https://elpais.com/america-colombia/elecciones-presidenciales/2026-06-13/sin-constituyente-y-sin-paz-total-ivan-cepeda-publica-un-plan-de-gobierno-mas-moderado.html</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="5" t="inlineStr"/>
+      <c r="A77" s="5" t="inlineStr">
+        <is>
+          <t>12/06/2026 10:45 p. m.</t>
+        </is>
+      </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2482,22 +2546,26 @@
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D77" s="6" t="inlineStr">
         <is>
-          <t>Colombia deberá pagar $83,9 billones en intereses de su deuda pública en 2027</t>
+          <t>¿Puedes batir nuestra predicción? Juega a pronosticar el Mundial</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/negocios/intereses-deuda-publica-colombia-2027-marco-fiscal-minhacienda-DF37674142</t>
+          <t>https://elpais.com/deportes/mundial-futbol/2026-06-13/puedes-batir-nuestra-prediccion-juega-a-pronosticar-el-mundial.html</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="inlineStr"/>
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>12/06/2026 10:30 p. m.</t>
+        </is>
+      </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2505,22 +2573,26 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>Elecciones en Perú: Sánchez se resiste a reconocer los resultados y propone a Fujimori revisar “todos los votos”</t>
+          <t>Viviendas, sanidad y otros servicios: los suizos se preguntan hasta dónde pueden crecer</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/internacional/roberto-sanchez-no-acepta-resultados-fujimori-elecciones-segunda-vuelta-peru-EE37660576</t>
+          <t>https://elpais.com/internacional/2026-06-13/viviendas-sanidad-y-otros-servicios-los-suizos-se-preguntan-hasta-donde-pueden-crecer.html</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="5" t="inlineStr"/>
+      <c r="A79" s="5" t="inlineStr">
+        <is>
+          <t>12/06/2026 10:30 p. m.</t>
+        </is>
+      </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2528,22 +2600,26 @@
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
         <is>
-          <t>Bombardeo contra el Clan del Golfo en zona rural de Chocó dejó al menos 9 criminales muertos</t>
+          <t>Los excursionistas que auxiliaron a Jonathan Andic, el quebradero de cabeza de los Mossos</t>
         </is>
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/bombardeo-contra-clan-golfo-choco-muertos-nuqui-OE37660680</t>
+          <t>https://elpais.com/espana/catalunya/2026-06-13/los-excursionistas-que-auxiliaron-a-jonathan-andic-el-quebradero-de-cabeza-de-los-mossos.html</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="inlineStr"/>
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>12/06/2026 10:30 p. m.</t>
+        </is>
+      </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2551,22 +2627,26 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>¿Es posible que le dé un ataque al corazón por la emoción de un gol?</t>
+          <t>La investigación a Zapatero por posible delito fiscal con las joyas limita cualquier regularización ante Hacienda</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/tendencias/mundial-2026-fifa-ataque-corazon-paro-cardiaco-salud-gol-ME37668774</t>
+          <t>https://elpais.com/economia/2026-06-13/la-investigacion-a-zapatero-por-posible-delito-fiscal-con-las-joyas-limita-cualquier-regularizacion-ante-hacienda.html</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="5" t="inlineStr"/>
+      <c r="A81" s="5" t="inlineStr">
+        <is>
+          <t>12/06/2026 10:30 p. m.</t>
+        </is>
+      </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2574,22 +2654,26 @@
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D81" s="6" t="inlineStr">
         <is>
-          <t>Encontraron un cadáver frente al estadio donde entrena la Selección de Irán en México</t>
+          <t>¿Está quemando Telecinco ‘Supervivientes’ y ‘La isla de las tentaciones’? La respuesta de los datos de audiencia</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/internacional/cadaver-frente-estadio-seleccion-iran-en-mexico-mundial-2026-FF37672124</t>
+          <t>https://elpais.com/television/2026-06-13/esta-quemando-telecinco-supervivientes-y-la-isla-de-las-tentaciones-la-respuesta-de-los-datos-de-audiencia.html</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="inlineStr"/>
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>12/06/2026 10:30 p. m.</t>
+        </is>
+      </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2597,22 +2681,26 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>Prográmese: Catar se enfrenta a Suiza este sábado en Santa Clara, por el Grupo B del Mundial</t>
+          <t>Los primeros estudiantes del grado de Matemáticas y Filosofía, único en España: “Hay que aprender a utilizar la IA con ética”</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/mundial-2026/catar-partido-suiza-sabado-santa-clara-grupo-b-del-mundial-KE37667850</t>
+          <t>https://elpais.com/educacion/2026-06-13/los-primeros-estudiantes-del-grado-de-matematicas-y-filosofia-unico-en-espana-hay-que-aprender-a-utilizar-la-ia-con-etica.html</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="5" t="inlineStr"/>
+      <c r="A83" s="5" t="inlineStr">
+        <is>
+          <t>12/06/2026 10:30 p. m.</t>
+        </is>
+      </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2620,22 +2708,26 @@
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D83" s="6" t="inlineStr">
         <is>
-          <t>Cerraron motel en Medellín señalado por la Fiscalía de permitir la explotación de niñas</t>
+          <t>El paso al frente de Marruecos con su nuevo seleccionador Mohamed Ouahbi</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/medellin/fiscalia-cierra-motel-centro-medellin-prostitucion-menores-AF37670617</t>
+          <t>https://elpais.com/deportes/mundial-futbol/2026-06-13/el-paso-al-frente-de-marruecos-con-su-nuevo-seleccionador-mohamed-ouahbi.html</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="inlineStr"/>
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>12/06/2026 10:30 p. m.</t>
+        </is>
+      </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2643,22 +2735,26 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>Aprueban la Ley Bartolo: este municipio de Antioquia se convierte en la Capital Mundial de la Mula de Silla</t>
+          <t>El vértigo de viajar solo en verano: “Llevo demasiado tiempo viviendo como si mi vida estuviera en pausa”</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/antioquia/ley-bartolo-burro-capital-mundial-de-la-mula-de-silla-titiribi-antioquia-PE37665785</t>
+          <t>https://elpais.com/estilo-de-vida/2026-06-13/el-vertigo-de-viajar-solo-en-verano-llevo-demasiado-tiempo-viviendo-como-si-mi-vida-estuviera-en-pausa.html</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="5" t="inlineStr"/>
+      <c r="A85" s="5" t="inlineStr">
+        <is>
+          <t>12/06/2026 08:15 p. m.</t>
+        </is>
+      </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2666,22 +2762,26 @@
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D85" s="6" t="inlineStr">
         <is>
-          <t>Pagos con QR y celular se disparan en Colombia: ¿está llegando el fin del efectivo?</t>
+          <t>Trump anuncia que el ejército de Estados Unidos ha matado en Venezuela al Niño Guerrero, líder del Tren de Aragua</t>
         </is>
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/negocios/pagos-qr-celular-colombia-fin-efectivo-bre-b-nequi-CE37661726</t>
+          <t>https://elpais.com/america/2026-06-13/trump-anuncia-que-el-ejercito-de-estados-unidos-ha-matado-al-nino-guerrero-lider-del-tren-de-aragua.html</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="inlineStr"/>
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>12/06/2026 02:45 a. m.</t>
+        </is>
+      </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2689,17 +2789,17 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>Iván Cepeda cerrará su campaña presidencial en la Plaza La Santamaría de Bogotá antes de la segunda vuelta</t>
+          <t>Maxi Iglesias: “Intento seguir mi vida sin hacer mucho caso al ruido que generan mis decisiones”</t>
         </is>
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/elecciones-2026/ivan-cepeda-cerrara-su-campana-presidencial-en-la-plaza-la-santamaria-de-bogota-antes-de-la-segunda-vuelta-OH37657018</t>
+          <t>https://elpais.com/icon/2026-06-12/maxi-iglesias-intento-seguir-mi-vida-sin-hacer-mucho-caso-al-ruido-que-generan-mis-decisiones.html</t>
         </is>
       </c>
     </row>
@@ -2712,17 +2812,17 @@
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D87" s="6" t="inlineStr">
         <is>
-          <t>Disidencias de alias Calarcá obligan a votantes a tomarle foto al tarjetón: la grave denuncia de constreñimiento en Caquetá</t>
+          <t>Predicciones</t>
         </is>
       </c>
       <c r="E87" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/disidencias-farc-fotos-voto-caqueta-HG37640236</t>
+          <t>https://elpais.com/deportes/mundial-futbol/2026-06-11/quien-ganara-el-mundial-asi-arrancan-nuestras-predicciones.html</t>
         </is>
       </c>
     </row>
@@ -2735,24 +2835,24 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>¿Guiño a De la Espriella? Oviedo visitó a Uribe en Rionegro</t>
+          <t>Selecciones</t>
         </is>
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/elecciones-2026/juan-daniel-oviedo-reunion-alvaro-uribe-elecciones-FG37641361</t>
+          <t>https://elpais.com/deportes/mundial-futbol/2026-06-05/todas-las-selecciones-del-mundial-de-estados-unidos-canada-y-mexico.html</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 05:50 a. m.</t>
+          <t>13/06/2026 06:00 a. m.</t>
         </is>
       </c>
       <c r="B89" s="5" t="inlineStr">
@@ -2762,24 +2862,24 @@
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D89" s="6" t="inlineStr">
         <is>
-          <t>Mundial 2026, ultimas noticias en directo | EEUU vence a Paraguay y Brasil y Marruecos preparan el primer choque entre selecciones candidatas</t>
+          <t>Las 8 obras en carpeta para no embotellar a Medellín con el tráfico de las 4G</t>
         </is>
       </c>
       <c r="E89" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/deportes/mundial-futbol/2026-06-13/resumen-y-ultimas-noticias-de-la-copa-mundial-de-futbol.html</t>
+          <t>https://www.elcolombiano.com/medellin/medellin-obras-viales-intercambios-autopistas-4g-GK37680701</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 05:27 a. m.</t>
+          <t>13/06/2026 05:40 a. m.</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -2789,24 +2889,24 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>El Kennedy Center cumple con la orden judicial de retirar el nombre de Donald Trump de su fachada</t>
+          <t>Hidroavión promete vuelo de 17 minutos entre Medellín y embalse de Guatapé: ¿cómo operaría?</t>
         </is>
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/internacional/2026-06-13/el-kennedy-center-cumple-con-la-orden-judicial-de-retirar-el-nombre-de-donald-trump-de-su-fachada.html</t>
+          <t>https://www.elcolombiano.com/antioquia/hidroavion-medellin-guatape-asi-operaria-FF37678739</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 05:17 a. m.</t>
+          <t>13/06/2026 12:40 a. m.</t>
         </is>
       </c>
       <c r="B91" s="5" t="inlineStr">
@@ -2816,24 +2916,24 @@
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D91" s="6" t="inlineStr">
         <is>
-          <t>Rodalies comienza el fin de semana con dos incidencias semana en la R3 y la R 11</t>
+          <t>Comiendo por Colombia: los 11 magníficos, segunda parte</t>
         </is>
       </c>
       <c r="E91" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/espana/catalunya/2026-06-13/rodalies-comienza-el-fin-de-semana-con-dos-incidencias-semana-en-la-r3-y-la-r-11.html</t>
+          <t>https://www.elcolombiano.com/cultura/gastronomia/platos-de-la-gastronomia-colombiana-alvaro-molina-sancocho-lechona-MK37682169</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 04:34 a. m.</t>
+          <t>13/06/2026 12:40 a. m.</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -2843,26 +2943,22 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>Anthropic suspende el acceso a sus modelos más avanzados de inteligencia artificial por el veto de EE UU a los extranjeros</t>
+          <t>“El nombramiento de Quintero nos hizo perder cientos de votos en Antioquia”: Carlos Carrillo</t>
         </is>
       </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/economia/2026-06-13/anthropic-suspende-el-acceso-a-sus-modelos-mas-avanzados-de-inteligencia-artificial-por-el-veto-de-ee-uu-a-los-extranjeros.html</t>
+          <t>https://www.elcolombiano.com/colombia/carlos-carrillo-habla-de-daniel-quintero-gobierno-gustavo-petro-y-campana-ivan-cepeda-AK37681472</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="5" t="inlineStr">
-        <is>
-          <t>13/06/2026 04:21 a. m.</t>
-        </is>
-      </c>
+      <c r="A93" s="5" t="inlineStr"/>
       <c r="B93" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2870,26 +2966,22 @@
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D93" s="6" t="inlineStr">
         <is>
-          <t>Trece detenidos en Barcelona en una operación policial contra el uso de armas de fuego</t>
+          <t>Dos modelos de país muy distintos: ¿quién gobernaría mejor a Colombia entre De la Espriella y Cepeda?</t>
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/espana/catalunya/2026-06-11/los-mossos-atribuyen-al-crimen-organizado-los-ultimos-seis-muertos-a-tiros-en-cataluna.html</t>
+          <t>https://www.elcolombiano.com/especiales/elecciones-2026/abelardo-cepeda-modelos-pais-distintos-gobernar-colombia-AK37682112</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="2" t="inlineStr">
-        <is>
-          <t>13/06/2026 04:06 a. m.</t>
-        </is>
-      </c>
+      <c r="A94" s="2" t="inlineStr"/>
       <c r="B94" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2897,26 +2989,22 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>Última hora de la guerra de Estados Unidos e Israel contra Irán, en directo | Israel emite una orden de evacuación para 20 localidades en el sur de Líbano y reanuda los bombardeos</t>
+          <t>Buga y Bogotá, las plazas donde Abelardo y Cepeda libran su último pulso</t>
         </is>
       </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/internacional/2026-06-13/ultima-hora-de-la-guerra-de-estados-unidos-e-israel-contra-iran-en-directo.html</t>
+          <t>https://www.elcolombiano.com/especiales/elecciones-2026/elecciones-2026-abelardo-cepeda-buga-bogota-pulso-campana-NK37681729</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="5" t="inlineStr">
-        <is>
-          <t>13/06/2026 02:28 a. m.</t>
-        </is>
-      </c>
+      <c r="A95" s="5" t="inlineStr"/>
       <c r="B95" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2924,26 +3012,22 @@
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D95" s="6" t="inlineStr">
         <is>
-          <t>Sarral, el Huntington y la Copa del Mundo</t>
+          <t>Trump dice que Estados Unidos mató al ‘Niño Guerrero’, jefe del Tren de Aragua</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/espana/catalunya/2026-06-13/sarral-el-huntington-y-la-copa-del-mundo.html</t>
+          <t>https://www.elcolombiano.com/internacional/estados-unidos-mato-nino-guerrero-jefe-del-tren-de-aragua-venezuela-KF37679407</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="2" t="inlineStr">
-        <is>
-          <t>13/06/2026 02:03 a. m.</t>
-        </is>
-      </c>
+      <c r="A96" s="2" t="inlineStr"/>
       <c r="B96" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2951,26 +3035,22 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>Lotería Nacional: sorteo del sábado 13 de junio</t>
+          <t>¿Por qué le está fallando la estrategia a Cepeda?</t>
         </is>
       </c>
       <c r="E96" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/sorteos/2026-06-13/loteria-nacional-sorteo-del-sabado-13-de-junio.html</t>
+          <t>https://www.elcolombiano.com/multimedia/videos/por-que-le-esta-fallando-la-estrategia-a-cepeda-JF37671787</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="5" t="inlineStr">
-        <is>
-          <t>13/06/2026 12:39 a. m.</t>
-        </is>
-      </c>
+      <c r="A97" s="5" t="inlineStr"/>
       <c r="B97" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2978,26 +3058,22 @@
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D97" s="6" t="inlineStr">
         <is>
-          <t>Un tiro en un pie: salir del CIADI le puede salir caro a Colombia</t>
+          <t>Contratista de Coljuegos pagó campaña del hijo de director al Congreso: es del Pacto</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/america-colombia/2026-06-13/un-tiro-en-un-pie-salir-del-ciadi-le-puede-salir-caro-a-colombia.html</t>
+          <t>https://www.elcolombiano.com/colombia/politica/contratista-coljuegos-pago-campana-hijo-director-congreso-pacto-historico-GF37670688</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="inlineStr">
-        <is>
-          <t>13/06/2026 12:08 a. m.</t>
-        </is>
-      </c>
+      <c r="A98" s="2" t="inlineStr"/>
       <c r="B98" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3005,26 +3081,22 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>Niño Guerrero, de una barriada de Venezuela a conquistar América Latina con el Tren de Aragua</t>
+          <t>Precio del dólar se desploma a $3.475, nivel que no se veía desde el 2021</t>
         </is>
       </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/america/2026-06-13/nino-guerrero-de-una-barriada-de-venezuela-a-conquistar-america-latina-con-el-tren-de-aragua.html</t>
+          <t>https://www.elcolombiano.com/negocios/dolar-precio-hoy-12-junio-colombia-cierre-desplome-PH37659215</t>
         </is>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="5" t="inlineStr">
-        <is>
-          <t>13/06/2026 12:05 a. m.</t>
-        </is>
-      </c>
+      <c r="A99" s="5" t="inlineStr"/>
       <c r="B99" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3032,26 +3104,22 @@
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D99" s="6" t="inlineStr">
         <is>
-          <t>Trump alaba al Tigre y reta a la izquierda, mientras Cepeda acude a la CPI</t>
+          <t>Operativo destapa helicóptero con pasado oscuro y motor Rolls-Royce</t>
         </is>
       </c>
       <c r="E99" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/america-colombia/elecciones-presidenciales/2026-06-13/trump-alaba-al-tigre-y-reta-a-la-izquierda-mientras-cepeda-acude-a-la-cpi.html</t>
+          <t>https://www.elcolombiano.com/colombia/ejercito-incauta-helicoptero-de-la-mafia-NG33717192</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="inlineStr">
-        <is>
-          <t>13/06/2026 12:01 a. m.</t>
-        </is>
-      </c>
+      <c r="A100" s="2" t="inlineStr"/>
       <c r="B100" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3059,26 +3127,22 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>Los creyentes progresistas que le disputan el voto religioso a Abelardo de la Espriella</t>
+          <t>¿Va a viajar este puente? Así estará la movilidad en las vías de Antioquia y Medellín</t>
         </is>
       </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/america-colombia/2026-06-13/los-creyentes-progresistas-que-le-disputan-el-voto-religioso-a-abelardo-de-la-espriella.html</t>
+          <t>https://www.elcolombiano.com/antioquia/puente-festivo-cierres-restricciones-viales-antioquia-medellin-FK37681411</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="5" t="inlineStr">
-        <is>
-          <t>13/06/2026 12:00 a. m.</t>
-        </is>
-      </c>
+      <c r="A101" s="5" t="inlineStr"/>
       <c r="B101" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3086,26 +3150,22 @@
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D101" s="6" t="inlineStr">
         <is>
-          <t>Vinicius, tras la estela de Garrincha en Brasil</t>
+          <t>¿El fin de la guerra? Irán anunció que el acuerdo de paz con EE. UU. está a solo días de firmarse</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/deportes/mundial-futbol/2026-06-13/vinicius-tras-la-estela-de-garrincha-en-brasil.html</t>
+          <t>https://www.elcolombiano.com/internacional/iran-anuncia-acuerdo-paz-ee-uu-dias-firmar-fin-guerra-DF37675314</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="2" t="inlineStr">
-        <is>
-          <t>13/06/2026 12:00 a. m.</t>
-        </is>
-      </c>
+      <c r="A102" s="2" t="inlineStr"/>
       <c r="B102" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3113,26 +3173,22 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>Pickleball: por qué todo el mundo está jugando (y qué necesitas para empezar)</t>
+          <t>Julieta Venegas responde a polémica por “La niña futbolista”: ¿por qué la canción mundialista fue tan criticada?</t>
         </is>
       </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/hemeroteca/2026-06-13/</t>
+          <t>https://www.elcolombiano.com/cultura/musica/julieta-venegas-responde-polemica-nina-futbolista-cancion-criticas-HF37675002</t>
         </is>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="5" t="inlineStr">
-        <is>
-          <t>12/06/2026 11:55 p. m.</t>
-        </is>
-      </c>
+      <c r="A103" s="5" t="inlineStr"/>
       <c r="B103" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3140,26 +3196,22 @@
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D103" s="6" t="inlineStr">
         <is>
-          <t>Abelardo de la Espriella matiza sus propuestas ‘milagro’</t>
+          <t>Modelo webcam se fotografió semidesnuda en una iglesia de Guarne: ¿podría enfrentar sanciones?</t>
         </is>
       </c>
       <c r="E103" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/america-colombia/elecciones-presidenciales/2026-06-13/abelardo-de-la-espriella-matiza-sus-propuestas-milagro.html</t>
+          <t>https://www.elcolombiano.com/antioquia/modelo-webcam-iglesia-guarne-fotos-KF37676963</t>
         </is>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="2" t="inlineStr">
-        <is>
-          <t>12/06/2026 11:52 p. m.</t>
-        </is>
-      </c>
+      <c r="A104" s="2" t="inlineStr"/>
       <c r="B104" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3167,26 +3219,22 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>Sin constituyente y sin paz total: Iván Cepeda publica un plan de gobierno más moderado</t>
+          <t>Luis7Lunes: rapero a tiempo completo</t>
         </is>
       </c>
       <c r="E104" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/america-colombia/elecciones-presidenciales/2026-06-13/sin-constituyente-y-sin-paz-total-ivan-cepeda-publica-un-plan-de-gobierno-mas-moderado.html</t>
+          <t>https://www.elcolombiano.com/cultura/luis7lunes-nuevo-disco-v-sabor-rap-afterclass-FF37675415</t>
         </is>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="5" t="inlineStr">
-        <is>
-          <t>12/06/2026 11:13 p. m.</t>
-        </is>
-      </c>
+      <c r="A105" s="5" t="inlineStr"/>
       <c r="B105" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3194,26 +3242,22 @@
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D105" s="6" t="inlineStr">
         <is>
-          <t>Pilar Rueda, esposa de Iván Cepeda: “En esta elección está en juego la libertad de ser”</t>
+          <t>Colombia redujo su desigualdad en 2025; el nivel más bajo de los últimos seis años</t>
         </is>
       </c>
       <c r="E105" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/america-colombia/elecciones-presidenciales/2026-06-13/pilar-rueda-esposa-de-ivan-cepeda-en-esta-eleccion-esta-en-juego-la-libertad-de-ser.html</t>
+          <t>https://www.elcolombiano.com/negocios/desigualdad-colombia-cae-2025-nivel-bajo-dane-BF37675510</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="2" t="inlineStr">
-        <is>
-          <t>12/06/2026 11:00 p. m.</t>
-        </is>
-      </c>
+      <c r="A106" s="2" t="inlineStr"/>
       <c r="B106" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3221,26 +3265,22 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D106" s="3" t="inlineStr">
         <is>
-          <t>CÓMIC | ¿Por qué les gusta el fútbol?</t>
+          <t>Cristiano Ronaldo respondió a las críticas antes del debut: “Estoy bien, ¿no has visto los partidos?”</t>
         </is>
       </c>
       <c r="E106" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/mexico/2026-06-13/comic-por-que-les-gusta-el-futbol.html</t>
+          <t>https://www.elcolombiano.com/deportes/futbol/cristiano-ronaldo-responde-criticas-antes-debut-mundial-2026-portugal-IF37670945</t>
         </is>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="5" t="inlineStr">
-        <is>
-          <t>12/06/2026 10:45 p. m.</t>
-        </is>
-      </c>
+      <c r="A107" s="5" t="inlineStr"/>
       <c r="B107" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3248,26 +3288,22 @@
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D107" s="6" t="inlineStr">
         <is>
-          <t>¿Puedes batir nuestra predicción? Juega a pronosticar el Mundial</t>
+          <t>Colombia deberá pagar $83,9 billones en intereses de su deuda pública en 2027</t>
         </is>
       </c>
       <c r="E107" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/deportes/mundial-futbol/2026-06-13/puedes-batir-nuestra-prediccion-juega-a-pronosticar-el-mundial.html</t>
+          <t>https://www.elcolombiano.com/negocios/intereses-deuda-publica-colombia-2027-marco-fiscal-minhacienda-DF37674142</t>
         </is>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="inlineStr">
-        <is>
-          <t>12/06/2026 10:30 p. m.</t>
-        </is>
-      </c>
+      <c r="A108" s="2" t="inlineStr"/>
       <c r="B108" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3275,26 +3311,22 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D108" s="3" t="inlineStr">
         <is>
-          <t>Viviendas, sanidad y otros servicios: los suizos se preguntan hasta dónde pueden crecer</t>
+          <t>Elecciones en Perú: Sánchez se resiste a reconocer los resultados y propone a Fujimori revisar “todos los votos”</t>
         </is>
       </c>
       <c r="E108" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/internacional/2026-06-13/viviendas-sanidad-y-otros-servicios-los-suizos-se-preguntan-hasta-donde-pueden-crecer.html</t>
+          <t>https://www.elcolombiano.com/internacional/roberto-sanchez-no-acepta-resultados-fujimori-elecciones-segunda-vuelta-peru-EE37660576</t>
         </is>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="5" t="inlineStr">
-        <is>
-          <t>12/06/2026 10:30 p. m.</t>
-        </is>
-      </c>
+      <c r="A109" s="5" t="inlineStr"/>
       <c r="B109" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3302,26 +3334,22 @@
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D109" s="6" t="inlineStr">
         <is>
-          <t>Los excursionistas que auxiliaron a Jonathan Andic, el quebradero de cabeza de los Mossos</t>
+          <t>Bombardeo contra el Clan del Golfo en zona rural de Chocó dejó al menos 9 criminales muertos</t>
         </is>
       </c>
       <c r="E109" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/espana/catalunya/2026-06-13/los-excursionistas-que-auxiliaron-a-jonathan-andic-el-quebradero-de-cabeza-de-los-mossos.html</t>
+          <t>https://www.elcolombiano.com/colombia/bombardeo-contra-clan-golfo-choco-muertos-nuqui-OE37660680</t>
         </is>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="2" t="inlineStr">
-        <is>
-          <t>12/06/2026 10:30 p. m.</t>
-        </is>
-      </c>
+      <c r="A110" s="2" t="inlineStr"/>
       <c r="B110" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3329,26 +3357,22 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D110" s="3" t="inlineStr">
         <is>
-          <t>La investigación a Zapatero por posible delito fiscal con las joyas limita cualquier regularización ante Hacienda</t>
+          <t>¿Es posible que le dé un ataque al corazón por la emoción de un gol?</t>
         </is>
       </c>
       <c r="E110" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/economia/2026-06-13/la-investigacion-a-zapatero-por-posible-delito-fiscal-con-las-joyas-limita-cualquier-regularizacion-ante-hacienda.html</t>
+          <t>https://www.elcolombiano.com/tendencias/mundial-2026-fifa-ataque-corazon-paro-cardiaco-salud-gol-ME37668774</t>
         </is>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="5" t="inlineStr">
-        <is>
-          <t>12/06/2026 10:30 p. m.</t>
-        </is>
-      </c>
+      <c r="A111" s="5" t="inlineStr"/>
       <c r="B111" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3356,26 +3380,22 @@
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D111" s="6" t="inlineStr">
         <is>
-          <t>¿Está quemando Telecinco ‘Supervivientes’ y ‘La isla de las tentaciones’? La respuesta de los datos de audiencia</t>
+          <t>Encontraron un cadáver frente al estadio donde entrena la Selección de Irán en México</t>
         </is>
       </c>
       <c r="E111" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/television/2026-06-13/esta-quemando-telecinco-supervivientes-y-la-isla-de-las-tentaciones-la-respuesta-de-los-datos-de-audiencia.html</t>
+          <t>https://www.elcolombiano.com/internacional/cadaver-frente-estadio-seleccion-iran-en-mexico-mundial-2026-FF37672124</t>
         </is>
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="2" t="inlineStr">
-        <is>
-          <t>12/06/2026 10:30 p. m.</t>
-        </is>
-      </c>
+      <c r="A112" s="2" t="inlineStr"/>
       <c r="B112" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3383,26 +3403,22 @@
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D112" s="3" t="inlineStr">
         <is>
-          <t>Los primeros estudiantes del grado de Matemáticas y Filosofía, único en España: “Hay que aprender a utilizar la IA con ética”</t>
+          <t>Prográmese: Catar se enfrenta a Suiza este sábado en Santa Clara, por el Grupo B del Mundial</t>
         </is>
       </c>
       <c r="E112" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/educacion/2026-06-13/los-primeros-estudiantes-del-grado-de-matematicas-y-filosofia-unico-en-espana-hay-que-aprender-a-utilizar-la-ia-con-etica.html</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/catar-partido-suiza-sabado-santa-clara-grupo-b-del-mundial-KE37667850</t>
         </is>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="5" t="inlineStr">
-        <is>
-          <t>12/06/2026 10:30 p. m.</t>
-        </is>
-      </c>
+      <c r="A113" s="5" t="inlineStr"/>
       <c r="B113" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3410,26 +3426,22 @@
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D113" s="6" t="inlineStr">
         <is>
-          <t>El paso al frente de Marruecos con su nuevo seleccionador Mohamed Ouahbi</t>
+          <t>Cerraron motel en Medellín señalado por la Fiscalía de permitir la explotación de niñas</t>
         </is>
       </c>
       <c r="E113" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/deportes/mundial-futbol/2026-06-13/el-paso-al-frente-de-marruecos-con-su-nuevo-seleccionador-mohamed-ouahbi.html</t>
+          <t>https://www.elcolombiano.com/medellin/fiscalia-cierra-motel-centro-medellin-prostitucion-menores-AF37670617</t>
         </is>
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="2" t="inlineStr">
-        <is>
-          <t>12/06/2026 10:30 p. m.</t>
-        </is>
-      </c>
+      <c r="A114" s="2" t="inlineStr"/>
       <c r="B114" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3437,26 +3449,22 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D114" s="3" t="inlineStr">
         <is>
-          <t>El vértigo de viajar solo en verano: “Llevo demasiado tiempo viviendo como si mi vida estuviera en pausa”</t>
+          <t>Aprueban la Ley Bartolo: este municipio de Antioquia se convierte en la Capital Mundial de la Mula de Silla</t>
         </is>
       </c>
       <c r="E114" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/estilo-de-vida/2026-06-13/el-vertigo-de-viajar-solo-en-verano-llevo-demasiado-tiempo-viviendo-como-si-mi-vida-estuviera-en-pausa.html</t>
+          <t>https://www.elcolombiano.com/antioquia/ley-bartolo-burro-capital-mundial-de-la-mula-de-silla-titiribi-antioquia-PE37665785</t>
         </is>
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="5" t="inlineStr">
-        <is>
-          <t>12/06/2026 08:15 p. m.</t>
-        </is>
-      </c>
+      <c r="A115" s="5" t="inlineStr"/>
       <c r="B115" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3464,26 +3472,22 @@
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D115" s="6" t="inlineStr">
         <is>
-          <t>Trump anuncia que el ejército de Estados Unidos ha matado en Venezuela al Niño Guerrero, líder del Tren de Aragua</t>
+          <t>Pagos con QR y celular se disparan en Colombia: ¿está llegando el fin del efectivo?</t>
         </is>
       </c>
       <c r="E115" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/america/2026-06-13/trump-anuncia-que-el-ejercito-de-estados-unidos-ha-matado-al-nino-guerrero-lider-del-tren-de-aragua.html</t>
+          <t>https://www.elcolombiano.com/negocios/pagos-qr-celular-colombia-fin-efectivo-bre-b-nequi-CE37661726</t>
         </is>
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="2" t="inlineStr">
-        <is>
-          <t>12/06/2026 02:45 a. m.</t>
-        </is>
-      </c>
+      <c r="A116" s="2" t="inlineStr"/>
       <c r="B116" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3491,17 +3495,17 @@
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D116" s="3" t="inlineStr">
         <is>
-          <t>Maxi Iglesias: “Intento seguir mi vida sin hacer mucho caso al ruido que generan mis decisiones”</t>
+          <t>Iván Cepeda cerrará su campaña presidencial en la Plaza La Santamaría de Bogotá antes de la segunda vuelta</t>
         </is>
       </c>
       <c r="E116" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/icon/2026-06-12/maxi-iglesias-intento-seguir-mi-vida-sin-hacer-mucho-caso-al-ruido-que-generan-mis-decisiones.html</t>
+          <t>https://www.elcolombiano.com/especiales/elecciones-2026/ivan-cepeda-cerrara-su-campana-presidencial-en-la-plaza-la-santamaria-de-bogota-antes-de-la-segunda-vuelta-OH37657018</t>
         </is>
       </c>
     </row>
@@ -3514,17 +3518,17 @@
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D117" s="6" t="inlineStr">
         <is>
-          <t>Predicciones</t>
+          <t>Disidencias de alias Calarcá obligan a votantes a tomarle foto al tarjetón: la grave denuncia de constreñimiento en Caquetá</t>
         </is>
       </c>
       <c r="E117" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/deportes/mundial-futbol/2026-06-11/quien-ganara-el-mundial-asi-arrancan-nuestras-predicciones.html</t>
+          <t>https://www.elcolombiano.com/colombia/disidencias-farc-fotos-voto-caqueta-HG37640236</t>
         </is>
       </c>
     </row>
@@ -3537,17 +3541,17 @@
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D118" s="3" t="inlineStr">
         <is>
-          <t>Selecciones</t>
+          <t>¿Guiño a De la Espriella? Oviedo visitó a Uribe en Rionegro</t>
         </is>
       </c>
       <c r="E118" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/deportes/mundial-futbol/2026-06-05/todas-las-selecciones-del-mundial-de-estados-unidos-canada-y-mexico.html</t>
+          <t>https://www.elcolombiano.com/especiales/elecciones-2026/juan-daniel-oviedo-reunion-alvaro-uribe-elecciones-FG37641361</t>
         </is>
       </c>
     </row>
@@ -4402,7 +4406,7 @@
     <row r="151">
       <c r="A151" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 03:52 a. m.</t>
+          <t>13/06/2026 03:40 a. m.</t>
         </is>
       </c>
       <c r="B151" s="5" t="inlineStr">
@@ -4429,7 +4433,7 @@
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 03:52 a. m.</t>
+          <t>13/06/2026 03:40 a. m.</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
@@ -4456,7 +4460,7 @@
     <row r="153">
       <c r="A153" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 03:52 a. m.</t>
+          <t>13/06/2026 03:40 a. m.</t>
         </is>
       </c>
       <c r="B153" s="5" t="inlineStr">
@@ -4483,7 +4487,7 @@
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 03:52 a. m.</t>
+          <t>13/06/2026 03:40 a. m.</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
@@ -4510,7 +4514,7 @@
     <row r="155">
       <c r="A155" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 03:52 a. m.</t>
+          <t>13/06/2026 03:40 a. m.</t>
         </is>
       </c>
       <c r="B155" s="5" t="inlineStr">
@@ -4525,19 +4529,19 @@
       </c>
       <c r="D155" s="6" t="inlineStr">
         <is>
-          <t>Piden a Estados Unidos que investigue e incluya en la Lista Clinton a Ricardo Roa, presidente de Ecopetrol, por transacciones en la campaña de Petro</t>
+          <t>Max Henriquez lanza alerta por fenómeno del superniño en Colombia: “Es posible que haya racionamiento de agua y energía”</t>
         </is>
       </c>
       <c r="E155" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/piden-a-estados-unidos-que-investigue-e-incluya-en-la-lista-clinton-a-ricardo-roa-presidente-de-ecopetrol-por-transacciones-en-la-campana-de-petro/202620/</t>
+          <t>https://www.semana.com/nacion/articulo/max-henriquez-lanza-alerta-por-fenomeno-del-supernino-en-colombia-es-posible-que-haya-racionamiento-de-agua-y-energia/202629/</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 03:52 a. m.</t>
+          <t>13/06/2026 03:40 a. m.</t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
@@ -4552,19 +4556,19 @@
       </c>
       <c r="D156" s="3" t="inlineStr">
         <is>
-          <t>Estos son los políticos cuestionados que apoyan la candidatura de Iván Cepeda: son señalados por presunta corrupción</t>
+          <t>Piden a Estados Unidos que investigue e incluya en la Lista Clinton a Ricardo Roa, presidente de Ecopetrol, por transacciones en la campaña de Petro</t>
         </is>
       </c>
       <c r="E156" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/estos-son-los-politicos-cuestionados-que-apoyan-la-candidatura-de-ivan-cepeda-son-senalados-por-presunta-corrupcion/202608/</t>
+          <t>https://www.semana.com/nacion/articulo/piden-a-estados-unidos-que-investigue-e-incluya-en-la-lista-clinton-a-ricardo-roa-presidente-de-ecopetrol-por-transacciones-en-la-campana-de-petro/202620/</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 03:52 a. m.</t>
+          <t>13/06/2026 03:40 a. m.</t>
         </is>
       </c>
       <c r="B157" s="5" t="inlineStr">
@@ -4579,19 +4583,19 @@
       </c>
       <c r="D157" s="6" t="inlineStr">
         <is>
-          <t>Mauricio Vargas dice que Abelardo de la Espriella ganaría la presidencia y que “Iván Cepeda y Gustavo Petro competirán por la oposición”</t>
+          <t>Añorado regreso de la Selección Colombia: ocho años deseándolo y así llega a la gran cita de la Copa del Mundo</t>
         </is>
       </c>
       <c r="E157" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/mauricio-vargas-dice-que-abelardo-de-la-espriella-ganara-la-presidencia-y-que-ivan-cepeda-y-gustavo-petro-competiran-por-la-oposicion/202627/</t>
+          <t>https://www.semana.com/deportes/articulo/anorado-regreso-de-la-seleccion-colombia-ocho-anos-deseandolo-y-asi-llega-a-la-gran-cita-de-la-copa-del-mundo/202656/</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 03:52 a. m.</t>
+          <t>13/06/2026 03:40 a. m.</t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
@@ -4618,7 +4622,7 @@
     <row r="159">
       <c r="A159" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 03:52 a. m.</t>
+          <t>13/06/2026 03:40 a. m.</t>
         </is>
       </c>
       <c r="B159" s="5" t="inlineStr">
@@ -4645,7 +4649,7 @@
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 03:52 a. m.</t>
+          <t>13/06/2026 03:40 a. m.</t>
         </is>
       </c>
       <c r="B160" s="2" t="inlineStr">
@@ -4660,19 +4664,19 @@
       </c>
       <c r="D160" s="3" t="inlineStr">
         <is>
-          <t>Salud Hernández-Mora recorrió el Guaviare y comprobó cómo alias Calarcá será un desafío para el próximo presidente</t>
+          <t>Estos son los políticos cuestionados que apoyan la candidatura de Iván Cepeda: son señalados por presunta corrupción</t>
         </is>
       </c>
       <c r="E160" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/salud-hernandez-mora-recorrio-el-guaviare-y-comprobo-como-alias-calarca-sera-un-desafio-para-el-proximo-presidente/202620/</t>
+          <t>https://www.semana.com/politica/articulo/estos-son-los-politicos-cuestionados-que-apoyan-la-candidatura-de-ivan-cepeda-son-senalados-por-presunta-corrupcion/202608/</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 02:52 a. m.</t>
+          <t>13/06/2026 03:40 a. m.</t>
         </is>
       </c>
       <c r="B161" s="5" t="inlineStr">
@@ -4687,19 +4691,19 @@
       </c>
       <c r="D161" s="6" t="inlineStr">
         <is>
-          <t>Selección Colombia: SEMANA conversó con los familiares de los convocados al Mundial 2026. Historias de sacrificio, temple y mucho amor</t>
+          <t>Mauricio Vargas dice que Abelardo de la Espriella ganaría la presidencia y que “Iván Cepeda y Gustavo Petro competirán por la oposición”</t>
         </is>
       </c>
       <c r="E161" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/seleccion-colombia-semana-converso-con-los-familiares-de-los-convocados-al-mundial-2026-historias-de-sacrificio-temple-y-mucho-amor/202621/</t>
+          <t>https://www.semana.com/politica/articulo/mauricio-vargas-dice-que-abelardo-de-la-espriella-ganara-la-presidencia-y-que-ivan-cepeda-y-gustavo-petro-competiran-por-la-oposicion/202627/</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 02:52 a. m.</t>
+          <t>13/06/2026 03:40 a. m.</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
@@ -4714,19 +4718,19 @@
       </c>
       <c r="D162" s="3" t="inlineStr">
         <is>
-          <t>Max Henriquez lanza alerta por fenómeno del superniño en Colombia: “Es posible que haya racionamiento de agua y energía”</t>
+          <t>Salud Hernández-Mora recorrió el Guaviare y comprobó cómo alias Calarcá será un desafío para el próximo presidente</t>
         </is>
       </c>
       <c r="E162" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/max-henriquez-lanza-alerta-por-fenomeno-del-supernino-en-colombia-es-posible-que-haya-racionamiento-de-agua-y-energia/202629/</t>
+          <t>https://www.semana.com/nacion/articulo/salud-hernandez-mora-recorrio-el-guaviare-y-comprobo-como-alias-calarca-sera-un-desafio-para-el-proximo-presidente/202620/</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 02:52 a. m.</t>
+          <t>13/06/2026 02:40 a. m.</t>
         </is>
       </c>
       <c r="B163" s="5" t="inlineStr">
@@ -4741,19 +4745,19 @@
       </c>
       <c r="D163" s="6" t="inlineStr">
         <is>
-          <t>Habla Sofía Otero, la doctora de la mafia</t>
+          <t>Selección Colombia: SEMANA conversó con los familiares de los convocados al Mundial 2026. Historias de sacrificio, temple y mucho amor</t>
         </is>
       </c>
       <c r="E163" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/habla-sofia-otero-la-doctora-de-la-mafia/202636/</t>
+          <t>https://www.semana.com/deportes/articulo/seleccion-colombia-semana-converso-con-los-familiares-de-los-convocados-al-mundial-2026-historias-de-sacrificio-temple-y-mucho-amor/202621/</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 02:52 a. m.</t>
+          <t>13/06/2026 02:40 a. m.</t>
         </is>
       </c>
       <c r="B164" s="2" t="inlineStr">
@@ -4768,19 +4772,19 @@
       </c>
       <c r="D164" s="3" t="inlineStr">
         <is>
-          <t>Añorado regreso de la Selección Colombia: ocho años deseándolo y así llega a la gran cita de la Copa del Mundo</t>
+          <t>Habla Sofía Otero, la doctora de la mafia</t>
         </is>
       </c>
       <c r="E164" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/anorado-regreso-de-la-seleccion-colombia-ocho-anos-deseandolo-y-asi-llega-a-la-gran-cita-de-la-copa-del-mundo/202656/</t>
+          <t>https://www.semana.com/nacion/articulo/habla-sofia-otero-la-doctora-de-la-mafia/202636/</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 02:52 a. m.</t>
+          <t>13/06/2026 02:40 a. m.</t>
         </is>
       </c>
       <c r="B165" s="5" t="inlineStr">
@@ -4807,7 +4811,7 @@
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 01:52 a. m.</t>
+          <t>13/06/2026 01:40 a. m.</t>
         </is>
       </c>
       <c r="B166" s="2" t="inlineStr">
@@ -4834,7 +4838,7 @@
     <row r="167">
       <c r="A167" s="5" t="inlineStr">
         <is>
-          <t>13/06/2026 01:52 a. m.</t>
+          <t>13/06/2026 01:40 a. m.</t>
         </is>
       </c>
       <c r="B167" s="5" t="inlineStr">
@@ -4861,7 +4865,7 @@
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026 01:52 a. m.</t>
+          <t>13/06/2026 01:40 a. m.</t>
         </is>
       </c>
       <c r="B168" s="2" t="inlineStr">
@@ -5854,12 +5858,12 @@
       </c>
       <c r="D206" s="3" t="inlineStr">
         <is>
-          <t>Militares ecuatorianos resultaron heridos en combate con grupo armado cerca de la frontera con Colombia: Ejército reporta posibles bajas</t>
+          <t>Abelardo De la Espriella supera a Iván Cepeda en la recta final de la segunda vuelta presidencial, según encuesta de Guarumo y Ecoanalítica</t>
         </is>
       </c>
       <c r="E206" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/militares-ecuatorianos-resultaron-heridos-en-combate-con-grupo-armado-cerca-de-la-frontera-con-colombia-ejercito-reporta-posibles-bajas/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/abelardo-de-la-espriella-supera-a-ivan-cepeda-en-la-recta-final-de-la-segunda-vuelta-presidencial-segun-encuesta-de-guarumo-y-ecoanalitica/</t>
         </is>
       </c>
     </row>
@@ -5881,12 +5885,12 @@
       </c>
       <c r="D207" s="6" t="inlineStr">
         <is>
-          <t>Mindefensa desestima denuncias de Uribe sobre presunto fraude del Eln en Arauca y cita informes de la MOE</t>
+          <t>Militares ecuatorianos resultaron heridos en combate con grupo armado cerca de la frontera con Colombia: Ejército reporta posibles bajas</t>
         </is>
       </c>
       <c r="E207" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/mindefensa-desestima-denuncias-de-uribe-sobre-presunto-fraude-del-eln-en-arauca-y-cita-informes-de-la-moe/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/militares-ecuatorianos-resultaron-heridos-en-combate-con-grupo-armado-cerca-de-la-frontera-con-colombia-ejercito-reporta-posibles-bajas/</t>
         </is>
       </c>
     </row>
@@ -5908,12 +5912,12 @@
       </c>
       <c r="D208" s="3" t="inlineStr">
         <is>
-          <t>Ideam advierte que Colombia enfrentaría el fenómeno de El Niño más fuerte desde 1950 y que su pico llegaría a fin de año</t>
+          <t>Mindefensa desestima denuncias de Uribe sobre presunto fraude del Eln en Arauca y cita informes de la MOE</t>
         </is>
       </c>
       <c r="E208" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/ideam-advierte-que-colombia-enfrentaria-el-fenomeno-de-el-nino-mas-fuerte-desde-1950-y-que-su-pico-llegaria-a-fin-de-ano/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/mindefensa-desestima-denuncias-de-uribe-sobre-presunto-fraude-del-eln-en-arauca-y-cita-informes-de-la-moe/</t>
         </is>
       </c>
     </row>
@@ -5935,12 +5939,12 @@
       </c>
       <c r="D209" s="6" t="inlineStr">
         <is>
-          <t>Clima: las temperaturas que predominarán este 13 de junio en Barranquilla</t>
+          <t>Ideam advierte que Colombia enfrentaría el fenómeno de El Niño más fuerte desde 1950 y que su pico llegaría a fin de año</t>
         </is>
       </c>
       <c r="E209" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/clima-las-temperaturas-que-predominaran-este-13-de-junio-en-barranquilla/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/ideam-advierte-que-colombia-enfrentaria-el-fenomeno-de-el-nino-mas-fuerte-desde-1950-y-que-su-pico-llegaria-a-fin-de-ano/</t>
         </is>
       </c>
     </row>
@@ -5962,12 +5966,12 @@
       </c>
       <c r="D210" s="3" t="inlineStr">
         <is>
-          <t>Clima: las temperaturas que predominarán este 13 de junio en Bogotá</t>
+          <t>Clima: las temperaturas que predominarán este 13 de junio en Barranquilla</t>
         </is>
       </c>
       <c r="E210" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/clima-las-temperaturas-que-predominaran-este-13-de-junio-en-bogota/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/clima-las-temperaturas-que-predominaran-este-13-de-junio-en-barranquilla/</t>
         </is>
       </c>
     </row>
@@ -5989,12 +5993,12 @@
       </c>
       <c r="D211" s="6" t="inlineStr">
         <is>
-          <t>¿Cuál es la temperatura promedio en Medellín?</t>
+          <t>Clima: las temperaturas que predominarán este 13 de junio en Bogotá</t>
         </is>
       </c>
       <c r="E211" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/cual-es-la-temperatura-promedio-en-medellin/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/clima-las-temperaturas-que-predominaran-este-13-de-junio-en-bogota/</t>
         </is>
       </c>
     </row>
@@ -6016,12 +6020,12 @@
       </c>
       <c r="D212" s="3" t="inlineStr">
         <is>
-          <t>Clima hoy en Colombia: temperaturas para Cali este 13 de junio</t>
+          <t>¿Cuál es la temperatura promedio en Medellín?</t>
         </is>
       </c>
       <c r="E212" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/clima-hoy-en-colombia-temperaturas-para-cali-este-13-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/cual-es-la-temperatura-promedio-en-medellin/</t>
         </is>
       </c>
     </row>
@@ -6043,12 +6047,12 @@
       </c>
       <c r="D213" s="6" t="inlineStr">
         <is>
-          <t>Clima hoy en Colombia: temperaturas para Cartagena de Indias este 13 de junio</t>
+          <t>Clima hoy en Colombia: temperaturas para Cali este 13 de junio</t>
         </is>
       </c>
       <c r="E213" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/clima-hoy-en-colombia-temperaturas-para-cartagena-de-indias-este-13-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/clima-hoy-en-colombia-temperaturas-para-cali-este-13-de-junio/</t>
         </is>
       </c>
     </row>
@@ -6070,12 +6074,12 @@
       </c>
       <c r="D214" s="3" t="inlineStr">
         <is>
-          <t>Resultado Sinuano Noche hoy 12 de junio</t>
+          <t>Clima hoy en Colombia: temperaturas para Cartagena de Indias este 13 de junio</t>
         </is>
       </c>
       <c r="E214" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/resultado-sinuano-noche-hoy-12-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/clima-hoy-en-colombia-temperaturas-para-cartagena-de-indias-este-13-de-junio/</t>
         </is>
       </c>
     </row>
@@ -6097,12 +6101,12 @@
       </c>
       <c r="D215" s="6" t="inlineStr">
         <is>
-          <t>Mindefensa alerta por posibles disturbios tras la segunda vuelta y anticipa medidas por información de inteligencia</t>
+          <t>Resultado Sinuano Noche hoy 12 de junio</t>
         </is>
       </c>
       <c r="E215" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/mindefensa-alerta-por-posibles-disturbios-tras-la-segunda-vuelta-y-anticipa-medidas-por-informacion-de-inteligencia/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/resultado-sinuano-noche-hoy-12-de-junio/</t>
         </is>
       </c>
     </row>
@@ -6124,12 +6128,12 @@
       </c>
       <c r="D216" s="3" t="inlineStr">
         <is>
-          <t>JEP ha identificado plenamente a 1.956 víctimas de falsos positivos y aún busca establecer quiénes son otras 418</t>
+          <t>Mindefensa alerta por posibles disturbios tras la segunda vuelta y anticipa medidas por información de inteligencia</t>
         </is>
       </c>
       <c r="E216" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/jep-ha-identificado-plenamente-a-1956-victimas-de-falsos-positivos-y-aun-busca-establecer-quienes-son-otras-418/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/mindefensa-alerta-por-posibles-disturbios-tras-la-segunda-vuelta-y-anticipa-medidas-por-informacion-de-inteligencia/</t>
         </is>
       </c>
     </row>
@@ -6151,12 +6155,12 @@
       </c>
       <c r="D217" s="6" t="inlineStr">
         <is>
-          <t>“Costó 30.000 pesos y hoy estoy pagando con todo este dolor”: influencer denuncia procedimiento estético que casi le cuesta la vida</t>
+          <t>JEP ha identificado plenamente a 1.956 víctimas de falsos positivos y aún busca establecer quiénes son otras 418</t>
         </is>
       </c>
       <c r="E217" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/costo-30000-pesos-y-hoy-estoy-pagando-con-todo-este-dolor-influencer-denuncia-procedimiento-estetico-que-casi-le-cuesta-la-vida/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/jep-ha-identificado-plenamente-a-1956-victimas-de-falsos-positivos-y-aun-busca-establecer-quienes-son-otras-418/</t>
         </is>
       </c>
     </row>
@@ -6178,12 +6182,12 @@
       </c>
       <c r="D218" s="3" t="inlineStr">
         <is>
-          <t>Resultados Lotería de Santander hoy 13 de junio: revise su billete y cobre el premio mayor</t>
+          <t>“Costó 30.000 pesos y hoy estoy pagando con todo este dolor”: influencer denuncia procedimiento estético que casi le cuesta la vida</t>
         </is>
       </c>
       <c r="E218" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/resultados-loteria-de-santander-hoy-13-de-junio-revise-su-billete-y-cobre-el-premio-mayor/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/costo-30000-pesos-y-hoy-estoy-pagando-con-todo-este-dolor-influencer-denuncia-procedimiento-estetico-que-casi-le-cuesta-la-vida/</t>
         </is>
       </c>
     </row>
@@ -6205,12 +6209,12 @@
       </c>
       <c r="D219" s="6" t="inlineStr">
         <is>
-          <t>Iván Cepeda firma pacto por el agua en Bucaramanga y busca sumar apoyos en Santander para la segunda vuelta</t>
+          <t>Resultados Lotería de Santander hoy 13 de junio: revise su billete y cobre el premio mayor</t>
         </is>
       </c>
       <c r="E219" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/ivan-cepeda-firma-pacto-por-el-agua-en-bucaramanga-y-busca-sumar-apoyos-en-santander-para-la-segunda-vuelta/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/resultados-loteria-de-santander-hoy-13-de-junio-revise-su-billete-y-cobre-el-premio-mayor/</t>
         </is>
       </c>
     </row>
@@ -6232,12 +6236,12 @@
       </c>
       <c r="D220" s="3" t="inlineStr">
         <is>
-          <t>Generadoras alertan que deuda de Air-e podría superar los $3 billones y ponen sobre la mesa riesgo por fenómeno de El Niño</t>
+          <t>Iván Cepeda firma pacto por el agua en Bucaramanga y busca sumar apoyos en Santander para la segunda vuelta</t>
         </is>
       </c>
       <c r="E220" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/generadoras-alertan-que-deuda-de-air-e-podria-superar-los-3-billones-y-ponen-sobre-la-mesa-riesgo-por-fenomeno-de-el-nino/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/ivan-cepeda-firma-pacto-por-el-agua-en-bucaramanga-y-busca-sumar-apoyos-en-santander-para-la-segunda-vuelta/</t>
         </is>
       </c>
     </row>
@@ -6259,12 +6263,12 @@
       </c>
       <c r="D221" s="6" t="inlineStr">
         <is>
-          <t>Resultado Chontico Noche: números ganadores del último sorteo hoy, viernes 12 de junio de 2026</t>
+          <t>Generadoras alertan que deuda de Air-e podría superar los $3 billones y ponen sobre la mesa riesgo por fenómeno de El Niño</t>
         </is>
       </c>
       <c r="E221" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/resultado-chontico-noche-numeros-ganadores-del-ultimo-sorteo-hoy-viernes-12-de-junio-de-2026/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/generadoras-alertan-que-deuda-de-air-e-podria-superar-los-3-billones-y-ponen-sobre-la-mesa-riesgo-por-fenomeno-de-el-nino/</t>
         </is>
       </c>
     </row>
@@ -6286,12 +6290,12 @@
       </c>
       <c r="D222" s="3" t="inlineStr">
         <is>
-          <t>Lotería de Risaralda: resultados ganadores del sábado 13 de junio</t>
+          <t>Resultado Chontico Noche: números ganadores del último sorteo hoy, viernes 12 de junio de 2026</t>
         </is>
       </c>
       <c r="E222" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/loteria-de-risaralda-resultados-ganadores-del-sabado-13-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/resultado-chontico-noche-numeros-ganadores-del-ultimo-sorteo-hoy-viernes-12-de-junio-de-2026/</t>
         </is>
       </c>
     </row>
@@ -6313,12 +6317,12 @@
       </c>
       <c r="D223" s="6" t="inlineStr">
         <is>
-          <t>Resultados Lotería de Medellín 12 de junio: números ganadores del último sorteo</t>
+          <t>Lotería de Risaralda: resultados ganadores del sábado 13 de junio</t>
         </is>
       </c>
       <c r="E223" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/resultados-loteria-de-medellin-12-de-junio-numeros-ganadores-del-ultimo-sorteo/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/loteria-de-risaralda-resultados-ganadores-del-sabado-13-de-junio/</t>
         </is>
       </c>
     </row>
@@ -6340,12 +6344,12 @@
       </c>
       <c r="D224" s="3" t="inlineStr">
         <is>
-          <t>Resultado Super Astro Luna HOY: número ganador del viernes 12 de junio</t>
+          <t>Resultados Lotería de Medellín 12 de junio: números ganadores del último sorteo</t>
         </is>
       </c>
       <c r="E224" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/resultado-super-astro-luna-hoy-numero-ganador-del-viernes-12-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/resultados-loteria-de-medellin-12-de-junio-numeros-ganadores-del-ultimo-sorteo/</t>
         </is>
       </c>
     </row>
@@ -6367,12 +6371,12 @@
       </c>
       <c r="D225" s="6" t="inlineStr">
         <is>
-          <t>Alias Samantha, la vocera de las disidencias de las Farc por la que ofrecen 100 millones de pesos de recompensa</t>
+          <t>Resultado Super Astro Luna HOY: número ganador del viernes 12 de junio</t>
         </is>
       </c>
       <c r="E225" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/13/alias-samantha-la-vocera-de-las-disidencias-de-las-farc-por-la-que-ofrecen-100-millones-de-pesos-de-recompensa/</t>
+          <t>https://www.infobae.com/colombia/2026/06/13/resultado-super-astro-luna-hoy-numero-ganador-del-viernes-12-de-junio/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 Noticias actualizadas 18/06/2026 09:37
</commit_message>
<xml_diff>
--- a/docs/ultimahora.xlsx
+++ b/docs/ultimahora.xlsx
@@ -515,7 +515,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 02:44 a. m.</t>
+          <t>18/06/2026 04:09 a. m.</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -530,19 +530,19 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Elecciones presidenciales Colombia 2026: todo sobre la segunda vuelta presidencial que definirá al próximo presidente</t>
+          <t>Néstor Lorenzo, director técnico de la selección, sobre la victoria de Colombia frente a Uzbekistán: 'Sabíamos que iba a ser un partido difícil'</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/elecciones-presidenciales-colombia-2026-todo-sobre-la-segunda-vuelta-presidencial-que-definira-al-proximo-presidente-3565112</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/nestor-lorenzo-director-tecnico-de-la-seleccion-sobre-la-victoria-de-colombia-frente-a-uzbekistan-sabiamos-que-iba-a-ser-un-partido-dificil-3565115</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 02:31 a. m.</t>
+          <t>18/06/2026 03:44 a. m.</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -557,19 +557,19 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>Queda solo un mes de la ventana de traslado pensional: si quiere aprovechar, ¿le conviene más un fondo privado que Colpensiones?</t>
+          <t>Los mejores memes del partido Colombia vs. Uzbekistán: así reaccionaron las redes al debut de la Tricolor en el Mundial 2026 en México</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/economia/finanzas-personales/queda-solo-un-mes-de-la-ventana-de-traslado-pensional-si-quiere-aprovechar-le-conviene-mas-un-fondo-privado-que-colpensiones-3564894</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/los-mejores-memes-del-partido-colombia-vs-uzbekistan-asi-reaccionaron-las-redes-al-debut-de-la-tricolor-en-el-mundial-2026-en-mexico-3565114</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 02:30 a. m.</t>
+          <t>18/06/2026 02:44 a. m.</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -584,19 +584,19 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>¡Atención conductores! Pico y placa en Pereira para el jueves 18 de junio de 2026: así regirá la medida</t>
+          <t>Elecciones presidenciales Colombia 2026: todo sobre la segunda vuelta presidencial que definirá al próximo presidente</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/otras-ciudades/atencion-conductores-pico-y-placa-en-pereira-para-el-jueves-18-de-junio-de-2026-asi-regira-la-medida-3564946</t>
+          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/elecciones-presidenciales-colombia-2026-todo-sobre-la-segunda-vuelta-presidencial-que-definira-al-proximo-presidente-3565112</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 02:30 a. m.</t>
+          <t>18/06/2026 02:31 a. m.</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -611,12 +611,12 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>¡Evite contratiempos! Pico y placa en Bucaramanga para el jueves 18 de junio de 2026</t>
+          <t>Queda solo un mes de la ventana de traslado pensional: si quiere aprovechar, ¿le conviene más un fondo privado que Colpensiones?</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/santander/evite-contratiempos-pico-y-placa-en-bucaramanga-para-el-jueves-18-de-junio-de-3564945</t>
+          <t>https://www.eltiempo.com/economia/finanzas-personales/queda-solo-un-mes-de-la-ventana-de-traslado-pensional-si-quiere-aprovechar-le-conviene-mas-un-fondo-privado-que-colpensiones-3564894</t>
         </is>
       </c>
     </row>
@@ -638,12 +638,12 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>¡Siga la medida de movilidad! Pico y placa en Medellín para el jueves 18 de junio de 2026: así funciona la restricción</t>
+          <t>¡Atención conductores! Pico y placa en Pereira para el jueves 18 de junio de 2026: así regirá la medida</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/medellin/siga-la-medida-de-movilidad-pico-y-placa-en-medellin-para-el-jueves-18-de-junio-de-2026-asi-funciona-la-restriccion-3564942</t>
+          <t>https://www.eltiempo.com/colombia/otras-ciudades/atencion-conductores-pico-y-placa-en-pereira-para-el-jueves-18-de-junio-de-2026-asi-regira-la-medida-3564946</t>
         </is>
       </c>
     </row>
@@ -665,19 +665,19 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>¡Evite multas! Pico y placa en Cali para el jueves 18 de junio de 2026: así opera la medida</t>
+          <t>¡Evite contratiempos! Pico y placa en Bucaramanga para el jueves 18 de junio de 2026</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/cali/evite-multas-pico-y-placa-en-cali-para-el-jueves-18-de-junio-de-2026-asi-opera-la-medida-3564941</t>
+          <t>https://www.eltiempo.com/colombia/santander/evite-contratiempos-pico-y-placa-en-bucaramanga-para-el-jueves-18-de-junio-de-3564945</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 02:20 a. m.</t>
+          <t>18/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -692,19 +692,19 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>¡Pilas en las vías! Pico y placa en Bogotá para el jueves 18 de junio de 2026</t>
+          <t>¡Siga la medida de movilidad! Pico y placa en Medellín para el jueves 18 de junio de 2026: así funciona la restricción</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/bogota/pilas-en-las-vias-pico-y-placa-en-bogota-para-el-jueves-18-de-junio-de-3564940</t>
+          <t>https://www.eltiempo.com/colombia/medellin/siga-la-medida-de-movilidad-pico-y-placa-en-medellin-para-el-jueves-18-de-junio-de-2026-asi-funciona-la-restriccion-3564942</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 02:14 a. m.</t>
+          <t>18/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -719,19 +719,19 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Mundial 2026 hoy jueves 18 de junio: partidos, goles, clasificaciones y últimas noticias de la Copa del Mundo</t>
+          <t>¡Evite multas! Pico y placa en Cali para el jueves 18 de junio de 2026: así opera la medida</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/mundial-2026-hoy-jueves-18-de-junio-partidos-goles-clasificaciones-y-ultimas-noticias-de-la-copa-del-mundo-3565111</t>
+          <t>https://www.eltiempo.com/colombia/cali/evite-multas-pico-y-placa-en-cali-para-el-jueves-18-de-junio-de-2026-asi-opera-la-medida-3564941</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 01:50 a. m.</t>
+          <t>18/06/2026 02:20 a. m.</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -746,19 +746,19 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Colombia ganó y Luis Díaz brilló: así arrancó el Mundial 2026 (día 7 del Mundial)</t>
+          <t>¡Pilas en las vías! Pico y placa en Bogotá para el jueves 18 de junio de 2026</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/podcast/contraataque/colombia-gano-y-luis-diaz-brillo-asi-arranco-el-mundial-2026-dia-7-del-mundial-3565110</t>
+          <t>https://www.eltiempo.com/bogota/pilas-en-las-vias-pico-y-placa-en-bogota-para-el-jueves-18-de-junio-de-3564940</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 01:05 a. m.</t>
+          <t>18/06/2026 02:14 a. m.</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -773,19 +773,19 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>El tercer Major del año, con presencia colombiana: Marcelo Rozo y Nico Echavarría, listos para jugar el US Open</t>
+          <t>Mundial 2026 hoy jueves 18 de junio: partidos, goles, clasificaciones y últimas noticias de la Copa del Mundo</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/otros-deportes/el-tercer-major-del-ano-con-presencia-colombiana-marcelo-rozo-y-nico-echavarria-listos-para-jugar-el-us-open-3565109</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/mundial-2026-hoy-jueves-18-de-junio-partidos-goles-clasificaciones-y-ultimas-noticias-de-la-copa-del-mundo-3565111</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 12:42 a. m.</t>
+          <t>18/06/2026 01:50 a. m.</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -800,19 +800,19 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Selección Colombia, bien acompañada: las mujeres lideran la marea amarilla en México</t>
+          <t>Colombia ganó y Luis Díaz brilló: así arrancó el Mundial 2026 (día 7 del Mundial)</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/seleccion-colombia-bien-acompanada-las-mujeres-lideran-la-marea-amarilla-en-mexico-3565107</t>
+          <t>https://www.eltiempo.com/podcast/contraataque/colombia-gano-y-luis-diaz-brillo-asi-arranco-el-mundial-2026-dia-7-del-mundial-3565110</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 12:31 a. m.</t>
+          <t>18/06/2026 01:05 a. m.</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -827,19 +827,19 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>La Selección Colombia y su balance individual tras ganarle a Uzbekistán: Luis Díaz, la pieza fundamental para la victoria</t>
+          <t>El tercer Major del año, con presencia colombiana: Marcelo Rozo y Nico Echavarría, listos para jugar el US Open</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/la-seleccion-colombia-y-su-balance-individual-tras-ganarle-a-uzbekistan-luis-diaz-la-pieza-fundamental-para-la-victoria-3565106</t>
+          <t>https://www.eltiempo.com/deportes/otros-deportes/el-tercer-major-del-ano-con-presencia-colombiana-marcelo-rozo-y-nico-echavarria-listos-para-jugar-el-us-open-3565109</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 12:29 a. m.</t>
+          <t>18/06/2026 12:42 a. m.</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -854,19 +854,19 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Aprobación de asilos para colombianos cae a mínimos históricos en EE. UU. bajo la era Trump: ¿cómo afecta a quienes tienen solicitudes pendientes?</t>
+          <t>Selección Colombia, bien acompañada: las mujeres lideran la marea amarilla en México</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/aprobacion-de-asilos-para-colombianos-cae-a-minimos-historicos-en-ee-uu-bajo-la-era-trump-como-afecta-a-quienes-tienen-solicitudes-pendientes-3564891</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/seleccion-colombia-bien-acompanada-las-mujeres-lideran-la-marea-amarilla-en-mexico-3565107</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 12:21 a. m.</t>
+          <t>18/06/2026 12:31 a. m.</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -881,19 +881,19 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Colombia, entre la ilusión y el momento de caos... No sé si decirlo (Opinión)</t>
+          <t>La Selección Colombia y su balance individual tras ganarle a Uzbekistán: Luis Díaz, la pieza fundamental para la victoria</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/colombia-entre-la-ilusion-y-el-momento-de-caos-no-se-si-decirlo-opinion-3565103</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/la-seleccion-colombia-y-su-balance-individual-tras-ganarle-a-uzbekistan-luis-diaz-la-pieza-fundamental-para-la-victoria-3565106</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 12:18 a. m.</t>
+          <t>18/06/2026 12:29 a. m.</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -908,19 +908,19 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Suiza y Bosnia Herzegovina, hora de empezar a ganar para ambos en el grupo B: hora y TV en vivo</t>
+          <t>Aprobación de asilos para colombianos cae a mínimos históricos en EE. UU. bajo la era Trump: ¿cómo afecta a quienes tienen solicitudes pendientes?</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/suiza-y-bosnia-herzegovina-hora-de-empezar-a-ganar-para-ambos-en-el-grupo-b-hora-y-tv-en-vivo-3565035</t>
+          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/aprobacion-de-asilos-para-colombianos-cae-a-minimos-historicos-en-ee-uu-bajo-la-era-trump-como-afecta-a-quienes-tienen-solicitudes-pendientes-3564891</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 12:06 a. m.</t>
+          <t>18/06/2026 12:21 a. m.</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -935,19 +935,19 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>Luis Díaz la tiene clara: contundente tras ser elegido la gran estrella de Colombia contra Uzbekistán en el Mundial</t>
+          <t>Colombia, entre la ilusión y el momento de caos... No sé si decirlo (Opinión)</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/luis-diaz-la-tiene-clara-contundente-tras-ser-elegido-la-gran-estrella-de-colombia-contra-uzbekistan-en-el-mundial-3565105</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/colombia-entre-la-ilusion-y-el-momento-de-caos-no-se-si-decirlo-opinion-3565103</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 12:05 a. m.</t>
+          <t>18/06/2026 12:18 a. m.</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -962,19 +962,19 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Centros de retorno, arrestos y expulsión a terceros países: así será la nueva política migratoria que cierra aún más el acceso a Europa</t>
+          <t>Suiza y Bosnia Herzegovina, hora de empezar a ganar para ambos en el grupo B: hora y TV en vivo</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/europa/centros-de-retorno-arrestos-y-expulsion-a-terceros-paises-asi-sera-la-nueva-politica-migratoria-que-cierra-aun-mas-el-acceso-a-europa-3564931</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/suiza-y-bosnia-herzegovina-hora-de-empezar-a-ganar-para-ambos-en-el-grupo-b-hora-y-tv-en-vivo-3565035</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>17/06/2026 11:44 p. m.</t>
+          <t>18/06/2026 12:06 a. m.</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -989,19 +989,19 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Responsabilidad en el debate</t>
+          <t>Luis Díaz la tiene clara: contundente tras ser elegido la gran estrella de Colombia contra Uzbekistán en el Mundial</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/cartas/responsabilidad-en-el-debate-3565104</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/luis-diaz-la-tiene-clara-contundente-tras-ser-elegido-la-gran-estrella-de-colombia-contra-uzbekistan-en-el-mundial-3565105</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>17/06/2026 11:32 p. m.</t>
+          <t>18/06/2026 12:05 a. m.</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1016,19 +1016,19 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Baloto y Baloto Revancha: conozca aquí los resultados del último sorteo del miércoles 17 de junio de 2026</t>
+          <t>Centros de retorno, arrestos y expulsión a terceros países: así será la nueva política migratoria que cierra aún más el acceso a Europa</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/economia/finanzas-personales/baloto-y-baloto-revancha-conozca-aqui-los-resultados-del-ultimo-sorteo-del-miercoles-17-de-junio-de-3565099</t>
+          <t>https://www.eltiempo.com/mundo/europa/centros-de-retorno-arrestos-y-expulsion-a-terceros-paises-asi-sera-la-nueva-politica-migratoria-que-cierra-aun-mas-el-acceso-a-europa-3564931</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>17/06/2026 11:29 p. m.</t>
+          <t>17/06/2026 11:44 p. m.</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
@@ -1043,12 +1043,12 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Así quedó la tabla de posiciones del Grupo K tras la victoria 3 a 1 de Colombia ante Uzbekistán en su debut de la Copa del Mundo 2026</t>
+          <t>Responsabilidad en el debate</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/asi-quedo-la-tabla-de-posiciones-del-grupo-k-tras-la-victoria-3-a-1-de-colombia-ante-uzbekistan-en-su-debut-de-la-copa-del-mundo-3565064</t>
+          <t>https://www.eltiempo.com/opinion/cartas/responsabilidad-en-el-debate-3565104</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 12:14 a. m.</t>
+          <t>18/06/2026 04:12 a. m.</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -1097,19 +1097,19 @@
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Luis Díaz tras su debut en el Mundial y el gol para Colombia: “Luché para estar en estos momentos”</t>
+          <t>Fujimori incrementa a más 39.000 votos su ventaja sobre Sánchez en las elecciones en Perú</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/18/luis-diaz-tras-su-debut-en-el-mundial-y-el-gol-para-colombia-luche-para-estar-en-estos-momentos/</t>
+          <t>https://caracol.com.co/2026/06/18/fujimori-incrementa-a-mas-39000-votos-su-ventaja-sobre-sanchez-en-las-elecciones-en-peru/</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>17/06/2026 11:58 p. m.</t>
+          <t>18/06/2026 12:14 a. m.</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1124,19 +1124,19 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Trump pide ‘salir a votar por De La Espriella’ de cara a la segunda vuelta</t>
+          <t>Luis Díaz tras su debut en el Mundial y el gol para Colombia: “Luché para estar en estos momentos”</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/18/trump-pide-salir-a-votar-por-la-de-espriella-de-cara-a-la-segunda-vuelta/</t>
+          <t>https://caracol.com.co/2026/06/18/luis-diaz-tras-su-debut-en-el-mundial-y-el-gol-para-colombia-luche-para-estar-en-estos-momentos/</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>17/06/2026 11:21 p. m.</t>
+          <t>17/06/2026 11:58 p. m.</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
@@ -1151,19 +1151,19 @@
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Ibagué fortalece la estrategia Caza Cochinos 2.0 con monitoreo y control de infractores ambientales</t>
+          <t>Trump pide ‘salir a votar por De La Espriella’ de cara a la segunda vuelta</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/18/ibague-fortalece-la-estrategia-caza-cochinos-20-con-monitoreo-y-control-de-infractores-ambientales/</t>
+          <t>https://caracol.com.co/2026/06/18/trump-pide-salir-a-votar-por-la-de-espriella-de-cara-a-la-segunda-vuelta/</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>17/06/2026 11:03 p. m.</t>
+          <t>17/06/2026 11:21 p. m.</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1178,19 +1178,19 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Colombia inicia con triunfo ante Uzbekistán en el Mundial 2026: goles y mejores momentos del partido</t>
+          <t>Ibagué fortalece la estrategia Caza Cochinos 2.0 con monitoreo y control de infractores ambientales</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/18/colombia-vs-uzbekistan-en-vivo-mundial-2026-transmision-y-minuto-a-minuto-del-partido-hoy/</t>
+          <t>https://caracol.com.co/2026/06/18/ibague-fortalece-la-estrategia-caza-cochinos-20-con-monitoreo-y-control-de-infractores-ambientales/</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>17/06/2026 10:00 p. m.</t>
+          <t>17/06/2026 11:03 p. m.</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -1205,19 +1205,19 @@
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>¿Pidió factura electrónica en 2025? Así puede aplicar al descuento DIAN en la declaración de renta</t>
+          <t>Colombia inicia con triunfo ante Uzbekistán en el Mundial 2026: goles y mejores momentos del partido</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/18/pidio-factura-electronica-en-2025-asi-puede-aplicar-al-descuento-dian-en-la-declaracion-de-renta/</t>
+          <t>https://caracol.com.co/2026/06/18/colombia-vs-uzbekistan-en-vivo-mundial-2026-transmision-y-minuto-a-minuto-del-partido-hoy/</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>17/06/2026 09:49 p. m.</t>
+          <t>17/06/2026 10:00 p. m.</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1232,19 +1232,19 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>ICETEX ofrece becas del 50% para estudiar maestrías virtuales en España: Así puede postularse</t>
+          <t>¿Pidió factura electrónica en 2025? Así puede aplicar al descuento DIAN en la declaración de renta</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/18/icetex-ofrece-becas-del-50-para-estudiar-maestrias-virtuales-en-espana-asi-puede-postularse/</t>
+          <t>https://caracol.com.co/2026/06/18/pidio-factura-electronica-en-2025-asi-puede-aplicar-al-descuento-dian-en-la-declaracion-de-renta/</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>17/06/2026 09:17 p. m.</t>
+          <t>17/06/2026 09:49 p. m.</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -1259,19 +1259,19 @@
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>Congresistas demócratas piden al Departamento de Justicia investigar a candidato De la Espriella</t>
+          <t>ICETEX ofrece becas del 50% para estudiar maestrías virtuales en España: Así puede postularse</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/18/congresistas-democratas-piden-al-departamento-de-justicia-investigar-a-candidato-de-la-espriella/</t>
+          <t>https://caracol.com.co/2026/06/18/icetex-ofrece-becas-del-50-para-estudiar-maestrias-virtuales-en-espana-asi-puede-postularse/</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>17/06/2026 08:04 p. m.</t>
+          <t>17/06/2026 09:17 p. m.</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1286,19 +1286,19 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>SENA ofrece curso virtual GRATUITO de cocina internacional: pasos para aplicar y LINK oficial</t>
+          <t>Congresistas demócratas piden al Departamento de Justicia investigar a candidato De la Espriella</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/18/sena-ofrece-curso-virtual-gratuito-de-cocina-internacional-pasos-para-aplicar-y-link-oficial/</t>
+          <t>https://caracol.com.co/2026/06/18/congresistas-democratas-piden-al-departamento-de-justicia-investigar-a-candidato-de-la-espriella/</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>17/06/2026 07:40 p. m.</t>
+          <t>17/06/2026 08:04 p. m.</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -1313,19 +1313,19 @@
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Tiroteo en Aeropuerto de Guayaquil deja al menos una persona muerta</t>
+          <t>SENA ofrece curso virtual GRATUITO de cocina internacional: pasos para aplicar y LINK oficial</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/18/tiroteo-en-aeropuerto-de-guayaquil-deja-al-menos-una-persona-muerta/</t>
+          <t>https://caracol.com.co/2026/06/18/sena-ofrece-curso-virtual-gratuito-de-cocina-internacional-pasos-para-aplicar-y-link-oficial/</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>17/06/2026 07:23 p. m.</t>
+          <t>17/06/2026 07:40 p. m.</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1340,19 +1340,19 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Supersalud detecta medicamentos disponibles en bodega que no estaban siendo entregados a usuarios</t>
+          <t>Tiroteo en Aeropuerto de Guayaquil deja al menos una persona muerta</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/18/supersalud-detecta-medicamentos-disponibles-en-bodega-que-no-estaban-siendo-entregados-a-usuarios/</t>
+          <t>https://caracol.com.co/2026/06/18/tiroteo-en-aeropuerto-de-guayaquil-deja-al-menos-una-persona-muerta/</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>17/06/2026 07:07 p. m.</t>
+          <t>17/06/2026 07:23 p. m.</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
@@ -1367,19 +1367,19 @@
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>Presidente Gustavo Petro reitera en que la EPS Coosalud, estaría  relacionada con lavado de activos</t>
+          <t>Supersalud detecta medicamentos disponibles en bodega que no estaban siendo entregados a usuarios</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/18/presidente-gustavo-petro-reitera-en-que-la-eps-coosalud-esta-relacionada-con-lavado-de-activos/</t>
+          <t>https://caracol.com.co/2026/06/18/supersalud-detecta-medicamentos-disponibles-en-bodega-que-no-estaban-siendo-entregados-a-usuarios/</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>17/06/2026 07:04 p. m.</t>
+          <t>17/06/2026 07:07 p. m.</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1394,19 +1394,19 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Medio día libre por votar: ¿es posible unir el beneficio de las dos vueltas electorales?</t>
+          <t>Presidente Gustavo Petro reitera en que la EPS Coosalud, estaría  relacionada con lavado de activos</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/18/medio-dia-libre-por-votar-es-posible-unir-el-beneficio-de-las-dos-vueltas-electorales/</t>
+          <t>https://caracol.com.co/2026/06/18/presidente-gustavo-petro-reitera-en-que-la-eps-coosalud-esta-relacionada-con-lavado-de-activos/</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>17/06/2026 06:49 p. m.</t>
+          <t>17/06/2026 07:04 p. m.</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
@@ -1421,19 +1421,19 @@
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>Embajada de Colombia interviene tras captura de Beto Coral y señala indicios de motivación política</t>
+          <t>Medio día libre por votar: ¿es posible unir el beneficio de las dos vueltas electorales?</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/17/embajada-de-colombia-interviene-tras-captura-de-beto-coral-y-senala-indicios-de-motivacion-politica/</t>
+          <t>https://caracol.com.co/2026/06/18/medio-dia-libre-por-votar-es-posible-unir-el-beneficio-de-las-dos-vueltas-electorales/</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>17/06/2026 06:35 p. m.</t>
+          <t>17/06/2026 06:49 p. m.</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1448,19 +1448,19 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Procuraduría indaga a Aerocivil y Enterritorio por fracaso de cuatro aeródromos prometidos por Petro</t>
+          <t>Embajada de Colombia interviene tras captura de Beto Coral y señala indicios de motivación política</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/17/procuraduria-indaga-a-la-aerocivil-por-fracaso-de-aeropuertos-rurales-del-gobierno-petro/</t>
+          <t>https://caracol.com.co/2026/06/17/embajada-de-colombia-interviene-tras-captura-de-beto-coral-y-senala-indicios-de-motivacion-politica/</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>17/06/2026 06:31 p. m.</t>
+          <t>17/06/2026 06:35 p. m.</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
@@ -1475,19 +1475,19 @@
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>¿Le faltan semanas para pensionarse? Puede usar sus ahorros BEPS de Colpensiones para completarlas</t>
+          <t>Procuraduría indaga a Aerocivil y Enterritorio por fracaso de cuatro aeródromos prometidos por Petro</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/17/le-faltan-semanas-para-pensionarse-puede-usar-sus-ahorros-beps-de-colpensiones-para-completarlas/</t>
+          <t>https://caracol.com.co/2026/06/17/procuraduria-indaga-a-la-aerocivil-por-fracaso-de-aeropuertos-rurales-del-gobierno-petro/</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>17/06/2026 06:13 p. m.</t>
+          <t>17/06/2026 06:31 p. m.</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -1502,19 +1502,19 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Maratón de Magdalena ingresa al calendario internacional de la Federación colombiana de Atletismo</t>
+          <t>¿Le faltan semanas para pensionarse? Puede usar sus ahorros BEPS de Colpensiones para completarlas</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/17/maraton-de-magdalena-ingresa-al-calendario-internacional-de-la-federacion-colombiana-de-atletismo/</t>
+          <t>https://caracol.com.co/2026/06/17/le-faltan-semanas-para-pensionarse-puede-usar-sus-ahorros-beps-de-colpensiones-para-completarlas/</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>17/06/2026 06:04 p. m.</t>
+          <t>17/06/2026 06:13 p. m.</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
@@ -1529,19 +1529,19 @@
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>Gobierno le baja el tono y reconocerá resultados electorales si “queda nítida la voluntad popular”</t>
+          <t>Maratón de Magdalena ingresa al calendario internacional de la Federación colombiana de Atletismo</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/17/gobierno-le-baja-el-tono-y-reconocera-resultados-electorales-si-queda-nitida-la-voluntad-popular/</t>
+          <t>https://caracol.com.co/2026/06/17/maraton-de-magdalena-ingresa-al-calendario-internacional-de-la-federacion-colombiana-de-atletismo/</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>17/06/2026 05:41 p. m.</t>
+          <t>17/06/2026 06:04 p. m.</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -1556,19 +1556,19 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>UNAD abrió inscripciones para Política de Gratuidad: Consulte requisitos y estudie GRATIS</t>
+          <t>Gobierno le baja el tono y reconocerá resultados electorales si “queda nítida la voluntad popular”</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/17/unad-abrio-inscripciones-para-politica-de-gratuidad-consulte-requisitos-y-estudie-gratis/</t>
+          <t>https://caracol.com.co/2026/06/17/gobierno-le-baja-el-tono-y-reconocera-resultados-electorales-si-queda-nitida-la-voluntad-popular/</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>17/06/2026 05:32 p. m.</t>
+          <t>17/06/2026 05:41 p. m.</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
@@ -1583,19 +1583,19 @@
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>Extienden por un año más la medida intramural contra presuntos asesinos de Sara Millerey González</t>
+          <t>UNAD abrió inscripciones para Política de Gratuidad: Consulte requisitos y estudie GRATIS</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/17/extienden-por-un-ano-mas-la-medida-intramural-contra-presuntos-asesinos-de-sara-millerey-gonzalez/</t>
+          <t>https://caracol.com.co/2026/06/17/unad-abrio-inscripciones-para-politica-de-gratuidad-consulte-requisitos-y-estudie-gratis/</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 06:13 a. m.</t>
+          <t>18/06/2026 08:12 a. m.</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -1610,19 +1610,19 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>Fuertes lluvias provocan inundaciones y emergencias en Segovia, Antioquia</t>
+          <t>Estados Unidos revela acuerdo de 14 puntos con Irán para el fin de la crisis</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/actualidad/fuertes-lluvias-provocan-inundaciones-y-emergencias-en-segovia-antioquia-402570</t>
+          <t>https://www.lafm.com.co/internacional/estados-unidos-revela-acuerdo-de-14-puntos-con-iran-para-el-fin-de-la-crisis-402572</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 05:28 a. m.</t>
+          <t>18/06/2026 06:13 a. m.</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
@@ -1637,19 +1637,19 @@
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>El detalle que preocupó a Néstor Lorenzo pese al triunfo de Colombia en su debut mundialista</t>
+          <t>Fuertes lluvias provocan inundaciones y emergencias en Segovia, Antioquia</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/deportes/nestor-lorenzo-rueda-de-prensa-colombia-uzbekistan-402569</t>
+          <t>https://www.lafm.com.co/actualidad/fuertes-lluvias-provocan-inundaciones-y-emergencias-en-segovia-antioquia-402570</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 04:35 a. m.</t>
+          <t>18/06/2026 05:28 a. m.</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -1664,12 +1664,12 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Colombia vs. Uzbekistán: Calificación y 1x1 de la 'Tricolor' en el arranque del Mundial 2026</t>
+          <t>El detalle que preocupó a Néstor Lorenzo pese al triunfo de Colombia en su debut mundialista</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/deportes/seleccion-colombia-calificacion-jugadores-debut-uzbekistan-mundial-2026-402568</t>
+          <t>https://www.lafm.com.co/deportes/nestor-lorenzo-rueda-de-prensa-colombia-uzbekistan-402569</t>
         </is>
       </c>
     </row>
@@ -1838,7 +1838,7 @@
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 01:04 a. m.</t>
+          <t>18/06/2026 01:39 a. m.</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
@@ -1853,19 +1853,19 @@
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>DIAN devolverá saldos a favor automáticamente en 2026: estos son los requisitos</t>
+          <t>¿Cuándo vuelve a jugar la Selección Colombia en el Mundial? Fecha, hora y rival tras la victoria ante Uzbekistán</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/economia/dian-devolvera-saldos-a-favor-2026-requisitos-402555</t>
+          <t>https://www.lafm.com.co/deportes/mundial-2026-cuando-juega-colombia-fecha-hora-partido-vs-republica-democratica-congo-402556</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 12:44 a. m.</t>
+          <t>18/06/2026 01:04 a. m.</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -1880,19 +1880,19 @@
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Agónica victoria de Ghana sobre Panamá; así fue el gol en la última del partido</t>
+          <t>DIAN devolverá saldos a favor automáticamente en 2026: estos son los requisitos</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/deportes/ghana-vs-panama-mundial-2026-fifa-resultado-mejores-momentos-grupo-l-402544</t>
+          <t>https://www.lafm.com.co/economia/dian-devolvera-saldos-a-favor-2026-requisitos-402555</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>17/06/2026 11:56 p. m.</t>
+          <t>18/06/2026 12:44 a. m.</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
@@ -1907,12 +1907,12 @@
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>“Yo nunca voy a emprender el camino de una constituyente si no hay un acuerdo entre todas las fuerzas del país”: Iván Cepeda</t>
+          <t>Agónica victoria de Ghana sobre Panamá; así fue el gol en la última del partido</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/entrevista-ivan-cepeda-noticias-rcn-abelardo-de-la-espriella-aida-quilcue-segunda-vuelta-402550</t>
+          <t>https://www.lafm.com.co/deportes/ghana-vs-panama-mundial-2026-fifa-resultado-mejores-momentos-grupo-l-402544</t>
         </is>
       </c>
     </row>
@@ -2038,12 +2038,12 @@
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Las cuentas de la Selección Colombia para clasificar tras victoria con Uzbekistán en el debut del Mundial 2026</t>
+          <t>Colombia vs. Uzbekistán: Calificación y 1x1 de la 'Tricolor' en el arranque del Mundial 2026</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/deportes/mundial-2026-cuentas-de-colombia-para-clasificar-402567</t>
+          <t>https://www.lafm.com.co/deportes/seleccion-colombia-calificacion-jugadores-debut-uzbekistan-mundial-2026-402568</t>
         </is>
       </c>
     </row>
@@ -2061,12 +2061,12 @@
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>¿Cuándo vuelve a jugar la Selección Colombia en el Mundial? Fecha, hora y rival tras la victoria ante Uzbekistán</t>
+          <t>Las cuentas de la Selección Colombia para clasificar tras victoria con Uzbekistán en el debut del Mundial 2026</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/deportes/mundial-2026-cuando-juega-colombia-fecha-hora-partido-vs-republica-democratica-congo-402556</t>
+          <t>https://www.lafm.com.co/deportes/mundial-2026-cuentas-de-colombia-para-clasificar-402567</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 02:43 a. m.</t>
+          <t>18/06/2026 04:28 a. m.</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -2134,19 +2134,19 @@
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>¿Para qué sirve la escuela cuando la información está a un clic?</t>
+          <t>El discurso de Tüchel que liberó a Inglaterra ante Croacia: “Nos dijo que nos calmáramos, que le enseñáramos al mundo quiénes podemos ser”</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/economia/formacion/2026-06-18/para-que-sirve-la-escuela-cuando-la-informacion-esta-a-un-clic.html</t>
+          <t>https://elpais.com/deportes/mundial-futbol/2026-06-18/el-discurso-de-tuchel-que-libero-a-inglaterra-ante-croacia-nos-dijo-que-nos-calmaramos-que-le-ensenaramos-al-mundo-quienes-podemos-ser.html</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 02:42 a. m.</t>
+          <t>18/06/2026 04:27 a. m.</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
@@ -2161,19 +2161,19 @@
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
-          <t>Decenas de páginas que narraban tragedias quedaron esparcidas sobre las vías del tren en Adamuz</t>
+          <t>Anna Castillo habla de la bifobia que sufrió cuando empezó con Álvaro Mel: “Mi insulto favorito siempre fue ‘bollera traicionera”</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/espana/andalucia/2026-06-18/decenas-de-paginas-que-narraban-tragedias-quedaron-esparcidas-sobre-las-vias-del-tren-en-adamuz.html</t>
+          <t>https://elpais.com/gente/2026-06-18/anna-castillo-habla-de-la-bifobia-que-sufrio-cuando-empezo-con-alvaro-mel-mi-insulto-favorito-siempre-fue-bollera-traicionera.html</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 02:32 a. m.</t>
+          <t>18/06/2026 04:23 a. m.</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -2188,19 +2188,19 @@
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Resumen de la jornada del 18 de junio del Mundial 2026: Inglaterra vence a Croacia y Portugal no pasa del empate</t>
+          <t>El Real Madrid hace oficial el fichaje de Konaté por cuatro temporadas</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/deportes/mundial-futbol/2026-06-17/resumen-y-ultimas-noticias-de-la-copa-mundial-de-futbol.html</t>
+          <t>https://elpais.com/deportes/2026-06-18/el-real-madrid-hace-oficial-el-fichaje-de-konate-por-cuatro-temporadas.html</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 02:29 a. m.</t>
+          <t>18/06/2026 04:20 a. m.</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
@@ -2215,19 +2215,19 @@
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>Resumen y últimas noticias de la Copa Mundial de fútbol</t>
+          <t>EE UU lanza una revisión de su presencia militar en Europa y del compromiso de los aliados con Trump</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/deportes/mundial-futbol/2026-06-18/resumen-y-ultimas-noticias-de-la-copa-mundial-de-futbol.html</t>
+          <t>https://elpais.com/internacional/2026-06-18/ee-uu-lanza-una-revision-de-su-presencia-militar-en-europa-y-del-compromiso-de-los-aliados-con-trump.html</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 02:26 a. m.</t>
+          <t>18/06/2026 04:18 a. m.</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -2242,19 +2242,19 @@
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Carles Lalueza-Fox, genetista: “Todos tenemos más de un doble en algún lugar del planeta”</t>
+          <t>Israel rompe “todo contacto” con la jefa de la diplomacia de la UE, Kaja Kallas</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/ciencia/2026-06-18/carles-lalueza-fox-genetista-todos-tenemos-mas-de-un-doble-en-algun-lugar-del-planeta.html</t>
+          <t>https://elpais.com/internacional/2026-06-18/israel-rompe-todo-contacto-con-la-jefa-de-la-diplomacia-europea-kaja-kallas.html</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 02:18 a. m.</t>
+          <t>18/06/2026 03:50 a. m.</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr">
@@ -2269,19 +2269,19 @@
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>La pareja de Pérez Llorca no se presentará a la renovación de la plaza en la Diputación de Valencia por la que cobraba 52.070 euros</t>
+          <t>El sector inmobiliario como impulso a la regeneración urbana</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/espana/comunidad-valenciana/2026-06-18/la-pareja-de-perez-llorca-no-se-presentara-a-la-renovacion-de-la-plaza-en-la-diputacion-por-la-que-cobraba-52070-euros.html</t>
+          <t>https://elpais.com/economia/negocios/2026-06-18/el-sector-inmobiliario-como-impulso-a-la-regeneracion-urbana.html</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 02:17 a. m.</t>
+          <t>18/06/2026 03:48 a. m.</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -2296,19 +2296,19 @@
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>Un incendio en una nave de trasteros de Madrid provoca una gran columna de humo y obliga a desalojar una gasolinera</t>
+          <t>Mundial 2026, últimas noticias en directo | Comienza la segunda jornada de la Copa del Mundo</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/espana/madrid/2026-06-18/un-incendio-en-una-nave-de-trasteros-de-madrid-provoca-una-gran-columna-de-humo-y-obliga-a-desalojar-una-gasolinera.html</t>
+          <t>https://elpais.com/deportes/mundial-futbol/2026-06-18/resumen-y-ultimas-noticias-de-la-copa-mundial-de-futbol.html</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 02:12 a. m.</t>
+          <t>18/06/2026 03:22 a. m.</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
@@ -2323,19 +2323,19 @@
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>Román, elegido triunfador de San Isidro por la Unión de Abonados y el Real Casino de Madrid</t>
+          <t>Ayuso pide “corresponsabilidad financiera” al resto de regiones para que sus ciudadanos tengan la tarjeta de transportes de Madrid</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/cultura/2026-06-18/roman-elegido-triunfador-de-san-isidro-por-la-union-de-abonados-y-el-real-casino-de-madrid.html</t>
+          <t>https://elpais.com/espana/madrid/2026-06-18/ayuso-pide-corresponsabilidad-financiera-al-resto-de-regiones-para-que-sus-ciudadanos-tengan-la-tarjeta-de-transportes-de-madrid.html</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 02:12 a. m.</t>
+          <t>18/06/2026 03:20 a. m.</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -2350,19 +2350,19 @@
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>Néstor Lorenzo celebra la victoria de Colombia, pero exige más contundencia a sus jugadores</t>
+          <t>Fallece de cáncer Eric Roy, entrenador del Brest y exjugador del Rayo Vallecano</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/america-colombia/2026-06-18/nestor-lorenzo-celebra-la-victoria-de-colombia-pero-exige-mas-contundencia-a-sus-jugadores.html</t>
+          <t>https://elpais.com/deportes/2026-06-18/fallece-de-cancer-eric-roy-entrenador-del-brest-y-exjugador-del-rayo-vallecano.html</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 12:27 a. m.</t>
+          <t>18/06/2026 03:18 a. m.</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr">
@@ -2377,19 +2377,19 @@
       </c>
       <c r="D71" s="6" t="inlineStr">
         <is>
-          <t>Última hora de la actualidad política, en directo</t>
+          <t>Si n’aprens, n’aprens, i si no, no (dels llibres que expliquen com s’escriu o com no s’escriu)</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/espana/2026-06-18/ultima-hora-de-la-actualidad-politica-en-directo.html</t>
+          <t>https://elpais.com/quadern/2026-06-18/si-naprens-naprens-i-si-no-no-dels-llibres-que-expliquen-com-sescriu-o-com-no-sescriu.html</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 12:25 a. m.</t>
+          <t>18/06/2026 03:13 a. m.</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -2404,19 +2404,19 @@
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>He probado cuatro dispositivos de ‘peeling’ ultrasónico y pocas veces he tenido la piel tan limpia</t>
+          <t>La Fiscalía investiga a Pilar Rahola por incitación al odio por su defensa de Israel</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/hemeroteca/2026-06-18/</t>
+          <t>https://elpais.com/espana/catalunya/2026-06-18/la-fiscalia-investiga-a-pilar-rahola-por-incitacion-al-odio-por-su-defensa-de-israel.html</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 12:02 a. m.</t>
+          <t>18/06/2026 03:11 a. m.</t>
         </is>
       </c>
       <c r="B73" s="5" t="inlineStr">
@@ -2431,19 +2431,19 @@
       </c>
       <c r="D73" s="6" t="inlineStr">
         <is>
-          <t>El Mundial empuja de vuelta a la mesa al Gobierno y a la CNTE, pero no acercan posturas</t>
+          <t>Entradas para Quevedo en Madrid y Barcelona: guía de la venta general, precios y fechas</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/mexico/2026-06-18/el-mundial-empuja-de-vuelta-a-la-mesa-al-gobierno-y-a-la-cnte-pero-no-acercan-posturas.html</t>
+          <t>https://elpais.com/cultura/2026-06-18/entradas-para-quevedo-en-madrid-y-barcelona-guia-de-la-venta-general-precios-y-fechas.html</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 12:01 a. m.</t>
+          <t>18/06/2026 03:09 a. m.</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -2458,19 +2458,19 @@
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>Maluma y un tsunami amarillo aúpan a Colombia en su regreso a los Mundiales</t>
+          <t>Sabrina Carpenter obtiene una orden de alejamiento de cinco años contra su presunto acosador</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/america-colombia/2026-06-18/maluma-y-un-tsunami-amarillo-aupan-a-colombia-en-su-regreso-a-los-mundiales.html</t>
+          <t>https://elpais.com/gente/2026-06-18/sabrina-carpenter-obtiene-una-orden-de-alejamiento-de-cinco-anos-contra-su-presunto-acosador.html</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 12:00 a. m.</t>
+          <t>18/06/2026 03:07 a. m.</t>
         </is>
       </c>
       <c r="B75" s="5" t="inlineStr">
@@ -2485,19 +2485,19 @@
       </c>
       <c r="D75" s="6" t="inlineStr">
         <is>
-          <t>Valencia Basket - Barcelona, horario del partido final de la Liga ACB</t>
+          <t>Ucrania golpea de nuevo la mayor refinería de Moscú y causa una gran humareda en la ciudad</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/deportes/baloncesto/2026-06-18/valencia-basket-barcelona-horario-del-partido-final-de-la-liga-acb.html</t>
+          <t>https://elpais.com/internacional/2026-06-18/ucrania-golpea-de-nuevo-la-mayor-refineria-de-moscu-y-causa-una-gran-humareda-en-la-ciudad.html</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>17/06/2026 11:35 p. m.</t>
+          <t>18/06/2026 03:04 a. m.</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -2512,19 +2512,19 @@
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>Kast convoca a los tres poderes del Estado para coordinar la búsqueda de más de 200 niños haitianos a los que Chile les perdió el rastro</t>
+          <t>Patti Smith declara su amor por Rosalía (otra vez): “Conquistó un corazón que ya estaba conquistado”</t>
         </is>
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/chile/2026-06-18/kast-convoca-a-los-tres-poderes-del-estado-para-coordinar-la-busqueda-de-mas-de-200-ninos-haitianos-a-los-que-chile-les-perdio-el-rastro.html</t>
+          <t>https://elpais.com/cultura/2026-06-18/patti-smith-declara-su-amor-por-rosalia-otra-vez-conquisto-un-corazon-que-ya-estaba-conquistado.html</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>17/06/2026 11:22 p. m.</t>
+          <t>18/06/2026 02:53 a. m.</t>
         </is>
       </c>
       <c r="B77" s="5" t="inlineStr">
@@ -2539,19 +2539,19 @@
       </c>
       <c r="D77" s="6" t="inlineStr">
         <is>
-          <t>Colombia tiene su fiesta en el Azteca con un triunfo ante Uzbekistán</t>
+          <t>Movistar Plus renueva ‘Se tiene que morir mucha gente’ por una segunda temporada</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/america-colombia/2026-06-18/colombia-tiene-su-fiesta-en-el-azteca-con-un-triunfo-ante-uzbekistan.html</t>
+          <t>https://elpais.com/television/series/2026-06-18/movistar-plus-renueva-se-tiene-que-morir-mucha-gente-por-una-segunda-temporada.html</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>17/06/2026 11:21 p. m.</t>
+          <t>18/06/2026 02:26 a. m.</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -2566,12 +2566,12 @@
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>Los manifestantes en Bolivia exigen la libertad de los sindicalistas presos para levantar las protestas</t>
+          <t>Carles Lalueza-Fox, genetista: “Todos tenemos más de un doble en algún lugar del planeta”</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/america/2026-06-18/los-manifestantes-en-bolivia-exigen-la-libertad-de-los-sindicalistas-presos-para-levantar-las-protestas.html</t>
+          <t>https://elpais.com/ciencia/2026-06-18/carles-lalueza-fox-genetista-todos-tenemos-mas-de-un-doble-en-algun-lugar-del-planeta.html</t>
         </is>
       </c>
     </row>
@@ -2728,7 +2728,7 @@
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>Diez universidades españolas debutan en el ranking mundial QS que escoge a las 1.500 mejores</t>
+          <t>Diez universidades españolas debutan en el ‘ranking’ mundial QS que escoge a las 1.500 mejores</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
@@ -2936,12 +2936,12 @@
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>No es una elección cualquiera</t>
+          <t>El avión que nunca despegó</t>
         </is>
       </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/18/no-es-una-eleccion-cualquiera/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/18/el-avion-que-nunca-despego/</t>
         </is>
       </c>
     </row>
@@ -2990,12 +2990,12 @@
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>¿Comité para la defensa de qué?</t>
+          <t>No es una elección cualquiera</t>
         </is>
       </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/18/comite-para-la-defensa-de-que/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/18/no-es-una-eleccion-cualquiera/</t>
         </is>
       </c>
     </row>
@@ -3017,12 +3017,12 @@
       </c>
       <c r="D95" s="6" t="inlineStr">
         <is>
-          <t>Maniqueísmos</t>
+          <t>Hay que votar para salvar a Colombia</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/18/maniqueismos/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/18/hay-que-votar-para-salvar-a-colombia/</t>
         </is>
       </c>
     </row>
@@ -3044,12 +3044,12 @@
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>Hay que votar para salvar a Colombia</t>
+          <t>¿Comité para la defensa de qué?</t>
         </is>
       </c>
       <c r="E96" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/18/hay-que-votar-para-salvar-a-colombia/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/18/comite-para-la-defensa-de-que/</t>
         </is>
       </c>
     </row>
@@ -3530,12 +3530,12 @@
       </c>
       <c r="D114" s="3" t="inlineStr">
         <is>
-          <t>Ciudadanos responsables: antes, durante y después de la elección</t>
+          <t>Votar responsablemente por la nación</t>
         </is>
       </c>
       <c r="E114" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/columnista-invitado-ee/ciudadanos-responsables-antes-durante-y-despues-de-la-eleccion/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/javier-ortiz/votar-responsablemente-por-la-nacion/</t>
         </is>
       </c>
     </row>
@@ -3557,12 +3557,12 @@
       </c>
       <c r="D115" s="6" t="inlineStr">
         <is>
-          <t>El pato cojo</t>
+          <t>Tiempo de ruptura</t>
         </is>
       </c>
       <c r="E115" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/cristinacarrizosa/el-pato-cojo/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/brigitte-lg-baptiste/tiempo-de-ruptura/</t>
         </is>
       </c>
     </row>
@@ -3584,12 +3584,12 @@
       </c>
       <c r="D116" s="3" t="inlineStr">
         <is>
-          <t>Tiempo de ruptura</t>
+          <t>Ciudadanos responsables: antes, durante y después de la elección</t>
         </is>
       </c>
       <c r="E116" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/brigitte-lg-baptiste/tiempo-de-ruptura/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/columnista-invitado-ee/ciudadanos-responsables-antes-durante-y-despues-de-la-eleccion/</t>
         </is>
       </c>
     </row>
@@ -3611,12 +3611,12 @@
       </c>
       <c r="D117" s="6" t="inlineStr">
         <is>
-          <t>Votar responsablemente por la nación</t>
+          <t>El pato cojo</t>
         </is>
       </c>
       <c r="E117" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/javier-ortiz/votar-responsablemente-por-la-nacion/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/cristinacarrizosa/el-pato-cojo/</t>
         </is>
       </c>
     </row>
@@ -4691,12 +4691,12 @@
       </c>
       <c r="D157" s="6" t="inlineStr">
         <is>
-          <t>CNE levanta definitivamente las restricciones a AtlasIntel y permite la publicación de encuestas electorales</t>
+          <t>Yeferson Cossio ganó una millonaria apuesta por la Selección Colombia y prometió donar 200 millones a fundaciones de perros</t>
         </is>
       </c>
       <c r="E157" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/18/cne-levanta-definitivamente-las-restricciones-a-atlasintel-y-permite-la-publicacion-de-encuestas-electorales/</t>
+          <t>https://www.infobae.com/colombia/2026/06/18/yeferson-cossio-gano-una-millonaria-apuesta-por-la-seleccion-colombia-y-prometio-donar-200-millones-a-fundaciones-de-perros/</t>
         </is>
       </c>
     </row>
@@ -4718,12 +4718,12 @@
       </c>
       <c r="D158" s="3" t="inlineStr">
         <is>
-          <t>Supersalud halló medicamentos en bodega que no eran entregados a usuarios de Famisanar</t>
+          <t>Pronóstico del estado del tiempo: las temperaturas que se esperan en Cartagena de Indias este 18 de junio</t>
         </is>
       </c>
       <c r="E158" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/18/supersalud-hallo-medicamentos-en-bodega-que-no-eran-entregados-a-usuarios-de-famisanar/</t>
+          <t>https://www.infobae.com/colombia/2026/06/18/pronostico-del-estado-del-tiempo-las-temperaturas-que-se-esperan-en-cartagena-de-indias-este-18-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4745,12 +4745,12 @@
       </c>
       <c r="D159" s="6" t="inlineStr">
         <is>
-          <t>Pico y Placa en Bogotá: restricciones vehiculares para evitar multas este jueves</t>
+          <t>Adiós a la incertidumbre, conoce las condiciones climáticas en Barranquilla</t>
         </is>
       </c>
       <c r="E159" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/18/pico-y-placa-en-bogota-restricciones-vehiculares-para-evitar-multas-este-jueves/</t>
+          <t>https://www.infobae.com/colombia/2026/06/18/adios-a-la-incertidumbre-conoce-las-condiciones-climaticas-en-barranquilla/</t>
         </is>
       </c>
     </row>
@@ -4772,12 +4772,12 @@
       </c>
       <c r="D160" s="3" t="inlineStr">
         <is>
-          <t>Elecciones presidenciales de Colombia 2026 en VIVO: Trump acusa de “marxista” a Iván Cepeda y respalda a De la Espriella en la segunda vuelta</t>
+          <t>Cali: el pronóstico del tiempo para este 18 de junio</t>
         </is>
       </c>
       <c r="E160" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/18/elecciones-presidenciales-de-colombia-2026-en-vivo-ivan-cepeda-insiste-en-debatir-con-abelardo-de-la-espriella/</t>
+          <t>https://www.infobae.com/colombia/2026/06/18/cali-el-pronostico-del-tiempo-para-este-18-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4799,12 +4799,12 @@
       </c>
       <c r="D161" s="6" t="inlineStr">
         <is>
-          <t>Los mejores memes de la victoria de Colombia ante Uzbekistán en el Mundial 2026: las redes no perdonaron a James Rodríguez y Camilo Vargas</t>
+          <t>Clima en Colombia: el estado del tiempo para Medellín este 18 de junio</t>
         </is>
       </c>
       <c r="E161" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/06/18/los-mejores-memes-de-la-victoria-de-colombia-ante-uzbekistan-en-el-mundial-2026-las-redes-no-perdonaron-a-james-rodriguez-y-camilo-vargas/</t>
+          <t>https://www.infobae.com/colombia/2026/06/18/clima-en-colombia-el-estado-del-tiempo-para-medellin-este-18-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4826,12 +4826,12 @@
       </c>
       <c r="D162" s="3" t="inlineStr">
         <is>
-          <t>Factura electrónica en 2025: así aplica el descuento en la declaración de renta en Colombia</t>
+          <t>Pronóstico del clima: las temperaturas que se esperan en Bogotá este 18 de junio</t>
         </is>
       </c>
       <c r="E162" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/18/factura-electronica-en-2025-asi-aplica-el-descuento-en-la-declaracion-de-renta-en-colombia/</t>
+          <t>https://www.infobae.com/colombia/2026/06/18/pronostico-del-clima-las-temperaturas-que-se-esperan-en-bogota-este-18-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4853,12 +4853,12 @@
       </c>
       <c r="D163" s="6" t="inlineStr">
         <is>
-          <t>Baloto y Revancha: números ganadores del miércoles 17 de junio</t>
+          <t>FNA hará jornada nacional para destrabar créditos de vivienda aprobados del 25 al 27 de junio</t>
         </is>
       </c>
       <c r="E163" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/18/baloto-y-revancha-numeros-ganadores-del-miercoles-17-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/18/fna-hara-jornada-nacional-para-destrabar-creditos-de-vivienda-aprobados-del-25-al-27-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4880,12 +4880,12 @@
       </c>
       <c r="D164" s="3" t="inlineStr">
         <is>
-          <t>“No vamos a permitir que este país se incendie”: autoridades piden respetar resultado electoral</t>
+          <t>La autocrítica de Néstor Lorenzo pese al triunfo de Colombia 3-1 sobre Uzbekistán: “Hay que mejorar”</t>
         </is>
       </c>
       <c r="E164" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/18/no-vamos-a-permitir-que-este-pais-se-incendie-autoridades-piden-respetar-resultado-electoral/</t>
+          <t>https://www.infobae.com/colombia/deportes/2026/06/18/la-autocritica-de-nestor-lorenzo-pese-al-triunfo-de-colombia-3-1-sobre-uzbekistan-hay-que-mejorar/</t>
         </is>
       </c>
     </row>
@@ -4907,12 +4907,12 @@
       </c>
       <c r="D165" s="6" t="inlineStr">
         <is>
-          <t>Déficit y crisis de confianza: sector salud pide plan de emergencia al próximo gobierno</t>
+          <t>Resultado Sinuano Noche hoy 17 de junio</t>
         </is>
       </c>
       <c r="E165" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/18/deficit-y-crisis-de-confianza-sector-salud-pide-plan-de-emergencia-al-proximo-gobierno/</t>
+          <t>https://www.infobae.com/colombia/2026/06/18/resultado-sinuano-noche-hoy-17-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4934,12 +4934,12 @@
       </c>
       <c r="D166" s="3" t="inlineStr">
         <is>
-          <t>Lotería del Valle resultados 17 de junio: números ganadores del premio mayor y los 30 secos millonarios</t>
+          <t>CNE levanta definitivamente las restricciones a AtlasIntel y permite la publicación de encuestas electorales</t>
         </is>
       </c>
       <c r="E166" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/18/loteria-del-valle-resultados-17-de-junio-numeros-ganadores-del-premio-mayor-y-los-30-secos-millonarios/</t>
+          <t>https://www.infobae.com/colombia/2026/06/18/cne-levanta-definitivamente-las-restricciones-a-atlasintel-y-permite-la-publicacion-de-encuestas-electorales/</t>
         </is>
       </c>
     </row>
@@ -4961,12 +4961,12 @@
       </c>
       <c r="D167" s="6" t="inlineStr">
         <is>
-          <t>Luis Díaz debutó con gol y asistencia en un Mundial: así va en la lista de máximos goleadores de la Selección Colombia</t>
+          <t>Supersalud halló medicamentos en bodega que no eran entregados a usuarios de Famisanar</t>
         </is>
       </c>
       <c r="E167" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/06/18/luis-diaz-debuto-con-gol-y-asistencia-en-un-mundial-asi-va-en-la-lista-de-maximos-goleadores-de-la-seleccion-colombia/</t>
+          <t>https://www.infobae.com/colombia/2026/06/18/supersalud-hallo-medicamentos-en-bodega-que-no-eran-entregados-a-usuarios-de-famisanar/</t>
         </is>
       </c>
     </row>
@@ -4988,12 +4988,12 @@
       </c>
       <c r="D168" s="3" t="inlineStr">
         <is>
-          <t>Reviva los goles de la Selección Colombia ante Uzbekistán en su debut en el Mundial 2026: la Tricolor sufrió, reaccionó y festejó</t>
+          <t>Pico y Placa en Bogotá: restricciones vehiculares para evitar multas este jueves</t>
         </is>
       </c>
       <c r="E168" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/06/18/reviva-los-goles-de-la-seleccion-colombia-ante-uzbekistan-en-su-debut-en-el-mundial-2026-la-tricolor-sufrio-reacciono-y-festejo/</t>
+          <t>https://www.infobae.com/colombia/2026/06/18/pico-y-placa-en-bogota-restricciones-vehiculares-para-evitar-multas-este-jueves/</t>
         </is>
       </c>
     </row>
@@ -5015,12 +5015,12 @@
       </c>
       <c r="D169" s="6" t="inlineStr">
         <is>
-          <t>Lotería de Manizales resultados miércoles 17 de junio: quién ganó el premio mayor de $2.600 millones</t>
+          <t>Elecciones presidenciales de Colombia 2026 en VIVO: Trump acusa de “marxista” a Iván Cepeda y respalda a De la Espriella en la segunda vuelta</t>
         </is>
       </c>
       <c r="E169" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/18/loteria-de-manizales-resultados-miercoles-17-de-junio-quien-gano-el-premio-mayor-de-2600-millones/</t>
+          <t>https://www.infobae.com/colombia/2026/06/18/elecciones-presidenciales-de-colombia-2026-en-vivo-ivan-cepeda-insiste-en-debatir-con-abelardo-de-la-espriella/</t>
         </is>
       </c>
     </row>
@@ -5042,12 +5042,12 @@
       </c>
       <c r="D170" s="3" t="inlineStr">
         <is>
-          <t>Así celebraron los colombianos la victoria 3-1 de la Tricolor en su debut mundialista</t>
+          <t>Los mejores memes de la victoria de Colombia ante Uzbekistán en el Mundial 2026: las redes no perdonaron a James Rodríguez y Camilo Vargas</t>
         </is>
       </c>
       <c r="E170" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/06/18/asi-celebraron-los-colombianos-la-victoria-3-1-de-la-seleccion-colombia-en-su-debut-mundialista/</t>
+          <t>https://www.infobae.com/colombia/deportes/2026/06/18/los-mejores-memes-de-la-victoria-de-colombia-ante-uzbekistan-en-el-mundial-2026-las-redes-no-perdonaron-a-james-rodriguez-y-camilo-vargas/</t>
         </is>
       </c>
     </row>
@@ -5069,12 +5069,12 @@
       </c>
       <c r="D171" s="6" t="inlineStr">
         <is>
-          <t>Congreso aprueba bonificación judicial como factor salarial: más de 36.000 servidores públicos serán beneficiados</t>
+          <t>Factura electrónica en 2025: así aplica el descuento en la declaración de renta en Colombia</t>
         </is>
       </c>
       <c r="E171" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/18/congreso-aprueba-bonificacion-judicial-como-factor-salarial-mas-de-36000-servidores-publicos-seran-beneficiados/</t>
+          <t>https://www.infobae.com/colombia/2026/06/18/factura-electronica-en-2025-asi-aplica-el-descuento-en-la-declaracion-de-renta-en-colombia/</t>
         </is>
       </c>
     </row>
@@ -5096,12 +5096,12 @@
       </c>
       <c r="D172" s="3" t="inlineStr">
         <is>
-          <t>Resultados Baloto y Revancha, último sorteo del lunes 15 de junio</t>
+          <t>Baloto y Revancha: números ganadores del miércoles 17 de junio</t>
         </is>
       </c>
       <c r="E172" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/18/resultados-baloto-y-revancha-ultimo-sorteo-del-lunes-15-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/18/baloto-y-revancha-numeros-ganadores-del-miercoles-17-de-junio/</t>
         </is>
       </c>
     </row>
@@ -5123,12 +5123,12 @@
       </c>
       <c r="D173" s="6" t="inlineStr">
         <is>
-          <t>Resultado Super Astro Luna HOY: número ganador del miércoles 17 de junio</t>
+          <t>“No vamos a permitir que este país se incendie”: autoridades piden respetar resultado electoral</t>
         </is>
       </c>
       <c r="E173" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/18/resultado-super-astro-luna-hoy-numero-ganador-del-miercoles-17-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/18/no-vamos-a-permitir-que-este-pais-se-incendie-autoridades-piden-respetar-resultado-electoral/</t>
         </is>
       </c>
     </row>
@@ -5150,12 +5150,12 @@
       </c>
       <c r="D174" s="3" t="inlineStr">
         <is>
-          <t>Daniel Muñoz, Luis Díaz y Jáminton Campaz le dieron una sufrida victoria a Colombia en su estreno en el Mundial 2026</t>
+          <t>Déficit y crisis de confianza: sector salud pide plan de emergencia al próximo gobierno</t>
         </is>
       </c>
       <c r="E174" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/06/18/daniel-munoz-luis-diaz-y-jaminton-campaz-le-dieron-una-sufrida-victoria-a-colombia-en-su-estreno-en-el-mundial-2026/</t>
+          <t>https://www.infobae.com/colombia/2026/06/18/deficit-y-crisis-de-confianza-sector-salud-pide-plan-de-emergencia-al-proximo-gobierno/</t>
         </is>
       </c>
     </row>
@@ -5177,19 +5177,19 @@
       </c>
       <c r="D175" s="6" t="inlineStr">
         <is>
-          <t>“Con votos, no con amenazas”: Consejo Gremial pide respetar resultado de segunda vuelta electoral en Colombia</t>
+          <t>Lotería del Valle resultados 17 de junio: números ganadores del premio mayor y los 30 secos millonarios</t>
         </is>
       </c>
       <c r="E175" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/18/con-votos-no-con-amenazas-consejo-gremial-pide-respetar-resultado-de-segunda-vuelta-electoral-en-colombia/</t>
+          <t>https://www.infobae.com/colombia/2026/06/18/loteria-del-valle-resultados-17-de-junio-numeros-ganadores-del-premio-mayor-y-los-30-secos-millonarios/</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>17/06/2026 12:00 a. m.</t>
+          <t>18/06/2026 12:00 a. m.</t>
         </is>
       </c>
       <c r="B176" s="2" t="inlineStr">
@@ -5204,12 +5204,12 @@
       </c>
       <c r="D176" s="3" t="inlineStr">
         <is>
-          <t>La Selección Colombia debutó con victoria en el Mundial 2026: triunfo 3-1 sobre Uzbekistán en Ciudad de México</t>
+          <t>Luis Díaz debutó con gol y asistencia en un Mundial: así va en la lista de máximos goleadores de la Selección Colombia</t>
         </is>
       </c>
       <c r="E176" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/17/seleccion-colombia-vs-uzbekistan-en-vivo-siga-el-minuto-a-minuto-del-debut-en-el-grupo-k-del-mundial-2026/</t>
+          <t>https://www.infobae.com/colombia/deportes/2026/06/18/luis-diaz-debuto-con-gol-y-asistencia-en-un-mundial-asi-va-en-la-lista-de-maximos-goleadores-de-la-seleccion-colombia/</t>
         </is>
       </c>
     </row>
@@ -6884,17 +6884,17 @@
       </c>
       <c r="C243" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D243" s="6" t="inlineStr">
         <is>
-          <t>Colombia bailó al son de Luis Díaz y le ganó a Uzbekistán: tres puntos y paso firme en el Mundial 2026</t>
+          <t>Colombia vs Uzbekistán: la Tricolor debutó con victoria 3-1</t>
         </is>
       </c>
       <c r="E243" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/colombia-bailo-al-son-de-luis-diaz-y-le-gano-a-uzbekistan-tres-puntos-y-paso-firme-en-el-mundial-2026/202625/</t>
+          <t>https://canaltrece.com.co/noticias/colombia-vs-uzbekistan-mundial-2026/</t>
         </is>
       </c>
     </row>
@@ -6907,17 +6907,17 @@
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D244" s="3" t="inlineStr">
         <is>
-          <t>Colombia vs. RD Congo, próximo partido de la Tricolor en el Mundial 2026: fecha y hora confirmadas</t>
+          <t>Morat Tu Cárcel alcanza el No. 1 en Billboard Latin Airplay</t>
         </is>
       </c>
       <c r="E244" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/colombia-vs-rd-congo-proximo-partido-de-la-tricolor-en-el-mundial-2026-fecha-y-hora-confirmadas/202659/</t>
+          <t>https://canaltrece.com.co/noticias/morat-tu-carcel-billboard/</t>
         </is>
       </c>
     </row>
@@ -6930,17 +6930,17 @@
       </c>
       <c r="C245" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D245" s="6" t="inlineStr">
         <is>
-          <t>El gol de Jaminton Campaz que liquidó a Uzbekistán: locura en Colombia tras la jugada del Cucho Hernández</t>
+          <t>Colombia vs Uzbekistán: así terminó el primer tiempo del debut</t>
         </is>
       </c>
       <c r="E245" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/el-gol-de-jaminton-campaz-que-liquido-a-uzbekistan-locura-en-colombia-tras-la-jugada-del-cucho-hernandez/202642/</t>
+          <t>https://canaltrece.com.co/noticias/colombia-vs-uzbekistan/</t>
         </is>
       </c>
     </row>
@@ -6953,17 +6953,17 @@
       </c>
       <c r="C246" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D246" s="3" t="inlineStr">
         <is>
-          <t>Magistral jugada de Luis Díaz que resuena en el Mundial 2026: magia ante Uzbekistán es viral</t>
+          <t>Penelope Robin inicia una nueva etapa con Diosa de Cien Colores</t>
         </is>
       </c>
       <c r="E246" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/magistral-jugada-de-luis-diaz-que-resuena-en-el-mundial-2026-magia-ante-uzbekistan-es-viral-en-el-mundo/202652/</t>
+          <t>https://canaltrece.com.co/noticias/penelope-robin-diosa-de-cien-colores/</t>
         </is>
       </c>
     </row>
@@ -6976,17 +6976,17 @@
       </c>
       <c r="C247" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D247" s="6" t="inlineStr">
         <is>
-          <t>Tabla de posiciones en el grupo K del Mundial 2026: Colombia vence a Uzbekistán y lanza aviso a Portugal</t>
+          <t>Narra Tu Territorio abre segundo corte tras recibir 764 propuestas</t>
         </is>
       </c>
       <c r="E247" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/tabla-de-posiciones-en-el-grupo-k-del-mundial-2026-colombia-vence-a-uzbekistan-y-lanza-aviso-a-portugal/202608/</t>
+          <t>https://canaltrece.com.co/noticias/narra-tu-territorio-segundo-corte/</t>
         </is>
       </c>
     </row>
@@ -6999,17 +6999,17 @@
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D248" s="3" t="inlineStr">
         <is>
-          <t>La reacción de Lorenzo tras la victoria ante Uzbekistán con tres goles en el Mundial 2026: “Hay que mejorar”</t>
+          <t>Colombia vs Uzbekistán: fecha, hora, estadio y dónde ver</t>
         </is>
       </c>
       <c r="E248" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/la-reaccion-de-lorenzo-tras-la-victoria-ante-uzbekistan-con-tres-goles-en-el-mundial-2026-hay-que-mejorar/202635/</t>
+          <t>https://canaltrece.com.co/noticias/colombia-vs-uzbekistan-fecha-hora-estadio-y-donde-ver/</t>
         </is>
       </c>
     </row>
@@ -7022,17 +7022,17 @@
       </c>
       <c r="C249" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D249" s="6" t="inlineStr">
         <is>
-          <t>Blooper de Camilo Vargas, pero Luis Díaz lo salvó: momento sublime de Colombia que resuena en el Mundial 2026</t>
+          <t>Fanzones en Bogotá para ver a Colombia: boletas y horarios</t>
         </is>
       </c>
       <c r="E249" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/blooper-de-camilo-vargas-pero-luis-diaz-lo-salvo-momento-sublime-de-colombia-que-resuena-en-el-mundial-2026/202653/</t>
+          <t>https://canaltrece.com.co/noticias/fanzones-en-bogota-para-ver-a-colombia-boletas-y-horarios/</t>
         </is>
       </c>
     </row>
@@ -7045,17 +7045,17 @@
       </c>
       <c r="C250" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D250" s="3" t="inlineStr">
         <is>
-          <t>Daniel Muñoz marcó el primer golazo de Colombia en el Mundial 2026: excelsa asistencia de Luis Díaz</t>
+          <t>¿Estreno hoy? Todo sobre la llegada de Toy Story 5 a las salas de cine</t>
         </is>
       </c>
       <c r="E250" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/daniel-munoz-marca-el-primer-golazo-de-colombia-en-el-mundial-2026-excelsa-asistencia-de-luis-diaz/202653/</t>
+          <t>https://canaltrece.com.co/noticias/estreno-hoy-todo-sobre-la-llegada-de-toy-story-5-a-las-salas-de-cine/</t>
         </is>
       </c>
     </row>
@@ -7068,17 +7068,17 @@
       </c>
       <c r="C251" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D251" s="6" t="inlineStr">
         <is>
-          <t>Uzbekistán 1 vs. 3 Colombia: reviva el minuto a minuto del debut mundialista de la Tricolor</t>
+          <t>Cierre de legislatura en el Congreso de la República: Proyectos clave que se juegan la vida en el remate del periodo legislativo</t>
         </is>
       </c>
       <c r="E251" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/uzbekistan-vs-colombia-en-vivo-hoy-siga-en-directo-el-debut-de-la-seleccion-colombia-en-el-mundial-2026-y-las-ultimas-noticias/202606/</t>
+          <t>https://canaltrece.com.co/noticias/cierre-de-legislatura-en-el-congreso-de-la-republica-proyectos-clave-que-se-juegan-la-vida-en-el-remate-del-periodo-legislativo/</t>
         </is>
       </c>
     </row>
@@ -7091,17 +7091,17 @@
       </c>
       <c r="C252" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D252" s="3" t="inlineStr">
         <is>
-          <t>Las tablas de todos los grupos del Mundial 2026, jugada la primera fecha</t>
+          <t>¿Qué pasará con Blessd? Claves para entender su situación jurídica tras el fallo sobre presunto secuestro</t>
         </is>
       </c>
       <c r="E252" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/las-tablas-de-todos-los-grupos-del-mundial-2026-jugada-la-primera-fecha/202610/</t>
+          <t>https://canaltrece.com.co/noticias/que-pasara-con-blessd-claves-para-entender-su-situacion-juridica-tras-el-fallo-sobre-presunto-secuestro/</t>
         </is>
       </c>
     </row>
@@ -7114,17 +7114,17 @@
       </c>
       <c r="C253" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D253" s="6" t="inlineStr">
         <is>
-          <t>¿Qué partidos del Mundial 2026 se juegan este 18 de junio? Horarios y canal de TV</t>
+          <t>Colombia define su futuro: Avance en vivo de la jornada de segunda vuelta presidencial de 2026</t>
         </is>
       </c>
       <c r="E253" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/que-partidos-del-mundial-2026-se-juegan-este-18-de-junio-horarios-y-canal-de-tv/202639/</t>
+          <t>https://canaltrece.com.co/noticias/colombia-define-su-futuro-avance-en-vivo-de-la-jornada-de-segunda-vuelta-presidencial-de-2026/</t>
         </is>
       </c>
     </row>
@@ -7137,17 +7137,17 @@
       </c>
       <c r="C254" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D254" s="3" t="inlineStr">
         <is>
-          <t>Trump llama marxista a Iván Cepeda y vuelve a respaldar a Abelardo de la Espriella para la segunda vuelta presidencial</t>
+          <t>Falcao Mundial 2026: el Tigre cree que Colombia puede superar lo hecho en 2014</t>
         </is>
       </c>
       <c r="E254" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/mundo/articulo/trump-llama-marxista-a-ivan-cepeda-y-vuelve-a-respaldar-a-abelardo-de-la-espriella-para-la-segunda-vuelta-presidencial/202613/</t>
+          <t>https://canaltrece.com.co/noticias/falcao-mundial-2026-colombia/</t>
         </is>
       </c>
     </row>
@@ -7160,17 +7160,17 @@
       </c>
       <c r="C255" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D255" s="6" t="inlineStr">
         <is>
-          <t>De crítica feroz a aliada: las veces que Claudia López cuestionó a Iván Cepeda antes de apoyarlo</t>
+          <t>Colombia vs Uzbekistán: hora y dónde ver EN VIVO el debut de la Selección en el Mundial 2026</t>
         </is>
       </c>
       <c r="E255" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/de-critica-feroz-a-aliada-las-veces-que-claudia-lopez-cuestiono-a-ivan-cepeda-antes-de-apoyarlo/202626/</t>
+          <t>https://canaltrece.com.co/noticias/colombia-vs-uzbekistan-hora-colombia/</t>
         </is>
       </c>
     </row>
@@ -7183,17 +7183,17 @@
       </c>
       <c r="C256" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D256" s="3" t="inlineStr">
         <is>
-          <t>Delcy Rodríguez sigue con la limpieza en Venezuela: destituyó a edecán de Maduro y a hija de Hugo Chávez</t>
+          <t>Ley seca Bogotá: Galán cambia el horario para las elecciones 2026</t>
         </is>
       </c>
       <c r="E256" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/mundo/articulo/delcy-rodriguez-sigue-con-la-limpieza-en-venezuela-destituyo-a-edecan-de-maduro-y-a-hija-de-hugo-chavez/202658/</t>
+          <t>https://canaltrece.com.co/noticias/ley-seca-bogota-elecciones-2026/</t>
         </is>
       </c>
     </row>
@@ -7206,17 +7206,17 @@
       </c>
       <c r="C257" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D257" s="6" t="inlineStr">
         <is>
-          <t>Video | Alimentador de TransMilenio se volcó y cayó en zona verde al sur de Bogotá</t>
+          <t>Premios Jaime Garzón 2026: así cerró con éxito el Encuentro de Medios Alternativos</t>
         </is>
       </c>
       <c r="E257" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/video-alimentador-de-transmilenio-se-volco-y-cayo-en-zona-verde-al-sur-de-bogota/202648/</t>
+          <t>https://canaltrece.com.co/noticias/premios-jaime-garzon-2026-encuentro-medios-alternativos/</t>
         </is>
       </c>
     </row>
@@ -7229,17 +7229,17 @@
       </c>
       <c r="C258" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D258" s="3" t="inlineStr">
         <is>
-          <t>“Casi me desmayo”: Yeferson Cossio ganó más de 4.000 millones de pesos tras el triunfo de la Selección Colombia</t>
+          <t>Reina del Carnaval de Negros y Blancos 2027 será la Reina del Centenario</t>
         </is>
       </c>
       <c r="E258" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/gente/articulo/casi-me-desmayo-yeferson-cossio-gano-mas-de-4000-millones-de-pesos-tras-el-triunfo-de-la-seleccion-colombia/202650/</t>
+          <t>https://canaltrece.com.co/noticias/reina-del-carnaval-de-negros-y-blancos-2027-sera-la-reina-del-centenario/</t>
         </is>
       </c>
     </row>
@@ -7252,17 +7252,17 @@
       </c>
       <c r="C259" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D259" s="6" t="inlineStr">
         <is>
-          <t>La inesperada película de intriga que destronó a los grandes éxitos del año y la puede ver online</t>
+          <t>Viva La Salsa Tour 2026: Rubén Blades, La India y más en Bogotá</t>
         </is>
       </c>
       <c r="E259" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/cultura/television/articulo/la-inesperada-pelicula-de-intriga-que-destrono-a-los-grandes-exitos-del-ano-y-la-puede-ver-online/202641/</t>
+          <t>https://canaltrece.com.co/noticias/viva-la-salsa-tour-2026-ruben-blades-la-india-y-mas-en-bogota/</t>
         </is>
       </c>
     </row>
@@ -7275,17 +7275,17 @@
       </c>
       <c r="C260" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D260" s="3" t="inlineStr">
         <is>
-          <t>El coloso de agua entre Islandia y Groenlandia: la impresionante cascada que la humanidad no puede ver a simple vista</t>
+          <t>Teatro Astor Plaza transmitirá el Mundial 2026 con experiencia en vivo</t>
         </is>
       </c>
       <c r="E260" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/tecnologia/articulo/el-coloso-de-agua-entre-islandia-y-groenlandia-la-impresionante-cascada-que-la-humanidad-no-puede-ver-a-simple-vista/202625/</t>
+          <t>https://canaltrece.com.co/noticias/teatro-astor-plaza-transmitira-el-mundial-2026-con-experiencia-en-vivo/</t>
         </is>
       </c>
     </row>
@@ -7298,17 +7298,17 @@
       </c>
       <c r="C261" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D261" s="6" t="inlineStr">
         <is>
-          <t>El pueblo colonial cerca de Bogotá que se convirtió en el destino preferido de las parejas para el fin de semana</t>
+          <t>La Gente de Omar Geles revive su legado con “Amor Hecho en Letras”</t>
         </is>
       </c>
       <c r="E261" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/turismo/articulo/el-pueblo-colonial-cerca-de-bogota-que-se-convirtio-en-el-destino-preferido-de-las-parejas-para-el-fin-de-semana/202645/</t>
+          <t>https://canaltrece.com.co/noticias/la-gente-de-omar-geles-revive-su-legado-con-amor-hecho-en-letras/</t>
         </is>
       </c>
     </row>
@@ -7321,17 +7321,17 @@
       </c>
       <c r="C262" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D262" s="3" t="inlineStr">
         <is>
-          <t>Beto Coral será deportado a Colombia por estar de manera “irregular” durante 10 años en Estados Unidos</t>
+          <t>Los Tigres del Norte celebrarán 60 años de carrera con show en Bogotá</t>
         </is>
       </c>
       <c r="E262" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/beto-coral-sera-deportado-a-colombia-por-estar-de-manera-irregular-durante-10-anos-en-estados-unidos/202627/</t>
+          <t>https://canaltrece.com.co/noticias/los-tigres-del-norte-celebraran-60-anos-de-carrera-con-show-en-bogota/</t>
         </is>
       </c>
     </row>
@@ -7344,17 +7344,17 @@
       </c>
       <c r="C263" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D263" s="6" t="inlineStr">
         <is>
-          <t>Tentativa de secuestro, calumnia y más: las graves consecuencias que enfrentarían quienes acusaron falsamente a extranjero de abusar de un niño</t>
+          <t>Atención conductores: Alcaldía de Bogotá anuncia nuevas restricciones de movilidad para el segundo semestre de 2026</t>
         </is>
       </c>
       <c r="E263" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/semana-tv/semana-el-debate/articulo/tentativa-de-secuestro-calumnia-y-mas-las-graves-consecuencias-que-enfrentarian-quienes-acusaron-falsamente-a-extranjero-de-abusar-de-un-nino/202612/</t>
+          <t>https://canaltrece.com.co/noticias/atencion-conductores-alcaldia-de-bogota-anuncia-nuevas-restricciones-de-movilidad-para-el-segundo-semestre-de-2026/</t>
         </is>
       </c>
     </row>
@@ -7367,17 +7367,17 @@
       </c>
       <c r="C264" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D264" s="3" t="inlineStr">
         <is>
-          <t>Armando Benedetti confirma empalme con De la Espriella si es elegido presidente: “Yo no voy a ser obstáculo ni piedra para él”</t>
+          <t>Furor en Bogotá: Álvaro Díaz agota su primer concierto y anuncia segunda fecha en el Movistar Arena</t>
         </is>
       </c>
       <c r="E264" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/semana-tv/semana-el-debate/articulo/armando-benedetti-confirma-empalme-con-de-la-espriella-si-es-elegido-presidente-yo-no-voy-a-ser-obstaculo-ni-piedra-para-el/202652/</t>
+          <t>https://canaltrece.com.co/noticias/furor-en-bogota-alvaro-diaz-agota-su-primer-concierto-y-anuncia-segunda-fecha-en-el-movistar-arena/</t>
         </is>
       </c>
     </row>
@@ -7390,17 +7390,17 @@
       </c>
       <c r="C265" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D265" s="6" t="inlineStr">
         <is>
-          <t>Congreso condecoró a Paloma Valencia: este es el importante galardón que recibió</t>
+          <t>De la calle a la gloria: El freestyler Fat N rinde homenaje a Luis Díaz con su nuevo sencillo «DÍAZ LUCHO»</t>
         </is>
       </c>
       <c r="E265" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/congreso-condecoro-a-paloma-valencia-este-es-el-importante-galardon-que-recibio/202649/</t>
+          <t>https://canaltrece.com.co/noticias/de-la-calle-a-la-gloria-el-freestyler-fat-n-rinde-homenaje-a-luis-diaz-con-su-nuevo-sencillo-diaz-lucho/</t>
         </is>
       </c>
     </row>
@@ -7413,17 +7413,17 @@
       </c>
       <c r="C266" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D266" s="3" t="inlineStr">
         <is>
-          <t>Policía de Bogotá hizo macabro hallazgo en la localidad de Kennedy: Medicina Legal investiga</t>
+          <t>El rey del house actual llega a Bogotá: John Summit se presentará en Chamorro City Hall este 10 de septiembre</t>
         </is>
       </c>
       <c r="E266" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/policia-de-bogota-hizo-macabro-hallazgo-en-la-localidad-de-kennedy-medicina-legal-investiga/202609/</t>
+          <t>https://canaltrece.com.co/noticias/el-rey-del-house-actual-llega-a-bogota-john-summit-se-presentara-en-chamorro-city-hall-este-10-de-septiembre/</t>
         </is>
       </c>
     </row>
@@ -7436,17 +7436,17 @@
       </c>
       <c r="C267" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D267" s="6" t="inlineStr">
         <is>
-          <t>Gobierno anuncia paso clave para poner en marcha el Túnel del Toyo: arrancó instalación de sistemas para su operación</t>
+          <t>Caso Blessd: Jueza rechaza medida de aseguramiento y descarta delito de secuestro en proceso judicial</t>
         </is>
       </c>
       <c r="E267" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/gobierno-anuncia-paso-clave-para-poner-en-marcha-el-tunel-del-toyo-arranco-instalacion-de-sistemas-para-su-operacion/202625/</t>
+          <t>https://canaltrece.com.co/noticias/caso-blessd-jueza-rechaza-medida-de-aseguramiento-y-descarta-delito-de-secuestro-en-proceso-judicial/</t>
         </is>
       </c>
     </row>
@@ -7459,17 +7459,17 @@
       </c>
       <c r="C268" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D268" s="3" t="inlineStr">
         <is>
-          <t>¿Nueva modalidad de robo a carros en Bogotá? Denuncian que usarían “ondas de radio” para copiar la señal del control y abrirlos</t>
+          <t>El trágico accidente en Brasil que apagó la vida de Oliver Tree: Una pérdida irreparable para la música alternativa</t>
         </is>
       </c>
       <c r="E268" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/vehiculos/articulo/nueva-modalidad-de-robo-a-carros-en-bogota-denuncia-que-usarian-ondas-de-radio-para-copiar-la-senal-del-control-y-abrirlos/202629/</t>
+          <t>https://canaltrece.com.co/noticias/el-tragico-accidente-en-brasil-que-apago-la-vida-de-oliver-tree-una-perdida-irreparable-para-la-musica-alternativa/</t>
         </is>
       </c>
     </row>
@@ -7482,17 +7482,17 @@
       </c>
       <c r="C269" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D269" s="6" t="inlineStr">
         <is>
-          <t>Elizabeth Serna, lideresa social que votará por Abelardo de la Espriella, afirmó haber recibido amenazas: “Me llamaron vendida”</t>
+          <t>El adiós a una leyenda del internet: ¿Quién era Gaspi y por qué su partida conmocionó a las redes sociales?</t>
         </is>
       </c>
       <c r="E269" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/elizabeth-serna-lideresa-social-que-votara-por-abelardo-de-la-espriella-afirmo-haber-recibido-amenazas-me-llamaron-vendida/202654/</t>
+          <t>https://canaltrece.com.co/noticias/el-adios-a-una-leyenda-del-internet-quien-era-gaspi-y-por-que-su-partida-conmociono-a-las-redes-sociales/</t>
         </is>
       </c>
     </row>
@@ -7505,17 +7505,17 @@
       </c>
       <c r="C270" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D270" s="3" t="inlineStr">
         <is>
-          <t>50 municipios de Cundinamarca aumentaron hasta 15 % el recaudo de la sobretasa a la gasolina</t>
+          <t>Dónde ver los partidos de Colombia en el Mundial 2026</t>
         </is>
       </c>
       <c r="E270" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/bogota/articulo/50-municipios-de-cundinamarca-aumentaron-hasta-15-el-recaudo-de-la-sobretasa-a-la-gasolina/202610/</t>
+          <t>https://canaltrece.com.co/noticias/donde-ver-los-partidos-de-colombia-en-el-mundial-2026-2/</t>
         </is>
       </c>
     </row>
@@ -7528,17 +7528,17 @@
       </c>
       <c r="C271" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D271" s="6" t="inlineStr">
         <is>
-          <t>En imágenes | Capturan a los “Bonnie y Clyde” colombianos: Policía dio los detalles del caso</t>
+          <t>Dónde ver Colombia vs Uzbekistán: canal, hora y streaming</t>
         </is>
       </c>
       <c r="E271" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/en-imagenes-capturan-a-los-bonnie-y-clyde-colombianos-policia-dio-los-detalles-del-caso/202656/</t>
+          <t>https://canaltrece.com.co/noticias/donde-ver-colombia-vs-uzbekistan-canal-hora-y-streaming/</t>
         </is>
       </c>
     </row>
@@ -7551,17 +7551,17 @@
       </c>
       <c r="C272" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D272" s="3" t="inlineStr">
         <is>
-          <t>🔴 Calendario y fixture de la Copa Mundial de la FIFA 2026</t>
+          <t>Ryan Castro y Spotify sorprendieron con canción inédita en Bogotá</t>
         </is>
       </c>
       <c r="E272" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/especiales-multimedia/articulo/mundial-2026-el-simulador-con-el-que-usted-puede-jugar-y-atinar-hasta-que-haya-campeon/202529/</t>
+          <t>https://canaltrece.com.co/noticias/ryan-castro-y-spotify-sorprendieron-con-cancion-inedita-en-bogota/</t>
         </is>
       </c>
     </row>
@@ -7574,17 +7574,17 @@
       </c>
       <c r="C273" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D273" s="6" t="inlineStr">
         <is>
-          <t>Colombia vs Uzbekistán: la Tricolor debutó con victoria 3-1</t>
+          <t>Colombia bailó al son de Luis Díaz y le ganó a Uzbekistán: tres puntos y paso firme en el Mundial 2026</t>
         </is>
       </c>
       <c r="E273" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/colombia-vs-uzbekistan-mundial-2026/</t>
+          <t>https://www.semana.com/deportes/articulo/colombia-bailo-al-son-de-luis-diaz-y-le-gano-a-uzbekistan-tres-puntos-y-paso-firme-en-el-mundial-2026/202625/</t>
         </is>
       </c>
     </row>
@@ -7597,17 +7597,17 @@
       </c>
       <c r="C274" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D274" s="3" t="inlineStr">
         <is>
-          <t>Morat Tu Cárcel alcanza el No. 1 en Billboard Latin Airplay</t>
+          <t>Colombia vs. RD Congo, próximo partido de la Tricolor en el Mundial 2026: fecha y hora confirmadas</t>
         </is>
       </c>
       <c r="E274" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/morat-tu-carcel-billboard/</t>
+          <t>https://www.semana.com/deportes/articulo/colombia-vs-rd-congo-proximo-partido-de-la-tricolor-en-el-mundial-2026-fecha-y-hora-confirmadas/202659/</t>
         </is>
       </c>
     </row>
@@ -7620,17 +7620,17 @@
       </c>
       <c r="C275" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D275" s="6" t="inlineStr">
         <is>
-          <t>Colombia vs Uzbekistán: así terminó el primer tiempo del debut</t>
+          <t>El gol de Jaminton Campaz que liquidó a Uzbekistán: locura en Colombia tras la jugada del Cucho Hernández</t>
         </is>
       </c>
       <c r="E275" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/colombia-vs-uzbekistan/</t>
+          <t>https://www.semana.com/deportes/articulo/el-gol-de-jaminton-campaz-que-liquido-a-uzbekistan-locura-en-colombia-tras-la-jugada-del-cucho-hernandez/202642/</t>
         </is>
       </c>
     </row>
@@ -7643,17 +7643,17 @@
       </c>
       <c r="C276" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D276" s="3" t="inlineStr">
         <is>
-          <t>Penelope Robin inicia una nueva etapa con Diosa de Cien Colores</t>
+          <t>Magistral jugada de Luis Díaz que resuena en el Mundial 2026: magia ante Uzbekistán es viral</t>
         </is>
       </c>
       <c r="E276" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/penelope-robin-diosa-de-cien-colores/</t>
+          <t>https://www.semana.com/deportes/articulo/magistral-jugada-de-luis-diaz-que-resuena-en-el-mundial-2026-magia-ante-uzbekistan-es-viral-en-el-mundo/202652/</t>
         </is>
       </c>
     </row>
@@ -7666,17 +7666,17 @@
       </c>
       <c r="C277" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D277" s="6" t="inlineStr">
         <is>
-          <t>Narra Tu Territorio abre segundo corte tras recibir 764 propuestas</t>
+          <t>Tabla de posiciones en el grupo K del Mundial 2026: Colombia vence a Uzbekistán y lanza aviso a Portugal</t>
         </is>
       </c>
       <c r="E277" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/narra-tu-territorio-segundo-corte/</t>
+          <t>https://www.semana.com/deportes/articulo/tabla-de-posiciones-en-el-grupo-k-del-mundial-2026-colombia-vence-a-uzbekistan-y-lanza-aviso-a-portugal/202608/</t>
         </is>
       </c>
     </row>
@@ -7689,17 +7689,17 @@
       </c>
       <c r="C278" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D278" s="3" t="inlineStr">
         <is>
-          <t>Colombia vs Uzbekistán: fecha, hora, estadio y dónde ver</t>
+          <t>La reacción de Lorenzo tras la victoria ante Uzbekistán con tres goles en el Mundial 2026: “Hay que mejorar”</t>
         </is>
       </c>
       <c r="E278" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/colombia-vs-uzbekistan-fecha-hora-estadio-y-donde-ver/</t>
+          <t>https://www.semana.com/deportes/articulo/la-reaccion-de-lorenzo-tras-la-victoria-ante-uzbekistan-con-tres-goles-en-el-mundial-2026-hay-que-mejorar/202635/</t>
         </is>
       </c>
     </row>
@@ -7712,17 +7712,17 @@
       </c>
       <c r="C279" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D279" s="6" t="inlineStr">
         <is>
-          <t>Fanzones en Bogotá para ver a Colombia: boletas y horarios</t>
+          <t>Blooper de Camilo Vargas, pero Luis Díaz lo salvó: momento sublime de Colombia que resuena en el Mundial 2026</t>
         </is>
       </c>
       <c r="E279" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/fanzones-en-bogota-para-ver-a-colombia-boletas-y-horarios/</t>
+          <t>https://www.semana.com/deportes/articulo/blooper-de-camilo-vargas-pero-luis-diaz-lo-salvo-momento-sublime-de-colombia-que-resuena-en-el-mundial-2026/202653/</t>
         </is>
       </c>
     </row>
@@ -7735,17 +7735,17 @@
       </c>
       <c r="C280" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D280" s="3" t="inlineStr">
         <is>
-          <t>¿Estreno hoy? Todo sobre la llegada de Toy Story 5 a las salas de cine</t>
+          <t>Daniel Muñoz marcó el primer golazo de Colombia en el Mundial 2026: excelsa asistencia de Luis Díaz</t>
         </is>
       </c>
       <c r="E280" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/estreno-hoy-todo-sobre-la-llegada-de-toy-story-5-a-las-salas-de-cine/</t>
+          <t>https://www.semana.com/deportes/articulo/daniel-munoz-marca-el-primer-golazo-de-colombia-en-el-mundial-2026-excelsa-asistencia-de-luis-diaz/202653/</t>
         </is>
       </c>
     </row>
@@ -7758,17 +7758,17 @@
       </c>
       <c r="C281" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D281" s="6" t="inlineStr">
         <is>
-          <t>Cierre de legislatura en el Congreso de la República: Proyectos clave que se juegan la vida en el remate del periodo legislativo</t>
+          <t>Uzbekistán 1 vs. 3 Colombia: reviva el minuto a minuto del debut mundialista de la Tricolor</t>
         </is>
       </c>
       <c r="E281" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/cierre-de-legislatura-en-el-congreso-de-la-republica-proyectos-clave-que-se-juegan-la-vida-en-el-remate-del-periodo-legislativo/</t>
+          <t>https://www.semana.com/deportes/articulo/uzbekistan-vs-colombia-en-vivo-hoy-siga-en-directo-el-debut-de-la-seleccion-colombia-en-el-mundial-2026-y-las-ultimas-noticias/202606/</t>
         </is>
       </c>
     </row>
@@ -7781,17 +7781,17 @@
       </c>
       <c r="C282" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D282" s="3" t="inlineStr">
         <is>
-          <t>¿Qué pasará con Blessd? Claves para entender su situación jurídica tras el fallo sobre presunto secuestro</t>
+          <t>Las tablas de todos los grupos del Mundial 2026, jugada la primera fecha</t>
         </is>
       </c>
       <c r="E282" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/que-pasara-con-blessd-claves-para-entender-su-situacion-juridica-tras-el-fallo-sobre-presunto-secuestro/</t>
+          <t>https://www.semana.com/deportes/articulo/las-tablas-de-todos-los-grupos-del-mundial-2026-jugada-la-primera-fecha/202610/</t>
         </is>
       </c>
     </row>
@@ -7804,17 +7804,17 @@
       </c>
       <c r="C283" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D283" s="6" t="inlineStr">
         <is>
-          <t>Colombia define su futuro: Avance en vivo de la jornada de segunda vuelta presidencial de 2026</t>
+          <t>¿Qué partidos del Mundial 2026 se juegan este 18 de junio? Horarios y canal de TV</t>
         </is>
       </c>
       <c r="E283" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/colombia-define-su-futuro-avance-en-vivo-de-la-jornada-de-segunda-vuelta-presidencial-de-2026/</t>
+          <t>https://www.semana.com/deportes/articulo/que-partidos-del-mundial-2026-se-juegan-este-18-de-junio-horarios-y-canal-de-tv/202639/</t>
         </is>
       </c>
     </row>
@@ -7827,17 +7827,17 @@
       </c>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D284" s="3" t="inlineStr">
         <is>
-          <t>Falcao Mundial 2026: el Tigre cree que Colombia puede superar lo hecho en 2014</t>
+          <t>Trump llama marxista a Iván Cepeda y vuelve a respaldar a Abelardo de la Espriella para la segunda vuelta presidencial</t>
         </is>
       </c>
       <c r="E284" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/falcao-mundial-2026-colombia/</t>
+          <t>https://www.semana.com/mundo/articulo/trump-llama-marxista-a-ivan-cepeda-y-vuelve-a-respaldar-a-abelardo-de-la-espriella-para-la-segunda-vuelta-presidencial/202613/</t>
         </is>
       </c>
     </row>
@@ -7850,17 +7850,17 @@
       </c>
       <c r="C285" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D285" s="6" t="inlineStr">
         <is>
-          <t>Colombia vs Uzbekistán: hora y dónde ver EN VIVO el debut de la Selección en el Mundial 2026</t>
+          <t>De crítica feroz a aliada: las veces que Claudia López cuestionó a Iván Cepeda antes de apoyarlo</t>
         </is>
       </c>
       <c r="E285" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/colombia-vs-uzbekistan-hora-colombia/</t>
+          <t>https://www.semana.com/politica/articulo/de-critica-feroz-a-aliada-las-veces-que-claudia-lopez-cuestiono-a-ivan-cepeda-antes-de-apoyarlo/202626/</t>
         </is>
       </c>
     </row>
@@ -7873,17 +7873,17 @@
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D286" s="3" t="inlineStr">
         <is>
-          <t>Ley seca Bogotá: Galán cambia el horario para las elecciones 2026</t>
+          <t>Delcy Rodríguez sigue con la limpieza en Venezuela: destituyó a edecán de Maduro y a hija de Hugo Chávez</t>
         </is>
       </c>
       <c r="E286" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/ley-seca-bogota-elecciones-2026/</t>
+          <t>https://www.semana.com/mundo/articulo/delcy-rodriguez-sigue-con-la-limpieza-en-venezuela-destituyo-a-edecan-de-maduro-y-a-hija-de-hugo-chavez/202658/</t>
         </is>
       </c>
     </row>
@@ -7896,17 +7896,17 @@
       </c>
       <c r="C287" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D287" s="6" t="inlineStr">
         <is>
-          <t>Premios Jaime Garzón 2026: así cerró con éxito el Encuentro de Medios Alternativos</t>
+          <t>Video | Alimentador de TransMilenio se volcó y cayó en zona verde al sur de Bogotá</t>
         </is>
       </c>
       <c r="E287" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/premios-jaime-garzon-2026-encuentro-medios-alternativos/</t>
+          <t>https://www.semana.com/nacion/articulo/video-alimentador-de-transmilenio-se-volco-y-cayo-en-zona-verde-al-sur-de-bogota/202648/</t>
         </is>
       </c>
     </row>
@@ -7919,17 +7919,17 @@
       </c>
       <c r="C288" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D288" s="3" t="inlineStr">
         <is>
-          <t>Reina del Carnaval de Negros y Blancos 2027 será la Reina del Centenario</t>
+          <t>“Casi me desmayo”: Yeferson Cossio ganó más de 4.000 millones de pesos tras el triunfo de la Selección Colombia</t>
         </is>
       </c>
       <c r="E288" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/reina-del-carnaval-de-negros-y-blancos-2027-sera-la-reina-del-centenario/</t>
+          <t>https://www.semana.com/gente/articulo/casi-me-desmayo-yeferson-cossio-gano-mas-de-4000-millones-de-pesos-tras-el-triunfo-de-la-seleccion-colombia/202650/</t>
         </is>
       </c>
     </row>
@@ -7942,17 +7942,17 @@
       </c>
       <c r="C289" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D289" s="6" t="inlineStr">
         <is>
-          <t>Viva La Salsa Tour 2026: Rubén Blades, La India y más en Bogotá</t>
+          <t>La inesperada película de intriga que destronó a los grandes éxitos del año y la puede ver online</t>
         </is>
       </c>
       <c r="E289" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/viva-la-salsa-tour-2026-ruben-blades-la-india-y-mas-en-bogota/</t>
+          <t>https://www.semana.com/cultura/television/articulo/la-inesperada-pelicula-de-intriga-que-destrono-a-los-grandes-exitos-del-ano-y-la-puede-ver-online/202641/</t>
         </is>
       </c>
     </row>
@@ -7965,17 +7965,17 @@
       </c>
       <c r="C290" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D290" s="3" t="inlineStr">
         <is>
-          <t>Teatro Astor Plaza transmitirá el Mundial 2026 con experiencia en vivo</t>
+          <t>El coloso de agua entre Islandia y Groenlandia: la impresionante cascada que la humanidad no puede ver a simple vista</t>
         </is>
       </c>
       <c r="E290" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/teatro-astor-plaza-transmitira-el-mundial-2026-con-experiencia-en-vivo/</t>
+          <t>https://www.semana.com/tecnologia/articulo/el-coloso-de-agua-entre-islandia-y-groenlandia-la-impresionante-cascada-que-la-humanidad-no-puede-ver-a-simple-vista/202625/</t>
         </is>
       </c>
     </row>
@@ -7988,17 +7988,17 @@
       </c>
       <c r="C291" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D291" s="6" t="inlineStr">
         <is>
-          <t>La Gente de Omar Geles revive su legado con “Amor Hecho en Letras”</t>
+          <t>El pueblo colonial cerca de Bogotá que se convirtió en el destino preferido de las parejas para el fin de semana</t>
         </is>
       </c>
       <c r="E291" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/la-gente-de-omar-geles-revive-su-legado-con-amor-hecho-en-letras/</t>
+          <t>https://www.semana.com/turismo/articulo/el-pueblo-colonial-cerca-de-bogota-que-se-convirtio-en-el-destino-preferido-de-las-parejas-para-el-fin-de-semana/202645/</t>
         </is>
       </c>
     </row>
@@ -8011,17 +8011,17 @@
       </c>
       <c r="C292" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D292" s="3" t="inlineStr">
         <is>
-          <t>Los Tigres del Norte celebrarán 60 años de carrera con show en Bogotá</t>
+          <t>Beto Coral será deportado a Colombia por estar de manera “irregular” durante 10 años en Estados Unidos</t>
         </is>
       </c>
       <c r="E292" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/los-tigres-del-norte-celebraran-60-anos-de-carrera-con-show-en-bogota/</t>
+          <t>https://www.semana.com/politica/articulo/beto-coral-sera-deportado-a-colombia-por-estar-de-manera-irregular-durante-10-anos-en-estados-unidos/202627/</t>
         </is>
       </c>
     </row>
@@ -8034,17 +8034,17 @@
       </c>
       <c r="C293" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D293" s="6" t="inlineStr">
         <is>
-          <t>Atención conductores: Alcaldía de Bogotá anuncia nuevas restricciones de movilidad para el segundo semestre de 2026</t>
+          <t>Tentativa de secuestro, calumnia y más: las graves consecuencias que enfrentarían quienes acusaron falsamente a extranjero de abusar de un niño</t>
         </is>
       </c>
       <c r="E293" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/atencion-conductores-alcaldia-de-bogota-anuncia-nuevas-restricciones-de-movilidad-para-el-segundo-semestre-de-2026/</t>
+          <t>https://www.semana.com/semana-tv/semana-el-debate/articulo/tentativa-de-secuestro-calumnia-y-mas-las-graves-consecuencias-que-enfrentarian-quienes-acusaron-falsamente-a-extranjero-de-abusar-de-un-nino/202612/</t>
         </is>
       </c>
     </row>
@@ -8057,17 +8057,17 @@
       </c>
       <c r="C294" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D294" s="3" t="inlineStr">
         <is>
-          <t>Furor en Bogotá: Álvaro Díaz agota su primer concierto y anuncia segunda fecha en el Movistar Arena</t>
+          <t>Armando Benedetti confirma empalme con De la Espriella si es elegido presidente: “Yo no voy a ser obstáculo ni piedra para él”</t>
         </is>
       </c>
       <c r="E294" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/furor-en-bogota-alvaro-diaz-agota-su-primer-concierto-y-anuncia-segunda-fecha-en-el-movistar-arena/</t>
+          <t>https://www.semana.com/semana-tv/semana-el-debate/articulo/armando-benedetti-confirma-empalme-con-de-la-espriella-si-es-elegido-presidente-yo-no-voy-a-ser-obstaculo-ni-piedra-para-el/202652/</t>
         </is>
       </c>
     </row>
@@ -8080,17 +8080,17 @@
       </c>
       <c r="C295" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D295" s="6" t="inlineStr">
         <is>
-          <t>De la calle a la gloria: El freestyler Fat N rinde homenaje a Luis Díaz con su nuevo sencillo «DÍAZ LUCHO»</t>
+          <t>Congreso condecoró a Paloma Valencia: este es el importante galardón que recibió</t>
         </is>
       </c>
       <c r="E295" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/de-la-calle-a-la-gloria-el-freestyler-fat-n-rinde-homenaje-a-luis-diaz-con-su-nuevo-sencillo-diaz-lucho/</t>
+          <t>https://www.semana.com/politica/articulo/congreso-condecoro-a-paloma-valencia-este-es-el-importante-galardon-que-recibio/202649/</t>
         </is>
       </c>
     </row>
@@ -8103,17 +8103,17 @@
       </c>
       <c r="C296" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D296" s="3" t="inlineStr">
         <is>
-          <t>El rey del house actual llega a Bogotá: John Summit se presentará en Chamorro City Hall este 10 de septiembre</t>
+          <t>Policía de Bogotá hizo macabro hallazgo en la localidad de Kennedy: Medicina Legal investiga</t>
         </is>
       </c>
       <c r="E296" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/el-rey-del-house-actual-llega-a-bogota-john-summit-se-presentara-en-chamorro-city-hall-este-10-de-septiembre/</t>
+          <t>https://www.semana.com/nacion/articulo/policia-de-bogota-hizo-macabro-hallazgo-en-la-localidad-de-kennedy-medicina-legal-investiga/202609/</t>
         </is>
       </c>
     </row>
@@ -8126,17 +8126,17 @@
       </c>
       <c r="C297" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D297" s="6" t="inlineStr">
         <is>
-          <t>Caso Blessd: Jueza rechaza medida de aseguramiento y descarta delito de secuestro en proceso judicial</t>
+          <t>Gobierno anuncia paso clave para poner en marcha el Túnel del Toyo: arrancó instalación de sistemas para su operación</t>
         </is>
       </c>
       <c r="E297" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/caso-blessd-jueza-rechaza-medida-de-aseguramiento-y-descarta-delito-de-secuestro-en-proceso-judicial/</t>
+          <t>https://www.semana.com/nacion/articulo/gobierno-anuncia-paso-clave-para-poner-en-marcha-el-tunel-del-toyo-arranco-instalacion-de-sistemas-para-su-operacion/202625/</t>
         </is>
       </c>
     </row>
@@ -8149,17 +8149,17 @@
       </c>
       <c r="C298" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D298" s="3" t="inlineStr">
         <is>
-          <t>El trágico accidente en Brasil que apagó la vida de Oliver Tree: Una pérdida irreparable para la música alternativa</t>
+          <t>¿Nueva modalidad de robo a carros en Bogotá? Denuncian que usarían “ondas de radio” para copiar la señal del control y abrirlos</t>
         </is>
       </c>
       <c r="E298" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/el-tragico-accidente-en-brasil-que-apago-la-vida-de-oliver-tree-una-perdida-irreparable-para-la-musica-alternativa/</t>
+          <t>https://www.semana.com/vehiculos/articulo/nueva-modalidad-de-robo-a-carros-en-bogota-denuncia-que-usarian-ondas-de-radio-para-copiar-la-senal-del-control-y-abrirlos/202629/</t>
         </is>
       </c>
     </row>
@@ -8172,17 +8172,17 @@
       </c>
       <c r="C299" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D299" s="6" t="inlineStr">
         <is>
-          <t>El adiós a una leyenda del internet: ¿Quién era Gaspi y por qué su partida conmocionó a las redes sociales?</t>
+          <t>Elizabeth Serna, lideresa social que votará por Abelardo de la Espriella, afirmó haber recibido amenazas: “Me llamaron vendida”</t>
         </is>
       </c>
       <c r="E299" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/el-adios-a-una-leyenda-del-internet-quien-era-gaspi-y-por-que-su-partida-conmociono-a-las-redes-sociales/</t>
+          <t>https://www.semana.com/nacion/articulo/elizabeth-serna-lideresa-social-que-votara-por-abelardo-de-la-espriella-afirmo-haber-recibido-amenazas-me-llamaron-vendida/202654/</t>
         </is>
       </c>
     </row>
@@ -8195,17 +8195,17 @@
       </c>
       <c r="C300" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D300" s="3" t="inlineStr">
         <is>
-          <t>Dónde ver los partidos de Colombia en el Mundial 2026</t>
+          <t>50 municipios de Cundinamarca aumentaron hasta 15 % el recaudo de la sobretasa a la gasolina</t>
         </is>
       </c>
       <c r="E300" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/donde-ver-los-partidos-de-colombia-en-el-mundial-2026-2/</t>
+          <t>https://www.semana.com/nacion/bogota/articulo/50-municipios-de-cundinamarca-aumentaron-hasta-15-el-recaudo-de-la-sobretasa-a-la-gasolina/202610/</t>
         </is>
       </c>
     </row>
@@ -8218,17 +8218,17 @@
       </c>
       <c r="C301" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D301" s="6" t="inlineStr">
         <is>
-          <t>Dónde ver Colombia vs Uzbekistán: canal, hora y streaming</t>
+          <t>En imágenes | Capturan a los “Bonnie y Clyde” colombianos: Policía dio los detalles del caso</t>
         </is>
       </c>
       <c r="E301" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/donde-ver-colombia-vs-uzbekistan-canal-hora-y-streaming/</t>
+          <t>https://www.semana.com/nacion/articulo/en-imagenes-capturan-a-los-bonnie-y-clyde-colombianos-policia-dio-los-detalles-del-caso/202656/</t>
         </is>
       </c>
     </row>
@@ -8241,17 +8241,17 @@
       </c>
       <c r="C302" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D302" s="3" t="inlineStr">
         <is>
-          <t>Ryan Castro y Spotify sorprendieron con canción inédita en Bogotá</t>
+          <t>🔴 Calendario y fixture de la Copa Mundial de la FIFA 2026</t>
         </is>
       </c>
       <c r="E302" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/ryan-castro-y-spotify-sorprendieron-con-cancion-inedita-en-bogota/</t>
+          <t>https://www.semana.com/deportes/especiales-multimedia/articulo/mundial-2026-el-simulador-con-el-que-usted-puede-jugar-y-atinar-hasta-que-haya-campeon/202529/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 Noticias actualizadas 19/06/2026 09:13
</commit_message>
<xml_diff>
--- a/docs/ultimahora.xlsx
+++ b/docs/ultimahora.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Todas las noticias" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Todas las noticias'!$A$1:$E$279</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Todas las noticias'!$A$1:$E$259</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E279"/>
+  <dimension ref="A1:E259"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -543,7 +543,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>19/06/2026 02:01 a. m.</t>
+          <t>19/06/2026 03:30 a. m.</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -558,19 +558,19 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Diez años de arresto por desacatos: el curioso caso de la exgerente de Nueva EPS que terminó en la Corte Suprema</t>
+          <t>Suiza confirma aplazamiento de reunión entre Irán, Estados Unidos y mediadores en medio de negociaciones de tregua</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/justicia/cortes/diez-anos-de-arresto-por-desacatos-el-curioso-caso-de-la-exgerente-de-nueva-eps-que-termino-en-la-corte-suprema-3565376</t>
+          <t>https://www.eltiempo.com/mundo/europa/suiza-confirma-aplazamiento-de-reunion-entre-iran-estados-unidos-y-mediadores-en-medio-de-negociaciones-de-tregua-3565414</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>19/06/2026 01:59 a. m.</t>
+          <t>19/06/2026 03:01 a. m.</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -585,19 +585,19 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>Mundial 2026: México clasifica a dieciseisavos, Canadá golea a Catar y Brasil espera el regreso de Neymar</t>
+          <t>Israel intensifica ataques en el sur del Líbano: al menos 18 muertos pese al acuerdo de cese de hostilidades impulsado por Estados Unidos e Irán</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/mundial-2026-mexico-clasifica-a-dieciseisavos-canada-golea-a-catar-y-brasil-espera-el-regreso-de-neymar-3565411</t>
+          <t>https://www.eltiempo.com/mundo/medio-oriente/israel-intensifica-ataques-en-el-sur-del-libano-al-menos-18-muertos-pese-al-acuerdo-de-cese-de-hostilidades-impulsado-por-estados-unidos-e-iran-3565413</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>19/06/2026 01:41 a. m.</t>
+          <t>19/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -612,19 +612,19 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Elecciones presidenciales Colombia 2026: últimas noticias de la segunda vuelta presidencial entre Iván Cepeda y Abelardo de la Espriella</t>
+          <t>Hermano del narcotraficante Fito llega a Ecuador y es enviado a cárcel de máxima seguridad</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/elecciones-presidenciales-colombia-2026-ultimas-noticias-de-la-segunda-vuelta-presidencial-entre-ivan-cepeda-y-abelardo-de-la-espriella-3565410</t>
+          <t>https://www.eltiempo.com/justicia/hermano-del-narcotraficante-fito-llega-a-ecuador-y-es-enviado-a-carcel-de-maxima-seguridad-3565412</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>19/06/2026 01:25 a. m.</t>
+          <t>19/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -639,19 +639,19 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Murió Dalita Navarro, artista y viuda del expresidente Belisario Betancur: su legado marcó la cerámica y la gestión cultural en Colombia</t>
+          <t>¡Atención conductores! Pico y placa en Pereira para el viernes 19 de junio de 2026: así regirá la medida</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/cultura/murio-dalita-navarro-artista-y-viuda-del-expresidente-belisario-betancur-su-legado-marco-la-ceramica-y-la-gestion-cultural-en-colombia-3565409</t>
+          <t>https://www.eltiempo.com/colombia/otras-ciudades/atencion-conductores-pico-y-placa-en-pereira-para-el-viernes-19-de-junio-de-2026-asi-regira-la-medida-3565384</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>19/06/2026 12:10 a. m.</t>
+          <t>19/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -666,19 +666,19 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Cinco colombianos demandan a Marco Rubio por el freno a visas de residencia: caso podría redefinir los límites de la política migratoria de Trump</t>
+          <t>¡Ojo, conductor! Pico y placa en Bucaramanga para el viernes 19 de junio de 2026</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/cinco-colombianos-demandan-a-marco-rubio-por-el-freno-a-visas-de-residencia-caso-podria-redefinir-los-limites-de-la-politica-migratoria-de-trump-3565176</t>
+          <t>https://www.eltiempo.com/colombia/santander/ojo-conductor-pico-y-placa-en-bucaramanga-para-el-viernes-19-de-junio-de-3565381</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>19/06/2026 12:01 a. m.</t>
+          <t>19/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -693,19 +693,19 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Procuraduría reunió a medios regionales para respaldar la paz electoral y defender la institucionalidad</t>
+          <t>¡Siga la medida de movilidad! Pico y placa en Medellín para el viernes 19 de junio de 2026: así funciona la restricción</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mas-contenido/procuraduria-reunio-a-medios-regionales-para-respaldar-la-paz-electoral-y-defender-la-institucionalidad-3565406</t>
+          <t>https://www.eltiempo.com/colombia/medellin/siga-la-medida-de-movilidad-pico-y-placa-en-medellin-para-el-viernes-19-de-junio-de-2026-asi-funciona-la-restriccion-3565377</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 11:40 p. m.</t>
+          <t>19/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -720,19 +720,19 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Paraguay quiere salir del túnel y busca que Turquía pague los platos rotos en el Mundial: día, hora y dónde ver el partido</t>
+          <t>¡Evite multas! Pico y placa en Cali para el viernes 19 de junio de 2026: así opera la medida</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/paraguay-quiere-salir-del-tunel-y-busca-que-turquia-pague-los-platos-rotos-en-el-mundial-dia-hora-y-donde-ver-el-partido-3565387</t>
+          <t>https://www.eltiempo.com/colombia/cali/evite-multas-pico-y-placa-en-cali-para-el-viernes-19-de-junio-de-2026-asi-opera-la-medida-3565369</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 11:31 p. m.</t>
+          <t>19/06/2026 02:19 a. m.</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -747,19 +747,19 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>¿Cuál de los dos candidatos será el mejor guardián de la Constitución? / La entrevista de María Isabel Rueda</t>
+          <t>¡Pilas en las vías! Pico y placa en Bogotá para el viernes 19 de junio de 2026</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/politica/cual-de-los-dos-candidatos-sera-el-mejor-guardian-de-la-constitucion-la-entrevista-de-maria-isabel-rueda-3565401</t>
+          <t>https://www.eltiempo.com/bogota/pilas-en-las-vias-pico-y-placa-en-bogota-para-el-viernes-19-de-junio-de-3565365</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 11:27 p. m.</t>
+          <t>19/06/2026 02:01 a. m.</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -774,19 +774,19 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Noveno día del Mundial de Estados Unidos, Canadá y México 2026: ¿qué partidos se juegan este viernes 19 de junio? Canal y hora para ver en vivo</t>
+          <t>Diez años de arresto por desacatos: el curioso caso de la exgerente de Nueva EPS que terminó en la Corte Suprema</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/noveno-dia-del-mundial-de-estados-unidos-canada-y-mexico-2026-que-partidos-se-juegan-este-viernes-19-de-junio-canal-y-hora-para-ver-en-vivo-3565403</t>
+          <t>https://www.eltiempo.com/justicia/cortes/diez-anos-de-arresto-por-desacatos-el-curioso-caso-de-la-exgerente-de-nueva-eps-que-termino-en-la-corte-suprema-3565376</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 11:20 p. m.</t>
+          <t>19/06/2026 01:59 a. m.</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -801,19 +801,19 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Turista murió tras intentar salvar la vida de su mamá en medio de paseo en caballo por Central Park, en Estados Unidos: fuertes imágenes de la caída</t>
+          <t>Mundial 2026: México clasifica a dieciseisavos, Canadá golea a Catar y Brasil espera el regreso de Neymar</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/turista-murio-tras-intentar-salvar-la-vida-de-su-mama-en-medio-de-paseo-en-caballo-por-central-park-en-estados-unidos-fuertes-imagenes-de-la-caida-3565404</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/mundial-2026-mexico-clasifica-a-dieciseisavos-canada-golea-a-catar-y-brasil-espera-el-regreso-de-neymar-3565411</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 11:18 p. m.</t>
+          <t>19/06/2026 01:41 a. m.</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -828,19 +828,19 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>1,3 toneladas de cocaína que iban a ser enviadas a Europa fueron incautadas por la Policía en el Urabá antioqueño: estaban ocultas en un contenedor</t>
+          <t>Elecciones presidenciales Colombia 2026: últimas noticias de la segunda vuelta presidencial entre Iván Cepeda y Abelardo de la Espriella</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/medellin/1-3-toneladas-de-cocaina-que-iban-a-ser-enviadas-a-europa-fueron-incautadas-por-la-policia-en-el-uraba-antioqueno-estaban-ocultas-en-un-contenedor-3565402</t>
+          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/elecciones-presidenciales-colombia-2026-ultimas-noticias-de-la-segunda-vuelta-presidencial-entre-ivan-cepeda-y-abelardo-de-la-espriella-3565410</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 11:14 p. m.</t>
+          <t>19/06/2026 01:25 a. m.</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -855,19 +855,19 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Nicolás Echavarría y Marcelo Rozo, en la lucha en el US Open de golf, en el que Wyndham Clark picaba en punta</t>
+          <t>Murió Dalita Navarro, artista y viuda del expresidente Belisario Betancur: su legado marcó la cerámica y la gestión cultural en Colombia</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/otros-deportes/nicolas-echavarria-y-marcelo-rozo-en-la-lucha-en-el-us-open-de-golf-en-el-que-wyndham-clark-picaba-en-punta-3565407</t>
+          <t>https://www.eltiempo.com/cultura/murio-dalita-navarro-artista-y-viuda-del-expresidente-belisario-betancur-su-legado-marco-la-ceramica-y-la-gestion-cultural-en-colombia-3565409</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 11:02 p. m.</t>
+          <t>19/06/2026 12:10 a. m.</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -882,19 +882,19 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Elecciones 2026: Valle del Cauca establece hoja de ruta con delegados de la ONU y la Unión Europea</t>
+          <t>Cinco colombianos demandan a Marco Rubio por el freno a visas de residencia: caso podría redefinir los límites de la política migratoria de Trump</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/cali/elecciones-2026-valle-del-cauca-establece-hoja-de-ruta-con-delegados-de-la-onu-y-la-union-europea-3565405</t>
+          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/cinco-colombianos-demandan-a-marco-rubio-por-el-freno-a-visas-de-residencia-caso-podria-redefinir-los-limites-de-la-politica-migratoria-de-trump-3565176</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 11:01 p. m.</t>
+          <t>19/06/2026 12:01 a. m.</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -909,19 +909,19 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Emigrantes desde Colombia: se triplicó el número de personas que salen del país y que no regresan</t>
+          <t>Procuraduría reunió a medios regionales para respaldar la paz electoral y defender la institucionalidad</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/economia/sectores/emigrantes-desde-colombia-se-triplico-el-numero-de-personas-que-salen-del-pais-y-que-no-regresan-3564832</t>
+          <t>https://www.eltiempo.com/mas-contenido/procuraduria-reunio-a-medios-regionales-para-respaldar-la-paz-electoral-y-defender-la-institucionalidad-3565406</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 10:44 p. m.</t>
+          <t>18/06/2026 11:40 p. m.</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -936,19 +936,19 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>El extraño caso de Luis Suárez en la Selección Colombia: ¿‘killer’ o jugador de equipo?</t>
+          <t>Paraguay quiere salir del túnel y busca que Turquía pague los platos rotos en el Mundial: día, hora y dónde ver el partido</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/el-extrano-caso-de-luis-suarez-en-la-seleccion-colombia-killer-o-jugador-de-equipo-3565397</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/paraguay-quiere-salir-del-tunel-y-busca-que-turquia-pague-los-platos-rotos-en-el-mundial-dia-hora-y-donde-ver-el-partido-3565387</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 10:38 p. m.</t>
+          <t>18/06/2026 11:31 p. m.</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -963,19 +963,19 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>La propuesta del candidato Abelardo de la Espriella para estabilizar el sistema de salud en Colombia con una inversión de 10 billones en 90 días</t>
+          <t>¿Cuál de los dos candidatos será el mejor guardián de la Constitución? / La entrevista de María Isabel Rueda</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/la-propuesta-de-abelardo-de-la-espriella-para-estabilizar-el-sistema-de-salud-en-colombia-con-una-inversion-de-10-billones-en-90-dias-3565391</t>
+          <t>https://www.eltiempo.com/politica/cual-de-los-dos-candidatos-sera-el-mejor-guardian-de-la-constitucion-la-entrevista-de-maria-isabel-rueda-3565401</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 10:36 p. m.</t>
+          <t>18/06/2026 11:27 p. m.</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -990,19 +990,19 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Video del violento atraco con arma de fuego en salón de belleza en el sur de Bogotá: ladrones se llevaron al menos seis celulares</t>
+          <t>Noveno día del Mundial de Estados Unidos, Canadá y México 2026: ¿qué partidos se juegan este viernes 19 de junio? Canal y hora para ver en vivo</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/bogota/video-de-violento-atraco-de-dos-sujetos-con-arma-de-fuego-en-salon-de-belleza-al-sur-de-bogota-hablo-testigo-y-revelo-detalles-clave-del-caso-3565396</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/noveno-dia-del-mundial-de-estados-unidos-canada-y-mexico-2026-que-partidos-se-juegan-este-viernes-19-de-junio-canal-y-hora-para-ver-en-vivo-3565403</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 10:36 p. m.</t>
+          <t>18/06/2026 11:20 p. m.</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -1017,19 +1017,19 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Certezas y preguntas tras el debut de la Selección Colombia en el Mundial: no todo lo cubrió la marea amarilla</t>
+          <t>Turista murió tras intentar salvar la vida de su mamá en medio de paseo en caballo por Central Park, en Estados Unidos: fuertes imágenes de la caída</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/certezas-y-preguntas-tras-el-debut-de-la-seleccion-colombia-en-el-mundial-no-todo-lo-cubrio-la-marea-amarilla-3565400</t>
+          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/turista-murio-tras-intentar-salvar-la-vida-de-su-mama-en-medio-de-paseo-en-caballo-por-central-park-en-estados-unidos-fuertes-imagenes-de-la-caida-3565404</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 10:30 p. m.</t>
+          <t>18/06/2026 11:18 p. m.</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1044,19 +1044,19 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Sánchez en Perú</t>
+          <t>1,3 toneladas de cocaína que iban a ser enviadas a Europa fueron incautadas por la Policía en el Urabá antioqueño: estaban ocultas en un contenedor</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/caricaturas/sanchez-en-peru-3565386</t>
+          <t>https://www.eltiempo.com/colombia/medellin/1-3-toneladas-de-cocaina-que-iban-a-ser-enviadas-a-europa-fueron-incautadas-por-la-policia-en-el-uraba-antioqueno-estaban-ocultas-en-un-contenedor-3565402</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 10:30 p. m.</t>
+          <t>18/06/2026 11:14 p. m.</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
@@ -1071,12 +1071,12 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Confusión felina</t>
+          <t>Nicolás Echavarría y Marcelo Rozo, en la lucha en el US Open de golf, en el que Wyndham Clark picaba en punta</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/caricaturas/confusion-felina-3565383</t>
+          <t>https://www.eltiempo.com/deportes/otros-deportes/nicolas-echavarria-y-marcelo-rozo-en-la-lucha-en-el-us-open-de-golf-en-el-que-wyndham-clark-picaba-en-punta-3565407</t>
         </is>
       </c>
     </row>
@@ -1110,7 +1110,7 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>19/06/2026 01:27 a. m.</t>
+          <t>19/06/2026 04:01 a. m.</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -1125,19 +1125,19 @@
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Defensoría pide frenar violencia política y alarmas de fraude ante segunda vuelta presidencial</t>
+          <t>Suiza confirma el aplazamiento de la reunión entre EEUU, Irán y los mediadores</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/19/defensoria-pide-frenar-violencia-politica-y-alarmas-de-fraude-ante-segunda-vuelta-presidencial/</t>
+          <t>https://caracol.com.co/2026/06/19/suiza-confirma-el-aplazamiento-de-la-reunion-entre-eeuu-iran-y-los-mediadores/</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 10:35 p. m.</t>
+          <t>19/06/2026 03:16 a. m.</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1152,19 +1152,19 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Tribunal concluye que no había motivos para frenar publicidad de campaña de Abelardo De la Espriella</t>
+          <t>Hermano de ‘Fito’ ya está en una cárcel de máxima seguridad en Ecuador</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/19/tribunal-concluye-que-no-habia-motivos-para-frenar-publicidad-de-campana-de-abelardo-de-la-espriella/</t>
+          <t>https://caracol.com.co/2026/06/19/hermano-de-fito-ya-esta-en-una-carcel-de-maxima-seguridad-en-ecuador/</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 10:34 p. m.</t>
+          <t>19/06/2026 01:27 a. m.</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
@@ -1179,19 +1179,19 @@
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Presidente Petro entregó 77.118 hectáreas para comunidades rurales que producen arroz y maíz</t>
+          <t>Defensoría pide frenar violencia política y alarmas de fraude ante segunda vuelta presidencial</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/19/presidente-petro-entrego-77118-hectareas-para-comunidades-rurales-que-producen-arroz-y-maiz/</t>
+          <t>https://caracol.com.co/2026/06/19/defensoria-pide-frenar-violencia-politica-y-alarmas-de-fraude-ante-segunda-vuelta-presidencial/</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 09:56 p. m.</t>
+          <t>18/06/2026 10:35 p. m.</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1206,19 +1206,19 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>México vence a Corea del Sur y clasifica a dieciseisavos de final del Mundial: resumen del partido</t>
+          <t>Tribunal concluye que no había motivos para frenar publicidad de campaña de Abelardo De la Espriella</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/18/en-vivo-mexico-vs-corea-del-sur-minuto-a-minuto-y-transmision-del-partido-hoy/</t>
+          <t>https://caracol.com.co/2026/06/19/tribunal-concluye-que-no-habia-motivos-para-frenar-publicidad-de-campana-de-abelardo-de-la-espriella/</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 09:52 p. m.</t>
+          <t>18/06/2026 10:34 p. m.</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -1233,19 +1233,19 @@
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>¿Puede el empleador determinar el medio día de descanso obligatorio por votar? Esto dice la ley</t>
+          <t>Presidente Petro entregó 77.118 hectáreas para comunidades rurales que producen arroz y maíz</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/19/puede-el-empleador-determinar-el-dia-de-descanso-obligatorio-por-votar-esto-dice-la-ley/</t>
+          <t>https://caracol.com.co/2026/06/19/presidente-petro-entrego-77118-hectareas-para-comunidades-rurales-que-producen-arroz-y-maiz/</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 09:30 p. m.</t>
+          <t>18/06/2026 09:56 p. m.</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1260,19 +1260,19 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Comprar vivienda sin cuota inicial en 2026: ¿Qué entidad ofrece esta opción? Entérese</t>
+          <t>México vence a Corea del Sur y clasifica a dieciseisavos de final del Mundial: resumen del partido</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/19/comprar-vivienda-sin-cuota-inicial-en-2026-que-entidad-ofrece-esta-opcion-enterese/</t>
+          <t>https://caracol.com.co/2026/06/18/en-vivo-mexico-vs-corea-del-sur-minuto-a-minuto-y-transmision-del-partido-hoy/</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 09:24 p. m.</t>
+          <t>18/06/2026 09:52 p. m.</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -1287,19 +1287,19 @@
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>“Siempre voy a defender mi legado, que es el del proceso de paz”: Santos dio pistas sobre su voto</t>
+          <t>¿Puede el empleador determinar el medio día de descanso obligatorio por votar? Esto dice la ley</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/19/siempre-voy-a-defender-mi-legado-que-es-el-del-proceso-de-paz-santos-dio-pistas-sobre-su-voto/</t>
+          <t>https://caracol.com.co/2026/06/19/puede-el-empleador-determinar-el-dia-de-descanso-obligatorio-por-votar-esto-dice-la-ley/</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 09:22 p. m.</t>
+          <t>18/06/2026 09:30 p. m.</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1314,19 +1314,19 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>¿Cuba es el siguiente? Vicepresidente JD Vance llama a la isla a tomar “decisiones inteligentes”</t>
+          <t>Comprar vivienda sin cuota inicial en 2026: ¿Qué entidad ofrece esta opción? Entérese</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/19/cuba-es-el-siguiente-vicepresidente-jd-vance-llama-a-la-isla-a-tomar-decisiones-inteligentes/</t>
+          <t>https://caracol.com.co/2026/06/19/comprar-vivienda-sin-cuota-inicial-en-2026-que-entidad-ofrece-esta-opcion-enterese/</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 07:55 p. m.</t>
+          <t>18/06/2026 09:24 p. m.</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -1341,19 +1341,19 @@
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Histórico del dólar en Colombia: ¿cuál ha sido el punto más bajo y más alto de la moneda? Análisis</t>
+          <t>“Siempre voy a defender mi legado, que es el del proceso de paz”: Santos dio pistas sobre su voto</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/19/historico-del-dolar-en-colombia-cual-ha-sido-el-punto-mas-bajo-y-mas-alto-de-la-moneda-analisis/</t>
+          <t>https://caracol.com.co/2026/06/19/siempre-voy-a-defender-mi-legado-que-es-el-del-proceso-de-paz-santos-dio-pistas-sobre-su-voto/</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 07:33 p. m.</t>
+          <t>18/06/2026 09:22 p. m.</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1368,19 +1368,19 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Así fue la dejación de armas de 100 hombres de la Coordinadora Nacional en Putumayo</t>
+          <t>¿Cuba es el siguiente? Vicepresidente JD Vance llama a la isla a tomar “decisiones inteligentes”</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/19/asi-fue-la-dejacion-de-armas-de-100-hombres-de-la-coordinadora-nacional-en-putumayo/</t>
+          <t>https://caracol.com.co/2026/06/19/cuba-es-el-siguiente-vicepresidente-jd-vance-llama-a-la-isla-a-tomar-decisiones-inteligentes/</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 07:29 p. m.</t>
+          <t>18/06/2026 07:55 p. m.</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
@@ -1395,19 +1395,19 @@
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>Gobierno convocará a sesiones extraordinarias para salvar la Jurisdicción agraria y el MinIgualdad</t>
+          <t>Histórico del dólar en Colombia: ¿cuál ha sido el punto más bajo y más alto de la moneda? Análisis</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/19/gobierno-convocara-a-sesiones-extraordinarias-para-salvar-la-jurisdiccion-agraria-y-el-minigualdad/</t>
+          <t>https://caracol.com.co/2026/06/19/historico-del-dolar-en-colombia-cual-ha-sido-el-punto-mas-bajo-y-mas-alto-de-la-moneda-analisis/</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 07:28 p. m.</t>
+          <t>18/06/2026 07:33 p. m.</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1422,19 +1422,19 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Gobierno venezolano se reunió con oposición para dialogar sobre transición democrática</t>
+          <t>Así fue la dejación de armas de 100 hombres de la Coordinadora Nacional en Putumayo</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/19/gobierno-venezolano-se-reunio-con-oposicion-para-dialogar-sobre-transicion-democratica/</t>
+          <t>https://caracol.com.co/2026/06/19/asi-fue-la-dejacion-de-armas-de-100-hombres-de-la-coordinadora-nacional-en-putumayo/</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 07:21 p. m.</t>
+          <t>18/06/2026 07:29 p. m.</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
@@ -1449,19 +1449,19 @@
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>Corte ordena detención de la senadora Martha Peralta para su indagatoria por el desfalco de la UNGRD</t>
+          <t>Gobierno convocará a sesiones extraordinarias para salvar la Jurisdicción agraria y el MinIgualdad</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/19/corte-ordena-detencion-de-la-senadora-martha-peralta-para-su-indagatoria-por-el-desfalco-de-la-ungrd/</t>
+          <t>https://caracol.com.co/2026/06/19/gobierno-convocara-a-sesiones-extraordinarias-para-salvar-la-jurisdiccion-agraria-y-el-minigualdad/</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 07:13 p. m.</t>
+          <t>18/06/2026 07:28 p. m.</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1476,19 +1476,19 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Supersalud impone medida cautelar a Medic Colombia por fallas en entrega de medicamentos</t>
+          <t>Gobierno venezolano se reunió con oposición para dialogar sobre transición democrática</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/19/supersalud-impone-medida-cautelar-a-medic-colombia-por-fallas-en-entrega-de-medicamentos/</t>
+          <t>https://caracol.com.co/2026/06/19/gobierno-venezolano-se-reunio-con-oposicion-para-dialogar-sobre-transicion-democratica/</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 07:09 p. m.</t>
+          <t>18/06/2026 07:21 p. m.</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
@@ -1503,19 +1503,19 @@
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>Paola Holguín renunció al Centro Democrático tras manifestar diferencias con el partido</t>
+          <t>Corte ordena detención de la senadora Martha Peralta para su indagatoria por el desfalco de la UNGRD</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/19/paola-holguin-renuncio-al-centro-democratico-tras-manifestar-diferencias-con-el-partido/</t>
+          <t>https://caracol.com.co/2026/06/19/corte-ordena-detencion-de-la-senadora-martha-peralta-para-su-indagatoria-por-el-desfalco-de-la-ungrd/</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 07:00 p. m.</t>
+          <t>18/06/2026 07:13 p. m.</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -1530,19 +1530,19 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>CNE amplió plazo para postulación de testigos electorales para segunda vuelta hasta mañana viernes</t>
+          <t>Supersalud impone medida cautelar a Medic Colombia por fallas en entrega de medicamentos</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/19/cne-amplio-plazo-para-postulacion-de-testigos-electorales-para-segunda-vuelta-hasta-manana-viernes/</t>
+          <t>https://caracol.com.co/2026/06/19/supersalud-impone-medida-cautelar-a-medic-colombia-por-fallas-en-entrega-de-medicamentos/</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 06:58 p. m.</t>
+          <t>18/06/2026 07:09 p. m.</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
@@ -1557,19 +1557,19 @@
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>Estos son los descuentos que puede reclamar con el certificado electoral 2026: hasta cuándo aplican</t>
+          <t>Paola Holguín renunció al Centro Democrático tras manifestar diferencias con el partido</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/18/estos-son-los-descuentos-que-puede-reclamar-con-el-certificado-electoral-2026-hasta-cuando-aplican/</t>
+          <t>https://caracol.com.co/2026/06/19/paola-holguin-renuncio-al-centro-democratico-tras-manifestar-diferencias-con-el-partido/</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 06:54 p. m.</t>
+          <t>18/06/2026 07:00 p. m.</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -1584,19 +1584,19 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Locker de Zulma Guzmán sigue bajo análisis: Medicina Legal aún no ha emitido informe oficial</t>
+          <t>CNE amplió plazo para postulación de testigos electorales para segunda vuelta hasta mañana viernes</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/18/locker-de-zulma-guzman-sigue-bajo-analisis-medicina-legal-aun-no-ha-emitido-informe-oficial/</t>
+          <t>https://caracol.com.co/2026/06/19/cne-amplio-plazo-para-postulacion-de-testigos-electorales-para-segunda-vuelta-hasta-manana-viernes/</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 06:46 p. m.</t>
+          <t>18/06/2026 06:58 p. m.</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
@@ -1611,12 +1611,12 @@
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>EE.UU. anunció nuevas recompensas para la captura de líderes de la Mara Salvatrucha en Honduras</t>
+          <t>Estos son los descuentos que puede reclamar con el certificado electoral 2026: hasta cuándo aplican</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/18/eeuu-anuncio-nuevas-recompensas-para-la-captura-de-lideres-de-la-mara-salvatrucha-en-honduras/</t>
+          <t>https://caracol.com.co/2026/06/18/estos-son-los-descuentos-que-puede-reclamar-con-el-certificado-electoral-2026-hasta-cuando-aplican/</t>
         </is>
       </c>
     </row>
@@ -1638,12 +1638,12 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>¿En vilo negociaciones de paz entre EEUU e Irán?</t>
+          <t>¿En vilo negociaciones de paz entre EE. UU. e Irán?</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/internacional/en-vilo-negociaciones-de-paz-entre-eeuu-e-iran-402678</t>
+          <t>https://www.lafm.com.co/internacional/en-vilo-negociaciones-de-paz-entre-ee-uu-e-iran-402678</t>
         </is>
       </c>
     </row>
@@ -2540,12 +2540,12 @@
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>Clima indeciso</t>
+          <t>¿Y mañana?</t>
         </is>
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/caricaturas/2026/06/19/clima-indeciso/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/19/y-manana/</t>
         </is>
       </c>
     </row>
@@ -2567,12 +2567,12 @@
       </c>
       <c r="D77" s="6" t="inlineStr">
         <is>
-          <t>Caricaturas</t>
+          <t>Columnistas</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/caricaturas/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/</t>
         </is>
       </c>
     </row>
@@ -2594,12 +2594,12 @@
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>Colombia milagro</t>
+          <t>Clima indeciso</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/19/colombia-milagro/</t>
+          <t>https://www.vanguardia.com/opinion/caricaturas/2026/06/19/clima-indeciso/</t>
         </is>
       </c>
     </row>
@@ -2621,12 +2621,12 @@
       </c>
       <c r="D79" s="6" t="inlineStr">
         <is>
-          <t>Columnistas</t>
+          <t>Caricaturas</t>
         </is>
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/</t>
+          <t>https://www.vanguardia.com/opinion/caricaturas/</t>
         </is>
       </c>
     </row>
@@ -2648,12 +2648,12 @@
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>Reflexión de viernes para domingo</t>
+          <t>Colombia milagro</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/19/reflexion-de-viernes-para-domingo/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/19/colombia-milagro/</t>
         </is>
       </c>
     </row>
@@ -2675,12 +2675,12 @@
       </c>
       <c r="D81" s="6" t="inlineStr">
         <is>
-          <t>El lamento por los migrantes</t>
+          <t>Reflexión de viernes para domingo</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/19/el-lamento-por-los-migrantes/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/19/reflexion-de-viernes-para-domingo/</t>
         </is>
       </c>
     </row>
@@ -2984,7 +2984,7 @@
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>19/06/2026 12:05 a. m.</t>
+          <t>19/06/2026 12:59 a. m.</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
@@ -2999,12 +2999,12 @@
       </c>
       <c r="D93" s="6" t="inlineStr">
         <is>
-          <t>¿En vísperas del desastre?</t>
+          <t>El desastre del Gobierno con el Minigualdad</t>
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/patricia-lara-salive/en-visperas-del-desastre/</t>
+          <t>https://www.elespectador.com/opinion/editorial/el-desastre-del-gobierno-con-el-minigualdad/</t>
         </is>
       </c>
     </row>
@@ -3026,12 +3026,12 @@
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>¿Qué sigue ahora?</t>
+          <t>¿En vísperas del desastre?</t>
         </is>
       </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/lectores/cartas/que-sigue-ahora/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/patricia-lara-salive/en-visperas-del-desastre/</t>
         </is>
       </c>
     </row>
@@ -3053,12 +3053,12 @@
       </c>
       <c r="D95" s="6" t="inlineStr">
         <is>
-          <t>Por qué voto en blanco, otra vez</t>
+          <t>¿Qué sigue ahora?</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/juan-carlos-botero/por-que-voto-en-blanco-otra-vez/</t>
+          <t>https://www.elespectador.com/opinion/lectores/cartas/que-sigue-ahora/</t>
         </is>
       </c>
     </row>
@@ -3080,12 +3080,12 @@
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>A Cali NO la van a incendiar</t>
+          <t>Por qué voto en blanco, otra vez</t>
         </is>
       </c>
       <c r="E96" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/mario-fernando-prado/a-cali-no-la-van-a-incendiar/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/juan-carlos-botero/por-que-voto-en-blanco-otra-vez/</t>
         </is>
       </c>
     </row>
@@ -3107,12 +3107,12 @@
       </c>
       <c r="D97" s="6" t="inlineStr">
         <is>
-          <t>Una vez más, Spielberg repite su fórmula: ‘El día de la revelación’ (’Disclosure day’, 2026)</t>
+          <t>A Cali NO la van a incendiar</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/criticadecine/una-vez-mas-spielberg-repite-su-formula-el-dia-de-la-revelacion-disclosure-day-2026/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/mario-fernando-prado/a-cali-no-la-van-a-incendiar/</t>
         </is>
       </c>
     </row>
@@ -3161,19 +3161,19 @@
       </c>
       <c r="D99" s="6" t="inlineStr">
         <is>
-          <t>Riesgo extremo</t>
+          <t>Una vez más, Spielberg repite su fórmula: ‘El día de la revelación’ (’Disclosure day’, 2026)</t>
         </is>
       </c>
       <c r="E99" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/francisco-gutierrez-sanin/riesgo-extremo/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/criticadecine/una-vez-mas-spielberg-repite-su-formula-el-dia-de-la-revelacion-disclosure-day-2026/</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 10:20 p. m.</t>
+          <t>19/06/2026 12:05 a. m.</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -3188,66 +3188,58 @@
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
+          <t>Riesgo extremo</t>
+        </is>
+      </c>
+      <c r="E100" s="4" t="inlineStr">
+        <is>
+          <t>https://www.elespectador.com/opinion/columnistas/francisco-gutierrez-sanin/riesgo-extremo/</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="5" t="inlineStr"/>
+      <c r="B101" s="5" t="inlineStr">
+        <is>
+          <t>Medio de Comunicación</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>El Espectador</t>
+        </is>
+      </c>
+      <c r="D101" s="6" t="inlineStr">
+        <is>
           <t>Así quedó la tabla de posiciones del Grupo A del Mundial 2026 tras nueva victoria de México</t>
         </is>
       </c>
-      <c r="E100" s="4" t="inlineStr">
+      <c r="E101" s="7" t="inlineStr">
         <is>
           <t>https://www.elespectador.com/deportes/mundial-2026/asi-quedo-la-tabla-de-posiciones-del-grupo-a-del-mundial-2026-tras-nueva-victoria-de-mexico/</t>
         </is>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" s="5" t="inlineStr">
-        <is>
-          <t>18/06/2026 09:56 p. m.</t>
-        </is>
-      </c>
-      <c r="B101" s="5" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C101" s="5" t="inlineStr">
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr"/>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>Medio de Comunicación</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
         <is>
           <t>El Espectador</t>
         </is>
       </c>
-      <c r="D101" s="6" t="inlineStr">
+      <c r="D102" s="3" t="inlineStr">
         <is>
           <t>México clasificó a los dieciseisavos del Mundial 2026 tras vencer a Corea del Sur</t>
         </is>
       </c>
-      <c r="E101" s="7" t="inlineStr">
+      <c r="E102" s="4" t="inlineStr">
         <is>
           <t>https://www.elespectador.com/deportes/mundial-2026/en-vivo-mexico-vs-corea-del-sur-en-el-mundial-2026-siga-el-minuto-a-minuto-partidos-hoy/</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" s="2" t="inlineStr">
-        <is>
-          <t>18/06/2026 09:49 p. m.</t>
-        </is>
-      </c>
-      <c r="B102" s="2" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C102" s="2" t="inlineStr">
-        <is>
-          <t>El Espectador</t>
-        </is>
-      </c>
-      <c r="D102" s="3" t="inlineStr">
-        <is>
-          <t>JEP imputa a cinco exjefes de las Farc por 243 crímenes contra indígenas y afro en el Caribe</t>
-        </is>
-      </c>
-      <c r="E102" s="4" t="inlineStr">
-        <is>
-          <t>https://www.elespectador.com/judicial/jep-imputa-a-cinco-exjefes-de-las-farc-por-243-crimenes-contra-indigenas-y-afro-en-el-caribe/</t>
         </is>
       </c>
     </row>
@@ -4106,12 +4098,12 @@
       </c>
       <c r="D134" s="3" t="inlineStr">
         <is>
-          <t>Medellín llegó a 123 homicidios tras asesinato de menor y ataque durante partido de Colombia</t>
+          <t>Previsión meteorológica del clima en Cali para este 19 de junio</t>
         </is>
       </c>
       <c r="E134" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/19/medellin-llego-a-123-homicidios-tras-asesinato-de-menor-y-ataque-durante-partido-de-colombia/</t>
+          <t>https://www.infobae.com/colombia/2026/06/19/prevision-meteorologica-del-clima-en-cali-para-este-19-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4133,12 +4125,12 @@
       </c>
       <c r="D135" s="6" t="inlineStr">
         <is>
-          <t>Pico y Placa Bogotá: evita multas este 19 de junio</t>
+          <t>Clima en Medellín: conoce el pronóstico y prepárate antes de salir</t>
         </is>
       </c>
       <c r="E135" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/19/pico-y-placa-bogota-evita-multas-este-19-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/19/clima-en-medellin-conoce-el-pronostico-y-preparate-antes-de-salir/</t>
         </is>
       </c>
     </row>
@@ -4160,12 +4152,12 @@
       </c>
       <c r="D136" s="3" t="inlineStr">
         <is>
-          <t>Resultados de la Lotería de Bogotá hoy, jueves 18 de junio de 2026: número ganador</t>
+          <t>Clima en Cartagena de Indias: temperatura y probabilidad de lluvia para este 19 de junio</t>
         </is>
       </c>
       <c r="E136" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/19/resultados-de-la-loteria-de-bogota-hoy-jueves-18-de-junio-de-2026-numero-ganador/</t>
+          <t>https://www.infobae.com/colombia/2026/06/19/clima-en-cartagena-de-indias-temperatura-y-probabilidad-de-lluvia-para-este-19-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4187,12 +4179,12 @@
       </c>
       <c r="D137" s="6" t="inlineStr">
         <is>
-          <t>“Reconsidere sus planes”: EE. UU. alerta por posibles protestas tras segunda vuelta en Colombia</t>
+          <t>Barranquilla: el pronóstico del clima para este 19 de junio</t>
         </is>
       </c>
       <c r="E137" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/19/reconsidere-sus-planes-ee-uu-alerta-por-posibles-protestas-tras-segunda-vuelta-en-colombia/</t>
+          <t>https://www.infobae.com/colombia/2026/06/19/barranquilla-el-pronostico-del-clima-para-este-19-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4214,12 +4206,12 @@
       </c>
       <c r="D138" s="3" t="inlineStr">
         <is>
-          <t>Más de 350 desplazados en Antioquia por choques entre disidencias Farc y Clan del Golfo</t>
+          <t>¿Cómo estará el clima en Bogotá?</t>
         </is>
       </c>
       <c r="E138" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/19/mas-de-350-desplazados-en-antioquia-por-choques-entre-disidencias-farc-y-clan-del-golfo/</t>
+          <t>https://www.infobae.com/colombia/2026/06/19/como-estara-el-clima-en-bogota/</t>
         </is>
       </c>
     </row>
@@ -4241,12 +4233,12 @@
       </c>
       <c r="D139" s="6" t="inlineStr">
         <is>
-          <t>“Nos jugamos nuestra estabilidad”: empleados de Air-e harán plantón contra liquidación</t>
+          <t>Resultado Sinuano Noche hoy 18 de junio</t>
         </is>
       </c>
       <c r="E139" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/19/nos-jugamos-nuestra-estabilidad-empleados-de-air-e-haran-planton-contra-liquidacion/</t>
+          <t>https://www.infobae.com/colombia/2026/06/19/resultado-sinuano-noche-hoy-18-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4268,12 +4260,12 @@
       </c>
       <c r="D140" s="3" t="inlineStr">
         <is>
-          <t>Coronel Portillo, Ucayali - Perú registró un sismo de 4.8 de intensidad este 18 de junio</t>
+          <t>Medellín llegó a 123 homicidios tras asesinato de menor y ataque durante partido de Colombia</t>
         </is>
       </c>
       <c r="E140" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/19/coronel-portillo-ucayali-peru-registro-un-sismo-de-48-de-intensidad-este-18-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/19/medellin-llego-a-123-homicidios-tras-asesinato-de-menor-y-ataque-durante-partido-de-colombia/</t>
         </is>
       </c>
     </row>
@@ -4295,12 +4287,12 @@
       </c>
       <c r="D141" s="6" t="inlineStr">
         <is>
-          <t>Resultado Chontico Noche: números ganadores del último sorteo hoy, jueves 18 de junio de 2026</t>
+          <t>Pico y Placa Bogotá: evita multas este 19 de junio</t>
         </is>
       </c>
       <c r="E141" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/19/resultado-chontico-noche-numeros-ganadores-del-ultimo-sorteo-hoy-jueves-18-de-junio-de-2026/</t>
+          <t>https://www.infobae.com/colombia/2026/06/19/pico-y-placa-bogota-evita-multas-este-19-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4322,12 +4314,12 @@
       </c>
       <c r="D142" s="3" t="inlineStr">
         <is>
-          <t>Resultado Super Astro Luna HOY: número ganador del jueves 18 de junio</t>
+          <t>Resultados de la Lotería de Bogotá hoy, jueves 18 de junio de 2026: número ganador</t>
         </is>
       </c>
       <c r="E142" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/19/resultado-super-astro-luna-hoy-numero-ganador-del-jueves-18-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/19/resultados-de-la-loteria-de-bogota-hoy-jueves-18-de-junio-de-2026-numero-ganador/</t>
         </is>
       </c>
     </row>
@@ -4349,12 +4341,12 @@
       </c>
       <c r="D143" s="6" t="inlineStr">
         <is>
-          <t>Tenga en cuenta: Así regirá el pico y placa en Cartagena este viernes</t>
+          <t>“Reconsidere sus planes”: EE. UU. alerta por posibles protestas tras segunda vuelta en Colombia</t>
         </is>
       </c>
       <c r="E143" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/19/tenga-en-cuenta-asi-regira-el-pico-y-placa-en-cartagena-este-viernes/</t>
+          <t>https://www.infobae.com/colombia/2026/06/19/reconsidere-sus-planes-ee-uu-alerta-por-posibles-protestas-tras-segunda-vuelta-en-colombia/</t>
         </is>
       </c>
     </row>
@@ -4376,12 +4368,12 @@
       </c>
       <c r="D144" s="3" t="inlineStr">
         <is>
-          <t>Pico y placa en Villavicencio hoy 19 de junio de 2026, así regirá la medida</t>
+          <t>Más de 350 desplazados en Antioquia por choques entre disidencias Farc y Clan del Golfo</t>
         </is>
       </c>
       <c r="E144" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/19/pico-y-placa-en-villavicencio-hoy-19-de-junio-de-2026-asi-regira-la-medida/</t>
+          <t>https://www.infobae.com/colombia/2026/06/19/mas-de-350-desplazados-en-antioquia-por-choques-entre-disidencias-farc-y-clan-del-golfo/</t>
         </is>
       </c>
     </row>
@@ -4403,12 +4395,12 @@
       </c>
       <c r="D145" s="6" t="inlineStr">
         <is>
-          <t>Este es el Pico y Placa en Cali para este viernes 19 de junio</t>
+          <t>“Nos jugamos nuestra estabilidad”: empleados de Air-e harán plantón contra liquidación</t>
         </is>
       </c>
       <c r="E145" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/19/este-es-el-pico-y-placa-en-cali-para-este-viernes-19-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/19/nos-jugamos-nuestra-estabilidad-empleados-de-air-e-haran-planton-contra-liquidacion/</t>
         </is>
       </c>
     </row>
@@ -4430,12 +4422,12 @@
       </c>
       <c r="D146" s="3" t="inlineStr">
         <is>
-          <t>Tenga en cuenta: así regirá el Pico y Placa en Medellín este viernes 19 de junio</t>
+          <t>Coronel Portillo, Ucayali - Perú registró un sismo de 4.8 de intensidad este 18 de junio</t>
         </is>
       </c>
       <c r="E146" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/19/tenga-en-cuenta-asi-regira-el-pico-y-placa-en-medellin-este-viernes-19-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/19/coronel-portillo-ucayali-peru-registro-un-sismo-de-48-de-intensidad-este-18-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4457,12 +4449,12 @@
       </c>
       <c r="D147" s="6" t="inlineStr">
         <is>
-          <t>Inseguridad en Bogotá: ¿percepción o realidad?, expertos y autoridades respondieron a la ciudadanía</t>
+          <t>Resultado Chontico Noche: números ganadores del último sorteo hoy, jueves 18 de junio de 2026</t>
         </is>
       </c>
       <c r="E147" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/19/inseguridad-en-bogota-percepcion-o-realidad-expertos-y-autoridades-respondieron-a-la-ciudadania/</t>
+          <t>https://www.infobae.com/colombia/2026/06/19/resultado-chontico-noche-numeros-ganadores-del-ultimo-sorteo-hoy-jueves-18-de-junio-de-2026/</t>
         </is>
       </c>
     </row>
@@ -4484,12 +4476,12 @@
       </c>
       <c r="D148" s="3" t="inlineStr">
         <is>
-          <t>Un jugador de la Selección Colombia apareció en el once menos deseado de la Copa del Mundo</t>
+          <t>Resultado Super Astro Luna HOY: número ganador del jueves 18 de junio</t>
         </is>
       </c>
       <c r="E148" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/06/19/un-jugador-de-la-seleccion-colombia-aparecio-en-el-once-menos-deseado-de-la-copa-del-mundo/</t>
+          <t>https://www.infobae.com/colombia/2026/06/19/resultado-super-astro-luna-hoy-numero-ganador-del-jueves-18-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4511,12 +4503,12 @@
       </c>
       <c r="D149" s="6" t="inlineStr">
         <is>
-          <t>Jhonny Ramírez sugirió cómo debe ser el mercado de pases para Millonarios: “Necesita jugadores de experiencia”</t>
+          <t>Tenga en cuenta: Así regirá el pico y placa en Cartagena este viernes</t>
         </is>
       </c>
       <c r="E149" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/06/19/jhonny-ramirez-sugirio-como-debe-ser-el-mercado-de-pases-para-millonarios-necesita-jugadores-de-experiencia/</t>
+          <t>https://www.infobae.com/colombia/2026/06/19/tenga-en-cuenta-asi-regira-el-pico-y-placa-en-cartagena-este-viernes/</t>
         </is>
       </c>
     </row>
@@ -4538,12 +4530,12 @@
       </c>
       <c r="D150" s="3" t="inlineStr">
         <is>
-          <t>Jugador con pasado en Junior afirmó que Millonarios es el equipo más grande del fútbol colombiano: “Por su hinchada”</t>
+          <t>Pico y placa en Villavicencio hoy 19 de junio de 2026, así regirá la medida</t>
         </is>
       </c>
       <c r="E150" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/06/19/jugador-con-pasado-en-junior-afirmo-que-millonarios-es-el-equipo-mas-grande-del-futbol-colombiano-por-su-hinchada/</t>
+          <t>https://www.infobae.com/colombia/2026/06/19/pico-y-placa-en-villavicencio-hoy-19-de-junio-de-2026-asi-regira-la-medida/</t>
         </is>
       </c>
     </row>
@@ -4565,12 +4557,12 @@
       </c>
       <c r="D151" s="6" t="inlineStr">
         <is>
-          <t>Gury Rodríguez se retractó con Esteban Restrepo tras fallo de un juez, pero causó polémica al hacerlo: “Le dije rata, pero no lo es”</t>
+          <t>Este es el Pico y Placa en Cali para este viernes 19 de junio</t>
         </is>
       </c>
       <c r="E151" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/19/gury-rodriguez-se-retracto-con-esteban-restrepo-tras-fallo-de-un-juez-pero-causo-polemica-al-hacerlo-le-dije-rata-pero-no-lo-es/</t>
+          <t>https://www.infobae.com/colombia/2026/06/19/este-es-el-pico-y-placa-en-cali-para-este-viernes-19-de-junio/</t>
         </is>
       </c>
     </row>
@@ -4592,19 +4584,19 @@
       </c>
       <c r="D152" s="3" t="inlineStr">
         <is>
-          <t>Ley seca en Bogotá hasta el lunes 22 de junio: estas son las multas y sanciones para las personas y locales que incumplan la restricción</t>
+          <t>Tenga en cuenta: así regirá el Pico y Placa en Medellín este viernes 19 de junio</t>
         </is>
       </c>
       <c r="E152" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/19/ley-seca-en-bogota-hasta-el-lunes-22-de-junio-estas-son-las-multas-y-sanciones-para-las-personas-y-locales-que-incumplan-la-restriccion/</t>
+          <t>https://www.infobae.com/colombia/2026/06/19/tenga-en-cuenta-asi-regira-el-pico-y-placa-en-medellin-este-viernes-19-de-junio/</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 12:00 a. m.</t>
+          <t>19/06/2026 12:00 a. m.</t>
         </is>
       </c>
       <c r="B153" s="5" t="inlineStr">
@@ -4619,19 +4611,19 @@
       </c>
       <c r="D153" s="6" t="inlineStr">
         <is>
-          <t>Elecciones presidenciales de Colombia 2026 en VIVO: el Pacto Histórico exige a la Procuraduría garantías para las elecciones del domingo</t>
+          <t>Inseguridad en Bogotá: ¿percepción o realidad?, expertos y autoridades respondieron a la ciudadanía</t>
         </is>
       </c>
       <c r="E153" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/18/elecciones-presidenciales-de-colombia-2026-en-vivo-ivan-cepeda-insiste-en-debatir-con-abelardo-de-la-espriella/</t>
+          <t>https://www.infobae.com/colombia/2026/06/19/inseguridad-en-bogota-percepcion-o-realidad-expertos-y-autoridades-respondieron-a-la-ciudadania/</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 07:52 p. m.</t>
+          <t>18/06/2026 06:30 p. m.</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
@@ -4641,24 +4633,24 @@
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D154" s="3" t="inlineStr">
         <is>
-          <t>Duerma informado con las movidas de este 18 de junio de 2026</t>
+          <t>La Fiscalía abre investigación contra el expresidente Álvaro Uribe por “su presunta responsabilidad en la conformación y acción de grupos paramilitares en Antioquia”</t>
         </is>
       </c>
       <c r="E154" s="4" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/duerma-informado-con-las-movidas-de-este-18-de-junio-de-2026/</t>
+          <t>https://cambiocolombia.com/poder/articulo/2026/6/la-fiscalia-abre-investigacion-contra-el-expresidente-alvaro-uribe-por-su-presunta-responsabilidad-en-la-conformacion-y-accion-de-grupos-paramilitares-en-antioquia</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 07:50 p. m.</t>
+          <t>18/06/2026 05:30 p. m.</t>
         </is>
       </c>
       <c r="B155" s="5" t="inlineStr">
@@ -4668,24 +4660,24 @@
       </c>
       <c r="C155" s="5" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D155" s="6" t="inlineStr">
         <is>
-          <t>Últimos días para acceder a la experiencia ABC de la Democracia</t>
+          <t>Tribunal niega tutela que pedía suspender piezas publicitarias de la campaña de Abelardo de la Espriella y Defensores de la Patria</t>
         </is>
       </c>
       <c r="E155" s="7" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/ultimos-dias-para-acceder-a-la-experiencia-abc-de-la-democracia/</t>
+          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/tribunal-niega-tutela-que-pedia-suspender-piezas-publicitarias-de-la-campana-de-abelardo-de-la-espriella-y-defensores-de-la-patria</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 07:33 p. m.</t>
+          <t>18/06/2026 04:00 p. m.</t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
@@ -4695,24 +4687,24 @@
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D156" s="3" t="inlineStr">
         <is>
-          <t>Fiscalía llama a indagatoria a Álvaro Uribe por las masacres de El Aro y La Granja</t>
+          <t>Alerta en Leticia por la desaparición de un jaguar rescatado en la Universidad Nacional, sede Amazonia</t>
         </is>
       </c>
       <c r="E156" s="4" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/fiscalia-llama-a-indagatoria-a-alvaro-uribe-por-las-masacres-de-el-aro-y-la-granja/</t>
+          <t>https://cambiocolombia.com/medio-ambiente/articulo/2026/6/alerta-en-leticia-por-la-desaparicion-de-un-jaguar-rescatado-en-la-universidad-nacional-sede-amazonia</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 06:22 p. m.</t>
+          <t>18/06/2026 03:45 p. m.</t>
         </is>
       </c>
       <c r="B157" s="5" t="inlineStr">
@@ -4722,24 +4714,24 @@
       </c>
       <c r="C157" s="5" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D157" s="6" t="inlineStr">
         <is>
-          <t>Cepeda promete pruebas contra De la Espriella por presunta compra de votos</t>
+          <t>¿Por qué Bogotá declaró alerta amarilla hospitalaria para la segunda vuelta?</t>
         </is>
       </c>
       <c r="E157" s="7" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/cepeda-promete-pruebas-contra-de-la-espriella-por-presunta-compra-de-votos/</t>
+          <t>https://cambiocolombia.com/salud-y-bienestar/articulo/2026/6/por-que-bogota-declaro-alerta-amarilla-hospitalaria-para-la-segunda-vuelta</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 05:49 p. m.</t>
+          <t>18/06/2026 03:15 p. m.</t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
@@ -4749,24 +4741,24 @@
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D158" s="3" t="inlineStr">
         <is>
-          <t>Oficialmente se hundió en Cámara el proyecto de ley de reforma agraria</t>
+          <t>Más de 1.500 motociclistas en Bogotá podrían perder la licencia por reincidir en infracciones de tránsito</t>
         </is>
       </c>
       <c r="E158" s="4" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/oficialmente-se-hundio-en-camara-el-proyecto-de-ley-de-reforma-agraria/</t>
+          <t>https://cambiocolombia.com/pais/articulo/2026/6/mas-de-1500-motociclistas-en-bogota-podrian-perder-la-licencia-por-reincidir-en-infracciones-de-transito</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 05:05 p. m.</t>
+          <t>18/06/2026 01:46 p. m.</t>
         </is>
       </c>
       <c r="B159" s="5" t="inlineStr">
@@ -4776,24 +4768,24 @@
       </c>
       <c r="C159" s="5" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D159" s="6" t="inlineStr">
         <is>
-          <t>Flip vuelve a alertar por ataques de Abelardo de la Espriella a la prensa</t>
+          <t>ELN afirma que está listo para negociar la paz o continuar la guerra con el próximo gobierno</t>
         </is>
       </c>
       <c r="E159" s="7" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/flip-vuelve-a-alertar-por-ataques-de-abelardo-de-la-espriella-a-la-prensa/</t>
+          <t>https://cambiocolombia.com/conflicto-armado-en-colombia/articulo/2026/6/eln-afirma-que-esta-listo-para-negociar-la-paz-o-continuar-la-guerra-con-el-proximo-gobierno</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 03:57 p. m.</t>
+          <t>18/06/2026 01:00 p. m.</t>
         </is>
       </c>
       <c r="B160" s="2" t="inlineStr">
@@ -4803,24 +4795,24 @@
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D160" s="3" t="inlineStr">
         <is>
-          <t>Martha Peralta rinde indagatoria ante la Corte Suprema por caso Ungrd</t>
+          <t>Guillermo Reyes le responde a Gustavo Petro: niega campaña contra Verónica Alcocer y apunta a la primera dama</t>
         </is>
       </c>
       <c r="E160" s="4" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/martha-peralta-rinde-indagatoria-ante-la-corte-suprema-por-caso-ungrd/</t>
+          <t>https://cambiocolombia.com/poder/articulo/2026/6/guillermo-reyes-le-responde-a-gustavo-petro-niega-campana-contra-veronica-alcocer-y-apunta-a-la-primera-dama</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 02:32 p. m.</t>
+          <t>18/06/2026 12:30 p. m.</t>
         </is>
       </c>
       <c r="B161" s="5" t="inlineStr">
@@ -4830,24 +4822,24 @@
       </c>
       <c r="C161" s="5" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D161" s="6" t="inlineStr">
         <is>
-          <t>MOE alerta presiones laborales para influir en el voto en Bogotá y Antioquia</t>
+          <t>Javier Pava regresa a la UNGRD tras la salida de Carlos Carrillo: asumirá la preparación del país para el Fenómeno de El Niño</t>
         </is>
       </c>
       <c r="E161" s="7" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/moe-alerta-presiones-laborales-para-votar-en-bogota-y-antioquia/</t>
+          <t>https://cambiocolombia.com/pais/articulo/2026/6/javier-pava-regresa-a-la-ungrd-tras-la-salida-de-carlos-carrillo-asumira-la-preparacion-del-pais-para-el-fenomeno-de-el-nino</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 01:08 p. m.</t>
+          <t>18/06/2026 11:30 a. m.</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
@@ -4857,24 +4849,24 @@
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D162" s="3" t="inlineStr">
         <is>
-          <t>Diario de Campaña: Trump con Abelardo. Benedetti critica a Carrillo</t>
+          <t>¿Información imprecisa? Ministerio de Defensa rechazó el informe del Financial Times sobre narcotráfico y defendió resultados del gobierno</t>
         </is>
       </c>
       <c r="E162" s="4" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/diario-de-campana-trump-con-abelardo-benedetti-critica-a-carrillo/</t>
+          <t>https://cambiocolombia.com/conflicto-armado-en-colombia/articulo/2026/6/informacion-imprecisa-ministerio-de-defensa-rechazo-el-informe-del-financial-times-sobre-narcotrafico-y-defendio-resultados-del-gobierno</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 12:38 p. m.</t>
+          <t>18/06/2026 09:05 a. m.</t>
         </is>
       </c>
       <c r="B163" s="5" t="inlineStr">
@@ -4884,24 +4876,24 @@
       </c>
       <c r="C163" s="5" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D163" s="6" t="inlineStr">
         <is>
-          <t>Dane: Actividad económica creció 3,3% en abril de 2026</t>
+          <t>Bogotá se prepara para un mes de orgullo, memoria y reivindicación con cuatro marchas LGBTIQ+</t>
         </is>
       </c>
       <c r="E163" s="7" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/dane-economia-crecio-33-en-abril-de-2026-respecto-a-2025/</t>
+          <t>https://cambiocolombia.com/pais/articulo/2026/6/bogota-se-prepara-para-un-mes-de-orgullo-memoria-y-reivindicacion-con-cuatro-marchas-lgbtiq</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 12:21 p. m.</t>
+          <t>18/06/2026 08:30 a. m.</t>
         </is>
       </c>
       <c r="B164" s="2" t="inlineStr">
@@ -4911,24 +4903,24 @@
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D164" s="3" t="inlineStr">
         <is>
-          <t>Guiño de Christian Daes a Abelardo en evento de la Selección Colombia</t>
+          <t>¿Cuándo y dónde juega Colombia su próximo partido en el Mundial 2026?</t>
         </is>
       </c>
       <c r="E164" s="4" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/guino-de-christian-daes-a-abelardo-en-evento-de-la-seleccion-colombia/</t>
+          <t>https://cambiocolombia.com/pais/articulo/2026/6/cuando-y-donde-juega-colombia-su-proximo-partido-en-el-mundial-2026</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 11:25 a. m.</t>
+          <t>18/06/2026 07:15 a. m.</t>
         </is>
       </c>
       <c r="B165" s="5" t="inlineStr">
@@ -4938,24 +4930,24 @@
       </c>
       <c r="C165" s="5" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D165" s="6" t="inlineStr">
         <is>
-          <t>Van 181 expedientes contra funcionarios por participación en política</t>
+          <t>Trump intervino de nuevo en la contienda electoral colombiana pidiendo votar por Abelardo de la Espriella</t>
         </is>
       </c>
       <c r="E165" s="7" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/van-181-expedientes-contra-funcionarios-por-participacion-en-politica/</t>
+          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/trump-intervino-de-nuevo-en-la-contienda-electoral-colombiana-pidiendo-votar-por-abelardo-de-la-espriella</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 10:24 a. m.</t>
+          <t>18/06/2026 02:00 a. m.</t>
         </is>
       </c>
       <c r="B166" s="2" t="inlineStr">
@@ -4965,24 +4957,24 @@
       </c>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D166" s="3" t="inlineStr">
         <is>
-          <t>Embajador en Suecia niega campaña de desprestigio contra primera dama</t>
+          <t>Procuraduría abrió indagación sobre aeropuertos rurales del Gobierno Petro tras revelaciones sobre que ninguno supera el 20 por ciento de avance</t>
         </is>
       </c>
       <c r="E166" s="4" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/embajador-en-suecia-niega-campana-de-desprestigio-contra-primera-dama/</t>
+          <t>https://cambiocolombia.com/pais/articulo/2026/6/procuraduria-abrio-indagacion-sobre-aeropuertos-rurales-del-gobierno-petro-tras-revelaciones-sobre-que-ninguno-supera-el-20-por-ciento-de-avance</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 10:23 a. m.</t>
+          <t>17/06/2026 05:30 p. m.</t>
         </is>
       </c>
       <c r="B167" s="5" t="inlineStr">
@@ -4992,24 +4984,24 @@
       </c>
       <c r="C167" s="5" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D167" s="6" t="inlineStr">
         <is>
-          <t>Más de 50 organizaciones llaman a campañas a aceptar resultados electorales</t>
+          <t>¿Qué pasa si queda en empate la segunda vuelta o si gana el voto en blanco?</t>
         </is>
       </c>
       <c r="E167" s="7" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/mas-de-50-organizaciones-llaman-a-campanas-a-aceptar-resultados-electorales/</t>
+          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/que-pasa-si-queda-en-empate-la-segunda-vuelta-o-si-gana-el-voto-en-blanco</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026 09:28 a. m.</t>
+          <t>17/06/2026 02:30 p. m.</t>
         </is>
       </c>
       <c r="B168" s="2" t="inlineStr">
@@ -5019,24 +5011,24 @@
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D168" s="3" t="inlineStr">
         <is>
-          <t>Trump replica apoyo a Abelardo tras petición de no incidir en elecciones</t>
+          <t>Ley Jineth Bedoya: ¿cómo funcionará la nueva ley para minimizar la revictimización desde el Estado para mujeres y niñas?</t>
         </is>
       </c>
       <c r="E168" s="4" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/trump-replica-apoyo-a-abelardo-tras-peticion-de-no-incidir-en-elecciones/</t>
+          <t>https://cambiocolombia.com/genero/articulo/2026/6/ley-jineth-bedoya-como-funcionara-la-nueva-ley-para-minimizar-la-revictimizacion-desde-el-estado-para-mujeres-y-ninas</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="5" t="inlineStr">
         <is>
-          <t>18/06/2026 08:28 a. m.</t>
+          <t>17/06/2026 01:45 p. m.</t>
         </is>
       </c>
       <c r="B169" s="5" t="inlineStr">
@@ -5046,26 +5038,22 @@
       </c>
       <c r="C169" s="5" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>Cambio Colombia</t>
         </is>
       </c>
       <c r="D169" s="6" t="inlineStr">
         <is>
-          <t>Cepeda en RCN: Acuerdo Nacional, debates y acusaciones de De la Espriella</t>
+          <t>Los nuevos detalles que reveló la esteticista que estuvo en la cirugía que causó muerte de Yulixa Toloza</t>
         </is>
       </c>
       <c r="E169" s="7" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/cepeda-en-rcn-acuerdo-nacional-debates-y-acusaciones-de-de-la-espriella/</t>
+          <t>https://cambiocolombia.com/los-nuevos-detalles-que-revelo-la-esteticista-que-estuvo-en-la-cirugia-que-causo-muerte-de-yulixa-toloza</t>
         </is>
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="2" t="inlineStr">
-        <is>
-          <t>18/06/2026 07:18 a. m.</t>
-        </is>
-      </c>
+      <c r="A170" s="2" t="inlineStr"/>
       <c r="B170" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5073,26 +5061,22 @@
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D170" s="3" t="inlineStr">
         <is>
-          <t>Desayune informado con las claves de este 18 de junio de 2026</t>
+          <t>Corte Suprema ordena captura de la senadora Martha Peralta en plena diligencia por caso de la UNGRD</t>
         </is>
       </c>
       <c r="E170" s="4" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/desayune-informado-con-las-claves-de-este-18-de-junio-de-2026/</t>
+          <t>https://www.elcolombiano.com/colombia/corte-detuvo-a-la-senadora-martha-peralta-CF37895315</t>
         </is>
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="5" t="inlineStr">
-        <is>
-          <t>17/06/2026 08:12 p. m.</t>
-        </is>
-      </c>
+      <c r="A171" s="5" t="inlineStr"/>
       <c r="B171" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5100,26 +5084,22 @@
       </c>
       <c r="C171" s="5" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D171" s="6" t="inlineStr">
         <is>
-          <t>Duerma informado con las movidas de este 17 de junio de 2026</t>
+          <t>El país dice a candidatos: “Aceptar los resultados es un deber democrático”</t>
         </is>
       </c>
       <c r="E171" s="7" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/duerma-informado-con-las-movidas-de-este-17-de-junio-de-2026/</t>
+          <t>https://www.elcolombiano.com/colombia/abelardo-de-la-espriella-e-ivan-cepeda-los-llaman-a-aceptar-resultados-electorales-AF37899180</t>
         </is>
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="2" t="inlineStr">
-        <is>
-          <t>17/06/2026 07:51 p. m.</t>
-        </is>
-      </c>
+      <c r="A172" s="2" t="inlineStr"/>
       <c r="B172" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5127,26 +5107,22 @@
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D172" s="3" t="inlineStr">
         <is>
-          <t>Economistas y políticos progresistas dan apoyo al modelo económico Petro-Cepeda</t>
+          <t>La Selección de México encontró el gol, el alivio y la clasificación en Guadalajara</t>
         </is>
       </c>
       <c r="E172" s="4" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/economistas-y-politicos-de-izquierda-dan-apoyo-al-modelo-economico-petro-cepeda/</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/en-vivo-seleccion-mexico-vs-corea-del-sur-mundial-2026-LF37895790</t>
         </is>
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="5" t="inlineStr">
-        <is>
-          <t>17/06/2026 07:33 p. m.</t>
-        </is>
-      </c>
+      <c r="A173" s="5" t="inlineStr"/>
       <c r="B173" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5154,26 +5130,22 @@
       </c>
       <c r="C173" s="5" t="inlineStr">
         <is>
-          <t>La Silla Vacía</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D173" s="6" t="inlineStr">
         <is>
-          <t>Congresistas gringos piden a Trump “no interferir” en las elecciones</t>
+          <t>A tres días de elecciones, Fiscalía llama a indagatoria a Álvaro Uribe por masacres de El Aro y La Granja ocurridas hace 30 años</t>
         </is>
       </c>
       <c r="E173" s="7" t="inlineStr">
         <is>
-          <t>https://www.lasillavacia.com/en-vivo/congresistas-gringos-piden-a-trump-no-interferir-en-las-elecciones/</t>
+          <t>https://www.elcolombiano.com/colombia/alvaro-uribe-velez-fiscalia-lo-cita-a-indagatoria-por-masacres-del-aro-y-la-granja-HF37891897</t>
         </is>
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="2" t="inlineStr">
-        <is>
-          <t>18/06/2026 06:30 p. m.</t>
-        </is>
-      </c>
+      <c r="A174" s="2" t="inlineStr"/>
       <c r="B174" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5181,26 +5153,22 @@
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D174" s="3" t="inlineStr">
         <is>
-          <t>La Fiscalía abre investigación contra el expresidente Álvaro Uribe por “su presunta responsabilidad en la conformación y acción de grupos paramilitares en Antioquia”</t>
+          <t>La lección del texano</t>
         </is>
       </c>
       <c r="E174" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/poder/articulo/2026/6/la-fiscalia-abre-investigacion-contra-el-expresidente-alvaro-uribe-por-su-presunta-responsabilidad-en-la-conformacion-y-accion-de-grupos-paramilitares-en-antioquia</t>
+          <t>https://www.elcolombiano.com/multimedia/videos/la-leccion-del-texano-IE37884491</t>
         </is>
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="5" t="inlineStr">
-        <is>
-          <t>18/06/2026 05:30 p. m.</t>
-        </is>
-      </c>
+      <c r="A175" s="5" t="inlineStr"/>
       <c r="B175" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5208,26 +5176,22 @@
       </c>
       <c r="C175" s="5" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D175" s="6" t="inlineStr">
         <is>
-          <t>Tribunal niega tutela que pedía suspender piezas publicitarias de la campaña de Abelardo de la Espriella y Defensores de la Patria</t>
+          <t>A sus 111 años murió don Luis, el nacido en Antioquia que era el hombre más viejo en Estados Unidos</t>
         </is>
       </c>
       <c r="E175" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/tribunal-niega-tutela-que-pedia-suspender-piezas-publicitarias-de-la-campana-de-abelardo-de-la-espriella-y-defensores-de-la-patria</t>
+          <t>https://www.elcolombiano.com/antioquia/hombre-nacido-en-andes-antioquia-murio-a-los-111-anos-en-estados-unidos-HF37897606</t>
         </is>
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="2" t="inlineStr">
-        <is>
-          <t>18/06/2026 04:00 p. m.</t>
-        </is>
-      </c>
+      <c r="A176" s="2" t="inlineStr"/>
       <c r="B176" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5235,26 +5199,22 @@
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D176" s="3" t="inlineStr">
         <is>
-          <t>Alerta en Leticia por la desaparición de un jaguar rescatado en la Universidad Nacional, sede Amazonia</t>
+          <t>¿Está Colombia clasificada a segunda ronda en el Mundial o qué le falta para asegurarse? Estas son las opciones</t>
         </is>
       </c>
       <c r="E176" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/medio-ambiente/articulo/2026/6/alerta-en-leticia-por-la-desaparicion-de-un-jaguar-rescatado-en-la-universidad-nacional-sede-amazonia</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/que-necesita-colombia-para-clasificar-a-la-siguiente-fase-del-mundial-de-norteamerica-IE37882138</t>
         </is>
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="5" t="inlineStr">
-        <is>
-          <t>18/06/2026 03:45 p. m.</t>
-        </is>
-      </c>
+      <c r="A177" s="5" t="inlineStr"/>
       <c r="B177" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5262,26 +5222,22 @@
       </c>
       <c r="C177" s="5" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D177" s="6" t="inlineStr">
         <is>
-          <t>¿Por qué Bogotá declaró alerta amarilla hospitalaria para la segunda vuelta?</t>
+          <t>Otras tres derrotas en el Congreso: al Gobierno Petro le archivaron estas iniciativas</t>
         </is>
       </c>
       <c r="E177" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/salud-y-bienestar/articulo/2026/6/por-que-bogota-declaro-alerta-amarilla-hospitalaria-para-la-segunda-vuelta</t>
+          <t>https://www.elcolombiano.com/colombia/congreso-archivo-tres-iniciativas-del-gobierno-petro-KL37870497</t>
         </is>
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="2" t="inlineStr">
-        <is>
-          <t>18/06/2026 03:15 p. m.</t>
-        </is>
-      </c>
+      <c r="A178" s="2" t="inlineStr"/>
       <c r="B178" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5289,26 +5245,22 @@
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D178" s="3" t="inlineStr">
         <is>
-          <t>Más de 1.500 motociclistas en Bogotá podrían perder la licencia por reincidir en infracciones de tránsito</t>
+          <t>Más de 50 organizaciones piden compromiso público de Cepeda y Abelardo de reconocer resultados de segunda vuelta presidencial</t>
         </is>
       </c>
       <c r="E178" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/pais/articulo/2026/6/mas-de-1500-motociclistas-en-bogota-podrian-perder-la-licencia-por-reincidir-en-infracciones-de-transito</t>
+          <t>https://www.elcolombiano.com/especiales/elecciones-2026/mas-50-organizaciones-piden-reconocer-resultados-segunda-vuelta-presidencia-HF37897077</t>
         </is>
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="5" t="inlineStr">
-        <is>
-          <t>18/06/2026 01:46 p. m.</t>
-        </is>
-      </c>
+      <c r="A179" s="5" t="inlineStr"/>
       <c r="B179" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5316,26 +5268,22 @@
       </c>
       <c r="C179" s="5" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D179" s="6" t="inlineStr">
         <is>
-          <t>ELN afirma que está listo para negociar la paz o continuar la guerra con el próximo gobierno</t>
+          <t>A tres días de la segunda vuelta, 21 municipios de Antioquia están en riesgo extraordinario electoral ¿Cuáles son?</t>
         </is>
       </c>
       <c r="E179" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/conflicto-armado-en-colombia/articulo/2026/6/eln-afirma-que-esta-listo-para-negociar-la-paz-o-continuar-la-guerra-con-el-proximo-gobierno</t>
+          <t>https://www.elcolombiano.com/antioquia/municipios-riesgo-electoral-2026-lista-completa-seguridad-votaciones-PL37879350</t>
         </is>
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="2" t="inlineStr">
-        <is>
-          <t>18/06/2026 01:00 p. m.</t>
-        </is>
-      </c>
+      <c r="A180" s="2" t="inlineStr"/>
       <c r="B180" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5343,26 +5291,22 @@
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D180" s="3" t="inlineStr">
         <is>
-          <t>Guillermo Reyes le responde a Gustavo Petro: niega campaña contra Verónica Alcocer y apunta a la primera dama</t>
+          <t>CNE ratifica candidatura de De la Espriella y cierra discusión sobre su nacionalidad</t>
         </is>
       </c>
       <c r="E180" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/poder/articulo/2026/6/guillermo-reyes-le-responde-a-gustavo-petro-niega-campana-contra-veronica-alcocer-y-apunta-a-la-primera-dama</t>
+          <t>https://www.elcolombiano.com/especiales/elecciones-2026/cne-ratifica-candidatura-abelardo-de-la-espriella-nacionalidad-EL37877434</t>
         </is>
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="5" t="inlineStr">
-        <is>
-          <t>18/06/2026 12:30 p. m.</t>
-        </is>
-      </c>
+      <c r="A181" s="5" t="inlineStr"/>
       <c r="B181" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5370,26 +5314,22 @@
       </c>
       <c r="C181" s="5" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D181" s="6" t="inlineStr">
         <is>
-          <t>Javier Pava regresa a la UNGRD tras la salida de Carlos Carrillo: asumirá la preparación del país para el Fenómeno de El Niño</t>
+          <t>MOE y 51 organizaciones exigen a Cepeda y Abelardo comprometerse a respetar los resultados</t>
         </is>
       </c>
       <c r="E181" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/pais/articulo/2026/6/javier-pava-regresa-a-la-ungrd-tras-la-salida-de-carlos-carrillo-asumira-la-preparacion-del-pais-para-el-fenomeno-de-el-nino</t>
+          <t>https://www.elcolombiano.com/colombia/moe-exige-candidatos-reconocer-resultados-elecciones-presidenciales-HK37868807</t>
         </is>
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="2" t="inlineStr">
-        <is>
-          <t>18/06/2026 11:30 a. m.</t>
-        </is>
-      </c>
+      <c r="A182" s="2" t="inlineStr"/>
       <c r="B182" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5397,26 +5337,22 @@
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D182" s="3" t="inlineStr">
         <is>
-          <t>¿Información imprecisa? Ministerio de Defensa rechazó el informe del Financial Times sobre narcotráfico y defendió resultados del gobierno</t>
+          <t>Así se mueven Cepeda y De la Espriella a cinco días del voto final</t>
         </is>
       </c>
       <c r="E182" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/conflicto-armado-en-colombia/articulo/2026/6/informacion-imprecisa-ministerio-de-defensa-rechazo-el-informe-del-financial-times-sobre-narcotrafico-y-defendio-resultados-del-gobierno</t>
+          <t>https://www.elcolombiano.com/especiales/elecciones-2026/ivan-cepeda-abelardo-de-la-espriella-apoyos-analisis-JL37787680</t>
         </is>
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="5" t="inlineStr">
-        <is>
-          <t>18/06/2026 09:05 a. m.</t>
-        </is>
-      </c>
+      <c r="A183" s="5" t="inlineStr"/>
       <c r="B183" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5424,26 +5360,22 @@
       </c>
       <c r="C183" s="5" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D183" s="6" t="inlineStr">
         <is>
-          <t>Bogotá se prepara para un mes de orgullo, memoria y reivindicación con cuatro marchas LGBTIQ+</t>
+          <t>Pilas con usar el celular en el puesto de votación: estas son las razones</t>
         </is>
       </c>
       <c r="E183" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/pais/articulo/2026/6/bogota-se-prepara-para-un-mes-de-orgullo-memoria-y-reivindicacion-con-cuatro-marchas-lgbtiq</t>
+          <t>https://www.elcolombiano.com/especiales/elecciones-2026/elecciones-segunda-vuelta-uso-celular-puesto-votacion-EB37501500</t>
         </is>
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="2" t="inlineStr">
-        <is>
-          <t>18/06/2026 08:30 a. m.</t>
-        </is>
-      </c>
+      <c r="A184" s="2" t="inlineStr"/>
       <c r="B184" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5451,26 +5383,22 @@
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D184" s="3" t="inlineStr">
         <is>
-          <t>¿Cuándo y dónde juega Colombia su próximo partido en el Mundial 2026?</t>
+          <t>Operativo destapa helicóptero con pasado oscuro y motor Rolls-Royce</t>
         </is>
       </c>
       <c r="E184" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/pais/articulo/2026/6/cuando-y-donde-juega-colombia-su-proximo-partido-en-el-mundial-2026</t>
+          <t>https://www.elcolombiano.com/colombia/ejercito-incauta-helicoptero-de-la-mafia-NG33717192</t>
         </is>
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="5" t="inlineStr">
-        <is>
-          <t>18/06/2026 07:15 a. m.</t>
-        </is>
-      </c>
+      <c r="A185" s="5" t="inlineStr"/>
       <c r="B185" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5478,26 +5406,22 @@
       </c>
       <c r="C185" s="5" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D185" s="6" t="inlineStr">
         <is>
-          <t>Trump intervino de nuevo en la contienda electoral colombiana pidiendo votar por Abelardo de la Espriella</t>
+          <t>Tres de los siete futbolistas que marcaron los primeros goles de Colombia en Mundiales nacieron en Antioquia, ¿quiénes son?</t>
         </is>
       </c>
       <c r="E185" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/trump-intervino-de-nuevo-en-la-contienda-electoral-colombiana-pidiendo-votar-por-abelardo-de-la-espriella</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/seleccion-colombia-futbolistas-que-han-marcado-primer-gol-en-mundiales-daniel-munoz-juanfer-quintero-pablo-armero-AF37897667</t>
         </is>
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="2" t="inlineStr">
-        <is>
-          <t>18/06/2026 02:00 a. m.</t>
-        </is>
-      </c>
+      <c r="A186" s="2" t="inlineStr"/>
       <c r="B186" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5505,26 +5429,22 @@
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D186" s="3" t="inlineStr">
         <is>
-          <t>Procuraduría abrió indagación sobre aeropuertos rurales del Gobierno Petro tras revelaciones sobre que ninguno supera el 20 por ciento de avance</t>
+          <t>Camarógrafo arrollado en partido Colombia vs. Uzbekistán recibió detallazo de Khusanov: “lo siento”</t>
         </is>
       </c>
       <c r="E186" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/pais/articulo/2026/6/procuraduria-abrio-indagacion-sobre-aeropuertos-rurales-del-gobierno-petro-tras-revelaciones-sobre-que-ninguno-supera-el-20-por-ciento-de-avance</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/khusanov-camiseta-camarografo-lesionado-colombia-uzbekistan-LF37897419</t>
         </is>
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="5" t="inlineStr">
-        <is>
-          <t>17/06/2026 05:30 p. m.</t>
-        </is>
-      </c>
+      <c r="A187" s="5" t="inlineStr"/>
       <c r="B187" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5532,26 +5452,22 @@
       </c>
       <c r="C187" s="5" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D187" s="6" t="inlineStr">
         <is>
-          <t>¿Qué pasa si queda en empate la segunda vuelta o si gana el voto en blanco?</t>
+          <t>Uribe denuncia que fiscal que lo llamó a indagatoria ejerce “clara presión política”; “no recibió una sola declaración mía”</t>
         </is>
       </c>
       <c r="E187" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/elecciones-colombia-2026/articulo/2026/6/que-pasa-si-queda-en-empate-la-segunda-vuelta-o-si-gana-el-voto-en-blanco</t>
+          <t>https://www.elcolombiano.com/colombia/alvaro-uribe-intereses-politicos-fiscalia-masacres-el-aro-las-granjas-GF37892985</t>
         </is>
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="2" t="inlineStr">
-        <is>
-          <t>17/06/2026 02:30 p. m.</t>
-        </is>
-      </c>
+      <c r="A188" s="2" t="inlineStr"/>
       <c r="B188" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5559,26 +5475,22 @@
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D188" s="3" t="inlineStr">
         <is>
-          <t>Ley Jineth Bedoya: ¿cómo funcionará la nueva ley para minimizar la revictimización desde el Estado para mujeres y niñas?</t>
+          <t>Gobierno Petro quiere que empresas postales manejen dinero como un banco, sin que nadie los vigile</t>
         </is>
       </c>
       <c r="E188" s="4" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/genero/articulo/2026/6/ley-jineth-bedoya-como-funcionara-la-nueva-ley-para-minimizar-la-revictimizacion-desde-el-estado-para-mujeres-y-ninas</t>
+          <t>https://www.elcolombiano.com/negocios/decreto-mintic-empresas-postales-colombia-riesgo-lavado-activos-CF37893274</t>
         </is>
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="5" t="inlineStr">
-        <is>
-          <t>17/06/2026 01:45 p. m.</t>
-        </is>
-      </c>
+      <c r="A189" s="5" t="inlineStr"/>
       <c r="B189" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -5586,17 +5498,17 @@
       </c>
       <c r="C189" s="5" t="inlineStr">
         <is>
-          <t>Cambio Colombia</t>
+          <t>El Colombiano</t>
         </is>
       </c>
       <c r="D189" s="6" t="inlineStr">
         <is>
-          <t>Los nuevos detalles que reveló la esteticista que estuvo en la cirugía que causó muerte de Yulixa Toloza</t>
+          <t>Consternación en Vancouver: Ismaël Koné, de Canadá, salió gravemente lesionado tras una falta de Catar; así quedó en video</t>
         </is>
       </c>
       <c r="E189" s="7" t="inlineStr">
         <is>
-          <t>https://cambiocolombia.com/los-nuevos-detalles-que-revelo-la-esteticista-que-estuvo-en-la-cirugia-que-causo-muerte-de-yulixa-toloza</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/lesion-ismael-kone-canada-falta-catar-video-vancouver-mundial-2026-LF37891956</t>
         </is>
       </c>
     </row>
@@ -5614,12 +5526,12 @@
       </c>
       <c r="D190" s="3" t="inlineStr">
         <is>
-          <t>Corte Suprema ordena captura de la senadora Martha Peralta en plena diligencia por caso de la UNGRD</t>
+          <t>Denuncian desplazamiento de 355 campesinos en Zaragoza por choque entre grupos ilegales</t>
         </is>
       </c>
       <c r="E190" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/corte-detuvo-a-la-senadora-martha-peralta-CF37895315</t>
+          <t>https://www.elcolombiano.com/antioquia/desplazamiento-campesinos-zaragoza-antioquia-choques-farc-y-clan-del-golfo-FF37891488</t>
         </is>
       </c>
     </row>
@@ -5637,12 +5549,12 @@
       </c>
       <c r="D191" s="6" t="inlineStr">
         <is>
-          <t>El país dice a candidatos: “Aceptar los resultados es un deber democrático”</t>
+          <t>¿Qué gana Atlético Nacional con el retorno de Víctor Marulanda como director deportivo?</t>
         </is>
       </c>
       <c r="E191" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/abelardo-de-la-espriella-e-ivan-cepeda-los-llaman-a-aceptar-resultados-electorales-AF37899180</t>
+          <t>https://www.elcolombiano.com/deportes/futbol/victor-marulanda-nuevo-director-deportivo-de-atletico-nacional-los-retos-que-le-esperan-HF37891314</t>
         </is>
       </c>
     </row>
@@ -5660,12 +5572,12 @@
       </c>
       <c r="D192" s="3" t="inlineStr">
         <is>
-          <t>La Selección de México encontró el gol, el alivio y la clasificación en Guadalajara</t>
+          <t>Video | Así fue la polémica expulsión de un jugador de Catar tras presunta falta vs. Canadá, ¿favorecieron al local?</t>
         </is>
       </c>
       <c r="E192" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/mundial-2026/en-vivo-seleccion-mexico-vs-corea-del-sur-mundial-2026-LF37895790</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/video-polemica-expulsion-jugador-catar-falta-vs-canada-mundial-2026-KE37889928</t>
         </is>
       </c>
     </row>
@@ -5683,12 +5595,12 @@
       </c>
       <c r="D193" s="6" t="inlineStr">
         <is>
-          <t>A tres días de elecciones, Fiscalía llama a indagatoria a Álvaro Uribe por masacres de El Aro y La Granja ocurridas hace 30 años</t>
+          <t>Video | ¡De aplaudir! Niño de Uzbekistán fue consolado por hinchas colombianos en el Azteca</t>
         </is>
       </c>
       <c r="E193" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/alvaro-uribe-velez-fiscalia-lo-cita-a-indagatoria-por-masacres-del-aro-y-la-granja-HF37891897</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/hinchas-colombianos-consuelan-nino-llorando-uzbekistan-estadio-azteca-EE37883135</t>
         </is>
       </c>
     </row>
@@ -5706,12 +5618,12 @@
       </c>
       <c r="D194" s="3" t="inlineStr">
         <is>
-          <t>La lección del texano</t>
+          <t>Al menos 500 voluntarios se sumarán a la “limpiatón” del río Medellín, ¿cómo sumarse?</t>
         </is>
       </c>
       <c r="E194" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/multimedia/videos/la-leccion-del-texano-IE37884491</t>
+          <t>https://www.elcolombiano.com/medellin/voluntarios-limpieza-rio-medellin-dia-del-rio-HE37886274</t>
         </is>
       </c>
     </row>
@@ -5729,12 +5641,12 @@
       </c>
       <c r="D195" s="6" t="inlineStr">
         <is>
-          <t>A sus 111 años murió don Luis, el nacido en Antioquia que era el hombre más viejo en Estados Unidos</t>
+          <t>Gobierno Petro creó un monopolio en la deuda colombiana: fondo de EE. UU. controla el 30%</t>
         </is>
       </c>
       <c r="E195" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/antioquia/hombre-nacido-en-andes-antioquia-murio-a-los-111-anos-en-estados-unidos-HF37897606</t>
+          <t>https://www.elcolombiano.com/negocios/pimco-mayor-tenedor-tes-deuda-colombiana-42-billones-GL37877122</t>
         </is>
       </c>
     </row>
@@ -5752,12 +5664,12 @@
       </c>
       <c r="D196" s="3" t="inlineStr">
         <is>
-          <t>¿Está Colombia clasificada a segunda ronda en el Mundial o qué le falta para asegurarse? Estas son las opciones</t>
+          <t>A prisión presunto integrante de disidencias señalado de planear el atentado contra el periodista Gustavo Chicangana</t>
         </is>
       </c>
       <c r="E196" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/mundial-2026/que-necesita-colombia-para-clasificar-a-la-siguiente-fase-del-mundial-de-norteamerica-IE37882138</t>
+          <t>https://www.elcolombiano.com/colombia/carcel-disidente-farc-atentado-periodista-gustavo-chicangana-guaviare-GL37877540</t>
         </is>
       </c>
     </row>
@@ -5775,12 +5687,12 @@
       </c>
       <c r="D197" s="6" t="inlineStr">
         <is>
-          <t>Otras tres derrotas en el Congreso: al Gobierno Petro le archivaron estas iniciativas</t>
+          <t>Efectos del alza de 23% del salario mínimo: menos desempleo, más concentración salarial y presión sobre la informalidad</t>
         </is>
       </c>
       <c r="E197" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/congreso-archivo-tres-iniciativas-del-gobierno-petro-KL37870497</t>
+          <t>https://www.elcolombiano.com/negocios/efectos-alza-salario-minimo-2026-mercado-laboral-colombia-anif-CE37883256</t>
         </is>
       </c>
     </row>
@@ -5798,12 +5710,12 @@
       </c>
       <c r="D198" s="3" t="inlineStr">
         <is>
-          <t>Más de 50 organizaciones piden compromiso público de Cepeda y Abelardo de reconocer resultados de segunda vuelta presidencial</t>
+          <t>Estos serán los partidos de este viernes en el Mundial 2026: Brasil y Paraguay necesitan la victoria</t>
         </is>
       </c>
       <c r="E198" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/elecciones-2026/mas-50-organizaciones-piden-reconocer-resultados-segunda-vuelta-presidencia-HF37897077</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/proximos-partidos-18-junio-mundial-2026-ee-uu-australia-brasil-haiti-escocia-marruecos-turquia-paraguay-ME37885595</t>
         </is>
       </c>
     </row>
@@ -5821,12 +5733,12 @@
       </c>
       <c r="D199" s="6" t="inlineStr">
         <is>
-          <t>A tres días de la segunda vuelta, 21 municipios de Antioquia están en riesgo extraordinario electoral ¿Cuáles son?</t>
+          <t>Bomberos voluntarios de Colombia quedarán exentos del impuesto vehicular tras iniciativa promovida desde Antioquia</t>
         </is>
       </c>
       <c r="E199" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/antioquia/municipios-riesgo-electoral-2026-lista-completa-seguridad-votaciones-PL37879350</t>
+          <t>https://www.elcolombiano.com/colombia/bomberos-voluntarios-colombia-exentos-impuesto-vehicular-IE37885418</t>
         </is>
       </c>
     </row>
@@ -5839,17 +5751,17 @@
       </c>
       <c r="C200" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D200" s="3" t="inlineStr">
         <is>
-          <t>CNE ratifica candidatura de De la Espriella y cierra discusión sobre su nacionalidad</t>
+          <t>¿Quién es Marcela Abadía, la fiscal que ordenó el llamado a indagatoria contra el expresidente Álvaro Uribe Vélez?</t>
         </is>
       </c>
       <c r="E200" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/elecciones-2026/cne-ratifica-candidatura-abelardo-de-la-espriella-nacionalidad-EL37877434</t>
+          <t>https://www.semana.com/nacion/articulo/quien-es-marcela-abadia-la-fiscal-que-ordeno-el-llamado-a-indagatoria-contra-el-expresidente-alvaro-uribe-velez/202612/</t>
         </is>
       </c>
     </row>
@@ -5862,17 +5774,17 @@
       </c>
       <c r="C201" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D201" s="6" t="inlineStr">
         <is>
-          <t>MOE y 51 organizaciones exigen a Cepeda y Abelardo comprometerse a respetar los resultados</t>
+          <t>El día definitivo: Abelardo de la Espriella conversará con Vicky Dávila, en vivo desde Barranquilla, este sábado a las 8:00 p. m.</t>
         </is>
       </c>
       <c r="E201" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/moe-exige-candidatos-reconocer-resultados-elecciones-presidenciales-HK37868807</t>
+          <t>https://www.semana.com/politica/articulo/el-dia-definitivo-abelardo-de-la-espriella-conversara-con-vicky-davila-en-vivo-desde-barranquilla-este-sabado-a-las-800-pm/202658/</t>
         </is>
       </c>
     </row>
@@ -5885,17 +5797,17 @@
       </c>
       <c r="C202" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D202" s="3" t="inlineStr">
         <is>
-          <t>Así se mueven Cepeda y De la Espriella a cinco días del voto final</t>
+          <t>Este es el juez que hostiga judicialmente y quiere silenciar a SEMANA por artículos sobre la JEP</t>
         </is>
       </c>
       <c r="E202" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/elecciones-2026/ivan-cepeda-abelardo-de-la-espriella-apoyos-analisis-JL37787680</t>
+          <t>https://www.semana.com/nacion/articulo/este-es-el-juez-que-hostiga-judicialmente-y-quiere-silenciar-a-semana-por-articulos-sobre-la-jep/202601/</t>
         </is>
       </c>
     </row>
@@ -5908,17 +5820,17 @@
       </c>
       <c r="C203" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D203" s="6" t="inlineStr">
         <is>
-          <t>Pilas con usar el celular en el puesto de votación: estas son las razones</t>
+          <t>Murió Dalita Navarro, la artista que convirtió la cerámica en un puente entre el arte y la historia política de Colombia</t>
         </is>
       </c>
       <c r="E203" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/elecciones-2026/elecciones-segunda-vuelta-uso-celular-puesto-votacion-EB37501500</t>
+          <t>https://www.semana.com/cultura/arte/articulo/murio-dalita-navarro-la-artista-que-convirtio-la-ceramica-en-un-puente-entre-el-arte-y-la-historia-politica-de-colombia/202601/</t>
         </is>
       </c>
     </row>
@@ -5931,17 +5843,17 @@
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D204" s="3" t="inlineStr">
         <is>
-          <t>Operativo destapa helicóptero con pasado oscuro y motor Rolls-Royce</t>
+          <t>“Es una trama electoral”: Álvaro Uribe Vélez estalla tras llamado a indagatoria y arremete contra Gustavo Petro</t>
         </is>
       </c>
       <c r="E204" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/ejercito-incauta-helicoptero-de-la-mafia-NG33717192</t>
+          <t>https://www.semana.com/politica/articulo/es-una-trama-electoral-alvaro-uribe-velez-estalla-tras-llamado-a-indagatoria-y-arremete-contra-gustavo-petro/202617/</t>
         </is>
       </c>
     </row>
@@ -5954,17 +5866,17 @@
       </c>
       <c r="C205" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D205" s="6" t="inlineStr">
         <is>
-          <t>Tres de los siete futbolistas que marcaron los primeros goles de Colombia en Mundiales nacieron en Antioquia, ¿quiénes son?</t>
+          <t>Corte Suprema capturó a la senadora Martha Peralta, del Pacto Histórico, en medio de la indagatoria por caso UNGRD</t>
         </is>
       </c>
       <c r="E205" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/mundial-2026/seleccion-colombia-futbolistas-que-han-marcado-primer-gol-en-mundiales-daniel-munoz-juanfer-quintero-pablo-armero-AF37897667</t>
+          <t>https://www.semana.com/nacion/articulo/primicia-corte-suprema-capturo-a-la-senadora-martha-peralta-del-pacto-historico-en-medio-de-la-indagatoria-por-caso-ungrd/202659/</t>
         </is>
       </c>
     </row>
@@ -5977,17 +5889,17 @@
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D206" s="3" t="inlineStr">
         <is>
-          <t>Camarógrafo arrollado en partido Colombia vs. Uzbekistán recibió detallazo de Khusanov: “lo siento”</t>
+          <t>Petro reacciona al llamado a indagatoria hecho a Álvaro Uribe: “Vayamos a la Justicia Especial para la Paz”</t>
         </is>
       </c>
       <c r="E206" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/mundial-2026/khusanov-camiseta-camarografo-lesionado-colombia-uzbekistan-LF37897419</t>
+          <t>https://www.semana.com/politica/articulo/petro-reacciona-al-llamado-a-indagatoria-hecho-a-alvaro-uribe-vayamos-a-la-justicia-especial-para-la-paz/202635/</t>
         </is>
       </c>
     </row>
@@ -6000,17 +5912,17 @@
       </c>
       <c r="C207" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D207" s="6" t="inlineStr">
         <is>
-          <t>Uribe denuncia que fiscal que lo llamó a indagatoria ejerce “clara presión política”; “no recibió una sola declaración mía”</t>
+          <t>Gobierno convocará a sesiones extraordinarias al Congreso; Jurisdicción Agraria y Ministerio de la Igualdad, sus intereses</t>
         </is>
       </c>
       <c r="E207" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/alvaro-uribe-intereses-politicos-fiscalia-masacres-el-aro-las-granjas-GF37892985</t>
+          <t>https://www.semana.com/politica/articulo/gobierno-convocara-a-sesiones-extraordinarias-al-congreso-jurisdiccion-agraria-y-ministerio-de-la-igualdad-sus-intereses/202608/</t>
         </is>
       </c>
     </row>
@@ -6023,17 +5935,17 @@
       </c>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D208" s="3" t="inlineStr">
         <is>
-          <t>Gobierno Petro quiere que empresas postales manejen dinero como un banco, sin que nadie los vigile</t>
+          <t>Tribunal rechazó la tutela que pedía suspender el uso de símbolos patrios en la campaña presidencial de Abelardo de la Espriella</t>
         </is>
       </c>
       <c r="E208" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/negocios/decreto-mintic-empresas-postales-colombia-riesgo-lavado-activos-CF37893274</t>
+          <t>https://www.semana.com/nacion/articulo/tribunal-rechazo-la-tutela-que-pedia-suspender-el-uso-de-simbolos-patrios-en-la-campana-presidencial-de-abelardo-de-la-espriella/202648/</t>
         </is>
       </c>
     </row>
@@ -6046,17 +5958,17 @@
       </c>
       <c r="C209" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D209" s="6" t="inlineStr">
         <is>
-          <t>Consternación en Vancouver: Ismaël Koné, de Canadá, salió gravemente lesionado tras una falta de Catar; así quedó en video</t>
+          <t>Caso Talio: Medicina Legal rompe el silencio sobre el locker de Zulma Guzmán y hace aclaración clave</t>
         </is>
       </c>
       <c r="E209" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/mundial-2026/lesion-ismael-kone-canada-falta-catar-video-vancouver-mundial-2026-LF37891956</t>
+          <t>https://www.semana.com/nacion/articulo/caso-talio-medicina-legal-rompe-el-silencio-sobre-el-locker-de-zulma-guzman-y-hace-aclaracion-clave/202650/</t>
         </is>
       </c>
     </row>
@@ -6069,17 +5981,17 @@
       </c>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D210" s="3" t="inlineStr">
         <is>
-          <t>Denuncian desplazamiento de 355 campesinos en Zaragoza por choque entre grupos ilegales</t>
+          <t>“Trampas de Petro, Cepeda y Farc”: opinión de Salud Hernández-Mora</t>
         </is>
       </c>
       <c r="E210" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/antioquia/desplazamiento-campesinos-zaragoza-antioquia-choques-farc-y-clan-del-golfo-FF37891488</t>
+          <t>https://www.semana.com/semana-tv/salud-hernandez/articulo/trampas-de-petro-cepeda-y-farc-opinion-de-salud-hernandez-mora/202631/</t>
         </is>
       </c>
     </row>
@@ -6092,17 +6004,17 @@
       </c>
       <c r="C211" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D211" s="6" t="inlineStr">
         <is>
-          <t>¿Qué gana Atlético Nacional con el retorno de Víctor Marulanda como director deportivo?</t>
+          <t>Primer gesto de Khusanov tras golpear al camarógrafo y caer ante Colombia en el Mundial: da ejemplo al mundo</t>
         </is>
       </c>
       <c r="E211" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/deportes/futbol/victor-marulanda-nuevo-director-deportivo-de-atletico-nacional-los-retos-que-le-esperan-HF37891314</t>
+          <t>https://www.semana.com/deportes/articulo/primer-gesto-de-khusanov-tras-golpear-al-camarografo-y-caer-ante-colombia-en-el-mundial-da-ejemplo-al-mundo/202619/</t>
         </is>
       </c>
     </row>
@@ -6115,17 +6027,17 @@
       </c>
       <c r="C212" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D212" s="3" t="inlineStr">
         <is>
-          <t>Video | Así fue la polémica expulsión de un jugador de Catar tras presunta falta vs. Canadá, ¿favorecieron al local?</t>
+          <t>Petro revive encuentro con Trump y lanza duro mensaje: “No me entendió”</t>
         </is>
       </c>
       <c r="E212" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/mundial-2026/video-polemica-expulsion-jugador-catar-falta-vs-canada-mundial-2026-KE37889928</t>
+          <t>https://www.semana.com/politica/articulo/petro-revive-encuentro-con-trump-y-lanza-duro-mensaje-no-me-entendio/202615/</t>
         </is>
       </c>
     </row>
@@ -6138,17 +6050,17 @@
       </c>
       <c r="C213" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D213" s="6" t="inlineStr">
         <is>
-          <t>Video | ¡De aplaudir! Niño de Uzbekistán fue consolado por hinchas colombianos en el Azteca</t>
+          <t>Impactante lesión en el Mundial 2026: jugador de Canadá sufre durísima fractura; imágenes sensibles</t>
         </is>
       </c>
       <c r="E213" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/mundial-2026/hinchas-colombianos-consuelan-nino-llorando-uzbekistan-estadio-azteca-EE37883135</t>
+          <t>https://www.semana.com/deportes/articulo/impactante-lesion-en-el-mundial-2026-jugador-de-canada-sufre-durisima-fractura-imagenes-sensibles/202616/</t>
         </is>
       </c>
     </row>
@@ -6161,17 +6073,17 @@
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D214" s="3" t="inlineStr">
         <is>
-          <t>Al menos 500 voluntarios se sumarán a la “limpiatón” del río Medellín, ¿cómo sumarse?</t>
+          <t>El Ejército de EE. UU. confirma el fin del bloqueo a los puertos iraníes en el estrecho de Ormuz</t>
         </is>
       </c>
       <c r="E214" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/medellin/voluntarios-limpieza-rio-medellin-dia-del-rio-HE37886274</t>
+          <t>https://www.semana.com/mundo/articulo/el-ejercito-de-ee-uu-confirma-el-fin-del-bloqueo-a-los-puertos-iranies-en-el-estrecho-de-ormuz/202658/</t>
         </is>
       </c>
     </row>
@@ -6184,17 +6096,17 @@
       </c>
       <c r="C215" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D215" s="6" t="inlineStr">
         <is>
-          <t>Gobierno Petro creó un monopolio en la deuda colombiana: fondo de EE. UU. controla el 30%</t>
+          <t>Gianni Infantino quedó atónito por lo que pasó en el Colombia vs. Uzbekistán: dejó contundente mensaje</t>
         </is>
       </c>
       <c r="E215" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/negocios/pimco-mayor-tenedor-tes-deuda-colombiana-42-billones-GL37877122</t>
+          <t>https://www.semana.com/deportes/articulo/gianni-infantino-quedo-atonito-por-lo-que-paso-en-el-colombia-vs-uzbekistan-dejo-contundente-mensaje/202603/</t>
         </is>
       </c>
     </row>
@@ -6207,17 +6119,17 @@
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D216" s="3" t="inlineStr">
         <is>
-          <t>A prisión presunto integrante de disidencias señalado de planear el atentado contra el periodista Gustavo Chicangana</t>
+          <t>La “última voluntad” de Yeison Jiménez: el sorpresivo respaldo de su esposa Sonia a la campaña de Abelardo de la Espriella</t>
         </is>
       </c>
       <c r="E216" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/carcel-disidente-farc-atentado-periodista-gustavo-chicangana-guaviare-GL37877540</t>
+          <t>https://www.semana.com/gente/articulo/la-ultima-voluntad-de-yeison-jimenez-el-sorpresivo-respaldo-de-su-esposa-sonia-a-la-campana-de-abelardo-de-la-espriella/202600/</t>
         </is>
       </c>
     </row>
@@ -6230,17 +6142,17 @@
       </c>
       <c r="C217" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D217" s="6" t="inlineStr">
         <is>
-          <t>Efectos del alza de 23% del salario mínimo: menos desempleo, más concentración salarial y presión sobre la informalidad</t>
+          <t>“Le presto mi canal”: Yeferson Cossio invitó a Iván Cepeda a transmitir su mensaje de campaña en la recta final electoral</t>
         </is>
       </c>
       <c r="E217" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/negocios/efectos-alza-salario-minimo-2026-mercado-laboral-colombia-anif-CE37883256</t>
+          <t>https://www.semana.com/politica/articulo/le-presto-mi-canal-yeferson-cossio-invito-a-ivan-cepeda-a-transmitir-su-mensaje-de-campana-en-la-recta-final-electoral/202601/</t>
         </is>
       </c>
     </row>
@@ -6253,17 +6165,17 @@
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D218" s="3" t="inlineStr">
         <is>
-          <t>Estos serán los partidos de este viernes en el Mundial 2026: Brasil y Paraguay necesitan la victoria</t>
+          <t>Partidos del Mundial 2026 que se juegan este 19 de junio: horarios y canal de TV</t>
         </is>
       </c>
       <c r="E218" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/mundial-2026/proximos-partidos-18-junio-mundial-2026-ee-uu-australia-brasil-haiti-escocia-marruecos-turquia-paraguay-ME37885595</t>
+          <t>https://www.semana.com/deportes/articulo/partidos-del-mundial-2026-que-se-juegan-este-19-de-junio-horarios-y-canal-de-tv/202639/</t>
         </is>
       </c>
     </row>
@@ -6276,17 +6188,17 @@
       </c>
       <c r="C219" s="5" t="inlineStr">
         <is>
-          <t>El Colombiano</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D219" s="6" t="inlineStr">
         <is>
-          <t>Bomberos voluntarios de Colombia quedarán exentos del impuesto vehicular tras iniciativa promovida desde Antioquia</t>
+          <t>Paulino Riascos alerta que su vida está en riesgo por no respaldar a Iván Cepeda: “Ya me tienen programado para matarme”</t>
         </is>
       </c>
       <c r="E219" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/bomberos-voluntarios-colombia-exentos-impuesto-vehicular-IE37885418</t>
+          <t>https://www.semana.com/politica/articulo/paulino-riascos-alerta-que-su-vida-esta-en-riesgo-por-no-respaldar-a-ivan-cepeda-ya-me-tienen-programado-para-matarme/202630/</t>
         </is>
       </c>
     </row>
@@ -6299,17 +6211,17 @@
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D220" s="3" t="inlineStr">
         <is>
-          <t>Prensa mundial Colombia: así reaccionó al triunfo en el Mundial 2026</t>
+          <t>Lidio García hace llamado a respetar los resultados electorales y rechaza supuestas protestas tras la segunda vuelta</t>
         </is>
       </c>
       <c r="E220" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/prensa-mundial-colombia-mundial-2026/</t>
+          <t>https://www.semana.com/politica/articulo/lidio-garcia-hace-llamado-a-respetar-los-resultados-electorales-y-rechaza-supuestas-protestas-tras-la-segunda-vuelta/202648/</t>
         </is>
       </c>
     </row>
@@ -6322,17 +6234,17 @@
       </c>
       <c r="C221" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D221" s="6" t="inlineStr">
         <is>
-          <t>Lineup EDC Colombia 2026: Alesso, Deadmau5, Armin y más de 80 artistas</t>
+          <t>Siguen las salidas en el Centro Democrático: Paola Holguín renunció al partido y a su curul en el Senado</t>
         </is>
       </c>
       <c r="E221" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/lineup-edc-colombia-2026/</t>
+          <t>https://www.semana.com/politica/articulo/siguen-las-salidas-en-el-centro-democratico-paola-holguin-renuncio-al-partido-y-a-su-curul-en-el-senado/202607/</t>
         </is>
       </c>
     </row>
@@ -6345,17 +6257,17 @@
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D222" s="3" t="inlineStr">
         <is>
-          <t>Yisell La Voz Rosa, la cantante vallenata que busca conquistar el 2026</t>
+          <t>El registrador Hernán Penagos reveló qué le preocupa de cara a las elecciones presidenciales del domingo 21 de junio: “Mentira pura y dura”</t>
         </is>
       </c>
       <c r="E222" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/yisell-la-voz-rosa/</t>
+          <t>https://www.semana.com/semana-tv/semana-el-debate/articulo/el-registrador-hernan-penagos-revelo-que-le-preocupa-de-cara-a-las-elecciones-presidenciales-del-domingo-21-de-junio-mentira-pura-y-dura/202649/</t>
         </is>
       </c>
     </row>
@@ -6368,17 +6280,17 @@
       </c>
       <c r="C223" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D223" s="6" t="inlineStr">
         <is>
-          <t>Catedral de Sal de Zipaquirá se une a una histórica mina de Polonia</t>
+          <t>Capturan en Medellín a dos mexicanos que serían enlace del Cartel de Sinaloa en Colombia</t>
         </is>
       </c>
       <c r="E223" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/catedral-de-sal-de-zipaquira-polonia/</t>
+          <t>https://www.semana.com/nacion/articulo/capturan-en-medellin-a-dos-mexicanos-que-serian-enlace-del-cartel-de-sinaloa-en-colombia/202627/</t>
         </is>
       </c>
     </row>
@@ -6391,17 +6303,17 @@
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D224" s="3" t="inlineStr">
         <is>
-          <t>El indie se toma Bogotá: El Festival Nuevas Voces 2026 enciende el circuito alternativo nacional</t>
+          <t>100 hombres de la Coordinadora Nacional Ejército Bolivariano entregaron sus armas en Putumayo</t>
         </is>
       </c>
       <c r="E224" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/el-indie-se-toma-bogota-el-festival-nuevas-voces-2026-enciende-el-circuito-alternativo-nacional/</t>
+          <t>https://www.semana.com/nacion/articulo/100-hombres-de-la-coordinadora-nacional-ejercito-bolivariano-entregaron-sus-armas-en-putumayo/202659/</t>
         </is>
       </c>
     </row>
@@ -6414,17 +6326,17 @@
       </c>
       <c r="C225" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D225" s="6" t="inlineStr">
         <is>
-          <t>Lujo con sello propio: Johnnie Walker Blue Label y Mario Hernández se unen para celebrar el estilo atemporal</t>
+          <t>“Trampas de Petro, Cepeda y las Farc”: Salud Hernández-Mora habla de presiones y amenazas</t>
         </is>
       </c>
       <c r="E225" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/lujo-con-sello-propio-johnnie-walker-blue-label-y-mario-hernandez-se-unen-para-celebrar-el-estilo-atemporal/</t>
+          <t>https://www.semana.com/nacion/articulo/trampas-de-petro-cepeda-y-las-farc-salud-hernandez-mora-habla-de-presiones-y-amenazas/202604/</t>
         </is>
       </c>
     </row>
@@ -6437,17 +6349,17 @@
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D226" s="3" t="inlineStr">
         <is>
-          <t>Vacaciones urbanas: Salitre Mágico se posiciona como el epicentro del entretenimiento familiar sin salir de Bogotá</t>
+          <t>Tribunal Superior rechazó la medida que buscaba suspender la candidatura de Abelardo de la Espriella para la segunda vuelta</t>
         </is>
       </c>
       <c r="E226" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/vacaciones-urbanas-salitre-magico-se-posiciona-como-el-epicentro-del-entretenimiento-familiar-sin-salir-de-bogota/</t>
+          <t>https://www.semana.com/nacion/articulo/tribunal-superior-rechazo-la-medida-que-buscaba-suspender-la-candidatura-de-abelardo-de-la-espriella-para-la-segunda-vuelta/202637/</t>
         </is>
       </c>
     </row>
@@ -6460,17 +6372,17 @@
       </c>
       <c r="C227" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D227" s="6" t="inlineStr">
         <is>
-          <t>Inteligencia artificial «invisible»: Samsung transforma la experiencia audiovisual desde las pantallas</t>
+          <t>Senadora Martha Peralta llegó a la indagatoria por caso UNGRD alegando que todo sería una “persecución política”</t>
         </is>
       </c>
       <c r="E227" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/inteligencia-artificial-invisible-samsung-transforma-la-experiencia-audiovisual-desde-las-pantallas/</t>
+          <t>https://www.semana.com/nacion/articulo/senadora-martha-peralta-llego-a-la-indagatoria-por-caso-ungrd-alegando-que-todo-seria-una-persecucion-politica/202646/</t>
         </is>
       </c>
     </row>
@@ -6483,17 +6395,17 @@
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D228" s="3" t="inlineStr">
         <is>
-          <t>Economía circular en la belleza: L’Oréal Groupe le apuesta a los formatos «refill» para reducir hasta un 77% de plástico</t>
+          <t>🔴 Calendario y fixture de la Copa Mundial de la FIFA 2026</t>
         </is>
       </c>
       <c r="E228" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/economia-circular-en-la-belleza-loreal-groupe-le-apuesta-a-los-formatos-refill-para-reducir-hasta-un-77-de-plastico/</t>
+          <t>https://www.semana.com/deportes/especiales-multimedia/articulo/mundial-2026-el-simulador-con-el-que-usted-puede-jugar-y-atinar-hasta-que-haya-campeon/202529/</t>
         </is>
       </c>
     </row>
@@ -6506,17 +6418,17 @@
       </c>
       <c r="C229" s="5" t="inlineStr">
         <is>
-          <t>Canal Trece</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D229" s="6" t="inlineStr">
         <is>
-          <t>La magia de Toy Story 5 llega a Cine Colombia con tiendas temáticas exclusivas y por tiempo limitado</t>
+          <t>Craso error de Corea del Sur acabó en la clasificación de México en el Mundial: el portero se equivocó</t>
         </is>
       </c>
       <c r="E229" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/la-magia-de-toy-story-5-llega-a-cine-colombia-con-tiendas-tematicas-exclusivas-y-por-tiempo-limitado/</t>
+          <t>https://www.semana.com/deportes/articulo/craso-error-de-corea-del-sur-acabo-en-la-clasificacion-de-mexico-en-el-mundial-el-portero-se-equivoco/202653/</t>
         </is>
       </c>
     </row>
@@ -6534,12 +6446,12 @@
       </c>
       <c r="D230" s="3" t="inlineStr">
         <is>
-          <t>Casos de éxito de la industria pet llegarán a Expopet 2026 como protagonistas de la muestra comercial</t>
+          <t>Prensa mundial Colombia: así reaccionó al triunfo en el Mundial 2026</t>
         </is>
       </c>
       <c r="E230" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/casos-de-exito-de-la-industria-pet-llegaran-a-expopet-2026-como-protagonistas-de-la-muestra-comercial/</t>
+          <t>https://canaltrece.com.co/noticias/prensa-mundial-colombia-mundial-2026/</t>
         </is>
       </c>
     </row>
@@ -6557,12 +6469,12 @@
       </c>
       <c r="D231" s="6" t="inlineStr">
         <is>
-          <t>«Magia»: El primer sencillo de Luisa Chimá inspirado en el poder de sanar</t>
+          <t>Lineup EDC Colombia 2026: Alesso, Deadmau5, Armin y más de 80 artistas</t>
         </is>
       </c>
       <c r="E231" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/magia-el-primer-sencillo-de-luisa-chima-inspirado-en-el-poder-de-sanar/</t>
+          <t>https://canaltrece.com.co/noticias/lineup-edc-colombia-2026/</t>
         </is>
       </c>
     </row>
@@ -6580,12 +6492,12 @@
       </c>
       <c r="D232" s="3" t="inlineStr">
         <is>
-          <t>«Así suena lo nuestro»: El Festival Francisco el Hombre 2026 celebra sus 18 años en Riohacha</t>
+          <t>Yisell La Voz Rosa, la cantante vallenata que busca conquistar el 2026</t>
         </is>
       </c>
       <c r="E232" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/asi-suena-lo-nuestro-el-festival-francisco-el-hombre-2026-celebra-sus-18-anos-en-riohacha/</t>
+          <t>https://canaltrece.com.co/noticias/yisell-la-voz-rosa/</t>
         </is>
       </c>
     </row>
@@ -6603,12 +6515,12 @@
       </c>
       <c r="D233" s="6" t="inlineStr">
         <is>
-          <t>Movilidad sostenible: BYD lanza camiones 100% eléctricos para transformar la logística de carga en Colombia</t>
+          <t>Catedral de Sal de Zipaquirá se une a una histórica mina de Polonia</t>
         </is>
       </c>
       <c r="E233" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/movilidad-sostenible-byd-lanza-camiones-100-electricos-para-transformar-la-logistica-de-carga-en-colombia/</t>
+          <t>https://canaltrece.com.co/noticias/catedral-de-sal-de-zipaquira-polonia/</t>
         </is>
       </c>
     </row>
@@ -6626,12 +6538,12 @@
       </c>
       <c r="D234" s="3" t="inlineStr">
         <is>
-          <t>Maná conmemora 40 años de trayectoria con su gira «Vivir Sin Aire Tour» y confirma concierto en BogotáManá conmemora 40 años de trayectoria con su gira «Vivir Sin Aire Tour» y confirma concierto en Bogotá</t>
+          <t>El indie se toma Bogotá: El Festival Nuevas Voces 2026 enciende el circuito alternativo nacional</t>
         </is>
       </c>
       <c r="E234" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/mana-conmemora-40-anos-de-trayectoria-con-su-gira-vivir-sin-aire-tour-y-confirma-concierto-en-bogotamana-conmemora-40-anos-de-trayectoria-con-su-gira-vivir-sin-aire-tour-y-confirma-concierto-e/</t>
+          <t>https://canaltrece.com.co/noticias/el-indie-se-toma-bogota-el-festival-nuevas-voces-2026-enciende-el-circuito-alternativo-nacional/</t>
         </is>
       </c>
     </row>
@@ -6649,12 +6561,12 @@
       </c>
       <c r="D235" s="6" t="inlineStr">
         <is>
-          <t>Colombia vs. RD del Congo: Horario, sede y canales de transmisión para el segundo examen de la Tricolor en la Copa del Mundo</t>
+          <t>Lujo con sello propio: Johnnie Walker Blue Label y Mario Hernández se unen para celebrar el estilo atemporal</t>
         </is>
       </c>
       <c r="E235" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/colombia-vs-rd-del-congo-horario-sede-y-canales-de-transmision-para-el-segundo-examen-de-la-tricolor-en-la-copa-del-mundo/</t>
+          <t>https://canaltrece.com.co/noticias/lujo-con-sello-propio-johnnie-walker-blue-label-y-mario-hernandez-se-unen-para-celebrar-el-estilo-atemporal/</t>
         </is>
       </c>
     </row>
@@ -6672,12 +6584,12 @@
       </c>
       <c r="D236" s="3" t="inlineStr">
         <is>
-          <t>Colombia vs Uzbekistán: la Tricolor debutó con victoria 3-1</t>
+          <t>Vacaciones urbanas: Salitre Mágico se posiciona como el epicentro del entretenimiento familiar sin salir de Bogotá</t>
         </is>
       </c>
       <c r="E236" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/colombia-vs-uzbekistan-mundial-2026/</t>
+          <t>https://canaltrece.com.co/noticias/vacaciones-urbanas-salitre-magico-se-posiciona-como-el-epicentro-del-entretenimiento-familiar-sin-salir-de-bogota/</t>
         </is>
       </c>
     </row>
@@ -6695,12 +6607,12 @@
       </c>
       <c r="D237" s="6" t="inlineStr">
         <is>
-          <t>Morat Tu Cárcel alcanza el No. 1 en Billboard Latin Airplay</t>
+          <t>Inteligencia artificial «invisible»: Samsung transforma la experiencia audiovisual desde las pantallas</t>
         </is>
       </c>
       <c r="E237" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/morat-tu-carcel-billboard/</t>
+          <t>https://canaltrece.com.co/noticias/inteligencia-artificial-invisible-samsung-transforma-la-experiencia-audiovisual-desde-las-pantallas/</t>
         </is>
       </c>
     </row>
@@ -6718,12 +6630,12 @@
       </c>
       <c r="D238" s="3" t="inlineStr">
         <is>
-          <t>Colombia vs Uzbekistán: así terminó el primer tiempo del debut</t>
+          <t>Economía circular en la belleza: L’Oréal Groupe le apuesta a los formatos «refill» para reducir hasta un 77% de plástico</t>
         </is>
       </c>
       <c r="E238" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/colombia-vs-uzbekistan/</t>
+          <t>https://canaltrece.com.co/noticias/economia-circular-en-la-belleza-loreal-groupe-le-apuesta-a-los-formatos-refill-para-reducir-hasta-un-77-de-plastico/</t>
         </is>
       </c>
     </row>
@@ -6741,12 +6653,12 @@
       </c>
       <c r="D239" s="6" t="inlineStr">
         <is>
-          <t>Penelope Robin inicia una nueva etapa con Diosa de Cien Colores</t>
+          <t>La magia de Toy Story 5 llega a Cine Colombia con tiendas temáticas exclusivas y por tiempo limitado</t>
         </is>
       </c>
       <c r="E239" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/penelope-robin-diosa-de-cien-colores/</t>
+          <t>https://canaltrece.com.co/noticias/la-magia-de-toy-story-5-llega-a-cine-colombia-con-tiendas-tematicas-exclusivas-y-por-tiempo-limitado/</t>
         </is>
       </c>
     </row>
@@ -6764,12 +6676,12 @@
       </c>
       <c r="D240" s="3" t="inlineStr">
         <is>
-          <t>Narra Tu Territorio abre segundo corte tras recibir 764 propuestas</t>
+          <t>Casos de éxito de la industria pet llegarán a Expopet 2026 como protagonistas de la muestra comercial</t>
         </is>
       </c>
       <c r="E240" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/narra-tu-territorio-segundo-corte/</t>
+          <t>https://canaltrece.com.co/noticias/casos-de-exito-de-la-industria-pet-llegaran-a-expopet-2026-como-protagonistas-de-la-muestra-comercial/</t>
         </is>
       </c>
     </row>
@@ -6787,12 +6699,12 @@
       </c>
       <c r="D241" s="6" t="inlineStr">
         <is>
-          <t>Colombia vs Uzbekistán: fecha, hora, estadio y dónde ver</t>
+          <t>«Magia»: El primer sencillo de Luisa Chimá inspirado en el poder de sanar</t>
         </is>
       </c>
       <c r="E241" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/colombia-vs-uzbekistan-fecha-hora-estadio-y-donde-ver/</t>
+          <t>https://canaltrece.com.co/noticias/magia-el-primer-sencillo-de-luisa-chima-inspirado-en-el-poder-de-sanar/</t>
         </is>
       </c>
     </row>
@@ -6810,12 +6722,12 @@
       </c>
       <c r="D242" s="3" t="inlineStr">
         <is>
-          <t>Fanzones en Bogotá para ver a Colombia: boletas y horarios</t>
+          <t>«Así suena lo nuestro»: El Festival Francisco el Hombre 2026 celebra sus 18 años en Riohacha</t>
         </is>
       </c>
       <c r="E242" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/fanzones-en-bogota-para-ver-a-colombia-boletas-y-horarios/</t>
+          <t>https://canaltrece.com.co/noticias/asi-suena-lo-nuestro-el-festival-francisco-el-hombre-2026-celebra-sus-18-anos-en-riohacha/</t>
         </is>
       </c>
     </row>
@@ -6833,12 +6745,12 @@
       </c>
       <c r="D243" s="6" t="inlineStr">
         <is>
-          <t>¿Estreno hoy? Todo sobre la llegada de Toy Story 5 a las salas de cine</t>
+          <t>Movilidad sostenible: BYD lanza camiones 100% eléctricos para transformar la logística de carga en Colombia</t>
         </is>
       </c>
       <c r="E243" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/estreno-hoy-todo-sobre-la-llegada-de-toy-story-5-a-las-salas-de-cine/</t>
+          <t>https://canaltrece.com.co/noticias/movilidad-sostenible-byd-lanza-camiones-100-electricos-para-transformar-la-logistica-de-carga-en-colombia/</t>
         </is>
       </c>
     </row>
@@ -6856,12 +6768,12 @@
       </c>
       <c r="D244" s="3" t="inlineStr">
         <is>
-          <t>Cierre de legislatura en el Congreso de la República: Proyectos clave que se juegan la vida en el remate del periodo legislativo</t>
+          <t>Maná conmemora 40 años de trayectoria con su gira «Vivir Sin Aire Tour» y confirma concierto en BogotáManá conmemora 40 años de trayectoria con su gira «Vivir Sin Aire Tour» y confirma concierto en Bogotá</t>
         </is>
       </c>
       <c r="E244" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/cierre-de-legislatura-en-el-congreso-de-la-republica-proyectos-clave-que-se-juegan-la-vida-en-el-remate-del-periodo-legislativo/</t>
+          <t>https://canaltrece.com.co/noticias/mana-conmemora-40-anos-de-trayectoria-con-su-gira-vivir-sin-aire-tour-y-confirma-concierto-en-bogotamana-conmemora-40-anos-de-trayectoria-con-su-gira-vivir-sin-aire-tour-y-confirma-concierto-e/</t>
         </is>
       </c>
     </row>
@@ -6879,12 +6791,12 @@
       </c>
       <c r="D245" s="6" t="inlineStr">
         <is>
-          <t>¿Qué pasará con Blessd? Claves para entender su situación jurídica tras el fallo sobre presunto secuestro</t>
+          <t>Colombia vs. RD del Congo: Horario, sede y canales de transmisión para el segundo examen de la Tricolor en la Copa del Mundo</t>
         </is>
       </c>
       <c r="E245" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/que-pasara-con-blessd-claves-para-entender-su-situacion-juridica-tras-el-fallo-sobre-presunto-secuestro/</t>
+          <t>https://canaltrece.com.co/noticias/colombia-vs-rd-del-congo-horario-sede-y-canales-de-transmision-para-el-segundo-examen-de-la-tricolor-en-la-copa-del-mundo/</t>
         </is>
       </c>
     </row>
@@ -6902,12 +6814,12 @@
       </c>
       <c r="D246" s="3" t="inlineStr">
         <is>
-          <t>Colombia define su futuro: Avance en vivo de la jornada de segunda vuelta presidencial de 2026</t>
+          <t>Colombia vs Uzbekistán: la Tricolor debutó con victoria 3-1</t>
         </is>
       </c>
       <c r="E246" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/colombia-define-su-futuro-avance-en-vivo-de-la-jornada-de-segunda-vuelta-presidencial-de-2026/</t>
+          <t>https://canaltrece.com.co/noticias/colombia-vs-uzbekistan-mundial-2026/</t>
         </is>
       </c>
     </row>
@@ -6925,12 +6837,12 @@
       </c>
       <c r="D247" s="6" t="inlineStr">
         <is>
-          <t>Falcao Mundial 2026: el Tigre cree que Colombia puede superar lo hecho en 2014</t>
+          <t>Morat Tu Cárcel alcanza el No. 1 en Billboard Latin Airplay</t>
         </is>
       </c>
       <c r="E247" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/falcao-mundial-2026-colombia/</t>
+          <t>https://canaltrece.com.co/noticias/morat-tu-carcel-billboard/</t>
         </is>
       </c>
     </row>
@@ -6948,12 +6860,12 @@
       </c>
       <c r="D248" s="3" t="inlineStr">
         <is>
-          <t>Colombia vs Uzbekistán: hora y dónde ver EN VIVO el debut de la Selección en el Mundial 2026</t>
+          <t>Colombia vs Uzbekistán: así terminó el primer tiempo del debut</t>
         </is>
       </c>
       <c r="E248" s="4" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/colombia-vs-uzbekistan-hora-colombia/</t>
+          <t>https://canaltrece.com.co/noticias/colombia-vs-uzbekistan/</t>
         </is>
       </c>
     </row>
@@ -6971,12 +6883,12 @@
       </c>
       <c r="D249" s="6" t="inlineStr">
         <is>
-          <t>Ley seca Bogotá: Galán cambia el horario para las elecciones 2026</t>
+          <t>Penelope Robin inicia una nueva etapa con Diosa de Cien Colores</t>
         </is>
       </c>
       <c r="E249" s="7" t="inlineStr">
         <is>
-          <t>https://canaltrece.com.co/noticias/ley-seca-bogota-elecciones-2026/</t>
+          <t>https://canaltrece.com.co/noticias/penelope-robin-diosa-de-cien-colores/</t>
         </is>
       </c>
     </row>
@@ -6989,17 +6901,17 @@
       </c>
       <c r="C250" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D250" s="3" t="inlineStr">
         <is>
-          <t>¿Quién es Marcela Abadía, la fiscal que ordenó el llamado a indagatoria contra el expresidente Álvaro Uribe Vélez?</t>
+          <t>Narra Tu Territorio abre segundo corte tras recibir 764 propuestas</t>
         </is>
       </c>
       <c r="E250" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/quien-es-marcela-abadia-la-fiscal-que-ordeno-el-llamado-a-indagatoria-contra-el-expresidente-alvaro-uribe-velez/202612/</t>
+          <t>https://canaltrece.com.co/noticias/narra-tu-territorio-segundo-corte/</t>
         </is>
       </c>
     </row>
@@ -7012,17 +6924,17 @@
       </c>
       <c r="C251" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D251" s="6" t="inlineStr">
         <is>
-          <t>El día definitivo: Abelardo de la Espriella conversará con Vicky Dávila, en vivo desde Barranquilla, este sábado a las 8:00 p. m.</t>
+          <t>Colombia vs Uzbekistán: fecha, hora, estadio y dónde ver</t>
         </is>
       </c>
       <c r="E251" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/el-dia-definitivo-abelardo-de-la-espriella-conversara-con-vicky-davila-en-vivo-desde-barranquilla-este-sabado-a-las-800-pm/202658/</t>
+          <t>https://canaltrece.com.co/noticias/colombia-vs-uzbekistan-fecha-hora-estadio-y-donde-ver/</t>
         </is>
       </c>
     </row>
@@ -7035,17 +6947,17 @@
       </c>
       <c r="C252" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D252" s="3" t="inlineStr">
         <is>
-          <t>Este es el juez que hostiga judicialmente y quiere silenciar a SEMANA por artículos sobre la JEP</t>
+          <t>Fanzones en Bogotá para ver a Colombia: boletas y horarios</t>
         </is>
       </c>
       <c r="E252" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/este-es-el-juez-que-hostiga-judicialmente-y-quiere-silenciar-a-semana-por-articulos-sobre-la-jep/202601/</t>
+          <t>https://canaltrece.com.co/noticias/fanzones-en-bogota-para-ver-a-colombia-boletas-y-horarios/</t>
         </is>
       </c>
     </row>
@@ -7058,17 +6970,17 @@
       </c>
       <c r="C253" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D253" s="6" t="inlineStr">
         <is>
-          <t>Murió Dalita Navarro, la artista que convirtió la cerámica en un puente entre el arte y la historia política de Colombia</t>
+          <t>¿Estreno hoy? Todo sobre la llegada de Toy Story 5 a las salas de cine</t>
         </is>
       </c>
       <c r="E253" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/cultura/arte/articulo/murio-dalita-navarro-la-artista-que-convirtio-la-ceramica-en-un-puente-entre-el-arte-y-la-historia-politica-de-colombia/202601/</t>
+          <t>https://canaltrece.com.co/noticias/estreno-hoy-todo-sobre-la-llegada-de-toy-story-5-a-las-salas-de-cine/</t>
         </is>
       </c>
     </row>
@@ -7081,17 +6993,17 @@
       </c>
       <c r="C254" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D254" s="3" t="inlineStr">
         <is>
-          <t>“Es una trama electoral”: Álvaro Uribe Vélez estalla tras llamado a indagatoria y arremete contra Gustavo Petro</t>
+          <t>Cierre de legislatura en el Congreso de la República: Proyectos clave que se juegan la vida en el remate del periodo legislativo</t>
         </is>
       </c>
       <c r="E254" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/es-una-trama-electoral-alvaro-uribe-velez-estalla-tras-llamado-a-indagatoria-y-arremete-contra-gustavo-petro/202617/</t>
+          <t>https://canaltrece.com.co/noticias/cierre-de-legislatura-en-el-congreso-de-la-republica-proyectos-clave-que-se-juegan-la-vida-en-el-remate-del-periodo-legislativo/</t>
         </is>
       </c>
     </row>
@@ -7104,17 +7016,17 @@
       </c>
       <c r="C255" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D255" s="6" t="inlineStr">
         <is>
-          <t>Corte Suprema capturó a la senadora Martha Peralta, del Pacto Histórico, en medio de la indagatoria por caso UNGRD</t>
+          <t>¿Qué pasará con Blessd? Claves para entender su situación jurídica tras el fallo sobre presunto secuestro</t>
         </is>
       </c>
       <c r="E255" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/primicia-corte-suprema-capturo-a-la-senadora-martha-peralta-del-pacto-historico-en-medio-de-la-indagatoria-por-caso-ungrd/202659/</t>
+          <t>https://canaltrece.com.co/noticias/que-pasara-con-blessd-claves-para-entender-su-situacion-juridica-tras-el-fallo-sobre-presunto-secuestro/</t>
         </is>
       </c>
     </row>
@@ -7127,17 +7039,17 @@
       </c>
       <c r="C256" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D256" s="3" t="inlineStr">
         <is>
-          <t>Petro reacciona al llamado a indagatoria hecho a Álvaro Uribe: “Vayamos a la Justicia Especial para la Paz”</t>
+          <t>Colombia define su futuro: Avance en vivo de la jornada de segunda vuelta presidencial de 2026</t>
         </is>
       </c>
       <c r="E256" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/petro-reacciona-al-llamado-a-indagatoria-hecho-a-alvaro-uribe-vayamos-a-la-justicia-especial-para-la-paz/202635/</t>
+          <t>https://canaltrece.com.co/noticias/colombia-define-su-futuro-avance-en-vivo-de-la-jornada-de-segunda-vuelta-presidencial-de-2026/</t>
         </is>
       </c>
     </row>
@@ -7150,17 +7062,17 @@
       </c>
       <c r="C257" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D257" s="6" t="inlineStr">
         <is>
-          <t>Gobierno convocará a sesiones extraordinarias al Congreso; Jurisdicción Agraria y Ministerio de la Igualdad, sus intereses</t>
+          <t>Falcao Mundial 2026: el Tigre cree que Colombia puede superar lo hecho en 2014</t>
         </is>
       </c>
       <c r="E257" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/gobierno-convocara-a-sesiones-extraordinarias-al-congreso-jurisdiccion-agraria-y-ministerio-de-la-igualdad-sus-intereses/202608/</t>
+          <t>https://canaltrece.com.co/noticias/falcao-mundial-2026-colombia/</t>
         </is>
       </c>
     </row>
@@ -7173,17 +7085,17 @@
       </c>
       <c r="C258" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D258" s="3" t="inlineStr">
         <is>
-          <t>Tribunal rechazó la tutela que pedía suspender el uso de símbolos patrios en la campaña presidencial de Abelardo de la Espriella</t>
+          <t>Colombia vs Uzbekistán: hora y dónde ver EN VIVO el debut de la Selección en el Mundial 2026</t>
         </is>
       </c>
       <c r="E258" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/tribunal-rechazo-la-tutela-que-pedia-suspender-el-uso-de-simbolos-patrios-en-la-campana-presidencial-de-abelardo-de-la-espriella/202648/</t>
+          <t>https://canaltrece.com.co/noticias/colombia-vs-uzbekistan-hora-colombia/</t>
         </is>
       </c>
     </row>
@@ -7196,482 +7108,22 @@
       </c>
       <c r="C259" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Canal Trece</t>
         </is>
       </c>
       <c r="D259" s="6" t="inlineStr">
         <is>
-          <t>Caso Talio: Medicina Legal rompe el silencio sobre el locker de Zulma Guzmán y hace aclaración clave</t>
+          <t>Ley seca Bogotá: Galán cambia el horario para las elecciones 2026</t>
         </is>
       </c>
       <c r="E259" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/caso-talio-medicina-legal-rompe-el-silencio-sobre-el-locker-de-zulma-guzman-y-hace-aclaracion-clave/202650/</t>
-        </is>
-      </c>
-    </row>
-    <row r="260">
-      <c r="A260" s="2" t="inlineStr"/>
-      <c r="B260" s="2" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C260" s="2" t="inlineStr">
-        <is>
-          <t>Semana</t>
-        </is>
-      </c>
-      <c r="D260" s="3" t="inlineStr">
-        <is>
-          <t>“Trampas de Petro, Cepeda y Farc”: opinión de Salud Hernández-Mora</t>
-        </is>
-      </c>
-      <c r="E260" s="4" t="inlineStr">
-        <is>
-          <t>https://www.semana.com/semana-tv/salud-hernandez/articulo/trampas-de-petro-cepeda-y-farc-opinion-de-salud-hernandez-mora/202631/</t>
-        </is>
-      </c>
-    </row>
-    <row r="261">
-      <c r="A261" s="5" t="inlineStr"/>
-      <c r="B261" s="5" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C261" s="5" t="inlineStr">
-        <is>
-          <t>Semana</t>
-        </is>
-      </c>
-      <c r="D261" s="6" t="inlineStr">
-        <is>
-          <t>Primer gesto de Khusanov tras golpear al camarógrafo y caer ante Colombia en el Mundial: da ejemplo al mundo</t>
-        </is>
-      </c>
-      <c r="E261" s="7" t="inlineStr">
-        <is>
-          <t>https://www.semana.com/deportes/articulo/primer-gesto-de-khusanov-tras-golpear-al-camarografo-y-caer-ante-colombia-en-el-mundial-da-ejemplo-al-mundo/202619/</t>
-        </is>
-      </c>
-    </row>
-    <row r="262">
-      <c r="A262" s="2" t="inlineStr"/>
-      <c r="B262" s="2" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C262" s="2" t="inlineStr">
-        <is>
-          <t>Semana</t>
-        </is>
-      </c>
-      <c r="D262" s="3" t="inlineStr">
-        <is>
-          <t>Petro revive encuentro con Trump y lanza duro mensaje: “No me entendió”</t>
-        </is>
-      </c>
-      <c r="E262" s="4" t="inlineStr">
-        <is>
-          <t>https://www.semana.com/politica/articulo/petro-revive-encuentro-con-trump-y-lanza-duro-mensaje-no-me-entendio/202615/</t>
-        </is>
-      </c>
-    </row>
-    <row r="263">
-      <c r="A263" s="5" t="inlineStr"/>
-      <c r="B263" s="5" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C263" s="5" t="inlineStr">
-        <is>
-          <t>Semana</t>
-        </is>
-      </c>
-      <c r="D263" s="6" t="inlineStr">
-        <is>
-          <t>Impactante lesión en el Mundial 2026: jugador de Canadá sufre durísima fractura; imágenes sensibles</t>
-        </is>
-      </c>
-      <c r="E263" s="7" t="inlineStr">
-        <is>
-          <t>https://www.semana.com/deportes/articulo/impactante-lesion-en-el-mundial-2026-jugador-de-canada-sufre-durisima-fractura-imagenes-sensibles/202616/</t>
-        </is>
-      </c>
-    </row>
-    <row r="264">
-      <c r="A264" s="2" t="inlineStr"/>
-      <c r="B264" s="2" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C264" s="2" t="inlineStr">
-        <is>
-          <t>Semana</t>
-        </is>
-      </c>
-      <c r="D264" s="3" t="inlineStr">
-        <is>
-          <t>El Ejército de EE. UU. confirma el fin del bloqueo a los puertos iraníes en el estrecho de Ormuz</t>
-        </is>
-      </c>
-      <c r="E264" s="4" t="inlineStr">
-        <is>
-          <t>https://www.semana.com/mundo/articulo/el-ejercito-de-ee-uu-confirma-el-fin-del-bloqueo-a-los-puertos-iranies-en-el-estrecho-de-ormuz/202658/</t>
-        </is>
-      </c>
-    </row>
-    <row r="265">
-      <c r="A265" s="5" t="inlineStr"/>
-      <c r="B265" s="5" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C265" s="5" t="inlineStr">
-        <is>
-          <t>Semana</t>
-        </is>
-      </c>
-      <c r="D265" s="6" t="inlineStr">
-        <is>
-          <t>Gianni Infantino quedó atónito por lo que pasó en el Colombia vs. Uzbekistán: dejó contundente mensaje</t>
-        </is>
-      </c>
-      <c r="E265" s="7" t="inlineStr">
-        <is>
-          <t>https://www.semana.com/deportes/articulo/gianni-infantino-quedo-atonito-por-lo-que-paso-en-el-colombia-vs-uzbekistan-dejo-contundente-mensaje/202603/</t>
-        </is>
-      </c>
-    </row>
-    <row r="266">
-      <c r="A266" s="2" t="inlineStr"/>
-      <c r="B266" s="2" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C266" s="2" t="inlineStr">
-        <is>
-          <t>Semana</t>
-        </is>
-      </c>
-      <c r="D266" s="3" t="inlineStr">
-        <is>
-          <t>La “última voluntad” de Yeison Jiménez: el sorpresivo respaldo de su esposa Sonia a la campaña de Abelardo de la Espriella</t>
-        </is>
-      </c>
-      <c r="E266" s="4" t="inlineStr">
-        <is>
-          <t>https://www.semana.com/gente/articulo/la-ultima-voluntad-de-yeison-jimenez-el-sorpresivo-respaldo-de-su-esposa-sonia-a-la-campana-de-abelardo-de-la-espriella/202600/</t>
-        </is>
-      </c>
-    </row>
-    <row r="267">
-      <c r="A267" s="5" t="inlineStr"/>
-      <c r="B267" s="5" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C267" s="5" t="inlineStr">
-        <is>
-          <t>Semana</t>
-        </is>
-      </c>
-      <c r="D267" s="6" t="inlineStr">
-        <is>
-          <t>“Le presto mi canal”: Yeferson Cossio invitó a Iván Cepeda a transmitir su mensaje de campaña en la recta final electoral</t>
-        </is>
-      </c>
-      <c r="E267" s="7" t="inlineStr">
-        <is>
-          <t>https://www.semana.com/politica/articulo/le-presto-mi-canal-yeferson-cossio-invito-a-ivan-cepeda-a-transmitir-su-mensaje-de-campana-en-la-recta-final-electoral/202601/</t>
-        </is>
-      </c>
-    </row>
-    <row r="268">
-      <c r="A268" s="2" t="inlineStr"/>
-      <c r="B268" s="2" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C268" s="2" t="inlineStr">
-        <is>
-          <t>Semana</t>
-        </is>
-      </c>
-      <c r="D268" s="3" t="inlineStr">
-        <is>
-          <t>Partidos del Mundial 2026 que se juegan este 19 de junio: horarios y canal de TV</t>
-        </is>
-      </c>
-      <c r="E268" s="4" t="inlineStr">
-        <is>
-          <t>https://www.semana.com/deportes/articulo/partidos-del-mundial-2026-que-se-juegan-este-19-de-junio-horarios-y-canal-de-tv/202639/</t>
-        </is>
-      </c>
-    </row>
-    <row r="269">
-      <c r="A269" s="5" t="inlineStr"/>
-      <c r="B269" s="5" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C269" s="5" t="inlineStr">
-        <is>
-          <t>Semana</t>
-        </is>
-      </c>
-      <c r="D269" s="6" t="inlineStr">
-        <is>
-          <t>Paulino Riascos alerta que su vida está en riesgo por no respaldar a Iván Cepeda: “Ya me tienen programado para matarme”</t>
-        </is>
-      </c>
-      <c r="E269" s="7" t="inlineStr">
-        <is>
-          <t>https://www.semana.com/politica/articulo/paulino-riascos-alerta-que-su-vida-esta-en-riesgo-por-no-respaldar-a-ivan-cepeda-ya-me-tienen-programado-para-matarme/202630/</t>
-        </is>
-      </c>
-    </row>
-    <row r="270">
-      <c r="A270" s="2" t="inlineStr"/>
-      <c r="B270" s="2" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C270" s="2" t="inlineStr">
-        <is>
-          <t>Semana</t>
-        </is>
-      </c>
-      <c r="D270" s="3" t="inlineStr">
-        <is>
-          <t>Lidio García hace llamado a respetar los resultados electorales y rechaza supuestas protestas tras la segunda vuelta</t>
-        </is>
-      </c>
-      <c r="E270" s="4" t="inlineStr">
-        <is>
-          <t>https://www.semana.com/politica/articulo/lidio-garcia-hace-llamado-a-respetar-los-resultados-electorales-y-rechaza-supuestas-protestas-tras-la-segunda-vuelta/202648/</t>
-        </is>
-      </c>
-    </row>
-    <row r="271">
-      <c r="A271" s="5" t="inlineStr"/>
-      <c r="B271" s="5" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C271" s="5" t="inlineStr">
-        <is>
-          <t>Semana</t>
-        </is>
-      </c>
-      <c r="D271" s="6" t="inlineStr">
-        <is>
-          <t>Siguen las salidas en el Centro Democrático: Paola Holguín renunció al partido y a su curul en el Senado</t>
-        </is>
-      </c>
-      <c r="E271" s="7" t="inlineStr">
-        <is>
-          <t>https://www.semana.com/politica/articulo/siguen-las-salidas-en-el-centro-democratico-paola-holguin-renuncio-al-partido-y-a-su-curul-en-el-senado/202607/</t>
-        </is>
-      </c>
-    </row>
-    <row r="272">
-      <c r="A272" s="2" t="inlineStr"/>
-      <c r="B272" s="2" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C272" s="2" t="inlineStr">
-        <is>
-          <t>Semana</t>
-        </is>
-      </c>
-      <c r="D272" s="3" t="inlineStr">
-        <is>
-          <t>El registrador Hernán Penagos reveló qué le preocupa de cara a las elecciones presidenciales del domingo 21 de junio: “Mentira pura y dura”</t>
-        </is>
-      </c>
-      <c r="E272" s="4" t="inlineStr">
-        <is>
-          <t>https://www.semana.com/semana-tv/semana-el-debate/articulo/el-registrador-hernan-penagos-revelo-que-le-preocupa-de-cara-a-las-elecciones-presidenciales-del-domingo-21-de-junio-mentira-pura-y-dura/202649/</t>
-        </is>
-      </c>
-    </row>
-    <row r="273">
-      <c r="A273" s="5" t="inlineStr"/>
-      <c r="B273" s="5" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C273" s="5" t="inlineStr">
-        <is>
-          <t>Semana</t>
-        </is>
-      </c>
-      <c r="D273" s="6" t="inlineStr">
-        <is>
-          <t>Capturan en Medellín a dos mexicanos que serían enlace del Cartel de Sinaloa en Colombia</t>
-        </is>
-      </c>
-      <c r="E273" s="7" t="inlineStr">
-        <is>
-          <t>https://www.semana.com/nacion/articulo/capturan-en-medellin-a-dos-mexicanos-que-serian-enlace-del-cartel-de-sinaloa-en-colombia/202627/</t>
-        </is>
-      </c>
-    </row>
-    <row r="274">
-      <c r="A274" s="2" t="inlineStr"/>
-      <c r="B274" s="2" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C274" s="2" t="inlineStr">
-        <is>
-          <t>Semana</t>
-        </is>
-      </c>
-      <c r="D274" s="3" t="inlineStr">
-        <is>
-          <t>100 hombres de la Coordinadora Nacional Ejército Bolivariano entregaron sus armas en Putumayo</t>
-        </is>
-      </c>
-      <c r="E274" s="4" t="inlineStr">
-        <is>
-          <t>https://www.semana.com/nacion/articulo/100-hombres-de-la-coordinadora-nacional-ejercito-bolivariano-entregaron-sus-armas-en-putumayo/202659/</t>
-        </is>
-      </c>
-    </row>
-    <row r="275">
-      <c r="A275" s="5" t="inlineStr"/>
-      <c r="B275" s="5" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C275" s="5" t="inlineStr">
-        <is>
-          <t>Semana</t>
-        </is>
-      </c>
-      <c r="D275" s="6" t="inlineStr">
-        <is>
-          <t>“Trampas de Petro, Cepeda y las Farc”: Salud Hernández-Mora habla de presiones y amenazas</t>
-        </is>
-      </c>
-      <c r="E275" s="7" t="inlineStr">
-        <is>
-          <t>https://www.semana.com/nacion/articulo/trampas-de-petro-cepeda-y-las-farc-salud-hernandez-mora-habla-de-presiones-y-amenazas/202604/</t>
-        </is>
-      </c>
-    </row>
-    <row r="276">
-      <c r="A276" s="2" t="inlineStr"/>
-      <c r="B276" s="2" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C276" s="2" t="inlineStr">
-        <is>
-          <t>Semana</t>
-        </is>
-      </c>
-      <c r="D276" s="3" t="inlineStr">
-        <is>
-          <t>Tribunal Superior rechazó la medida que buscaba suspender la candidatura de Abelardo de la Espriella para la segunda vuelta</t>
-        </is>
-      </c>
-      <c r="E276" s="4" t="inlineStr">
-        <is>
-          <t>https://www.semana.com/nacion/articulo/tribunal-superior-rechazo-la-medida-que-buscaba-suspender-la-candidatura-de-abelardo-de-la-espriella-para-la-segunda-vuelta/202637/</t>
-        </is>
-      </c>
-    </row>
-    <row r="277">
-      <c r="A277" s="5" t="inlineStr"/>
-      <c r="B277" s="5" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C277" s="5" t="inlineStr">
-        <is>
-          <t>Semana</t>
-        </is>
-      </c>
-      <c r="D277" s="6" t="inlineStr">
-        <is>
-          <t>Senadora Martha Peralta llegó a la indagatoria por caso UNGRD alegando que todo sería una “persecución política”</t>
-        </is>
-      </c>
-      <c r="E277" s="7" t="inlineStr">
-        <is>
-          <t>https://www.semana.com/nacion/articulo/senadora-martha-peralta-llego-a-la-indagatoria-por-caso-ungrd-alegando-que-todo-seria-una-persecucion-politica/202646/</t>
-        </is>
-      </c>
-    </row>
-    <row r="278">
-      <c r="A278" s="2" t="inlineStr"/>
-      <c r="B278" s="2" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C278" s="2" t="inlineStr">
-        <is>
-          <t>Semana</t>
-        </is>
-      </c>
-      <c r="D278" s="3" t="inlineStr">
-        <is>
-          <t>🔴 Calendario y fixture de la Copa Mundial de la FIFA 2026</t>
-        </is>
-      </c>
-      <c r="E278" s="4" t="inlineStr">
-        <is>
-          <t>https://www.semana.com/deportes/especiales-multimedia/articulo/mundial-2026-el-simulador-con-el-que-usted-puede-jugar-y-atinar-hasta-que-haya-campeon/202529/</t>
-        </is>
-      </c>
-    </row>
-    <row r="279">
-      <c r="A279" s="5" t="inlineStr"/>
-      <c r="B279" s="5" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C279" s="5" t="inlineStr">
-        <is>
-          <t>Semana</t>
-        </is>
-      </c>
-      <c r="D279" s="6" t="inlineStr">
-        <is>
-          <t>Craso error de Corea del Sur acabó en la clasificación de México en el Mundial: el portero se equivocó</t>
-        </is>
-      </c>
-      <c r="E279" s="7" t="inlineStr">
-        <is>
-          <t>https://www.semana.com/deportes/articulo/craso-error-de-corea-del-sur-acabo-en-la-clasificacion-de-mexico-en-el-mundial-el-portero-se-equivoco/202653/</t>
+          <t>https://canaltrece.com.co/noticias/ley-seca-bogota-elecciones-2026/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E279"/>
+  <autoFilter ref="A1:E259"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
@@ -7931,26 +7383,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E257" r:id="rId256"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E258" r:id="rId257"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E259" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E260" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E261" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E262" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E263" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E264" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E265" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E266" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E267" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E268" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E269" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E270" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E271" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E272" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E273" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E274" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E275" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E276" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E277" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E278" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E279" r:id="rId278"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Noticias actualizadas 21/06/2026 09:22
</commit_message>
<xml_diff>
--- a/docs/ultimahora.xlsx
+++ b/docs/ultimahora.xlsx
@@ -515,7 +515,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>21/06/2026 02:32 a. m.</t>
+          <t>21/06/2026 03:55 a. m.</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -530,19 +530,19 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Japón no tuvo piedad de Túnez y lo goleó con cuatro tantos para subir al segundo lugar del grupo F en el Mundial 2026</t>
+          <t>Resultado elecciones presidenciales en segunda vuelta Colombia 2026: desde las 8 de la mañana se abren urnas, siga la jornada de votación</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/japon-no-tuvo-piedad-de-tunez-y-lo-goleo-con-cuatro-tantos-para-subir-al-segundo-lugar-del-grupo-f-en-el-mundial-3565830</t>
+          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/resultado-elecciones-presidenciales-en-segunda-vuelta-colombia-2026-desde-las-8-de-la-manana-se-abren-urnas-siga-la-jornada-de-votacion-3565831</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>21/06/2026 01:27 a. m.</t>
+          <t>21/06/2026 03:01 a. m.</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -557,19 +557,19 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>'La ficción está demasiado invadida por la realidad': Rosa Montero, escritora española</t>
+          <t>Uruguay busca su primera victoria en el Mundial, pero al frente tiene a Cabo Verde y a su arquerazo, Vozinha: día, hora y dónde ver el juego</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/cultura/musica-y-libros/la-ficcion-esta-demasiado-invadida-por-la-realidad-rosa-montero-escritora-espanola-3565743</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/uruguay-busca-su-primera-victoria-en-el-mundial-pero-al-frente-tiene-a-cabo-verde-y-a-su-arquerazo-vozinha-dia-hora-y-donde-ver-el-juego-3565780</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>21/06/2026 12:11 a. m.</t>
+          <t>21/06/2026 02:32 a. m.</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -584,19 +584,19 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>El dilema de Brasil: buenos indicadores económicos, percepción social pesimista</t>
+          <t>Japón no tuvo piedad de Túnez y lo goleó con cuatro tantos para subir al segundo lugar del grupo F en el Mundial 2026</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/latinoamerica/el-dilema-de-brasil-buenos-indicadores-economicos-percepcion-social-pesimista-3565668</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/japon-no-tuvo-piedad-de-tunez-y-lo-goleo-con-cuatro-tantos-para-subir-al-segundo-lugar-del-grupo-f-en-el-mundial-3565830</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>21/06/2026 12:01 a. m.</t>
+          <t>21/06/2026 01:27 a. m.</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -611,19 +611,19 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Un deber ciudadano</t>
+          <t>'La ficción está demasiado invadida por la realidad': Rosa Montero, escritora española</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/cartas/un-deber-ciudadano-3565827</t>
+          <t>https://www.eltiempo.com/cultura/musica-y-libros/la-ficcion-esta-demasiado-invadida-por-la-realidad-rosa-montero-escritora-espanola-3565743</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>21/06/2026 12:01 a. m.</t>
+          <t>21/06/2026 12:11 a. m.</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -638,19 +638,19 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>El avance imparable de la Avenida Cañasgordas: la obra que transformará a Cali y a Jamundí</t>
+          <t>El dilema de Brasil: buenos indicadores económicos, percepción social pesimista</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mas-contenido/el-avance-imparable-de-la-avenida-canasgordas-la-obra-que-transformara-a-cali-y-a-jamundi-3565283</t>
+          <t>https://www.eltiempo.com/mundo/latinoamerica/el-dilema-de-brasil-buenos-indicadores-economicos-percepcion-social-pesimista-3565668</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 11:30 p. m.</t>
+          <t>21/06/2026 12:01 a. m.</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -665,19 +665,19 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>¿Cómo ha cambiado la manera de estudiar de las generaciones hiperconectadas?</t>
+          <t>Un deber ciudadano</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/vida/educacion/como-ha-cambiado-la-manera-de-estudiar-de-las-generaciones-hiperconectadas-3565799</t>
+          <t>https://www.eltiempo.com/opinion/cartas/un-deber-ciudadano-3565827</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 11:25 p. m.</t>
+          <t>21/06/2026 12:01 a. m.</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -692,19 +692,19 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Cómo cumplir sin plata / Análisis de Ricardo Ávila</t>
+          <t>El avance imparable de la Avenida Cañasgordas: la obra que transformará a Cali y a Jamundí</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/economia/sectores/como-cumplir-sin-plata-analisis-de-ricardo-avila-3565808</t>
+          <t>https://www.eltiempo.com/mas-contenido/el-avance-imparable-de-la-avenida-canasgordas-la-obra-que-transformara-a-cali-y-a-jamundi-3565283</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 11:20 p. m.</t>
+          <t>20/06/2026 11:30 p. m.</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -719,19 +719,19 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Cuentas Claras / Subsidios, tajadas y zarpazos</t>
+          <t>¿Cómo ha cambiado la manera de estudiar de las generaciones hiperconectadas?</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/economia/sectores/cuentas-claras-subsidios-tajadas-y-zarpazos-3565809</t>
+          <t>https://www.eltiempo.com/vida/educacion/como-ha-cambiado-la-manera-de-estudiar-de-las-generaciones-hiperconectadas-3565799</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 11:15 p. m.</t>
+          <t>20/06/2026 11:25 p. m.</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -746,19 +746,19 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>El contrabando mundialista se dispara en Bogotá: estas son las rutas, movimientos y millonarios negocios detrás de la fiebre del fútbol</t>
+          <t>Cómo cumplir sin plata / Análisis de Ricardo Ávila</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/bogota/el-contrabando-mundialista-se-dispara-en-bogota-estas-son-las-rutas-movimientos-y-millonarios-negocios-detras-de-la-fiebre-del-futbol-3565758</t>
+          <t>https://www.eltiempo.com/economia/sectores/como-cumplir-sin-plata-analisis-de-ricardo-avila-3565808</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 11:14 p. m.</t>
+          <t>20/06/2026 11:20 p. m.</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -773,19 +773,19 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>‘Nuestra casa influye en quiénes somos y quiénes podemos llegar a ser’: la arquitecta y neuropsicóloga Ana Mombiedro</t>
+          <t>Cuentas Claras / Subsidios, tajadas y zarpazos</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/vida/tendencias/nuestra-casa-influye-en-quienes-somos-y-quienes-podemos-llegar-a-ser-3565746</t>
+          <t>https://www.eltiempo.com/economia/sectores/cuentas-claras-subsidios-tajadas-y-zarpazos-3565809</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 11:01 p. m.</t>
+          <t>20/06/2026 11:15 p. m.</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -800,19 +800,19 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Goles de ternura</t>
+          <t>El contrabando mundialista se dispara en Bogotá: estas son las rutas, movimientos y millonarios negocios detrás de la fiebre del fútbol</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/columnistas/goles-de-ternura-3565826</t>
+          <t>https://www.eltiempo.com/bogota/el-contrabando-mundialista-se-dispara-en-bogota-estas-son-las-rutas-movimientos-y-millonarios-negocios-detras-de-la-fiebre-del-futbol-3565758</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 11:01 p. m.</t>
+          <t>20/06/2026 11:14 p. m.</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -827,12 +827,12 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>¿Estallido social 2.0?</t>
+          <t>‘Nuestra casa influye en quiénes somos y quiénes podemos llegar a ser’: la arquitecta y neuropsicóloga Ana Mombiedro</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/columnistas/estallido-social-2-3565825</t>
+          <t>https://www.eltiempo.com/vida/tendencias/nuestra-casa-influye-en-quienes-somos-y-quienes-podemos-llegar-a-ser-3565746</t>
         </is>
       </c>
     </row>
@@ -854,12 +854,12 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>100 primeros días</t>
+          <t>Goles de ternura</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/columnistas/100-primeros-dias-3565824</t>
+          <t>https://www.eltiempo.com/opinion/columnistas/goles-de-ternura-3565826</t>
         </is>
       </c>
     </row>
@@ -881,12 +881,12 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Incendiar al país</t>
+          <t>¿Estallido social 2.0?</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/columnistas/incendiar-al-pais-3565823</t>
+          <t>https://www.eltiempo.com/opinion/columnistas/estallido-social-2-3565825</t>
         </is>
       </c>
     </row>
@@ -908,12 +908,12 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Cómo decidir el voto</t>
+          <t>100 primeros días</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/columnistas/como-decidir-el-voto-3565821</t>
+          <t>https://www.eltiempo.com/opinion/columnistas/100-primeros-dias-3565824</t>
         </is>
       </c>
     </row>
@@ -935,12 +935,12 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>El día después</t>
+          <t>Incendiar al país</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/columnistas/el-dia-despues-3565820</t>
+          <t>https://www.eltiempo.com/opinion/columnistas/incendiar-al-pais-3565823</t>
         </is>
       </c>
     </row>
@@ -962,12 +962,12 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Megatsunami de votos</t>
+          <t>Cómo decidir el voto</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/columnistas/megatsunami-de-votos-3565819</t>
+          <t>https://www.eltiempo.com/opinion/columnistas/como-decidir-el-voto-3565821</t>
         </is>
       </c>
     </row>
@@ -989,12 +989,12 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>El llamado es a votar y acatar</t>
+          <t>El día después</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/editorial/el-llamado-es-a-votar-y-acatar-3565818</t>
+          <t>https://www.eltiempo.com/opinion/columnistas/el-dia-despues-3565820</t>
         </is>
       </c>
     </row>
@@ -1016,12 +1016,12 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Puerta al cielo: la historia de la revelación de la Selección Colombia en el Mundial</t>
+          <t>Megatsunami de votos</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/puerta-al-cielo-la-historia-de-la-revelacion-de-la-seleccion-colombia-en-el-mundial-3565802</t>
+          <t>https://www.eltiempo.com/opinion/columnistas/megatsunami-de-votos-3565819</t>
         </is>
       </c>
     </row>
@@ -1043,12 +1043,12 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Voy y vuelvo| ¿Queremos repetir la historia? ¡A votar!</t>
+          <t>El llamado es a votar y acatar</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/bogota/voy-y-vuelvo-queremos-repetir-la-historia-a-votar-3565793</t>
+          <t>https://www.eltiempo.com/opinion/editorial/el-llamado-es-a-votar-y-acatar-3565818</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 11:29 p. m.</t>
+          <t>21/06/2026 03:19 a. m.</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -1097,19 +1097,19 @@
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>“Neutralización de alias Marlon es un golpe estratégico al terrorismo”: Mindefensa</t>
+          <t>El vicepresidente de EE.UU. llega a Suiza para iniciar las negociaciones de paz con Irán</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/21/neutralizacion-de-alias-marlon-es-un-golpe-estrategico-al-terrorismo-mindefensa/</t>
+          <t>https://caracol.com.co/2026/06/21/el-vicepresidente-de-eeuu-llega-a-suiza-para-iniciar-las-negociaciones-de-paz-con-iran/</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 09:04 p. m.</t>
+          <t>20/06/2026 11:29 p. m.</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1124,19 +1124,19 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Ecuador se estrelló ante un gigante Eloy Room y empató con Curazao en el Grupo E</t>
+          <t>“Neutralización de alias Marlon es un golpe estratégico al terrorismo”: Mindefensa</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/20/en-vivo-ecuador-vs-curazao-minuto-a-minuto-y-la-transmision-del-partido-hoy/</t>
+          <t>https://caracol.com.co/2026/06/21/neutralizacion-de-alias-marlon-es-un-golpe-estrategico-al-terrorismo-mindefensa/</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 08:40 p. m.</t>
+          <t>20/06/2026 09:04 p. m.</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
@@ -1151,19 +1151,19 @@
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Transportadores alertan riesgos por plan para flexibilizar viajes de taxis entre municipios</t>
+          <t>Ecuador se estrelló ante un gigante Eloy Room y empató con Curazao en el Grupo E</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/21/transportadores-alertan-riesgos-por-plan-para-flexibilizar-viajes-de-taxis-entre-municipios/</t>
+          <t>https://caracol.com.co/2026/06/20/en-vivo-ecuador-vs-curazao-minuto-a-minuto-y-la-transmision-del-partido-hoy/</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 08:37 p. m.</t>
+          <t>20/06/2026 08:40 p. m.</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1178,19 +1178,19 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>COPPPAL inicia observación electoral en Colombia y acompaña segunda vuelta presidencial</t>
+          <t>Transportadores alertan riesgos por plan para flexibilizar viajes de taxis entre municipios</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/21/copppal-inicia-observacion-electoral-en-colombia-y-acompana-segunda-vuelta-presidencial/</t>
+          <t>https://caracol.com.co/2026/06/21/transportadores-alertan-riesgos-por-plan-para-flexibilizar-viajes-de-taxis-entre-municipios/</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 08:36 p. m.</t>
+          <t>20/06/2026 08:37 p. m.</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -1205,19 +1205,19 @@
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>¿Habrá restricción de parrillero en moto en la segunda vuelta 2026? Esto dice nuevo decreto 0612</t>
+          <t>COPPPAL inicia observación electoral en Colombia y acompaña segunda vuelta presidencial</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/21/habra-restriccion-de-parrillero-en-moto-en-la-segunda-vuelta-2026-esto-dice-nuevo-decreto-0612/</t>
+          <t>https://caracol.com.co/2026/06/21/copppal-inicia-observacion-electoral-en-colombia-y-acompana-segunda-vuelta-presidencial/</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 08:30 p. m.</t>
+          <t>20/06/2026 08:36 p. m.</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1232,19 +1232,19 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Supersalud reporta caída del 22 % en quejas por entrega de medicamentos</t>
+          <t>¿Habrá restricción de parrillero en moto en la segunda vuelta 2026? Esto dice nuevo decreto 0612</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/21/supersalud-reporta-caida-del-22-en-quejas-por-entrega-de-medicamentos/</t>
+          <t>https://caracol.com.co/2026/06/21/habra-restriccion-de-parrillero-en-moto-en-la-segunda-vuelta-2026-esto-dice-nuevo-decreto-0612/</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 08:09 p. m.</t>
+          <t>20/06/2026 08:30 p. m.</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -1259,19 +1259,19 @@
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>“Se requieren acciones urgentes en el Meta”: Gobernadora alerta por seguridad electoral</t>
+          <t>Supersalud reporta caída del 22 % en quejas por entrega de medicamentos</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/21/se-requieren-acciones-urgentes-en-el-meta-gobernadora-alerta-por-seguridad-electoral/</t>
+          <t>https://caracol.com.co/2026/06/21/supersalud-reporta-caida-del-22-en-quejas-por-entrega-de-medicamentos/</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 07:54 p. m.</t>
+          <t>20/06/2026 08:09 p. m.</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1286,19 +1286,19 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Murió alias ‘Marlon’, cabecilla de las disidencias en operación militar en el suroccidente del país</t>
+          <t>“Se requieren acciones urgentes en el Meta”: Gobernadora alerta por seguridad electoral</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/21/habrian-abatido-a-alias-marlon-cabecilla-de-las-disidencias-de-mordisco-en-operacion-en-cauca/</t>
+          <t>https://caracol.com.co/2026/06/21/se-requieren-acciones-urgentes-en-el-meta-gobernadora-alerta-por-seguridad-electoral/</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 06:57 p. m.</t>
+          <t>20/06/2026 07:54 p. m.</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -1313,19 +1313,19 @@
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Fue capturado en Cali alias ‘El Sueco’, uno de los narcotraficantes más buscados por Suecia</t>
+          <t>Murió alias ‘Marlon’, cabecilla de las disidencias en operación militar en el suroccidente del país</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/20/fue-capturado-en-cali-alias-el-sueco-uno-de-los-narcotraficantes-mas-buscados-por-suecia/</t>
+          <t>https://caracol.com.co/2026/06/21/habrian-abatido-a-alias-marlon-cabecilla-de-las-disidencias-de-mordisco-en-operacion-en-cauca/</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 06:21 p. m.</t>
+          <t>20/06/2026 06:57 p. m.</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1340,19 +1340,19 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Funcionario del Congreso alerta inconvenientes en aeropuertos internacionales por nuevo pasaporte</t>
+          <t>Fue capturado en Cali alias ‘El Sueco’, uno de los narcotraficantes más buscados por Suecia</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/20/funcionario-del-congreso-alerta-inconvenientes-en-aeropuertos-internacionales-por-nuevo-pasaporte/</t>
+          <t>https://caracol.com.co/2026/06/20/fue-capturado-en-cali-alias-el-sueco-uno-de-los-narcotraficantes-mas-buscados-por-suecia/</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 05:21 p. m.</t>
+          <t>20/06/2026 06:21 p. m.</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
@@ -1367,19 +1367,19 @@
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>Bernie Moreno llega a Bogotá para elecciones: “El futuro de Colombia reside en sus propias manos”</t>
+          <t>Funcionario del Congreso alerta inconvenientes en aeropuertos internacionales por nuevo pasaporte</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/20/bernie-moreno-llega-a-bogota-para-elecciones-el-futuro-de-colombia-reside-en-sus-propias-manos/</t>
+          <t>https://caracol.com.co/2026/06/20/funcionario-del-congreso-alerta-inconvenientes-en-aeropuertos-internacionales-por-nuevo-pasaporte/</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 05:19 p. m.</t>
+          <t>20/06/2026 05:21 p. m.</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1394,19 +1394,19 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>¿Desde qué hora se puede votar este domingo, 21 de junio? Detalles de la segunda vuelta presidencial</t>
+          <t>Bernie Moreno llega a Bogotá para elecciones: “El futuro de Colombia reside en sus propias manos”</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/20/desde-que-hora-se-puede-votar-este-domingo-21-de-junio-detalles-de-la-segunda-vuelta-presidencial/</t>
+          <t>https://caracol.com.co/2026/06/20/bernie-moreno-llega-a-bogota-para-elecciones-el-futuro-de-colombia-reside-en-sus-propias-manos/</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 04:57 p. m.</t>
+          <t>20/06/2026 05:19 p. m.</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
@@ -1421,19 +1421,19 @@
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>“No hubo manipulaciones de resultados electorales en primera vuelta”: auditoría internacional</t>
+          <t>¿Desde qué hora se puede votar este domingo, 21 de junio? Detalles de la segunda vuelta presidencial</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/20/no-hubo-manipulaciones-en-resultados-electorales-de-primera-vuelta-auditoria-internacional/</t>
+          <t>https://caracol.com.co/2026/06/20/desde-que-hora-se-puede-votar-este-domingo-21-de-junio-detalles-de-la-segunda-vuelta-presidencial/</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 04:50 p. m.</t>
+          <t>20/06/2026 04:57 p. m.</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1448,19 +1448,19 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Elecciones Presidenciales en Bolívar: más de 1.600 policías garantizarán la seguridad</t>
+          <t>“No hubo manipulaciones de resultados electorales en primera vuelta”: auditoría internacional</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/20/elecciones-presidenciales-en-bolivar-mas-de-1600-policias-garantizaran-la-seguridad/</t>
+          <t>https://caracol.com.co/2026/06/20/no-hubo-manipulaciones-en-resultados-electorales-de-primera-vuelta-auditoria-internacional/</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 04:40 p. m.</t>
+          <t>20/06/2026 04:50 p. m.</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
@@ -1475,19 +1475,19 @@
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>Segunda vuelta presidencial: estos son los consulados de Colombia en Venezuela donde podrá votar</t>
+          <t>Elecciones Presidenciales en Bolívar: más de 1.600 policías garantizarán la seguridad</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/20/segunda-vuelta-presidencial-estos-son-los-consulados-de-colombia-en-venezuela-donde-podra-votar/</t>
+          <t>https://caracol.com.co/2026/06/20/elecciones-presidenciales-en-bolivar-mas-de-1600-policias-garantizaran-la-seguridad/</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 04:37 p. m.</t>
+          <t>20/06/2026 04:40 p. m.</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -1502,19 +1502,19 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>¿Qué es el código hash utilizado en el escrutinio para garantizar la transparencia electoral?</t>
+          <t>Segunda vuelta presidencial: estos son los consulados de Colombia en Venezuela donde podrá votar</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/20/que-es-el-codigo-hash-utilizado-en-el-escrutinio-para-garantizar-la-transparencia-electoral/</t>
+          <t>https://caracol.com.co/2026/06/20/segunda-vuelta-presidencial-estos-son-los-consulados-de-colombia-en-venezuela-donde-podra-votar/</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 03:53 p. m.</t>
+          <t>20/06/2026 04:37 p. m.</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
@@ -1529,19 +1529,19 @@
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>Segunda vuelta 2026: cierre de fronteras, ley seca y prohibiciones; consulte aquí el ABC electoral</t>
+          <t>¿Qué es el código hash utilizado en el escrutinio para garantizar la transparencia electoral?</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/20/segunda-vuelta-2026-cierre-de-fronteras-ley-seca-y-prohibiciones-consulte-aqui-el-abc-electoral/</t>
+          <t>https://caracol.com.co/2026/06/20/que-es-el-codigo-hash-utilizado-en-el-escrutinio-para-garantizar-la-transparencia-electoral/</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 03:47 p. m.</t>
+          <t>20/06/2026 03:53 p. m.</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -1556,19 +1556,19 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Registrador Penagos se reunió con Misión de la Unión Europea para la segunda vuelta presidencial</t>
+          <t>Segunda vuelta 2026: cierre de fronteras, ley seca y prohibiciones; consulte aquí el ABC electoral</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/20/registrador-penagos-se-reunio-con-mision-de-la-union-europea-para-la-segunda-vuelta-presidencial/</t>
+          <t>https://caracol.com.co/2026/06/20/segunda-vuelta-2026-cierre-de-fronteras-ley-seca-y-prohibiciones-consulte-aqui-el-abc-electoral/</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 03:40 p. m.</t>
+          <t>20/06/2026 03:47 p. m.</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
@@ -1583,12 +1583,12 @@
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>El puerto de Tumaco recibió 100 mil barriles de combustible enviados desde Cartagena</t>
+          <t>Registrador Penagos se reunió con Misión de la Unión Europea para la segunda vuelta presidencial</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>https://caracol.com.co/2026/06/20/el-puerto-de-tumaco-recibio-100-mil-barriles-de-combustible-enviados-desde-cartagena/</t>
+          <t>https://caracol.com.co/2026/06/20/registrador-penagos-se-reunio-con-mision-de-la-union-europea-para-la-segunda-vuelta-presidencial/</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2027,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>21/06/2026 03:21 a. m.</t>
+          <t>21/06/2026 09:13 a. m.</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -2037,24 +2037,24 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Mindefensa: muerte de alias ‘Marlon’ es un duro golpe contra las disidencias de ‘Mordisco’</t>
+          <t>Petro exige a Trump que se revele la ubicación del influencer Beto Coral</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/orden-publico/mindefensa-muerte-de-alias-marlon-es-un-duro-golpe-contra-las-disidencias-de-mordisco-402844</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/20/petro-exige-a-trump-que-se-revele-la-ubicacion-del-influencer-beto-coral/</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>21/06/2026 02:43 a. m.</t>
+          <t>21/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
@@ -2064,24 +2064,24 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>Ecuador no pudo con Curazao y quedó contra las cuerdas en el Mundial 2026</t>
+          <t>Análisis de las elecciones presidenciales (III): Los errores de la campaña de Cepeda</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/deportes/mundial-2026-ecuador-empato-con-curazo-402843</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/21/analisis-de-las-elecciones-presidenciales-iii-los-errores-de-la-campana-de-cepeda/</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>21/06/2026 01:55 a. m.</t>
+          <t>21/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -2091,24 +2091,24 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Gobernador del Cauca tras muerte de alias 'Marlon': "No daremos tregua a las estructuras criminales"</t>
+          <t>Columnistas</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/orden-publico/gobernador-del-cauca-octavio-guzman-habla-tras-muerte-de-alias-marlon-402839</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>21/06/2026 01:06 a. m.</t>
+          <t>21/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
@@ -2118,24 +2118,24 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>Fue abatido alias 'Marlon', máximo cabecilla de las disidencias en Cauca y quien sería el futuro sucesor de 'Mordisco'</t>
+          <t>Participación, serenidad y unión</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/orden-publico/abatido-alias-marlon-cabecilla-disidencias-mordisco-cauca-402838</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/21/participacion-serenidad-y-union/</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>21/06/2026 12:19 a. m.</t>
+          <t>21/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -2145,24 +2145,24 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Así quedan las rutas de TransMilenio con la nueva estación Calle 26 - Atrio</t>
+          <t>Píldoras para la memoria: lo que Colombia no debe olvidar antes de elegir</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/actualidad/estacion-calle-26-atrio-transmilenio-como-seran-las-rutas-402836</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/maria-juliana-acebedo/2026/06/21/pildoras-para-la-memoria-lo-que-colombia-no-debe-olvidar-antes-de-elegir/</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 11:38 p. m.</t>
+          <t>21/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
@@ -2172,24 +2172,24 @@
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
-          <t>Gobernadora del Meta denuncia presunto intento de secuestro del alcalde de Mesetas</t>
+          <t>Maria Juliana Acebedo</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/orden-publico/meta-gobernadora-denuncia-aparente-intento-secuestro-alcalde-mesetas-402833</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/maria-juliana-acebedo/</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 11:33 p. m.</t>
+          <t>21/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -2199,24 +2199,24 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>¿Marco Rubio autorizó el documento para detener al activista Beto Coral en EE.UU.? Esto revela The New York Times</t>
+          <t>¡Salvemos a Colombia!</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/internacional/marco-rubio-autorizo-el-documento-para-detener-al-activista-beto-coral-en-eeuu-esto-revela-el-new-york-times-402835</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/alberto-montoya/2026/06/21/salvemos-a-colombia/</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 11:26 p. m.</t>
+          <t>21/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
@@ -2226,24 +2226,24 @@
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>Se conoce la razón por la que Georgina Rodríguez no acompañó a Cristinao Ronaldo al Mundial 2026</t>
+          <t>Alberto Montoya</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/entretenimiento/mundial-2026-cristiano-ronaldo-por-que-georgina-rodriguez-no-fue-a-verlo-402834</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/alberto-montoya/</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 10:49 p. m.</t>
+          <t>20/06/2026 11:11 p. m.</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -2253,24 +2253,24 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Estos son los ocho municipios colombianos que buscan llegar a la vitrina turística de ONU Turismo</t>
+          <t>Ejército abatió a alias ‘Marlon’, jefe clave de disidencias de ‘Iván Mordisco’ en Cauca</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/sociedad/onu-turismo-ocho-municipios-colombianos-buscan-reconocimiento-mundial-turismo-rural-402832</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/20/ejercito-abatio-a-alias-marlon-jefe-clave-de-disidencias-de-ivan-mordisco-en-cauca/</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 10:34 p. m.</t>
+          <t>20/06/2026 11:11 p. m.</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr">
@@ -2280,24 +2280,24 @@
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>Bernie Moreno llegó a Bogotá para ser observador internacional en la segunda vuelta de las presidenciales</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/bernie-moreno-llega-a-bogota-como-observador-internacional-para-la-segunda-vuelta-presidencial-402831</t>
+          <t>https://www.vanguardia.com/colombia/</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 10:18 p. m.</t>
+          <t>20/06/2026 10:53 p. m.</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -2307,24 +2307,24 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>¿Se podrá operar drones durante las elecciones en segunda vuelta presidencial? Aerocivil hace dura advertencia</t>
+          <t>Pensionado fue víctima de estafa dirigida desde Sudáfrica: así perdió $93 millones</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/sociedad/aerocivil-restringe-operaciones-drones-segunda-vuelta-presidencial-402829</t>
+          <t>https://www.vanguardia.com/contenido-registrados/2026/06/20/pensionado-fue-victima-de-estafa-dirigida-desde-sudafrica-asi-perdio-93-millones/</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 10:09 p. m.</t>
+          <t>20/06/2026 10:53 p. m.</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
@@ -2334,24 +2334,24 @@
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>Alemania remonta ante Costa de Marfil y clasifica a dieciseisavos del Mundial 2026</t>
+          <t>Contenido registrados</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/deportes/mundial-2026-alemania-remonta-costa-de-marfil-clasifica-dieciseisavos-402830</t>
+          <t>https://www.vanguardia.com/contenido-registrados/</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 09:43 p. m.</t>
+          <t>20/06/2026 07:29 p. m.</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -2361,24 +2361,24 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>Colombianos en Venezuela se quedaron sin votar en Cúcuta por cierre fronterizo</t>
+          <t>Capturan en Cali a ‘El Sueco’, clave en el envío de cocaína hacia Europa y Medio Oriente</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/actualidad/colombianos-en-venezuela-sin-votar-por-cierre-imprevisto-de-frontera-402827</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/20/capturan-en-cali-a-el-sueco-clave-en-el-envio-de-cocaina-hacia-europa-y-medio-oriente/</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 09:33 p. m.</t>
+          <t>20/06/2026 04:04 p. m.</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr">
@@ -2388,24 +2388,24 @@
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D71" s="6" t="inlineStr">
         <is>
-          <t>Último sorteo de la Lotería de Boyacá: resultado premio mayor hoy 20 de junio</t>
+          <t>El drama de una familia atrapada en la guerra del Catatumbo: niño murió y una bebé lucha por su vida</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/sociedad/ultimo-sorteo-de-la-loteria-de-boyaca-resultado-premio-mayor-hoy-20-de-junio-402828</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/20/el-drama-de-una-familia-atrapada-en-la-guerra-del-catatumbo-nino-murio-y-una-bebe-lucha-por-su-vida/</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 08:40 p. m.</t>
+          <t>20/06/2026 03:29 p. m.</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -2415,24 +2415,24 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>Tragedia en hotel de República Dominicana: un muerto y múltiples heridos tras incendio de gran magnitud</t>
+          <t>Asesinan a Mónica Eugenia Sánchez, reconocida lideresa social de Santa Bárbara, Antioquia</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/internacional/republica-dominicana-incendio-tragedia-muerte-turista-italiana-402825</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/20/asesinan-a-monica-eugenia-sanchez-reconocida-lideresa-social-de-santa-barbara-antioquia/</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 08:37 p. m.</t>
+          <t>20/06/2026 03:15 p. m.</t>
         </is>
       </c>
       <c r="B73" s="5" t="inlineStr">
@@ -2442,24 +2442,24 @@
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D73" s="6" t="inlineStr">
         <is>
-          <t>¿Qué pasa con la Transversal del Sisga? Reabre, pero con restricciones: solo estos vehículos pueden circular</t>
+          <t>Senadora Martha Peralta seguirá privada de la libertad por caso Ungrd: niegan habeas corpus</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/sociedad/transversal-del-sisga-reabre-con-restricciones-y-estos-son-los-vehiculos-autorizados-402824</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/20/senadora-martha-peralta-seguira-privada-de-la-libertad-niegan-habeas-corpus/</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>31/05/2026 03:32 p. m.</t>
+          <t>20/06/2026 12:12 p. m.</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -2469,24 +2469,24 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>Transporte para elecciones presidenciales: ajustes y medidas adoptadas por MinTransporte para la movilidad de votantes</t>
+          <t>Fiscalía judicializó a cinco profesores en el Magdalena por irregularidades en proceso de selección de docentes</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/sociedad/movilidad-para-elecciones-presidenciales-mintransporte-anuncia-medidas-especiales-para-votantes-402826</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/20/fiscalia-judicializo-a-cinco-profesores-en-el-magdalena-por-irregularidades-en-proceso-de-seleccion-de-docentes/</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>04/11/2025 07:23 p. m.</t>
+          <t>20/06/2026 09:49 a. m.</t>
         </is>
       </c>
       <c r="B75" s="5" t="inlineStr">
@@ -2496,17 +2496,17 @@
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>LaFM</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr">
         <is>
-          <t>¿Qué riesgos enfrentan las grandes ciudades de cara a la segunda vuelta presidencial? Asocapitales les pone la lupa</t>
+          <t>Defensa de Manuela Echeverri niega millonario acuerdo de divorcio con Santiago Botero</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/politica/segunda-vuelta-presidencial-riesgos-que-electorales-enfrentan-las-ciudades-asocapitales-toma-medidas-402649</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/20/el-millonario-acuerdo-de-divorcio-entre-el-excandidato-presidencial-santiago-botero-y-manuela-echeverry/</t>
         </is>
       </c>
     </row>
@@ -2519,47 +2519,51 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
+          <t>Vanguardia</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>Video | Jorge Barón le dio la tradicional ‘patadita de la buena suerte’ a Abelardo De La Espriella</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>https://www.vanguardia.com/colombia/2026/06/19/video-jorge-baron-le-dio-la-tradicional-patadita-de-la-buena-suerte-a-abelardo-de-la-espriella/</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="5" t="inlineStr">
+        <is>
+          <t>21/06/2026 03:21 a. m.</t>
+        </is>
+      </c>
+      <c r="B77" s="5" t="inlineStr">
+        <is>
+          <t>Medio de Comunicación</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
           <t>LaFM</t>
         </is>
       </c>
-      <c r="D76" s="3" t="inlineStr">
-        <is>
-          <t>Mandatarios del Valle del Cauca piden al Gobierno Nacional mantener la ofensiva tras la muerte de alias 'Marlon'</t>
-        </is>
-      </c>
-      <c r="E76" s="4" t="inlineStr">
-        <is>
-          <t>https://www.lafm.com.co/orden-publico/alcalde-de-cali-y-gobernadora-del-valle-instan-al-gobierno-nacional-a-continuar-acciones-tras-muerte-de-alias-marlon-402842</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="5" t="inlineStr"/>
-      <c r="B77" s="5" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C77" s="5" t="inlineStr">
-        <is>
-          <t>LaFM</t>
-        </is>
-      </c>
       <c r="D77" s="6" t="inlineStr">
         <is>
-          <t>Abatido alias Marlon durante operativos militares: “Es el golpe más duro a las estructuras armadas de la mafia”, dijo Petro</t>
+          <t>Mindefensa: muerte de alias ‘Marlon’ es un duro golpe contra las disidencias de ‘Mordisco’</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/orden-publico/alias-marlon-fue-abatido-en-operativos-militares-y-gustavo-petro-lo-califica-como-golpe-duro-402840</t>
+          <t>https://www.lafm.com.co/orden-publico/mindefensa-muerte-de-alias-marlon-es-un-duro-golpe-contra-las-disidencias-de-mordisco-402844</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>21/06/2026 01:30 a. m.</t>
+          <t>21/06/2026 02:43 a. m.</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -2569,24 +2573,24 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>Así quedaron las tablas del Mundial 2026 tras los partidos de este sábado 20 de junio</t>
+          <t>Ecuador no pudo con Curazao y quedó contra las cuerdas en el Mundial 2026</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/deportes/mundial-2026/asi-quedaron-las-tablas-del-mundial-2026-tras-los-partidos-de-este-sabado-20-de-junio-norteamerica-2026/</t>
+          <t>https://www.lafm.com.co/deportes/mundial-2026-ecuador-empato-con-curazo-402843</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>21/06/2026 01:10 a. m.</t>
+          <t>21/06/2026 01:55 a. m.</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
@@ -2596,24 +2600,24 @@
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
         <is>
-          <t>Japón 4-0 Túnez: partido 1.000 en la historia de la Copa Mundial de la FIFA</t>
+          <t>Gobernador del Cauca tras muerte de alias 'Marlon': "No daremos tregua a las estructuras criminales"</t>
         </is>
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/deportes/mundial-2026/tunez-vs-japon-partido-1000-en-la-historia-de-la-copa-mundial-de-la-fifa-mundial-2026-norteamerica-2026/</t>
+          <t>https://www.lafm.com.co/orden-publico/gobernador-del-cauca-octavio-guzman-habla-tras-muerte-de-alias-marlon-402839</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>21/06/2026 01:00 a. m.</t>
+          <t>21/06/2026 01:06 a. m.</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -2623,24 +2627,24 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>No estamos en economía de demanda</t>
+          <t>Fue abatido alias 'Marlon', máximo cabecilla de las disidencias en Cauca y quien sería el futuro sucesor de 'Mordisco'</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/eduardo-sarmiento/no-estamos-en-economia-de-demanda/</t>
+          <t>https://www.lafm.com.co/orden-publico/abatido-alias-marlon-cabecilla-disidencias-mordisco-cauca-402838</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>21/06/2026 12:07 a. m.</t>
+          <t>21/06/2026 12:19 a. m.</t>
         </is>
       </c>
       <c r="B81" s="5" t="inlineStr">
@@ -2650,24 +2654,24 @@
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D81" s="6" t="inlineStr">
         <is>
-          <t>Entre los palos</t>
+          <t>Así quedan las rutas de TransMilenio con la nueva estación Calle 26 - Atrio</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/piedad-bonnett/entre-los-palos/</t>
+          <t>https://www.lafm.com.co/actualidad/estacion-calle-26-atrio-transmilenio-como-seran-las-rutas-402836</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>21/06/2026 12:07 a. m.</t>
+          <t>20/06/2026 11:38 p. m.</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -2677,24 +2681,24 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>Gane quien gane</t>
+          <t>Gobernadora del Meta denuncia presunto intento de secuestro del alcalde de Mesetas</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/rodrigo-uprimny/gane-quien-gane/</t>
+          <t>https://www.lafm.com.co/orden-publico/meta-gobernadora-denuncia-aparente-intento-secuestro-alcalde-mesetas-402833</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>21/06/2026 12:07 a. m.</t>
+          <t>20/06/2026 11:33 p. m.</t>
         </is>
       </c>
       <c r="B83" s="5" t="inlineStr">
@@ -2704,24 +2708,24 @@
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D83" s="6" t="inlineStr">
         <is>
-          <t>La poesía es un arma cargada de sentido</t>
+          <t>¿Marco Rubio autorizó el documento para detener al activista Beto Coral en EE.UU.? Esto revela The New York Times</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/hector-abad-faciolince/la-poesia-es-un-arma-cargada-de-sentido/</t>
+          <t>https://www.lafm.com.co/internacional/marco-rubio-autorizo-el-documento-para-detener-al-activista-beto-coral-en-eeuu-esto-revela-el-new-york-times-402835</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>21/06/2026 12:06 a. m.</t>
+          <t>20/06/2026 11:26 p. m.</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -2731,24 +2735,24 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>Campaña grotesca</t>
+          <t>Se conoce la razón por la que Georgina Rodríguez no acompañó a Cristinao Ronaldo al Mundial 2026</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/ramiro-bejarano-guzman/campana-grotesca/</t>
+          <t>https://www.lafm.com.co/entretenimiento/mundial-2026-cristiano-ronaldo-por-que-georgina-rodriguez-no-fue-a-verlo-402834</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>21/06/2026 12:06 a. m.</t>
+          <t>20/06/2026 10:49 p. m.</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr">
@@ -2758,24 +2762,24 @@
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D85" s="6" t="inlineStr">
         <is>
-          <t>Mañana (tras las elecciones del odio)</t>
+          <t>Estos son los ocho municipios colombianos que buscan llegar a la vitrina turística de ONU Turismo</t>
         </is>
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/laura-ardila-arrieta/manana-tras-las-elecciones-del-odio/</t>
+          <t>https://www.lafm.com.co/sociedad/onu-turismo-ocho-municipios-colombianos-buscan-reconocimiento-mundial-turismo-rural-402832</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>21/06/2026 12:06 a. m.</t>
+          <t>20/06/2026 10:34 p. m.</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -2785,24 +2789,24 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>De repartir riqueza pasan es a administrar pobreza</t>
+          <t>Bernie Moreno llegó a Bogotá para ser observador internacional en la segunda vuelta de las presidenciales</t>
         </is>
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/mauricio-botero-caicedo/de-repartir-riqueza-pasan-es-a-administrar-pobreza/</t>
+          <t>https://www.lafm.com.co/politica/bernie-moreno-llega-a-bogota-como-observador-internacional-para-la-segunda-vuelta-presidencial-402831</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>21/06/2026 12:06 a. m.</t>
+          <t>20/06/2026 10:18 p. m.</t>
         </is>
       </c>
       <c r="B87" s="5" t="inlineStr">
@@ -2812,24 +2816,24 @@
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>El Espectador</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D87" s="6" t="inlineStr">
         <is>
-          <t>Narcopolítica: ¿por la vida?</t>
+          <t>¿Se podrá operar drones durante las elecciones en segunda vuelta presidencial? Aerocivil hace dura advertencia</t>
         </is>
       </c>
       <c r="E87" s="7" t="inlineStr">
         <is>
-          <t>https://www.elespectador.com/opinion/columnistas/carlos-enrique-moreno/narcopolitica-por-la-vida/</t>
+          <t>https://www.lafm.com.co/sociedad/aerocivil-restringe-operaciones-drones-segunda-vuelta-presidencial-402829</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>21/06/2026 01:11 a. m.</t>
+          <t>20/06/2026 10:09 p. m.</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -2839,24 +2843,24 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>Mundial 2026: Japón goleó a Túnez y sueña en grande</t>
+          <t>Alemania remonta ante Costa de Marfil y clasifica a dieciseisavos del Mundial 2026</t>
         </is>
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/deportes/2026/06/21/mundial-2026-japon-le-gano-a-tunez-y-suena-en-grande/</t>
+          <t>https://www.lafm.com.co/deportes/mundial-2026-alemania-remonta-costa-de-marfil-clasifica-dieciseisavos-402830</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>21/06/2026 01:11 a. m.</t>
+          <t>20/06/2026 09:43 p. m.</t>
         </is>
       </c>
       <c r="B89" s="5" t="inlineStr">
@@ -2866,24 +2870,24 @@
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D89" s="6" t="inlineStr">
         <is>
-          <t>Deportes</t>
+          <t>Colombianos en Venezuela se quedaron sin votar en Cúcuta por cierre fronterizo</t>
         </is>
       </c>
       <c r="E89" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/deportes/</t>
+          <t>https://www.lafm.com.co/actualidad/colombianos-en-venezuela-sin-votar-por-cierre-imprevisto-de-frontera-402827</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>21/06/2026 12:56 a. m.</t>
+          <t>20/06/2026 09:33 p. m.</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -2893,24 +2897,24 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>Países Bajos y Japón golearon; Alemania clasificó y Ecuador se complicó</t>
+          <t>Último sorteo de la Lotería de Boyacá: resultado premio mayor hoy 20 de junio</t>
         </is>
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/deportes/2026/06/21/paises-bajos-y-japon-golearon-alemania-clasifico-y-ecuador-se-complico/</t>
+          <t>https://www.lafm.com.co/sociedad/ultimo-sorteo-de-la-loteria-de-boyaca-resultado-premio-mayor-hoy-20-de-junio-402828</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>21/06/2026 12:00 a. m.</t>
+          <t>20/06/2026 08:40 p. m.</t>
         </is>
       </c>
       <c r="B91" s="5" t="inlineStr">
@@ -2920,24 +2924,24 @@
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D91" s="6" t="inlineStr">
         <is>
-          <t>Cepeda vs. Abelardo en elecciones presidenciales: lo que puede definir el voto</t>
+          <t>Tragedia en hotel de República Dominicana: un muerto y múltiples heridos tras incendio de gran magnitud</t>
         </is>
       </c>
       <c r="E91" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/politica/2026/06/21/cepeda-vs-abelardo-en-elecciones-presidenciales-lo-que-puede-definir-el-voto/</t>
+          <t>https://www.lafm.com.co/internacional/republica-dominicana-incendio-tragedia-muerte-turista-italiana-402825</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>21/06/2026 12:00 a. m.</t>
+          <t>20/06/2026 08:37 p. m.</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -2947,24 +2951,24 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>Política</t>
+          <t>¿Qué pasa con la Transversal del Sisga? Reabre, pero con restricciones: solo estos vehículos pueden circular</t>
         </is>
       </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/politica/</t>
+          <t>https://www.lafm.com.co/sociedad/transversal-del-sisga-reabre-con-restricciones-y-estos-son-los-vehiculos-autorizados-402824</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>21/06/2026 12:00 a. m.</t>
+          <t>31/05/2026 03:32 p. m.</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
@@ -2974,24 +2978,24 @@
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D93" s="6" t="inlineStr">
         <is>
-          <t>Emiratos Árabes Unidos prohíbe redes sociales a menores de 15 años</t>
+          <t>Transporte para elecciones presidenciales: ajustes y medidas adoptadas por MinTransporte para la movilidad de votantes</t>
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/tecnologia/2026/06/21/emiratos-arabes-unidos-prohibe-redes-sociales-a-menores-de-15-anos/</t>
+          <t>https://www.lafm.com.co/sociedad/movilidad-para-elecciones-presidenciales-mintransporte-anuncia-medidas-especiales-para-votantes-402826</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>21/06/2026 12:00 a. m.</t>
+          <t>04/11/2025 07:23 p. m.</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -3001,26 +3005,22 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>Tecnología</t>
+          <t>¿Qué riesgos enfrentan las grandes ciudades de cara a la segunda vuelta presidencial? Asocapitales les pone la lupa</t>
         </is>
       </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/tecnologia/</t>
+          <t>https://www.lafm.com.co/politica/segunda-vuelta-presidencial-riesgos-que-electorales-enfrentan-las-ciudades-asocapitales-toma-medidas-402649</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="5" t="inlineStr">
-        <is>
-          <t>21/06/2026 12:00 a. m.</t>
-        </is>
-      </c>
+      <c r="A95" s="5" t="inlineStr"/>
       <c r="B95" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3028,26 +3028,22 @@
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D95" s="6" t="inlineStr">
         <is>
-          <t>Todo lo que debe saber sobre la segunda vuelta presidencial en Cartagena</t>
+          <t>Mandatarios del Valle del Cauca piden al Gobierno Nacional mantener la ofensiva tras la muerte de alias 'Marlon'</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/cartagena/2026/06/21/todo-lo-que-debe-saber-sobre-la-segunda-vuelta-presidencial-en-cartagena/</t>
+          <t>https://www.lafm.com.co/orden-publico/alcalde-de-cali-y-gobernadora-del-valle-instan-al-gobierno-nacional-a-continuar-acciones-tras-muerte-de-alias-marlon-402842</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="2" t="inlineStr">
-        <is>
-          <t>21/06/2026 12:00 a. m.</t>
-        </is>
-      </c>
+      <c r="A96" s="2" t="inlineStr"/>
       <c r="B96" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3055,24 +3051,24 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>LaFM</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>Cartagena</t>
+          <t>Abatido alias Marlon durante operativos militares: “Es el golpe más duro a las estructuras armadas de la mafia”, dijo Petro</t>
         </is>
       </c>
       <c r="E96" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/cartagena/</t>
+          <t>https://www.lafm.com.co/orden-publico/alias-marlon-fue-abatido-en-operativos-militares-y-gustavo-petro-lo-califica-como-golpe-duro-402840</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>21/06/2026 12:00 a. m.</t>
+          <t>21/06/2026 01:30 a. m.</t>
         </is>
       </c>
       <c r="B97" s="5" t="inlineStr">
@@ -3082,24 +3078,24 @@
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D97" s="6" t="inlineStr">
         <is>
-          <t>FIFA eliminó casi 400 mil publicaciones daniñas en internet por el Mundial</t>
+          <t>Así quedaron las tablas del Mundial 2026 tras los partidos de este sábado 20 de junio</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/tecnologia/2026/06/21/fifa-elimino-casi-400-mil-publicaciones-daninas-en-internet-por-el-mundial/</t>
+          <t>https://www.elespectador.com/deportes/mundial-2026/asi-quedaron-las-tablas-del-mundial-2026-tras-los-partidos-de-este-sabado-20-de-junio-norteamerica-2026/</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>21/06/2026 12:00 a. m.</t>
+          <t>21/06/2026 01:10 a. m.</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -3109,24 +3105,24 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>Domingo emocionante en el Mundial 2026: estos son los partidos de este 21 de junio</t>
+          <t>Japón 4-0 Túnez: partido 1.000 en la historia de la Copa Mundial de la FIFA</t>
         </is>
       </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/deportes/2026/06/21/domingo-emocionante-en-el-mundial-2026-estos-son-los-partidos-de-este-21-de-junio/</t>
+          <t>https://www.elespectador.com/deportes/mundial-2026/tunez-vs-japon-partido-1000-en-la-historia-de-la-copa-mundial-de-la-fifa-mundial-2026-norteamerica-2026/</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 11:31 p. m.</t>
+          <t>21/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B99" s="5" t="inlineStr">
@@ -3136,24 +3132,24 @@
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D99" s="6" t="inlineStr">
         <is>
-          <t>Video: gol de taco le está dando la victoria a Japón ante Túnez en el Mundial 2026</t>
+          <t>No estamos en economía de demanda</t>
         </is>
       </c>
       <c r="E99" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/deportes/2026/06/20/video-gol-de-taco-le-esta-dando-la-victoria-a-japon-ante-tunez-en-el-mundial-2026/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/eduardo-sarmiento/no-estamos-en-economia-de-demanda/</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 10:41 p. m.</t>
+          <t>21/06/2026 12:07 a. m.</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -3163,24 +3159,24 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>Petro confirmó la muerte de alias Marlon, segundo al mando de Iván Mordisco</t>
+          <t>Entre los palos</t>
         </is>
       </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/colombia/2026/06/20/petro-confirmo-la-muerte-de-alias-marlon-segundo-al-mando-de-ivan-mordisco/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/piedad-bonnett/entre-los-palos/</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 10:41 p. m.</t>
+          <t>21/06/2026 12:07 a. m.</t>
         </is>
       </c>
       <c r="B101" s="5" t="inlineStr">
@@ -3190,24 +3186,24 @@
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D101" s="6" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Gane quien gane</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/colombia/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/rodrigo-uprimny/gane-quien-gane/</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 09:54 p. m.</t>
+          <t>21/06/2026 12:07 a. m.</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -3217,24 +3213,24 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>¿Habrá peajes en el estrecho de Ormuz? Esto dijo Donald Trump</t>
+          <t>La poesía es un arma cargada de sentido</t>
         </is>
       </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/mundo/2026/06/20/habra-peajes-en-el-estrecho-de-ormuz-esto-dijo-donald-trump/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/hector-abad-faciolince/la-poesia-es-un-arma-cargada-de-sentido/</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 09:24 p. m.</t>
+          <t>21/06/2026 12:06 a. m.</t>
         </is>
       </c>
       <c r="B103" s="5" t="inlineStr">
@@ -3244,24 +3240,24 @@
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D103" s="6" t="inlineStr">
         <is>
-          <t>Video: las mejores atajadas de Eloy Room, arquero de Curazao, ante Ecuador</t>
+          <t>Campaña grotesca</t>
         </is>
       </c>
       <c r="E103" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/deportes/2026/06/20/video-las-mejores-atajadas-de-eloy-room-arquero-de-curazao-ante-ecuador/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/ramiro-bejarano-guzman/campana-grotesca/</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 08:12 p. m.</t>
+          <t>21/06/2026 12:06 a. m.</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
@@ -3271,24 +3267,24 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>Hombre fue asesinado a tiros en Villas de Aranjuez: otro resultó herido</t>
+          <t>Mañana (tras las elecciones del odio)</t>
         </is>
       </c>
       <c r="E104" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/sucesos/2026/06/20/hombre-fue-asesinado-a-tiros-en-villa-aranjuez-otro-resulto-herido/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/laura-ardila-arrieta/manana-tras-las-elecciones-del-odio/</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 07:37 p. m.</t>
+          <t>21/06/2026 12:06 a. m.</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
@@ -3298,24 +3294,24 @@
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D105" s="6" t="inlineStr">
         <is>
-          <t>Sábado lluvioso en Cartagena: reportan fuerte aguacero en sectores de la ciudad</t>
+          <t>De repartir riqueza pasan es a administrar pobreza</t>
         </is>
       </c>
       <c r="E105" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/cartagena/2026/06/20/sabado-lluvioso-en-cartagena-reportan-fuerte-aguacero-en-sectores-de-la-ciudad/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/mauricio-botero-caicedo/de-repartir-riqueza-pasan-es-a-administrar-pobreza/</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 07:05 p. m.</t>
+          <t>21/06/2026 12:06 a. m.</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
@@ -3325,24 +3321,24 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>El Universal</t>
+          <t>El Espectador</t>
         </is>
       </c>
       <c r="D106" s="3" t="inlineStr">
         <is>
-          <t>Defensa de Manuela Echeverri niega millonario acuerdo de divorcio con Santiago Botero</t>
+          <t>Narcopolítica: ¿por la vida?</t>
         </is>
       </c>
       <c r="E106" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/colombia/2026/06/20/defensa-de-manuela-echeverri-niega-millonario-acuerdo-de-divorcio-con-santiago-botero/</t>
+          <t>https://www.elespectador.com/opinion/columnistas/carlos-enrique-moreno/narcopolitica-por-la-vida/</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 05:06 p. m.</t>
+          <t>21/06/2026 01:11 a. m.</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
@@ -3357,19 +3353,19 @@
       </c>
       <c r="D107" s="6" t="inlineStr">
         <is>
-          <t>Cayeron ‘Kike’ y ‘Alex’ en Cartagena: eran buscados y suman anotaciones judiciales</t>
+          <t>Mundial 2026: Japón goleó a Túnez y sueña en grande</t>
         </is>
       </c>
       <c r="E107" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/sucesos/2026/06/20/capturan-a-kike-y-alex-en-cartagena-eran-buscados-y-suman-anotaciones-judiciales/</t>
+          <t>https://www.eluniversal.com.co/deportes/2026/06/21/mundial-2026-japon-le-gano-a-tunez-y-suena-en-grande/</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 05:04 p. m.</t>
+          <t>21/06/2026 01:11 a. m.</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
@@ -3384,19 +3380,19 @@
       </c>
       <c r="D108" s="3" t="inlineStr">
         <is>
-          <t>Capturan a alias ‘Bisolvón’ con arma de fuego en un operativo en Arjona</t>
+          <t>Deportes</t>
         </is>
       </c>
       <c r="E108" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/sucesos/2026/06/20/capturan-a-alias-bisolvon-con-artefacto-en-un-operativo-en-arjona/</t>
+          <t>https://www.eluniversal.com.co/deportes/</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 04:50 p. m.</t>
+          <t>21/06/2026 12:56 a. m.</t>
         </is>
       </c>
       <c r="B109" s="5" t="inlineStr">
@@ -3411,19 +3407,19 @@
       </c>
       <c r="D109" s="6" t="inlineStr">
         <is>
-          <t>Ataque sicarial dejó a un hombre herido en San Isidro: tiene 10 anotaciones</t>
+          <t>Países Bajos y Japón golearon; Alemania clasificó y Ecuador se complicó</t>
         </is>
       </c>
       <c r="E109" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/sucesos/2026/06/20/ataque-sicarial-dejo-a-un-hombre-herido-en-san-isidro-tiene-10-anotaciones/</t>
+          <t>https://www.eluniversal.com.co/deportes/2026/06/21/paises-bajos-y-japon-golearon-alemania-clasifico-y-ecuador-se-complico/</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 04:39 p. m.</t>
+          <t>21/06/2026 12:00 a. m.</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
@@ -3438,19 +3434,19 @@
       </c>
       <c r="D110" s="3" t="inlineStr">
         <is>
-          <t>Mientras esperaban el bus, sicarios atacaron a bala a 2 hermanos: uno perdió la vida</t>
+          <t>Cepeda vs. Abelardo en elecciones presidenciales: lo que puede definir el voto</t>
         </is>
       </c>
       <c r="E110" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/sucesos/2026/06/20/mientras-esperaban-el-bus-sicarios-atacaron-a-dos-hermanos-uno-perdio-la-vida/</t>
+          <t>https://www.eluniversal.com.co/politica/2026/06/21/cepeda-vs-abelardo-en-elecciones-presidenciales-lo-que-puede-definir-el-voto/</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 03:57 p. m.</t>
+          <t>21/06/2026 12:00 a. m.</t>
         </is>
       </c>
       <c r="B111" s="5" t="inlineStr">
@@ -3465,19 +3461,19 @@
       </c>
       <c r="D111" s="6" t="inlineStr">
         <is>
-          <t>Hallan sin vida al bañista de 28 años, desaparecido en playas de Puerto Colombia</t>
+          <t>Política</t>
         </is>
       </c>
       <c r="E111" s="7" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/sucesos/2026/06/20/hallan-sin-vida-al-banista-de-28-anos-desaparecido-en-playas-de-puerto-colombia/</t>
+          <t>https://www.eluniversal.com.co/politica/</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 10:27 a. m.</t>
+          <t>21/06/2026 12:00 a. m.</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
@@ -3492,19 +3488,19 @@
       </c>
       <c r="D112" s="3" t="inlineStr">
         <is>
-          <t>Condenan a 7 integrantes de red que explotaba a niños indígenas para mendigar</t>
+          <t>Emiratos Árabes Unidos prohíbe redes sociales a menores de 15 años</t>
         </is>
       </c>
       <c r="E112" s="4" t="inlineStr">
         <is>
-          <t>https://www.eluniversal.com.co/sucesos/2026/06/20/condenan-a-7-integrantes-de-red-que-explotaba-a-ninos-indigenas-para-mendigar/</t>
+          <t>https://www.eluniversal.com.co/tecnologia/2026/06/21/emiratos-arabes-unidos-prohibe-redes-sociales-a-menores-de-15-anos/</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
-          <t>21/06/2026 01:00 a. m.</t>
+          <t>21/06/2026 12:00 a. m.</t>
         </is>
       </c>
       <c r="B113" s="5" t="inlineStr">
@@ -3514,24 +3510,24 @@
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D113" s="6" t="inlineStr">
         <is>
-          <t>Análisis de las elecciones presidenciales (III): Los errores de la campaña de Cepeda</t>
+          <t>Tecnología</t>
         </is>
       </c>
       <c r="E113" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/21/analisis-de-las-elecciones-presidenciales-iii-los-errores-de-la-campana-de-cepeda/</t>
+          <t>https://www.eluniversal.com.co/tecnologia/</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>21/06/2026 01:00 a. m.</t>
+          <t>21/06/2026 12:00 a. m.</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
@@ -3541,24 +3537,24 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D114" s="3" t="inlineStr">
         <is>
-          <t>Columnistas</t>
+          <t>Todo lo que debe saber sobre la segunda vuelta presidencial en Cartagena</t>
         </is>
       </c>
       <c r="E114" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/</t>
+          <t>https://www.eluniversal.com.co/cartagena/2026/06/21/todo-lo-que-debe-saber-sobre-la-segunda-vuelta-presidencial-en-cartagena/</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="5" t="inlineStr">
         <is>
-          <t>21/06/2026 01:00 a. m.</t>
+          <t>21/06/2026 12:00 a. m.</t>
         </is>
       </c>
       <c r="B115" s="5" t="inlineStr">
@@ -3568,24 +3564,24 @@
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D115" s="6" t="inlineStr">
         <is>
-          <t>Participación, serenidad y unión</t>
+          <t>Cartagena</t>
         </is>
       </c>
       <c r="E115" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/21/participacion-serenidad-y-union/</t>
+          <t>https://www.eluniversal.com.co/cartagena/</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>21/06/2026 01:00 a. m.</t>
+          <t>21/06/2026 12:00 a. m.</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
@@ -3595,24 +3591,24 @@
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D116" s="3" t="inlineStr">
         <is>
-          <t>Píldoras para la memoria: lo que Colombia no debe olvidar antes de elegir</t>
+          <t>FIFA eliminó casi 400 mil publicaciones daniñas en internet por el Mundial</t>
         </is>
       </c>
       <c r="E116" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/maria-juliana-acebedo/2026/06/21/pildoras-para-la-memoria-lo-que-colombia-no-debe-olvidar-antes-de-elegir/</t>
+          <t>https://www.eluniversal.com.co/tecnologia/2026/06/21/fifa-elimino-casi-400-mil-publicaciones-daninas-en-internet-por-el-mundial/</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="5" t="inlineStr">
         <is>
-          <t>21/06/2026 01:00 a. m.</t>
+          <t>21/06/2026 12:00 a. m.</t>
         </is>
       </c>
       <c r="B117" s="5" t="inlineStr">
@@ -3622,24 +3618,24 @@
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D117" s="6" t="inlineStr">
         <is>
-          <t>Maria Juliana Acebedo</t>
+          <t>Domingo emocionante en el Mundial 2026: estos son los partidos de este 21 de junio</t>
         </is>
       </c>
       <c r="E117" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/maria-juliana-acebedo/</t>
+          <t>https://www.eluniversal.com.co/deportes/2026/06/21/domingo-emocionante-en-el-mundial-2026-estos-son-los-partidos-de-este-21-de-junio/</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>21/06/2026 01:00 a. m.</t>
+          <t>20/06/2026 11:31 p. m.</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
@@ -3649,24 +3645,24 @@
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D118" s="3" t="inlineStr">
         <is>
-          <t>¡Salvemos a Colombia!</t>
+          <t>Video: gol de taco le está dando la victoria a Japón ante Túnez en el Mundial 2026</t>
         </is>
       </c>
       <c r="E118" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/alberto-montoya/2026/06/21/salvemos-a-colombia/</t>
+          <t>https://www.eluniversal.com.co/deportes/2026/06/20/video-gol-de-taco-le-esta-dando-la-victoria-a-japon-ante-tunez-en-el-mundial-2026/</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="5" t="inlineStr">
         <is>
-          <t>21/06/2026 01:00 a. m.</t>
+          <t>20/06/2026 10:41 p. m.</t>
         </is>
       </c>
       <c r="B119" s="5" t="inlineStr">
@@ -3676,24 +3672,24 @@
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D119" s="6" t="inlineStr">
         <is>
-          <t>Alberto Montoya</t>
+          <t>Petro confirmó la muerte de alias Marlon, segundo al mando de Iván Mordisco</t>
         </is>
       </c>
       <c r="E119" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/alberto-montoya/</t>
+          <t>https://www.eluniversal.com.co/colombia/2026/06/20/petro-confirmo-la-muerte-de-alias-marlon-segundo-al-mando-de-ivan-mordisco/</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 11:11 p. m.</t>
+          <t>20/06/2026 10:41 p. m.</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
@@ -3703,24 +3699,24 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D120" s="3" t="inlineStr">
         <is>
-          <t>Ejército abatió a alias ‘Marlon’, jefe clave de disidencias de ‘Iván Mordisco’ en Cauca</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E120" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/20/ejercito-abatio-a-alias-marlon-jefe-clave-de-disidencias-de-ivan-mordisco-en-cauca/</t>
+          <t>https://www.eluniversal.com.co/colombia/</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 11:11 p. m.</t>
+          <t>20/06/2026 09:54 p. m.</t>
         </is>
       </c>
       <c r="B121" s="5" t="inlineStr">
@@ -3730,24 +3726,24 @@
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D121" s="6" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>¿Habrá peajes en el estrecho de Ormuz? Esto dijo Donald Trump</t>
         </is>
       </c>
       <c r="E121" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/</t>
+          <t>https://www.eluniversal.com.co/mundo/2026/06/20/habra-peajes-en-el-estrecho-de-ormuz-esto-dijo-donald-trump/</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 10:53 p. m.</t>
+          <t>20/06/2026 09:24 p. m.</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
@@ -3757,24 +3753,24 @@
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D122" s="3" t="inlineStr">
         <is>
-          <t>Pensionado fue víctima de estafa dirigida desde Sudáfrica: así perdió $93 millones</t>
+          <t>Video: las mejores atajadas de Eloy Room, arquero de Curazao, ante Ecuador</t>
         </is>
       </c>
       <c r="E122" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/contenido-registrados/2026/06/20/pensionado-fue-victima-de-estafa-dirigida-desde-sudafrica-asi-perdio-93-millones/</t>
+          <t>https://www.eluniversal.com.co/deportes/2026/06/20/video-las-mejores-atajadas-de-eloy-room-arquero-de-curazao-ante-ecuador/</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 10:53 p. m.</t>
+          <t>20/06/2026 08:12 p. m.</t>
         </is>
       </c>
       <c r="B123" s="5" t="inlineStr">
@@ -3784,24 +3780,24 @@
       </c>
       <c r="C123" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D123" s="6" t="inlineStr">
         <is>
-          <t>Contenido registrados</t>
+          <t>Hombre fue asesinado a tiros en Villas de Aranjuez: otro resultó herido</t>
         </is>
       </c>
       <c r="E123" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/contenido-registrados/</t>
+          <t>https://www.eluniversal.com.co/sucesos/2026/06/20/hombre-fue-asesinado-a-tiros-en-villa-aranjuez-otro-resulto-herido/</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 07:29 p. m.</t>
+          <t>20/06/2026 07:37 p. m.</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
@@ -3811,24 +3807,24 @@
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D124" s="3" t="inlineStr">
         <is>
-          <t>Capturan en Cali a ‘El Sueco’, clave en el envío de cocaína hacia Europa y Medio Oriente</t>
+          <t>Sábado lluvioso en Cartagena: reportan fuerte aguacero en sectores de la ciudad</t>
         </is>
       </c>
       <c r="E124" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/20/capturan-en-cali-a-el-sueco-clave-en-el-envio-de-cocaina-hacia-europa-y-medio-oriente/</t>
+          <t>https://www.eluniversal.com.co/cartagena/2026/06/20/sabado-lluvioso-en-cartagena-reportan-fuerte-aguacero-en-sectores-de-la-ciudad/</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 04:04 p. m.</t>
+          <t>20/06/2026 07:05 p. m.</t>
         </is>
       </c>
       <c r="B125" s="5" t="inlineStr">
@@ -3838,24 +3834,24 @@
       </c>
       <c r="C125" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D125" s="6" t="inlineStr">
         <is>
-          <t>El drama de una familia atrapada en la guerra del Catatumbo: niño murió y una bebé lucha por su vida</t>
+          <t>Defensa de Manuela Echeverri niega millonario acuerdo de divorcio con Santiago Botero</t>
         </is>
       </c>
       <c r="E125" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/20/el-drama-de-una-familia-atrapada-en-la-guerra-del-catatumbo-nino-murio-y-una-bebe-lucha-por-su-vida/</t>
+          <t>https://www.eluniversal.com.co/colombia/2026/06/20/defensa-de-manuela-echeverri-niega-millonario-acuerdo-de-divorcio-con-santiago-botero/</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 03:29 p. m.</t>
+          <t>20/06/2026 05:06 p. m.</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
@@ -3865,24 +3861,24 @@
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D126" s="3" t="inlineStr">
         <is>
-          <t>Asesinan a Mónica Eugenia Sánchez, reconocida lideresa social de Santa Bárbara, Antioquia</t>
+          <t>Cayeron ‘Kike’ y ‘Alex’ en Cartagena: eran buscados y suman anotaciones judiciales</t>
         </is>
       </c>
       <c r="E126" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/20/asesinan-a-monica-eugenia-sanchez-reconocida-lideresa-social-de-santa-barbara-antioquia/</t>
+          <t>https://www.eluniversal.com.co/sucesos/2026/06/20/capturan-a-kike-y-alex-en-cartagena-eran-buscados-y-suman-anotaciones-judiciales/</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 03:15 p. m.</t>
+          <t>20/06/2026 05:04 p. m.</t>
         </is>
       </c>
       <c r="B127" s="5" t="inlineStr">
@@ -3892,24 +3888,24 @@
       </c>
       <c r="C127" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D127" s="6" t="inlineStr">
         <is>
-          <t>Senadora Martha Peralta seguirá privada de la libertad por caso Ungrd: niegan habeas corpus</t>
+          <t>Capturan a alias ‘Bisolvón’ con arma de fuego en un operativo en Arjona</t>
         </is>
       </c>
       <c r="E127" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/20/senadora-martha-peralta-seguira-privada-de-la-libertad-niegan-habeas-corpus/</t>
+          <t>https://www.eluniversal.com.co/sucesos/2026/06/20/capturan-a-alias-bisolvon-con-artefacto-en-un-operativo-en-arjona/</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 12:12 p. m.</t>
+          <t>20/06/2026 04:50 p. m.</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
@@ -3919,24 +3915,24 @@
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D128" s="3" t="inlineStr">
         <is>
-          <t>Fiscalía judicializó a cinco profesores en el Magdalena por irregularidades en proceso de selección de docentes</t>
+          <t>Ataque sicarial dejó a un hombre herido en San Isidro: tiene 10 anotaciones</t>
         </is>
       </c>
       <c r="E128" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/20/fiscalia-judicializo-a-cinco-profesores-en-el-magdalena-por-irregularidades-en-proceso-de-seleccion-de-docentes/</t>
+          <t>https://www.eluniversal.com.co/sucesos/2026/06/20/ataque-sicarial-dejo-a-un-hombre-herido-en-san-isidro-tiene-10-anotaciones/</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 09:49 a. m.</t>
+          <t>20/06/2026 04:39 p. m.</t>
         </is>
       </c>
       <c r="B129" s="5" t="inlineStr">
@@ -3946,24 +3942,24 @@
       </c>
       <c r="C129" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D129" s="6" t="inlineStr">
         <is>
-          <t>Defensa de Manuela Echeverri niega millonario acuerdo de divorcio con Santiago Botero</t>
+          <t>Mientras esperaban el bus, sicarios atacaron a bala a 2 hermanos: uno perdió la vida</t>
         </is>
       </c>
       <c r="E129" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/20/el-millonario-acuerdo-de-divorcio-entre-el-excandidato-presidencial-santiago-botero-y-manuela-echeverry/</t>
+          <t>https://www.eluniversal.com.co/sucesos/2026/06/20/mientras-esperaban-el-bus-sicarios-atacaron-a-dos-hermanos-uno-perdio-la-vida/</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026 09:13 a. m.</t>
+          <t>20/06/2026 03:57 p. m.</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
@@ -3973,22 +3969,26 @@
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D130" s="3" t="inlineStr">
         <is>
-          <t>Petro exige a Trump que se revele la ubicación del influencer Beto Coral</t>
+          <t>Hallan sin vida al bañista de 28 años, desaparecido en playas de Puerto Colombia</t>
         </is>
       </c>
       <c r="E130" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/20/petro-exige-a-trump-que-se-revele-la-ubicacion-del-influencer-beto-coral/</t>
+          <t>https://www.eluniversal.com.co/sucesos/2026/06/20/hallan-sin-vida-al-banista-de-28-anos-desaparecido-en-playas-de-puerto-colombia/</t>
         </is>
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="5" t="inlineStr"/>
+      <c r="A131" s="5" t="inlineStr">
+        <is>
+          <t>20/06/2026 10:27 a. m.</t>
+        </is>
+      </c>
       <c r="B131" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3996,24 +3996,24 @@
       </c>
       <c r="C131" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El Universal</t>
         </is>
       </c>
       <c r="D131" s="6" t="inlineStr">
         <is>
-          <t>Video | Jorge Barón le dio la tradicional ‘patadita de la buena suerte’ a Abelardo De La Espriella</t>
+          <t>Condenan a 7 integrantes de red que explotaba a niños indígenas para mendigar</t>
         </is>
       </c>
       <c r="E131" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/19/video-jorge-baron-le-dio-la-tradicional-patadita-de-la-buena-suerte-a-abelardo-de-la-espriella/</t>
+          <t>https://www.eluniversal.com.co/sucesos/2026/06/20/condenan-a-7-integrantes-de-red-que-explotaba-a-ninos-indigenas-para-mendigar/</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>21/06/2026 12:46 a. m.</t>
+          <t>21/06/2026 12:22 a. m.</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
@@ -4040,7 +4040,7 @@
     <row r="133">
       <c r="A133" s="5" t="inlineStr">
         <is>
-          <t>21/06/2026 12:46 a. m.</t>
+          <t>21/06/2026 12:22 a. m.</t>
         </is>
       </c>
       <c r="B133" s="5" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>21/06/2026 12:46 a. m.</t>
+          <t>21/06/2026 12:22 a. m.</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
@@ -4094,7 +4094,7 @@
     <row r="135">
       <c r="A135" s="5" t="inlineStr">
         <is>
-          <t>21/06/2026 12:46 a. m.</t>
+          <t>21/06/2026 12:22 a. m.</t>
         </is>
       </c>
       <c r="B135" s="5" t="inlineStr">
@@ -4121,7 +4121,7 @@
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>21/06/2026 12:46 a. m.</t>
+          <t>21/06/2026 12:22 a. m.</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
@@ -4148,7 +4148,7 @@
     <row r="137">
       <c r="A137" s="5" t="inlineStr">
         <is>
-          <t>21/06/2026 12:46 a. m.</t>
+          <t>21/06/2026 12:22 a. m.</t>
         </is>
       </c>
       <c r="B137" s="5" t="inlineStr">
@@ -4175,7 +4175,7 @@
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>21/06/2026 12:46 a. m.</t>
+          <t>21/06/2026 12:22 a. m.</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
@@ -4420,12 +4420,12 @@
       </c>
       <c r="D148" s="3" t="inlineStr">
         <is>
-          <t>¿Batalla de algoritmos? Así se han movido los candidatos en redes: Abelardo con un 52% de impacto frente al 48% de Cepeda</t>
+          <t>Pilas con usar el celular en el puesto de votación: estas son las razones</t>
         </is>
       </c>
       <c r="E148" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/elecciones-2026/impacto-redes-sociales-abelardo-espriella-ivan-cepeda-segunda-vuelta-2026-OI37954947</t>
+          <t>https://www.elcolombiano.com/especiales/elecciones-2026/elecciones-segunda-vuelta-uso-celular-puesto-votacion-EB37501500</t>
         </is>
       </c>
     </row>
@@ -4443,12 +4443,12 @@
       </c>
       <c r="D149" s="6" t="inlineStr">
         <is>
-          <t>Pilas con usar el celular en el puesto de votación: estas son las razones</t>
+          <t>Operativo destapa helicóptero con pasado oscuro y motor Rolls-Royce</t>
         </is>
       </c>
       <c r="E149" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/elecciones-2026/elecciones-segunda-vuelta-uso-celular-puesto-votacion-EB37501500</t>
+          <t>https://www.elcolombiano.com/colombia/ejercito-incauta-helicoptero-de-la-mafia-NG33717192</t>
         </is>
       </c>
     </row>
@@ -4466,12 +4466,12 @@
       </c>
       <c r="D150" s="3" t="inlineStr">
         <is>
-          <t>Operativo destapa helicóptero con pasado oscuro y motor Rolls-Royce</t>
+          <t>Proantioquia y la OEA, así como distintas personalidades, hacen un llamado a respetar los resultados de este domingo.</t>
         </is>
       </c>
       <c r="E150" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/ejercito-incauta-helicoptero-de-la-mafia-NG33717192</t>
+          <t>https://www.elcolombiano.com/colombia/abelardo-de-la-espriella-e-ivan-cepeda-todo-listo-para-observar-elecciones-HK37976331</t>
         </is>
       </c>
     </row>
@@ -4489,12 +4489,12 @@
       </c>
       <c r="D151" s="6" t="inlineStr">
         <is>
-          <t>Proantioquia y la OEA, así como distintas personalidades, hacen un llamado a respetar los resultados de este domingo.</t>
+          <t>Raphinha se somete a un “tratamiento intensivo” y será baja de Brasil ante Escocia</t>
         </is>
       </c>
       <c r="E151" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/abelardo-de-la-espriella-e-ivan-cepeda-todo-listo-para-observar-elecciones-HK37976331</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/raphinha-es-baja-de-brasil-para-el-duelo-ante-escocia-en-el-mundial-de-norteamerica-LK37976195</t>
         </is>
       </c>
     </row>
@@ -4512,12 +4512,12 @@
       </c>
       <c r="D152" s="3" t="inlineStr">
         <is>
-          <t>Raphinha se somete a un “tratamiento intensivo” y será baja de Brasil ante Escocia</t>
+          <t>Aguacero terminó tumbando árboles en vía principal del Valle de Aburrá: ¿qué pasó?</t>
         </is>
       </c>
       <c r="E152" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/mundial-2026/raphinha-es-baja-de-brasil-para-el-duelo-ante-escocia-en-el-mundial-de-norteamerica-LK37976195</t>
+          <t>https://www.elcolombiano.com/antioquia/caida-arboles-variante-caldas-medellin-carros-danados-EK37973788</t>
         </is>
       </c>
     </row>
@@ -4535,12 +4535,12 @@
       </c>
       <c r="D153" s="6" t="inlineStr">
         <is>
-          <t>Aguacero terminó tumbando árboles en vía principal del Valle de Aburrá: ¿qué pasó?</t>
+          <t>Fact check: video de Fajardo haciendo un corazón, como si apoyara a Cepeda, no es actual</t>
         </is>
       </c>
       <c r="E153" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/antioquia/caida-arboles-variante-caldas-medellin-carros-danados-EK37973788</t>
+          <t>https://www.elcolombiano.com/colombia/fact-check-video-de-fajardo-haciendo-un-corazon-como-si-apoyara-a-cepeda-no-es-actual-GK37974516</t>
         </is>
       </c>
     </row>
@@ -4558,12 +4558,12 @@
       </c>
       <c r="D154" s="3" t="inlineStr">
         <is>
-          <t>Fact check: video de Fajardo haciendo un corazón, como si apoyara a Cepeda, no es actual</t>
+          <t>Alemania sufrió, pero al final logró la victoria ante Costa de Marfil y es líder del Grupo E del Mundial de Norteamérica</t>
         </is>
       </c>
       <c r="E154" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/fact-check-video-de-fajardo-haciendo-un-corazon-como-si-apoyara-a-cepeda-no-es-actual-GK37974516</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/alemania-gano-ane-costa-marfil-y-se-clasifico-a-dieciseisavos-en-norteamerica-NK37973428</t>
         </is>
       </c>
     </row>
@@ -4581,12 +4581,12 @@
       </c>
       <c r="D155" s="6" t="inlineStr">
         <is>
-          <t>Alemania sufrió, pero al final logró la victoria ante Costa de Marfil y es líder del Grupo E del Mundial de Norteamérica</t>
+          <t>Bernie Moreno ya está en Colombia para observar las elecciones: “el futuro está en sus propias manos”</t>
         </is>
       </c>
       <c r="E155" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/mundial-2026/alemania-gano-ane-costa-marfil-y-se-clasifico-a-dieciseisavos-en-norteamerica-NK37973428</t>
+          <t>https://www.elcolombiano.com/colombia/bernie-moreno-ya-esta-en-colombia-para-observar-las-elecciones-de-segunda-vuelta-PK37972490</t>
         </is>
       </c>
     </row>
@@ -4604,12 +4604,12 @@
       </c>
       <c r="D156" s="3" t="inlineStr">
         <is>
-          <t>Bernie Moreno ya está en Colombia para observar las elecciones: “el futuro está en sus propias manos”</t>
+          <t>Auditoría internacional también concluye que no hubo fraude o irregularidades en la primera vuelta presidencial en Colombia</t>
         </is>
       </c>
       <c r="E156" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/bernie-moreno-ya-esta-en-colombia-para-observar-las-elecciones-de-segunda-vuelta-PK37972490</t>
+          <t>https://www.elcolombiano.com/colombia/auditoria-no-hubo-fraude-irregularidades-primera-vuelta-presidencial-colombia-HK37971512</t>
         </is>
       </c>
     </row>
@@ -4627,12 +4627,12 @@
       </c>
       <c r="D157" s="6" t="inlineStr">
         <is>
-          <t>Auditoría internacional también concluye que no hubo fraude o irregularidades en la primera vuelta presidencial en Colombia</t>
+          <t>Vuelve “la novela de los domingos”: se estrena la tercera temporada de La casa del dragón</t>
         </is>
       </c>
       <c r="E157" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/auditoria-no-hubo-fraude-irregularidades-primera-vuelta-presidencial-colombia-HK37971512</t>
+          <t>https://www.elcolombiano.com/entretenimiento/television/la-casa-del-dragon-house-of-the-dragon-temporada-tres-hbo-NK37971149</t>
         </is>
       </c>
     </row>
@@ -4650,12 +4650,12 @@
       </c>
       <c r="D158" s="3" t="inlineStr">
         <is>
-          <t>Vuelve “la novela de los domingos”: se estrena la tercera temporada de La casa del dragón</t>
+          <t>¡Vote aunque truene y llueva! Ideam pronostica lluvias durante la segunda vuelta presidencial en Colombia</t>
         </is>
       </c>
       <c r="E158" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/entretenimiento/television/la-casa-del-dragon-house-of-the-dragon-temporada-tres-hbo-NK37971149</t>
+          <t>https://www.elcolombiano.com/especiales/elecciones-2026/lluvias-colombia-elecciones-presidenciales-segunda-vuelta-ideam-JK37970393</t>
         </is>
       </c>
     </row>
@@ -4673,12 +4673,12 @@
       </c>
       <c r="D159" s="6" t="inlineStr">
         <is>
-          <t>¡Vote aunque truene y llueva! Ideam pronostica lluvias durante la segunda vuelta presidencial en Colombia</t>
+          <t>Julián Quiñones vive un sueño: le renovaron contrato en Arabia con una cláusula carísima después de su gol en el Mundial</t>
         </is>
       </c>
       <c r="E159" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/elecciones-2026/lluvias-colombia-elecciones-presidenciales-segunda-vuelta-ideam-JK37970393</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/julian-quinones-seleccion-mexico-colombia-goleador-arabia-clausura-recesion-contrato-nuevo-CK37971452</t>
         </is>
       </c>
     </row>
@@ -4696,12 +4696,12 @@
       </c>
       <c r="D160" s="3" t="inlineStr">
         <is>
-          <t>¿Cómo se moverá el voto decisivo en segunda vuelta?</t>
+          <t>Brecha de 40 años separa al DT más joven, del más veterano del Mundial 2026, ¿quiénes son?</t>
         </is>
       </c>
       <c r="E160" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/elecciones-2026/como-se-movera-el-voto-decisivo-en-segunda-vuelta-NI37956957</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/tecnico-mas-joven-y-mas-veterano-mundial-norteamerica-2026-julian-naggelsman-seleccion-alemania-BK37973673</t>
         </is>
       </c>
     </row>
@@ -4719,12 +4719,12 @@
       </c>
       <c r="D161" s="6" t="inlineStr">
         <is>
-          <t>Julián Quiñones vive un sueño: le renovaron contrato en Arabia con una cláusula carísima después de su gol en el Mundial</t>
+          <t>Video | El defensa inglés Harry Maguire, que quedó fuera de la convocatoria, fue visto vendiendo láminas de Panini en las calles de EE. UU.</t>
         </is>
       </c>
       <c r="E161" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/mundial-2026/julian-quinones-seleccion-mexico-colombia-goleador-arabia-clausura-recesion-contrato-nuevo-CK37971452</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/video-defensa-ingles-harry-maguire-vende-laminas-album-panini-estados-unidos-JK37971945</t>
         </is>
       </c>
     </row>
@@ -4854,7 +4854,7 @@
       </c>
       <c r="D166" s="3" t="inlineStr">
         <is>
-          <t>Éder y Dilian destacan muerte de alias ‘Marlon’, responsable de atentados en Cali y el Valle</t>
+          <t>Alcalde de Cali y gobernadora del Valle destacan muerte de alias 'Marlon'</t>
         </is>
       </c>
       <c r="E166" s="4" t="inlineStr">
@@ -5070,12 +5070,12 @@
       </c>
       <c r="D174" s="3" t="inlineStr">
         <is>
-          <t>Resultado Chontico Noche: números ganadores del último sorteo hoy, sábado 20 de junio de 2026</t>
+          <t>Nueva Zelanda vs Egipto, en VIVO: Siga el minuto a minuto de la segunda fecha del Grupo G del Mundial 2026</t>
         </is>
       </c>
       <c r="E174" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/21/resultado-chontico-noche-numeros-ganadores-del-ultimo-sorteo-hoy-sabado-20-de-junio-de-2026/</t>
+          <t>https://www.infobae.com/colombia/deportes/2026/06/21/nueva-zelanda-vs-egipto-en-vivo-siga-el-minuto-a-minuto-de-la-segunda-fecha-del-grupo-g-del-mundial-2026/</t>
         </is>
       </c>
     </row>
@@ -5097,12 +5097,12 @@
       </c>
       <c r="D175" s="6" t="inlineStr">
         <is>
-          <t>Resultado Lotería del Cauca hoy 20 de junio</t>
+          <t>Las últimas previsiones para Medellín: temperatura, lluvias y viento</t>
         </is>
       </c>
       <c r="E175" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/21/resultado-loteria-del-cauca-hoy-20-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/21/las-ultimas-previsiones-para-medellin-temperatura-lluvias-y-viento/</t>
         </is>
       </c>
     </row>
@@ -5124,12 +5124,12 @@
       </c>
       <c r="D176" s="3" t="inlineStr">
         <is>
-          <t>Iván Cepeda | Elecciones 2026 en VIVO: Apertura de mesas y reporte de orden público en Colombia</t>
+          <t>Clima en Cali: la predicción para este 21 de junio</t>
         </is>
       </c>
       <c r="E176" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/21/ivan-cepeda-elecciones-2026-en-vivo-apertura-de-mesas-y-reporte-de-orden-publico-en-colombia/</t>
+          <t>https://www.infobae.com/colombia/2026/06/21/clima-en-cali-la-prediccion-para-este-21-de-junio/</t>
         </is>
       </c>
     </row>
@@ -5151,12 +5151,12 @@
       </c>
       <c r="D177" s="6" t="inlineStr">
         <is>
-          <t>Abelardo de la Espriella | Elecciones 2026 en VIVO: Apertura de mesas y reporte de orden público en Colombia</t>
+          <t>Bogotá: el pronóstico del clima para este 21 de junio</t>
         </is>
       </c>
       <c r="E177" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/21/abelardo-de-la-espriella-elecciones-2026-en-vivo-apertura-de-mesas-y-reporte-de-orden-publico-en-colombia/</t>
+          <t>https://www.infobae.com/colombia/2026/06/21/bogota-el-pronostico-del-clima-para-este-21-de-junio/</t>
         </is>
       </c>
     </row>
@@ -5178,12 +5178,12 @@
       </c>
       <c r="D178" s="3" t="inlineStr">
         <is>
-          <t>Elecciones Presidenciales EN VIVO desde Barranquilla, hoy 21 de junio: siga el minuto a minuto de las votaciones electorales</t>
+          <t>Clima en Barranquilla: pronóstico de lluvias y ráfagas de viento</t>
         </is>
       </c>
       <c r="E178" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/21/elecciones-presidenciales-en-vivo-desde-barranquilla-hoy-21-de-junio-siga-el-minuto-a-minuto-de-las-votaciones-electorales/</t>
+          <t>https://www.infobae.com/colombia/2026/06/21/clima-en-barranquilla-pronostico-de-lluvias-y-rafagas-de-viento/</t>
         </is>
       </c>
     </row>
@@ -5205,12 +5205,12 @@
       </c>
       <c r="D179" s="6" t="inlineStr">
         <is>
-          <t>Elecciones Presidenciales EN VIVO desde Bogotá, hoy 21 de junio: siga el minuto a minuto de las votaciones</t>
+          <t>Las últimas previsiones para Cartagena de Indias: temperatura, lluvias y viento</t>
         </is>
       </c>
       <c r="E179" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/21/elecciones-presidenciales-en-vivo-desde-bogota-hoy-21-de-junio-siga-el-minuto-a-minuto-de-las-votaciones/</t>
+          <t>https://www.infobae.com/colombia/2026/06/21/las-ultimas-previsiones-para-cartagena-de-indias-temperatura-lluvias-y-viento/</t>
         </is>
       </c>
     </row>
@@ -5232,12 +5232,12 @@
       </c>
       <c r="D180" s="3" t="inlineStr">
         <is>
-          <t>Elecciones Presidenciales EN VIVO desde Antioquia, hoy 21 de junio: siga el minuto a minuto de las votaciones</t>
+          <t>Resultado Chontico Noche: números ganadores del último sorteo hoy, sábado 20 de junio de 2026</t>
         </is>
       </c>
       <c r="E180" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/21/elecciones-presidenciales-en-vivo-desde-antioquia-hoy-21-de-junio-siga-el-minuto-a-minuto-de-las-votaciones/</t>
+          <t>https://www.infobae.com/colombia/2026/06/21/resultado-chontico-noche-numeros-ganadores-del-ultimo-sorteo-hoy-sabado-20-de-junio-de-2026/</t>
         </is>
       </c>
     </row>
@@ -5259,12 +5259,12 @@
       </c>
       <c r="D181" s="6" t="inlineStr">
         <is>
-          <t>Qué se vota hoy en Colombia: claves para entender la segunda vuelta presidencial del 21 de junio de 2026</t>
+          <t>Resultado Lotería del Cauca hoy 20 de junio</t>
         </is>
       </c>
       <c r="E181" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/21/que-se-vota-hoy-en-colombia-claves-para-entender-la-segunda-vuelta-presidencial-del-21-de-junio-de-2026/</t>
+          <t>https://www.infobae.com/colombia/2026/06/21/resultado-loteria-del-cauca-hoy-20-de-junio/</t>
         </is>
       </c>
     </row>
@@ -5286,12 +5286,12 @@
       </c>
       <c r="D182" s="3" t="inlineStr">
         <is>
-          <t>Resultado Super Astro Luna HOY: número ganador del sábado 20 de junio</t>
+          <t>Iván Cepeda | Elecciones 2026 en VIVO: Apertura de mesas y reporte de orden público en Colombia</t>
         </is>
       </c>
       <c r="E182" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/21/resultado-super-astro-luna-hoy-numero-ganador-del-sabado-20-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/21/ivan-cepeda-elecciones-2026-en-vivo-apertura-de-mesas-y-reporte-de-orden-publico-en-colombia/</t>
         </is>
       </c>
     </row>
@@ -5313,12 +5313,12 @@
       </c>
       <c r="D183" s="6" t="inlineStr">
         <is>
-          <t>Resultado Sinuano Noche hoy 20 de junio</t>
+          <t>Abelardo de la Espriella | Elecciones 2026 en VIVO: Apertura de mesas y reporte de orden público en Colombia</t>
         </is>
       </c>
       <c r="E183" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/21/resultado-sinuano-noche-hoy-20-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/21/abelardo-de-la-espriella-elecciones-2026-en-vivo-apertura-de-mesas-y-reporte-de-orden-publico-en-colombia/</t>
         </is>
       </c>
     </row>
@@ -5340,12 +5340,12 @@
       </c>
       <c r="D184" s="3" t="inlineStr">
         <is>
-          <t>Costa de Marfil sonríe en el Mundial 2026 gracias a Ecuador y Curazao: estas son sus cuentas</t>
+          <t>Elecciones Presidenciales EN VIVO desde Barranquilla, hoy 21 de junio: siga el minuto a minuto de las votaciones electorales</t>
         </is>
       </c>
       <c r="E184" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/06/21/costa-de-marfil-sonrie-en-el-mundial-2026-gracias-a-ecuador-y-curazao-estas-son-sus-cuentas/</t>
+          <t>https://www.infobae.com/colombia/2026/06/21/elecciones-presidenciales-en-vivo-desde-barranquilla-hoy-21-de-junio-siga-el-minuto-a-minuto-de-las-votaciones-electorales/</t>
         </is>
       </c>
     </row>
@@ -5367,12 +5367,12 @@
       </c>
       <c r="D185" s="6" t="inlineStr">
         <is>
-          <t>Resultados de auditorías de Iidh descartan manipulación en la primera vuelta presidencial: “Sin ningún percance”</t>
+          <t>Elecciones Presidenciales EN VIVO desde Bogotá, hoy 21 de junio: siga el minuto a minuto de las votaciones</t>
         </is>
       </c>
       <c r="E185" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/21/resultados-de-auditorias-de-iidh-descartan-manipulacion-en-la-primera-vuelta-presidencial-sin-ningun-percance/</t>
+          <t>https://www.infobae.com/colombia/2026/06/21/elecciones-presidenciales-en-vivo-desde-bogota-hoy-21-de-junio-siga-el-minuto-a-minuto-de-las-votaciones/</t>
         </is>
       </c>
     </row>
@@ -5394,12 +5394,12 @@
       </c>
       <c r="D186" s="3" t="inlineStr">
         <is>
-          <t>Emerse Fae explicó la derrota de Costa de Marfil ante Alemania en el Mundial 2026: “La diferencia fue la experiencia”</t>
+          <t>Elecciones Presidenciales EN VIVO desde Antioquia, hoy 21 de junio: siga el minuto a minuto de las votaciones</t>
         </is>
       </c>
       <c r="E186" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/06/21/emerse-fae-explico-la-derrota-de-costa-de-marfil-ante-alemania-en-el-mundial-2026-la-diferencia-fue-la-experiencia/</t>
+          <t>https://www.infobae.com/colombia/2026/06/21/elecciones-presidenciales-en-vivo-desde-antioquia-hoy-21-de-junio-siga-el-minuto-a-minuto-de-las-votaciones/</t>
         </is>
       </c>
     </row>
@@ -5421,12 +5421,12 @@
       </c>
       <c r="D187" s="6" t="inlineStr">
         <is>
-          <t>Sancionan al Gimnasio Campestre Los Laureles, donde falleció Valeria Afanador: ordenaron la cancelación de la licencia de funcionamiento</t>
+          <t>Qué se vota hoy en Colombia: claves para entender la segunda vuelta presidencial del 21 de junio de 2026</t>
         </is>
       </c>
       <c r="E187" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/21/sancionan-al-gimnasio-campestre-los-laureles-donde-fallecio-valeria-afanador-ordenaron-la-cancelacion-de-la-licencia-de-funcionamiento/</t>
+          <t>https://www.infobae.com/colombia/2026/06/21/que-se-vota-hoy-en-colombia-claves-para-entender-la-segunda-vuelta-presidencial-del-21-de-junio-de-2026/</t>
         </is>
       </c>
     </row>
@@ -5448,12 +5448,12 @@
       </c>
       <c r="D188" s="3" t="inlineStr">
         <is>
-          <t>Gobernador del Quindío reaccionó a montaje hecho con IA en apoyo a un candidato presidencial: “Ya tengo definido mi voto”</t>
+          <t>Resultado Super Astro Luna HOY: número ganador del sábado 20 de junio</t>
         </is>
       </c>
       <c r="E188" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/21/gobernador-del-quindio-reacciono-a-montaje-hecho-con-ia-en-apoyo-a-un-candidato-presidencial-ya-tengo-definido-mi-voto/</t>
+          <t>https://www.infobae.com/colombia/2026/06/21/resultado-super-astro-luna-hoy-numero-ganador-del-sabado-20-de-junio/</t>
         </is>
       </c>
     </row>
@@ -5475,12 +5475,12 @@
       </c>
       <c r="D189" s="6" t="inlineStr">
         <is>
-          <t>Nelson Deossa tiene opciones de salir de Real Betis: lo buscaría un reconocido club de Brasil</t>
+          <t>Resultado Sinuano Noche hoy 20 de junio</t>
         </is>
       </c>
       <c r="E189" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/06/21/nelson-deossa-tiene-opciones-de-salir-de-real-betis-lo-buscaria-un-reconocido-club-de-brasil/</t>
+          <t>https://www.infobae.com/colombia/2026/06/21/resultado-sinuano-noche-hoy-20-de-junio/</t>
         </is>
       </c>
     </row>
@@ -5502,12 +5502,12 @@
       </c>
       <c r="D190" s="3" t="inlineStr">
         <is>
-          <t>Atlético Nacional fue sancionado por la Dimayor tras la final de la Liga BetPlay: duro castigo por desmanes</t>
+          <t>Costa de Marfil sonríe en el Mundial 2026 gracias a Ecuador y Curazao: estas son sus cuentas</t>
         </is>
       </c>
       <c r="E190" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/06/21/atletico-nacional-fue-sancionado-por-la-dimayor-tras-la-final-de-la-liga-betplay-duro-castigo-por-desmanes/</t>
+          <t>https://www.infobae.com/colombia/deportes/2026/06/21/costa-de-marfil-sonrie-en-el-mundial-2026-gracias-a-ecuador-y-curazao-estas-son-sus-cuentas/</t>
         </is>
       </c>
     </row>
@@ -5529,12 +5529,12 @@
       </c>
       <c r="D191" s="6" t="inlineStr">
         <is>
-          <t>Abelardo de la Espriella sumó otro apoyo, el expresidente de México Vicente Fox anunció su respaldo: el candidato le agradeció</t>
+          <t>Resultados de auditorías de Iidh descartan manipulación en la primera vuelta presidencial: “Sin ningún percance”</t>
         </is>
       </c>
       <c r="E191" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/21/abelardo-de-la-espriella-sumo-otro-apoyo-el-expresidente-de-mexico-vicente-fox-anuncio-su-respaldo-el-candidato-le-agradecio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/21/resultados-de-auditorias-de-iidh-descartan-manipulacion-en-la-primera-vuelta-presidencial-sin-ningun-percance/</t>
         </is>
       </c>
     </row>
@@ -5556,12 +5556,12 @@
       </c>
       <c r="D192" s="3" t="inlineStr">
         <is>
-          <t>Fabrizio Romano elogió a Luis Díaz tras su debut en el Mundial 2026: “No debemos subestimar lo especial que está siendo lo que hace por Colombia”</t>
+          <t>Emerse Fae explicó la derrota de Costa de Marfil ante Alemania en el Mundial 2026: “La diferencia fue la experiencia”</t>
         </is>
       </c>
       <c r="E192" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/06/21/fabrizio-romano-elogio-a-luis-diaz-tras-su-debut-en-el-mundial-2026-no-debemos-subestimar-lo-especial-que-esta-siendo-lo-que-hace-por-colombia/</t>
+          <t>https://www.infobae.com/colombia/deportes/2026/06/21/emerse-fae-explico-la-derrota-de-costa-de-marfil-ante-alemania-en-el-mundial-2026-la-diferencia-fue-la-experiencia/</t>
         </is>
       </c>
     </row>
@@ -5583,12 +5583,12 @@
       </c>
       <c r="D193" s="6" t="inlineStr">
         <is>
-          <t>Aproveche su certificado de votación hay descuentos y promociones: estas son las marcas que se han sumado a la tendencia</t>
+          <t>Sancionan al Gimnasio Campestre Los Laureles, donde falleció Valeria Afanador: ordenaron la cancelación de la licencia de funcionamiento</t>
         </is>
       </c>
       <c r="E193" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/21/aproveche-su-certificado-de-votacion-hay-descuentos-y-promociones-estas-son-las-marcas-que-se-han-sumado-a-la-tendencia/</t>
+          <t>https://www.infobae.com/colombia/2026/06/21/sancionan-al-gimnasio-campestre-los-laureles-donde-fallecio-valeria-afanador-ordenaron-la-cancelacion-de-la-licencia-de-funcionamiento/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 Noticias actualizadas 23/06/2026 07:50
</commit_message>
<xml_diff>
--- a/docs/ultimahora.xlsx
+++ b/docs/ultimahora.xlsx
@@ -515,7 +515,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 11:55 p. m.</t>
+          <t>23/06/2026 01:49 a. m.</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -530,19 +530,19 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Día trece del Mundial Estados Unidos, Canadá y México 2026: ¿qué partidos se juegan este martes 23 de junio? Canal y hora para ver en vivo</t>
+          <t>Colombia, por la clasificación contra Congo en el Mundial 2026 | Previo del partido, en 'Contraataque'</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/dia-trece-del-mundial-estados-unidos-canada-y-mexico-2026-que-partidos-se-juegan-este-martes-23-de-junio-canal-y-hora-para-ver-en-vivo-3566279</t>
+          <t>https://www.eltiempo.com/podcast/contraataque/colombia-por-la-clasificacion-contra-congo-en-el-mundial-2026-previo-del-partido-en-contraataque-3566301</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 11:14 p. m.</t>
+          <t>23/06/2026 01:43 a. m.</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -557,19 +557,19 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>Así funciona el 'cartel del arroz' en Venezuela, el entramado corporativo que usa influencias y privilegios arancelarios para asfixiar a campesinos</t>
+          <t>La selección de Argelia logró remontar el marcador ante Jordania y ganó 2-1 en San Francisco; el equipo jordano quedó eliminado del Mundial 2026</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/venezuela/asi-funciona-el-cartel-del-arroz-en-venezuela-el-entramado-corporativo-que-usa-influencias-y-privilegios-arancelarios-para-asfixiar-a-campesinos-3566183</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/la-seleccion-de-argelia-logro-remontar-el-marcador-ante-jordania-y-gano-2-1-en-san-francisco-el-equipo-jordano-quedo-eliminado-del-mundial-3566300</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 11:01 p. m.</t>
+          <t>22/06/2026 11:55 p. m.</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -584,19 +584,19 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Abogado del Gimnasio Campestre Los Laureles se pronunció tras la sanción de la Gobernación de Cundinamarca por la muerte de Valeria Afanador en Cajicá</t>
+          <t>Día trece del Mundial Estados Unidos, Canadá y México 2026: ¿qué partidos se juegan este martes 23 de junio? Canal y hora para ver en vivo</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/bogota/abogado-del-gimnasio-campestre-los-laureles-se-pronuncio-tras-la-sancion-de-la-gobernacion-de-cundinamarca-por-la-muerte-de-valeria-afanador-en-cajica-3566298</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/dia-trece-del-mundial-estados-unidos-canada-y-mexico-2026-que-partidos-se-juegan-este-martes-23-de-junio-canal-y-hora-para-ver-en-vivo-3566279</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 11:00 p. m.</t>
+          <t>22/06/2026 11:14 p. m.</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -611,19 +611,19 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Administración de lujoso edificio del norte de Bogotá se pronunció tras hallazgo de mujer muerta dentro de maleta en un apartamento: 'Manejo del caso'</t>
+          <t>Así funciona el 'cartel del arroz' en Venezuela, el entramado corporativo que usa influencias y privilegios arancelarios para asfixiar a campesinos</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/bogota/administracion-de-lujoso-edificio-del-norte-de-bogota-se-pronuncio-tras-hallazgo-de-mujer-muerta-dentro-de-maleta-en-un-apartamento-manejo-del-caso-3566299</t>
+          <t>https://www.eltiempo.com/mundo/venezuela/asi-funciona-el-cartel-del-arroz-en-venezuela-el-entramado-corporativo-que-usa-influencias-y-privilegios-arancelarios-para-asfixiar-a-campesinos-3566183</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 10:58 p. m.</t>
+          <t>22/06/2026 11:01 p. m.</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -638,19 +638,19 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Colombia desafía a Congo: ¡a clasificar sin demoras!</t>
+          <t>Abogado del Gimnasio Campestre Los Laureles se pronunció tras la sanción de la Gobernación de Cundinamarca por la muerte de Valeria Afanador en Cajicá</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/colombia-desafia-a-congo-a-clasificar-sin-demoras-3566293</t>
+          <t>https://www.eltiempo.com/bogota/abogado-del-gimnasio-campestre-los-laureles-se-pronuncio-tras-la-sancion-de-la-gobernacion-de-cundinamarca-por-la-muerte-de-valeria-afanador-en-cajica-3566298</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 10:45 p. m.</t>
+          <t>22/06/2026 11:00 p. m.</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -665,19 +665,19 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>República del Congo advierte a Colombia: ‘Luchamos por la clasificación’</t>
+          <t>Administración de lujoso edificio del norte de Bogotá se pronunció tras hallazgo de mujer muerta dentro de maleta en un apartamento: 'Manejo del caso'</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/republica-del-congo-advierte-a-colombia-luchamos-por-la-clasificacion-3566297</t>
+          <t>https://www.eltiempo.com/bogota/administracion-de-lujoso-edificio-del-norte-de-bogota-se-pronuncio-tras-hallazgo-de-mujer-muerta-dentro-de-maleta-en-un-apartamento-manejo-del-caso-3566299</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 10:37 p. m.</t>
+          <t>22/06/2026 10:58 p. m.</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -692,19 +692,19 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Elecciones en Perú 2026: Roberto Sánchez presentó solicitud que podría cambiar el rumbo de la segunda vuelta y le permitiría superar a Keiko Fujimori</t>
+          <t>Colombia desafía a Congo: ¡a clasificar sin demoras!</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/latinoamerica/elecciones-en-peru-2026-roberto-sanchez-presento-solicitud-que-podria-cambiar-el-rumbo-de-la-segunda-vuelta-y-le-permitiria-superar-a-keiko-fujimori-3566296</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/colombia-desafia-a-congo-a-clasificar-sin-demoras-3566293</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 10:37 p. m.</t>
+          <t>22/06/2026 10:45 p. m.</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -719,19 +719,19 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Esta es la razón de la suspensión del partido de Francia vs. Irak en el Mundial 2026: así funciona el protocolo de tormentas en Estados Unidos</t>
+          <t>República del Congo advierte a Colombia: ‘Luchamos por la clasificación’</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/esta-es-la-razon-de-la-suspension-del-partido-de-francia-vs-irak-en-el-mundial-2026-asi-funciona-el-protocolo-de-tormentas-en-estados-unidos-3566289</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/republica-del-congo-advierte-a-colombia-luchamos-por-la-clasificacion-3566297</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 10:33 p. m.</t>
+          <t>22/06/2026 10:37 p. m.</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -746,19 +746,19 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Tormenta altera la preparación de Colombia antes del decisivo duelo contra RD Congo</t>
+          <t>Elecciones en Perú 2026: Roberto Sánchez presentó solicitud que podría cambiar el rumbo de la segunda vuelta y le permitiría superar a Keiko Fujimori</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/tormenta-altera-la-preparacion-de-colombia-antes-del-decisivo-duelo-contra-rd-congo-3566294</t>
+          <t>https://www.eltiempo.com/mundo/latinoamerica/elecciones-en-peru-2026-roberto-sanchez-presento-solicitud-que-podria-cambiar-el-rumbo-de-la-segunda-vuelta-y-le-permitiria-superar-a-keiko-fujimori-3566296</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 10:30 p. m.</t>
+          <t>22/06/2026 10:37 p. m.</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -773,19 +773,19 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Iván Cepeda ganó en 102 de los 139 municipios en riesgo extremo electoral en segunda vuelta: en 15 lo hizo con más del 90 por ciento de los votos</t>
+          <t>Esta es la razón de la suspensión del partido de Francia vs. Irak en el Mundial 2026: así funciona el protocolo de tormentas en Estados Unidos</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/ivan-cepeda-gano-en-102-de-los-139-municipios-en-riesgo-extremo-electoral-en-segunda-vuelta-en-15-lo-hizo-con-mas-del-90-por-ciento-de-los-votos-3566209</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/esta-es-la-razon-de-la-suspension-del-partido-de-francia-vs-irak-en-el-mundial-2026-asi-funciona-el-protocolo-de-tormentas-en-estados-unidos-3566289</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 10:30 p. m.</t>
+          <t>22/06/2026 10:33 p. m.</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -800,19 +800,19 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Andy Burnham, el favorito para suceder a Keir Starmer como primer ministro: así busca el Partido Laborista mantener el poder en Reino Unido</t>
+          <t>Tormenta altera la preparación de Colombia antes del decisivo duelo contra RD Congo</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/europa/andy-burnham-el-favorito-para-suceder-a-keir-starmer-como-primer-ministro-asi-busca-el-partido-laborista-mantener-el-poder-en-reino-unido-3566208</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/tormenta-altera-la-preparacion-de-colombia-antes-del-decisivo-duelo-contra-rd-congo-3566294</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 10:28 p. m.</t>
+          <t>22/06/2026 10:30 p. m.</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -827,19 +827,19 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Selección Colombia: con prisa, pero con calma (opinión)</t>
+          <t>Iván Cepeda ganó en 102 de los 139 municipios en riesgo extremo electoral en segunda vuelta: en 15 lo hizo con más del 90 por ciento de los votos</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/seleccion-colombia-con-prisa-pero-con-calma-opinion-3566295</t>
+          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/ivan-cepeda-gano-en-102-de-los-139-municipios-en-riesgo-extremo-electoral-en-segunda-vuelta-en-15-lo-hizo-con-mas-del-90-por-ciento-de-los-votos-3566209</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 10:20 p. m.</t>
+          <t>22/06/2026 10:30 p. m.</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -854,19 +854,19 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Tadej Pogacar: este es el motivo por el que podría cambiar de manera drástica su asalto al Tour de Francia</t>
+          <t>Andy Burnham, el favorito para suceder a Keir Starmer como primer ministro: así busca el Partido Laborista mantener el poder en Reino Unido</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/ciclismo/tadej-pogacar-este-es-el-motivo-por-el-que-podria-cambiar-de-manera-drastica-su-asalto-al-tour-de-francia-3566265</t>
+          <t>https://www.eltiempo.com/mundo/europa/andy-burnham-el-favorito-para-suceder-a-keir-starmer-como-primer-ministro-asi-busca-el-partido-laborista-mantener-el-poder-en-reino-unido-3566208</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 10:08 p. m.</t>
+          <t>22/06/2026 10:28 p. m.</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -881,19 +881,19 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Este es el escolta del líder de campaña de Abelardo de la Espriella en Medellín al que se le incautó un arma sin papeles durante los escrutinios</t>
+          <t>Selección Colombia: con prisa, pero con calma (opinión)</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/medellin/este-es-el-escolta-del-lider-de-campana-de-abelardo-de-la-espriella-en-medellin-al-que-se-le-incauto-un-arma-sin-papeles-durante-los-escrutinios-3566285</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/seleccion-colombia-con-prisa-pero-con-calma-opinion-3566295</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 09:50 p. m.</t>
+          <t>22/06/2026 10:20 p. m.</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -908,19 +908,19 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Antes del primer día de clases</t>
+          <t>Tadej Pogacar: este es el motivo por el que podría cambiar de manera drástica su asalto al Tour de Francia</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/columnistas/antes-del-primer-dia-de-clases-3566292</t>
+          <t>https://www.eltiempo.com/deportes/ciclismo/tadej-pogacar-este-es-el-motivo-por-el-que-podria-cambiar-de-manera-drastica-su-asalto-al-tour-de-francia-3566265</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 09:43 p. m.</t>
+          <t>22/06/2026 10:08 p. m.</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -935,19 +935,19 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>La insólita incertidumbre que agobia a la parafiscalidad cafetera</t>
+          <t>Este es el escolta del líder de campaña de Abelardo de la Espriella en Medellín al que se le incautó un arma sin papeles durante los escrutinios</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/columnistas/la-insolita-incertidumbre-que-agobia-a-la-parafiscalidad-cafetera-3566291</t>
+          <t>https://www.eltiempo.com/colombia/medellin/este-es-el-escolta-del-lider-de-campana-de-abelardo-de-la-espriella-en-medellin-al-que-se-le-incauto-un-arma-sin-papeles-durante-los-escrutinios-3566285</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 09:40 p. m.</t>
+          <t>22/06/2026 09:50 p. m.</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -962,19 +962,19 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Familia campesina recupera tierras despojadas por alias ‘Terror’, el heredero de los paramilitares del Magdalena Medio</t>
+          <t>Antes del primer día de clases</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/justicia/paz-y-derechos-humanos/familia-campesina-recupera-tierras-despojadas-por-alias-terror-el-heredero-de-los-paramilitares-del-magdalena-medio-3566287</t>
+          <t>https://www.eltiempo.com/opinion/columnistas/antes-del-primer-dia-de-clases-3566292</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 09:35 p. m.</t>
+          <t>22/06/2026 09:43 p. m.</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -989,19 +989,19 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Ganó la democracia</t>
+          <t>La insólita incertidumbre que agobia a la parafiscalidad cafetera</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/cartas/gano-la-democracia-3566290</t>
+          <t>https://www.eltiempo.com/opinion/columnistas/la-insolita-incertidumbre-que-agobia-a-la-parafiscalidad-cafetera-3566291</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 09:27 p. m.</t>
+          <t>22/06/2026 09:40 p. m.</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1016,19 +1016,19 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>¿De regreso al pasado?</t>
+          <t>Familia campesina recupera tierras despojadas por alias ‘Terror’, el heredero de los paramilitares del Magdalena Medio</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/columnistas/de-regreso-al-pasado-3566286</t>
+          <t>https://www.eltiempo.com/justicia/paz-y-derechos-humanos/familia-campesina-recupera-tierras-despojadas-por-alias-terror-el-heredero-de-los-paramilitares-del-magdalena-medio-3566287</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 09:23 p. m.</t>
+          <t>22/06/2026 09:35 p. m.</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
@@ -1043,12 +1043,12 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Aceptan acción de tutela en contra de James Rodríguez, Luis Díaz y la Federación de Fútbol por ‘traición a la patria’: los detalles</t>
+          <t>Ganó la democracia</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/aceptan-accion-de-tutela-en-contra-de-james-rodriguez-luis-diaz-y-la-federacion-de-futbol-por-traicion-a-la-patria-los-detalles-3566284</t>
+          <t>https://www.eltiempo.com/opinion/cartas/gano-la-democracia-3566290</t>
         </is>
       </c>
     </row>
@@ -2123,7 +2123,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 01:12 a. m.</t>
+          <t>23/06/2026 02:39 a. m.</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -2133,24 +2133,24 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Resultados loterías de Cundinamarca, Tolima, Baloto, MiLoto y ColorLoto del 22 de junio de 2026</t>
+          <t>La periodista Anna Bosch anuncia su jubilación y se despide emocionada de TVE: “Me han dejado sin habla”</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/economia/juegos-de-azar/resultados-loterias-de-cundinamarca-tolima-baloto-miloto-y-colorloto-del-22-de-junio-de-2026-so35</t>
+          <t>https://elpais.com/television/2026-06-23/la-periodista-anna-bosch-anuncia-su-jubilacion-y-se-despide-emocionada-de-tve-me-han-dejado-sin-habla.html</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>23/06/2026 12:53 a. m.</t>
+          <t>23/06/2026 02:37 a. m.</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
@@ -2160,24 +2160,24 @@
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
-          <t>ColorLoto, resultado del último sorteo lunes 22 de junio de 2026</t>
+          <t>El Gobierno aprobará la mayor inyección económica en dependencia hasta superar los 7.000 millones en 2027</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/economia/juegos-de-azar/colorloto-resultado-del-ultimo-sorteo-lunes-22-de-junio-de-2026-so35</t>
+          <t>https://elpais.com/sociedad/2026-06-23/el-gobierno-aprobara-la-mayor-inyeccion-economica-en-dependencia-hasta-superar-los-7000-millones-en-2027.html</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 12:07 a. m.</t>
+          <t>23/06/2026 02:32 a. m.</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -2187,24 +2187,24 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Aceptan tutela contra Luis Díaz y James Rodríguez por "traición a la patria"</t>
+          <t>Resumen y últimas noticias de la Copa Mundial de fútbol</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/judicial/aceptan-tutela-contra-luis-diaz-y-james-rodriguez-por-traicion-a-la-patria-so35</t>
+          <t>https://elpais.com/deportes/mundial-futbol/2026-06-23/resumen-y-ultimas-noticias-de-la-copa-mundial-de-futbol.html</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 11:38 p. m.</t>
+          <t>23/06/2026 01:39 a. m.</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
@@ -2214,24 +2214,24 @@
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>Predicción Colombia vs. República del Congo: así van las apuestas de este duelo</t>
+          <t>La italiana Camila Angelucci gana ‘Masterchef’ 14: “Tu plato es un triple salto mortal con éxito”</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/deportes/futbol/copa-mundial-de-la-fifa-2026/prediccion-colombia-vs-republica-del-congo-asi-van-las-apuestas-de-este-duelo-so35</t>
+          <t>https://elpais.com/television/2026-06-23/la-italiana-camila-angelucci-gana-masterchef-14-tu-plato-es-un-triple-salto-mortal-con-exito.html</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 11:18 p. m.</t>
+          <t>23/06/2026 01:35 a. m.</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -2241,24 +2241,24 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Trump le envía mensaje a De La Espriella: afirma que será un "gran presidente"</t>
+          <t>¿Quiénes serán los rivales de España en dieciseisavos? Así es su camino a la final</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion/trump-le-envia-mensaje-a-de-la-espriella-afirma-que-sera-un-gran-presidente-cb20</t>
+          <t>https://elpais.com/deportes/mundial-futbol/2026-06-23/quienes-seran-los-rivales-de-espana-en-dieciseisavos-asi-es-su-camino-a-la-final.html</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 11:09 p. m.</t>
+          <t>23/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr">
@@ -2268,24 +2268,24 @@
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>MiLoto, resultado del último sorteo hoy lunes 22 de junio de 2026</t>
+          <t>He probado durante una semana las Skechers que arrasan en Amazon Prime Day: cómodas, ligeras y ahora en oferta</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/economia/juegos-de-azar/miloto-resultado-del-ultimo-sorteo-hoy-lunes-22-de-junio-de-2026-so35</t>
+          <t>https://elpais.com/hemeroteca/2026-06-23/</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 11:06 p. m.</t>
+          <t>23/06/2026 12:33 a. m.</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -2295,24 +2295,24 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>Tras doblete contra Irak, Mbappé le envía mensaje a Messi: "No me fijo en lo que hace"</t>
+          <t>Última hora de la guerra de Estados Unidos e Israel contra Irán, en directo | Irán dice que las negociaciones técnicas con EE UU han concluido y que pasan a la siguiente fase</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/deportes/futbol/copa-mundial-de-la-fifa-2026/tras-doblete-contra-irak-mbappe-le-envia-mensaje-a-messi-no-me-fijo-en-lo-que-hace-cb20</t>
+          <t>https://elpais.com/internacional/2026-06-23/ultima-hora-de-la-guerra-de-estados-unidos-e-israel-contra-iran-en-directo.html</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 11:06 p. m.</t>
+          <t>23/06/2026 12:17 a. m.</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
@@ -2322,24 +2322,24 @@
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>Baloto y Revancha, resultado del útimo sorteo hoy lunes 22 de junio de 2026</t>
+          <t>“Vándalos” y amenazas de hasta 10 años de cárcel: Trump desvía la culpa por el fracaso de la piscina reflectante del Monumento a Lincoln</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/economia/juegos-de-azar/baloto-y-revancha-resultado-del-utimo-sorteo-hoy-lunes-22-de-junio-de-2026-so35</t>
+          <t>https://elpais.com/us/2026-06-24/vandalos-y-amenazas-de-hasta-10-anos-de-carcel-trump-desvia-la-culpa-por-el-fracaso-de-la-piscina-reflectante-del-monumento-a-lincoln.html</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 11:03 p. m.</t>
+          <t>22/06/2026 11:50 p. m.</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -2349,24 +2349,24 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>Martha Peralta recobró la libertad tras terminar su indagatoria por caso UNGRD</t>
+          <t>Las mejores imágenes de la Copa del Mundo de Fútbol | Imágenes del 22 de junio</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/judicial/martha-peralta-recobro-la-libertad-tras-terminar-su-indagatoria-por-caso-ungrd-rg10</t>
+          <t>https://elpais.com/deportes/mundial-futbol/2026-06-23/las-mejores-imagenes-de-la-copa-del-mundo-de-futbol.html</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 10:44 p. m.</t>
+          <t>22/06/2026 11:17 p. m.</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr">
@@ -2376,24 +2376,24 @@
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D71" s="6" t="inlineStr">
         <is>
-          <t>El Pentágono de EEUU propone a De la Espriella reforzar la alianza contra el narcotráfico</t>
+          <t>Los sueños rotos de Guillermo y Zafar: de huir de la pesadilla de Trump a encontrar su muerte en México</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/nacion/el-pentagono-de-eeuu-propone-a-de-la-espriella-reforzar-la-alianza-contra-el-narcotrafico-cb20</t>
+          <t>https://elpais.com/mexico/2026-06-23/los-suenos-rotos-de-guillermo-y-zafar-de-huir-de-la-pesadilla-de-trump-a-encontrar-su-muerte-en-mexico.html</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 10:04 p. m.</t>
+          <t>22/06/2026 11:10 p. m.</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -2403,24 +2403,24 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>Argentina clasifica a dieciseisavos de final: 22 junio 2026-Blog Deportivo, programa completo</t>
+          <t>México y Colombia le dan la bienvenida a Lumumba, el hincha más político</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/blog-deportivo/argentina-clasifica-a-dieciseisavos-de-final-22-junio-2026-blog-deportivo-programa-completo-pr30</t>
+          <t>https://elpais.com/mexico/2026-06-23/mexico-y-colombia-le-dan-la-bienvenida-a-lumumba-el-hincha-mas-politico.html</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 09:51 p. m.</t>
+          <t>22/06/2026 11:04 p. m.</t>
         </is>
       </c>
       <c r="B73" s="5" t="inlineStr">
@@ -2430,24 +2430,24 @@
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D73" s="6" t="inlineStr">
         <is>
-          <t>Lotería del Tolima, resultado del último sorteo hoy lunes 22 de junio de 2026</t>
+          <t>Joyas por 18 millones de pesos, siete vehículos de lujo, 10 casas y un edificio: Gertz Manero transparenta por primera vez su riqueza</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/economia/juegos-de-azar/loteria-del-tolima-resultado-del-ultimo-sorteo-hoy-lunes-22-de-junio-de-2026-so35</t>
+          <t>https://elpais.com/mexico/2026-06-23/joyas-por-18-millones-de-pesos-siete-vehiculos-de-lujo-10-casas-y-un-edificio-gertz-manero-transparenta-por-primera-vez-su-riqueza.html</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 01:00 a. m.</t>
+          <t>22/06/2026 11:00 p. m.</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -2457,24 +2457,24 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>El ‘memorando de entendimiento’ entre Irán y E.E.U.U.</t>
+          <t>Colombia se divide en las urnas y se reencuentra en la Constitución</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/23/el-memorando-de-entendimiento-entre-iran-y-eeuu/</t>
+          <t>https://elpais.com/america-colombia/elecciones-presidenciales/2026-06-23/colombia-se-divide-en-las-urnas-y-se-reencuentra-en-la-constitucion.html</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>23/06/2026 01:00 a. m.</t>
+          <t>22/06/2026 11:00 p. m.</t>
         </is>
       </c>
       <c r="B75" s="5" t="inlineStr">
@@ -2484,24 +2484,24 @@
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr">
         <is>
-          <t>Columnistas</t>
+          <t>El idioma nacional</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/</t>
+          <t>https://elpais.com/america/iberoamerica-democracia/2026-06-23/el-idioma-nacional.html</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 01:00 a. m.</t>
+          <t>22/06/2026 11:00 p. m.</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -2511,24 +2511,24 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>Un cielo nublado</t>
+          <t>El dibujante boliviano Al-Azar interpela al poder a través de la caricatura política</t>
         </is>
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/23/un-cielo-nublado/</t>
+          <t>https://elpais.com/america-futura/2026-06-23/el-dibujante-boliviano-al-azar-interpela-al-poder-a-traves-de-la-caricatura-politica.html</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>23/06/2026 01:00 a. m.</t>
+          <t>22/06/2026 11:00 p. m.</t>
         </is>
       </c>
       <c r="B77" s="5" t="inlineStr">
@@ -2538,24 +2538,24 @@
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D77" s="6" t="inlineStr">
         <is>
-          <t>Cambio de chip</t>
+          <t>El precio de investigar al Gobierno en Ecuador alcanza a la familia de un periodista</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/caricaturas/2026/06/23/cambio-de-chip/</t>
+          <t>https://elpais.com/america/2026-06-23/el-precio-de-investigar-al-gobierno-en-ecuador-alcanza-a-la-familia-de-un-periodista.html</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 01:00 a. m.</t>
+          <t>22/06/2026 11:00 p. m.</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -2565,24 +2565,24 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>Caricaturas</t>
+          <t>Sin cheque en blanco: el reto de Abelardo de la Espriella de gobernar con medio país en contra</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/caricaturas/</t>
+          <t>https://elpais.com/america-colombia/elecciones-presidenciales/2026-06-23/sin-cheque-en-blanco-el-reto-de-abelardo-de-la-espriella-de-gobernar-con-medio-pais-en-contra.html</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>23/06/2026 01:00 a. m.</t>
+          <t>22/06/2026 10:45 p. m.</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
@@ -2592,24 +2592,24 @@
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
         <is>
-          <t>Ideas conservadoras en Palacio</t>
+          <t>Las promesas incumplidas del Brexit: por qué el Reino Unido está peor que antes de salir de la UE</t>
         </is>
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/23/ideas-conservadoras-en-palacio/</t>
+          <t>https://elpais.com/internacional/2026-06-23/las-promesas-incumplidas-del-brexit-por-que-el-reino-unido-esta-peor-que-antes-de-salir-de-la-ue.html</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 10:59 p. m.</t>
+          <t>22/06/2026 10:45 p. m.</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -2619,24 +2619,24 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>¿Traición a la patria? La insólita “tutela” contra James Rodríguez y Luis Díaz en pleno Mundial</t>
+          <t>Estados Unidos versus Irán, la guerra de fuerzas desiguales que ningún bando pudo ganar</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/deportes/mundial-de-futbol/2026/06/22/traicion-a-la-patria-la-insolita-tutela-contra-james-rodriguez-y-luis-diaz-en-pleno-mundial/</t>
+          <t>https://elpais.com/internacional/2026-06-23/estados-unidos-versus-iran-la-guerra-de-fuerzas-desiguales-que-ningun-bando-pudo-ganar.html</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 10:59 p. m.</t>
+          <t>22/06/2026 10:45 p. m.</t>
         </is>
       </c>
       <c r="B81" s="5" t="inlineStr">
@@ -2646,24 +2646,24 @@
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D81" s="6" t="inlineStr">
         <is>
-          <t>Mundial de Fútbol</t>
+          <t>Las nuevas viviendas en España apenas cubrieron el 40% de los hogares que se constituyeron el año pasado</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/deportes/mundial-de-futbol/</t>
+          <t>https://elpais.com/economia/vivienda/2026-06-23/las-nuevas-viviendas-en-espana-apenas-cubrieron-el-40-de-los-hogares-que-se-constituyeron-el-ano-pasado.html</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 10:43 p. m.</t>
+          <t>22/06/2026 10:30 p. m.</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -2673,24 +2673,24 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>Gobierno inicia la liquidación del Ministerio de la Igualdad en medio de protestas laborales</t>
+          <t>Recorrido visual por la sentencia del Supremo que condena a Ábalos, Koldo y Aldama</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/22/gobierno-inicia-la-liquidacion-del-ministerio-de-la-igualdad-en-medio-de-protestas-laborales/</t>
+          <t>https://elpais.com/espana/2026-06-23/recorrido-visual-por-la-sentencia-del-supremo-que-condena-a-abalos-koldo-y-aldama.html</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 10:43 p. m.</t>
+          <t>22/06/2026 10:30 p. m.</t>
         </is>
       </c>
       <c r="B83" s="5" t="inlineStr">
@@ -2700,24 +2700,24 @@
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D83" s="6" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Ayuso multa con hasta 13.000 euros a pequeños comercios gallegos por incumplir la normativa de venta ‘online’</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/</t>
+          <t>https://elpais.com/espana/galicia/2026-06-23/ayuso-multa-con-hasta-13000-euros-a-pequenos-comercios-gallegos-por-incumplir-la-normativa-de-venta-online.html</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 10:39 p. m.</t>
+          <t>22/06/2026 10:30 p. m.</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -2727,24 +2727,24 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>Voto en el exterior, clave para victoria de Abelardo De La Espriella: así quedaron los resultados</t>
+          <t>Ian Gibson: “Un Gobierno que sacó a Franco del Valle de los Caídos haría muy bien en seguir buscando el cadáver de Lorca”</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/22/voto-en-el-exterior-fue-clave-para-la-victoria-de-abelardo-de-la-espriella-asi-quedaron-los-resultados/</t>
+          <t>https://elpais.com/cultura/2026-06-23/ian-gibson-un-gobierno-que-saco-a-franco-del-valle-de-los-caidos-haria-muy-bien-en-seguir-buscando-el-cadaver-de-lorca.html</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 07:51 p. m.</t>
+          <t>22/06/2026 10:30 p. m.</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr">
@@ -2754,24 +2754,24 @@
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D85" s="6" t="inlineStr">
         <is>
-          <t>Martha Peralta recupera su libertad tras declarar ante la Corte por investigación de contratos en la Ungrd</t>
+          <t>Cómo Ikea se metió en ocho de cada diez hogares españoles: 30 años del desembarco del gigante sueco</t>
         </is>
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/22/martha-peralta-recupera-su-libertad-tras-declarar-ante-la-corte-por-investigacion-de-contratos-en-la-ungrd/</t>
+          <t>https://elpais.com/icon-design/2026-06-23/como-ikea-se-metio-en-ocho-de-cada-diez-hogares-espanoles-30-anos-del-desembarco-del-gigante-sueco.html</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 07:00 p. m.</t>
+          <t>22/06/2026 08:37 p. m.</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -2781,24 +2781,24 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>Simpatizantes de Iván Cepeda marchan en Bogotá mientras avanza el escrutinio electoral</t>
+          <t>Francia brilla con un doblete de Mbappé en un partido pasado por agua</t>
         </is>
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/22/simpatizantes-de-ivan-cepeda-marchan-en-bogota-mientras-avanza-el-escrutinio-electoral/</t>
+          <t>https://elpais.com/deportes/mundial-futbol/2026-06-23/una-francia-pasada-por-agua-brilla-con-un-doblete-de-mbappe.html</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 04:40 p. m.</t>
+          <t>22/06/2026 04:26 p. m.</t>
         </is>
       </c>
       <c r="B87" s="5" t="inlineStr">
@@ -2808,24 +2808,24 @@
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D87" s="6" t="inlineStr">
         <is>
-          <t>Hallan a una mujer muerta dentro de una maleta en Bogotá: investigan a un extranjero que estuvo con ella</t>
+          <t>Julián Alvarez pide salir del Atlético y el club rojiblanco se plantea denunciar al Barça ante la FIFA: “No puedo esconderme, lo mejor es una transferencia, quiero cumplir mi sueño”</t>
         </is>
       </c>
       <c r="E87" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/22/hallan-a-una-mujer-muerta-dentro-de-una-maleta-en-bogota-investigan-a-un-extranjero-que-estuvo-con-ella/</t>
+          <t>https://elpais.com/deportes/mundial-futbol/2026-06-22/julian-alvarez-pide-salir-del-atletico-no-puedo-esconderme-lo-mejor-es-una-transferencia-quiero-cumplir-mi-sueno.html</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 04:11 p. m.</t>
+          <t>22/06/2026 03:09 p. m.</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -2835,24 +2835,24 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>Isabella Echeverri: de defender el arco a contar las historias de la Selección Colombia</t>
+          <t>El viejo Messi emociona al mundo: otro doblete lo convierte en el máximo goleador de la historia del torneo</t>
         </is>
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/22/isabella-echeverri-de-defender-el-arco-a-contar-las-historias-de-la-seleccion-colombia/</t>
+          <t>https://elpais.com/deportes/mundial-futbol/2026-06-22/el-viejo-messi-conmueve-al-mundo.html</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 03:51 p. m.</t>
+          <t>22/06/2026 09:27 a. m.</t>
         </is>
       </c>
       <c r="B89" s="5" t="inlineStr">
@@ -2862,26 +2862,22 @@
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D89" s="6" t="inlineStr">
         <is>
-          <t>Gustavo Petro celebra posible salida de la lista Clinton y agita la polémica</t>
+          <t>Bear, el hijo de 9 años de Liam Payne, ya puede beneficiarse de los 25 millones de herencia del fallecido cantante</t>
         </is>
       </c>
       <c r="E89" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/22/petro-celebra-posible-salida-de-la-lista-ofac-ya-no-se-enfrentan-a-guerrilleros-sino-a-pueblos/</t>
+          <t>https://elpais.com/gente/2026-06-22/bear-el-hijo-de-9-anos-de-liam-payne-ya-puede-beneficiarse-de-los-25-millones-de-herencia-del-fallecido-cantante.html</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="inlineStr">
-        <is>
-          <t>22/06/2026 03:38 p. m.</t>
-        </is>
-      </c>
+      <c r="A90" s="2" t="inlineStr"/>
       <c r="B90" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2889,26 +2885,22 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>Cepeda pide diálogo y responde a De La Espriella tras su discurso: “No nos asustan sus rugidos”</t>
+          <t>Predicciones</t>
         </is>
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/22/cepeda-pide-dialogo-y-responde-a-de-la-espriella-tras-su-discurso-no-nos-asustan-sus-rugidos/</t>
+          <t>https://elpais.com/deportes/mundial-futbol/2026-06-11/quien-ganara-el-mundial-asi-arrancan-nuestras-predicciones.html</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="5" t="inlineStr">
-        <is>
-          <t>22/06/2026 03:00 p. m.</t>
-        </is>
-      </c>
+      <c r="A91" s="5" t="inlineStr"/>
       <c r="B91" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -2916,24 +2908,24 @@
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>Vanguardia</t>
+          <t>El País</t>
         </is>
       </c>
       <c r="D91" s="6" t="inlineStr">
         <is>
-          <t>Los nombres que suenan para el gabinete de De La Espriella: entre figuras políticas y apuestas técnicas</t>
+          <t>Selecciones</t>
         </is>
       </c>
       <c r="E91" s="7" t="inlineStr">
         <is>
-          <t>https://www.vanguardia.com/colombia/2026/06/22/los-nombres-que-empiezan-a-sonar-para-el-gabinete-de-abelardo-de-la-espriella-entre-figuras-politicas-y-apuestas-tecnicas/</t>
+          <t>https://elpais.com/deportes/mundial-futbol/2026-06-05/todas-las-selecciones-del-mundial-de-estados-unidos-canada-y-mexico.html</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 01:00 a. m.</t>
+          <t>23/06/2026 01:12 a. m.</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -2943,24 +2935,24 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>He probado durante una semana las Skechers que arrasan en Amazon Prime Day: cómodas, ligeras y ahora en oferta</t>
+          <t>Resultados loterías de Cundinamarca, Tolima, Baloto, MiLoto y ColorLoto del 22 de junio de 2026</t>
         </is>
       </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/hemeroteca/2026-06-23/</t>
+          <t>https://www.bluradio.com/economia/juegos-de-azar/resultados-loterias-de-cundinamarca-tolima-baloto-miloto-y-colorloto-del-22-de-junio-de-2026-so35</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>23/06/2026 12:33 a. m.</t>
+          <t>23/06/2026 12:53 a. m.</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
@@ -2970,24 +2962,24 @@
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D93" s="6" t="inlineStr">
         <is>
-          <t>Última hora de la guerra de Estados Unidos e Israel contra Irán, en directo | Irán dice que las negociaciones técnicas con EE UU han concluido y que pasan a la siguiente fase</t>
+          <t>ColorLoto, resultado del último sorteo lunes 22 de junio de 2026</t>
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/internacional/2026-06-23/ultima-hora-de-la-guerra-de-estados-unidos-e-israel-contra-iran-en-directo.html</t>
+          <t>https://www.bluradio.com/economia/juegos-de-azar/colorloto-resultado-del-ultimo-sorteo-lunes-22-de-junio-de-2026-so35</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 12:17 a. m.</t>
+          <t>23/06/2026 12:07 a. m.</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -2997,24 +2989,24 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>“Vándalos” y amenazas de hasta 10 años de cárcel: Trump desvía la culpa por el fracaso de la piscina reflectante del Monumento a Lincoln</t>
+          <t>Aceptan tutela contra Luis Díaz y James Rodríguez por "traición a la patria"</t>
         </is>
       </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/us/2026-06-24/vandalos-y-amenazas-de-hasta-10-anos-de-carcel-trump-desvia-la-culpa-por-el-fracaso-de-la-piscina-reflectante-del-monumento-a-lincoln.html</t>
+          <t>https://www.bluradio.com/judicial/aceptan-tutela-contra-luis-diaz-y-james-rodriguez-por-traicion-a-la-patria-so35</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 11:50 p. m.</t>
+          <t>22/06/2026 11:38 p. m.</t>
         </is>
       </c>
       <c r="B95" s="5" t="inlineStr">
@@ -3024,24 +3016,24 @@
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D95" s="6" t="inlineStr">
         <is>
-          <t>Las mejores imágenes de la Copa del Mundo de Fútbol | Imágenes del 22 de junio</t>
+          <t>Predicción Colombia vs. República del Congo: así van las apuestas de este duelo</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/deportes/mundial-futbol/2026-06-23/las-mejores-imagenes-de-la-copa-del-mundo-de-futbol.html</t>
+          <t>https://www.bluradio.com/deportes/futbol/copa-mundial-de-la-fifa-2026/prediccion-colombia-vs-republica-del-congo-asi-van-las-apuestas-de-este-duelo-so35</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 11:17 p. m.</t>
+          <t>22/06/2026 11:18 p. m.</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -3051,24 +3043,24 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>Los sueños rotos de Guillermo y Zafar: de huir de la pesadilla de Trump a encontrar su muerte en México</t>
+          <t>Trump le envía mensaje a De La Espriella: afirma que será un "gran presidente"</t>
         </is>
       </c>
       <c r="E96" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/mexico/2026-06-23/los-suenos-rotos-de-guillermo-y-zafar-de-huir-de-la-pesadilla-de-trump-a-encontrar-su-muerte-en-mexico.html</t>
+          <t>https://www.bluradio.com/nacion/trump-le-envia-mensaje-a-de-la-espriella-afirma-que-sera-un-gran-presidente-cb20</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 11:10 p. m.</t>
+          <t>22/06/2026 11:09 p. m.</t>
         </is>
       </c>
       <c r="B97" s="5" t="inlineStr">
@@ -3078,24 +3070,24 @@
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D97" s="6" t="inlineStr">
         <is>
-          <t>México y Colombia le dan la bienvenida a Lumumba, el hincha más político</t>
+          <t>MiLoto, resultado del último sorteo hoy lunes 22 de junio de 2026</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/mexico/2026-06-23/mexico-y-colombia-le-dan-la-bienvenida-a-lumumba-el-hincha-mas-politico.html</t>
+          <t>https://www.bluradio.com/economia/juegos-de-azar/miloto-resultado-del-ultimo-sorteo-hoy-lunes-22-de-junio-de-2026-so35</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 11:04 p. m.</t>
+          <t>22/06/2026 11:06 p. m.</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -3105,24 +3097,24 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>Joyas por 18 millones de pesos, siete vehículos de lujo, 10 casas y un edificio: Gertz Manero transparenta por primera vez su riqueza</t>
+          <t>Tras doblete contra Irak, Mbappé le envía mensaje a Messi: "No me fijo en lo que hace"</t>
         </is>
       </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/mexico/2026-06-23/joyas-por-18-millones-de-pesos-siete-vehiculos-de-lujo-10-casas-y-un-edificio-gertz-manero-transparenta-por-primera-vez-su-riqueza.html</t>
+          <t>https://www.bluradio.com/deportes/futbol/copa-mundial-de-la-fifa-2026/tras-doblete-contra-irak-mbappe-le-envia-mensaje-a-messi-no-me-fijo-en-lo-que-hace-cb20</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 11:00 p. m.</t>
+          <t>22/06/2026 11:06 p. m.</t>
         </is>
       </c>
       <c r="B99" s="5" t="inlineStr">
@@ -3132,24 +3124,24 @@
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D99" s="6" t="inlineStr">
         <is>
-          <t>Colombia se divide en las urnas y se reencuentra en la Constitución</t>
+          <t>Baloto y Revancha, resultado del útimo sorteo hoy lunes 22 de junio de 2026</t>
         </is>
       </c>
       <c r="E99" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/america-colombia/elecciones-presidenciales/2026-06-23/colombia-se-divide-en-las-urnas-y-se-reencuentra-en-la-constitucion.html</t>
+          <t>https://www.bluradio.com/economia/juegos-de-azar/baloto-y-revancha-resultado-del-utimo-sorteo-hoy-lunes-22-de-junio-de-2026-so35</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 11:00 p. m.</t>
+          <t>22/06/2026 11:03 p. m.</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -3159,24 +3151,24 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>El idioma nacional</t>
+          <t>Martha Peralta recobró la libertad tras terminar su indagatoria por caso UNGRD</t>
         </is>
       </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/america/iberoamerica-democracia/2026-06-23/el-idioma-nacional.html</t>
+          <t>https://www.bluradio.com/judicial/martha-peralta-recobro-la-libertad-tras-terminar-su-indagatoria-por-caso-ungrd-rg10</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 11:00 p. m.</t>
+          <t>22/06/2026 10:44 p. m.</t>
         </is>
       </c>
       <c r="B101" s="5" t="inlineStr">
@@ -3186,24 +3178,24 @@
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D101" s="6" t="inlineStr">
         <is>
-          <t>El dibujante boliviano Al-Azar interpela al poder a través de la caricatura política</t>
+          <t>El Pentágono de EEUU propone a De la Espriella reforzar la alianza contra el narcotráfico</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/america-futura/2026-06-23/el-dibujante-boliviano-al-azar-interpela-al-poder-a-traves-de-la-caricatura-politica.html</t>
+          <t>https://www.bluradio.com/nacion/el-pentagono-de-eeuu-propone-a-de-la-espriella-reforzar-la-alianza-contra-el-narcotrafico-cb20</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 11:00 p. m.</t>
+          <t>22/06/2026 10:04 p. m.</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -3213,24 +3205,24 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>El precio de investigar al Gobierno en Ecuador alcanza a la familia de un periodista</t>
+          <t>Argentina clasifica a dieciseisavos de final: 22 junio 2026-Blog Deportivo, programa completo</t>
         </is>
       </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/america/2026-06-23/el-precio-de-investigar-al-gobierno-en-ecuador-alcanza-a-la-familia-de-un-periodista.html</t>
+          <t>https://www.bluradio.com/blog-deportivo/argentina-clasifica-a-dieciseisavos-de-final-22-junio-2026-blog-deportivo-programa-completo-pr30</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 11:00 p. m.</t>
+          <t>22/06/2026 09:51 p. m.</t>
         </is>
       </c>
       <c r="B103" s="5" t="inlineStr">
@@ -3240,24 +3232,24 @@
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D103" s="6" t="inlineStr">
         <is>
-          <t>Sin cheque en blanco: el reto de Abelardo de la Espriella de gobernar con medio país en contra</t>
+          <t>Lotería del Tolima, resultado del último sorteo hoy lunes 22 de junio de 2026</t>
         </is>
       </c>
       <c r="E103" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/america-colombia/elecciones-presidenciales/2026-06-23/sin-cheque-en-blanco-el-reto-de-abelardo-de-la-espriella-de-gobernar-con-medio-pais-en-contra.html</t>
+          <t>https://www.bluradio.com/economia/juegos-de-azar/loteria-del-tolima-resultado-del-ultimo-sorteo-hoy-lunes-22-de-junio-de-2026-so35</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 11:00 p. m.</t>
+          <t>23/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
@@ -3267,24 +3259,24 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>Videoanálisis | La oposición al Gobierno de Abelardo de la Espriella será robusta</t>
+          <t>Fracking: la fractura humana de la palabra</t>
         </is>
       </c>
       <c r="E104" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/america-colombia/elecciones-presidenciales/2026-06-23/videoanalisis-la-oposicion-al-gobierno-de-abelardo-de-la-espriella-sera-robusta.html</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/23/fracking-la-fractura-humana-de-la-palabra/</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 11:00 p. m.</t>
+          <t>23/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
@@ -3294,24 +3286,24 @@
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D105" s="6" t="inlineStr">
         <is>
-          <t>Gustavo Puerta, una estrella en ascenso fuera del radar de la selección de Colombia</t>
+          <t>Columnistas</t>
         </is>
       </c>
       <c r="E105" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/america-colombia/2026-06-23/gustavo-puerta-una-estrella-en-ascenso-fuera-del-radar-de-la-seleccion-de-colombia.html</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 11:00 p. m.</t>
+          <t>23/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
@@ -3321,24 +3313,24 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D106" s="3" t="inlineStr">
         <is>
-          <t>Juan David Velasco, investigador: “La derecha necesitaba dejar morir al uribismo para volver al poder”</t>
+          <t>El ‘memorando de entendimiento’ entre Irán y E.E.U.U.</t>
         </is>
       </c>
       <c r="E106" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/america-colombia/elecciones-presidenciales/2026-06-23/juan-david-velasco-investigador-la-derecha-necesitaba-dejar-morir-al-uribismo-para-volver-al-poder.html</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/23/el-memorando-de-entendimiento-entre-iran-y-eeuu/</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 10:45 p. m.</t>
+          <t>23/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
@@ -3348,24 +3340,24 @@
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D107" s="6" t="inlineStr">
         <is>
-          <t>Las promesas incumplidas del Brexit: por qué el Reino Unido está peor que antes de salir de la UE</t>
+          <t>Un cielo nublado</t>
         </is>
       </c>
       <c r="E107" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/internacional/2026-06-23/las-promesas-incumplidas-del-brexit-por-que-el-reino-unido-esta-peor-que-antes-de-salir-de-la-ue.html</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/23/un-cielo-nublado/</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 10:45 p. m.</t>
+          <t>23/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
@@ -3375,24 +3367,24 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D108" s="3" t="inlineStr">
         <is>
-          <t>Estados Unidos versus Irán, la guerra de fuerzas desiguales que ningún bando pudo ganar</t>
+          <t>Cambio de chip</t>
         </is>
       </c>
       <c r="E108" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/internacional/2026-06-23/estados-unidos-versus-iran-la-guerra-de-fuerzas-desiguales-que-ningun-bando-pudo-ganar.html</t>
+          <t>https://www.vanguardia.com/opinion/caricaturas/2026/06/23/cambio-de-chip/</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 10:45 p. m.</t>
+          <t>23/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B109" s="5" t="inlineStr">
@@ -3402,24 +3394,24 @@
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D109" s="6" t="inlineStr">
         <is>
-          <t>Las nuevas viviendas en España apenas cubrieron el 40% de los hogares que se constituyeron el año pasado</t>
+          <t>Caricaturas</t>
         </is>
       </c>
       <c r="E109" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/economia/vivienda/2026-06-23/las-nuevas-viviendas-en-espana-apenas-cubrieron-el-40-de-los-hogares-que-se-constituyeron-el-ano-pasado.html</t>
+          <t>https://www.vanguardia.com/opinion/caricaturas/</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 10:30 p. m.</t>
+          <t>22/06/2026 10:59 p. m.</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
@@ -3429,24 +3421,24 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D110" s="3" t="inlineStr">
         <is>
-          <t>Recorrido visual por la sentencia del Supremo que condena a Ábalos, Koldo y Aldama</t>
+          <t>¿Traición a la patria? La insólita “tutela” contra James Rodríguez y Luis Díaz en pleno Mundial</t>
         </is>
       </c>
       <c r="E110" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/espana/2026-06-23/recorrido-visual-por-la-sentencia-del-supremo-que-condena-a-abalos-koldo-y-aldama.html</t>
+          <t>https://www.vanguardia.com/deportes/mundial-de-futbol/2026/06/22/traicion-a-la-patria-la-insolita-tutela-contra-james-rodriguez-y-luis-diaz-en-pleno-mundial/</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 10:30 p. m.</t>
+          <t>22/06/2026 10:59 p. m.</t>
         </is>
       </c>
       <c r="B111" s="5" t="inlineStr">
@@ -3456,24 +3448,24 @@
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D111" s="6" t="inlineStr">
         <is>
-          <t>Ayuso multa con hasta 13.000 euros a pequeños comercios gallegos por incumplir la normativa de venta ‘online’</t>
+          <t>Mundial de Fútbol</t>
         </is>
       </c>
       <c r="E111" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/espana/galicia/2026-06-23/ayuso-multa-con-hasta-13000-euros-a-pequenos-comercios-gallegos-por-incumplir-la-normativa-de-venta-online.html</t>
+          <t>https://www.vanguardia.com/deportes/mundial-de-futbol/</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 10:30 p. m.</t>
+          <t>22/06/2026 10:43 p. m.</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
@@ -3483,24 +3475,24 @@
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D112" s="3" t="inlineStr">
         <is>
-          <t>Ian Gibson: “Un Gobierno que sacó a Franco del Valle de los Caídos haría muy bien en seguir buscando el cadáver de Lorca”</t>
+          <t>Gobierno inicia la liquidación del Ministerio de la Igualdad en medio de protestas laborales</t>
         </is>
       </c>
       <c r="E112" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/cultura/2026-06-23/ian-gibson-un-gobierno-que-saco-a-franco-del-valle-de-los-caidos-haria-muy-bien-en-seguir-buscando-el-cadaver-de-lorca.html</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/22/gobierno-inicia-la-liquidacion-del-ministerio-de-la-igualdad-en-medio-de-protestas-laborales/</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 10:30 p. m.</t>
+          <t>22/06/2026 10:43 p. m.</t>
         </is>
       </c>
       <c r="B113" s="5" t="inlineStr">
@@ -3510,24 +3502,24 @@
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D113" s="6" t="inlineStr">
         <is>
-          <t>Calor, sol o picaduras en niños: cómo prevenir los riesgos más frecuentes durante el verano</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E113" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/mamas-papas/actualidad/2026-06-23/calor-sol-o-picaduras-en-ninos-como-prevenir-los-riesgos-mas-frecuentes-durante-el-verano.html</t>
+          <t>https://www.vanguardia.com/colombia/</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 10:30 p. m.</t>
+          <t>22/06/2026 10:39 p. m.</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
@@ -3537,24 +3529,24 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D114" s="3" t="inlineStr">
         <is>
-          <t>España, cuando la calma está en el vértigo</t>
+          <t>Voto en el exterior, clave para victoria de Abelardo De La Espriella: así quedaron los resultados</t>
         </is>
       </c>
       <c r="E114" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/deportes/mundial-futbol/2026-06-23/espana-cuando-la-calma-esta-en-el-vertigo.html</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/22/voto-en-el-exterior-fue-clave-para-la-victoria-de-abelardo-de-la-espriella-asi-quedaron-los-resultados/</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 10:30 p. m.</t>
+          <t>22/06/2026 07:51 p. m.</t>
         </is>
       </c>
       <c r="B115" s="5" t="inlineStr">
@@ -3564,24 +3556,24 @@
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D115" s="6" t="inlineStr">
         <is>
-          <t>Cómo Ikea se metió en ocho de cada diez hogares españoles: 30 años del desembarco del gigante sueco</t>
+          <t>Martha Peralta recupera su libertad tras declarar ante la Corte por investigación de contratos en la Ungrd</t>
         </is>
       </c>
       <c r="E115" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/icon-design/2026-06-23/como-ikea-se-metio-en-ocho-de-cada-diez-hogares-espanoles-30-anos-del-desembarco-del-gigante-sueco.html</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/22/martha-peralta-recupera-su-libertad-tras-declarar-ante-la-corte-por-investigacion-de-contratos-en-la-ungrd/</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 08:37 p. m.</t>
+          <t>22/06/2026 07:00 p. m.</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
@@ -3591,24 +3583,24 @@
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D116" s="3" t="inlineStr">
         <is>
-          <t>Francia brilla con un doblete de Mbappé en un partido pasado por agua</t>
+          <t>Simpatizantes de Iván Cepeda marchan en Bogotá mientras avanza el escrutinio electoral</t>
         </is>
       </c>
       <c r="E116" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/deportes/mundial-futbol/2026-06-23/una-francia-pasada-por-agua-brilla-con-un-doblete-de-mbappe.html</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/22/simpatizantes-de-ivan-cepeda-marchan-en-bogota-mientras-avanza-el-escrutinio-electoral/</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 04:26 p. m.</t>
+          <t>22/06/2026 04:40 p. m.</t>
         </is>
       </c>
       <c r="B117" s="5" t="inlineStr">
@@ -3618,24 +3610,24 @@
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D117" s="6" t="inlineStr">
         <is>
-          <t>Julián Alvarez pide salir del Atlético y el club rojiblanco se plantea denunciar al Barça ante la FIFA: “No puedo esconderme, lo mejor es una transferencia, quiero cumplir mi sueño”</t>
+          <t>Hallan a una mujer muerta dentro de una maleta en Bogotá: investigan a un extranjero que estuvo con ella</t>
         </is>
       </c>
       <c r="E117" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/deportes/mundial-futbol/2026-06-22/julian-alvarez-pide-salir-del-atletico-no-puedo-esconderme-lo-mejor-es-una-transferencia-quiero-cumplir-mi-sueno.html</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/22/hallan-a-una-mujer-muerta-dentro-de-una-maleta-en-bogota-investigan-a-un-extranjero-que-estuvo-con-ella/</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 03:09 p. m.</t>
+          <t>22/06/2026 04:11 p. m.</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
@@ -3645,24 +3637,24 @@
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D118" s="3" t="inlineStr">
         <is>
-          <t>El viejo Messi emociona al mundo: otro doblete lo convierte en el máximo goleador de la historia del torneo</t>
+          <t>Isabella Echeverri: de defender el arco a contar las historias de la Selección Colombia</t>
         </is>
       </c>
       <c r="E118" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/deportes/mundial-futbol/2026-06-22/el-viejo-messi-conmueve-al-mundo.html</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/22/isabella-echeverri-de-defender-el-arco-a-contar-las-historias-de-la-seleccion-colombia/</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="5" t="inlineStr">
         <is>
-          <t>22/06/2026 09:27 a. m.</t>
+          <t>22/06/2026 03:51 p. m.</t>
         </is>
       </c>
       <c r="B119" s="5" t="inlineStr">
@@ -3672,22 +3664,26 @@
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D119" s="6" t="inlineStr">
         <is>
-          <t>Bear, el hijo de 9 años de Liam Payne, ya puede beneficiarse de los 25 millones de herencia del fallecido cantante</t>
+          <t>Gustavo Petro celebra posible salida de la lista Clinton y agita la polémica</t>
         </is>
       </c>
       <c r="E119" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/gente/2026-06-22/bear-el-hijo-de-9-anos-de-liam-payne-ya-puede-beneficiarse-de-los-25-millones-de-herencia-del-fallecido-cantante.html</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/22/petro-celebra-posible-salida-de-la-lista-ofac-ya-no-se-enfrentan-a-guerrilleros-sino-a-pueblos/</t>
         </is>
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="2" t="inlineStr"/>
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>22/06/2026 03:38 p. m.</t>
+        </is>
+      </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3695,22 +3691,26 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D120" s="3" t="inlineStr">
         <is>
-          <t>Predicciones</t>
+          <t>Cepeda pide diálogo y responde a De La Espriella tras su discurso: “No nos asustan sus rugidos”</t>
         </is>
       </c>
       <c r="E120" s="4" t="inlineStr">
         <is>
-          <t>https://elpais.com/deportes/mundial-futbol/2026-06-11/quien-ganara-el-mundial-asi-arrancan-nuestras-predicciones.html</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/22/cepeda-pide-dialogo-y-responde-a-de-la-espriella-tras-su-discurso-no-nos-asustan-sus-rugidos/</t>
         </is>
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="5" t="inlineStr"/>
+      <c r="A121" s="5" t="inlineStr">
+        <is>
+          <t>22/06/2026 03:00 p. m.</t>
+        </is>
+      </c>
       <c r="B121" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3718,24 +3718,24 @@
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>El País</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D121" s="6" t="inlineStr">
         <is>
-          <t>Selecciones</t>
+          <t>Los nombres que suenan para el gabinete de De La Espriella: entre figuras políticas y apuestas técnicas</t>
         </is>
       </c>
       <c r="E121" s="7" t="inlineStr">
         <is>
-          <t>https://elpais.com/deportes/mundial-futbol/2026-06-05/todas-las-selecciones-del-mundial-de-estados-unidos-canada-y-mexico.html</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/22/los-nombres-que-empiezan-a-sonar-para-el-gabinete-de-abelardo-de-la-espriella-entre-figuras-politicas-y-apuestas-tecnicas/</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 12:26 a. m.</t>
+          <t>23/06/2026 12:49 a. m.</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
@@ -3762,7 +3762,7 @@
     <row r="123">
       <c r="A123" s="5" t="inlineStr">
         <is>
-          <t>23/06/2026 12:26 a. m.</t>
+          <t>23/06/2026 12:49 a. m.</t>
         </is>
       </c>
       <c r="B123" s="5" t="inlineStr">
@@ -3789,7 +3789,7 @@
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 12:26 a. m.</t>
+          <t>23/06/2026 12:49 a. m.</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
@@ -5370,12 +5370,12 @@
       </c>
       <c r="D186" s="3" t="inlineStr">
         <is>
-          <t>Pico y Placa: qué automóviles no circulan en Bogotá este martes 23 de junio</t>
+          <t>Resultado Sinuano Noche hoy 22 de junio</t>
         </is>
       </c>
       <c r="E186" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/23/pico-y-placa-que-automoviles-no-circulan-en-bogota-este-martes-23-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/23/resultado-sinuano-noche-hoy-22-de-junio/</t>
         </is>
       </c>
     </row>
@@ -5397,12 +5397,12 @@
       </c>
       <c r="D187" s="6" t="inlineStr">
         <is>
-          <t>Video de seguridad revela presunto secuestro de un hombre en Cajibío, Cauca por sujetos armados en motocicletas</t>
+          <t>Tutela contra James Rodríguez, Luis Díaz y la FCF por presunta “traición a la patria” fue admitida por un juzgado</t>
         </is>
       </c>
       <c r="E187" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/23/video-de-seguridad-revela-presunto-secuestro-de-un-hombre-en-cajibio-cauca-por-sujetos-armados-en-motocicletas/</t>
+          <t>https://www.infobae.com/colombia/deportes/2026/06/23/tutela-contra-james-rodriguez-luis-diaz-y-la-fcf-por-presunta-traicion-a-la-patria-fue-admitida-por-un-juzgado/</t>
         </is>
       </c>
     </row>
@@ -5424,12 +5424,12 @@
       </c>
       <c r="D188" s="3" t="inlineStr">
         <is>
-          <t>Lotería de Cundinamarca, resultados oficiales, hoy lunes 22 de junio de 2026</t>
+          <t>Supersalud defiende inspección a la FLA y dice que visitará más fábricas de licores</t>
         </is>
       </c>
       <c r="E188" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/23/loteria-de-cundinamarca-resultados-oficiales-hoy-lunes-22-de-junio-de-2026/</t>
+          <t>https://www.infobae.com/colombia/2026/06/23/supersalud-defiende-inspeccion-a-la-fla-y-dice-que-visitara-mas-fabricas-de-licores/</t>
         </is>
       </c>
     </row>
@@ -5451,12 +5451,12 @@
       </c>
       <c r="D189" s="6" t="inlineStr">
         <is>
-          <t>Felipe Harman volvería a la ANT tras apoyar la campaña de Iván Cepeda: Presidencia publicó su hoja de vida tras elecciones</t>
+          <t>Dos menores resultan heridos en grave accidente en Usaquén, Bogotá, tras choque con volqueta en Tibabita 2</t>
         </is>
       </c>
       <c r="E189" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/23/felipe-harman-volveria-a-la-ant-tras-apoyar-la-campana-de-ivan-cepeda-presidencia-publico-su-hoja-de-vida-tras-elecciones/</t>
+          <t>https://www.infobae.com/colombia/2026/06/23/dos-menores-resultan-heridos-en-grave-accidente-en-usaquen-bogota-tras-choque-con-volqueta-en-tibabita-2/</t>
         </is>
       </c>
     </row>
@@ -5478,12 +5478,12 @@
       </c>
       <c r="D190" s="3" t="inlineStr">
         <is>
-          <t>Resultado Super Astro Luna HOY: número ganador del lunes 22 de junio</t>
+          <t>Pico y Placa: qué automóviles no circulan en Bogotá este martes 23 de junio</t>
         </is>
       </c>
       <c r="E190" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/23/resultado-super-astro-luna-hoy-numero-ganador-del-lunes-22-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/23/pico-y-placa-que-automoviles-no-circulan-en-bogota-este-martes-23-de-junio/</t>
         </is>
       </c>
     </row>
@@ -5505,12 +5505,12 @@
       </c>
       <c r="D191" s="6" t="inlineStr">
         <is>
-          <t>Resultado Chontico Noche: números ganadores del último sorteo hoy, lunes 22 de junio de 2026</t>
+          <t>Video de seguridad revela presunto secuestro de un hombre en Cajibío, Cauca por sujetos armados en motocicletas</t>
         </is>
       </c>
       <c r="E191" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/23/resultado-chontico-noche-numeros-ganadores-del-ultimo-sorteo-hoy-lunes-22-de-junio-de-2026/</t>
+          <t>https://www.infobae.com/colombia/2026/06/23/video-de-seguridad-revela-presunto-secuestro-de-un-hombre-en-cajibio-cauca-por-sujetos-armados-en-motocicletas/</t>
         </is>
       </c>
     </row>
@@ -5532,12 +5532,12 @@
       </c>
       <c r="D192" s="3" t="inlineStr">
         <is>
-          <t>“Cuando les da la gana”: Bolívar defiende esperar escrutinio antes de reconocer triunfo de De La Espriella</t>
+          <t>Lotería de Cundinamarca, resultados oficiales, hoy lunes 22 de junio de 2026</t>
         </is>
       </c>
       <c r="E192" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/23/cuando-les-da-la-gana-bolivar-defiende-esperar-escrutinio-antes-de-reconocer-triunfo-de-de-la-espriella/</t>
+          <t>https://www.infobae.com/colombia/2026/06/23/loteria-de-cundinamarca-resultados-oficiales-hoy-lunes-22-de-junio-de-2026/</t>
         </is>
       </c>
     </row>
@@ -5559,12 +5559,12 @@
       </c>
       <c r="D193" s="6" t="inlineStr">
         <is>
-          <t>“Entre la crisis y la esperanza”: Fernando Ruiz señala cómo De la Espriella podría recuperar el sistema de salud colombiano</t>
+          <t>Felipe Harman volvería a la ANT tras apoyar la campaña de Iván Cepeda: Presidencia publicó su hoja de vida tras elecciones</t>
         </is>
       </c>
       <c r="E193" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/23/entre-la-crisis-y-la-esperanza-fernando-ruiz-senala-como-de-la-espriella-podria-recuperar-el-sistema-de-salud-colombiano/</t>
+          <t>https://www.infobae.com/colombia/2026/06/23/felipe-harman-volveria-a-la-ant-tras-apoyar-la-campana-de-ivan-cepeda-presidencia-publico-su-hoja-de-vida-tras-elecciones/</t>
         </is>
       </c>
     </row>
@@ -5586,12 +5586,12 @@
       </c>
       <c r="D194" s="3" t="inlineStr">
         <is>
-          <t>Tenga en cuenta: así regirá el Pico y Placa en Cartagena este martes 23 de junio</t>
+          <t>Resultado Super Astro Luna HOY: número ganador del lunes 22 de junio</t>
         </is>
       </c>
       <c r="E194" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/23/tenga-en-cuenta-asi-regira-el-pico-y-placa-en-cartagena-este-martes-23-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/23/resultado-super-astro-luna-hoy-numero-ganador-del-lunes-22-de-junio/</t>
         </is>
       </c>
     </row>
@@ -5613,12 +5613,12 @@
       </c>
       <c r="D195" s="6" t="inlineStr">
         <is>
-          <t>Pico y Placa: qué carros descansan en Villavicencio este martes 23 de junio</t>
+          <t>Resultado Chontico Noche: números ganadores del último sorteo hoy, lunes 22 de junio de 2026</t>
         </is>
       </c>
       <c r="E195" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/23/pico-y-placa-que-carros-descansan-en-villavicencio-este-martes-23-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/23/resultado-chontico-noche-numeros-ganadores-del-ultimo-sorteo-hoy-lunes-22-de-junio-de-2026/</t>
         </is>
       </c>
     </row>
@@ -5640,12 +5640,12 @@
       </c>
       <c r="D196" s="3" t="inlineStr">
         <is>
-          <t>Oxford Economics: triunfo de De La Espriella reduce riesgos económicos en Colombia, pero no los elimina</t>
+          <t>“Cuando les da la gana”: Bolívar defiende esperar escrutinio antes de reconocer triunfo de De La Espriella</t>
         </is>
       </c>
       <c r="E196" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/23/oxford-economics-triunfo-de-de-la-espriella-reduce-riesgos-economicos-en-colombia-pero-no-los-elimina/</t>
+          <t>https://www.infobae.com/colombia/2026/06/23/cuando-les-da-la-gana-bolivar-defiende-esperar-escrutinio-antes-de-reconocer-triunfo-de-de-la-espriella/</t>
         </is>
       </c>
     </row>
@@ -5667,12 +5667,12 @@
       </c>
       <c r="D197" s="6" t="inlineStr">
         <is>
-          <t>Miguel Ángel Pinto se declara inocente tras indagatoria por presunto acceso carnal violento ante la Corte Suprema</t>
+          <t>“Entre la crisis y la esperanza”: Fernando Ruiz señala cómo De la Espriella podría recuperar el sistema de salud colombiano</t>
         </is>
       </c>
       <c r="E197" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/23/miguel-angel-pinto-se-declara-inocente-tras-indagatoria-por-presunto-acceso-carnal-violento-ante-la-corte-suprema/</t>
+          <t>https://www.infobae.com/colombia/2026/06/23/entre-la-crisis-y-la-esperanza-fernando-ruiz-senala-como-de-la-espriella-podria-recuperar-el-sistema-de-salud-colombiano/</t>
         </is>
       </c>
     </row>
@@ -5694,12 +5694,12 @@
       </c>
       <c r="D198" s="3" t="inlineStr">
         <is>
-          <t>Desde la UAndes proponen un Pacto Nacional por la Educación Superior: “compromiso impostergable”</t>
+          <t>Tenga en cuenta: así regirá el Pico y Placa en Cartagena este martes 23 de junio</t>
         </is>
       </c>
       <c r="E198" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/23/desde-la-uandes-proponen-un-pacto-nacional-por-la-educacion-superior-compromiso-impostergable/</t>
+          <t>https://www.infobae.com/colombia/2026/06/23/tenga-en-cuenta-asi-regira-el-pico-y-placa-en-cartagena-este-martes-23-de-junio/</t>
         </is>
       </c>
     </row>
@@ -5721,12 +5721,12 @@
       </c>
       <c r="D199" s="6" t="inlineStr">
         <is>
-          <t>Los cortes de agua en Bogotá este 23 de junio</t>
+          <t>Pico y Placa: qué carros descansan en Villavicencio este martes 23 de junio</t>
         </is>
       </c>
       <c r="E199" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/23/los-cortes-de-agua-en-bogota-este-23-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/23/pico-y-placa-que-carros-descansan-en-villavicencio-este-martes-23-de-junio/</t>
         </is>
       </c>
     </row>
@@ -5748,12 +5748,12 @@
       </c>
       <c r="D200" s="3" t="inlineStr">
         <is>
-          <t>Pico y Placa: qué vehículos no circulan en Cali este martes 23 de junio</t>
+          <t>Oxford Economics: triunfo de De La Espriella reduce riesgos económicos en Colombia, pero no los elimina</t>
         </is>
       </c>
       <c r="E200" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/23/pico-y-placa-que-vehiculos-no-circulan-en-cali-este-martes-23-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/23/oxford-economics-triunfo-de-de-la-espriella-reduce-riesgos-economicos-en-colombia-pero-no-los-elimina/</t>
         </is>
       </c>
     </row>
@@ -5775,12 +5775,12 @@
       </c>
       <c r="D201" s="6" t="inlineStr">
         <is>
-          <t>Ponencia pide salvar con salvedades emergencia económica de Petro por inundaciones</t>
+          <t>Miguel Ángel Pinto se declara inocente tras indagatoria por presunto acceso carnal violento ante la Corte Suprema</t>
         </is>
       </c>
       <c r="E201" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/23/ponencia-pide-salvar-con-salvedades-emergencia-economica-de-petro-por-inundaciones/</t>
+          <t>https://www.infobae.com/colombia/2026/06/23/miguel-angel-pinto-se-declara-inocente-tras-indagatoria-por-presunto-acceso-carnal-violento-ante-la-corte-suprema/</t>
         </is>
       </c>
     </row>
@@ -5802,12 +5802,12 @@
       </c>
       <c r="D202" s="3" t="inlineStr">
         <is>
-          <t>Pilas: Así rotará el Pico y Placa en Medellín este martes 23 de junio</t>
+          <t>Desde la UAndes proponen un Pacto Nacional por la Educación Superior: “compromiso impostergable”</t>
         </is>
       </c>
       <c r="E202" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/23/pilas-asi-rotara-el-pico-y-placa-en-medellin-este-martes-23-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/23/desde-la-uandes-proponen-un-pacto-nacional-por-la-educacion-superior-compromiso-impostergable/</t>
         </is>
       </c>
     </row>
@@ -5829,12 +5829,12 @@
       </c>
       <c r="D203" s="6" t="inlineStr">
         <is>
-          <t>Álvaro Uribe se despachó contra estratega de Abelardo de la Espriella, pese a victoria del ‘Tigre’: este es el motivo de la polémica</t>
+          <t>Los cortes de agua en Bogotá este 23 de junio</t>
         </is>
       </c>
       <c r="E203" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/23/alvaro-uribe-se-despacho-contra-estratega-de-abelardo-de-la-espriella-pese-a-victoria-del-tigre-este-es-el-motivo-de-la-polemica/</t>
+          <t>https://www.infobae.com/colombia/2026/06/23/los-cortes-de-agua-en-bogota-este-23-de-junio/</t>
         </is>
       </c>
     </row>
@@ -5856,19 +5856,19 @@
       </c>
       <c r="D204" s="3" t="inlineStr">
         <is>
-          <t>El triunfo de Abelardo de la Espriella cambió el mapa político de América Latina: así se ve la región entre la derecha y la izquierda</t>
+          <t>Pico y Placa: qué vehículos no circulan en Cali este martes 23 de junio</t>
         </is>
       </c>
       <c r="E204" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/23/el-triunfo-de-abelardo-de-la-espriella-cambio-el-mapa-politico-de-america-latina-asi-se-ve-la-region-entre-la-derecha-y-la-izquierda/</t>
+          <t>https://www.infobae.com/colombia/2026/06/23/pico-y-placa-que-vehiculos-no-circulan-en-cali-este-martes-23-de-junio/</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="5" t="inlineStr">
         <is>
-          <t>20/06/2026 12:00 a. m.</t>
+          <t>23/06/2026 12:00 a. m.</t>
         </is>
       </c>
       <c r="B205" s="5" t="inlineStr">
@@ -5883,12 +5883,12 @@
       </c>
       <c r="D205" s="6" t="inlineStr">
         <is>
-          <t>Resultados elecciones Colombia EN VIVO: el procurador Gregorio Eljach descartó fraude electoral tras la victoria de De la Espriella: “No hay evidencia de adulteración”</t>
+          <t>Ponencia pide salvar con salvedades emergencia económica de Petro por inundaciones</t>
         </is>
       </c>
       <c r="E205" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/20/elecciones-presidenciales-de-colombia-2026-en-vivo-estas-son-las-ultimas-movidas-politicas-de-cara-a-la-segunda-vuelta/</t>
+          <t>https://www.infobae.com/colombia/2026/06/23/ponencia-pide-salvar-con-salvedades-emergencia-economica-de-petro-por-inundaciones/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 Noticias actualizadas 24/06/2026 09:14
</commit_message>
<xml_diff>
--- a/docs/ultimahora.xlsx
+++ b/docs/ultimahora.xlsx
@@ -515,7 +515,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>24/06/2026 12:56 a. m.</t>
+          <t>24/06/2026 04:03 a. m.</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -530,19 +530,19 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Vacaciones en el Mundial: ¡más que un lindo sueño de infancia!</t>
+          <t>Partidos del Mundial hoy 24 de junio en Estados Unidos, Canadá y México: canal y hora para ver en vivo</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/vacaciones-en-el-mundial-mas-que-un-lindo-sueno-de-infancia-3566615</t>
+          <t>https://www.eltiempo.com/deportes/futbol-colombiano/partidos-del-mundial-hoy-24-de-junio-en-estados-unidos-canada-y-mexico-canal-y-hora-para-ver-en-vivo-3566618</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>24/06/2026 12:20 a. m.</t>
+          <t>24/06/2026 02:55 a. m.</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -557,19 +557,19 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>Colombia vibra con el triunfo contra Congo: el panorama de la Selección en el Mundial, día, hora y dónde ver el juego contra Portugal</t>
+          <t>Presidente Gustavo Petro dice que 'empezará el empalme y mi retirada', en un mensaje en sus redes sociales</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/colombia-vibra-con-el-triunfo-contra-congo-el-panorama-de-la-seleccion-en-el-mundial-dia-hora-y-donde-ver-el-juego-contra-portugal-3566613</t>
+          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/presidente-gustavo-petro-dice-que-empezara-el-empalme-y-mi-retirada-en-un-mensaje-en-sus-redes-sociales-3566616</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>24/06/2026 12:11 a. m.</t>
+          <t>24/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -584,19 +584,19 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>La alerta de la presidenta de Naturgas tras fuerte caída de las reservas de gas al cierre de 2025: ‘Debemos actuar con sentido de urgencia’</t>
+          <t>¡Programe sus recorridos! Así regirá el pico y placa en Bucaramanga este miércoles 24 de junio de 2026</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/economia/sectores/la-alerta-de-la-presidenta-de-naturgas-tras-fuerte-caida-de-las-reservas-de-gas-al-cierre-de-2025-debemos-actuar-con-sentido-de-urgencia-3566614</t>
+          <t>https://www.eltiempo.com/colombia/santander/programe-sus-recorridos-asi-regira-el-pico-y-placa-en-bucaramanga-este-miercoles-24-de-junio-de-3566466</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>24/06/2026 12:04 a. m.</t>
+          <t>24/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -611,19 +611,19 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Venezuela es la provincia energética más rica del hemisferio, pero apagones son una constante: ¿cuál es la receta para reactivar el sector eléctrico?</t>
+          <t>¡Revise si puede circular, conductor! Pico y placa en Pereira para el miércoles 24 de junio de 2026</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/venezuela/venezuela-es-la-provincia-energetica-mas-rica-del-hemisferio-pero-apagones-son-una-constante-cual-es-la-receta-para-reactivar-el-sector-electrico-3566469</t>
+          <t>https://www.eltiempo.com/colombia/otras-ciudades/revise-si-puede-circular-conductor-pico-y-placa-en-pereira-para-el-miercoles-24-de-junio-de-3566465</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 11:58 p. m.</t>
+          <t>24/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -638,19 +638,19 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>El fútbol celebra a un Messi estelar en su cumpleaños 39</t>
+          <t>¡Consulte las restricciones! Así opera el pico y placa en Medellín este miércoles 24 de junio de 2026</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/el-futbol-celebra-a-un-messi-estelar-en-su-cumpleanos-3566570</t>
+          <t>https://www.eltiempo.com/colombia/medellin/consulte-las-restricciones-asi-opera-el-pico-y-placa-en-medellin-este-miercoles-24-de-junio-de-3566464</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>23/06/2026 11:56 p. m.</t>
+          <t>24/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -665,19 +665,19 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Las reacciones de los jugadores de Colombia tras vencer a la República del Congo y lograr la clasificación: celebración y abrazos en la cancha</t>
+          <t>Revise su placa: así funciona el pico y placa en Bogotá este miércoles 24 de junio de 2026</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/las-reacciones-de-los-jugadores-de-colombia-tras-vencer-a-la-republica-del-congo-y-lograr-la-clasificacion-celebracion-y-abrazos-en-el-cancha-3566612</t>
+          <t>https://www.eltiempo.com/bogota/revise-su-placa-asi-funciona-el-pico-y-placa-en-bogota-este-miercoles-24-de-junio-de-3566462</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 11:50 p. m.</t>
+          <t>24/06/2026 02:30 a. m.</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -692,19 +692,19 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>¿Por qué el Brexit es el gran culpable de la crisis en Reino Unido? Desgobierno, economía y migración sacuden al país / Análisis de Mauricio Vargas</t>
+          <t>¡Ojo al volante! Pico y placa en Cali para el miércoles 24 de junio de 2026: consulte si puede circular</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/europa/por-que-el-brexit-es-el-gran-culpable-de-la-crisis-en-reino-unido-desgobierno-economia-y-migracion-sacuden-al-pais-analisis-de-mauricio-vargas-3566540</t>
+          <t>https://www.eltiempo.com/colombia/cali/ojo-al-volante-pico-y-placa-en-cali-para-el-miercoles-24-de-junio-de-2026-consulte-si-puede-circular-3566461</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>23/06/2026 11:50 p. m.</t>
+          <t>24/06/2026 12:56 a. m.</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -719,19 +719,19 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Una universidad para mayores de 50 años que enseña a seguir viviendo</t>
+          <t>Vacaciones en el Mundial: ¡más que un lindo sueño de infancia!</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mas-cincuenta/una-universidad-para-mayores-de-50-anos-que-ensena-a-seguir-viviendo-3566553</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/vacaciones-en-el-mundial-mas-que-un-lindo-sueno-de-infancia-3566615</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 11:49 p. m.</t>
+          <t>24/06/2026 12:20 a. m.</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -746,19 +746,19 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Colombia es uno de los pocos países en los que Donald Trump tiene cierto nivel de favorabilidad: esto revela encuesta global</t>
+          <t>Colombia vibra con el triunfo contra Congo: el panorama de la Selección en el Mundial, día, hora y dónde ver el juego contra Portugal</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/colombia-es-uno-de-los-pocos-paises-en-los-que-donald-trump-tiene-cierto-nivel-de-favorabilidad-esto-revela-encuesta-global-3566496</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/colombia-vibra-con-el-triunfo-contra-congo-el-panorama-de-la-seleccion-en-el-mundial-dia-hora-y-donde-ver-el-juego-contra-portugal-3566613</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>23/06/2026 11:48 p. m.</t>
+          <t>24/06/2026 12:11 a. m.</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -773,19 +773,19 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>A falta de goleador, Daniel Muñoz... (Opinión)</t>
+          <t>La alerta de la presidenta de Naturgas tras fuerte caída de las reservas de gas al cierre de 2025: ‘Debemos actuar con sentido de urgencia’</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/a-falta-de-goleador-daniel-munoz-opinion-3566611</t>
+          <t>https://www.eltiempo.com/economia/sectores/la-alerta-de-la-presidenta-de-naturgas-tras-fuerte-caida-de-las-reservas-de-gas-al-cierre-de-2025-debemos-actuar-con-sentido-de-urgencia-3566614</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 11:47 p. m.</t>
+          <t>24/06/2026 12:04 a. m.</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -800,19 +800,19 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>'Vamos por otra presa': Daniel Muñoz explotó tras el triunfo de Colombia contra Congo en el Mundial</t>
+          <t>Venezuela es la provincia energética más rica del hemisferio, pero apagones son una constante: ¿cuál es la receta para reactivar el sector eléctrico?</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/vamos-por-otra-presa-daniel-munoz-exploto-tras-el-triunfo-de-colombia-contra-congo-en-el-mundial-3566609</t>
+          <t>https://www.eltiempo.com/mundo/venezuela/venezuela-es-la-provincia-energetica-mas-rica-del-hemisferio-pero-apagones-son-una-constante-cual-es-la-receta-para-reactivar-el-sector-electrico-3566469</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>23/06/2026 11:44 p. m.</t>
+          <t>23/06/2026 11:58 p. m.</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -827,19 +827,19 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Gerente de la Federación Nacional de Cafeteros se pronunció tras prórroga por cinco meses del contrato de administración del Fondo Nacional del Café</t>
+          <t>El fútbol celebra a un Messi estelar en su cumpleaños 39</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/economia/sectores/gerente-de-la-federacion-nacional-de-cafeteros-explico-en-que-consiste-la-prorroga-de-cinco-meses-para-administrar-el-fondo-nacional-del-cafe-3566604</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/el-futbol-celebra-a-un-messi-estelar-en-su-cumpleanos-3566570</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 11:39 p. m.</t>
+          <t>23/06/2026 11:56 p. m.</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -854,19 +854,19 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Nuevos detalles del exfutbolista colombiano señalado de matar y decapitar a su amigo en Chile, a donde se habrían trasladado temidas 'casas de pique'</t>
+          <t>Las reacciones de los jugadores de Colombia tras vencer a la República del Congo y lograr la clasificación: celebración y abrazos en la cancha</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/cali/nuevos-detalles-del-exfutbolista-colombiano-senalado-de-matar-y-decapitar-a-su-amigo-en-chile-a-donde-se-habrian-trasladado-temidas-casas-de-pique-3566569</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/las-reacciones-de-los-jugadores-de-colombia-tras-vencer-a-la-republica-del-congo-y-lograr-la-clasificacion-celebracion-y-abrazos-en-el-cancha-3566612</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>23/06/2026 11:39 p. m.</t>
+          <t>23/06/2026 11:50 p. m.</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -881,19 +881,19 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Así jugó la Selección Colombia, uno por uno: Daniel Muñoz, un goleador de emergencia que acabó como figura</t>
+          <t>¿Por qué el Brexit es el gran culpable de la crisis en Reino Unido? Desgobierno, economía y migración sacuden al país / Análisis de Mauricio Vargas</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/asi-jugo-la-seleccion-colombia-uno-por-uno-daniel-munoz-un-goleador-de-emergencia-que-acabo-como-figura-3566610</t>
+          <t>https://www.eltiempo.com/mundo/europa/por-que-el-brexit-es-el-gran-culpable-de-la-crisis-en-reino-unido-desgobierno-economia-y-migracion-sacuden-al-pais-analisis-de-mauricio-vargas-3566540</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 11:32 p. m.</t>
+          <t>23/06/2026 11:50 p. m.</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -908,19 +908,19 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>¿Cuándo volverá a jugar la Selección Colombia en el Mundial de la Fifa 2026? Detalles del partido contra Portugal por el liderato del Grupo K</t>
+          <t>Una universidad para mayores de 50 años que enseña a seguir viviendo</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/cuando-volvera-a-jugar-la-seleccion-colombia-en-el-mundial-de-la-fifa-2026-detalles-del-partido-decisivo-contra-portugal-por-el-liderato-del-grupo-k-3566603</t>
+          <t>https://www.eltiempo.com/mas-cincuenta/una-universidad-para-mayores-de-50-anos-que-ensena-a-seguir-viviendo-3566553</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>23/06/2026 11:24 p. m.</t>
+          <t>23/06/2026 11:49 p. m.</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -935,19 +935,19 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>¡Clasificados! La Selección Colombia esquivó la trampa con talento y venció a República Democrática del Congo</t>
+          <t>Colombia es uno de los pocos países en los que Donald Trump tiene cierto nivel de favorabilidad: esto revela encuesta global</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/clasificados-la-seleccion-colombia-esquivo-la-trampa-con-talento-y-vencio-a-republica-democratica-del-congo-3566608</t>
+          <t>https://www.eltiempo.com/mundo/eeuu-y-canada/colombia-es-uno-de-los-pocos-paises-en-los-que-donald-trump-tiene-cierto-nivel-de-favorabilidad-esto-revela-encuesta-global-3566496</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 11:14 p. m.</t>
+          <t>23/06/2026 11:48 p. m.</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -962,19 +962,19 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Néstor Lorenzo, lleno de orgullo: elogió a sus jugadores por el esfuerzo en el triunfo de Colombia contra Congo</t>
+          <t>A falta de goleador, Daniel Muñoz... (Opinión)</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/nestor-lorenzo-lleno-de-orgullo-elogio-a-sus-jugadores-por-el-esfuerzo-en-el-triunfo-de-colombia-contra-congo-3566607</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/a-falta-de-goleador-daniel-munoz-opinion-3566611</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>23/06/2026 11:07 p. m.</t>
+          <t>23/06/2026 11:47 p. m.</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -989,19 +989,19 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Videos | Reviva gol de la selección Colombia que le dio la victoria contra RD Congo y lo dejó como primero en el grupo: mejores jugadas y anulados</t>
+          <t>'Vamos por otra presa': Daniel Muñoz explotó tras el triunfo de Colombia contra Congo en el Mundial</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/videos-reviva-gol-de-la-seleccion-colombia-que-le-dio-la-victoria-contra-rd-congo-1-0-y-lo-dejo-como-primero-en-el-grupo-mejores-jugadas-y-anulados-3566606</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/vamos-por-otra-presa-daniel-munoz-exploto-tras-el-triunfo-de-colombia-contra-congo-en-el-mundial-3566609</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 10:55 p. m.</t>
+          <t>23/06/2026 11:44 p. m.</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1016,19 +1016,19 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>El triunfo de De la Espriella</t>
+          <t>Gerente de la Federación Nacional de Cafeteros se pronunció tras prórroga por cinco meses del contrato de administración del Fondo Nacional del Café</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/cartas/el-triunfo-de-de-la-espriella-3566599</t>
+          <t>https://www.eltiempo.com/economia/sectores/gerente-de-la-federacion-nacional-de-cafeteros-explico-en-que-consiste-la-prorroga-de-cinco-meses-para-administrar-el-fondo-nacional-del-cafe-3566604</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>23/06/2026 10:55 p. m.</t>
+          <t>23/06/2026 11:39 p. m.</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
@@ -1043,12 +1043,12 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Pobres infractores</t>
+          <t>Nuevos detalles del exfutbolista colombiano señalado de matar y decapitar a su amigo en Chile, a donde se habrían trasladado temidas 'casas de pique'</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/opinion/columnistas/pobres-infractores-3566598</t>
+          <t>https://www.eltiempo.com/colombia/cali/nuevos-detalles-del-exfutbolista-colombiano-senalado-de-matar-y-decapitar-a-su-amigo-en-chile-a-donde-se-habrian-trasladado-temidas-casas-de-pique-3566569</t>
         </is>
       </c>
     </row>
@@ -3500,7 +3500,7 @@
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
-          <t>24/06/2026 12:47 a. m.</t>
+          <t>24/06/2026 12:13 a. m.</t>
         </is>
       </c>
       <c r="B113" s="5" t="inlineStr">
@@ -4194,7 +4194,7 @@
     <row r="143">
       <c r="A143" s="5" t="inlineStr">
         <is>
-          <t>24/06/2026 12:47 a. m.</t>
+          <t>24/06/2026 12:13 a. m.</t>
         </is>
       </c>
       <c r="B143" s="5" t="inlineStr">
@@ -5227,12 +5227,12 @@
       </c>
       <c r="D185" s="6" t="inlineStr">
         <is>
-          <t>Devolución automática de saldos a favor en renta 2026: paso a paso para solicitarla ante la Dian</t>
+          <t>Sudáfrica vs. Corea del Sur, EN VIVO: siga el minuto a minuto del partido por la fecha 3 del Grupo A del Mundial 2026</t>
         </is>
       </c>
       <c r="E185" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/24/devolucion-automatica-de-saldos-a-favor-en-renta-2026-paso-a-paso-para-solicitarla-ante-la-dian/</t>
+          <t>https://www.infobae.com/colombia/deportes/2026/06/24/sudafrica-vs-corea-del-sur-en-vivo-siga-el-minuto-a-minuto-del-partido-por-la-fecha-3-del-grupo-a-del-mundial-2026/</t>
         </is>
       </c>
     </row>
@@ -5254,12 +5254,12 @@
       </c>
       <c r="D186" s="3" t="inlineStr">
         <is>
-          <t>Gobierno prorroga por cinco meses el contrato del Fondo Nacional del Café y deja nuevo acuerdo al próximo presidente</t>
+          <t>Suiza vs. Canadá, EN VIVO: siga el minuto a minuto del partido en el Grupo B del Mundial 2026</t>
         </is>
       </c>
       <c r="E186" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/24/gobierno-prorroga-por-cinco-meses-el-contrato-del-fondo-nacional-del-cafe-y-deja-nuevo-acuerdo-al-proximo-presidente/</t>
+          <t>https://www.infobae.com/colombia/deportes/2026/06/24/suiza-vs-canada-en-vivo-siga-el-minuto-a-minuto-del-partido-en-el-grupo-b-del-mundial-2026/</t>
         </is>
       </c>
     </row>
@@ -5281,12 +5281,12 @@
       </c>
       <c r="D187" s="6" t="inlineStr">
         <is>
-          <t>Investigan presunto intento de sicariato en Bucaramanga: dos heridos, entre ellos directivo de la Cámara de Comercio</t>
+          <t>“Es posible que lo esté haciendo”: misión de la UE cuestiona a Petro por señalamientos de fraude</t>
         </is>
       </c>
       <c r="E187" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/24/investigan-presunto-intento-de-sicariato-en-bucaramanga-dos-heridos-entre-ellos-directivo-de-la-camara-de-comercio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/24/es-posible-que-lo-este-haciendo-mision-de-la-ue-cuestiona-a-petro-por-senalamientos-de-fraude/</t>
         </is>
       </c>
     </row>
@@ -5308,12 +5308,12 @@
       </c>
       <c r="D188" s="3" t="inlineStr">
         <is>
-          <t>“Muy productiva”: De La Espriella y presidente de Panamá hablan de seguridad e inversión</t>
+          <t>Pasaporte con certificado electoral: así queda el precio con descuento del 10 % por votar</t>
         </is>
       </c>
       <c r="E188" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/24/muy-productiva-de-la-espriella-y-presidente-de-panama-hablan-de-seguridad-e-inversion/</t>
+          <t>https://www.infobae.com/colombia/2026/06/24/pasaporte-con-certificado-electoral-asi-queda-el-precio-con-descuento-del-10-por-votar/</t>
         </is>
       </c>
     </row>
@@ -5335,12 +5335,12 @@
       </c>
       <c r="D189" s="6" t="inlineStr">
         <is>
-          <t>Pico y Placa en Bogotá: qué automóviles no circulan este 24 de junio</t>
+          <t>Las últimas previsiones para Barranquilla: temperatura, lluvias y viento</t>
         </is>
       </c>
       <c r="E189" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/24/pico-y-placa-en-bogota-que-automoviles-no-circulan-este-24-de-junio/</t>
+          <t>https://www.infobae.com/colombia/2026/06/24/las-ultimas-previsiones-para-barranquilla-temperatura-lluvias-y-viento/</t>
         </is>
       </c>
     </row>
@@ -5362,12 +5362,12 @@
       </c>
       <c r="D190" s="3" t="inlineStr">
         <is>
-          <t>Shakira celebró el triunfo de Colombia ante República Democrática del Congo antes de su concierto</t>
+          <t>Conoce el clima de este día en Cali</t>
         </is>
       </c>
       <c r="E190" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/24/shakira-celebro-el-triunfo-de-colombia-ante-republica-democratica-del-congo-antes-de-su-concierto/</t>
+          <t>https://www.infobae.com/colombia/2026/06/24/conoce-el-clima-de-este-dia-en-cali/</t>
         </is>
       </c>
     </row>
@@ -5389,12 +5389,12 @@
       </c>
       <c r="D191" s="6" t="inlineStr">
         <is>
-          <t>Luis Díaz fue anulado por el arbitraje: le negaron dos goles en dos minutos</t>
+          <t>Las últimas previsiones para Bogotá: temperatura, lluvias y viento</t>
         </is>
       </c>
       <c r="E191" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/06/24/luis-diaz-fue-anulado-por-el-arbitraje-le-negaron-dos-goles-en-dos-minutos/</t>
+          <t>https://www.infobae.com/colombia/2026/06/24/las-ultimas-previsiones-para-bogota-temperatura-lluvias-y-viento/</t>
         </is>
       </c>
     </row>
@@ -5416,12 +5416,12 @@
       </c>
       <c r="D192" s="3" t="inlineStr">
         <is>
-          <t>Petro anuncia empalme con Abelardo de la Espriella, confirma su retirada y plantea “resistencia pacífica” tras la segunda vuelta presidencial</t>
+          <t>Clima en Medellín: el estado del tiempo para este 24 de junio</t>
         </is>
       </c>
       <c r="E192" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/24/petro-anuncia-empalme-con-abelardo-de-la-espriella-confirma-su-retirada-y-plantea-resistencia-pacifica-tras-la-segunda-vuelta-presidencial/</t>
+          <t>https://www.infobae.com/colombia/2026/06/24/clima-en-medellin-el-estado-del-tiempo-para-este-24-de-junio/</t>
         </is>
       </c>
     </row>
@@ -5443,12 +5443,12 @@
       </c>
       <c r="D193" s="6" t="inlineStr">
         <is>
-          <t>Néstor Lorenzo y los jugadores de la Selección Colombia reaccionaron tras vencer a RD Congo en el Mundial 2026: “Nadie nos regala nada”</t>
+          <t>Clima: las temperaturas que predominarán este 24 de junio en Cartagena de Indias</t>
         </is>
       </c>
       <c r="E193" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/06/24/nestor-lorenzo-y-los-jugadores-de-la-seleccion-colombia-reaccionaron-tras-vencer-a-rd-congo-en-el-mundial-2026-nadie-nos-regala-nada/</t>
+          <t>https://www.infobae.com/colombia/2026/06/24/clima-las-temperaturas-que-predominaran-este-24-de-junio-en-cartagena-de-indias/</t>
         </is>
       </c>
     </row>
@@ -5470,12 +5470,12 @@
       </c>
       <c r="D194" s="3" t="inlineStr">
         <is>
-          <t>“Reconozco como nuevo presidente a Abelardo de la Espriella”: Agmeth Escaf acepta derrota de Cepeda</t>
+          <t>Resultado Sinuano Noche hoy 23 de junio</t>
         </is>
       </c>
       <c r="E194" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/24/reconozco-como-nuevo-presidente-a-abelardo-de-la-espriella-agmeth-escaf-acepta-derrota-de-cepeda/</t>
+          <t>https://www.infobae.com/colombia/2026/06/24/resultado-sinuano-noche-hoy-23-de-junio/</t>
         </is>
       </c>
     </row>
@@ -5497,12 +5497,12 @@
       </c>
       <c r="D195" s="6" t="inlineStr">
         <is>
-          <t>De La Espriella propone ajuste fiscal: déficit de 4,8 % en 360 días y crecimiento de 5 %</t>
+          <t>Devolución automática de saldos a favor en renta 2026: paso a paso para solicitarla ante la Dian</t>
         </is>
       </c>
       <c r="E195" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/24/de-la-espriella-propone-ajuste-fiscal-deficit-de-48-en-360-dias-y-crecimiento-de-5/</t>
+          <t>https://www.infobae.com/colombia/2026/06/24/devolucion-automatica-de-saldos-a-favor-en-renta-2026-paso-a-paso-para-solicitarla-ante-la-dian/</t>
         </is>
       </c>
     </row>
@@ -5524,12 +5524,12 @@
       </c>
       <c r="D196" s="3" t="inlineStr">
         <is>
-          <t>Mesa Fiscal advierte crisis de finanzas públicas en Colombia y pide ajuste: deuda llegó a 58,5 % del PIB</t>
+          <t>Gobierno prorroga por cinco meses el contrato del Fondo Nacional del Café y deja nuevo acuerdo al próximo presidente</t>
         </is>
       </c>
       <c r="E196" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/24/mesa-fiscal-advierte-crisis-de-finanzas-publicas-en-colombia-y-pide-ajuste-deuda-llego-a-585-del-pib/</t>
+          <t>https://www.infobae.com/colombia/2026/06/24/gobierno-prorroga-por-cinco-meses-el-contrato-del-fondo-nacional-del-cafe-y-deja-nuevo-acuerdo-al-proximo-presidente/</t>
         </is>
       </c>
     </row>
@@ -5551,12 +5551,12 @@
       </c>
       <c r="D197" s="6" t="inlineStr">
         <is>
-          <t>Falsos policías secuestran a firmante de paz y sus hijos en Cauca: robaron camioneta de la UNP</t>
+          <t>Investigan presunto intento de sicariato en Bucaramanga: dos heridos, entre ellos directivo de la Cámara de Comercio</t>
         </is>
       </c>
       <c r="E197" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/24/falsos-policias-secuestran-a-firmante-de-paz-y-sus-hijos-en-cauca-robaron-camioneta-de-la-unp/</t>
+          <t>https://www.infobae.com/colombia/2026/06/24/investigan-presunto-intento-de-sicariato-en-bucaramanga-dos-heridos-entre-ellos-directivo-de-la-camara-de-comercio/</t>
         </is>
       </c>
     </row>
@@ -5578,12 +5578,12 @@
       </c>
       <c r="D198" s="3" t="inlineStr">
         <is>
-          <t>Colombia sufrió en Guadalajara, pero aseguró su tiquete a la segunda ronda en el Mundial 2026</t>
+          <t>“Muy productiva”: De La Espriella y presidente de Panamá hablan de seguridad e inversión</t>
         </is>
       </c>
       <c r="E198" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/06/24/colombia-sufrio-en-guadalajara-pero-aseguro-su-tiquete-a-la-segunda-ronda-en-el-mundial-2026/</t>
+          <t>https://www.infobae.com/colombia/2026/06/24/muy-productiva-de-la-espriella-y-presidente-de-panama-hablan-de-seguridad-e-inversion/</t>
         </is>
       </c>
     </row>
@@ -5605,12 +5605,12 @@
       </c>
       <c r="D199" s="6" t="inlineStr">
         <is>
-          <t>Resultados de la Lotería de la Cruz Roja martes 23 de junio: quién ganó el premio mayor de $7.000 millones</t>
+          <t>Pico y Placa en Bogotá: qué automóviles no circulan este 24 de junio</t>
         </is>
       </c>
       <c r="E199" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/24/resultados-de-la-loteria-de-la-cruz-roja-martes-23-de-junio-quien-gano-el-premio-mayor-de-7000-millones/</t>
+          <t>https://www.infobae.com/colombia/2026/06/24/pico-y-placa-en-bogota-que-automoviles-no-circulan-este-24-de-junio/</t>
         </is>
       </c>
     </row>
@@ -5632,12 +5632,12 @@
       </c>
       <c r="D200" s="3" t="inlineStr">
         <is>
-          <t>Estos son los mejores memes que dejó la victoria de la Selección Colombia ante RD Congo en el Mundial 2026</t>
+          <t>Shakira celebró el triunfo de Colombia ante República Democrática del Congo antes de su concierto</t>
         </is>
       </c>
       <c r="E200" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/06/24/estos-son-los-mejores-memes-que-dejo-la-victoria-de-la-seleccion-colombia-ante-rd-congo-en-el-mundial-2026/</t>
+          <t>https://www.infobae.com/colombia/2026/06/24/shakira-celebro-el-triunfo-de-colombia-ante-republica-democratica-del-congo-antes-de-su-concierto/</t>
         </is>
       </c>
     </row>
@@ -5659,12 +5659,12 @@
       </c>
       <c r="D201" s="6" t="inlineStr">
         <is>
-          <t>Resultado Super Astro Luna HOY: número ganador del martes 23 de junio</t>
+          <t>Luis Díaz fue anulado por el arbitraje: le negaron dos goles en dos minutos</t>
         </is>
       </c>
       <c r="E201" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/2026/06/24/resultado-super-astro-luna-hoy-numero-ganador-del-martes-23-de-junio/</t>
+          <t>https://www.infobae.com/colombia/deportes/2026/06/24/luis-diaz-fue-anulado-por-el-arbitraje-le-negaron-dos-goles-en-dos-minutos/</t>
         </is>
       </c>
     </row>
@@ -5686,12 +5686,12 @@
       </c>
       <c r="D202" s="3" t="inlineStr">
         <is>
-          <t>Este sería el próximo rival de la Selección Colombia en los dieciseisavos de final del Mundial 2026</t>
+          <t>Petro anuncia empalme con Abelardo de la Espriella, confirma su retirada y plantea “resistencia pacífica” tras la segunda vuelta presidencial</t>
         </is>
       </c>
       <c r="E202" s="4" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/colombia/deportes/2026/06/24/este-seria-el-proximo-rival-de-la-seleccion-colombia-en-los-dieciseisavos-de-final-del-mundial-2026/</t>
+          <t>https://www.infobae.com/colombia/2026/06/24/petro-anuncia-empalme-con-abelardo-de-la-espriella-confirma-su-retirada-y-plantea-resistencia-pacifica-tras-la-segunda-vuelta-presidencial/</t>
         </is>
       </c>
     </row>
@@ -5713,12 +5713,12 @@
       </c>
       <c r="D203" s="6" t="inlineStr">
         <is>
-          <t>Ahorrar en vacaciones 2026: cuáles son los destinos y meses más baratos para volar desde Colombia</t>
+          <t>Néstor Lorenzo y los jugadores de la Selección Colombia reaccionaron tras vencer a RD Congo en el Mundial 2026: “Nadie nos regala nada”</t>
         </is>
       </c>
       <c r="E203" s="7" t="inlineStr">
         <is>
-          <t>https://www.infobae.com/tecno/2026/06/24/ahorrar-en-vacaciones-2026-cuales-son-los-destinos-y-meses-mas-baratos-para-volar-desde-colombia/</t>
+          <t>https://www.infobae.com/colombia/deportes/2026/06/24/nestor-lorenzo-y-los-jugadores-de-la-seleccion-colombia-reaccionaron-tras-vencer-a-rd-congo-en-el-mundial-2026-nadie-nos-regala-nada/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 Noticias actualizadas 27/06/2026 11:07
</commit_message>
<xml_diff>
--- a/docs/ultimahora.xlsx
+++ b/docs/ultimahora.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Todas las noticias" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Todas las noticias'!$A$1:$E$252</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Todas las noticias'!$A$1:$E$255</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E252"/>
+  <dimension ref="A1:E255"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -515,7 +515,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>27/06/2026 05:03 a. m.</t>
+          <t>27/06/2026 05:54 a. m.</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -530,19 +530,19 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Movilidad Bogotá hoy sábado 27 de junio: plan éxodo para este puente festivo de San Pedro y San Pablo; se espera la salida de 1.251.588 vehículos</t>
+          <t>Elecciones presidenciales Colombia 2026: la primera dama, Verónica Alcocer, envió un mensaje al presidente electo del país, Abelardo de la Espriella</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/bogota/movilidad-bogota-hoy-sabado-27-de-junio-plan-exodo-para-este-puente-festivo-de-san-pedro-y-san-pablo-se-espera-la-salida-de-1-251-588-vehiculos-3567496</t>
+          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/elecciones-presidenciales-colombia-2026-la-primera-dama-veronica-alcocer-envio-un-mensaje-al-presidente-electo-del-pais-abelardo-de-la-espriella-3567498</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>27/06/2026 04:29 a. m.</t>
+          <t>27/06/2026 05:30 a. m.</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -557,19 +557,19 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>Marcelo Bielsa, técnico de Uruguay, se despide del Mundial con escándalo: gritó furioso a periodistas al final de la eliminación del equipo</t>
+          <t>Venezuela hoy 27 de junio tras terremotos que dejan 920 muertos: Delcy Rodríguez dice que la prioridad ahora es rescatar a las personas atrapadas</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/marcelo-bielsa-tecnico-de-uruguay-se-despide-del-mundial-con-escandalo-grito-furioso-a-periodistas-al-final-de-la-eliminacion-del-equipo-3567495</t>
+          <t>https://www.eltiempo.com/mundo/venezuela/venezuela-hoy-27-de-junio-tras-terremotos-que-dejan-920-muertos-delcy-rodriguez-dice-que-la-prioridad-ahora-es-rescatar-a-las-personas-atrapadas-3567497</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>27/06/2026 04:16 a. m.</t>
+          <t>27/06/2026 05:16 a. m.</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -584,19 +584,19 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>‘La Agencia’, la serie de espionaje que regresa con un elenco de primer nivel</t>
+          <t>La historia de amor de Anne Hathaway y su marido Adam Shulman: un flechazo inesperado que llegó en el peor momento de su vida</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/cultura/cine-y-tv/la-agencia-la-serie-de-espionaje-que-regresa-con-un-elenco-de-primer-nivel-3567125</t>
+          <t>https://www.eltiempo.com/cultura/entretenimiento/la-historia-de-amor-de-anne-hathaway-y-su-marido-adam-shulman-un-flechazo-inesperado-que-llego-en-el-peor-momento-de-su-vida-3567359</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>27/06/2026 03:15 a. m.</t>
+          <t>27/06/2026 05:03 a. m.</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -611,19 +611,19 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Cinco señales de que su celular ha sido hackeado</t>
+          <t>Movilidad Bogotá hoy sábado 27 de junio: plan éxodo para este puente festivo de San Pedro y San Pablo; se espera la salida de 1.251.588 vehículos</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/tecnosfera/cinco-senales-de-que-su-celular-ha-sido-hackeado-3567473</t>
+          <t>https://www.eltiempo.com/bogota/movilidad-bogota-hoy-sabado-27-de-junio-plan-exodo-para-este-puente-festivo-de-san-pedro-y-san-pablo-se-espera-la-salida-de-1-251-588-vehiculos-3567496</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>27/06/2026 02:46 a. m.</t>
+          <t>27/06/2026 04:29 a. m.</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -638,19 +638,19 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Así van las tablas de posiciones de los grupos en el Mundial de Estados Unidos, México y Canadá 2026</t>
+          <t>Marcelo Bielsa, técnico de Uruguay, se despide del Mundial con escándalo: gritó furioso a periodistas al final de la eliminación del equipo</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/asi-van-las-tablas-de-posiciones-de-los-grupos-en-el-mundial-de-estados-unidos-mexico-y-canada-3567476</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/marcelo-bielsa-tecnico-de-uruguay-se-despide-del-mundial-con-escandalo-grito-furioso-a-periodistas-al-final-de-la-eliminacion-del-equipo-3567495</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>27/06/2026 02:13 a. m.</t>
+          <t>27/06/2026 04:16 a. m.</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -665,19 +665,19 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Mentes creativas de ‘Toy Story 5’ profundizan sobre lo compleja que se ha vuelto la infancia: así ven la conexión entre juguetes y tecnología</t>
+          <t>‘La Agencia’, la serie de espionaje que regresa con un elenco de primer nivel</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/cultura/cine-y-tv/mentes-creativas-de-toy-story-5-profundizan-sobre-lo-compleja-que-se-ha-vuelto-la-infancia-asi-ven-la-conexion-entre-juguetes-y-tecnologia-3567393</t>
+          <t>https://www.eltiempo.com/cultura/cine-y-tv/la-agencia-la-serie-de-espionaje-que-regresa-con-un-elenco-de-primer-nivel-3567125</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>27/06/2026 02:01 a. m.</t>
+          <t>27/06/2026 03:15 a. m.</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -692,19 +692,19 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Guía legal para resolver la falta de constitución jurídica de copropiedades y para adaptar infraestructura de recarga de autos eléctricos</t>
+          <t>Cinco señales de que su celular ha sido hackeado</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/economia/finanzas-personales/guia-legal-para-resolver-la-falta-de-constitucion-juridica-de-copropiedades-y-para-adaptar-infraestructura-de-recarga-de-autos-electricos-3567264</t>
+          <t>https://www.eltiempo.com/tecnosfera/cinco-senales-de-que-su-celular-ha-sido-hackeado-3567473</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>27/06/2026 01:25 a. m.</t>
+          <t>27/06/2026 02:46 a. m.</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -719,19 +719,19 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Lo que está preparando la izquierda para hacerle oposición a Abelardo de la Espriella: así será el tono paa el cuatrenio</t>
+          <t>Así van las tablas de posiciones de los grupos en el Mundial de Estados Unidos, México y Canadá 2026</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/lo-que-esta-preparando-la-izquierda-para-hacerle-oposicion-a-abelardo-de-la-espriella-asi-sera-el-tono-paa-el-cuatrenio-3567493</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/asi-van-las-tablas-de-posiciones-de-los-grupos-en-el-mundial-de-estados-unidos-mexico-y-canada-3567476</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>27/06/2026 12:19 a. m.</t>
+          <t>27/06/2026 02:13 a. m.</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -746,19 +746,19 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Egipto empató, clasificó a dieciseisavos de final del Mundial 2026 y dejó a Irán con 'matrícula condicional'</t>
+          <t>Mentes creativas de ‘Toy Story 5’ profundizan sobre lo compleja que se ha vuelto la infancia: así ven la conexión entre juguetes y tecnología</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/egipto-empato-clasifico-a-dieciseisavos-de-final-del-mundial-2026-y-dejo-a-iran-con-matricula-condicional-3567491</t>
+          <t>https://www.eltiempo.com/cultura/cine-y-tv/mentes-creativas-de-toy-story-5-profundizan-sobre-lo-compleja-que-se-ha-vuelto-la-infancia-asi-ven-la-conexion-entre-juguetes-y-tecnologia-3567393</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>27/06/2026 12:07 a. m.</t>
+          <t>27/06/2026 02:01 a. m.</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -773,19 +773,19 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Bélgica liquida a Nueva Zelanda y termina primera de su grupo en el Mundial</t>
+          <t>Guía legal para resolver la falta de constitución jurídica de copropiedades y para adaptar infraestructura de recarga de autos eléctricos</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/belgica-liquida-a-nueva-zelanda-y-termina-primera-de-su-grupo-en-el-mundial-3567490</t>
+          <t>https://www.eltiempo.com/economia/finanzas-personales/guia-legal-para-resolver-la-falta-de-constitucion-juridica-de-copropiedades-y-para-adaptar-infraestructura-de-recarga-de-autos-electricos-3567264</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>26/06/2026 11:53 p. m.</t>
+          <t>27/06/2026 01:25 a. m.</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -800,19 +800,19 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Cartagena: tras casi dos décadas de espera, el Ministerio de Cultura aprobó el Plan de Protección para el Centro Histórico (PEMP)</t>
+          <t>Lo que está preparando la izquierda para hacerle oposición a Abelardo de la Espriella: así será el tono paa el cuatrenio</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/otras-ciudades/cartagena-tras-casi-dos-decadas-de-espera-el-ministerio-de-cultura-aprobo-el-plan-de-proteccion-para-el-centro-historico-pemp-3567483</t>
+          <t>https://www.eltiempo.com/politica/elecciones-colombia-2026/lo-que-esta-preparando-la-izquierda-para-hacerle-oposicion-a-abelardo-de-la-espriella-asi-sera-el-tono-paa-el-cuatrenio-3567493</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>26/06/2026 11:43 p. m.</t>
+          <t>27/06/2026 12:19 a. m.</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -827,19 +827,19 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Tomás Restrepo hizo historia: revalidó el título mundial juvenil de golf en Japón</t>
+          <t>Egipto empató, clasificó a dieciseisavos de final del Mundial 2026 y dejó a Irán con 'matrícula condicional'</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/otros-deportes/tomas-restrepo-hizo-historia-revalido-el-titulo-mundial-juvenil-de-golf-en-japon-3567489</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/egipto-empato-clasifico-a-dieciseisavos-de-final-del-mundial-2026-y-dejo-a-iran-con-matricula-condicional-3567491</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>26/06/2026 11:36 p. m.</t>
+          <t>27/06/2026 12:07 a. m.</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -854,19 +854,19 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>¡Colombia va por el batacazo contra Portugal y el liderato en su grupo en el Mundial!</t>
+          <t>Bélgica liquida a Nueva Zelanda y termina primera de su grupo en el Mundial</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/colombia-va-por-el-batacazo-contra-portugal-y-el-liderato-en-su-grupo-en-el-mundial-3567487</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/belgica-liquida-a-nueva-zelanda-y-termina-primera-de-su-grupo-en-el-mundial-3567490</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>26/06/2026 11:33 p. m.</t>
+          <t>26/06/2026 11:53 p. m.</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -881,19 +881,19 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Indignante: las monjas misioneras de la casa natal de Santa Laura Montoya en Jericó, Antioquia, fueron víctimas de un millonario robo</t>
+          <t>Cartagena: tras casi dos décadas de espera, el Ministerio de Cultura aprobó el Plan de Protección para el Centro Histórico (PEMP)</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/medellin/indignante-las-monjas-misioneras-de-la-casa-natal-de-santa-laura-montoya-en-jerico-antioquia-fueron-victimas-de-un-millonario-robo-3567488</t>
+          <t>https://www.eltiempo.com/colombia/otras-ciudades/cartagena-tras-casi-dos-decadas-de-espera-el-ministerio-de-cultura-aprobo-el-plan-de-proteccion-para-el-centro-historico-pemp-3567483</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>26/06/2026 11:20 p. m.</t>
+          <t>26/06/2026 11:43 p. m.</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -908,19 +908,19 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Terremoto en Venezuela, un 'cisne negro' que amenaza con frenar la lucha democrática, afirma experta de Wola</t>
+          <t>Tomás Restrepo hizo historia: revalidó el título mundial juvenil de golf en Japón</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/venezuela/terremoto-en-venezuela-un-cisne-negro-que-amenaza-con-frenar-la-lucha-democratica-afirma-experta-de-wola-3567418</t>
+          <t>https://www.eltiempo.com/deportes/otros-deportes/tomas-restrepo-hizo-historia-revalido-el-titulo-mundial-juvenil-de-golf-en-japon-3567489</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>26/06/2026 11:20 p. m.</t>
+          <t>26/06/2026 11:36 p. m.</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -935,19 +935,19 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>'No sabía nada sobre mi familia': bloqueo al internet y acceso a la información agravan la tragedia por terremotos en Venezuela</t>
+          <t>¡Colombia va por el batacazo contra Portugal y el liderato en su grupo en el Mundial!</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/venezuela/no-sabia-nada-sobre-mi-familia-bloqueo-al-internet-y-acceso-a-la-informacion-agravan-la-tragedia-por-terremotos-en-venezuela-3567034</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/colombia-va-por-el-batacazo-contra-portugal-y-el-liderato-en-su-grupo-en-el-mundial-3567487</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>26/06/2026 11:18 p. m.</t>
+          <t>26/06/2026 11:33 p. m.</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -962,19 +962,19 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>En el corazón del banderazo de los hinchas de la Selección Colombia en Fort Lauderdale: ríos de aguardiente, amor y fe</t>
+          <t>Indignante: las monjas misioneras de la casa natal de Santa Laura Montoya en Jericó, Antioquia, fueron víctimas de un millonario robo</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/en-el-corazon-del-banderazo-de-los-hinchas-de-la-seleccion-colombia-en-fort-lauderdale-rios-de-aguardiente-amor-y-fe-3567484</t>
+          <t>https://www.eltiempo.com/colombia/medellin/indignante-las-monjas-misioneras-de-la-casa-natal-de-santa-laura-montoya-en-jerico-antioquia-fueron-victimas-de-un-millonario-robo-3567488</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>26/06/2026 11:16 p. m.</t>
+          <t>26/06/2026 11:20 p. m.</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -989,19 +989,19 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>El contrato y la supuesta identidad falsa de británico capturado por muerte de Natalia Villalba: razón por la que víctima estaba en lujoso apartamento</t>
+          <t>Terremoto en Venezuela, un 'cisne negro' que amenaza con frenar la lucha democrática, afirma experta de Wola</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/bogota/el-contrato-y-la-supuesta-identidad-falsa-de-britanico-capturado-por-muerte-de-natalia-villalba-razon-por-la-que-victima-estaba-en-lujoso-apartamento-3567486</t>
+          <t>https://www.eltiempo.com/mundo/venezuela/terremoto-en-venezuela-un-cisne-negro-que-amenaza-con-frenar-la-lucha-democratica-afirma-experta-de-wola-3567418</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>26/06/2026 11:16 p. m.</t>
+          <t>26/06/2026 11:20 p. m.</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1016,19 +1016,19 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Vozinha y Cabo Verde hacen historia: clasifican en el Mundial y ahora van por un reto mayor contra la Argentina de Messi</t>
+          <t>'No sabía nada sobre mi familia': bloqueo al internet y acceso a la información agravan la tragedia por terremotos en Venezuela</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/vozinha-y-cabo-verde-hacen-historia-clasifican-en-el-mundial-y-ahora-van-por-un-reto-mayor-contra-la-argentina-de-messi-3567485</t>
+          <t>https://www.eltiempo.com/mundo/venezuela/no-sabia-nada-sobre-mi-familia-bloqueo-al-internet-y-acceso-a-la-informacion-agravan-la-tragedia-por-terremotos-en-venezuela-3567034</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>26/06/2026 10:58 p. m.</t>
+          <t>26/06/2026 11:18 p. m.</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
@@ -1043,12 +1043,12 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Tras cinco horas retenidos, el Gobierno de Venezuela autorizó el ingreso de los bomberos de Medellín para apoyar en la emergencia tras los terremotos</t>
+          <t>En el corazón del banderazo de los hinchas de la Selección Colombia en Fort Lauderdale: ríos de aguardiente, amor y fe</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/medellin/gobierno-de-venezuela-no-ha-dejado-entrar-a-la-escuadrilla-de-bomberos-de-medellin-que-viajaron-a-apoyar-tras-los-terremotos-federico-gutierrez-3567481</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/en-el-corazon-del-banderazo-de-los-hinchas-de-la-seleccion-colombia-en-fort-lauderdale-rios-de-aguardiente-amor-y-fe-3567484</t>
         </is>
       </c>
     </row>
@@ -2123,7 +2123,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>27/06/2026 05:16 a. m.</t>
+          <t>27/06/2026 06:06 a. m.</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -2138,19 +2138,19 @@
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Ludopatía crece 23% en el Valle de Aburrá: ¿una pandemia silenciosa?</t>
+          <t>Lo que le espera a Rodrigo Lara como ministro al armar la coalición de De la Espriella en el Congreso</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/antioquia/ludopatia-crece-valle-de-aburra-apuestas-deportivas-FM38256366</t>
+          <t>https://www.elcolombiano.com/colombia/rodrigo-lara-ministro-interior-abelardo-de-la-espriella-IM38254590</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>27/06/2026 12:16 a. m.</t>
+          <t>27/06/2026 05:06 a. m.</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
@@ -2165,35 +2165,39 @@
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
+          <t>Ludopatía crece 23% en el Valle de Aburrá: ¿una pandemia silenciosa?</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>https://www.elcolombiano.com/antioquia/ludopatia-crece-valle-de-aburra-apuestas-deportivas-FM38256366</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>27/06/2026 12:06 a. m.</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Medio de Comunicación</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>El Colombiano</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
           <t>Comiendo por Colombia: y bebiendo</t>
         </is>
       </c>
-      <c r="E63" s="7" t="inlineStr">
+      <c r="E64" s="4" t="inlineStr">
         <is>
           <t>https://www.elcolombiano.com/cultura/gastronomia/comiendo-por-colombia-y-bebiendo-FM38254221</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr"/>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>Medio de Comunicación</t>
-        </is>
-      </c>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t>El Colombiano</t>
-        </is>
-      </c>
-      <c r="D64" s="3" t="inlineStr">
-        <is>
-          <t>El ‘juicio’ de la Paz Total: ¿hasta dónde puede llegar De la Espriella para desmontarla?</t>
-        </is>
-      </c>
-      <c r="E64" s="4" t="inlineStr">
-        <is>
-          <t>https://www.elcolombiano.com/colombia/los-caminos-de-abelardo-para-tumbar-la-paz-total-gustavo-petro-IL38229625</t>
         </is>
       </c>
     </row>
@@ -2211,12 +2215,12 @@
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>Video | Con la mamá de Vozinha en la tribuna: La emocionante celebración de Cabo Verde tras clasificar a 16avos en el Mundial</t>
+          <t>El ‘juicio’ de la Paz Total: ¿hasta dónde puede llegar De la Espriella para desmontarla?</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/mundial-2026/video-celebracion-hinchas-cabo-verde-mama-vozinha-clasificacion-mundial-2026-EM38257928</t>
+          <t>https://www.elcolombiano.com/colombia/los-caminos-de-abelardo-para-tumbar-la-paz-total-gustavo-petro-IL38229625</t>
         </is>
       </c>
     </row>
@@ -2234,12 +2238,12 @@
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Uruguay perdió con España en Guadalajara y es el único equipo Suramericano eliminado en fase de grupos</t>
+          <t>Video | Con la mamá de Vozinha en la tribuna: La emocionante celebración de Cabo Verde tras clasificar a 16avos en el Mundial</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/mundial-2026/seleccion-uruguay-vs-espana-mundial-2026-eliminada-fase-de-grupos-GM38257463</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/video-celebracion-hinchas-cabo-verde-mama-vozinha-clasificacion-mundial-2026-EM38257928</t>
         </is>
       </c>
     </row>
@@ -2257,12 +2261,12 @@
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>Video | Así fue el banderazo de los hinchas de Colombia en Miami antes del partido con Portugal</t>
+          <t>Uruguay perdió con España en Guadalajara y es el único equipo Suramericano eliminado en fase de grupos</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/mundial-2026/seleccion-colombia-vs-portugal-mundial-2026-banderazo-hinchas-miami-hotel-dalmar-NM38255091</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/seleccion-uruguay-vs-espana-mundial-2026-eliminada-fase-de-grupos-GM38257463</t>
         </is>
       </c>
     </row>
@@ -2280,12 +2284,12 @@
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>¿Estados Unidos apretó a Petro?</t>
+          <t>Video | Así fue el banderazo de los hinchas de Colombia en Miami antes del partido con Portugal</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/multimedia/videos/estados-unidos-apreto-a-petro-GN38245344</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/seleccion-colombia-vs-portugal-mundial-2026-banderazo-hinchas-miami-hotel-dalmar-NM38255091</t>
         </is>
       </c>
     </row>
@@ -2303,12 +2307,12 @@
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>Imágenes satelitales muestran cómo quedó Venezuela tras el terremoto, ¿por qué La Guaira resultó tan afectada?</t>
+          <t>¿Estados Unidos apretó a Petro?</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/internacional/la-guaira-terremoto-tragedia-de-vargas-desastres-naturales-CI38219795</t>
+          <t>https://www.elcolombiano.com/multimedia/videos/estados-unidos-apreto-a-petro-GN38245344</t>
         </is>
       </c>
     </row>
@@ -2326,12 +2330,12 @@
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>Video | Con triplete, Dembelé igualó un registro que solo tenía Messi en el Mundial y Francia venció 4-1 a Noruega</t>
+          <t>Imágenes satelitales muestran cómo quedó Venezuela tras el terremoto, ¿por qué La Guaira resultó tan afectada?</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/especiales/mundial-2026/ousmane-dembele-triplete-seleccion-francia-vs-noruega-PN38242049</t>
+          <t>https://www.elcolombiano.com/internacional/la-guaira-terremoto-tragedia-de-vargas-desastres-naturales-CI38219795</t>
         </is>
       </c>
     </row>
@@ -2349,12 +2353,12 @@
       </c>
       <c r="D71" s="6" t="inlineStr">
         <is>
-          <t>Cronología: así el Gobierno Petro se acercó al Clan del Golfo para darle ‘gabelas’ hasta suspender traslado de sus miembros</t>
+          <t>Video | Con triplete, Dembelé igualó un registro que solo tenía Messi en el Mundial y Francia venció 4-1 a Noruega</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>https://www.elcolombiano.com/colombia/proceso-paz-total-clan-del-golfo-gobierno-gustavo-petro-cronologia-GL38228358</t>
+          <t>https://www.elcolombiano.com/especiales/mundial-2026/ousmane-dembele-triplete-seleccion-francia-vs-noruega-PN38242049</t>
         </is>
       </c>
     </row>
@@ -2821,7 +2825,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>27/06/2026 03:16 a. m.</t>
+          <t>27/06/2026 05:53 a. m.</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -2831,24 +2835,24 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>Las voces de la tragedia: colombianos relatan el terror que aún se vive en Venezuela</t>
+          <t>Así rige este sábado, 27 de junio, el pico y placa en Bucaramanga y el área</t>
         </is>
       </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/mundo/articulo/las-voces-de-la-tragedia-colombianos-relatan-el-terror-que-aun-se-vive-en-venezuela/202616/</t>
+          <t>https://www.vanguardia.com/area-metropolitana/bucaramanga/2026/06/27/asi-rige-este-sabado-27-de-junio-el-pico-y-placa-en-bucaramanga-y-el-area/</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>27/06/2026 02:16 a. m.</t>
+          <t>27/06/2026 05:53 a. m.</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
@@ -2858,24 +2862,24 @@
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D93" s="6" t="inlineStr">
         <is>
-          <t>Keiko Fujimori triunfa en Perú y América Latina consolida el giro a la derecha, en medio de denuncias de fraude y silencios de la izquierda</t>
+          <t>Bucaramanga</t>
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/mundo/articulo/keiko-fujimori-triunfa-en-peru-y-america-latina-consolida-el-giro-a-la-derecha-en-medio-de-denuncias-de-fraude-y-silencios-de-la-izquierda/202615/</t>
+          <t>https://www.vanguardia.com/area-metropolitana/bucaramanga/</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>27/06/2026 02:16 a. m.</t>
+          <t>27/06/2026 01:51 a. m.</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -2885,24 +2889,24 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>“No quiero ser Shakira, ni Carlos Vives”: Guillo Vives habla de su música, su familia y la relación con su hermano</t>
+          <t>Raúl Gómez Jattin y las mujeres (1)</t>
         </is>
       </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/gente/articulo/no-quiero-ser-shakira-ni-carlos-vives-guillo-vives-habla-de-su-musica-su-familia-y-la-relacion-con-su-hermano/202618/</t>
+          <t>https://www.vanguardia.com/entretenimiento/cultura/magazin-cultural/2026/06/27/raul-gomez-jattin-y-las-mujeres-1/</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>27/06/2026 02:16 a. m.</t>
+          <t>27/06/2026 01:51 a. m.</t>
         </is>
       </c>
       <c r="B95" s="5" t="inlineStr">
@@ -2912,24 +2916,24 @@
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D95" s="6" t="inlineStr">
         <is>
-          <t>Denuncia por presunto maltrato laboral sacude a Hocol: alta funcionaria señala al presidente por “hostigamiento” y “humillación” en público</t>
+          <t>Magazín cultural</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/denuncia-por-presunto-maltrato-laboral-sacude-a-hocol-alta-funcionaria-senala-al-presidente-por-hostigamiento-y-humillacion-en-publico/202644/</t>
+          <t>https://www.vanguardia.com/entretenimiento/cultura/magazin-cultural/</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>27/06/2026 02:16 a. m.</t>
+          <t>27/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -2939,24 +2943,24 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>Líder de la primera línea estaría dando instrucciones de “incendiar al país” tras la victoria de Abelardo De La Espriella</t>
+          <t>Más armas, menos Estado</t>
         </is>
       </c>
       <c r="E96" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/lider-de-la-primera-linea-estaria-dando-instrucciones-de-incendiar-al-pais-tras-la-victoria-de-abelardo-de-la-espriella/202602/</t>
+          <t>https://www.vanguardia.com/opinion/editorial/2026/06/27/mas-armas-menos-estado/</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>27/06/2026 02:16 a. m.</t>
+          <t>27/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B97" s="5" t="inlineStr">
@@ -2966,24 +2970,24 @@
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D97" s="6" t="inlineStr">
         <is>
-          <t>Exclusivo: SEMANA revela la denuncia por acoso sexual contra el representante Carlos Carreño, exmiembro de las Farc. “Me tocaba las nalgas”</t>
+          <t>Editorial</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/exclusivo-semana-revela-la-denuncia-por-acoso-sexual-contra-el-representante-carlos-carreno-exmiembro-de-las-farc-me-tocaba-las-nalgas/202613/</t>
+          <t>https://www.vanguardia.com/opinion/editorial/</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>27/06/2026 02:16 a. m.</t>
+          <t>27/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -2993,24 +2997,24 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>El FBI está al frente del caso del estadounidense acusado falsamente de abusar de menores de edad en Bogotá. Esta es la historia</t>
+          <t>La arquitectura invisible del mundo</t>
         </is>
       </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/el-fbi-esta-al-frente-del-caso-del-estadounidense-acusado-falsamente-de-abusar-de-menores-de-edad-en-bogota-esta-es-la-historia/202608/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/2026/06/27/la-arquitectura-invisible-del-mundo/</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="5" t="inlineStr">
         <is>
-          <t>27/06/2026 02:16 a. m.</t>
+          <t>27/06/2026 01:00 a. m.</t>
         </is>
       </c>
       <c r="B99" s="5" t="inlineStr">
@@ -3020,24 +3024,24 @@
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D99" s="6" t="inlineStr">
         <is>
-          <t>Rodrigo Lara alerta contratación exprés y anuncia bloque de búsqueda anticorrupción: “No habrá acuerdos burocráticos, oscuros o transaccionales”</t>
+          <t>Columnistas</t>
         </is>
       </c>
       <c r="E99" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/rodrigo-lara-alerta-contratacion-expres-y-anuncia-bloque-de-busqueda-anticorrupcion-no-habra-acuerdos-burocraticos-oscuros-o-transaccionales/202635/</t>
+          <t>https://www.vanguardia.com/opinion/columnistas/</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>27/06/2026 02:16 a. m.</t>
+          <t>26/06/2026 10:02 p. m.</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -3047,24 +3051,24 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>“No dañemos amistades por las elecciones”: el médico Santiago Rojas habla de la polarización y el duelo, y le da consejos a De la Espriella, Petro y Cepeda</t>
+          <t>Capturan en Ecuador al principal sospechoso del feminicidio de Natalia Villalba en Bogotá</t>
         </is>
       </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/no-danemos-amistades-por-las-elecciones-el-medico-santiago-rojas-habla-de-la-polarizacion-y-el-duelo-y-le-da-consejos-a-de-la-espriella-petro-y-cepeda/202614/</t>
+          <t>https://www.vanguardia.com/judicial/2026/06/26/capturan-en-ecuador-al-principal-sospechoso-del-feminicidio-de-natalia-villalba-en-bogota/</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>27/06/2026 02:16 a. m.</t>
+          <t>26/06/2026 10:02 p. m.</t>
         </is>
       </c>
       <c r="B101" s="5" t="inlineStr">
@@ -3074,24 +3078,24 @@
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D101" s="6" t="inlineStr">
         <is>
-          <t>Magnicidio de Miguel Uribe Turbay: SEMANA revela la declaración de alias Chipi. Contó poco y dejó ver una confianza con la fiscal. “¡Piénsame mucho!”</t>
+          <t>Judicial</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/magnicidio-de-miguel-uribe-turbay-semana-revela-la-declaracion-de-alias-chipi-conto-poco-y-dejo-ver-una-confianza-con-la-fiscal-piensame-mucho/202642/</t>
+          <t>https://www.vanguardia.com/judicial/</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>27/06/2026 02:16 a. m.</t>
+          <t>26/06/2026 08:14 p. m.</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -3101,24 +3105,24 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>Abelardo De La Espriella tendría mayorías en el Congreso para tramitar sus reformas. Esta será la estrategia para sacar adelante sus propuestas</t>
+          <t>Se cae el puente festivo: ley deja sin el descanso que esperaban millones de colombianos en 2026</t>
         </is>
       </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/abelardo-de-la-espriella-tendria-mayorias-en-el-congreso-para-tramitar-sus-reformas-esta-sera-la-estrategia-para-sacar-adelante-sus-propuestas/202611/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/26/se-cae-el-puente-festivo-ley-deja-sin-el-descanso-que-esperaban-millones-de-colombianos-en-2026/</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>27/06/2026 02:16 a. m.</t>
+          <t>26/06/2026 08:14 p. m.</t>
         </is>
       </c>
       <c r="B103" s="5" t="inlineStr">
@@ -3128,24 +3132,24 @@
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D103" s="6" t="inlineStr">
         <is>
-          <t>Colombia vs. Portugal, el partido más esperado: la Selección afronta su reto más fuerte en la cita mundialista contra Cristiano Ronaldo</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E103" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/colombia-vs-portugal-el-partido-mas-esperado-la-seleccion-afronta-su-reto-mas-fuerte-en-la-cita-mundialista-contra-cristiano-ronaldo/202621/</t>
+          <t>https://www.vanguardia.com/colombia/</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>27/06/2026 02:16 a. m.</t>
+          <t>26/06/2026 07:40 p. m.</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
@@ -3155,24 +3159,24 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>Feminicidio de Natalia Villalba: El señalado asesino compartió con ella durante dos horas en un apartamento en el norte de Bogotá</t>
+          <t>Niegan casa por cárcel a Walter Martínez investigado por red de contrabando vinculada a Lili Pink</t>
         </is>
       </c>
       <c r="E104" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/feminicidio-de-natalia-villalba-el-senalado-asesino-compartio-con-ella-durante-dos-horas-en-un-apartamento-en-el-norte-de-bogota/202614/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/26/niegan-casa-por-carcel-a-walter-martinez-investigado-por-red-de-contrabando-vinculada-a-lili-pink/</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>27/06/2026 02:16 a. m.</t>
+          <t>26/06/2026 06:32 p. m.</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
@@ -3182,24 +3186,24 @@
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D105" s="6" t="inlineStr">
         <is>
-          <t>Los detalles inéditos del paso de Abelardo De La Espriella por la Universidad Sergio Arboleda: buenas calificaciones en su maestría en derecho. Hablan los docentes</t>
+          <t>Gobierno pidió la renuncia del presidente de Fiduprevisora en medio de nueva crisis política</t>
         </is>
       </c>
       <c r="E105" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/los-detalles-ineditos-del-paso-de-abelardo-de-la-espriella-por-la-universidad-sergio-arboleda-buenas-calificaciones-en-su-maestria-en-derecho-hablan-los-docentes/202627/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/26/gobierno-pidio-la-renuncia-del-presidente-de-fiduprevisora-en-medio-de-nueva-crisis-politica/</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>27/06/2026 02:16 a. m.</t>
+          <t>26/06/2026 05:04 p. m.</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
@@ -3209,24 +3213,24 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D106" s="3" t="inlineStr">
         <is>
-          <t>El gabinete de Abelardo De La Espriella: SEMANA revela el listado de algunas personas que podrían conformar el nuevo Gobierno</t>
+          <t>Jaime Andrés Beltrán sería el ministro de Vivienda en el Gobierno de Abelardo De La Espriella</t>
         </is>
       </c>
       <c r="E106" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/el-gabinete-de-abelardo-de-la-espriella-semana-revela-el-listado-de-algunas-personas-que-podrian-conformar-el-nuevo-gobierno/202621/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/26/jaime-andres-beltran-sera-el-ministro-de-vivienda-en-el-gobierno-de-abelardo-de-la-espriella/</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>27/06/2026 02:16 a. m.</t>
+          <t>26/06/2026 04:21 p. m.</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
@@ -3236,24 +3240,24 @@
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D107" s="6" t="inlineStr">
         <is>
-          <t>Venezuela, qué dolor… Delcy Rodríguez recibe el apoyo del mundo para atender la tragedia ocasionada por los dos terremotos. Reportaje desde Caracas y La Guaira</t>
+          <t>Petro felicitó a De La Espriella, pero lanzó un comentario: “La supo hacer bien”</t>
         </is>
       </c>
       <c r="E107" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/mundo/articulo/venezuela-que-dolor-delcy-rodriguez-recibe-el-apoyo-del-mundo-para-atender-la-tragedia-ocasionada-por-los-dos-terremotos-reportaje-desde-caracas-y-la-guaira/202615/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/26/petro-felicito-a-de-la-espriella-pero-lanzo-un-comentario-la-supo-hacer-bien/</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>27/06/2026 01:16 a. m.</t>
+          <t>26/06/2026 04:13 p. m.</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
@@ -3263,24 +3267,24 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D108" s="3" t="inlineStr">
         <is>
-          <t>Unidos por Venezuela: así ha sido la avalancha de solidaridad internacional con el vecino país</t>
+          <t>Si los audios son reales habría delito advierte Mindefensa por caso Danilo Rueda</t>
         </is>
       </c>
       <c r="E108" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/mundo/articulo/unidos-por-venezuela-asi-ha-sido-la-avalancha-de-solidaridad-internacional-con-el-vecino-pais/202624/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/26/si-los-audios-son-reales-habria-delito-advierte-mindefensa-por-caso-danilo-rueda/</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>27/06/2026 01:16 a. m.</t>
+          <t>26/06/2026 03:45 p. m.</t>
         </is>
       </c>
       <c r="B109" s="5" t="inlineStr">
@@ -3290,22 +3294,26 @@
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D109" s="6" t="inlineStr">
         <is>
-          <t>Se acaba la paz total: Abelardo De La Espriella solo tendrá dos caminos para los grupos criminales</t>
+          <t>Al menos 51 menores fueron reclutados por grupos armados en Colombia durante 2026</t>
         </is>
       </c>
       <c r="E109" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/se-acaba-la-paz-total-abelardo-de-la-espriella-solo-tendra-dos-caminos-para-los-grupos-criminales/202630/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/26/al-menos-51-menores-fueron-reclutados-por-grupos-armados-en-colombia-durante-2026/</t>
         </is>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="2" t="inlineStr"/>
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>26/06/2026 03:41 p. m.</t>
+        </is>
+      </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3313,22 +3321,26 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D110" s="3" t="inlineStr">
         <is>
-          <t>Presupuesto 2027 se alista para salir al ruedo, hecho por el gobierno saliente para que lo defienda el entrante</t>
+          <t>Gustavo Petro dice que está listo para entregar el Gobierno a Abelardo de la Espriella</t>
         </is>
       </c>
       <c r="E110" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/economia/macroeconomia/articulo/presupuesto-2027-se-alista-para-salir-al-ruedo-hecho-por-el-gobierno-saliente-para-que-lo-defienda-el-entrante/202600/</t>
+          <t>https://www.vanguardia.com/colombia/2026/06/26/gustavo-petro-dice-que-esta-listo-para-entregar-el-gobierno-a-abelardo-de-la-espriella/</t>
         </is>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="5" t="inlineStr"/>
+      <c r="A111" s="5" t="inlineStr">
+        <is>
+          <t>26/06/2026 02:47 p. m.</t>
+        </is>
+      </c>
       <c r="B111" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3336,22 +3348,26 @@
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D111" s="6" t="inlineStr">
         <is>
-          <t>El registrador Hernán Penagos escribió una carta a los colombianos tras las elecciones. El funcionario fue ferozmente atacado por Gustavo Petro</t>
+          <t>¿Su celular puede avisarle antes de un terremoto? Así activar las alertas en Android y qué hacer en iPhone</t>
         </is>
       </c>
       <c r="E111" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/el-registrador-hernan-penagos-escribio-una-carta-a-los-colombianos-tras-las-elecciones-el-funcionario-fue-ferozmente-atacado-por-gustavo-petro/202635/</t>
+          <t>https://www.vanguardia.com/mundo/tecnologia/2026/06/26/su-celular-puede-avisarle-antes-de-un-terremoto-asi-puede-activar-las-alertas-en-android-y-que-hacer-si-tiene-iphone/</t>
         </is>
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="2" t="inlineStr"/>
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>26/06/2026 02:47 p. m.</t>
+        </is>
+      </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3359,22 +3375,26 @@
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Vanguardia</t>
         </is>
       </c>
       <c r="D112" s="3" t="inlineStr">
         <is>
-          <t>Iván Cepeda será el líder de la oposición en el Congreso, con el apoyo de Gustavo Petro como expresidente</t>
+          <t>Tecnología</t>
         </is>
       </c>
       <c r="E112" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/ivan-cepeda-sera-el-lider-de-la-oposicion-en-el-congreso-con-el-apoyo-de-gustavo-petro-como-expresidente/202649/</t>
+          <t>https://www.vanguardia.com/mundo/tecnologia/</t>
         </is>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="5" t="inlineStr"/>
+      <c r="A113" s="5" t="inlineStr">
+        <is>
+          <t>27/06/2026 03:09 a. m.</t>
+        </is>
+      </c>
       <c r="B113" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3382,22 +3402,26 @@
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D113" s="6" t="inlineStr">
         <is>
-          <t>El llamado “voto fusil”: estas son las zonas donde los grupos armados habrían intimidado a los colombianos para votar</t>
+          <t>Resultados de MiLoto del viernes 26 de junio de 2026</t>
         </is>
       </c>
       <c r="E113" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/el-llamado-voto-fusil-estas-son-las-zonas-donde-los-grupos-armados-habrian-intimidado-a-los-colombianos-para-votar/202659/</t>
+          <t>https://www.bluradio.com/economia/juegos-de-azar/resultados-de-miloto-del-viernes-26-de-junio-de-2026-so35</t>
         </is>
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="2" t="inlineStr"/>
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>27/06/2026 02:59 a. m.</t>
+        </is>
+      </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3405,22 +3429,26 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D114" s="3" t="inlineStr">
         <is>
-          <t>La puerta giratoria de Andrés Felipe Harmán: así fue la campaña del exdirector de la ANT en los municipios donde la agencia entregó tierras</t>
+          <t>Lotería de Risaralda, resultados del viernes 26 de junio de 2026</t>
         </is>
       </c>
       <c r="E114" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/la-puerta-giratoria-de-andres-felipe-harman-asi-fue-la-campana-del-exdirector-de-la-ant-en-los-municipios-donde-la-agencia-entrego-tierras/202631/</t>
+          <t>https://www.bluradio.com/economia/juegos-de-azar/loteria-de-risaralda-resultados-del-viernes-26-de-junio-de-2026-so35</t>
         </is>
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="5" t="inlineStr"/>
+      <c r="A115" s="5" t="inlineStr">
+        <is>
+          <t>27/06/2026 02:57 a. m.</t>
+        </is>
+      </c>
       <c r="B115" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3428,22 +3456,26 @@
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D115" s="6" t="inlineStr">
         <is>
-          <t>¿Está Colombia realmente preparada para un terremoto de gran magnitud? Esto dice el director de la UNGRD</t>
+          <t>Lotería de Santander, resultados del viernes 26 de junio de 2026</t>
         </is>
       </c>
       <c r="E115" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/articulo/esta-colombia-realmente-preparada-para-un-terremoto-de-gran-magnitud-esto-dice-el-director-de-la-ungrd/202613/</t>
+          <t>https://www.bluradio.com/economia/juegos-de-azar/loteria-de-santander-resultados-del-viernes-26-de-junio-de-2026-so35</t>
         </is>
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="2" t="inlineStr"/>
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>27/06/2026 02:52 a. m.</t>
+        </is>
+      </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3451,22 +3483,26 @@
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D116" s="3" t="inlineStr">
         <is>
-          <t>SuperTransporte sanciona a empresa por accidente de bus en La Línea; iban estudiantes y docentes, 10 murieron</t>
+          <t>Lotería de Medellín, resultado del viernes 26 de junio</t>
         </is>
       </c>
       <c r="E116" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/vehiculos/articulo/supertransporte-sanciona-a-empresa-por-accidente-de-bus-en-la-linea-iban-estudiantes-y-docentes-10-murieron/202659/</t>
+          <t>https://www.bluradio.com/economia/juegos-de-azar/loteria-de-medellin-resultado-del-viernes-26-de-junio-so35</t>
         </is>
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="5" t="inlineStr"/>
+      <c r="A117" s="5" t="inlineStr">
+        <is>
+          <t>26/06/2026 11:05 p. m.</t>
+        </is>
+      </c>
       <c r="B117" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3474,22 +3510,26 @@
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D117" s="6" t="inlineStr">
         <is>
-          <t>Detalles del intento de bloqueo promovieron vándalos en Cali con supuestos apoyos de estructuras armadas. La ciudad está en alerta</t>
+          <t>¿Dónde ver el partido Colombia vs. Portugal en Bogotá? Planes gratuitos para apoyar a la Tricolor</t>
         </is>
       </c>
       <c r="E117" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/cali/articulo/detalles-del-intento-de-bloqueo-promovieron-vandalos-en-cali-con-supuestos-apoyos-de-estructuras-armadas-la-ciudad-esta-en-alerta/202655/</t>
+          <t>https://www.bluradio.com/regiones/bogota/donde-ver-el-partido-colombia-vs-portugal-en-bogota-planes-gratuitos-para-apoyar-a-la-tricolor-so35</t>
         </is>
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="2" t="inlineStr"/>
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>26/06/2026 10:36 p. m.</t>
+        </is>
+      </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3497,22 +3537,26 @@
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D118" s="3" t="inlineStr">
         <is>
-          <t>Estos tres departamentos son los bastiones electorales de Abelardo De La Espriella: su votación fue arrolladora y ya plantean una fuerza política local</t>
+          <t>Bomberos de Medellín que apoyarán labores de rescate no han podido entrar a Venezuela</t>
         </is>
       </c>
       <c r="E118" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/politica/articulo/estos-tres-departamentos-son-los-bastiones-electorales-de-abelardo-de-la-espriella-su-votacion-fue-arrolladora-y-ya-plantean-una-fuerza-politica-local/202616/</t>
+          <t>https://www.bluradio.com/regiones/antioquia/bomberos-de-medellin-que-apoyaran-labores-de-rescate-no-han-podido-entrar-a-venezuela-rg10</t>
         </is>
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="5" t="inlineStr"/>
+      <c r="A119" s="5" t="inlineStr">
+        <is>
+          <t>26/06/2026 09:42 p. m.</t>
+        </is>
+      </c>
       <c r="B119" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3520,22 +3564,26 @@
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D119" s="6" t="inlineStr">
         <is>
-          <t>Las movidas políticas en el Atlántico tras el triunfo de Abelardo De La Espriella: hay promesas de apoyo para disputas por alcaldías y Gobernación</t>
+          <t>Uruguay, eliminada del Mundial 2026 tras una dura derrota contra España</t>
         </is>
       </c>
       <c r="E119" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/nacion/barranquilla/articulo/las-movidas-politicas-en-el-atlantico-tras-el-triunfo-de-abelardo-de-la-espriella-hay-promesas-de-apoyo-para-disputas-por-alcaldias-y-gobernacion/202653/</t>
+          <t>https://www.bluradio.com/deportes/futbol/copa-mundial-de-la-fifa-2026/uruguay-vs-espana-en-vivo-por-el-mundial-2026-vea-gratis-y-online-el-partido-rg10</t>
         </is>
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="2" t="inlineStr"/>
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>26/06/2026 09:39 p. m.</t>
+        </is>
+      </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3543,22 +3591,26 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D120" s="3" t="inlineStr">
         <is>
-          <t>Canal y hora para ver los últimos partidos de la fase de grupos del Mundial 2026: Colombia, Inglaterra y más</t>
+          <t>Vladimir Putin y líderes españoles felicitan a De La Espriella tras su triunfo electoral</t>
         </is>
       </c>
       <c r="E120" s="4" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/canal-y-hora-para-ver-los-ultimos-partidos-de-la-fase-de-grupos-del-mundial-2026-colombia-inglaterra-y-mas/202639/</t>
+          <t>https://www.bluradio.com/politica/vladimir-putin-y-lideres-espanoles-felicitan-a-de-la-espriella-tras-su-triunfo-electoral-rg10</t>
         </is>
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="5" t="inlineStr"/>
+      <c r="A121" s="5" t="inlineStr">
+        <is>
+          <t>26/06/2026 08:36 p. m.</t>
+        </is>
+      </c>
       <c r="B121" s="5" t="inlineStr">
         <is>
           <t>Medio de Comunicación</t>
@@ -3566,24 +3618,24 @@
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>Semana</t>
+          <t>Blu Radio</t>
         </is>
       </c>
       <c r="D121" s="6" t="inlineStr">
         <is>
-          <t>Lista de selecciones clasificadas y eliminadas del Mundial 2026, tras los partidos del 26 de junio</t>
+          <t>Caso Natalia Villalba: capturan en Ecuador a británico que sería el responsable</t>
         </is>
       </c>
       <c r="E121" s="7" t="inlineStr">
         <is>
-          <t>https://www.semana.com/deportes/articulo/lista-de-selecciones-clasificadas-y-eliminadas-del-mundial-2026-tras-los-partidos-del-26-de-junio/202603/</t>
+          <t>https://www.bluradio.com/judicial/caso-natalia-villalba-capturan-en-ecuador-a-britanico-que-seria-el-responsable-rs15</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>27/06/2026 03:09 a. m.</t>
+          <t>26/06/2026 08:23 p. m.</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
@@ -3598,19 +3650,19 @@
       </c>
       <c r="D122" s="3" t="inlineStr">
         <is>
-          <t>Resultados de MiLoto del viernes 26 de junio de 2026</t>
+          <t>Circos, conciertos y fiestas: así es la agenda cultural para este puente festivo en Antioquia</t>
         </is>
       </c>
       <c r="E122" s="4" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/economia/juegos-de-azar/resultados-de-miloto-del-viernes-26-de-junio-de-2026-so35</t>
+          <t>https://www.bluradio.com/regiones/antioquia/circos-conciertos-y-fiestas-asi-es-la-agenda-cultural-para-este-puente-festivo-en-antioquia-so35</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="5" t="inlineStr">
         <is>
-          <t>27/06/2026 02:59 a. m.</t>
+          <t>26/06/2026 08:09 p. m.</t>
         </is>
       </c>
       <c r="B123" s="5" t="inlineStr">
@@ -3625,19 +3677,19 @@
       </c>
       <c r="D123" s="6" t="inlineStr">
         <is>
-          <t>Lotería de Risaralda, resultados del viernes 26 de junio de 2026</t>
+          <t>Gobierno nacional abrió proceso de vigilancia especial a la Universidad de Medellín</t>
         </is>
       </c>
       <c r="E123" s="7" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/economia/juegos-de-azar/loteria-de-risaralda-resultados-del-viernes-26-de-junio-de-2026-so35</t>
+          <t>https://www.bluradio.com/regiones/antioquia/gobierno-nacional-abrio-proceso-de-vigilancia-especial-a-la-universidad-de-medellin-rg10</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>27/06/2026 02:57 a. m.</t>
+          <t>26/06/2026 08:04 p. m.</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
@@ -3652,19 +3704,19 @@
       </c>
       <c r="D124" s="3" t="inlineStr">
         <is>
-          <t>Lotería de Santander, resultados del viernes 26 de junio de 2026</t>
+          <t>Astro Luna, resultado del viernes 26 de junio de 2026</t>
         </is>
       </c>
       <c r="E124" s="4" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/economia/juegos-de-azar/loteria-de-santander-resultados-del-viernes-26-de-junio-de-2026-so35</t>
+          <t>https://www.bluradio.com/economia/juegos-de-azar/astro-luna-resultado-del-viernes-26-de-junio-de-2026-so35</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="5" t="inlineStr">
         <is>
-          <t>27/06/2026 02:52 a. m.</t>
+          <t>27/06/2026 03:06 a. m.</t>
         </is>
       </c>
       <c r="B125" s="5" t="inlineStr">
@@ -3674,24 +3726,24 @@
       </c>
       <c r="C125" s="5" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D125" s="6" t="inlineStr">
         <is>
-          <t>Lotería de Medellín, resultado del viernes 26 de junio</t>
+          <t>Las voces de la tragedia: colombianos relatan el terror que aún se vive en Venezuela</t>
         </is>
       </c>
       <c r="E125" s="7" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/economia/juegos-de-azar/loteria-de-medellin-resultado-del-viernes-26-de-junio-so35</t>
+          <t>https://www.semana.com/mundo/articulo/las-voces-de-la-tragedia-colombianos-relatan-el-terror-que-aun-se-vive-en-venezuela/202616/</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>26/06/2026 11:05 p. m.</t>
+          <t>27/06/2026 03:06 a. m.</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
@@ -3701,24 +3753,24 @@
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D126" s="3" t="inlineStr">
         <is>
-          <t>¿Dónde ver el partido Colombia vs. Portugal en Bogotá? Planes gratuitos para apoyar a la Tricolor</t>
+          <t>Rodrigo Lara alerta contratación exprés y anuncia bloque de búsqueda anticorrupción: “No habrá acuerdos burocráticos, oscuros o transaccionales”</t>
         </is>
       </c>
       <c r="E126" s="4" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/regiones/bogota/donde-ver-el-partido-colombia-vs-portugal-en-bogota-planes-gratuitos-para-apoyar-a-la-tricolor-so35</t>
+          <t>https://www.semana.com/politica/articulo/rodrigo-lara-alerta-contratacion-expres-y-anuncia-bloque-de-busqueda-anticorrupcion-no-habra-acuerdos-burocraticos-oscuros-o-transaccionales/202635/</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="5" t="inlineStr">
         <is>
-          <t>26/06/2026 10:36 p. m.</t>
+          <t>27/06/2026 03:06 a. m.</t>
         </is>
       </c>
       <c r="B127" s="5" t="inlineStr">
@@ -3728,24 +3780,24 @@
       </c>
       <c r="C127" s="5" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D127" s="6" t="inlineStr">
         <is>
-          <t>Bomberos de Medellín que apoyarán labores de rescate no han podido entrar a Venezuela</t>
+          <t>Abelardo De La Espriella tendría mayorías en el Congreso para tramitar sus reformas. Esta será la estrategia para sacar adelante sus propuestas</t>
         </is>
       </c>
       <c r="E127" s="7" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/regiones/antioquia/bomberos-de-medellin-que-apoyaran-labores-de-rescate-no-han-podido-entrar-a-venezuela-rg10</t>
+          <t>https://www.semana.com/politica/articulo/abelardo-de-la-espriella-tendria-mayorias-en-el-congreso-para-tramitar-sus-reformas-esta-sera-la-estrategia-para-sacar-adelante-sus-propuestas/202611/</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>26/06/2026 09:42 p. m.</t>
+          <t>27/06/2026 03:06 a. m.</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
@@ -3755,24 +3807,24 @@
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D128" s="3" t="inlineStr">
         <is>
-          <t>Uruguay, eliminada del Mundial 2026 tras una dura derrota contra España</t>
+          <t>El gabinete de Abelardo De La Espriella: SEMANA revela el listado de algunas personas que podrían conformar el nuevo Gobierno</t>
         </is>
       </c>
       <c r="E128" s="4" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/deportes/futbol/copa-mundial-de-la-fifa-2026/uruguay-vs-espana-en-vivo-por-el-mundial-2026-vea-gratis-y-online-el-partido-rg10</t>
+          <t>https://www.semana.com/politica/articulo/el-gabinete-de-abelardo-de-la-espriella-semana-revela-el-listado-de-algunas-personas-que-podrian-conformar-el-nuevo-gobierno/202621/</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="5" t="inlineStr">
         <is>
-          <t>26/06/2026 09:39 p. m.</t>
+          <t>27/06/2026 02:06 a. m.</t>
         </is>
       </c>
       <c r="B129" s="5" t="inlineStr">
@@ -3782,24 +3834,24 @@
       </c>
       <c r="C129" s="5" t="inlineStr">
         <is>
-          <t>Blu Radio</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="D129" s="6" t="inlineStr">
         <is>
-          <t>Vladimir Putin y líderes españoles felicitan a De La Espriella tras su triunfo electoral</t>
+          <t>Keiko Fujimori triunfa en Perú y América Latina consolida el giro a la derecha, en medio de denuncias de fraude y silencios de la izquierda</t>
         </is>
       </c>
       <c r="E129" s="7" t="inlineStr">
         <is>
-          <t>https://www.bluradio.com/politica/vladimir-putin-y-lideres-espanoles-felicitan-a-de-la-espriella-tras-su-triunfo-electoral-rg10</t>
+          <t>https://www.semana.com/mundo/articulo/keiko-fujimori-triunfa-en-peru-y-america-latina-consolida-el-giro-a-la-derecha-en-medio-de-denuncias-de-fraude-y-silencios-de-la-izquierda/202615/</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t